<commit_message>
feat(brand): add Procera brand assets, brand guide and design-system mapping (BPMS-034)
- assets/brand: original concept-board exports (source/) plus cleaned logo,
  symbol, dark-mode wordmark, square app icons, favicon set and marketing art
- assets/brand/README.md: brand copy, pillars, palette with WCAG contrast,
  file index, logo usage rules, production caveats
- docs/05 §7.1.1: brand roles (brand red for logo/focus/active, charcoal
  primary actions, distinct danger colour), verified contrast ratios
- README header banner + tagline + pillars; NOTICE/GOVERNANCE: brand assets
  are trademarks, not Apache-licensed
- tracker: BPMS-034 (vector masters + clearance); register U-16

Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BacklogT" displayName="BacklogT" ref="A1:O109" headerRowCount="1">
-  <autoFilter ref="A1:O109"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BacklogT" displayName="BacklogT" ref="A1:O110" headerRowCount="1">
+  <autoFilter ref="A1:O110"/>
   <tableColumns count="15">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Area"/>
@@ -340,8 +340,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="UnknownsT" displayName="UnknownsT" ref="A1:F16" headerRowCount="1">
-  <autoFilter ref="A1:F16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="UnknownsT" displayName="UnknownsT" ref="A1:F17" headerRowCount="1">
+  <autoFilter ref="A1:F17"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Source"/>
     <tableColumn id="2" name="ID"/>
@@ -824,7 +824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1323,25 +1323,57 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
+          <t>U-16</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Brand assets are raster concept extractions; production vector masters and a small-size symbol are needed</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Logo/favicon quality, print, app icons</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Commission or produce SVG masters (BPMS-034); re-export icon and favicon sets</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
           <t>U-15</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Browser support matrix</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>QA cost</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>Decide: last 2 versions of Chromium/Firefox/Safari; no IE/legacy Edge</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>M1</t>
         </is>
@@ -2808,7 +2840,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O109"/>
+  <dimension ref="A1:O110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4568,17 +4600,17 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>BPMS-040</t>
+          <t>BPMS-034</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>LIB</t>
+          <t>BRAND</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Artifacts, versions, lifecycle state machine, immutability trigger, SoD</t>
+          <t>Brand vector masters (SVG symbol/wordmark/lockups, small-size symbol), favicon/PWA icon set from vector, trademark &amp; domain search</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -4593,29 +4625,25 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Design + Product</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>FR-G04, T07</t>
+          <t>assets/brand, OQ-01, U-16</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>T07 passes</t>
+          <t>SVGs in assets/brand/vector; clearance memo</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J30" s="3" t="inlineStr">
-        <is>
-          <t>BPMS-024,026</t>
-        </is>
-      </c>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr"/>
       <c r="K30" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -4629,7 +4657,7 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>BPMS-041</t>
+          <t>BPMS-040</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -4639,7 +4667,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Landscape, collections, owners, RACI, visibility</t>
+          <t>Artifacts, versions, lifecycle state machine, immutability trigger, SoD</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -4654,27 +4682,27 @@
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Fullstack</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>FR-G01/G02</t>
+          <t>FR-G04, T07</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>Search authorized-only</t>
+          <t>T07 passes</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>BPMS-040</t>
+          <t>BPMS-024,026</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
@@ -4690,7 +4718,7 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>BPMS-042</t>
+          <t>BPMS-041</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -4700,7 +4728,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>SOP/policy block editor + renderer (web/PDF)</t>
+          <t>Landscape, collections, owners, RACI, visibility</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -4715,22 +4743,22 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>FE</t>
+          <t>Fullstack</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>FR-G03, ADR-0013, U-10</t>
+          <t>FR-G01/G02</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>Tagged PDF export</t>
+          <t>Search authorized-only</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr">
@@ -4751,7 +4779,7 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>BPMS-043</t>
+          <t>BPMS-042</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -4761,7 +4789,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Semantic diff across artifact kinds</t>
+          <t>SOP/policy block editor + renderer (web/PDF)</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -4776,22 +4804,22 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Fullstack</t>
+          <t>FE</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>FR-G05</t>
+          <t>FR-G03, ADR-0013, U-10</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>Diff covers bundle artifacts</t>
+          <t>Tagged PDF export</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
@@ -4812,7 +4840,7 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>BPMS-044</t>
+          <t>BPMS-043</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -4822,7 +4850,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Reviews, change requests, effective-date scheduling, renewal date, verification badge</t>
+          <t>Semantic diff across artifact kinds</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -4842,12 +4870,12 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>FR-G05/G07, FX-G01/G02</t>
+          <t>FR-G05</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>Expired flagged</t>
+          <t>Diff covers bundle artifacts</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -4873,7 +4901,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>BPMS-045</t>
+          <t>BPMS-044</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -4883,7 +4911,7 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Policy library + employee policy portal + applicability</t>
+          <t>Reviews, change requests, effective-date scheduling, renewal date, verification badge</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -4903,12 +4931,12 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>FR-PL01–PL03</t>
+          <t>FR-G05/G07, FX-G01/G02</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>Applicability enforced</t>
+          <t>Expired flagged</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
@@ -4918,7 +4946,7 @@
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>BPMS-042</t>
+          <t>BPMS-040</t>
         </is>
       </c>
       <c r="K35" s="3" t="inlineStr">
@@ -4934,17 +4962,17 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>BPMS-046</t>
+          <t>BPMS-045</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>CAMP</t>
+          <t>LIB</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Campaign engine: ack/quiz-lite, audience snapshot, reminders, escalation, new joiners, evidence export</t>
+          <t>Policy library + employee policy portal + applicability</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -4959,27 +4987,27 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Fullstack</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>FR-AK01–04, ADR-0017</t>
+          <t>FR-PL01–PL03</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>5k recipients/min</t>
+          <t>Applicability enforced</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>BPMS-029</t>
+          <t>BPMS-042</t>
         </is>
       </c>
       <c r="K36" s="3" t="inlineStr">
@@ -4995,17 +5023,17 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>BPMS-047</t>
+          <t>BPMS-046</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>COMMS</t>
+          <t>CAMP</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Announcements: compose, targeting, schedule/expiry, pin, required ack, approval, analytics</t>
+          <t>Campaign engine: ack/quiz-lite, audience snapshot, reminders, escalation, new joiners, evidence export</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -5020,17 +5048,17 @@
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Fullstack</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>FR-AN01–06, FX-C01</t>
+          <t>FR-AK01–04, ADR-0017</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>J14 passes</t>
+          <t>5k recipients/min</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
@@ -5040,7 +5068,7 @@
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>BPMS-046</t>
+          <t>BPMS-029</t>
         </is>
       </c>
       <c r="K37" s="3" t="inlineStr">
@@ -5056,17 +5084,17 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>BPMS-048</t>
+          <t>BPMS-047</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>NOTIF</t>
+          <t>COMMS</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>In-app notification centre + SMTP email + templates + digests</t>
+          <t>Announcements: compose, targeting, schedule/expiry, pin, required ack, approval, analytics</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -5086,22 +5114,22 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>FR-N01/N02/N04</t>
+          <t>FR-AN01–06, FX-C01</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>Bounce handling</t>
+          <t>J14 passes</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>BPMS-029</t>
+          <t>BPMS-046</t>
         </is>
       </c>
       <c r="K38" s="3" t="inlineStr">
@@ -5117,17 +5145,17 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>BPMS-049</t>
+          <t>BPMS-048</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>SRCH</t>
+          <t>NOTIF</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Postgres FTS + trgm, permission-filtered search</t>
+          <t>In-app notification centre + SMTP email + templates + digests</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -5142,17 +5170,17 @@
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Fullstack</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>04 §6</t>
+          <t>FR-N01/N02/N04</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>No restricted leakage</t>
+          <t>Bounce handling</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
@@ -5162,7 +5190,7 @@
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>BPMS-040</t>
+          <t>BPMS-029</t>
         </is>
       </c>
       <c r="K39" s="3" t="inlineStr">
@@ -5178,17 +5206,17 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>BPMS-060</t>
+          <t>BPMS-049</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>FILE</t>
+          <t>SRCH</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Files pipeline: resumable upload, hash, sniff, ClamAV, quarantine, signed URLs</t>
+          <t>Postgres FTS + trgm, permission-filtered search</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -5208,22 +5236,22 @@
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>FR-F01–F03, F05</t>
+          <t>04 §6</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>EICAR quarantined; SEC-10</t>
+          <t>No restricted leakage</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>BPMS-030</t>
+          <t>BPMS-040</t>
         </is>
       </c>
       <c r="K40" s="3" t="inlineStr">
@@ -5239,7 +5267,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>BPMS-061</t>
+          <t>BPMS-060</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -5249,7 +5277,7 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Previews (image/PDF) in sandbox; Office preview spike</t>
+          <t>Files pipeline: resumable upload, hash, sniff, ClamAV, quarantine, signed URLs</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -5269,22 +5297,22 @@
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>FR-F04, U-08</t>
+          <t>FR-F01–F03, F05</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>No active content</t>
+          <t>EICAR quarantined; SEC-10</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>BPMS-060</t>
+          <t>BPMS-030</t>
         </is>
       </c>
       <c r="K41" s="3" t="inlineStr">
@@ -5300,7 +5328,7 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>BPMS-062</t>
+          <t>BPMS-061</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -5310,7 +5338,7 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Workspace Files view, quotas, orphan cleanup</t>
+          <t>Previews (image/PDF) in sandbox; Office preview spike</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -5325,17 +5353,17 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>FE</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>FR-F06/F07</t>
+          <t>FR-F04, U-08</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>Held files undeletable</t>
+          <t>No active content</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
@@ -5345,7 +5373,7 @@
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>BPMS-060,028</t>
+          <t>BPMS-060</t>
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
@@ -5361,17 +5389,17 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>BPMS-063</t>
+          <t>BPMS-062</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>FILE</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard + people &amp; access monitor</t>
+          <t>Workspace Files view, quotas, orphan cleanup</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -5391,22 +5419,22 @@
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>FR-A01/A06</t>
+          <t>FR-F06/F07</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>Every tile drills down</t>
+          <t>Held files undeletable</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>BPMS-028</t>
+          <t>BPMS-060,028</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
@@ -5422,17 +5450,17 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>BPMS-064</t>
+          <t>BPMS-063</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>AUD</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Audit explorer, timelines, saved queries, export</t>
+          <t>Workspace overview dashboard + people &amp; access monitor</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -5447,17 +5475,17 @@
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>Fullstack</t>
+          <t>FE</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>FR-T03/T04</t>
+          <t>FR-A01/A06</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>P95&lt;2s @10M</t>
+          <t>Every tile drills down</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
@@ -5467,7 +5495,7 @@
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>BPMS-026</t>
+          <t>BPMS-028</t>
         </is>
       </c>
       <c r="K44" s="3" t="inlineStr">
@@ -5483,17 +5511,17 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>BPMS-065</t>
+          <t>BPMS-064</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>PLAT</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>System console: workspaces grid, quotas, health, system audit</t>
+          <t>Audit explorer, timelines, saved queries, export</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -5508,27 +5536,27 @@
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>FE</t>
+          <t>Fullstack</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>FR-S02–S09</t>
+          <t>FR-T03/T04</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P95&lt;2s @10M</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>BPMS-020</t>
+          <t>BPMS-026</t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr">
@@ -5544,17 +5572,17 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>BPMS-120</t>
+          <t>BPMS-065</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>PILOT</t>
+          <t>PLAT</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Pilot workspaces (Starter + Enterprise profile), 3–5 real processes, 4 weeks</t>
+          <t>System console: workspaces grid, quotas, health, system audit</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -5569,27 +5597,27 @@
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>FE</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>G3</t>
+          <t>FR-S02–S09</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>G3 checklist</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>M6</t>
+          <t>BPMS-020</t>
         </is>
       </c>
       <c r="K46" s="3" t="inlineStr">
@@ -5605,17 +5633,17 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>BPMS-080</t>
+          <t>BPMS-120</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>RT</t>
+          <t>PILOT</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>IR v1 model + compiler (§11 checks, diagnostics, semantic diff)</t>
+          <t>Pilot workspaces (Starter + Enterprise profile), 3–5 real processes, 4 weeks</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -5625,22 +5653,22 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Runtime</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>11, ADR-0003</t>
+          <t>G3</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>All checks covered</t>
+          <t>G3 checklist</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
@@ -5650,7 +5678,7 @@
       </c>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t>BPMS-009</t>
+          <t>M6</t>
         </is>
       </c>
       <c r="K47" s="3" t="inlineStr">
@@ -5666,7 +5694,7 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>BPMS-081</t>
+          <t>BPMS-080</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -5676,7 +5704,7 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Expression engine integration (typed, budgeted, WASM build)</t>
+          <t>IR v1 model + compiler (§11 checks, diagnostics, semantic diff)</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -5696,17 +5724,17 @@
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>ADR-0010</t>
+          <t>11, ADR-0003</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>Budget exhaustion = incident</t>
+          <t>All checks covered</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J48" s="3" t="inlineStr">
@@ -5727,7 +5755,7 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>BPMS-082</t>
+          <t>BPMS-081</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -5737,7 +5765,7 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Interpreter: advance loop, tokens, splits/joins, end/terminate</t>
+          <t>Expression engine integration (typed, budgeted, WASM build)</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -5757,22 +5785,22 @@
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>04 §4</t>
+          <t>ADR-0010</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>Conformance green</t>
+          <t>Budget exhaustion = incident</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J49" s="3" t="inlineStr">
         <is>
-          <t>BPMS-080</t>
+          <t>BPMS-009</t>
         </is>
       </c>
       <c r="K49" s="3" t="inlineStr">
@@ -5788,7 +5816,7 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>BPMS-083</t>
+          <t>BPMS-082</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -5798,7 +5826,7 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Jobs + timers + scheduler with leases/fencing; calendars; SLA clocks</t>
+          <t>Interpreter: advance loop, tokens, splits/joins, end/terminate</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -5818,12 +5846,12 @@
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>04 §4.4, FR-E12</t>
+          <t>04 §4</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>T06; lateness SLO</t>
+          <t>Conformance green</t>
         </is>
       </c>
       <c r="I50" s="3" t="inlineStr">
@@ -5833,7 +5861,7 @@
       </c>
       <c r="J50" s="3" t="inlineStr">
         <is>
-          <t>BPMS-082</t>
+          <t>BPMS-080</t>
         </is>
       </c>
       <c r="K50" s="3" t="inlineStr">
@@ -5849,7 +5877,7 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>BPMS-084</t>
+          <t>BPMS-083</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -5859,7 +5887,7 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Release bundles + publish integration</t>
+          <t>Jobs + timers + scheduler with leases/fencing; calendars; SLA clocks</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -5879,22 +5907,22 @@
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>ADR-0012</t>
+          <t>04 §4.4, FR-E12</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>T03 passes</t>
+          <t>T06; lateness SLO</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J51" s="3" t="inlineStr">
         <is>
-          <t>BPMS-040,080</t>
+          <t>BPMS-082</t>
         </is>
       </c>
       <c r="K51" s="3" t="inlineStr">
@@ -5910,17 +5938,17 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>BPMS-085</t>
+          <t>BPMS-084</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>WORK</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Work items, assignment strategies, manager chain, DoA matrix, quorum, per-group</t>
+          <t>Release bundles + publish integration</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -5935,27 +5963,27 @@
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Runtime</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>FR-E04/E05, FX-D01/D02, FX-E01</t>
+          <t>ADR-0012</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>T01 passes</t>
+          <t>T03 passes</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J52" s="3" t="inlineStr">
         <is>
-          <t>BPMS-082,023</t>
+          <t>BPMS-040,080</t>
         </is>
       </c>
       <c r="K52" s="3" t="inlineStr">
@@ -5971,7 +5999,7 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>BPMS-086</t>
+          <t>BPMS-085</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -5981,7 +6009,7 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Delegation, OOO substitution, SoD re-check, send-back</t>
+          <t>Work items, assignment strategies, manager chain, DoA matrix, quorum, per-group</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -6001,22 +6029,22 @@
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>12 §9/§10, FX-E05</t>
+          <t>FR-E04/E05, FX-D01/D02, FX-E01</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>T05 passes</t>
+          <t>T01 passes</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr">
         <is>
-          <t>BPMS-085</t>
+          <t>BPMS-082,023</t>
         </is>
       </c>
       <c r="K53" s="3" t="inlineStr">
@@ -6032,17 +6060,17 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>BPMS-087</t>
+          <t>BPMS-086</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>RT</t>
+          <t>WORK</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Rule tables (UNIQUE/FIRST/COLLECT)</t>
+          <t>Delegation, OOO substitution, SoD re-check, send-back</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -6057,17 +6085,17 @@
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>Runtime</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>FR-E10</t>
+          <t>12 §9/§10, FX-E05</t>
         </is>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>Deterministic</t>
+          <t>T05 passes</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
@@ -6077,7 +6105,7 @@
       </c>
       <c r="J54" s="3" t="inlineStr">
         <is>
-          <t>BPMS-081</t>
+          <t>BPMS-085</t>
         </is>
       </c>
       <c r="K54" s="3" t="inlineStr">
@@ -6093,7 +6121,7 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>BPMS-088</t>
+          <t>BPMS-087</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -6103,7 +6131,7 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Incidents, retry/skip/cancel, instance admin ops</t>
+          <t>Rule tables (UNIQUE/FIRST/COLLECT)</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -6118,17 +6146,17 @@
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Runtime</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>FR-E13</t>
+          <t>FR-E10</t>
         </is>
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>One open incident per failure</t>
+          <t>Deterministic</t>
         </is>
       </c>
       <c r="I55" s="3" t="inlineStr">
@@ -6138,7 +6166,7 @@
       </c>
       <c r="J55" s="3" t="inlineStr">
         <is>
-          <t>BPMS-082</t>
+          <t>BPMS-081</t>
         </is>
       </c>
       <c r="K55" s="3" t="inlineStr">
@@ -6154,17 +6182,17 @@
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>BPMS-089</t>
+          <t>BPMS-088</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Conformance suite + model-based tests + deterministic simulation harness</t>
+          <t>Incidents, retry/skip/cancel, instance admin ops</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -6179,22 +6207,22 @@
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>SDET/Runtime</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="G56" s="3" t="inlineStr">
         <is>
-          <t>15 §4–6</t>
+          <t>FR-E13</t>
         </is>
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>Nightly chaos green</t>
+          <t>One open incident per failure</t>
         </is>
       </c>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J56" s="3" t="inlineStr">
@@ -6215,17 +6243,17 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>BPMS-100</t>
+          <t>BPMS-089</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>DES</t>
+          <t>QA</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Step builder + React Flow canvas + properties + validate/test-run/review/publish</t>
+          <t>Conformance suite + model-based tests + deterministic simulation harness</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
@@ -6240,27 +6268,27 @@
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>FE</t>
+          <t>SDET/Runtime</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>FR-E01/E11, ADR-0018</t>
+          <t>15 §4–6</t>
         </is>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>T10 keyboard-only</t>
+          <t>Nightly chaos green</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>XL</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J57" s="3" t="inlineStr">
         <is>
-          <t>BPMS-080</t>
+          <t>BPMS-082</t>
         </is>
       </c>
       <c r="K57" s="3" t="inlineStr">
@@ -6276,17 +6304,17 @@
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>BPMS-101</t>
+          <t>BPMS-100</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>DES</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Form builder + renderer (calc, prefill, repeating, lookups, PDF of submission)</t>
+          <t>Step builder + React Flow canvas + properties + validate/test-run/review/publish</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
@@ -6306,12 +6334,12 @@
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>FR-E03, FX-F01–F04</t>
+          <t>FR-E01/E11, ADR-0018</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>Server = client validation</t>
+          <t>T10 keyboard-only</t>
         </is>
       </c>
       <c r="I58" s="3" t="inlineStr">
@@ -6321,7 +6349,7 @@
       </c>
       <c r="J58" s="3" t="inlineStr">
         <is>
-          <t>BPMS-081</t>
+          <t>BPMS-080</t>
         </is>
       </c>
       <c r="K58" s="3" t="inlineStr">
@@ -6337,17 +6365,17 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>BPMS-103</t>
+          <t>BPMS-101</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>REQ</t>
+          <t>FORM</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Request portal/catalogue, start form, request detail, comments/@mentions/watchers</t>
+          <t>Form builder + renderer (calc, prefill, repeating, lookups, PDF of submission)</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
@@ -6362,27 +6390,27 @@
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>Fullstack</t>
+          <t>FE</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>FR-R01/R02, FX-R01/R02</t>
+          <t>FR-E03, FX-F01–F04</t>
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>J0/J3 pass</t>
+          <t>Server = client validation</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>XL</t>
         </is>
       </c>
       <c r="J59" s="3" t="inlineStr">
         <is>
-          <t>BPMS-082</t>
+          <t>BPMS-081</t>
         </is>
       </c>
       <c r="K59" s="3" t="inlineStr">
@@ -6398,17 +6426,17 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>BPMS-105</t>
+          <t>BPMS-103</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>WORK</t>
+          <t>REQ</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>My Work 3-pane inbox (tasks, acks, signatures), bulk with preview</t>
+          <t>Request portal/catalogue, start form, request detail, comments/@mentions/watchers</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -6423,17 +6451,17 @@
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>FE</t>
+          <t>Fullstack</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>FR-R03, FR-AK02</t>
+          <t>FR-R01/R02, FX-R01/R02</t>
         </is>
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>Decision ≤3 interactions</t>
+          <t>J0/J3 pass</t>
         </is>
       </c>
       <c r="I60" s="3" t="inlineStr">
@@ -6443,7 +6471,7 @@
       </c>
       <c r="J60" s="3" t="inlineStr">
         <is>
-          <t>BPMS-085,046</t>
+          <t>BPMS-082</t>
         </is>
       </c>
       <c r="K60" s="3" t="inlineStr">
@@ -6459,17 +6487,17 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>BPMS-106</t>
+          <t>BPMS-105</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>TPL</t>
+          <t>WORK</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Template gallery + install wizard + Wave-1 templates (13)</t>
+          <t>My Work 3-pane inbox (tasks, acks, signatures), bulk with preview</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -6484,27 +6512,27 @@
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>Fullstack/SMEs</t>
+          <t>FE</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>FR-G08, TPL-001..</t>
+          <t>FR-R03, FR-AK02</t>
         </is>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>All W1 test-run green</t>
+          <t>Decision ≤3 interactions</t>
         </is>
       </c>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>XL</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J61" s="3" t="inlineStr">
         <is>
-          <t>BPMS-100,101</t>
+          <t>BPMS-085,046</t>
         </is>
       </c>
       <c r="K61" s="3" t="inlineStr">
@@ -6520,17 +6548,17 @@
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>BPMS-111</t>
+          <t>BPMS-106</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>E2E</t>
+          <t>TPL</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2 pack (R2-01…16 + ISO) + Firefox</t>
+          <t>Template gallery + install wizard + Wave-1 templates (13)</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -6545,27 +6573,27 @@
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>SDET + feature owners</t>
+          <t>Fullstack/SMEs</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>23 §5</t>
+          <t>FR-G08, TPL-001..</t>
         </is>
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>Green; race/restart/timer stable</t>
+          <t>All W1 test-run green</t>
         </is>
       </c>
       <c r="I62" s="3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>XL</t>
         </is>
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
-          <t>BPMS-032</t>
+          <t>BPMS-100,101</t>
         </is>
       </c>
       <c r="K62" s="3" t="inlineStr">
@@ -6581,17 +6609,17 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>BPMS-121</t>
+          <t>BPMS-111</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>E2E</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Usability round + SUS measurement + fixes</t>
+          <t>E2E-R2 pack (R2-01…16 + ISO) + Firefox</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -6606,27 +6634,27 @@
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>SDET + feature owners</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>02 §9</t>
+          <t>23 §5</t>
         </is>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>SUS targets</t>
+          <t>Green; race/restart/timer stable</t>
         </is>
       </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr">
         <is>
-          <t>BPMS-120</t>
+          <t>BPMS-032</t>
         </is>
       </c>
       <c r="K63" s="3" t="inlineStr">
@@ -6642,17 +6670,17 @@
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>BPMS-066</t>
+          <t>BPMS-121</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>AUD</t>
+          <t>UX</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Retention policy per record class (policy only)</t>
+          <t>Usability round + SUS measurement + fixes</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
@@ -6662,22 +6690,22 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
         <is>
-          <t>PRV-04</t>
+          <t>02 §9</t>
         </is>
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>Jobs honour classes</t>
+          <t>SUS targets</t>
         </is>
       </c>
       <c r="I64" s="3" t="inlineStr">
@@ -6687,7 +6715,7 @@
       </c>
       <c r="J64" s="3" t="inlineStr">
         <is>
-          <t>BPMS-026</t>
+          <t>BPMS-120</t>
         </is>
       </c>
       <c r="K64" s="3" t="inlineStr">
@@ -6703,17 +6731,17 @@
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>BPMS-102</t>
+          <t>BPMS-066</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>DATA</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Master-data tables (CSV import, lookups, versioned)</t>
+          <t>Retention policy per record class (policy only)</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
@@ -6728,17 +6756,17 @@
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Fullstack</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
         <is>
-          <t>FX-E02</t>
+          <t>PRV-04</t>
         </is>
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
-          <t>Cascading dropdowns</t>
+          <t>Jobs honour classes</t>
         </is>
       </c>
       <c r="I65" s="3" t="inlineStr">
@@ -6748,7 +6776,7 @@
       </c>
       <c r="J65" s="3" t="inlineStr">
         <is>
-          <t>BPMS-101</t>
+          <t>BPMS-026</t>
         </is>
       </c>
       <c r="K65" s="3" t="inlineStr">
@@ -6764,17 +6792,17 @@
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>BPMS-104</t>
+          <t>BPMS-102</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>REQ</t>
+          <t>DATA</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw, edit-after-submit, request-on-behalf, numbering</t>
+          <t>Master-data tables (CSV import, lookups, versioned)</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
@@ -6789,17 +6817,17 @@
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Fullstack</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
         <is>
-          <t>FX-E03/E04/E06</t>
+          <t>FX-E02</t>
         </is>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>Audited</t>
+          <t>Cascading dropdowns</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
@@ -6809,7 +6837,7 @@
       </c>
       <c r="J66" s="3" t="inlineStr">
         <is>
-          <t>BPMS-103</t>
+          <t>BPMS-101</t>
         </is>
       </c>
       <c r="K66" s="3" t="inlineStr">
@@ -6825,17 +6853,17 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>BPMS-107</t>
+          <t>BPMS-104</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>SIGN</t>
+          <t>REQ</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>E-sign v1: PDF, recipients/roles, routing, bulk, fields, consent step, ceremony, certificate</t>
+          <t>Recall/withdraw, edit-after-submit, request-on-behalf, numbering</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
@@ -6850,27 +6878,27 @@
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>Fullstack</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="G67" s="3" t="inlineStr">
         <is>
-          <t>FR-DS01–07, FX-S01/02/05/06/07</t>
+          <t>FX-E03/E04/E06</t>
         </is>
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>J13 passes</t>
+          <t>Audited</t>
         </is>
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>XL</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr">
         <is>
-          <t>BPMS-046,060</t>
+          <t>BPMS-103</t>
         </is>
       </c>
       <c r="K67" s="3" t="inlineStr">
@@ -6886,17 +6914,17 @@
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>BPMS-108</t>
+          <t>BPMS-107</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>SIGN</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>All requests / all work / workload / process health / ops monitor</t>
+          <t>E-sign v1: PDF, recipients/roles, routing, bulk, fields, consent step, ceremony, certificate</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
@@ -6911,27 +6939,27 @@
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>FE</t>
+          <t>Fullstack</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
         <is>
-          <t>FR-A02–A05</t>
+          <t>FR-DS01–07, FX-S01/02/05/06/07</t>
         </is>
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>Bulk audited</t>
+          <t>J13 passes</t>
         </is>
       </c>
       <c r="I68" s="3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>XL</t>
         </is>
       </c>
       <c r="J68" s="3" t="inlineStr">
         <is>
-          <t>BPMS-063,085</t>
+          <t>BPMS-046,060</t>
         </is>
       </c>
       <c r="K68" s="3" t="inlineStr">
@@ -6947,17 +6975,17 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>BPMS-109</t>
+          <t>BPMS-108</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>PWA (360px) for My Work, requests, acks, signing</t>
+          <t>All requests / all work / workload / process health / ops monitor</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
@@ -6977,22 +7005,22 @@
       </c>
       <c r="G69" s="3" t="inlineStr">
         <is>
-          <t>FR-P07</t>
+          <t>FR-A02–A05</t>
         </is>
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>Lighthouse PWA pass</t>
+          <t>Bulk audited</t>
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr">
         <is>
-          <t>BPMS-105</t>
+          <t>BPMS-063,085</t>
         </is>
       </c>
       <c r="K69" s="3" t="inlineStr">
@@ -7008,17 +7036,17 @@
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>BPMS-110</t>
+          <t>BPMS-109</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>LIB</t>
+          <t>UX</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>BPMN 2.0 XML import (subset) + compatibility report</t>
+          <t>PWA (360px) for My Work, requests, acks, signing</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
@@ -7033,17 +7061,17 @@
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>Runtime</t>
+          <t>FE</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
         <is>
-          <t>FR-G09, SP-06</t>
+          <t>FR-P07</t>
         </is>
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>Unsupported listed</t>
+          <t>Lighthouse PWA pass</t>
         </is>
       </c>
       <c r="I70" s="3" t="inlineStr">
@@ -7053,7 +7081,7 @@
       </c>
       <c r="J70" s="3" t="inlineStr">
         <is>
-          <t>BPMS-080</t>
+          <t>BPMS-105</t>
         </is>
       </c>
       <c r="K70" s="3" t="inlineStr">
@@ -7069,17 +7097,17 @@
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>BPMS-112</t>
+          <t>BPMS-110</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>E2E</t>
+          <t>LIB</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3 pack (R3-01…12 + MOB + ISO) + WebKit</t>
+          <t>BPMN 2.0 XML import (subset) + compatibility report</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
@@ -7094,27 +7122,27 @@
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>SDET + feature owners</t>
+          <t>Runtime</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr">
         <is>
-          <t>23 §5</t>
+          <t>FR-G09, SP-06</t>
         </is>
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>Green; bulk-sign 1000</t>
+          <t>Unsupported listed</t>
         </is>
       </c>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J71" s="3" t="inlineStr">
         <is>
-          <t>BPMS-111</t>
+          <t>BPMS-080</t>
         </is>
       </c>
       <c r="K71" s="3" t="inlineStr">
@@ -7130,42 +7158,42 @@
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>BPMS-140</t>
+          <t>BPMS-112</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>IAM</t>
+          <t>E2E</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO, SAML-broker, SSO enforcement, JIT</t>
+          <t>E2E-R3 pack (R3-01…12 + MOB + ISO) + WebKit</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>SDET + feature owners</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr">
         <is>
-          <t>FR-P02, INT-001/002</t>
+          <t>23 §5</t>
         </is>
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>Deprovision test</t>
+          <t>Green; bulk-sign 1000</t>
         </is>
       </c>
       <c r="I72" s="3" t="inlineStr">
@@ -7173,7 +7201,11 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J72" s="3" t="inlineStr"/>
+      <c r="J72" s="3" t="inlineStr">
+        <is>
+          <t>BPMS-111</t>
+        </is>
+      </c>
       <c r="K72" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -7187,7 +7219,7 @@
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>BPMS-141</t>
+          <t>BPMS-140</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
@@ -7197,7 +7229,7 @@
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>SCIM 2.0 server</t>
+          <t>OIDC SSO, SAML-broker, SSO enforcement, JIT</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
@@ -7217,24 +7249,20 @@
       </c>
       <c r="G73" s="3" t="inlineStr">
         <is>
-          <t>INT-003</t>
+          <t>FR-P02, INT-001/002</t>
         </is>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>&lt;5 min deprovision</t>
+          <t>Deprovision test</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J73" s="3" t="inlineStr">
-        <is>
-          <t>BPMS-140</t>
-        </is>
-      </c>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J73" s="3" t="inlineStr"/>
       <c r="K73" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -7248,7 +7276,7 @@
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>BPMS-142</t>
+          <t>BPMS-141</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
@@ -7258,7 +7286,7 @@
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>Scoped/delegated admins; IP allowlists</t>
+          <t>SCIM 2.0 server</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
@@ -7278,12 +7306,12 @@
       </c>
       <c r="G74" s="3" t="inlineStr">
         <is>
-          <t>CFG-018, FR-W06</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>No escalation</t>
+          <t>&lt;5 min deprovision</t>
         </is>
       </c>
       <c r="I74" s="3" t="inlineStr">
@@ -7293,7 +7321,7 @@
       </c>
       <c r="J74" s="3" t="inlineStr">
         <is>
-          <t>BPMS-024</t>
+          <t>BPMS-140</t>
         </is>
       </c>
       <c r="K74" s="3" t="inlineStr">
@@ -7309,17 +7337,17 @@
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>BPMS-143</t>
+          <t>BPMS-142</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>IAM</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Webhooks (Standard Webhooks), HTTP connector via egress proxy, inbound events</t>
+          <t>Scoped/delegated admins; IP allowlists</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
@@ -7334,27 +7362,27 @@
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
         <is>
-          <t>INT-*, WH/SSRF</t>
+          <t>CFG-018, FR-W06</t>
         </is>
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>SEC SSRF tests</t>
+          <t>No escalation</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr">
         <is>
-          <t>BPMS-029</t>
+          <t>BPMS-024</t>
         </is>
       </c>
       <c r="K75" s="3" t="inlineStr">
@@ -7370,7 +7398,7 @@
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>BPMS-144</t>
+          <t>BPMS-143</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
@@ -7380,7 +7408,7 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>Public API hardening, OpenAPI, CLI, TS/Python SDKs</t>
+          <t>Webhooks (Standard Webhooks), HTTP connector via egress proxy, inbound events</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
@@ -7400,20 +7428,24 @@
       </c>
       <c r="G76" s="3" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>INT-*, WH/SSRF</t>
         </is>
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>Spec published</t>
+          <t>SEC SSRF tests</t>
         </is>
       </c>
       <c r="I76" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J76" s="3" t="inlineStr"/>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J76" s="3" t="inlineStr">
+        <is>
+          <t>BPMS-029</t>
+        </is>
+      </c>
       <c r="K76" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -7427,17 +7459,17 @@
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>BPMS-145</t>
+          <t>BPMS-144</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>NOTIF</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approvals, reply-by-email, web push</t>
+          <t>Public API hardening, OpenAPI, CLI, TS/Python SDKs</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
@@ -7452,17 +7484,17 @@
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>Fullstack</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr">
         <is>
-          <t>FR-N03/N05, FX-R03</t>
+          <t>08</t>
         </is>
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
-          <t>Replay rejected</t>
+          <t>Spec published</t>
         </is>
       </c>
       <c r="I77" s="3" t="inlineStr">
@@ -7470,11 +7502,7 @@
           <t>M</t>
         </is>
       </c>
-      <c r="J77" s="3" t="inlineStr">
-        <is>
-          <t>BPMS-048</t>
-        </is>
-      </c>
+      <c r="J77" s="3" t="inlineStr"/>
       <c r="K77" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -7488,17 +7516,17 @@
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>BPMS-146</t>
+          <t>BPMS-145</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>IAM</t>
+          <t>NOTIF</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>Guests + external signers (magic link + OTP); self-serve signing links</t>
+          <t>Email-actionable approvals, reply-by-email, web push</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
@@ -7518,12 +7546,12 @@
       </c>
       <c r="G78" s="3" t="inlineStr">
         <is>
-          <t>FR-P08, FX-S10</t>
+          <t>FR-N03/N05, FX-R03</t>
         </is>
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>Single-use</t>
+          <t>Replay rejected</t>
         </is>
       </c>
       <c r="I78" s="3" t="inlineStr">
@@ -7533,7 +7561,7 @@
       </c>
       <c r="J78" s="3" t="inlineStr">
         <is>
-          <t>BPMS-107</t>
+          <t>BPMS-048</t>
         </is>
       </c>
       <c r="K78" s="3" t="inlineStr">
@@ -7549,17 +7577,17 @@
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>BPMS-147</t>
+          <t>BPMS-146</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>SIGN</t>
+          <t>IAM</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>E-sign v2: DOCX + merge, anchor tags, conditional fields, delegate, correction, embedded</t>
+          <t>Guests + external signers (magic link + OTP); self-serve signing links</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
@@ -7579,17 +7607,17 @@
       </c>
       <c r="G79" s="3" t="inlineStr">
         <is>
-          <t>FX-S03/04/08/09/12</t>
+          <t>FR-P08, FX-S10</t>
         </is>
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
-          <t>Audited corrections</t>
+          <t>Single-use</t>
         </is>
       </c>
       <c r="I79" s="3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J79" s="3" t="inlineStr">
@@ -7610,17 +7638,17 @@
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>BPMS-148</t>
+          <t>BPMS-147</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>SIGN</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>Public forms (privacy CAPTCHA), save &amp; resume, partials, form signature field</t>
+          <t>E-sign v2: DOCX + merge, anchor tags, conditional fields, delegate, correction, embedded</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
@@ -7640,22 +7668,22 @@
       </c>
       <c r="G80" s="3" t="inlineStr">
         <is>
-          <t>FX-F05–F07</t>
+          <t>FX-S03/04/08/09/12</t>
         </is>
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>Rate-limited</t>
+          <t>Audited corrections</t>
         </is>
       </c>
       <c r="I80" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J80" s="3" t="inlineStr">
         <is>
-          <t>BPMS-101</t>
+          <t>BPMS-107</t>
         </is>
       </c>
       <c r="K80" s="3" t="inlineStr">
@@ -7671,17 +7699,17 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>BPMS-149</t>
+          <t>BPMS-148</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>EXEC</t>
+          <t>FORM</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Subprocesses, reusable sub-flows, duplicate detection, bulk import, env promotion</t>
+          <t>Public forms (privacy CAPTCHA), save &amp; resume, partials, form signature field</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
@@ -7696,27 +7724,27 @@
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>Runtime</t>
+          <t>Fullstack</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr">
         <is>
-          <t>FR-E08, FX-E07–E09, FR-P09</t>
+          <t>FX-F05–F07</t>
         </is>
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rate-limited</t>
         </is>
       </c>
       <c r="I81" s="3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J81" s="3" t="inlineStr">
         <is>
-          <t>BPMS-082</t>
+          <t>BPMS-101</t>
         </is>
       </c>
       <c r="K81" s="3" t="inlineStr">
@@ -7732,17 +7760,17 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>BPMS-150</t>
+          <t>BPMS-149</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>LIB</t>
+          <t>EXEC</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>Auto-generated process documentation; policy exceptions; policy templates</t>
+          <t>Subprocesses, reusable sub-flows, duplicate detection, bulk import, env promotion</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
@@ -7757,12 +7785,12 @@
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>Fullstack</t>
+          <t>Runtime</t>
         </is>
       </c>
       <c r="G82" s="3" t="inlineStr">
         <is>
-          <t>FX-G04, FR-PL04, FX-G03</t>
+          <t>FR-E08, FX-E07–E09, FR-P09</t>
         </is>
       </c>
       <c r="H82" s="3" t="inlineStr">
@@ -7772,12 +7800,12 @@
       </c>
       <c r="I82" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J82" s="3" t="inlineStr">
         <is>
-          <t>BPMS-042</t>
+          <t>BPMS-082</t>
         </is>
       </c>
       <c r="K82" s="3" t="inlineStr">
@@ -7793,17 +7821,17 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>BPMS-151</t>
+          <t>BPMS-150</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>COMMS</t>
+          <t>LIB</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Emergency alerts, content validation period, moderation, quiz</t>
+          <t>Auto-generated process documentation; policy exceptions; policy templates</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
@@ -7823,7 +7851,7 @@
       </c>
       <c r="G83" s="3" t="inlineStr">
         <is>
-          <t>FX-C02–C04</t>
+          <t>FX-G04, FR-PL04, FX-G03</t>
         </is>
       </c>
       <c r="H83" s="3" t="inlineStr">
@@ -7838,7 +7866,7 @@
       </c>
       <c r="J83" s="3" t="inlineStr">
         <is>
-          <t>BPMS-047</t>
+          <t>BPMS-042</t>
         </is>
       </c>
       <c r="K83" s="3" t="inlineStr">
@@ -7854,17 +7882,17 @@
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>BPMS-152</t>
+          <t>BPMS-151</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>E2E</t>
+          <t>COMMS</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4 pack incl. Keycloak, SCIM, webhook receiver</t>
+          <t>Emergency alerts, content validation period, moderation, quiz</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
@@ -7879,27 +7907,27 @@
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>SDET + feature owners</t>
+          <t>Fullstack</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr">
         <is>
-          <t>23 §5</t>
+          <t>FX-C02–C04</t>
         </is>
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I84" s="3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J84" s="3" t="inlineStr">
         <is>
-          <t>BPMS-112</t>
+          <t>BPMS-047</t>
         </is>
       </c>
       <c r="K84" s="3" t="inlineStr">
@@ -7915,17 +7943,17 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>BPMS-160</t>
+          <t>BPMS-152</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>CASE</t>
+          <t>E2E</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Case types, queues, macros, SLAs, link/merge, restricted cases</t>
+          <t>E2E-R4 pack incl. Keycloak, SCIM, webhook receiver</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -7935,32 +7963,32 @@
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>Fullstack</t>
+          <t>SDET + feature owners</t>
         </is>
       </c>
       <c r="G85" s="3" t="inlineStr">
         <is>
-          <t>FR-C01, FX-K01–K06</t>
+          <t>23 §5</t>
         </is>
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
-          <t>J4 passes</t>
+          <t>Green</t>
         </is>
       </c>
       <c r="I85" s="3" t="inlineStr">
         <is>
-          <t>XL</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J85" s="3" t="inlineStr">
         <is>
-          <t>BPMS-082</t>
+          <t>BPMS-112</t>
         </is>
       </c>
       <c r="K85" s="3" t="inlineStr">
@@ -7976,17 +8004,17 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>BPMS-161</t>
+          <t>BPMS-160</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>AUD</t>
+          <t>CASE</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>Investigations: pins, legal hold, signed export, conflict-of-interest</t>
+          <t>Case types, queues, macros, SLAs, link/merge, restricted cases</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
@@ -8006,22 +8034,22 @@
       </c>
       <c r="G86" s="3" t="inlineStr">
         <is>
-          <t>FR-T05/T06, FX-K08, FX-L01</t>
+          <t>FR-C01, FX-K01–K06</t>
         </is>
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>J10 passes</t>
+          <t>J4 passes</t>
         </is>
       </c>
       <c r="I86" s="3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>XL</t>
         </is>
       </c>
       <c r="J86" s="3" t="inlineStr">
         <is>
-          <t>BPMS-064,160</t>
+          <t>BPMS-082</t>
         </is>
       </c>
       <c r="K86" s="3" t="inlineStr">
@@ -8037,7 +8065,7 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>BPMS-162</t>
+          <t>BPMS-161</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
@@ -8047,7 +8075,7 @@
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Checkpoints, RFC 3161, WORM export, procera-verify CLI</t>
+          <t>Investigations: pins, legal hold, signed export, conflict-of-interest</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
@@ -8062,27 +8090,27 @@
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Fullstack</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr">
         <is>
-          <t>AUD-02–05</t>
+          <t>FR-T05/T06, FX-K08, FX-L01</t>
         </is>
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>Verifier detects tamper</t>
+          <t>J10 passes</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J87" s="3" t="inlineStr">
         <is>
-          <t>BPMS-026</t>
+          <t>BPMS-064,160</t>
         </is>
       </c>
       <c r="K87" s="3" t="inlineStr">
@@ -8098,17 +8126,17 @@
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>BPMS-163</t>
+          <t>BPMS-162</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>GOV</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaigns, control mapping, access reviews</t>
+          <t>Checkpoints, RFC 3161, WORM export, procera-verify CLI</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
@@ -8123,17 +8151,17 @@
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>Fullstack</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="G88" s="3" t="inlineStr">
         <is>
-          <t>FR-G06, FR-W11</t>
+          <t>AUD-02–05</t>
         </is>
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>Evidence export</t>
+          <t>Verifier detects tamper</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
@@ -8143,7 +8171,7 @@
       </c>
       <c r="J88" s="3" t="inlineStr">
         <is>
-          <t>BPMS-046</t>
+          <t>BPMS-026</t>
         </is>
       </c>
       <c r="K88" s="3" t="inlineStr">
@@ -8159,7 +8187,7 @@
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>BPMS-164</t>
+          <t>BPMS-163</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
@@ -8169,7 +8197,7 @@
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>Retention disposition + certificates, DSAR template, legal hold engine</t>
+          <t>Attestation campaigns, control mapping, access reviews</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
@@ -8184,17 +8212,17 @@
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Fullstack</t>
         </is>
       </c>
       <c r="G89" s="3" t="inlineStr">
         <is>
-          <t>PRV-01/03/04</t>
+          <t>FR-G06, FR-W11</t>
         </is>
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
-          <t>Holds block deletion</t>
+          <t>Evidence export</t>
         </is>
       </c>
       <c r="I89" s="3" t="inlineStr">
@@ -8204,7 +8232,7 @@
       </c>
       <c r="J89" s="3" t="inlineStr">
         <is>
-          <t>BPMS-066</t>
+          <t>BPMS-046</t>
         </is>
       </c>
       <c r="K89" s="3" t="inlineStr">
@@ -8220,17 +8248,17 @@
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>BPMS-165</t>
+          <t>BPMS-164</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>SIGN</t>
+          <t>GOV</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode, PAdES-LTV, TSA; in-person/kiosk signing</t>
+          <t>Retention disposition + certificates, DSAR template, legal hold engine</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
@@ -8245,27 +8273,27 @@
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>Fullstack</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="G90" s="3" t="inlineStr">
         <is>
-          <t>ESIG-01–05, FR-DS05, FX-S11</t>
+          <t>PRV-01/03/04</t>
         </is>
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>Verification passes</t>
+          <t>Holds block deletion</t>
         </is>
       </c>
       <c r="I90" s="3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J90" s="3" t="inlineStr">
         <is>
-          <t>BPMS-107</t>
+          <t>BPMS-066</t>
         </is>
       </c>
       <c r="K90" s="3" t="inlineStr">
@@ -8281,17 +8309,17 @@
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>BPMS-166</t>
+          <t>BPMS-165</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>SIGN</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>Alert centre, custom dashboards, report builder, scheduled reports, KPI goals, usage analytics, CSAT</t>
+          <t>Part 11 mode, PAdES-LTV, TSA; in-person/kiosk signing</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
@@ -8311,22 +8339,22 @@
       </c>
       <c r="G91" s="3" t="inlineStr">
         <is>
-          <t>FR-A07–A09, FX-A01–A04, FX-R04</t>
+          <t>ESIG-01–05, FR-DS05, FX-S11</t>
         </is>
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
-          <t>RLS at run time</t>
+          <t>Verification passes</t>
         </is>
       </c>
       <c r="I91" s="3" t="inlineStr">
         <is>
-          <t>XL</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J91" s="3" t="inlineStr">
         <is>
-          <t>BPMS-063</t>
+          <t>BPMS-107</t>
         </is>
       </c>
       <c r="K91" s="3" t="inlineStr">
@@ -8342,17 +8370,17 @@
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>BPMS-167</t>
+          <t>BPMS-166</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>IAM</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>Separation mode; break-glass</t>
+          <t>Alert centre, custom dashboards, report builder, scheduled reports, KPI goals, usage analytics, CSAT</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
@@ -8367,27 +8395,27 @@
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Fullstack</t>
         </is>
       </c>
       <c r="G92" s="3" t="inlineStr">
         <is>
-          <t>12 §6.1, FR-S07</t>
+          <t>FR-A07–A09, FX-A01–A04, FX-R04</t>
         </is>
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>Visible to workspace</t>
+          <t>RLS at run time</t>
         </is>
       </c>
       <c r="I92" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>XL</t>
         </is>
       </c>
       <c r="J92" s="3" t="inlineStr">
         <is>
-          <t>BPMS-024</t>
+          <t>BPMS-063</t>
         </is>
       </c>
       <c r="K92" s="3" t="inlineStr">
@@ -8403,17 +8431,17 @@
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>BPMS-168</t>
+          <t>BPMS-167</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>LIB</t>
+          <t>IAM</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>Role-based onboarding/training paths</t>
+          <t>Separation mode; break-glass</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
@@ -8428,17 +8456,17 @@
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>Fullstack</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="G93" s="3" t="inlineStr">
         <is>
-          <t>FX-G07</t>
+          <t>12 §6.1, FR-S07</t>
         </is>
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
-          <t>Completion reports</t>
+          <t>Visible to workspace</t>
         </is>
       </c>
       <c r="I93" s="3" t="inlineStr">
@@ -8448,7 +8476,7 @@
       </c>
       <c r="J93" s="3" t="inlineStr">
         <is>
-          <t>BPMS-046</t>
+          <t>BPMS-024</t>
         </is>
       </c>
       <c r="K93" s="3" t="inlineStr">
@@ -8464,17 +8492,17 @@
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>BPMS-169</t>
+          <t>BPMS-168</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>E2E</t>
+          <t>LIB</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5 pack incl. investigations, Part 11, break-glass</t>
+          <t>Role-based onboarding/training paths</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
@@ -8489,27 +8517,27 @@
       </c>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>SDET + feature owners</t>
+          <t>Fullstack</t>
         </is>
       </c>
       <c r="G94" s="3" t="inlineStr">
         <is>
-          <t>23 §5</t>
+          <t>FX-G07</t>
         </is>
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>Completion reports</t>
         </is>
       </c>
       <c r="I94" s="3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J94" s="3" t="inlineStr">
         <is>
-          <t>BPMS-152</t>
+          <t>BPMS-046</t>
         </is>
       </c>
       <c r="K94" s="3" t="inlineStr">
@@ -8525,17 +8553,17 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>BPMS-186</t>
+          <t>BPMS-169</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>E2E</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>AI assistance P1 set (drafting, summaries, translate, Q&amp;A) behind kill switch</t>
+          <t>E2E-R5 pack incl. investigations, Part 11, break-glass</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
@@ -8550,17 +8578,17 @@
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>Fullstack</t>
+          <t>SDET + feature owners</t>
         </is>
       </c>
       <c r="G95" s="3" t="inlineStr">
         <is>
-          <t>16, ADR-0006</t>
+          <t>23 §5</t>
         </is>
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
-          <t>Eval thresholds</t>
+          <t>Green</t>
         </is>
       </c>
       <c r="I95" s="3" t="inlineStr">
@@ -8568,7 +8596,11 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J95" s="3" t="inlineStr"/>
+      <c r="J95" s="3" t="inlineStr">
+        <is>
+          <t>BPMS-152</t>
+        </is>
+      </c>
       <c r="K95" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -8582,17 +8614,17 @@
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>BPMS-180</t>
+          <t>BPMS-186</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>OPS</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>Load test at reference load; HA failover; RPO/RTO restore drill</t>
+          <t>AI assistance P1 set (drafting, summaries, translate, Q&amp;A) behind kill switch</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
@@ -8602,22 +8634,22 @@
       </c>
       <c r="E96" s="3" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>SRE</t>
+          <t>Fullstack</t>
         </is>
       </c>
       <c r="G96" s="3" t="inlineStr">
         <is>
-          <t>06, T09</t>
+          <t>16, ADR-0006</t>
         </is>
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
-          <t>Targets met</t>
+          <t>Eval thresholds</t>
         </is>
       </c>
       <c r="I96" s="3" t="inlineStr">
@@ -8639,17 +8671,17 @@
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>BPMS-181</t>
+          <t>BPMS-180</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>SEC</t>
+          <t>OPS</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>External pentest + ASVS L2 self-assessment + fixes</t>
+          <t>Load test at reference load; HA failover; RPO/RTO restore drill</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
@@ -8664,22 +8696,22 @@
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>SRE</t>
         </is>
       </c>
       <c r="G97" s="3" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>06, T09</t>
         </is>
       </c>
       <c r="H97" s="3" t="inlineStr">
         <is>
-          <t>0 crit/high</t>
+          <t>Targets met</t>
         </is>
       </c>
       <c r="I97" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J97" s="3" t="inlineStr"/>
@@ -8696,17 +8728,17 @@
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>BPMS-182</t>
+          <t>BPMS-181</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>SEC</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>WCAG 2.2 AA audit + VPAT 2.5 INT</t>
+          <t>External pentest + ASVS L2 self-assessment + fixes</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
@@ -8721,17 +8753,17 @@
       </c>
       <c r="F98" s="3" t="inlineStr">
         <is>
-          <t>Design/QA</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="G98" s="3" t="inlineStr">
         <is>
-          <t>A11Y-01/03</t>
+          <t>06</t>
         </is>
       </c>
       <c r="H98" s="3" t="inlineStr">
         <is>
-          <t>Audit pass</t>
+          <t>0 crit/high</t>
         </is>
       </c>
       <c r="I98" s="3" t="inlineStr">
@@ -8753,17 +8785,17 @@
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>BPMS-183</t>
+          <t>BPMS-182</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>I18N</t>
+          <t>UX</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>3 UI languages + RTL + pseudo-locale</t>
+          <t>WCAG 2.2 AA audit + VPAT 2.5 INT</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
@@ -8778,17 +8810,17 @@
       </c>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>FE</t>
+          <t>Design/QA</t>
         </is>
       </c>
       <c r="G99" s="3" t="inlineStr">
         <is>
-          <t>FR-P04, OQ-09</t>
+          <t>A11Y-01/03</t>
         </is>
       </c>
       <c r="H99" s="3" t="inlineStr">
         <is>
-          <t>Checks pass</t>
+          <t>Audit pass</t>
         </is>
       </c>
       <c r="I99" s="3" t="inlineStr">
@@ -8810,17 +8842,17 @@
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>BPMS-184</t>
+          <t>BPMS-183</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>OPS</t>
+          <t>I18N</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>Helm chart, air-gapped bundle, upgrade N-1→N tests, dedicated-DB tier</t>
+          <t>3 UI languages + RTL + pseudo-locale</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
@@ -8835,22 +8867,22 @@
       </c>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>DevOps</t>
+          <t>FE</t>
         </is>
       </c>
       <c r="G100" s="3" t="inlineStr">
         <is>
-          <t>FR-P06, FR-S10</t>
+          <t>FR-P04, OQ-09</t>
         </is>
       </c>
       <c r="H100" s="3" t="inlineStr">
         <is>
-          <t>Upgrade with live instances</t>
+          <t>Checks pass</t>
         </is>
       </c>
       <c r="I100" s="3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J100" s="3" t="inlineStr"/>
@@ -8867,17 +8899,17 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>BPMS-185</t>
+          <t>BPMS-184</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>DOC</t>
+          <t>OPS</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>Docs site, admin guide, API reference, trust pack</t>
+          <t>Helm chart, air-gapped bundle, upgrade N-1→N tests, dedicated-DB tier</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
@@ -8892,22 +8924,22 @@
       </c>
       <c r="F101" s="3" t="inlineStr">
         <is>
-          <t>Writer</t>
+          <t>DevOps</t>
         </is>
       </c>
       <c r="G101" s="3" t="inlineStr">
         <is>
-          <t>FX-P06</t>
+          <t>FR-P06, FR-S10</t>
         </is>
       </c>
       <c r="H101" s="3" t="inlineStr">
         <is>
-          <t>Published</t>
+          <t>Upgrade with live instances</t>
         </is>
       </c>
       <c r="I101" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J101" s="3" t="inlineStr"/>
@@ -8924,17 +8956,17 @@
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>BPMS-187</t>
+          <t>BPMS-185</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>E2E</t>
+          <t>DOC</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>E2E-GA regression: 3 browsers × 2 viewports, cache-off, upgrade-path R1→1.0, air-gapped</t>
+          <t>Docs site, admin guide, API reference, trust pack</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
@@ -8949,17 +8981,17 @@
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>SDET</t>
+          <t>Writer</t>
         </is>
       </c>
       <c r="G102" s="3" t="inlineStr">
         <is>
-          <t>23 §5</t>
+          <t>FX-P06</t>
         </is>
       </c>
       <c r="H102" s="3" t="inlineStr">
         <is>
-          <t>Green; flake &lt; 0.5 %</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="I102" s="3" t="inlineStr">
@@ -8967,11 +8999,7 @@
           <t>M</t>
         </is>
       </c>
-      <c r="J102" s="3" t="inlineStr">
-        <is>
-          <t>BPMS-169</t>
-        </is>
-      </c>
+      <c r="J102" s="3" t="inlineStr"/>
       <c r="K102" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -8985,17 +9013,17 @@
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>BPMS-190</t>
+          <t>BPMS-187</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>REL</t>
+          <t>E2E</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>GA release: signed artefacts, SBOM, provenance, runbooks</t>
+          <t>E2E-GA regression: 3 browsers × 2 viewports, cache-off, upgrade-path R1→1.0, air-gapped</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
@@ -9010,27 +9038,27 @@
       </c>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>Tech lead</t>
+          <t>SDET</t>
         </is>
       </c>
       <c r="G103" s="3" t="inlineStr">
         <is>
-          <t>G5</t>
+          <t>23 §5</t>
         </is>
       </c>
       <c r="H103" s="3" t="inlineStr">
         <is>
-          <t>Released</t>
+          <t>Green; flake &lt; 0.5 %</t>
         </is>
       </c>
       <c r="I103" s="3" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J103" s="3" t="inlineStr">
         <is>
-          <t>M10</t>
+          <t>BPMS-169</t>
         </is>
       </c>
       <c r="K103" s="3" t="inlineStr">
@@ -9046,50 +9074,54 @@
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>BPMS-200</t>
+          <t>BPMS-190</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>REL</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>Chat/host-platform connectors (identity, embed, cards, notifications, directory)</t>
+          <t>GA release: signed artefacts, SBOM, provenance, runbooks</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="E104" s="3" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="F104" s="3" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Tech lead</t>
         </is>
       </c>
       <c r="G104" s="3" t="inlineStr">
         <is>
-          <t>13 §4</t>
+          <t>G5</t>
         </is>
       </c>
       <c r="H104" s="3" t="inlineStr">
         <is>
-          <t>Demand gate</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="I104" s="3" t="inlineStr">
         <is>
-          <t>XL</t>
-        </is>
-      </c>
-      <c r="J104" s="3" t="inlineStr"/>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J104" s="3" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
       <c r="K104" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -9103,7 +9135,7 @@
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>BPMS-201</t>
+          <t>BPMS-200</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
@@ -9113,7 +9145,7 @@
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>Chat cards (Slack/Teams), M365/Google, HRIS, ERP connectors</t>
+          <t>Chat/host-platform connectors (identity, embed, cards, notifications, directory)</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
@@ -9133,12 +9165,12 @@
       </c>
       <c r="G105" s="3" t="inlineStr">
         <is>
-          <t>INT-*</t>
+          <t>13 §4</t>
         </is>
       </c>
       <c r="H105" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Demand gate</t>
         </is>
       </c>
       <c r="I105" s="3" t="inlineStr">
@@ -9160,17 +9192,17 @@
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>BPMS-202</t>
+          <t>BPMS-201</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>SIGN</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>QES via QTSP; Aadhaar eSign via ESP; SMS/IDV providers</t>
+          <t>Chat cards (Slack/Teams), M365/Google, HRIS, ERP connectors</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
@@ -9190,7 +9222,7 @@
       </c>
       <c r="G106" s="3" t="inlineStr">
         <is>
-          <t>FX-S13, FX-S07</t>
+          <t>INT-*</t>
         </is>
       </c>
       <c r="H106" s="3" t="inlineStr">
@@ -9200,7 +9232,7 @@
       </c>
       <c r="I106" s="3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>XL</t>
         </is>
       </c>
       <c r="J106" s="3" t="inlineStr"/>
@@ -9217,17 +9249,17 @@
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>BPMS-203</t>
+          <t>BPMS-202</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>EXEC</t>
+          <t>SIGN</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>BPMN view (diagram-js), DMN import/export, migration tool, simulation</t>
+          <t>QES via QTSP; Aadhaar eSign via ESP; SMS/IDV providers</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
@@ -9242,12 +9274,12 @@
       </c>
       <c r="F107" s="3" t="inlineStr">
         <is>
-          <t>Runtime/FE</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="G107" s="3" t="inlineStr">
         <is>
-          <t>ADR-0018, FR-E07/E10, FR-I04</t>
+          <t>FX-S13, FX-S07</t>
         </is>
       </c>
       <c r="H107" s="3" t="inlineStr">
@@ -9257,7 +9289,7 @@
       </c>
       <c r="I107" s="3" t="inlineStr">
         <is>
-          <t>XL</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J107" s="3" t="inlineStr"/>
@@ -9274,17 +9306,17 @@
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>BPMS-204</t>
+          <t>BPMS-203</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>INS</t>
+          <t>EXEC</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>Event-log export OCEL 2.0 / XES</t>
+          <t>BPMN view (diagram-js), DMN import/export, migration tool, simulation</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr">
@@ -9299,22 +9331,22 @@
       </c>
       <c r="F108" s="3" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Runtime/FE</t>
         </is>
       </c>
       <c r="G108" s="3" t="inlineStr">
         <is>
-          <t>FR-I03</t>
+          <t>ADR-0018, FR-E07/E10, FR-I04</t>
         </is>
       </c>
       <c r="H108" s="3" t="inlineStr">
         <is>
-          <t>Schema-valid</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I108" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>XL</t>
         </is>
       </c>
       <c r="J108" s="3" t="inlineStr"/>
@@ -9331,17 +9363,17 @@
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>BPMS-205</t>
+          <t>BPMS-204</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>INS</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>Governed AI agent steps</t>
+          <t>Event-log export OCEL 2.0 / XES</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr">
@@ -9356,22 +9388,22 @@
       </c>
       <c r="F109" s="3" t="inlineStr">
         <is>
-          <t>Fullstack</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="G109" s="3" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>FR-I03</t>
         </is>
       </c>
       <c r="H109" s="3" t="inlineStr">
         <is>
-          <t>Human gate</t>
+          <t>Schema-valid</t>
         </is>
       </c>
       <c r="I109" s="3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J109" s="3" t="inlineStr"/>
@@ -9385,8 +9417,65 @@
       <c r="N109" s="3" t="inlineStr"/>
       <c r="O109" s="3" t="inlineStr"/>
     </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>BPMS-205</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>Governed AI agent steps</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="F110" s="3" t="inlineStr">
+        <is>
+          <t>Fullstack</t>
+        </is>
+      </c>
+      <c r="G110" s="3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="H110" s="3" t="inlineStr">
+        <is>
+          <t>Human gate</t>
+        </is>
+      </c>
+      <c r="I110" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J110" s="3" t="inlineStr"/>
+      <c r="K110" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L110" s="3" t="inlineStr"/>
+      <c r="M110" s="3" t="inlineStr"/>
+      <c r="N110" s="3" t="inlineStr"/>
+      <c r="O110" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="K2:K109">
+  <conditionalFormatting sqref="K2:K110">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Blocked"</formula>
     </cfRule>
@@ -9398,7 +9487,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="K2:K109" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K110" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,In progress,Blocked,In review,Done,Deferred"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
build: Rust workspace, kernel crate, procera binary and CI gates (BPMS-011)
- Cargo workspace (edition 2024, toolchain 1.98.0) with workspace lints that
  forbid unsafe, unwrap/expect, dbg/todo and stdout printing (docs/24 §3.10)
- procera-kernel: Clock (+ ManualClock behind test-clock), UUIDv7 IdGen,
  RFC 9457 Problem
- procera binary: 'serve [--all]' with /healthz, /readyz, /version
- deny.toml licence gate: permissive-only allow list (ADR-0014)
- CI: fmt, clippy -D warnings, tests, release build, cargo-deny, CycloneDX SBOM
- tracker: STATUS map in build_tracker.py with progress summary; BPMS-011 in
  review, BPMS-014 done, BPMS-034 in progress (docs/24 §2.2)

JS licence check and axe a11y gate join CI with the web workspace (BPMS-010).

Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -3560,13 +3560,17 @@
       <c r="J12" s="3" t="inlineStr"/>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In review</t>
         </is>
       </c>
       <c r="L12" s="3" t="inlineStr"/>
       <c r="M12" s="3" t="inlineStr"/>
       <c r="N12" s="3" t="inlineStr"/>
-      <c r="O12" s="3" t="inlineStr"/>
+      <c r="O12" s="3" t="inlineStr">
+        <is>
+          <t>Rust workspace, kernel, procera binary, CI (fmt/clippy/test/deny/SBOM): PR feat/BPMS-011-monorepo-ci</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -3735,13 +3739,17 @@
       <c r="J15" s="3" t="inlineStr"/>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr"/>
       <c r="M15" s="3" t="inlineStr"/>
       <c r="N15" s="3" t="inlineStr"/>
-      <c r="O15" s="3" t="inlineStr"/>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>CLAUDE.md, AGENTS.md, PR template, CODEOWNERS, docs/24 rules on main</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -4646,13 +4654,17 @@
       <c r="J30" s="3" t="inlineStr"/>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L30" s="3" t="inlineStr"/>
       <c r="M30" s="3" t="inlineStr"/>
       <c r="N30" s="3" t="inlineStr"/>
-      <c r="O30" s="3" t="inlineStr"/>
+      <c r="O30" s="3" t="inlineStr">
+        <is>
+          <t>Raster assets + brand guide merged; SVG masters and trademark search pending</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">

</xml_diff>

<commit_message>
test(e2e): E2E harness with test-only controls and P0 smoke pack (BPMS-013)
- procera 'e2e' cargo feature: ManualClock-backed AppState and /__test/clock,
  /__test/drain, /__test/fault (501 until BPMS-089), /__test/audit/verify
  (501 until BPMS-026); unit test asserts routes are absent without the feature
- e2e/: Playwright config (api + browser projects), TestControls fixture,
  P0 smoke pack E2E-P0-01..04, no-fixed-sleeps lint (docs/23 §7)
- Dockerfile (distroless, nonroot) and deploy/compose.e2e.yml with
  Postgres 16, Valkey, SeaweedFS, Mailpit, ClamAV
- CI job e2e-smoke: validates compose, runs the smoke pack against an e2e
  build, and asserts the release binary returns 404 for /__test/clock
- docs/23: E2E-P0 scenarios; tracker: BPMS-013 in review

Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E226" headerRowCount="1">
-  <autoFilter ref="A1:E226"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E231" headerRowCount="1">
+  <autoFilter ref="A1:E231"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -3682,13 +3682,17 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In review</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr"/>
       <c r="M14" s="3" t="inlineStr"/>
       <c r="N14" s="3" t="inlineStr"/>
-      <c r="O14" s="3" t="inlineStr"/>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>procera e2e feature + /__test controls, Playwright harness, P0 smoke pack, compose.e2e stack, CI e2e-smoke job: PR feat/BPMS-013-e2e-harness (stacked on BPMS-011)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -9516,7 +9520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E226"/>
+  <dimension ref="A1:E231"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -13638,12 +13642,12 @@
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-P0-01</t>
         </is>
       </c>
       <c r="C153" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>`/healthz` and `/readyz` return 200 | Harness boots the stack</t>
         </is>
       </c>
       <c r="D153" s="3" t="inlineStr">
@@ -13665,12 +13669,12 @@
       </c>
       <c r="B154" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-P0-02</t>
         </is>
       </c>
       <c r="C154" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>`/version` reports name and server time | Clock wiring</t>
         </is>
       </c>
       <c r="D154" s="3" t="inlineStr">
@@ -13692,12 +13696,12 @@
       </c>
       <c r="B155" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-P0-03</t>
         </is>
       </c>
       <c r="C155" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>`__test/clock` advances only forward and drives server time; invalid durations get a 422 problem+json | docs/23 §4 controls</t>
         </is>
       </c>
       <c r="D155" s="3" t="inlineStr">
@@ -13719,12 +13723,12 @@
       </c>
       <c r="B156" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-P0-04</t>
         </is>
       </c>
       <c r="C156" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>`__test/drain` reports idle; unknown routes return 404 | Drain control; routing baseline</t>
         </is>
       </c>
       <c r="D156" s="3" t="inlineStr">
@@ -13746,12 +13750,12 @@
       </c>
       <c r="B157" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-P0-REL</t>
         </is>
       </c>
       <c r="C157" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>The release binary returns 404 for `/__test/clock` (CI step) | docs/24 §5.4</t>
         </is>
       </c>
       <c r="D157" s="3" t="inlineStr">
@@ -13773,12 +13777,12 @@
       </c>
       <c r="B158" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C158" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
         </is>
       </c>
       <c r="D158" s="3" t="inlineStr">
@@ -13800,12 +13804,12 @@
       </c>
       <c r="B159" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C159" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D159" s="3" t="inlineStr">
@@ -13827,12 +13831,12 @@
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C160" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D160" s="3" t="inlineStr">
@@ -13854,12 +13858,12 @@
       </c>
       <c r="B161" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C161" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
         </is>
       </c>
       <c r="D161" s="3" t="inlineStr">
@@ -13881,12 +13885,12 @@
       </c>
       <c r="B162" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C162" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
         </is>
       </c>
       <c r="D162" s="3" t="inlineStr">
@@ -13908,12 +13912,12 @@
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C163" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D163" s="3" t="inlineStr">
@@ -13935,12 +13939,12 @@
       </c>
       <c r="B164" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C164" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D164" s="3" t="inlineStr">
@@ -13962,12 +13966,12 @@
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C165" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
         </is>
       </c>
       <c r="D165" s="3" t="inlineStr">
@@ -13989,12 +13993,12 @@
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D166" s="3" t="inlineStr">
@@ -14016,12 +14020,12 @@
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C167" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D167" s="3" t="inlineStr">
@@ -14043,12 +14047,12 @@
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D168" s="3" t="inlineStr">
@@ -14070,12 +14074,12 @@
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C169" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D169" s="3" t="inlineStr">
@@ -14097,12 +14101,12 @@
       </c>
       <c r="B170" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C170" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
         </is>
       </c>
       <c r="D170" s="3" t="inlineStr">
@@ -14124,12 +14128,12 @@
       </c>
       <c r="B171" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C171" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
         </is>
       </c>
       <c r="D171" s="3" t="inlineStr">
@@ -14151,12 +14155,12 @@
       </c>
       <c r="B172" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C172" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
         </is>
       </c>
       <c r="D172" s="3" t="inlineStr">
@@ -14178,12 +14182,12 @@
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C173" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D173" s="3" t="inlineStr">
@@ -14205,12 +14209,12 @@
       </c>
       <c r="B174" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C174" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
         </is>
       </c>
       <c r="D174" s="3" t="inlineStr">
@@ -14232,12 +14236,12 @@
       </c>
       <c r="B175" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C175" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
         </is>
       </c>
       <c r="D175" s="3" t="inlineStr">
@@ -14259,12 +14263,12 @@
       </c>
       <c r="B176" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C176" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D176" s="3" t="inlineStr">
@@ -14286,12 +14290,12 @@
       </c>
       <c r="B177" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C177" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
         </is>
       </c>
       <c r="D177" s="3" t="inlineStr">
@@ -14313,12 +14317,12 @@
       </c>
       <c r="B178" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C178" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D178" s="3" t="inlineStr">
@@ -14340,12 +14344,12 @@
       </c>
       <c r="B179" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C179" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D179" s="3" t="inlineStr">
@@ -14367,12 +14371,12 @@
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C180" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D180" s="3" t="inlineStr">
@@ -14394,12 +14398,12 @@
       </c>
       <c r="B181" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C181" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D181" s="3" t="inlineStr">
@@ -14421,12 +14425,12 @@
       </c>
       <c r="B182" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C182" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D182" s="3" t="inlineStr">
@@ -14448,12 +14452,12 @@
       </c>
       <c r="B183" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C183" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D183" s="3" t="inlineStr">
@@ -14475,12 +14479,12 @@
       </c>
       <c r="B184" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C184" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D184" s="3" t="inlineStr">
@@ -14502,12 +14506,12 @@
       </c>
       <c r="B185" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D185" s="3" t="inlineStr">
@@ -14529,12 +14533,12 @@
       </c>
       <c r="B186" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C186" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D186" s="3" t="inlineStr">
@@ -14556,12 +14560,12 @@
       </c>
       <c r="B187" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D187" s="3" t="inlineStr">
@@ -14583,12 +14587,12 @@
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D188" s="3" t="inlineStr">
@@ -14610,12 +14614,12 @@
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D189" s="3" t="inlineStr">
@@ -14637,12 +14641,12 @@
       </c>
       <c r="B190" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C190" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D190" s="3" t="inlineStr">
@@ -14664,12 +14668,12 @@
       </c>
       <c r="B191" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D191" s="3" t="inlineStr">
@@ -14691,12 +14695,12 @@
       </c>
       <c r="B192" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C192" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D192" s="3" t="inlineStr">
@@ -14718,12 +14722,12 @@
       </c>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D193" s="3" t="inlineStr">
@@ -14745,12 +14749,12 @@
       </c>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C194" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D194" s="3" t="inlineStr">
@@ -14772,12 +14776,12 @@
       </c>
       <c r="B195" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D195" s="3" t="inlineStr">
@@ -14799,12 +14803,12 @@
       </c>
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C196" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D196" s="3" t="inlineStr">
@@ -14826,12 +14830,12 @@
       </c>
       <c r="B197" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D197" s="3" t="inlineStr">
@@ -14853,12 +14857,12 @@
       </c>
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C198" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D198" s="3" t="inlineStr">
@@ -14880,12 +14884,12 @@
       </c>
       <c r="B199" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D199" s="3" t="inlineStr">
@@ -14907,12 +14911,12 @@
       </c>
       <c r="B200" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C200" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D200" s="3" t="inlineStr">
@@ -14934,12 +14938,12 @@
       </c>
       <c r="B201" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D201" s="3" t="inlineStr">
@@ -14961,12 +14965,12 @@
       </c>
       <c r="B202" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C202" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D202" s="3" t="inlineStr">
@@ -14988,12 +14992,12 @@
       </c>
       <c r="B203" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D203" s="3" t="inlineStr">
@@ -15015,12 +15019,12 @@
       </c>
       <c r="B204" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C204" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D204" s="3" t="inlineStr">
@@ -15042,12 +15046,12 @@
       </c>
       <c r="B205" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C205" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D205" s="3" t="inlineStr">
@@ -15069,12 +15073,12 @@
       </c>
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D206" s="3" t="inlineStr">
@@ -15096,12 +15100,12 @@
       </c>
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D207" s="3" t="inlineStr">
@@ -15123,12 +15127,12 @@
       </c>
       <c r="B208" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D208" s="3" t="inlineStr">
@@ -15150,12 +15154,12 @@
       </c>
       <c r="B209" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D209" s="3" t="inlineStr">
@@ -15177,12 +15181,12 @@
       </c>
       <c r="B210" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D210" s="3" t="inlineStr">
@@ -15204,12 +15208,12 @@
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D211" s="3" t="inlineStr">
@@ -15231,12 +15235,12 @@
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D212" s="3" t="inlineStr">
@@ -15258,12 +15262,12 @@
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D213" s="3" t="inlineStr">
@@ -15285,12 +15289,12 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D214" s="3" t="inlineStr">
@@ -15312,12 +15316,12 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D215" s="3" t="inlineStr">
@@ -15339,12 +15343,12 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
@@ -15366,12 +15370,12 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -15393,12 +15397,12 @@
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
@@ -15420,12 +15424,12 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R4-11</t>
         </is>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
         </is>
       </c>
       <c r="D219" s="3" t="inlineStr">
@@ -15447,12 +15451,12 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R4-ISO</t>
         </is>
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
         </is>
       </c>
       <c r="D220" s="3" t="inlineStr">
@@ -15474,12 +15478,12 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R5-01</t>
         </is>
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
         </is>
       </c>
       <c r="D221" s="3" t="inlineStr">
@@ -15501,12 +15505,12 @@
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R5-02</t>
         </is>
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
         </is>
       </c>
       <c r="D222" s="3" t="inlineStr">
@@ -15528,12 +15532,12 @@
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R5-03</t>
         </is>
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
         </is>
       </c>
       <c r="D223" s="3" t="inlineStr">
@@ -15555,12 +15559,12 @@
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R5-04</t>
         </is>
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
         </is>
       </c>
       <c r="D224" s="3" t="inlineStr">
@@ -15582,12 +15586,12 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R5-05</t>
         </is>
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
         </is>
       </c>
       <c r="D225" s="3" t="inlineStr">
@@ -15609,20 +15613,155 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
+          <t>E2E-R5-06</t>
+        </is>
+      </c>
+      <c r="C226" s="3" t="inlineStr">
+        <is>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+        </is>
+      </c>
+      <c r="D226" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E226" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B227" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-07</t>
+        </is>
+      </c>
+      <c r="C227" s="3" t="inlineStr">
+        <is>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+        </is>
+      </c>
+      <c r="D227" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E227" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B228" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-08</t>
+        </is>
+      </c>
+      <c r="C228" s="3" t="inlineStr">
+        <is>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+        </is>
+      </c>
+      <c r="D228" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E228" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B229" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-09</t>
+        </is>
+      </c>
+      <c r="C229" s="3" t="inlineStr">
+        <is>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+        </is>
+      </c>
+      <c r="D229" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E229" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B230" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C230" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D230" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E230" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B231" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C226" s="3" t="inlineStr">
+      <c r="C231" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D226" s="3" t="inlineStr">
+      <c r="D231" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E226" s="3" t="inlineStr">
+      <c r="E231" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
docs(tracker): editor-friendly tracker dashboard + trunk-based workflow (BPMS-011, BPMS-013 done)
- trackers/README.md: generated dashboard with overall progress, current
  release, active items, done list and collapsible per-release checklists;
  CI freshness check now covers it
- docs/24 §7, CLAUDE.md, AGENTS.md, CONTRIBUTING.md: owner decision to commit
  directly to main (no PRs) with local gates before push, red-main-first rule,
  [protected] commits reviewed after they land; external contributors use PRs
- tracker: BPMS-011 and BPMS-013 marked Done (CI green on main)

Evidence: cargo fmt/clippy -D warnings/test ok; cargo deny ok; links ok.
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -3560,7 +3560,7 @@
       <c r="J12" s="3" t="inlineStr"/>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>In review</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L12" s="3" t="inlineStr"/>
@@ -3568,7 +3568,7 @@
       <c r="N12" s="3" t="inlineStr"/>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>Rust workspace, kernel, procera binary, CI (fmt/clippy/test/deny/SBOM): PR feat/BPMS-011-monorepo-ci</t>
+          <t>Rust workspace, kernel, procera binary, CI (fmt/clippy/test/deny/SBOM/E2E smoke); on main, CI green. JS licence + axe gates join with BPMS-010</t>
         </is>
       </c>
     </row>
@@ -3682,7 +3682,7 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>In review</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr"/>
@@ -3690,7 +3690,7 @@
       <c r="N14" s="3" t="inlineStr"/>
       <c r="O14" s="3" t="inlineStr">
         <is>
-          <t>procera e2e feature + /__test controls, Playwright harness, P0 smoke pack, compose.e2e stack, CI e2e-smoke job: PR feat/BPMS-013-e2e-harness (stacked on BPMS-011)</t>
+          <t>e2e feature + /__test controls, Playwright harness, P0 smoke pack (E2E-P0-01..04, REL), compose.e2e stack, CI e2e-smoke job; on main, CI green. Seed A/B + personas land with the first workspace APIs (BPMS-032); full compose boot pending a Docker run</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: complete local test suite, batch cadence, tracker update
- scripts/test-all.sh: complete suite (Rust fmt/clippy/tests with and without
  e2e feature, licence gates, spikes, tracker, links, compose, web, E2E API +
  a11y packs, release has no /__test routes)
- docs/24 §7.3, CLAUDE.md: batch 3-4 tasks, run test-all after 5-10, then push
- tracker: BPMS-002/004/005/006/007 done, BPMS-010 in progress
- .gitignore: ignore target/ in nested workspaces

Evidence: ./scripts/test-all.sh -> all checks passed.
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E231" headerRowCount="1">
-  <autoFilter ref="A1:E231"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E236" headerRowCount="1">
+  <autoFilter ref="A1:E236"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -3043,13 +3043,17 @@
       <c r="J3" s="3" t="inlineStr"/>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="3" t="inlineStr"/>
-      <c r="O3" s="3" t="inlineStr"/>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>5 reference processes as IR v1 fixtures (all 16 node kinds) + JSON Schema + structural checker IR-E001..E016 with negative tests; 12 IR spec clarifications (docs/spikes/BPMS-002)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -3157,13 +3161,17 @@
       <c r="J5" s="3" t="inlineStr"/>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="3" t="inlineStr"/>
-      <c r="O5" s="3" t="inlineStr"/>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>SP-07: Rust + JS dependency licences reviewed; approved set; JS licence gate (scripts/js-licence-gate.mjs) + CDLA-Permissive-2.0 for CA roots; fonts OFL — docs/spikes/SP-07</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -3214,13 +3222,17 @@
       <c r="J6" s="3" t="inlineStr"/>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr"/>
       <c r="M6" s="3" t="inlineStr"/>
       <c r="N6" s="3" t="inlineStr"/>
-      <c r="O6" s="3" t="inlineStr"/>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>SP-08: recommend CEL + decimal/stdlib/type-checker/budgets; FEEL rejected at runtime (quadratic loops, no WASM) — docs/spikes/SP-08; ADR-0010 recommended</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -3271,13 +3283,17 @@
       <c r="J7" s="3" t="inlineStr"/>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr"/>
       <c r="M7" s="3" t="inlineStr"/>
       <c r="N7" s="3" t="inlineStr"/>
-      <c r="O7" s="3" t="inlineStr"/>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>SP-09: Cedar 6/6 correct, 5.6µs P50; RLS via pool 0 leaks/5000; LLD fix NULLIF in RLS policy; partial-eval→SQL viable with fallback — docs/spikes/SP-09</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -3328,13 +3344,17 @@
       <c r="J8" s="3" t="inlineStr"/>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr"/>
       <c r="M8" s="3" t="inlineStr"/>
       <c r="N8" s="3" t="inlineStr"/>
-      <c r="O8" s="3" t="inlineStr"/>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>SP-10: head-lock 9.7k ev/s (P99 11ms), batched sealer 65k ev/s, explorer P95 &lt;0.6ms at 10M, verifier 536k ev/s + tamper detected — docs/spikes/SP-10</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -3503,13 +3523,17 @@
       <c r="J11" s="3" t="inlineStr"/>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr"/>
       <c r="M11" s="3" t="inlineStr"/>
       <c r="N11" s="3" t="inlineStr"/>
-      <c r="O11" s="3" t="inlineStr"/>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>Slice 1 done: web workspace (Vite/React/TS), tokens.json→CSS with 40 WCAG contrast checks, Button/TextField/Checkbox/Notice on React Aria, app shell, gallery, axe+keyboard+reflow+target E2E (E2E-P0-05..09). Next: Select, Dialog, DataGrid shell, Tabs</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -3568,7 +3592,7 @@
       <c r="N12" s="3" t="inlineStr"/>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>Rust workspace, kernel, procera binary, CI (fmt/clippy/test/deny/SBOM/E2E smoke); on main, CI green. JS licence + axe gates join with BPMS-010</t>
+          <t>Rust workspace, kernel, procera binary, CI (fmt/clippy/test/deny/SBOM/E2E smoke) + web check/build, JS licence gate and axe a11y job (added with BPMS-010)</t>
         </is>
       </c>
     </row>
@@ -9520,7 +9544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E231"/>
+  <dimension ref="A1:E236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -13777,12 +13801,12 @@
       </c>
       <c r="B158" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-P0-05</t>
         </is>
       </c>
       <c r="C158" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>Design-system gallery: zero axe violations for WCAG 2.0/2.1/2.2 A+AA (light theme) | BPMS-010, A11Y-01</t>
         </is>
       </c>
       <c r="D158" s="3" t="inlineStr">
@@ -13804,12 +13828,12 @@
       </c>
       <c r="B159" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-P0-06</t>
         </is>
       </c>
       <c r="C159" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>Same in the dark theme | docs/05 §7.1.1</t>
         </is>
       </c>
       <c r="D159" s="3" t="inlineStr">
@@ -13831,12 +13855,12 @@
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-P0-07</t>
         </is>
       </c>
       <c r="C160" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>Keyboard: skip link is the first tab stop and moves focus to main; every following tab stop shows a visible focus outline | WCAG 2.4.1, 2.4.7, 2.4.11</t>
         </is>
       </c>
       <c r="D160" s="3" t="inlineStr">
@@ -13858,12 +13882,12 @@
       </c>
       <c r="B161" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-P0-08</t>
         </is>
       </c>
       <c r="C161" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>Reflows at 320 px with no horizontal scrolling | WCAG 1.4.10</t>
         </is>
       </c>
       <c r="D161" s="3" t="inlineStr">
@@ -13885,12 +13909,12 @@
       </c>
       <c r="B162" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-P0-09</t>
         </is>
       </c>
       <c r="C162" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>Every visible interactive target is ≥ 24×24 px (visually hidden native inputs are measured through their label) | WCAG 2.5.8</t>
         </is>
       </c>
       <c r="D162" s="3" t="inlineStr">
@@ -13912,12 +13936,12 @@
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C163" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
         </is>
       </c>
       <c r="D163" s="3" t="inlineStr">
@@ -13939,12 +13963,12 @@
       </c>
       <c r="B164" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C164" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D164" s="3" t="inlineStr">
@@ -13966,12 +13990,12 @@
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C165" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D165" s="3" t="inlineStr">
@@ -13993,12 +14017,12 @@
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
         </is>
       </c>
       <c r="D166" s="3" t="inlineStr">
@@ -14020,12 +14044,12 @@
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C167" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
         </is>
       </c>
       <c r="D167" s="3" t="inlineStr">
@@ -14047,12 +14071,12 @@
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D168" s="3" t="inlineStr">
@@ -14074,12 +14098,12 @@
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C169" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D169" s="3" t="inlineStr">
@@ -14101,12 +14125,12 @@
       </c>
       <c r="B170" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C170" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
         </is>
       </c>
       <c r="D170" s="3" t="inlineStr">
@@ -14128,12 +14152,12 @@
       </c>
       <c r="B171" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C171" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D171" s="3" t="inlineStr">
@@ -14155,12 +14179,12 @@
       </c>
       <c r="B172" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C172" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D172" s="3" t="inlineStr">
@@ -14182,12 +14206,12 @@
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C173" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D173" s="3" t="inlineStr">
@@ -14209,12 +14233,12 @@
       </c>
       <c r="B174" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C174" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D174" s="3" t="inlineStr">
@@ -14236,12 +14260,12 @@
       </c>
       <c r="B175" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C175" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
         </is>
       </c>
       <c r="D175" s="3" t="inlineStr">
@@ -14263,12 +14287,12 @@
       </c>
       <c r="B176" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C176" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
         </is>
       </c>
       <c r="D176" s="3" t="inlineStr">
@@ -14290,12 +14314,12 @@
       </c>
       <c r="B177" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C177" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
         </is>
       </c>
       <c r="D177" s="3" t="inlineStr">
@@ -14317,12 +14341,12 @@
       </c>
       <c r="B178" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C178" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D178" s="3" t="inlineStr">
@@ -14344,12 +14368,12 @@
       </c>
       <c r="B179" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C179" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
         </is>
       </c>
       <c r="D179" s="3" t="inlineStr">
@@ -14371,12 +14395,12 @@
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C180" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
         </is>
       </c>
       <c r="D180" s="3" t="inlineStr">
@@ -14398,12 +14422,12 @@
       </c>
       <c r="B181" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C181" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D181" s="3" t="inlineStr">
@@ -14425,12 +14449,12 @@
       </c>
       <c r="B182" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C182" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
         </is>
       </c>
       <c r="D182" s="3" t="inlineStr">
@@ -14452,12 +14476,12 @@
       </c>
       <c r="B183" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C183" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D183" s="3" t="inlineStr">
@@ -14479,12 +14503,12 @@
       </c>
       <c r="B184" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C184" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D184" s="3" t="inlineStr">
@@ -14506,12 +14530,12 @@
       </c>
       <c r="B185" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D185" s="3" t="inlineStr">
@@ -14533,12 +14557,12 @@
       </c>
       <c r="B186" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C186" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D186" s="3" t="inlineStr">
@@ -14560,12 +14584,12 @@
       </c>
       <c r="B187" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D187" s="3" t="inlineStr">
@@ -14587,12 +14611,12 @@
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D188" s="3" t="inlineStr">
@@ -14614,12 +14638,12 @@
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D189" s="3" t="inlineStr">
@@ -14641,12 +14665,12 @@
       </c>
       <c r="B190" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C190" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D190" s="3" t="inlineStr">
@@ -14668,12 +14692,12 @@
       </c>
       <c r="B191" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D191" s="3" t="inlineStr">
@@ -14695,12 +14719,12 @@
       </c>
       <c r="B192" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C192" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D192" s="3" t="inlineStr">
@@ -14722,12 +14746,12 @@
       </c>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D193" s="3" t="inlineStr">
@@ -14749,12 +14773,12 @@
       </c>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C194" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D194" s="3" t="inlineStr">
@@ -14776,12 +14800,12 @@
       </c>
       <c r="B195" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D195" s="3" t="inlineStr">
@@ -14803,12 +14827,12 @@
       </c>
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C196" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D196" s="3" t="inlineStr">
@@ -14830,12 +14854,12 @@
       </c>
       <c r="B197" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D197" s="3" t="inlineStr">
@@ -14857,12 +14881,12 @@
       </c>
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C198" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D198" s="3" t="inlineStr">
@@ -14884,12 +14908,12 @@
       </c>
       <c r="B199" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D199" s="3" t="inlineStr">
@@ -14911,12 +14935,12 @@
       </c>
       <c r="B200" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C200" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D200" s="3" t="inlineStr">
@@ -14938,12 +14962,12 @@
       </c>
       <c r="B201" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D201" s="3" t="inlineStr">
@@ -14965,12 +14989,12 @@
       </c>
       <c r="B202" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C202" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D202" s="3" t="inlineStr">
@@ -14992,12 +15016,12 @@
       </c>
       <c r="B203" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D203" s="3" t="inlineStr">
@@ -15019,12 +15043,12 @@
       </c>
       <c r="B204" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C204" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D204" s="3" t="inlineStr">
@@ -15046,12 +15070,12 @@
       </c>
       <c r="B205" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C205" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D205" s="3" t="inlineStr">
@@ -15073,12 +15097,12 @@
       </c>
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D206" s="3" t="inlineStr">
@@ -15100,12 +15124,12 @@
       </c>
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D207" s="3" t="inlineStr">
@@ -15127,12 +15151,12 @@
       </c>
       <c r="B208" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D208" s="3" t="inlineStr">
@@ -15154,12 +15178,12 @@
       </c>
       <c r="B209" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D209" s="3" t="inlineStr">
@@ -15181,12 +15205,12 @@
       </c>
       <c r="B210" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D210" s="3" t="inlineStr">
@@ -15208,12 +15232,12 @@
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D211" s="3" t="inlineStr">
@@ -15235,12 +15259,12 @@
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D212" s="3" t="inlineStr">
@@ -15262,12 +15286,12 @@
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D213" s="3" t="inlineStr">
@@ -15289,12 +15313,12 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D214" s="3" t="inlineStr">
@@ -15316,12 +15340,12 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D215" s="3" t="inlineStr">
@@ -15343,12 +15367,12 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
@@ -15370,12 +15394,12 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -15397,12 +15421,12 @@
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
@@ -15424,12 +15448,12 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D219" s="3" t="inlineStr">
@@ -15451,12 +15475,12 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D220" s="3" t="inlineStr">
@@ -15478,12 +15502,12 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D221" s="3" t="inlineStr">
@@ -15505,12 +15529,12 @@
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D222" s="3" t="inlineStr">
@@ -15532,12 +15556,12 @@
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D223" s="3" t="inlineStr">
@@ -15559,12 +15583,12 @@
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R4-11</t>
         </is>
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
         </is>
       </c>
       <c r="D224" s="3" t="inlineStr">
@@ -15586,12 +15610,12 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R4-ISO</t>
         </is>
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
         </is>
       </c>
       <c r="D225" s="3" t="inlineStr">
@@ -15613,12 +15637,12 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R5-01</t>
         </is>
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
         </is>
       </c>
       <c r="D226" s="3" t="inlineStr">
@@ -15640,12 +15664,12 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R5-02</t>
         </is>
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
         </is>
       </c>
       <c r="D227" s="3" t="inlineStr">
@@ -15667,12 +15691,12 @@
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R5-03</t>
         </is>
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
         </is>
       </c>
       <c r="D228" s="3" t="inlineStr">
@@ -15694,12 +15718,12 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R5-04</t>
         </is>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
@@ -15721,12 +15745,12 @@
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R5-05</t>
         </is>
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
         </is>
       </c>
       <c r="D230" s="3" t="inlineStr">
@@ -15748,20 +15772,155 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
+          <t>E2E-R5-06</t>
+        </is>
+      </c>
+      <c r="C231" s="3" t="inlineStr">
+        <is>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+        </is>
+      </c>
+      <c r="D231" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E231" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B232" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-07</t>
+        </is>
+      </c>
+      <c r="C232" s="3" t="inlineStr">
+        <is>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+        </is>
+      </c>
+      <c r="D232" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E232" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B233" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-08</t>
+        </is>
+      </c>
+      <c r="C233" s="3" t="inlineStr">
+        <is>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+        </is>
+      </c>
+      <c r="D233" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E233" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B234" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-09</t>
+        </is>
+      </c>
+      <c r="C234" s="3" t="inlineStr">
+        <is>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+        </is>
+      </c>
+      <c r="D234" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E234" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B235" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C235" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D235" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E235" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B236" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C231" s="3" t="inlineStr">
+      <c r="C236" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D231" s="3" t="inlineStr">
+      <c r="D236" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E231" s="3" t="inlineStr">
+      <c r="E236" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
@@ -16715,7 +16874,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Proposed — decided by SP-08</t>
+          <t>Recommended: CEL with Procera extensions (SP-08, 2026-10-11); final acceptance at G1</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -16737,7 +16896,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Proposed — validated by SP-09</t>
+          <t>Validated by SP-09 (2026-10-11); acceptance at G1</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">

</xml_diff>

<commit_message>
chore: CI Postgres+Valkey services, test-all bootstraps throwaway servers, licence wording, tracker
- CI rust job: postgres:16 and valkey:8 services for integration tests
- test-all.sh: throwaway Postgres (:16432) and Redis/Valkey (:16391) when no
  URLs are set; cleans up on exit
- deny/JS gate: allow BSL-1.0 (Boost); policy text now says BUSL-1.1
  (Business Source) to avoid confusion
- tracker: BPMS-003/010/025/033 done; 026/029 in progress

Evidence: ./scripts/test-all.sh -> all checks passed.
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E236" headerRowCount="1">
-  <autoFilter ref="A1:E236"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E240" headerRowCount="1">
+  <autoFilter ref="A1:E240"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -3104,13 +3104,17 @@
       <c r="J4" s="3" t="inlineStr"/>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr"/>
       <c r="N4" s="3" t="inlineStr"/>
-      <c r="O4" s="3" t="inlineStr"/>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>SP-01..06 native runtime: 10k instances under 1329 crashes 0 lost; race exactly-once; join once; 410 retries 0 dup effects; 30-day pinning; BPMN 54-node lossless round trip — docs/spikes/SP-01-06; ADR-0015 recommended</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -3523,7 +3527,7 @@
       <c r="J11" s="3" t="inlineStr"/>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr"/>
@@ -3531,7 +3535,7 @@
       <c r="N11" s="3" t="inlineStr"/>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>Slice 1 done: web workspace (Vite/React/TS), tokens.json→CSS with 40 WCAG contrast checks, Button/TextField/Checkbox/Notice on React Aria, app shell, gallery, axe+keyboard+reflow+target E2E (E2E-P0-05..09). Next: Select, Dialog, DataGrid shell, Tabs</t>
+          <t>Tokens (41 contrast checks + forbidden-pair guard), Button/TextField/Checkbox/Notice/Select/ConfirmDialog/Tabs/DataGrid shell on React Aria + TanStack, app shell, gallery; axe light/dark, keyboard, focus trap, aria-sort, reflow, targets (E2E-P0-05..13)</t>
         </is>
       </c>
     </row>
@@ -4137,13 +4141,17 @@
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L21" s="3" t="inlineStr"/>
       <c r="M21" s="3" t="inlineStr"/>
       <c r="N21" s="3" t="inlineStr"/>
-      <c r="O21" s="3" t="inlineStr"/>
+      <c r="O21" s="3" t="inlineStr">
+        <is>
+          <t>procera-db: migrations (0001-0003), roles bootstrap (app/migrator/discovery), WsTx with tx-local set_config, procera_enable_workspace_rls() with NULLIF, procera_rls_violations guard (tested + enforced at startup), discovery.* functions with column grants; 6 DB tests</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -4198,13 +4206,17 @@
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L22" s="3" t="inlineStr"/>
       <c r="M22" s="3" t="inlineStr"/>
       <c r="N22" s="3" t="inlineStr"/>
-      <c r="O22" s="3" t="inlineStr"/>
+      <c r="O22" s="3" t="inlineStr">
+        <is>
+          <t>procera-audit: JCS/SHA-256 per-workspace chain in the business tx, batched sealer, verifier, monthly partitions with forced RLS, append-only grants + trigger; tamper test passes. Remaining: route audit-coverage contract test (with BPMS-020 routes)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -4381,13 +4393,17 @@
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L25" s="3" t="inlineStr"/>
       <c r="M25" s="3" t="inlineStr"/>
       <c r="N25" s="3" t="inlineStr"/>
-      <c r="O25" s="3" t="inlineStr"/>
+      <c r="O25" s="3" t="inlineStr">
+        <is>
+          <t>Outbox/inbox/idempotency tables + helpers with tests (disjoint SKIP LOCKED claims, replay/conflict). Remaining: dispatcher loop (LISTEN/NOTIFY + Bus trait)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -4625,13 +4641,17 @@
       </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L29" s="3" t="inlineStr"/>
       <c r="M29" s="3" t="inlineStr"/>
       <c r="N29" s="3" t="inlineStr"/>
-      <c r="O29" s="3" t="inlineStr"/>
+      <c r="O29" s="3" t="inlineStr">
+        <is>
+          <t>procera-cache: memory + Valkey/Redis (redis 1.7, BSD-3) with ws:/sys: key namespacing, TTL-only writes, Lua fixed-window rate limit with in-process fallback, degraded health; wired into procera (/readyz), CI Valkey service</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -9544,7 +9564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E236"/>
+  <dimension ref="A1:E240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -13936,12 +13956,12 @@
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-P0-10</t>
         </is>
       </c>
       <c r="C163" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>Confirm dialog: Cancel focused first, focus trapped, axe-clean, Esc closes and restores focus to the trigger; confirm performs the action | WCAG 2.4.3, 2.1.2; docs/05 §7.1.1</t>
         </is>
       </c>
       <c r="D163" s="3" t="inlineStr">
@@ -13963,12 +13983,12 @@
       </c>
       <c r="B164" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-P0-11</t>
         </is>
       </c>
       <c r="C164" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>Data grid: `aria-sort` none→ascending→descending, filter result count announced in a live region, select-all count | FR-V01/V02/V06/V08</t>
         </is>
       </c>
       <c r="D164" s="3" t="inlineStr">
@@ -13990,12 +14010,12 @@
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-P0-12</t>
         </is>
       </c>
       <c r="C165" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>Select operable by keyboard only (open, move, choose) | WCAG 2.1.1</t>
         </is>
       </c>
       <c r="D165" s="3" t="inlineStr">
@@ -14017,12 +14037,12 @@
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-P0-13</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>Tabs: arrow keys move focus and selection; the panel follows | WAI-ARIA tabs pattern</t>
         </is>
       </c>
       <c r="D166" s="3" t="inlineStr">
@@ -14044,12 +14064,12 @@
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C167" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
         </is>
       </c>
       <c r="D167" s="3" t="inlineStr">
@@ -14071,12 +14091,12 @@
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D168" s="3" t="inlineStr">
@@ -14098,12 +14118,12 @@
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C169" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D169" s="3" t="inlineStr">
@@ -14125,12 +14145,12 @@
       </c>
       <c r="B170" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C170" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
         </is>
       </c>
       <c r="D170" s="3" t="inlineStr">
@@ -14152,12 +14172,12 @@
       </c>
       <c r="B171" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C171" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
         </is>
       </c>
       <c r="D171" s="3" t="inlineStr">
@@ -14179,12 +14199,12 @@
       </c>
       <c r="B172" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C172" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D172" s="3" t="inlineStr">
@@ -14206,12 +14226,12 @@
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C173" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D173" s="3" t="inlineStr">
@@ -14233,12 +14253,12 @@
       </c>
       <c r="B174" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C174" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
         </is>
       </c>
       <c r="D174" s="3" t="inlineStr">
@@ -14260,12 +14280,12 @@
       </c>
       <c r="B175" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C175" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D175" s="3" t="inlineStr">
@@ -14287,12 +14307,12 @@
       </c>
       <c r="B176" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C176" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D176" s="3" t="inlineStr">
@@ -14314,12 +14334,12 @@
       </c>
       <c r="B177" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C177" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D177" s="3" t="inlineStr">
@@ -14341,12 +14361,12 @@
       </c>
       <c r="B178" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C178" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D178" s="3" t="inlineStr">
@@ -14368,12 +14388,12 @@
       </c>
       <c r="B179" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C179" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
         </is>
       </c>
       <c r="D179" s="3" t="inlineStr">
@@ -14395,12 +14415,12 @@
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C180" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
         </is>
       </c>
       <c r="D180" s="3" t="inlineStr">
@@ -14422,12 +14442,12 @@
       </c>
       <c r="B181" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C181" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
         </is>
       </c>
       <c r="D181" s="3" t="inlineStr">
@@ -14449,12 +14469,12 @@
       </c>
       <c r="B182" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C182" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D182" s="3" t="inlineStr">
@@ -14476,12 +14496,12 @@
       </c>
       <c r="B183" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C183" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
         </is>
       </c>
       <c r="D183" s="3" t="inlineStr">
@@ -14503,12 +14523,12 @@
       </c>
       <c r="B184" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C184" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
         </is>
       </c>
       <c r="D184" s="3" t="inlineStr">
@@ -14530,12 +14550,12 @@
       </c>
       <c r="B185" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D185" s="3" t="inlineStr">
@@ -14557,12 +14577,12 @@
       </c>
       <c r="B186" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C186" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
         </is>
       </c>
       <c r="D186" s="3" t="inlineStr">
@@ -14584,12 +14604,12 @@
       </c>
       <c r="B187" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D187" s="3" t="inlineStr">
@@ -14611,12 +14631,12 @@
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D188" s="3" t="inlineStr">
@@ -14638,12 +14658,12 @@
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D189" s="3" t="inlineStr">
@@ -14665,12 +14685,12 @@
       </c>
       <c r="B190" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C190" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D190" s="3" t="inlineStr">
@@ -14692,12 +14712,12 @@
       </c>
       <c r="B191" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D191" s="3" t="inlineStr">
@@ -14719,12 +14739,12 @@
       </c>
       <c r="B192" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C192" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D192" s="3" t="inlineStr">
@@ -14746,12 +14766,12 @@
       </c>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D193" s="3" t="inlineStr">
@@ -14773,12 +14793,12 @@
       </c>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C194" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D194" s="3" t="inlineStr">
@@ -14800,12 +14820,12 @@
       </c>
       <c r="B195" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D195" s="3" t="inlineStr">
@@ -14827,12 +14847,12 @@
       </c>
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C196" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D196" s="3" t="inlineStr">
@@ -14854,12 +14874,12 @@
       </c>
       <c r="B197" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D197" s="3" t="inlineStr">
@@ -14881,12 +14901,12 @@
       </c>
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C198" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D198" s="3" t="inlineStr">
@@ -14908,12 +14928,12 @@
       </c>
       <c r="B199" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D199" s="3" t="inlineStr">
@@ -14935,12 +14955,12 @@
       </c>
       <c r="B200" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C200" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D200" s="3" t="inlineStr">
@@ -14962,12 +14982,12 @@
       </c>
       <c r="B201" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D201" s="3" t="inlineStr">
@@ -14989,12 +15009,12 @@
       </c>
       <c r="B202" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C202" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D202" s="3" t="inlineStr">
@@ -15016,12 +15036,12 @@
       </c>
       <c r="B203" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D203" s="3" t="inlineStr">
@@ -15043,12 +15063,12 @@
       </c>
       <c r="B204" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C204" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D204" s="3" t="inlineStr">
@@ -15070,12 +15090,12 @@
       </c>
       <c r="B205" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C205" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D205" s="3" t="inlineStr">
@@ -15097,12 +15117,12 @@
       </c>
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D206" s="3" t="inlineStr">
@@ -15124,12 +15144,12 @@
       </c>
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D207" s="3" t="inlineStr">
@@ -15151,12 +15171,12 @@
       </c>
       <c r="B208" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D208" s="3" t="inlineStr">
@@ -15178,12 +15198,12 @@
       </c>
       <c r="B209" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D209" s="3" t="inlineStr">
@@ -15205,12 +15225,12 @@
       </c>
       <c r="B210" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D210" s="3" t="inlineStr">
@@ -15232,12 +15252,12 @@
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D211" s="3" t="inlineStr">
@@ -15259,12 +15279,12 @@
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D212" s="3" t="inlineStr">
@@ -15286,12 +15306,12 @@
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D213" s="3" t="inlineStr">
@@ -15313,12 +15333,12 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D214" s="3" t="inlineStr">
@@ -15340,12 +15360,12 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D215" s="3" t="inlineStr">
@@ -15367,12 +15387,12 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
@@ -15394,12 +15414,12 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -15421,12 +15441,12 @@
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
@@ -15448,12 +15468,12 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D219" s="3" t="inlineStr">
@@ -15475,12 +15495,12 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D220" s="3" t="inlineStr">
@@ -15502,12 +15522,12 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D221" s="3" t="inlineStr">
@@ -15529,12 +15549,12 @@
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D222" s="3" t="inlineStr">
@@ -15556,12 +15576,12 @@
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D223" s="3" t="inlineStr">
@@ -15583,12 +15603,12 @@
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D224" s="3" t="inlineStr">
@@ -15610,12 +15630,12 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D225" s="3" t="inlineStr">
@@ -15637,12 +15657,12 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D226" s="3" t="inlineStr">
@@ -15664,12 +15684,12 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D227" s="3" t="inlineStr">
@@ -15691,12 +15711,12 @@
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R4-11</t>
         </is>
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
         </is>
       </c>
       <c r="D228" s="3" t="inlineStr">
@@ -15718,12 +15738,12 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R4-ISO</t>
         </is>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
@@ -15745,12 +15765,12 @@
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R5-01</t>
         </is>
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
         </is>
       </c>
       <c r="D230" s="3" t="inlineStr">
@@ -15772,12 +15792,12 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R5-02</t>
         </is>
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
         </is>
       </c>
       <c r="D231" s="3" t="inlineStr">
@@ -15799,12 +15819,12 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R5-03</t>
         </is>
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
         </is>
       </c>
       <c r="D232" s="3" t="inlineStr">
@@ -15826,12 +15846,12 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R5-04</t>
         </is>
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
         </is>
       </c>
       <c r="D233" s="3" t="inlineStr">
@@ -15853,12 +15873,12 @@
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R5-05</t>
         </is>
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
         </is>
       </c>
       <c r="D234" s="3" t="inlineStr">
@@ -15880,12 +15900,12 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R5-06</t>
         </is>
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
         </is>
       </c>
       <c r="D235" s="3" t="inlineStr">
@@ -15907,20 +15927,128 @@
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
+          <t>E2E-R5-07</t>
+        </is>
+      </c>
+      <c r="C236" s="3" t="inlineStr">
+        <is>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+        </is>
+      </c>
+      <c r="D236" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E236" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B237" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-08</t>
+        </is>
+      </c>
+      <c r="C237" s="3" t="inlineStr">
+        <is>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+        </is>
+      </c>
+      <c r="D237" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E237" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B238" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-09</t>
+        </is>
+      </c>
+      <c r="C238" s="3" t="inlineStr">
+        <is>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+        </is>
+      </c>
+      <c r="D238" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E238" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B239" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C239" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D239" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E239" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B240" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C236" s="3" t="inlineStr">
+      <c r="C240" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D236" s="3" t="inlineStr">
+      <c r="D240" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E236" s="3" t="inlineStr">
+      <c r="E240" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
@@ -16984,7 +17112,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Proposed — decided at G1</t>
+          <t>Recommended: native interpreter (SP-01…06 all pass, 2026-10-11); final acceptance at G1</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(api): auth and system HTTP APIs, E2E packs R1-AUTH and R1-SYS, DB-backed E2E in CI
- /api/v1/auth/{login,mfa,refresh,logout}, /api/v1/me (+ sign-out-everywhere,
  TOTP enrol/confirm); /sysapi/v1 workspaces; RFC 9457 errors; per-IP login
  rate limit (configurable); serve wires one shared clock into identity and
  platform; logs go to stderr so 'procera keygen' output is clean
- Test-only controls: seed users, issue bootstrap token, grant system roles,
  verify audit chains (e2e feature only)
- E2E-R1-AUTH-01..07 and E2E-R1-SYS-01..05; TOTP fixtures use server time
- test-all.sh and CI create a fresh database, run roles + migrations and start
  a database-backed e2e server
- tracker: BPMS-020/021 done; 022/030 in progress

Evidence: ./scripts/test-all.sh -> all checks passed (25/25 E2E).
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E240" headerRowCount="1">
-  <autoFilter ref="A1:E240"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E252" headerRowCount="1">
+  <autoFilter ref="A1:E252"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -280,8 +280,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="DecisionsT" displayName="DecisionsT" ref="A1:D20" headerRowCount="1">
-  <autoFilter ref="A1:D20"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="DecisionsT" displayName="DecisionsT" ref="A1:D21" headerRowCount="1">
+  <autoFilter ref="A1:D21"/>
   <tableColumns count="4">
     <tableColumn id="1" name="ADR"/>
     <tableColumn id="2" name="Decision"/>
@@ -3836,13 +3836,17 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr"/>
       <c r="M16" s="3" t="inlineStr"/>
       <c r="N16" s="3" t="inlineStr"/>
-      <c r="O16" s="3" t="inlineStr"/>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>procera-platform + /sysapi/v1: one-time bootstrap token (printed at startup until bootstrapped), system.owner/admin/operator/auditor fixed authz table, MFA required for system plane, workspace create/list/get/rename/suspend/restore/schedule-deletion with If-Match + ETag, profile quotas, platform setting floors seeded, all audited; E2E-R1-SYS-01..05</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -3897,13 +3901,17 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr"/>
       <c r="M17" s="3" t="inlineStr"/>
       <c r="N17" s="3" t="inlineStr"/>
-      <c r="O17" s="3" t="inlineStr"/>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t>procera-identity + /api/v1/auth: users, Argon2id (policy, rehash, enumeration-safe), JWT access (ADR-0020) + rotating refresh with reuse detection, DB login throttling + per-IP rate limit, logout, sign-out-everywhere, deactivation via token_version; audited; E2E-R1-AUTH-01..05,07</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -3958,13 +3966,17 @@
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L18" s="3" t="inlineStr"/>
       <c r="M18" s="3" t="inlineStr"/>
       <c r="N18" s="3" t="inlineStr"/>
-      <c r="O18" s="3" t="inlineStr"/>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>TOTP (RFC 6238, replay-protected, sealed secrets) + 10 recovery codes + MFA login done (E2E-R1-AUTH-06). Remaining: WebAuthn/passkeys, step-up endpoint, MFA-required-by-role enforcement</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -4458,13 +4470,17 @@
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L26" s="3" t="inlineStr"/>
       <c r="M26" s="3" t="inlineStr"/>
       <c r="N26" s="3" t="inlineStr"/>
-      <c r="O26" s="3" t="inlineStr"/>
+      <c r="O26" s="3" t="inlineStr">
+        <is>
+          <t>procera-crypto: LocalKey (env root key, HMAC-derived purpose keys), AES-256-GCM seal/open bound to context, token helpers, procera keygen. Remaining: KMS/OpenBao adapters, per-workspace KEKs, rotation</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -9564,7 +9580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E240"/>
+  <dimension ref="A1:E252"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14064,12 +14080,12 @@
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-AUTH-01</t>
         </is>
       </c>
       <c r="C167" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>Login returns a ≤ 15 min Bearer JWT + HttpOnly/SameSite=Strict refresh cookie, `Cache-Control: no-store`; `/me` works only with a valid token; forged token → 401 problem+json | §3.2</t>
         </is>
       </c>
       <c r="D167" s="3" t="inlineStr">
@@ -14091,12 +14107,12 @@
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-AUTH-02</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>Wrong password and unknown account return the same error code | enumeration resistance</t>
         </is>
       </c>
       <c r="D168" s="3" t="inlineStr">
@@ -14118,12 +14134,12 @@
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-AUTH-03</t>
         </is>
       </c>
       <c r="C169" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>Refresh rotates the cookie; replaying the old refresh token → `token_reused` and the legitimate session is revoked too | SEC-14</t>
         </is>
       </c>
       <c r="D169" s="3" t="inlineStr">
@@ -14145,12 +14161,12 @@
       </c>
       <c r="B170" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-AUTH-04</t>
         </is>
       </c>
       <c r="C170" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>Cookie endpoints without `X-Requested-With: procera` → 403 `csrf` | CSRF</t>
         </is>
       </c>
       <c r="D170" s="3" t="inlineStr">
@@ -14172,12 +14188,12 @@
       </c>
       <c r="B171" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-AUTH-05</t>
         </is>
       </c>
       <c r="C171" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>Logout revokes the family and clears the cookie | §3.2</t>
         </is>
       </c>
       <c r="D171" s="3" t="inlineStr">
@@ -14199,12 +14215,12 @@
       </c>
       <c r="B172" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-AUTH-06</t>
         </is>
       </c>
       <c r="C172" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>TOTP enrolment (otpauth URI), MFA login (`amr=[pwd,otp]`), MFA token rejected as access token, TOTP replay rejected, recovery code single-use | §3.6</t>
         </is>
       </c>
       <c r="D172" s="3" t="inlineStr">
@@ -14226,12 +14242,12 @@
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-AUTH-07</t>
         </is>
       </c>
       <c r="C173" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>Sign-out-everywhere rejects another device's unexpired JWT and refresh; system audit chain verifies | SEC-04, AUD-01</t>
         </is>
       </c>
       <c r="D173" s="3" t="inlineStr">
@@ -14253,12 +14269,12 @@
       </c>
       <c r="B174" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-SYS-01</t>
         </is>
       </c>
       <c r="C174" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>Bootstrap: wrong token 401; one-time token creates `system.owner`; reuse 409; no further tokens | FR-S01 (= E2E-R1-01)</t>
         </is>
       </c>
       <c r="D174" s="3" t="inlineStr">
@@ -14280,12 +14296,12 @@
       </c>
       <c r="B175" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-SYS-02</t>
         </is>
       </c>
       <c r="C175" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>System API returns 404 to non-system users and 403 `mfa_required` to system users without MFA | docs/12 §1, docs/06 §3.6</t>
         </is>
       </c>
       <c r="D175" s="3" t="inlineStr">
@@ -14307,12 +14323,12 @@
       </c>
       <c r="B176" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-SYS-03</t>
         </is>
       </c>
       <c r="C176" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>Create workspaces A (starter) and B (enterprise): 201 + Location + ETag, profile quotas, duplicate slug 409, invalid slug 422, listing | FR-S02/S04 (= E2E-R1-02)</t>
         </is>
       </c>
       <c r="D176" s="3" t="inlineStr">
@@ -14334,12 +14350,12 @@
       </c>
       <c r="B177" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-SYS-04</t>
         </is>
       </c>
       <c r="C177" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>Suspend read-only with reason; stale `If-Match` → 412; restore with current ETag; invalid transition 409; schedule deletion (grace validated) | FR-S02 (= E2E-R1-17)</t>
         </is>
       </c>
       <c r="D177" s="3" t="inlineStr">
@@ -14361,12 +14377,12 @@
       </c>
       <c r="B178" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-SYS-05</t>
         </is>
       </c>
       <c r="C178" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>`system.operator` can read but not write; system audit chain verifies | docs/12 §4.1, FR-S09</t>
         </is>
       </c>
       <c r="D178" s="3" t="inlineStr">
@@ -14388,12 +14404,12 @@
       </c>
       <c r="B179" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C179" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
         </is>
       </c>
       <c r="D179" s="3" t="inlineStr">
@@ -14415,12 +14431,12 @@
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C180" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D180" s="3" t="inlineStr">
@@ -14442,12 +14458,12 @@
       </c>
       <c r="B181" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C181" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D181" s="3" t="inlineStr">
@@ -14469,12 +14485,12 @@
       </c>
       <c r="B182" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C182" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
         </is>
       </c>
       <c r="D182" s="3" t="inlineStr">
@@ -14496,12 +14512,12 @@
       </c>
       <c r="B183" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C183" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
         </is>
       </c>
       <c r="D183" s="3" t="inlineStr">
@@ -14523,12 +14539,12 @@
       </c>
       <c r="B184" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C184" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D184" s="3" t="inlineStr">
@@ -14550,12 +14566,12 @@
       </c>
       <c r="B185" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D185" s="3" t="inlineStr">
@@ -14577,12 +14593,12 @@
       </c>
       <c r="B186" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C186" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
         </is>
       </c>
       <c r="D186" s="3" t="inlineStr">
@@ -14604,12 +14620,12 @@
       </c>
       <c r="B187" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D187" s="3" t="inlineStr">
@@ -14631,12 +14647,12 @@
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D188" s="3" t="inlineStr">
@@ -14658,12 +14674,12 @@
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D189" s="3" t="inlineStr">
@@ -14685,12 +14701,12 @@
       </c>
       <c r="B190" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C190" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D190" s="3" t="inlineStr">
@@ -14712,12 +14728,12 @@
       </c>
       <c r="B191" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
         </is>
       </c>
       <c r="D191" s="3" t="inlineStr">
@@ -14739,12 +14755,12 @@
       </c>
       <c r="B192" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C192" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
         </is>
       </c>
       <c r="D192" s="3" t="inlineStr">
@@ -14766,12 +14782,12 @@
       </c>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
         </is>
       </c>
       <c r="D193" s="3" t="inlineStr">
@@ -14793,12 +14809,12 @@
       </c>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C194" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D194" s="3" t="inlineStr">
@@ -14820,12 +14836,12 @@
       </c>
       <c r="B195" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
         </is>
       </c>
       <c r="D195" s="3" t="inlineStr">
@@ -14847,12 +14863,12 @@
       </c>
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C196" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
         </is>
       </c>
       <c r="D196" s="3" t="inlineStr">
@@ -14874,12 +14890,12 @@
       </c>
       <c r="B197" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D197" s="3" t="inlineStr">
@@ -14901,12 +14917,12 @@
       </c>
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C198" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
         </is>
       </c>
       <c r="D198" s="3" t="inlineStr">
@@ -14928,12 +14944,12 @@
       </c>
       <c r="B199" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D199" s="3" t="inlineStr">
@@ -14955,12 +14971,12 @@
       </c>
       <c r="B200" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C200" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D200" s="3" t="inlineStr">
@@ -14982,12 +14998,12 @@
       </c>
       <c r="B201" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D201" s="3" t="inlineStr">
@@ -15009,12 +15025,12 @@
       </c>
       <c r="B202" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C202" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D202" s="3" t="inlineStr">
@@ -15036,12 +15052,12 @@
       </c>
       <c r="B203" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D203" s="3" t="inlineStr">
@@ -15063,12 +15079,12 @@
       </c>
       <c r="B204" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C204" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D204" s="3" t="inlineStr">
@@ -15090,12 +15106,12 @@
       </c>
       <c r="B205" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C205" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D205" s="3" t="inlineStr">
@@ -15117,12 +15133,12 @@
       </c>
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D206" s="3" t="inlineStr">
@@ -15144,12 +15160,12 @@
       </c>
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D207" s="3" t="inlineStr">
@@ -15171,12 +15187,12 @@
       </c>
       <c r="B208" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D208" s="3" t="inlineStr">
@@ -15198,12 +15214,12 @@
       </c>
       <c r="B209" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D209" s="3" t="inlineStr">
@@ -15225,12 +15241,12 @@
       </c>
       <c r="B210" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D210" s="3" t="inlineStr">
@@ -15252,12 +15268,12 @@
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D211" s="3" t="inlineStr">
@@ -15279,12 +15295,12 @@
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D212" s="3" t="inlineStr">
@@ -15306,12 +15322,12 @@
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D213" s="3" t="inlineStr">
@@ -15333,12 +15349,12 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D214" s="3" t="inlineStr">
@@ -15360,12 +15376,12 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D215" s="3" t="inlineStr">
@@ -15387,12 +15403,12 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
@@ -15414,12 +15430,12 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -15441,12 +15457,12 @@
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
@@ -15468,12 +15484,12 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D219" s="3" t="inlineStr">
@@ -15495,12 +15511,12 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D220" s="3" t="inlineStr">
@@ -15522,12 +15538,12 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D221" s="3" t="inlineStr">
@@ -15549,12 +15565,12 @@
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D222" s="3" t="inlineStr">
@@ -15576,12 +15592,12 @@
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D223" s="3" t="inlineStr">
@@ -15603,12 +15619,12 @@
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D224" s="3" t="inlineStr">
@@ -15630,12 +15646,12 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D225" s="3" t="inlineStr">
@@ -15657,12 +15673,12 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D226" s="3" t="inlineStr">
@@ -15684,12 +15700,12 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D227" s="3" t="inlineStr">
@@ -15711,12 +15727,12 @@
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D228" s="3" t="inlineStr">
@@ -15738,12 +15754,12 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
@@ -15765,12 +15781,12 @@
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D230" s="3" t="inlineStr">
@@ -15792,12 +15808,12 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D231" s="3" t="inlineStr">
@@ -15819,12 +15835,12 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D232" s="3" t="inlineStr">
@@ -15846,12 +15862,12 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D233" s="3" t="inlineStr">
@@ -15873,12 +15889,12 @@
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D234" s="3" t="inlineStr">
@@ -15900,12 +15916,12 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D235" s="3" t="inlineStr">
@@ -15927,12 +15943,12 @@
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D236" s="3" t="inlineStr">
@@ -15954,12 +15970,12 @@
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D237" s="3" t="inlineStr">
@@ -15981,12 +15997,12 @@
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D238" s="3" t="inlineStr">
@@ -16008,12 +16024,12 @@
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D239" s="3" t="inlineStr">
@@ -16035,20 +16051,344 @@
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
+          <t>E2E-R4-11</t>
+        </is>
+      </c>
+      <c r="C240" s="3" t="inlineStr">
+        <is>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+        </is>
+      </c>
+      <c r="D240" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E240" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B241" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-ISO</t>
+        </is>
+      </c>
+      <c r="C241" s="3" t="inlineStr">
+        <is>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+        </is>
+      </c>
+      <c r="D241" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E241" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B242" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-01</t>
+        </is>
+      </c>
+      <c r="C242" s="3" t="inlineStr">
+        <is>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+        </is>
+      </c>
+      <c r="D242" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E242" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B243" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-02</t>
+        </is>
+      </c>
+      <c r="C243" s="3" t="inlineStr">
+        <is>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+        </is>
+      </c>
+      <c r="D243" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E243" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B244" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-03</t>
+        </is>
+      </c>
+      <c r="C244" s="3" t="inlineStr">
+        <is>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+        </is>
+      </c>
+      <c r="D244" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E244" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B245" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-04</t>
+        </is>
+      </c>
+      <c r="C245" s="3" t="inlineStr">
+        <is>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+        </is>
+      </c>
+      <c r="D245" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E245" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B246" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-05</t>
+        </is>
+      </c>
+      <c r="C246" s="3" t="inlineStr">
+        <is>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+        </is>
+      </c>
+      <c r="D246" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E246" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B247" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-06</t>
+        </is>
+      </c>
+      <c r="C247" s="3" t="inlineStr">
+        <is>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+        </is>
+      </c>
+      <c r="D247" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E247" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B248" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-07</t>
+        </is>
+      </c>
+      <c r="C248" s="3" t="inlineStr">
+        <is>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+        </is>
+      </c>
+      <c r="D248" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E248" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B249" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-08</t>
+        </is>
+      </c>
+      <c r="C249" s="3" t="inlineStr">
+        <is>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+        </is>
+      </c>
+      <c r="D249" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E249" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B250" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-09</t>
+        </is>
+      </c>
+      <c r="C250" s="3" t="inlineStr">
+        <is>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+        </is>
+      </c>
+      <c r="D250" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E250" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B251" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C251" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D251" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E251" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B252" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C240" s="3" t="inlineStr">
+      <c r="C252" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D240" s="3" t="inlineStr">
+      <c r="D252" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E240" s="3" t="inlineStr">
+      <c r="E252" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
@@ -16760,7 +17100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -17206,6 +17546,28 @@
       <c r="D20" s="3" t="inlineStr">
         <is>
           <t>ADR-0019-valkey-redis-cache.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>ADR-0020</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>JWT access tokens with rotating refresh tokens (no server-side sessions)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>ADR-0020-jwt-access-tokens.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(api): workspace-plane members, roles and grants APIs with E2E pack R1-MEM (BPMS-023, BPMS-024)
/api/v1 gains workspace switching, invitation accept/register, members,
roles, role grants, permission catalogue and effective permissions. Every
handler authorizes through Cedar; the WsMember extractor enforces active
membership and the workspace state gate (423 when suspended). E2E-R1-MEM-01..06
added to docs/23; tracker updated.

Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E252" headerRowCount="1">
-  <autoFilter ref="A1:E252"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E258" headerRowCount="1">
+  <autoFilter ref="A1:E258"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -4031,13 +4031,17 @@
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L19" s="3" t="inlineStr"/>
       <c r="M19" s="3" t="inlineStr"/>
       <c r="N19" s="3" t="inlineStr"/>
-      <c r="O19" s="3" t="inlineStr"/>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>procera-members + /api/v1: memberships, invitations (hashed + sealed tokens, 7-day expiry, email-bound, single use), register-by-invite, owner onboarding activates the provisioning workspace, workspace switch (ws-scoped JWT), member list, deactivation with last-owner/self guards, state gate (423 when suspended); audited; E2E-R1-MEM-01..03,05,06. Remaining: directory (departments/groups/positions/managers), CSV import, invitation revoke/resend</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -4092,13 +4096,17 @@
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L20" s="3" t="inlineStr"/>
       <c r="M20" s="3" t="inlineStr"/>
       <c r="N20" s="3" t="inlineStr"/>
-      <c r="O20" s="3" t="inlineStr"/>
+      <c r="O20" s="3" t="inlineStr">
+        <is>
+          <t>procera-access: permission catalogue + 12 role templates, custom roles (no escalation, built-ins immutable, clone lineage), scoped grants with expiry compiled to Cedar, invariants (workspace isolation, active members only), per-workspace access_revisions cache; /api/v1 roles, role-grants, permission-catalog, me/permissions; E2E-R1-MEM-04. Remaining: access preview/explain endpoint, no-escalation property test</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -9580,7 +9588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E252"/>
+  <dimension ref="A1:E258"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14404,12 +14412,12 @@
       </c>
       <c r="B179" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-MEM-01</t>
         </is>
       </c>
       <c r="C179" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>Owner registers through the system-created invitation; workspace becomes `active`; owner holds owner permissions; invitation is single-use | FR-S01, FR-W01</t>
         </is>
       </c>
       <c r="D179" s="3" t="inlineStr">
@@ -14431,12 +14439,12 @@
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-MEM-02</t>
         </is>
       </c>
       <c r="C180" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>Invite → accept only by the invited email; the token is never returned to the inviter; member appears in the list | FR-W01, docs/06 §3</t>
         </is>
       </c>
       <c r="D180" s="3" t="inlineStr">
@@ -14458,12 +14466,12 @@
       </c>
       <c r="B181" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-MEM-03</t>
         </is>
       </c>
       <c r="C181" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>A non-member cannot switch into another workspace (404); workspace APIs need a selected workspace | docs/12 §1, SEC-01</t>
         </is>
       </c>
       <c r="D181" s="3" t="inlineStr">
@@ -14485,12 +14493,12 @@
       </c>
       <c r="B182" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-MEM-04</t>
         </is>
       </c>
       <c r="C182" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>Custom role: no escalation, built-ins immutable, grant/revoke takes effect on the next request | FR-W03, ADR-0011</t>
         </is>
       </c>
       <c r="D182" s="3" t="inlineStr">
@@ -14512,12 +14520,12 @@
       </c>
       <c r="B183" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-MEM-05</t>
         </is>
       </c>
       <c r="C183" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>Admin cannot invite an owner, cannot remove the last owner or themselves; a deactivated member loses access at once | FR-W01, docs/12 §6</t>
         </is>
       </c>
       <c r="D183" s="3" t="inlineStr">
@@ -14539,12 +14547,12 @@
       </c>
       <c r="B184" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-MEM-06</t>
         </is>
       </c>
       <c r="C184" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>Read-only suspension blocks workspace writes with 423, reads still work; restore re-enables writes | FR-S02</t>
         </is>
       </c>
       <c r="D184" s="3" t="inlineStr">
@@ -14566,12 +14574,12 @@
       </c>
       <c r="B185" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
         </is>
       </c>
       <c r="D185" s="3" t="inlineStr">
@@ -14593,12 +14601,12 @@
       </c>
       <c r="B186" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C186" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D186" s="3" t="inlineStr">
@@ -14620,12 +14628,12 @@
       </c>
       <c r="B187" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D187" s="3" t="inlineStr">
@@ -14647,12 +14655,12 @@
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
         </is>
       </c>
       <c r="D188" s="3" t="inlineStr">
@@ -14674,12 +14682,12 @@
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
         </is>
       </c>
       <c r="D189" s="3" t="inlineStr">
@@ -14701,12 +14709,12 @@
       </c>
       <c r="B190" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C190" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D190" s="3" t="inlineStr">
@@ -14728,12 +14736,12 @@
       </c>
       <c r="B191" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D191" s="3" t="inlineStr">
@@ -14755,12 +14763,12 @@
       </c>
       <c r="B192" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C192" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
         </is>
       </c>
       <c r="D192" s="3" t="inlineStr">
@@ -14782,12 +14790,12 @@
       </c>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D193" s="3" t="inlineStr">
@@ -14809,12 +14817,12 @@
       </c>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C194" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D194" s="3" t="inlineStr">
@@ -14836,12 +14844,12 @@
       </c>
       <c r="B195" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D195" s="3" t="inlineStr">
@@ -14863,12 +14871,12 @@
       </c>
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C196" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D196" s="3" t="inlineStr">
@@ -14890,12 +14898,12 @@
       </c>
       <c r="B197" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
         </is>
       </c>
       <c r="D197" s="3" t="inlineStr">
@@ -14917,12 +14925,12 @@
       </c>
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C198" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
         </is>
       </c>
       <c r="D198" s="3" t="inlineStr">
@@ -14944,12 +14952,12 @@
       </c>
       <c r="B199" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
         </is>
       </c>
       <c r="D199" s="3" t="inlineStr">
@@ -14971,12 +14979,12 @@
       </c>
       <c r="B200" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C200" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D200" s="3" t="inlineStr">
@@ -14998,12 +15006,12 @@
       </c>
       <c r="B201" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
         </is>
       </c>
       <c r="D201" s="3" t="inlineStr">
@@ -15025,12 +15033,12 @@
       </c>
       <c r="B202" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C202" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
         </is>
       </c>
       <c r="D202" s="3" t="inlineStr">
@@ -15052,12 +15060,12 @@
       </c>
       <c r="B203" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D203" s="3" t="inlineStr">
@@ -15079,12 +15087,12 @@
       </c>
       <c r="B204" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C204" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
         </is>
       </c>
       <c r="D204" s="3" t="inlineStr">
@@ -15106,12 +15114,12 @@
       </c>
       <c r="B205" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C205" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D205" s="3" t="inlineStr">
@@ -15133,12 +15141,12 @@
       </c>
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D206" s="3" t="inlineStr">
@@ -15160,12 +15168,12 @@
       </c>
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D207" s="3" t="inlineStr">
@@ -15187,12 +15195,12 @@
       </c>
       <c r="B208" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D208" s="3" t="inlineStr">
@@ -15214,12 +15222,12 @@
       </c>
       <c r="B209" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D209" s="3" t="inlineStr">
@@ -15241,12 +15249,12 @@
       </c>
       <c r="B210" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D210" s="3" t="inlineStr">
@@ -15268,12 +15276,12 @@
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D211" s="3" t="inlineStr">
@@ -15295,12 +15303,12 @@
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D212" s="3" t="inlineStr">
@@ -15322,12 +15330,12 @@
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D213" s="3" t="inlineStr">
@@ -15349,12 +15357,12 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D214" s="3" t="inlineStr">
@@ -15376,12 +15384,12 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D215" s="3" t="inlineStr">
@@ -15403,12 +15411,12 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
@@ -15430,12 +15438,12 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -15457,12 +15465,12 @@
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
@@ -15484,12 +15492,12 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D219" s="3" t="inlineStr">
@@ -15511,12 +15519,12 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D220" s="3" t="inlineStr">
@@ -15538,12 +15546,12 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D221" s="3" t="inlineStr">
@@ -15565,12 +15573,12 @@
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D222" s="3" t="inlineStr">
@@ -15592,12 +15600,12 @@
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D223" s="3" t="inlineStr">
@@ -15619,12 +15627,12 @@
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D224" s="3" t="inlineStr">
@@ -15646,12 +15654,12 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D225" s="3" t="inlineStr">
@@ -15673,12 +15681,12 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D226" s="3" t="inlineStr">
@@ -15700,12 +15708,12 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D227" s="3" t="inlineStr">
@@ -15727,12 +15735,12 @@
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D228" s="3" t="inlineStr">
@@ -15754,12 +15762,12 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
@@ -15781,12 +15789,12 @@
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D230" s="3" t="inlineStr">
@@ -15808,12 +15816,12 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D231" s="3" t="inlineStr">
@@ -15835,12 +15843,12 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D232" s="3" t="inlineStr">
@@ -15862,12 +15870,12 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D233" s="3" t="inlineStr">
@@ -15889,12 +15897,12 @@
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D234" s="3" t="inlineStr">
@@ -15916,12 +15924,12 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D235" s="3" t="inlineStr">
@@ -15943,12 +15951,12 @@
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D236" s="3" t="inlineStr">
@@ -15970,12 +15978,12 @@
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D237" s="3" t="inlineStr">
@@ -15997,12 +16005,12 @@
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D238" s="3" t="inlineStr">
@@ -16024,12 +16032,12 @@
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D239" s="3" t="inlineStr">
@@ -16051,12 +16059,12 @@
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D240" s="3" t="inlineStr">
@@ -16078,12 +16086,12 @@
       </c>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D241" s="3" t="inlineStr">
@@ -16105,12 +16113,12 @@
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D242" s="3" t="inlineStr">
@@ -16132,12 +16140,12 @@
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D243" s="3" t="inlineStr">
@@ -16159,12 +16167,12 @@
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D244" s="3" t="inlineStr">
@@ -16186,12 +16194,12 @@
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D245" s="3" t="inlineStr">
@@ -16213,12 +16221,12 @@
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R4-11</t>
         </is>
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
         </is>
       </c>
       <c r="D246" s="3" t="inlineStr">
@@ -16240,12 +16248,12 @@
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R4-ISO</t>
         </is>
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
         </is>
       </c>
       <c r="D247" s="3" t="inlineStr">
@@ -16267,12 +16275,12 @@
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R5-01</t>
         </is>
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
@@ -16294,12 +16302,12 @@
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R5-02</t>
         </is>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
         </is>
       </c>
       <c r="D249" s="3" t="inlineStr">
@@ -16321,12 +16329,12 @@
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R5-03</t>
         </is>
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
         </is>
       </c>
       <c r="D250" s="3" t="inlineStr">
@@ -16348,12 +16356,12 @@
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R5-04</t>
         </is>
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
         </is>
       </c>
       <c r="D251" s="3" t="inlineStr">
@@ -16375,20 +16383,182 @@
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
+          <t>E2E-R5-05</t>
+        </is>
+      </c>
+      <c r="C252" s="3" t="inlineStr">
+        <is>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+        </is>
+      </c>
+      <c r="D252" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E252" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B253" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-06</t>
+        </is>
+      </c>
+      <c r="C253" s="3" t="inlineStr">
+        <is>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+        </is>
+      </c>
+      <c r="D253" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E253" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B254" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-07</t>
+        </is>
+      </c>
+      <c r="C254" s="3" t="inlineStr">
+        <is>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+        </is>
+      </c>
+      <c r="D254" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E254" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B255" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-08</t>
+        </is>
+      </c>
+      <c r="C255" s="3" t="inlineStr">
+        <is>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+        </is>
+      </c>
+      <c r="D255" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E255" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B256" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-09</t>
+        </is>
+      </c>
+      <c r="C256" s="3" t="inlineStr">
+        <is>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+        </is>
+      </c>
+      <c r="D256" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E256" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B257" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C257" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D257" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E257" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B258" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C252" s="3" t="inlineStr">
+      <c r="C258" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D252" s="3" t="inlineStr">
+      <c r="D258" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E252" s="3" t="inlineStr">
+      <c r="E258" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
feat(api): invitation list/revoke/resend, role preview, audited role and grant changes; E2E-R1-MEM-07..08 (BPMS-023, BPMS-024)
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E258" headerRowCount="1">
-  <autoFilter ref="A1:E258"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E260" headerRowCount="1">
+  <autoFilter ref="A1:E260"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -4039,7 +4039,7 @@
       <c r="N19" s="3" t="inlineStr"/>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>procera-members + /api/v1: memberships, invitations (hashed + sealed tokens, 7-day expiry, email-bound, single use), register-by-invite, owner onboarding activates the provisioning workspace, workspace switch (ws-scoped JWT), member list, deactivation with last-owner/self guards, state gate (423 when suspended); audited; E2E-R1-MEM-01..03,05,06. Remaining: directory (departments/groups/positions/managers), CSV import, invitation revoke/resend</t>
+          <t>procera-members + /api/v1: memberships, invitations (hashed + sealed tokens, 7-day expiry, email-bound, single use; list, revoke, resend), register-by-invite, owner onboarding activates the provisioning workspace, workspace switch (ws-scoped JWT), member list, deactivation with last-owner/self guards, state gate (423 when suspended); audited; E2E-R1-MEM-01..03,05..07. Remaining: directory (departments/groups/positions/managers), CSV import</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       <c r="N20" s="3" t="inlineStr"/>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>procera-access: permission catalogue + 12 role templates, custom roles (no escalation, built-ins immutable, clone lineage), scoped grants with expiry compiled to Cedar, invariants (workspace isolation, active members only), per-workspace access_revisions cache; /api/v1 roles, role-grants, permission-catalog, me/permissions; E2E-R1-MEM-04. Remaining: access preview/explain endpoint, no-escalation property test</t>
+          <t>procera-access: permission catalogue + 12 role templates, custom roles (no escalation on create/edit/grant/revoke, built-ins immutable, clone lineage), scoped expiring grants compiled to Cedar, invariants (workspace isolation, active members only), last-owner protection, role change preview, per-workspace access_revisions cache; all role/grant changes audited; no-escalation property test (proptest, 64 cases vs Postgres); E2E-R1-MEM-04,08. Remaining: preview-matches-effect property test, group/directory-rule assignment (needs BPMS-023 directory)</t>
         </is>
       </c>
     </row>
@@ -9588,7 +9588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E258"/>
+  <dimension ref="A1:E260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14574,12 +14574,12 @@
       </c>
       <c r="B185" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-MEM-07</t>
         </is>
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>Pending invitations listed; revoking kills the token (404); resend issues a new working token | FR-W01</t>
         </is>
       </c>
       <c r="D185" s="3" t="inlineStr">
@@ -14601,12 +14601,12 @@
       </c>
       <c r="B186" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-MEM-08</t>
         </is>
       </c>
       <c r="C186" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>An admin cannot revoke the owner's grant (escalation); the last owner keeps the role; role preview shows added/removed/affected members; role and grant changes are on the verified audit chain | FR-W03, docs/12 §5, FR-T01</t>
         </is>
       </c>
       <c r="D186" s="3" t="inlineStr">
@@ -14628,12 +14628,12 @@
       </c>
       <c r="B187" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
         </is>
       </c>
       <c r="D187" s="3" t="inlineStr">
@@ -14655,12 +14655,12 @@
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D188" s="3" t="inlineStr">
@@ -14682,12 +14682,12 @@
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D189" s="3" t="inlineStr">
@@ -14709,12 +14709,12 @@
       </c>
       <c r="B190" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C190" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
         </is>
       </c>
       <c r="D190" s="3" t="inlineStr">
@@ -14736,12 +14736,12 @@
       </c>
       <c r="B191" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
         </is>
       </c>
       <c r="D191" s="3" t="inlineStr">
@@ -14763,12 +14763,12 @@
       </c>
       <c r="B192" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C192" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D192" s="3" t="inlineStr">
@@ -14790,12 +14790,12 @@
       </c>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D193" s="3" t="inlineStr">
@@ -14817,12 +14817,12 @@
       </c>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C194" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
         </is>
       </c>
       <c r="D194" s="3" t="inlineStr">
@@ -14844,12 +14844,12 @@
       </c>
       <c r="B195" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D195" s="3" t="inlineStr">
@@ -14871,12 +14871,12 @@
       </c>
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C196" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D196" s="3" t="inlineStr">
@@ -14898,12 +14898,12 @@
       </c>
       <c r="B197" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D197" s="3" t="inlineStr">
@@ -14925,12 +14925,12 @@
       </c>
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C198" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D198" s="3" t="inlineStr">
@@ -14952,12 +14952,12 @@
       </c>
       <c r="B199" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
         </is>
       </c>
       <c r="D199" s="3" t="inlineStr">
@@ -14979,12 +14979,12 @@
       </c>
       <c r="B200" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C200" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
         </is>
       </c>
       <c r="D200" s="3" t="inlineStr">
@@ -15006,12 +15006,12 @@
       </c>
       <c r="B201" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
         </is>
       </c>
       <c r="D201" s="3" t="inlineStr">
@@ -15033,12 +15033,12 @@
       </c>
       <c r="B202" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C202" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D202" s="3" t="inlineStr">
@@ -15060,12 +15060,12 @@
       </c>
       <c r="B203" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
         </is>
       </c>
       <c r="D203" s="3" t="inlineStr">
@@ -15087,12 +15087,12 @@
       </c>
       <c r="B204" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C204" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
         </is>
       </c>
       <c r="D204" s="3" t="inlineStr">
@@ -15114,12 +15114,12 @@
       </c>
       <c r="B205" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C205" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D205" s="3" t="inlineStr">
@@ -15141,12 +15141,12 @@
       </c>
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
         </is>
       </c>
       <c r="D206" s="3" t="inlineStr">
@@ -15168,12 +15168,12 @@
       </c>
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D207" s="3" t="inlineStr">
@@ -15195,12 +15195,12 @@
       </c>
       <c r="B208" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D208" s="3" t="inlineStr">
@@ -15222,12 +15222,12 @@
       </c>
       <c r="B209" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D209" s="3" t="inlineStr">
@@ -15249,12 +15249,12 @@
       </c>
       <c r="B210" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D210" s="3" t="inlineStr">
@@ -15276,12 +15276,12 @@
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D211" s="3" t="inlineStr">
@@ -15303,12 +15303,12 @@
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D212" s="3" t="inlineStr">
@@ -15330,12 +15330,12 @@
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D213" s="3" t="inlineStr">
@@ -15357,12 +15357,12 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D214" s="3" t="inlineStr">
@@ -15384,12 +15384,12 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D215" s="3" t="inlineStr">
@@ -15411,12 +15411,12 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
@@ -15438,12 +15438,12 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -15465,12 +15465,12 @@
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
@@ -15492,12 +15492,12 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D219" s="3" t="inlineStr">
@@ -15519,12 +15519,12 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D220" s="3" t="inlineStr">
@@ -15546,12 +15546,12 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D221" s="3" t="inlineStr">
@@ -15573,12 +15573,12 @@
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D222" s="3" t="inlineStr">
@@ -15600,12 +15600,12 @@
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D223" s="3" t="inlineStr">
@@ -15627,12 +15627,12 @@
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D224" s="3" t="inlineStr">
@@ -15654,12 +15654,12 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D225" s="3" t="inlineStr">
@@ -15681,12 +15681,12 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D226" s="3" t="inlineStr">
@@ -15708,12 +15708,12 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D227" s="3" t="inlineStr">
@@ -15735,12 +15735,12 @@
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D228" s="3" t="inlineStr">
@@ -15762,12 +15762,12 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
@@ -15789,12 +15789,12 @@
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D230" s="3" t="inlineStr">
@@ -15816,12 +15816,12 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D231" s="3" t="inlineStr">
@@ -15843,12 +15843,12 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D232" s="3" t="inlineStr">
@@ -15870,12 +15870,12 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D233" s="3" t="inlineStr">
@@ -15897,12 +15897,12 @@
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D234" s="3" t="inlineStr">
@@ -15924,12 +15924,12 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D235" s="3" t="inlineStr">
@@ -15951,12 +15951,12 @@
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D236" s="3" t="inlineStr">
@@ -15978,12 +15978,12 @@
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D237" s="3" t="inlineStr">
@@ -16005,12 +16005,12 @@
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D238" s="3" t="inlineStr">
@@ -16032,12 +16032,12 @@
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D239" s="3" t="inlineStr">
@@ -16059,12 +16059,12 @@
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D240" s="3" t="inlineStr">
@@ -16086,12 +16086,12 @@
       </c>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D241" s="3" t="inlineStr">
@@ -16113,12 +16113,12 @@
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D242" s="3" t="inlineStr">
@@ -16140,12 +16140,12 @@
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D243" s="3" t="inlineStr">
@@ -16167,12 +16167,12 @@
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D244" s="3" t="inlineStr">
@@ -16194,12 +16194,12 @@
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D245" s="3" t="inlineStr">
@@ -16221,12 +16221,12 @@
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D246" s="3" t="inlineStr">
@@ -16248,12 +16248,12 @@
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D247" s="3" t="inlineStr">
@@ -16275,12 +16275,12 @@
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-11</t>
         </is>
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
@@ -16302,12 +16302,12 @@
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R4-ISO</t>
         </is>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
         </is>
       </c>
       <c r="D249" s="3" t="inlineStr">
@@ -16329,12 +16329,12 @@
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R5-01</t>
         </is>
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
         </is>
       </c>
       <c r="D250" s="3" t="inlineStr">
@@ -16356,12 +16356,12 @@
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R5-02</t>
         </is>
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
         </is>
       </c>
       <c r="D251" s="3" t="inlineStr">
@@ -16383,12 +16383,12 @@
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R5-03</t>
         </is>
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
         </is>
       </c>
       <c r="D252" s="3" t="inlineStr">
@@ -16410,12 +16410,12 @@
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R5-04</t>
         </is>
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
         </is>
       </c>
       <c r="D253" s="3" t="inlineStr">
@@ -16437,12 +16437,12 @@
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R5-05</t>
         </is>
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
         </is>
       </c>
       <c r="D254" s="3" t="inlineStr">
@@ -16464,12 +16464,12 @@
       </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R5-06</t>
         </is>
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
         </is>
       </c>
       <c r="D255" s="3" t="inlineStr">
@@ -16491,12 +16491,12 @@
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R5-07</t>
         </is>
       </c>
       <c r="C256" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
         </is>
       </c>
       <c r="D256" s="3" t="inlineStr">
@@ -16518,12 +16518,12 @@
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R5-08</t>
         </is>
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
         </is>
       </c>
       <c r="D257" s="3" t="inlineStr">
@@ -16545,20 +16545,74 @@
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
+          <t>E2E-R5-09</t>
+        </is>
+      </c>
+      <c r="C258" s="3" t="inlineStr">
+        <is>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+        </is>
+      </c>
+      <c r="D258" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E258" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B259" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C259" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D259" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E259" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B260" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C258" s="3" t="inlineStr">
+      <c r="C260" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D258" s="3" t="inlineStr">
+      <c r="D260" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E258" s="3" t="inlineStr">
+      <c r="E260" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
test(audit): [protected] route audit contract with static route check and E2E-R1-AUD-01 (BPMS-026)
Every mutating route declares the audit actions a successful call appends,
or a written exemption. A unit test parses the router sources and fails on
a mutating route without an entry. E2E-R1-AUD-01 calls every route and
compares the appended events (attributed by User-Agent) with the contract.
Closes audit gaps for TOTP enrolment start and workspace selection.
docs/24 §3.5 now describes the declared-event-set rule.

Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E260" headerRowCount="1">
-  <autoFilter ref="A1:E260"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E261" headerRowCount="1">
+  <autoFilter ref="A1:E261"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -4226,7 +4226,7 @@
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L22" s="3" t="inlineStr"/>
@@ -4234,7 +4234,7 @@
       <c r="N22" s="3" t="inlineStr"/>
       <c r="O22" s="3" t="inlineStr">
         <is>
-          <t>procera-audit: JCS/SHA-256 per-workspace chain in the business tx, batched sealer, verifier, monthly partitions with forced RLS, append-only grants + trigger; tamper test passes. Remaining: route audit-coverage contract test (with BPMS-020 routes)</t>
+          <t>procera-audit: JCS/SHA-256 per-workspace chain in the business tx, batched sealer, verifier, monthly partitions with forced RLS, append-only grants + trigger; tamper test. Route audit contract (audit_contract.rs): a unit test fails on any mutating route without an entry; E2E-R1-AUD-01 checks every route's appended events against it. Gaps closed: TOTP enrolment start, workspace selection, role/grant changes. data_access events follow with restricted data (BPMS-040+)</t>
         </is>
       </c>
     </row>
@@ -9588,7 +9588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E260"/>
+  <dimension ref="A1:E261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14628,12 +14628,12 @@
       </c>
       <c r="B187" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-AUD-01</t>
         </is>
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>Every mutating route is called once and appends exactly the audit actions in its route contract (`/__test/audit/contract`); exempt routes append nothing; no route goes unexercised (bootstrap is one-shot and checked by the platform integration test) | FR-T01, docs/24 §3.5</t>
         </is>
       </c>
       <c r="D187" s="3" t="inlineStr">
@@ -14655,12 +14655,12 @@
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
         </is>
       </c>
       <c r="D188" s="3" t="inlineStr">
@@ -14682,12 +14682,12 @@
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D189" s="3" t="inlineStr">
@@ -14709,12 +14709,12 @@
       </c>
       <c r="B190" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C190" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D190" s="3" t="inlineStr">
@@ -14736,12 +14736,12 @@
       </c>
       <c r="B191" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
         </is>
       </c>
       <c r="D191" s="3" t="inlineStr">
@@ -14763,12 +14763,12 @@
       </c>
       <c r="B192" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C192" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
         </is>
       </c>
       <c r="D192" s="3" t="inlineStr">
@@ -14790,12 +14790,12 @@
       </c>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D193" s="3" t="inlineStr">
@@ -14817,12 +14817,12 @@
       </c>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C194" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D194" s="3" t="inlineStr">
@@ -14844,12 +14844,12 @@
       </c>
       <c r="B195" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
         </is>
       </c>
       <c r="D195" s="3" t="inlineStr">
@@ -14871,12 +14871,12 @@
       </c>
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C196" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D196" s="3" t="inlineStr">
@@ -14898,12 +14898,12 @@
       </c>
       <c r="B197" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D197" s="3" t="inlineStr">
@@ -14925,12 +14925,12 @@
       </c>
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C198" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D198" s="3" t="inlineStr">
@@ -14952,12 +14952,12 @@
       </c>
       <c r="B199" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D199" s="3" t="inlineStr">
@@ -14979,12 +14979,12 @@
       </c>
       <c r="B200" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C200" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
         </is>
       </c>
       <c r="D200" s="3" t="inlineStr">
@@ -15006,12 +15006,12 @@
       </c>
       <c r="B201" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
         </is>
       </c>
       <c r="D201" s="3" t="inlineStr">
@@ -15033,12 +15033,12 @@
       </c>
       <c r="B202" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C202" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
         </is>
       </c>
       <c r="D202" s="3" t="inlineStr">
@@ -15060,12 +15060,12 @@
       </c>
       <c r="B203" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D203" s="3" t="inlineStr">
@@ -15087,12 +15087,12 @@
       </c>
       <c r="B204" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C204" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
         </is>
       </c>
       <c r="D204" s="3" t="inlineStr">
@@ -15114,12 +15114,12 @@
       </c>
       <c r="B205" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C205" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
         </is>
       </c>
       <c r="D205" s="3" t="inlineStr">
@@ -15141,12 +15141,12 @@
       </c>
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D206" s="3" t="inlineStr">
@@ -15168,12 +15168,12 @@
       </c>
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
         </is>
       </c>
       <c r="D207" s="3" t="inlineStr">
@@ -15195,12 +15195,12 @@
       </c>
       <c r="B208" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D208" s="3" t="inlineStr">
@@ -15222,12 +15222,12 @@
       </c>
       <c r="B209" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D209" s="3" t="inlineStr">
@@ -15249,12 +15249,12 @@
       </c>
       <c r="B210" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D210" s="3" t="inlineStr">
@@ -15276,12 +15276,12 @@
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D211" s="3" t="inlineStr">
@@ -15303,12 +15303,12 @@
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D212" s="3" t="inlineStr">
@@ -15330,12 +15330,12 @@
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D213" s="3" t="inlineStr">
@@ -15357,12 +15357,12 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D214" s="3" t="inlineStr">
@@ -15384,12 +15384,12 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D215" s="3" t="inlineStr">
@@ -15411,12 +15411,12 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
@@ -15438,12 +15438,12 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -15465,12 +15465,12 @@
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
@@ -15492,12 +15492,12 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D219" s="3" t="inlineStr">
@@ -15519,12 +15519,12 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D220" s="3" t="inlineStr">
@@ -15546,12 +15546,12 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D221" s="3" t="inlineStr">
@@ -15573,12 +15573,12 @@
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D222" s="3" t="inlineStr">
@@ -15600,12 +15600,12 @@
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D223" s="3" t="inlineStr">
@@ -15627,12 +15627,12 @@
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D224" s="3" t="inlineStr">
@@ -15654,12 +15654,12 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D225" s="3" t="inlineStr">
@@ -15681,12 +15681,12 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D226" s="3" t="inlineStr">
@@ -15708,12 +15708,12 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D227" s="3" t="inlineStr">
@@ -15735,12 +15735,12 @@
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D228" s="3" t="inlineStr">
@@ -15762,12 +15762,12 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
@@ -15789,12 +15789,12 @@
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D230" s="3" t="inlineStr">
@@ -15816,12 +15816,12 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D231" s="3" t="inlineStr">
@@ -15843,12 +15843,12 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D232" s="3" t="inlineStr">
@@ -15870,12 +15870,12 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D233" s="3" t="inlineStr">
@@ -15897,12 +15897,12 @@
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D234" s="3" t="inlineStr">
@@ -15924,12 +15924,12 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D235" s="3" t="inlineStr">
@@ -15951,12 +15951,12 @@
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D236" s="3" t="inlineStr">
@@ -15978,12 +15978,12 @@
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D237" s="3" t="inlineStr">
@@ -16005,12 +16005,12 @@
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D238" s="3" t="inlineStr">
@@ -16032,12 +16032,12 @@
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D239" s="3" t="inlineStr">
@@ -16059,12 +16059,12 @@
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D240" s="3" t="inlineStr">
@@ -16086,12 +16086,12 @@
       </c>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D241" s="3" t="inlineStr">
@@ -16113,12 +16113,12 @@
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D242" s="3" t="inlineStr">
@@ -16140,12 +16140,12 @@
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D243" s="3" t="inlineStr">
@@ -16167,12 +16167,12 @@
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D244" s="3" t="inlineStr">
@@ -16194,12 +16194,12 @@
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D245" s="3" t="inlineStr">
@@ -16221,12 +16221,12 @@
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D246" s="3" t="inlineStr">
@@ -16248,12 +16248,12 @@
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D247" s="3" t="inlineStr">
@@ -16275,12 +16275,12 @@
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
@@ -16302,12 +16302,12 @@
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R4-11</t>
         </is>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
         </is>
       </c>
       <c r="D249" s="3" t="inlineStr">
@@ -16329,12 +16329,12 @@
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-ISO</t>
         </is>
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
         </is>
       </c>
       <c r="D250" s="3" t="inlineStr">
@@ -16356,12 +16356,12 @@
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R5-01</t>
         </is>
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
         </is>
       </c>
       <c r="D251" s="3" t="inlineStr">
@@ -16383,12 +16383,12 @@
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R5-02</t>
         </is>
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
         </is>
       </c>
       <c r="D252" s="3" t="inlineStr">
@@ -16410,12 +16410,12 @@
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R5-03</t>
         </is>
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
         </is>
       </c>
       <c r="D253" s="3" t="inlineStr">
@@ -16437,12 +16437,12 @@
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R5-04</t>
         </is>
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
         </is>
       </c>
       <c r="D254" s="3" t="inlineStr">
@@ -16464,12 +16464,12 @@
       </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R5-05</t>
         </is>
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
         </is>
       </c>
       <c r="D255" s="3" t="inlineStr">
@@ -16491,12 +16491,12 @@
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R5-06</t>
         </is>
       </c>
       <c r="C256" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
         </is>
       </c>
       <c r="D256" s="3" t="inlineStr">
@@ -16518,12 +16518,12 @@
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R5-07</t>
         </is>
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
         </is>
       </c>
       <c r="D257" s="3" t="inlineStr">
@@ -16545,12 +16545,12 @@
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R5-08</t>
         </is>
       </c>
       <c r="C258" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
         </is>
       </c>
       <c r="D258" s="3" t="inlineStr">
@@ -16572,12 +16572,12 @@
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R5-09</t>
         </is>
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
         </is>
       </c>
       <c r="D259" s="3" t="inlineStr">
@@ -16599,20 +16599,47 @@
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C260" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D260" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E260" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B261" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C260" s="3" t="inlineStr">
+      <c r="C261" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D260" s="3" t="inlineStr">
+      <c r="D261" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E260" s="3" t="inlineStr">
+      <c r="E261" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
chore(tracker): dashboard shows partial progress, test counts and recently shipped commits; BPMS-027 in progress
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -4291,13 +4291,17 @@
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L23" s="3" t="inlineStr"/>
       <c r="M23" s="3" t="inlineStr"/>
       <c r="N23" s="3" t="inlineStr"/>
-      <c r="O23" s="3" t="inlineStr"/>
+      <c r="O23" s="3" t="inlineStr">
+        <is>
+          <t>procera-settings: catalogue in code (P0 subset, 38 keys, comparators), platform floors (migration 0007), configuration profiles, effective-resolution with clamping, revision history. Wiring APIs + tests now</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(api): workspace settings and platform floor APIs, profiles at workspace creation; E2E-R1-CFG-01..05 (BPMS-027)
Workspace creation applies the chosen configuration profile. /api/v1/settings
lists effective values, explains a key, updates one key per PUT with
If-Match, and shows history; /sysapi/v1/settings reads and sets floors.
Changes are audited and in the route audit contract. docs/08 now specifies
per-key PUT; docs/20 records the as-built data model.

Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E261" headerRowCount="1">
-  <autoFilter ref="A1:E261"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E266" headerRowCount="1">
+  <autoFilter ref="A1:E266"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -4299,7 +4299,7 @@
       <c r="N23" s="3" t="inlineStr"/>
       <c r="O23" s="3" t="inlineStr">
         <is>
-          <t>procera-settings: catalogue in code (P0 subset, 38 keys, comparators), platform floors (migration 0007), configuration profiles, effective-resolution with clamping, revision history. Wiring APIs + tests now</t>
+          <t>procera-settings: catalogue in code (P0 subset, 38 keys) with comparators; platform floors + workspace values + append-only revisions (migration 0007, RLS); 4 configuration profiles applied at workspace creation; resolution with clamping when a floor is raised; explainer; /api/v1/settings (list, explainer, PUT per key with If-Match, history) and /sysapi/v1/settings floors; reasons for ⚡ keys, step-up = MFA session (interim); audited (setting.changed, platform.floor_changed); property test (512 cases, never looser than floor); E2E-R1-CFG-01..05. Remaining: department/collection overrides (needs directory), profile switch plan/apply (CFG-017), settings cache invalidation (CFG-004)</t>
         </is>
       </c>
     </row>
@@ -9592,7 +9592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E261"/>
+  <dimension ref="A1:E266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14659,12 +14659,12 @@
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-CFG-01</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>The creation profile seeds values (Starter: 8 h idle); the explainer lists default → platform floor → profile; unknown keys 404 | FR-W04, docs/20 §0-1</t>
         </is>
       </c>
       <c r="D188" s="3" t="inlineStr">
@@ -14686,12 +14686,12 @@
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-CFG-02</t>
         </is>
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>Looser than a floor → 422 `setting_below_floor`; ⚡ keys need a reason; stricter value saved with `ETag`/`If-Match` (stale → 412); floor-locked key 403; invalid value 422; history records the change | FR-S05, FR-W06</t>
         </is>
       </c>
       <c r="D189" s="3" t="inlineStr">
@@ -14713,12 +14713,12 @@
       </c>
       <c r="B190" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-CFG-03</t>
         </is>
       </c>
       <c r="C190" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>Step-up keys (`auth.mfa.required_roles`) need an MFA-verified session | docs/20 §2.3</t>
         </is>
       </c>
       <c r="D190" s="3" t="inlineStr">
@@ -14740,12 +14740,12 @@
       </c>
       <c r="B191" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-CFG-04</t>
         </is>
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>A member without settings permissions can neither view nor change settings | docs/12 §5</t>
         </is>
       </c>
       <c r="D191" s="3" t="inlineStr">
@@ -14767,12 +14767,12 @@
       </c>
       <c r="B192" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-CFG-05</t>
         </is>
       </c>
       <c r="C192" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>Raising a platform floor clamps a looser workspace value at resolution (stored value kept, `clamped: true`); floors need a reason; keys without floors are rejected | docs/20 §1 rules 4-5</t>
         </is>
       </c>
       <c r="D192" s="3" t="inlineStr">
@@ -14794,12 +14794,12 @@
       </c>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
         </is>
       </c>
       <c r="D193" s="3" t="inlineStr">
@@ -14821,12 +14821,12 @@
       </c>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C194" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D194" s="3" t="inlineStr">
@@ -14848,12 +14848,12 @@
       </c>
       <c r="B195" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D195" s="3" t="inlineStr">
@@ -14875,12 +14875,12 @@
       </c>
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C196" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
         </is>
       </c>
       <c r="D196" s="3" t="inlineStr">
@@ -14902,12 +14902,12 @@
       </c>
       <c r="B197" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
         </is>
       </c>
       <c r="D197" s="3" t="inlineStr">
@@ -14929,12 +14929,12 @@
       </c>
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C198" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D198" s="3" t="inlineStr">
@@ -14956,12 +14956,12 @@
       </c>
       <c r="B199" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D199" s="3" t="inlineStr">
@@ -14983,12 +14983,12 @@
       </c>
       <c r="B200" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C200" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
         </is>
       </c>
       <c r="D200" s="3" t="inlineStr">
@@ -15010,12 +15010,12 @@
       </c>
       <c r="B201" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D201" s="3" t="inlineStr">
@@ -15037,12 +15037,12 @@
       </c>
       <c r="B202" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C202" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D202" s="3" t="inlineStr">
@@ -15064,12 +15064,12 @@
       </c>
       <c r="B203" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D203" s="3" t="inlineStr">
@@ -15091,12 +15091,12 @@
       </c>
       <c r="B204" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C204" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D204" s="3" t="inlineStr">
@@ -15118,12 +15118,12 @@
       </c>
       <c r="B205" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C205" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
         </is>
       </c>
       <c r="D205" s="3" t="inlineStr">
@@ -15145,12 +15145,12 @@
       </c>
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
         </is>
       </c>
       <c r="D206" s="3" t="inlineStr">
@@ -15172,12 +15172,12 @@
       </c>
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
         </is>
       </c>
       <c r="D207" s="3" t="inlineStr">
@@ -15199,12 +15199,12 @@
       </c>
       <c r="B208" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D208" s="3" t="inlineStr">
@@ -15226,12 +15226,12 @@
       </c>
       <c r="B209" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
         </is>
       </c>
       <c r="D209" s="3" t="inlineStr">
@@ -15253,12 +15253,12 @@
       </c>
       <c r="B210" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
         </is>
       </c>
       <c r="D210" s="3" t="inlineStr">
@@ -15280,12 +15280,12 @@
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D211" s="3" t="inlineStr">
@@ -15307,12 +15307,12 @@
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
         </is>
       </c>
       <c r="D212" s="3" t="inlineStr">
@@ -15334,12 +15334,12 @@
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D213" s="3" t="inlineStr">
@@ -15361,12 +15361,12 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D214" s="3" t="inlineStr">
@@ -15388,12 +15388,12 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D215" s="3" t="inlineStr">
@@ -15415,12 +15415,12 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
@@ -15442,12 +15442,12 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -15469,12 +15469,12 @@
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
@@ -15496,12 +15496,12 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D219" s="3" t="inlineStr">
@@ -15523,12 +15523,12 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D220" s="3" t="inlineStr">
@@ -15550,12 +15550,12 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D221" s="3" t="inlineStr">
@@ -15577,12 +15577,12 @@
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D222" s="3" t="inlineStr">
@@ -15604,12 +15604,12 @@
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D223" s="3" t="inlineStr">
@@ -15631,12 +15631,12 @@
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D224" s="3" t="inlineStr">
@@ -15658,12 +15658,12 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D225" s="3" t="inlineStr">
@@ -15685,12 +15685,12 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D226" s="3" t="inlineStr">
@@ -15712,12 +15712,12 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D227" s="3" t="inlineStr">
@@ -15739,12 +15739,12 @@
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D228" s="3" t="inlineStr">
@@ -15766,12 +15766,12 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
@@ -15793,12 +15793,12 @@
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D230" s="3" t="inlineStr">
@@ -15820,12 +15820,12 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D231" s="3" t="inlineStr">
@@ -15847,12 +15847,12 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D232" s="3" t="inlineStr">
@@ -15874,12 +15874,12 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D233" s="3" t="inlineStr">
@@ -15901,12 +15901,12 @@
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D234" s="3" t="inlineStr">
@@ -15928,12 +15928,12 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D235" s="3" t="inlineStr">
@@ -15955,12 +15955,12 @@
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D236" s="3" t="inlineStr">
@@ -15982,12 +15982,12 @@
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D237" s="3" t="inlineStr">
@@ -16009,12 +16009,12 @@
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D238" s="3" t="inlineStr">
@@ -16036,12 +16036,12 @@
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D239" s="3" t="inlineStr">
@@ -16063,12 +16063,12 @@
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D240" s="3" t="inlineStr">
@@ -16090,12 +16090,12 @@
       </c>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D241" s="3" t="inlineStr">
@@ -16117,12 +16117,12 @@
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D242" s="3" t="inlineStr">
@@ -16144,12 +16144,12 @@
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D243" s="3" t="inlineStr">
@@ -16171,12 +16171,12 @@
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D244" s="3" t="inlineStr">
@@ -16198,12 +16198,12 @@
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D245" s="3" t="inlineStr">
@@ -16225,12 +16225,12 @@
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D246" s="3" t="inlineStr">
@@ -16252,12 +16252,12 @@
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D247" s="3" t="inlineStr">
@@ -16279,12 +16279,12 @@
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
@@ -16306,12 +16306,12 @@
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D249" s="3" t="inlineStr">
@@ -16333,12 +16333,12 @@
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D250" s="3" t="inlineStr">
@@ -16360,12 +16360,12 @@
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D251" s="3" t="inlineStr">
@@ -16387,12 +16387,12 @@
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D252" s="3" t="inlineStr">
@@ -16414,12 +16414,12 @@
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D253" s="3" t="inlineStr">
@@ -16441,12 +16441,12 @@
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R4-11</t>
         </is>
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
         </is>
       </c>
       <c r="D254" s="3" t="inlineStr">
@@ -16468,12 +16468,12 @@
       </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R4-ISO</t>
         </is>
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
         </is>
       </c>
       <c r="D255" s="3" t="inlineStr">
@@ -16495,12 +16495,12 @@
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R5-01</t>
         </is>
       </c>
       <c r="C256" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
         </is>
       </c>
       <c r="D256" s="3" t="inlineStr">
@@ -16522,12 +16522,12 @@
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R5-02</t>
         </is>
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
         </is>
       </c>
       <c r="D257" s="3" t="inlineStr">
@@ -16549,12 +16549,12 @@
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R5-03</t>
         </is>
       </c>
       <c r="C258" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
         </is>
       </c>
       <c r="D258" s="3" t="inlineStr">
@@ -16576,12 +16576,12 @@
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R5-04</t>
         </is>
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
         </is>
       </c>
       <c r="D259" s="3" t="inlineStr">
@@ -16603,12 +16603,12 @@
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R5-05</t>
         </is>
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
         </is>
       </c>
       <c r="D260" s="3" t="inlineStr">
@@ -16630,20 +16630,155 @@
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
+          <t>E2E-R5-06</t>
+        </is>
+      </c>
+      <c r="C261" s="3" t="inlineStr">
+        <is>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+        </is>
+      </c>
+      <c r="D261" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E261" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B262" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-07</t>
+        </is>
+      </c>
+      <c r="C262" s="3" t="inlineStr">
+        <is>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+        </is>
+      </c>
+      <c r="D262" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E262" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B263" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-08</t>
+        </is>
+      </c>
+      <c r="C263" s="3" t="inlineStr">
+        <is>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+        </is>
+      </c>
+      <c r="D263" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E263" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B264" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-09</t>
+        </is>
+      </c>
+      <c r="C264" s="3" t="inlineStr">
+        <is>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+        </is>
+      </c>
+      <c r="D264" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E264" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B265" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C265" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D265" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E265" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B266" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C261" s="3" t="inlineStr">
+      <c r="C266" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D261" s="3" t="inlineStr">
+      <c r="D266" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E261" s="3" t="inlineStr">
+      <c r="E266" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
docs: directory API, E2E plan and LLD path note; tracker marks BPMS-023 done
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E266" headerRowCount="1">
-  <autoFilter ref="A1:E266"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E270" headerRowCount="1">
+  <autoFilter ref="A1:E270"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -4031,7 +4031,7 @@
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L19" s="3" t="inlineStr"/>
@@ -4039,7 +4039,7 @@
       <c r="N19" s="3" t="inlineStr"/>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>procera-members + /api/v1: memberships, invitations (hashed + sealed tokens, 7-day expiry, email-bound, single use; list, revoke, resend), register-by-invite, owner onboarding activates the provisioning workspace, workspace switch (ws-scoped JWT), member list, deactivation with last-owner/self guards, state gate (423 when suspended); audited; E2E-R1-MEM-01..03,05..07. Remaining: directory (departments/groups/positions/managers), CSV import</t>
+          <t>procera-members + /api/v1: memberships, invitations (hashed + sealed tokens, 7-day expiry, email-bound, single use; list, revoke, resend), register-by-invite, owner onboarding activates the workspace, workspace switch (ws-scoped JWT), deactivation guards, state gate (423). Directory (migration 0008): department tree (uuid[] paths, sibling-unique names, no moves under descendants), static groups, positions (behind directory.positions.enabled), manager links with cycle rejection, deterministic manager resolution (explicit → nearest department head), per-field source attribution, CSV import with plan/apply. All audited; E2E-R1-MEM-01..03,05..07, E2E-R1-DIR-01..04</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       <c r="N20" s="3" t="inlineStr"/>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>procera-access: permission catalogue + 12 role templates, custom roles (no escalation on create/edit/grant/revoke, built-ins immutable, clone lineage), scoped expiring grants compiled to Cedar, invariants (workspace isolation, active members only), last-owner protection, role change preview, per-workspace access_revisions cache; all role/grant changes audited; no-escalation property test (proptest, 64 cases vs Postgres); E2E-R1-MEM-04,08. Remaining: preview-matches-effect property test, group/directory-rule assignment (needs BPMS-023 directory)</t>
+          <t>procera-access: permission catalogue + 12 role templates, custom roles (no escalation on create/edit/grant/revoke, built-ins immutable, clone lineage), scoped expiring grants compiled to Cedar, invariants (workspace isolation, active members only), last-owner protection, role change preview, per-workspace access_revisions cache; all role/grant changes audited; no-escalation property test (proptest, 64 cases vs Postgres); E2E-R1-MEM-04,08. Remaining: preview-matches-effect property test, grants to groups/directory rules, department-subtree ancestors in Cedar resource checks</t>
         </is>
       </c>
     </row>
@@ -9592,7 +9592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E266"/>
+  <dimension ref="A1:E270"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14794,12 +14794,12 @@
       </c>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-DIR-01</t>
         </is>
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>Department tree: sibling names unique (409), moving under a descendant rejected (422 `cycle`), deleting a non-empty department refused | FR-W02</t>
         </is>
       </c>
       <c r="D193" s="3" t="inlineStr">
@@ -14821,12 +14821,12 @@
       </c>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-DIR-02</t>
         </is>
       </c>
       <c r="C194" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>Manager cycles rejected; resolution is the explicit manager, else the nearest department head that is not the member; field sources recorded | FR-W02 (deterministic resolution)</t>
         </is>
       </c>
       <c r="D194" s="3" t="inlineStr">
@@ -14848,12 +14848,12 @@
       </c>
       <c r="B195" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-DIR-03</t>
         </is>
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>Static groups (duplicate member 409); positions blocked until `directory.positions.enabled`; members read the directory but cannot change it | FR-W02, docs/20 §2.5</t>
         </is>
       </c>
       <c r="D195" s="3" t="inlineStr">
@@ -14875,12 +14875,12 @@
       </c>
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-DIR-04</t>
         </is>
       </c>
       <c r="C196" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>CSV import: `mode=plan` changes nothing; `mode=apply` creates departments by path and links managers listed later in the file; unknown members reported per row; unknown columns 422 | FR-W02</t>
         </is>
       </c>
       <c r="D196" s="3" t="inlineStr">
@@ -14902,12 +14902,12 @@
       </c>
       <c r="B197" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
         </is>
       </c>
       <c r="D197" s="3" t="inlineStr">
@@ -14929,12 +14929,12 @@
       </c>
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C198" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D198" s="3" t="inlineStr">
@@ -14956,12 +14956,12 @@
       </c>
       <c r="B199" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D199" s="3" t="inlineStr">
@@ -14983,12 +14983,12 @@
       </c>
       <c r="B200" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C200" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
         </is>
       </c>
       <c r="D200" s="3" t="inlineStr">
@@ -15010,12 +15010,12 @@
       </c>
       <c r="B201" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
         </is>
       </c>
       <c r="D201" s="3" t="inlineStr">
@@ -15037,12 +15037,12 @@
       </c>
       <c r="B202" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C202" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D202" s="3" t="inlineStr">
@@ -15064,12 +15064,12 @@
       </c>
       <c r="B203" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D203" s="3" t="inlineStr">
@@ -15091,12 +15091,12 @@
       </c>
       <c r="B204" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C204" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
         </is>
       </c>
       <c r="D204" s="3" t="inlineStr">
@@ -15118,12 +15118,12 @@
       </c>
       <c r="B205" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C205" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D205" s="3" t="inlineStr">
@@ -15145,12 +15145,12 @@
       </c>
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D206" s="3" t="inlineStr">
@@ -15172,12 +15172,12 @@
       </c>
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D207" s="3" t="inlineStr">
@@ -15199,12 +15199,12 @@
       </c>
       <c r="B208" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D208" s="3" t="inlineStr">
@@ -15226,12 +15226,12 @@
       </c>
       <c r="B209" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
         </is>
       </c>
       <c r="D209" s="3" t="inlineStr">
@@ -15253,12 +15253,12 @@
       </c>
       <c r="B210" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
         </is>
       </c>
       <c r="D210" s="3" t="inlineStr">
@@ -15280,12 +15280,12 @@
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
         </is>
       </c>
       <c r="D211" s="3" t="inlineStr">
@@ -15307,12 +15307,12 @@
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D212" s="3" t="inlineStr">
@@ -15334,12 +15334,12 @@
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
         </is>
       </c>
       <c r="D213" s="3" t="inlineStr">
@@ -15361,12 +15361,12 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
         </is>
       </c>
       <c r="D214" s="3" t="inlineStr">
@@ -15388,12 +15388,12 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D215" s="3" t="inlineStr">
@@ -15415,12 +15415,12 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
@@ -15442,12 +15442,12 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -15469,12 +15469,12 @@
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
@@ -15496,12 +15496,12 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D219" s="3" t="inlineStr">
@@ -15523,12 +15523,12 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D220" s="3" t="inlineStr">
@@ -15550,12 +15550,12 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D221" s="3" t="inlineStr">
@@ -15577,12 +15577,12 @@
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D222" s="3" t="inlineStr">
@@ -15604,12 +15604,12 @@
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D223" s="3" t="inlineStr">
@@ -15631,12 +15631,12 @@
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D224" s="3" t="inlineStr">
@@ -15658,12 +15658,12 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D225" s="3" t="inlineStr">
@@ -15685,12 +15685,12 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D226" s="3" t="inlineStr">
@@ -15712,12 +15712,12 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D227" s="3" t="inlineStr">
@@ -15739,12 +15739,12 @@
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D228" s="3" t="inlineStr">
@@ -15766,12 +15766,12 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
@@ -15793,12 +15793,12 @@
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D230" s="3" t="inlineStr">
@@ -15820,12 +15820,12 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D231" s="3" t="inlineStr">
@@ -15847,12 +15847,12 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D232" s="3" t="inlineStr">
@@ -15874,12 +15874,12 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D233" s="3" t="inlineStr">
@@ -15901,12 +15901,12 @@
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D234" s="3" t="inlineStr">
@@ -15928,12 +15928,12 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D235" s="3" t="inlineStr">
@@ -15955,12 +15955,12 @@
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D236" s="3" t="inlineStr">
@@ -15982,12 +15982,12 @@
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D237" s="3" t="inlineStr">
@@ -16009,12 +16009,12 @@
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D238" s="3" t="inlineStr">
@@ -16036,12 +16036,12 @@
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D239" s="3" t="inlineStr">
@@ -16063,12 +16063,12 @@
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D240" s="3" t="inlineStr">
@@ -16090,12 +16090,12 @@
       </c>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D241" s="3" t="inlineStr">
@@ -16117,12 +16117,12 @@
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D242" s="3" t="inlineStr">
@@ -16144,12 +16144,12 @@
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D243" s="3" t="inlineStr">
@@ -16171,12 +16171,12 @@
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D244" s="3" t="inlineStr">
@@ -16198,12 +16198,12 @@
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D245" s="3" t="inlineStr">
@@ -16225,12 +16225,12 @@
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D246" s="3" t="inlineStr">
@@ -16252,12 +16252,12 @@
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D247" s="3" t="inlineStr">
@@ -16279,12 +16279,12 @@
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
@@ -16306,12 +16306,12 @@
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D249" s="3" t="inlineStr">
@@ -16333,12 +16333,12 @@
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D250" s="3" t="inlineStr">
@@ -16360,12 +16360,12 @@
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D251" s="3" t="inlineStr">
@@ -16387,12 +16387,12 @@
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D252" s="3" t="inlineStr">
@@ -16414,12 +16414,12 @@
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D253" s="3" t="inlineStr">
@@ -16441,12 +16441,12 @@
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D254" s="3" t="inlineStr">
@@ -16468,12 +16468,12 @@
       </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D255" s="3" t="inlineStr">
@@ -16495,12 +16495,12 @@
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C256" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D256" s="3" t="inlineStr">
@@ -16522,12 +16522,12 @@
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D257" s="3" t="inlineStr">
@@ -16549,12 +16549,12 @@
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R4-11</t>
         </is>
       </c>
       <c r="C258" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
         </is>
       </c>
       <c r="D258" s="3" t="inlineStr">
@@ -16576,12 +16576,12 @@
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R4-ISO</t>
         </is>
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
         </is>
       </c>
       <c r="D259" s="3" t="inlineStr">
@@ -16603,12 +16603,12 @@
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R5-01</t>
         </is>
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
         </is>
       </c>
       <c r="D260" s="3" t="inlineStr">
@@ -16630,12 +16630,12 @@
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R5-02</t>
         </is>
       </c>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
         </is>
       </c>
       <c r="D261" s="3" t="inlineStr">
@@ -16657,12 +16657,12 @@
       </c>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R5-03</t>
         </is>
       </c>
       <c r="C262" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
         </is>
       </c>
       <c r="D262" s="3" t="inlineStr">
@@ -16684,12 +16684,12 @@
       </c>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R5-04</t>
         </is>
       </c>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
         </is>
       </c>
       <c r="D263" s="3" t="inlineStr">
@@ -16711,12 +16711,12 @@
       </c>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R5-05</t>
         </is>
       </c>
       <c r="C264" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
         </is>
       </c>
       <c r="D264" s="3" t="inlineStr">
@@ -16738,12 +16738,12 @@
       </c>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R5-06</t>
         </is>
       </c>
       <c r="C265" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
         </is>
       </c>
       <c r="D265" s="3" t="inlineStr">
@@ -16765,20 +16765,128 @@
       </c>
       <c r="B266" s="3" t="inlineStr">
         <is>
+          <t>E2E-R5-07</t>
+        </is>
+      </c>
+      <c r="C266" s="3" t="inlineStr">
+        <is>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+        </is>
+      </c>
+      <c r="D266" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E266" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B267" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-08</t>
+        </is>
+      </c>
+      <c r="C267" s="3" t="inlineStr">
+        <is>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+        </is>
+      </c>
+      <c r="D267" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E267" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B268" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-09</t>
+        </is>
+      </c>
+      <c r="C268" s="3" t="inlineStr">
+        <is>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+        </is>
+      </c>
+      <c r="D268" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E268" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B269" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C269" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D269" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E269" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B270" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C266" s="3" t="inlineStr">
+      <c r="C270" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D266" s="3" t="inlineStr">
+      <c r="D270" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E266" s="3" t="inlineStr">
+      <c r="E270" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
docs: E2E-R1-MEM-09; tracker marks BPMS-024 done
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E270" headerRowCount="1">
-  <autoFilter ref="A1:E270"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E271" headerRowCount="1">
+  <autoFilter ref="A1:E271"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -4096,7 +4096,7 @@
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L20" s="3" t="inlineStr"/>
@@ -4104,7 +4104,7 @@
       <c r="N20" s="3" t="inlineStr"/>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>procera-access: permission catalogue + 12 role templates, custom roles (no escalation on create/edit/grant/revoke, built-ins immutable, clone lineage), scoped expiring grants compiled to Cedar, invariants (workspace isolation, active members only), last-owner protection, role change preview, per-workspace access_revisions cache; all role/grant changes audited; no-escalation property test (proptest, 64 cases vs Postgres); E2E-R1-MEM-04,08. Remaining: preview-matches-effect property test, grants to groups/directory rules, department-subtree ancestors in Cedar resource checks</t>
+          <t>procera-access: permission catalogue + 12 role templates; custom roles (no escalation on create/edit/grant/revoke, built-ins immutable, clone lineage); grants to members or static groups (migration 0009), scoped (workspace/department/collection/process/case) with expiry, compiled to Cedar; members inherit their department subtree so department-scoped admins reach only it; invariants (workspace isolation, active members only); last-owner protection; role change preview; access_revisions cache; all changes audited. Property tests: no escalation (64 cases) and preview matches effect (48 cases), both against Postgres. E2E-R1-MEM-04,08,09</t>
         </is>
       </c>
     </row>
@@ -9592,7 +9592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E270"/>
+  <dimension ref="A1:E271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14632,12 +14632,12 @@
       </c>
       <c r="B187" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUD-01</t>
+          <t>E2E-R1-MEM-09</t>
         </is>
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>Every mutating route is called once and appends exactly the audit actions in its route contract (`/__test/audit/contract`); exempt routes append nothing; no route goes unexercised (bootstrap is one-shot and checked by the platform integration test) | FR-T01, docs/24 §3.5</t>
+          <t>A role granted to a group applies while the member is in it and stops when removed; owner role cannot go to groups; a department-scoped admin reaches members in the subtree only | docs/12 §5, FR-W03</t>
         </is>
       </c>
       <c r="D187" s="3" t="inlineStr">
@@ -14659,12 +14659,12 @@
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CFG-01</t>
+          <t>E2E-R1-AUD-01</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
         <is>
-          <t>The creation profile seeds values (Starter: 8 h idle); the explainer lists default → platform floor → profile; unknown keys 404 | FR-W04, docs/20 §0-1</t>
+          <t>Every mutating route is called once and appends exactly the audit actions in its route contract (`/__test/audit/contract`); exempt routes append nothing; no route goes unexercised (bootstrap is one-shot and checked by the platform integration test) | FR-T01, docs/24 §3.5</t>
         </is>
       </c>
       <c r="D188" s="3" t="inlineStr">
@@ -14686,12 +14686,12 @@
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CFG-02</t>
+          <t>E2E-R1-CFG-01</t>
         </is>
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>Looser than a floor → 422 `setting_below_floor`; ⚡ keys need a reason; stricter value saved with `ETag`/`If-Match` (stale → 412); floor-locked key 403; invalid value 422; history records the change | FR-S05, FR-W06</t>
+          <t>The creation profile seeds values (Starter: 8 h idle); the explainer lists default → platform floor → profile; unknown keys 404 | FR-W04, docs/20 §0-1</t>
         </is>
       </c>
       <c r="D189" s="3" t="inlineStr">
@@ -14713,12 +14713,12 @@
       </c>
       <c r="B190" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CFG-03</t>
+          <t>E2E-R1-CFG-02</t>
         </is>
       </c>
       <c r="C190" s="3" t="inlineStr">
         <is>
-          <t>Step-up keys (`auth.mfa.required_roles`) need an MFA-verified session | docs/20 §2.3</t>
+          <t>Looser than a floor → 422 `setting_below_floor`; ⚡ keys need a reason; stricter value saved with `ETag`/`If-Match` (stale → 412); floor-locked key 403; invalid value 422; history records the change | FR-S05, FR-W06</t>
         </is>
       </c>
       <c r="D190" s="3" t="inlineStr">
@@ -14740,12 +14740,12 @@
       </c>
       <c r="B191" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CFG-04</t>
+          <t>E2E-R1-CFG-03</t>
         </is>
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>A member without settings permissions can neither view nor change settings | docs/12 §5</t>
+          <t>Step-up keys (`auth.mfa.required_roles`) need an MFA-verified session | docs/20 §2.3</t>
         </is>
       </c>
       <c r="D191" s="3" t="inlineStr">
@@ -14767,12 +14767,12 @@
       </c>
       <c r="B192" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CFG-05</t>
+          <t>E2E-R1-CFG-04</t>
         </is>
       </c>
       <c r="C192" s="3" t="inlineStr">
         <is>
-          <t>Raising a platform floor clamps a looser workspace value at resolution (stored value kept, `clamped: true`); floors need a reason; keys without floors are rejected | docs/20 §1 rules 4-5</t>
+          <t>A member without settings permissions can neither view nor change settings | docs/12 §5</t>
         </is>
       </c>
       <c r="D192" s="3" t="inlineStr">
@@ -14794,12 +14794,12 @@
       </c>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-DIR-01</t>
+          <t>E2E-R1-CFG-05</t>
         </is>
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>Department tree: sibling names unique (409), moving under a descendant rejected (422 `cycle`), deleting a non-empty department refused | FR-W02</t>
+          <t>Raising a platform floor clamps a looser workspace value at resolution (stored value kept, `clamped: true`); floors need a reason; keys without floors are rejected | docs/20 §1 rules 4-5</t>
         </is>
       </c>
       <c r="D193" s="3" t="inlineStr">
@@ -14821,12 +14821,12 @@
       </c>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-DIR-02</t>
+          <t>E2E-R1-DIR-01</t>
         </is>
       </c>
       <c r="C194" s="3" t="inlineStr">
         <is>
-          <t>Manager cycles rejected; resolution is the explicit manager, else the nearest department head that is not the member; field sources recorded | FR-W02 (deterministic resolution)</t>
+          <t>Department tree: sibling names unique (409), moving under a descendant rejected (422 `cycle`), deleting a non-empty department refused | FR-W02</t>
         </is>
       </c>
       <c r="D194" s="3" t="inlineStr">
@@ -14848,12 +14848,12 @@
       </c>
       <c r="B195" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-DIR-03</t>
+          <t>E2E-R1-DIR-02</t>
         </is>
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>Static groups (duplicate member 409); positions blocked until `directory.positions.enabled`; members read the directory but cannot change it | FR-W02, docs/20 §2.5</t>
+          <t>Manager cycles rejected; resolution is the explicit manager, else the nearest department head that is not the member; field sources recorded | FR-W02 (deterministic resolution)</t>
         </is>
       </c>
       <c r="D195" s="3" t="inlineStr">
@@ -14875,12 +14875,12 @@
       </c>
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-DIR-04</t>
+          <t>E2E-R1-DIR-03</t>
         </is>
       </c>
       <c r="C196" s="3" t="inlineStr">
         <is>
-          <t>CSV import: `mode=plan` changes nothing; `mode=apply` creates departments by path and links managers listed later in the file; unknown members reported per row; unknown columns 422 | FR-W02</t>
+          <t>Static groups (duplicate member 409); positions blocked until `directory.positions.enabled`; members read the directory but cannot change it | FR-W02, docs/20 §2.5</t>
         </is>
       </c>
       <c r="D196" s="3" t="inlineStr">
@@ -14902,12 +14902,12 @@
       </c>
       <c r="B197" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-DIR-04</t>
         </is>
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>CSV import: `mode=plan` changes nothing; `mode=apply` creates departments by path and links managers listed later in the file; unknown members reported per row; unknown columns 422 | FR-W02</t>
         </is>
       </c>
       <c r="D197" s="3" t="inlineStr">
@@ -14929,12 +14929,12 @@
       </c>
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C198" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
         </is>
       </c>
       <c r="D198" s="3" t="inlineStr">
@@ -14956,12 +14956,12 @@
       </c>
       <c r="B199" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D199" s="3" t="inlineStr">
@@ -14983,12 +14983,12 @@
       </c>
       <c r="B200" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C200" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D200" s="3" t="inlineStr">
@@ -15010,12 +15010,12 @@
       </c>
       <c r="B201" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
         </is>
       </c>
       <c r="D201" s="3" t="inlineStr">
@@ -15037,12 +15037,12 @@
       </c>
       <c r="B202" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C202" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
         </is>
       </c>
       <c r="D202" s="3" t="inlineStr">
@@ -15064,12 +15064,12 @@
       </c>
       <c r="B203" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D203" s="3" t="inlineStr">
@@ -15091,12 +15091,12 @@
       </c>
       <c r="B204" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C204" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D204" s="3" t="inlineStr">
@@ -15118,12 +15118,12 @@
       </c>
       <c r="B205" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C205" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
         </is>
       </c>
       <c r="D205" s="3" t="inlineStr">
@@ -15145,12 +15145,12 @@
       </c>
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D206" s="3" t="inlineStr">
@@ -15172,12 +15172,12 @@
       </c>
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D207" s="3" t="inlineStr">
@@ -15199,12 +15199,12 @@
       </c>
       <c r="B208" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D208" s="3" t="inlineStr">
@@ -15226,12 +15226,12 @@
       </c>
       <c r="B209" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D209" s="3" t="inlineStr">
@@ -15253,12 +15253,12 @@
       </c>
       <c r="B210" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
         </is>
       </c>
       <c r="D210" s="3" t="inlineStr">
@@ -15280,12 +15280,12 @@
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
         </is>
       </c>
       <c r="D211" s="3" t="inlineStr">
@@ -15307,12 +15307,12 @@
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
         </is>
       </c>
       <c r="D212" s="3" t="inlineStr">
@@ -15334,12 +15334,12 @@
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D213" s="3" t="inlineStr">
@@ -15361,12 +15361,12 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
         </is>
       </c>
       <c r="D214" s="3" t="inlineStr">
@@ -15388,12 +15388,12 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
         </is>
       </c>
       <c r="D215" s="3" t="inlineStr">
@@ -15415,12 +15415,12 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
@@ -15442,12 +15442,12 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -15469,12 +15469,12 @@
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
@@ -15496,12 +15496,12 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D219" s="3" t="inlineStr">
@@ -15523,12 +15523,12 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D220" s="3" t="inlineStr">
@@ -15550,12 +15550,12 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D221" s="3" t="inlineStr">
@@ -15577,12 +15577,12 @@
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D222" s="3" t="inlineStr">
@@ -15604,12 +15604,12 @@
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D223" s="3" t="inlineStr">
@@ -15631,12 +15631,12 @@
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D224" s="3" t="inlineStr">
@@ -15658,12 +15658,12 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D225" s="3" t="inlineStr">
@@ -15685,12 +15685,12 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D226" s="3" t="inlineStr">
@@ -15712,12 +15712,12 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D227" s="3" t="inlineStr">
@@ -15739,12 +15739,12 @@
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D228" s="3" t="inlineStr">
@@ -15766,12 +15766,12 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
@@ -15793,12 +15793,12 @@
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D230" s="3" t="inlineStr">
@@ -15820,12 +15820,12 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D231" s="3" t="inlineStr">
@@ -15847,12 +15847,12 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D232" s="3" t="inlineStr">
@@ -15874,12 +15874,12 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D233" s="3" t="inlineStr">
@@ -15901,12 +15901,12 @@
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D234" s="3" t="inlineStr">
@@ -15928,12 +15928,12 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D235" s="3" t="inlineStr">
@@ -15955,12 +15955,12 @@
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D236" s="3" t="inlineStr">
@@ -15982,12 +15982,12 @@
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D237" s="3" t="inlineStr">
@@ -16009,12 +16009,12 @@
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D238" s="3" t="inlineStr">
@@ -16036,12 +16036,12 @@
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D239" s="3" t="inlineStr">
@@ -16063,12 +16063,12 @@
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D240" s="3" t="inlineStr">
@@ -16090,12 +16090,12 @@
       </c>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D241" s="3" t="inlineStr">
@@ -16117,12 +16117,12 @@
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D242" s="3" t="inlineStr">
@@ -16144,12 +16144,12 @@
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D243" s="3" t="inlineStr">
@@ -16171,12 +16171,12 @@
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D244" s="3" t="inlineStr">
@@ -16198,12 +16198,12 @@
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D245" s="3" t="inlineStr">
@@ -16225,12 +16225,12 @@
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D246" s="3" t="inlineStr">
@@ -16252,12 +16252,12 @@
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D247" s="3" t="inlineStr">
@@ -16279,12 +16279,12 @@
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
@@ -16306,12 +16306,12 @@
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D249" s="3" t="inlineStr">
@@ -16333,12 +16333,12 @@
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D250" s="3" t="inlineStr">
@@ -16360,12 +16360,12 @@
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D251" s="3" t="inlineStr">
@@ -16387,12 +16387,12 @@
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D252" s="3" t="inlineStr">
@@ -16414,12 +16414,12 @@
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D253" s="3" t="inlineStr">
@@ -16441,12 +16441,12 @@
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D254" s="3" t="inlineStr">
@@ -16468,12 +16468,12 @@
       </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D255" s="3" t="inlineStr">
@@ -16495,12 +16495,12 @@
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C256" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D256" s="3" t="inlineStr">
@@ -16522,12 +16522,12 @@
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D257" s="3" t="inlineStr">
@@ -16549,12 +16549,12 @@
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C258" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D258" s="3" t="inlineStr">
@@ -16576,12 +16576,12 @@
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R4-11</t>
         </is>
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
         </is>
       </c>
       <c r="D259" s="3" t="inlineStr">
@@ -16603,12 +16603,12 @@
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-ISO</t>
         </is>
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
         </is>
       </c>
       <c r="D260" s="3" t="inlineStr">
@@ -16630,12 +16630,12 @@
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R5-01</t>
         </is>
       </c>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
         </is>
       </c>
       <c r="D261" s="3" t="inlineStr">
@@ -16657,12 +16657,12 @@
       </c>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R5-02</t>
         </is>
       </c>
       <c r="C262" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
         </is>
       </c>
       <c r="D262" s="3" t="inlineStr">
@@ -16684,12 +16684,12 @@
       </c>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R5-03</t>
         </is>
       </c>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
         </is>
       </c>
       <c r="D263" s="3" t="inlineStr">
@@ -16711,12 +16711,12 @@
       </c>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R5-04</t>
         </is>
       </c>
       <c r="C264" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
         </is>
       </c>
       <c r="D264" s="3" t="inlineStr">
@@ -16738,12 +16738,12 @@
       </c>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R5-05</t>
         </is>
       </c>
       <c r="C265" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
         </is>
       </c>
       <c r="D265" s="3" t="inlineStr">
@@ -16765,12 +16765,12 @@
       </c>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R5-06</t>
         </is>
       </c>
       <c r="C266" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
         </is>
       </c>
       <c r="D266" s="3" t="inlineStr">
@@ -16792,12 +16792,12 @@
       </c>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R5-07</t>
         </is>
       </c>
       <c r="C267" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
         </is>
       </c>
       <c r="D267" s="3" t="inlineStr">
@@ -16819,12 +16819,12 @@
       </c>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R5-08</t>
         </is>
       </c>
       <c r="C268" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
         </is>
       </c>
       <c r="D268" s="3" t="inlineStr">
@@ -16846,12 +16846,12 @@
       </c>
       <c r="B269" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R5-09</t>
         </is>
       </c>
       <c r="C269" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
         </is>
       </c>
       <c r="D269" s="3" t="inlineStr">
@@ -16873,20 +16873,47 @@
       </c>
       <c r="B270" s="3" t="inlineStr">
         <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C270" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D270" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E270" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B271" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C270" s="3" t="inlineStr">
+      <c r="C271" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D270" s="3" t="inlineStr">
+      <c r="D271" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E270" s="3" t="inlineStr">
+      <c r="E271" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
docs: step-up API and E2E scenarios; tracker BPMS-022
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E271" headerRowCount="1">
-  <autoFilter ref="A1:E271"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E272" headerRowCount="1">
+  <autoFilter ref="A1:E272"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -3974,7 +3974,7 @@
       <c r="N18" s="3" t="inlineStr"/>
       <c r="O18" s="3" t="inlineStr">
         <is>
-          <t>TOTP (RFC 6238, replay-protected, sealed secrets) + 10 recovery codes + MFA login done (E2E-R1-AUTH-06). Remaining: WebAuthn/passkeys, step-up endpoint, MFA-required-by-role enforcement</t>
+          <t>TOTP (RFC 6238, replay-protected, sealed secrets) + 10 recovery codes + MFA login (E2E-R1-AUTH-06). Step-up: POST /session/step-up (TOTP code, or password without MFA) re-issues the token with a fresh auth_time; enforced against auth.stepup.window (401 step_up_required) for step-up settings, role create/edit and grant/revoke (E2E-R1-CFG-03). MFA required by role (auth.mfa.required_roles) enforced at workspace entry, 403 mfa_required (E2E-R1-MEM-10). Remaining: WebAuthn/passkeys</t>
         </is>
       </c>
     </row>
@@ -9592,7 +9592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E271"/>
+  <dimension ref="A1:E272"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14659,12 +14659,12 @@
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUD-01</t>
+          <t>E2E-R1-MEM-10</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
         <is>
-          <t>Every mutating route is called once and appends exactly the audit actions in its route contract (`/__test/audit/contract`); exempt routes append nothing; no route goes unexercised (bootstrap is one-shot and checked by the platform integration test) | FR-T01, docs/24 §3.5</t>
+          <t>MFA by role: in a Standard workspace an admin signed in without MFA is refused at workspace entry (403 `mfa_required`); a plain member is not | docs/20 §2.3 `auth.mfa.required_roles`, FR-W06</t>
         </is>
       </c>
       <c r="D188" s="3" t="inlineStr">
@@ -14686,12 +14686,12 @@
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CFG-01</t>
+          <t>E2E-R1-AUD-01</t>
         </is>
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>The creation profile seeds values (Starter: 8 h idle); the explainer lists default → platform floor → profile; unknown keys 404 | FR-W04, docs/20 §0-1</t>
+          <t>Every mutating route is called once and appends exactly the audit actions in its route contract (`/__test/audit/contract`); exempt routes append nothing; no route goes unexercised (bootstrap is one-shot and checked by the platform integration test) | FR-T01, docs/24 §3.5</t>
         </is>
       </c>
       <c r="D189" s="3" t="inlineStr">
@@ -14713,12 +14713,12 @@
       </c>
       <c r="B190" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CFG-02</t>
+          <t>E2E-R1-CFG-01</t>
         </is>
       </c>
       <c r="C190" s="3" t="inlineStr">
         <is>
-          <t>Looser than a floor → 422 `setting_below_floor`; ⚡ keys need a reason; stricter value saved with `ETag`/`If-Match` (stale → 412); floor-locked key 403; invalid value 422; history records the change | FR-S05, FR-W06</t>
+          <t>The creation profile seeds values (Starter: 8 h idle); the explainer lists default → platform floor → profile; unknown keys 404 | FR-W04, docs/20 §0-1</t>
         </is>
       </c>
       <c r="D190" s="3" t="inlineStr">
@@ -14740,12 +14740,12 @@
       </c>
       <c r="B191" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CFG-03</t>
+          <t>E2E-R1-CFG-02</t>
         </is>
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>Step-up keys (`auth.mfa.required_roles`) need an MFA-verified session | docs/20 §2.3</t>
+          <t>Looser than a floor → 422 `setting_below_floor`; ⚡ keys need a reason; stricter value saved with `ETag`/`If-Match` (stale → 412); floor-locked key 403; invalid value 422; history records the change | FR-S05, FR-W06</t>
         </is>
       </c>
       <c r="D191" s="3" t="inlineStr">
@@ -14767,12 +14767,12 @@
       </c>
       <c r="B192" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CFG-04</t>
+          <t>E2E-R1-CFG-03</t>
         </is>
       </c>
       <c r="C192" s="3" t="inlineStr">
         <is>
-          <t>A member without settings permissions can neither view nor change settings | docs/12 §5</t>
+          <t>Step-up keys need a recent authentication: a 10-minute-old sign-in gets 401 `step_up_required`; a wrong code fails; `POST /session/step-up` with a current TOTP code issues a fresh token that succeeds | docs/12 §11, SEC-17</t>
         </is>
       </c>
       <c r="D192" s="3" t="inlineStr">
@@ -14794,12 +14794,12 @@
       </c>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CFG-05</t>
+          <t>E2E-R1-CFG-04</t>
         </is>
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>Raising a platform floor clamps a looser workspace value at resolution (stored value kept, `clamped: true`); floors need a reason; keys without floors are rejected | docs/20 §1 rules 4-5</t>
+          <t>A member without settings permissions can neither view nor change settings | docs/12 §5</t>
         </is>
       </c>
       <c r="D193" s="3" t="inlineStr">
@@ -14821,12 +14821,12 @@
       </c>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-DIR-01</t>
+          <t>E2E-R1-CFG-05</t>
         </is>
       </c>
       <c r="C194" s="3" t="inlineStr">
         <is>
-          <t>Department tree: sibling names unique (409), moving under a descendant rejected (422 `cycle`), deleting a non-empty department refused | FR-W02</t>
+          <t>Raising a platform floor clamps a looser workspace value at resolution (stored value kept, `clamped: true`); floors need a reason; keys without floors are rejected | docs/20 §1 rules 4-5</t>
         </is>
       </c>
       <c r="D194" s="3" t="inlineStr">
@@ -14848,12 +14848,12 @@
       </c>
       <c r="B195" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-DIR-02</t>
+          <t>E2E-R1-DIR-01</t>
         </is>
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>Manager cycles rejected; resolution is the explicit manager, else the nearest department head that is not the member; field sources recorded | FR-W02 (deterministic resolution)</t>
+          <t>Department tree: sibling names unique (409), moving under a descendant rejected (422 `cycle`), deleting a non-empty department refused | FR-W02</t>
         </is>
       </c>
       <c r="D195" s="3" t="inlineStr">
@@ -14875,12 +14875,12 @@
       </c>
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-DIR-03</t>
+          <t>E2E-R1-DIR-02</t>
         </is>
       </c>
       <c r="C196" s="3" t="inlineStr">
         <is>
-          <t>Static groups (duplicate member 409); positions blocked until `directory.positions.enabled`; members read the directory but cannot change it | FR-W02, docs/20 §2.5</t>
+          <t>Manager cycles rejected; resolution is the explicit manager, else the nearest department head that is not the member; field sources recorded | FR-W02 (deterministic resolution)</t>
         </is>
       </c>
       <c r="D196" s="3" t="inlineStr">
@@ -14902,12 +14902,12 @@
       </c>
       <c r="B197" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-DIR-04</t>
+          <t>E2E-R1-DIR-03</t>
         </is>
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>CSV import: `mode=plan` changes nothing; `mode=apply` creates departments by path and links managers listed later in the file; unknown members reported per row; unknown columns 422 | FR-W02</t>
+          <t>Static groups (duplicate member 409); positions blocked until `directory.positions.enabled`; members read the directory but cannot change it | FR-W02, docs/20 §2.5</t>
         </is>
       </c>
       <c r="D197" s="3" t="inlineStr">
@@ -14929,12 +14929,12 @@
       </c>
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-DIR-04</t>
         </is>
       </c>
       <c r="C198" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>CSV import: `mode=plan` changes nothing; `mode=apply` creates departments by path and links managers listed later in the file; unknown members reported per row; unknown columns 422 | FR-W02</t>
         </is>
       </c>
       <c r="D198" s="3" t="inlineStr">
@@ -14956,12 +14956,12 @@
       </c>
       <c r="B199" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
         </is>
       </c>
       <c r="D199" s="3" t="inlineStr">
@@ -14983,12 +14983,12 @@
       </c>
       <c r="B200" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C200" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D200" s="3" t="inlineStr">
@@ -15010,12 +15010,12 @@
       </c>
       <c r="B201" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D201" s="3" t="inlineStr">
@@ -15037,12 +15037,12 @@
       </c>
       <c r="B202" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C202" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
         </is>
       </c>
       <c r="D202" s="3" t="inlineStr">
@@ -15064,12 +15064,12 @@
       </c>
       <c r="B203" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
         </is>
       </c>
       <c r="D203" s="3" t="inlineStr">
@@ -15091,12 +15091,12 @@
       </c>
       <c r="B204" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C204" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D204" s="3" t="inlineStr">
@@ -15118,12 +15118,12 @@
       </c>
       <c r="B205" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C205" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D205" s="3" t="inlineStr">
@@ -15145,12 +15145,12 @@
       </c>
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
         </is>
       </c>
       <c r="D206" s="3" t="inlineStr">
@@ -15172,12 +15172,12 @@
       </c>
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D207" s="3" t="inlineStr">
@@ -15199,12 +15199,12 @@
       </c>
       <c r="B208" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D208" s="3" t="inlineStr">
@@ -15226,12 +15226,12 @@
       </c>
       <c r="B209" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D209" s="3" t="inlineStr">
@@ -15253,12 +15253,12 @@
       </c>
       <c r="B210" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D210" s="3" t="inlineStr">
@@ -15280,12 +15280,12 @@
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
         </is>
       </c>
       <c r="D211" s="3" t="inlineStr">
@@ -15307,12 +15307,12 @@
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
         </is>
       </c>
       <c r="D212" s="3" t="inlineStr">
@@ -15334,12 +15334,12 @@
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
         </is>
       </c>
       <c r="D213" s="3" t="inlineStr">
@@ -15361,12 +15361,12 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D214" s="3" t="inlineStr">
@@ -15388,12 +15388,12 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
         </is>
       </c>
       <c r="D215" s="3" t="inlineStr">
@@ -15415,12 +15415,12 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
@@ -15442,12 +15442,12 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -15469,12 +15469,12 @@
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
@@ -15496,12 +15496,12 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D219" s="3" t="inlineStr">
@@ -15523,12 +15523,12 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D220" s="3" t="inlineStr">
@@ -15550,12 +15550,12 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D221" s="3" t="inlineStr">
@@ -15577,12 +15577,12 @@
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D222" s="3" t="inlineStr">
@@ -15604,12 +15604,12 @@
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D223" s="3" t="inlineStr">
@@ -15631,12 +15631,12 @@
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D224" s="3" t="inlineStr">
@@ -15658,12 +15658,12 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D225" s="3" t="inlineStr">
@@ -15685,12 +15685,12 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D226" s="3" t="inlineStr">
@@ -15712,12 +15712,12 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D227" s="3" t="inlineStr">
@@ -15739,12 +15739,12 @@
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D228" s="3" t="inlineStr">
@@ -15766,12 +15766,12 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
@@ -15793,12 +15793,12 @@
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D230" s="3" t="inlineStr">
@@ -15820,12 +15820,12 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D231" s="3" t="inlineStr">
@@ -15847,12 +15847,12 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D232" s="3" t="inlineStr">
@@ -15874,12 +15874,12 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D233" s="3" t="inlineStr">
@@ -15901,12 +15901,12 @@
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D234" s="3" t="inlineStr">
@@ -15928,12 +15928,12 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D235" s="3" t="inlineStr">
@@ -15955,12 +15955,12 @@
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D236" s="3" t="inlineStr">
@@ -15982,12 +15982,12 @@
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D237" s="3" t="inlineStr">
@@ -16009,12 +16009,12 @@
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D238" s="3" t="inlineStr">
@@ -16036,12 +16036,12 @@
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D239" s="3" t="inlineStr">
@@ -16063,12 +16063,12 @@
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D240" s="3" t="inlineStr">
@@ -16090,12 +16090,12 @@
       </c>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D241" s="3" t="inlineStr">
@@ -16117,12 +16117,12 @@
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D242" s="3" t="inlineStr">
@@ -16144,12 +16144,12 @@
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D243" s="3" t="inlineStr">
@@ -16171,12 +16171,12 @@
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D244" s="3" t="inlineStr">
@@ -16198,12 +16198,12 @@
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D245" s="3" t="inlineStr">
@@ -16225,12 +16225,12 @@
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D246" s="3" t="inlineStr">
@@ -16252,12 +16252,12 @@
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D247" s="3" t="inlineStr">
@@ -16279,12 +16279,12 @@
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
@@ -16306,12 +16306,12 @@
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D249" s="3" t="inlineStr">
@@ -16333,12 +16333,12 @@
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D250" s="3" t="inlineStr">
@@ -16360,12 +16360,12 @@
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D251" s="3" t="inlineStr">
@@ -16387,12 +16387,12 @@
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D252" s="3" t="inlineStr">
@@ -16414,12 +16414,12 @@
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D253" s="3" t="inlineStr">
@@ -16441,12 +16441,12 @@
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D254" s="3" t="inlineStr">
@@ -16468,12 +16468,12 @@
       </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D255" s="3" t="inlineStr">
@@ -16495,12 +16495,12 @@
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C256" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D256" s="3" t="inlineStr">
@@ -16522,12 +16522,12 @@
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D257" s="3" t="inlineStr">
@@ -16549,12 +16549,12 @@
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C258" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D258" s="3" t="inlineStr">
@@ -16576,12 +16576,12 @@
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D259" s="3" t="inlineStr">
@@ -16603,12 +16603,12 @@
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R4-11</t>
         </is>
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
         </is>
       </c>
       <c r="D260" s="3" t="inlineStr">
@@ -16630,12 +16630,12 @@
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-ISO</t>
         </is>
       </c>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
         </is>
       </c>
       <c r="D261" s="3" t="inlineStr">
@@ -16657,12 +16657,12 @@
       </c>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R5-01</t>
         </is>
       </c>
       <c r="C262" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
         </is>
       </c>
       <c r="D262" s="3" t="inlineStr">
@@ -16684,12 +16684,12 @@
       </c>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R5-02</t>
         </is>
       </c>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
         </is>
       </c>
       <c r="D263" s="3" t="inlineStr">
@@ -16711,12 +16711,12 @@
       </c>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R5-03</t>
         </is>
       </c>
       <c r="C264" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
         </is>
       </c>
       <c r="D264" s="3" t="inlineStr">
@@ -16738,12 +16738,12 @@
       </c>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R5-04</t>
         </is>
       </c>
       <c r="C265" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
         </is>
       </c>
       <c r="D265" s="3" t="inlineStr">
@@ -16765,12 +16765,12 @@
       </c>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R5-05</t>
         </is>
       </c>
       <c r="C266" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
         </is>
       </c>
       <c r="D266" s="3" t="inlineStr">
@@ -16792,12 +16792,12 @@
       </c>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R5-06</t>
         </is>
       </c>
       <c r="C267" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
         </is>
       </c>
       <c r="D267" s="3" t="inlineStr">
@@ -16819,12 +16819,12 @@
       </c>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R5-07</t>
         </is>
       </c>
       <c r="C268" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
         </is>
       </c>
       <c r="D268" s="3" t="inlineStr">
@@ -16846,12 +16846,12 @@
       </c>
       <c r="B269" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R5-08</t>
         </is>
       </c>
       <c r="C269" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
         </is>
       </c>
       <c r="D269" s="3" t="inlineStr">
@@ -16873,12 +16873,12 @@
       </c>
       <c r="B270" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R5-09</t>
         </is>
       </c>
       <c r="C270" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
         </is>
       </c>
       <c r="D270" s="3" t="inlineStr">
@@ -16900,20 +16900,47 @@
       </c>
       <c r="B271" s="3" t="inlineStr">
         <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C271" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D271" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E271" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B272" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C271" s="3" t="inlineStr">
+      <c r="C272" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D271" s="3" t="inlineStr">
+      <c r="D272" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E271" s="3" t="inlineStr">
+      <c r="E272" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
docs: tracker marks BPMS-029 done
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -4417,7 +4417,7 @@
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L25" s="3" t="inlineStr"/>
@@ -4425,7 +4425,7 @@
       <c r="N25" s="3" t="inlineStr"/>
       <c r="O25" s="3" t="inlineStr">
         <is>
-          <t>Outbox/inbox/idempotency tables + helpers with tests (disjoint SKIP LOCKED claims, replay/conflict). Remaining: dispatcher loop (LISTEN/NOTIFY + Bus trait)</t>
+          <t>Outbox/inbox/idempotency tables + helpers (SKIP LOCKED claims, replay/conflict). Dispatcher (procera_db::dispatch, migration 0010): due-workspace discovery, per-workspace advisory lock, per-aggregate ordered delivery to a Bus, at-least-once with exponential backoff (max 5 min) and hold-back behind a failed event, NOTIFY trigger wake-ups + 1 s polling; runs in serve --all; /__test/drain really drains. Tests: order/backoff/hold-back/workspaces + NOTIFY wake-up; E2E-R1-MEM-07. Consumers (mailer) arrive with BPMS-048</t>
         </is>
       </c>
     </row>
@@ -14583,7 +14583,7 @@
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>Pending invitations listed; revoking kills the token (404); resend issues a new working token | FR-W01</t>
+          <t>Pending invitations listed; revoking kills the token (404); resend issues a new working token; `/__test/drain` dispatches the outbox to idle | FR-W01, docs/04 §2.11</t>
         </is>
       </c>
       <c r="D185" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: notifications API, LLD as-built note, E2E plan; tracker BPMS-048
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E272" headerRowCount="1">
-  <autoFilter ref="A1:E272"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E274" headerRowCount="1">
+  <autoFilter ref="A1:E274"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -5283,13 +5283,17 @@
       </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L39" s="3" t="inlineStr"/>
       <c r="M39" s="3" t="inlineStr"/>
       <c r="N39" s="3" t="inlineStr"/>
-      <c r="O39" s="3" t="inlineStr"/>
+      <c r="O39" s="3" t="inlineStr">
+        <is>
+          <t>procera-notify (migration 0011): templates in code (minijinja, strict, HTML auto-escaped), in-app inbox (list/unread/read/read-all), email queue with sealed bodies and dedupe, SMTP delivery via lettre (STARTTLS/TLS) with backoff (max 1 h, 12 tries), workspace sender name; outbox consumers: invitation email with accept link, member-joined in-app to the inviter. Flags --public-url, --smtp-url, --mail-from. E2E-R1-NOT-01..02. Remaining: digests + quiet hours (FR-N04), localisation + terminology (CFG-008), more event kinds as features land</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -9592,7 +9596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E272"/>
+  <dimension ref="A1:E274"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14956,12 +14960,12 @@
       </c>
       <c r="B199" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-NOT-01</t>
         </is>
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>An invitation queues an email (subject, HTML button, link); the link's token registers the invitee; the inviter gets an in-app "joined" notification; read / unread / read-all work | FR-N01, FR-N02, FR-W01</t>
         </is>
       </c>
       <c r="D199" s="3" t="inlineStr">
@@ -14983,12 +14987,12 @@
       </c>
       <c r="B200" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-NOT-02</t>
         </is>
       </c>
       <c r="C200" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>A member cannot mark another member's notification (404) | FR-N01, SEC-01</t>
         </is>
       </c>
       <c r="D200" s="3" t="inlineStr">
@@ -15010,12 +15014,12 @@
       </c>
       <c r="B201" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
         </is>
       </c>
       <c r="D201" s="3" t="inlineStr">
@@ -15037,12 +15041,12 @@
       </c>
       <c r="B202" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C202" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D202" s="3" t="inlineStr">
@@ -15064,12 +15068,12 @@
       </c>
       <c r="B203" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D203" s="3" t="inlineStr">
@@ -15091,12 +15095,12 @@
       </c>
       <c r="B204" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C204" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
         </is>
       </c>
       <c r="D204" s="3" t="inlineStr">
@@ -15118,12 +15122,12 @@
       </c>
       <c r="B205" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C205" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
         </is>
       </c>
       <c r="D205" s="3" t="inlineStr">
@@ -15145,12 +15149,12 @@
       </c>
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D206" s="3" t="inlineStr">
@@ -15172,12 +15176,12 @@
       </c>
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D207" s="3" t="inlineStr">
@@ -15199,12 +15203,12 @@
       </c>
       <c r="B208" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
         </is>
       </c>
       <c r="D208" s="3" t="inlineStr">
@@ -15226,12 +15230,12 @@
       </c>
       <c r="B209" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D209" s="3" t="inlineStr">
@@ -15253,12 +15257,12 @@
       </c>
       <c r="B210" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D210" s="3" t="inlineStr">
@@ -15280,12 +15284,12 @@
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D211" s="3" t="inlineStr">
@@ -15307,12 +15311,12 @@
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D212" s="3" t="inlineStr">
@@ -15334,12 +15338,12 @@
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
         </is>
       </c>
       <c r="D213" s="3" t="inlineStr">
@@ -15361,12 +15365,12 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
         </is>
       </c>
       <c r="D214" s="3" t="inlineStr">
@@ -15388,12 +15392,12 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
         </is>
       </c>
       <c r="D215" s="3" t="inlineStr">
@@ -15415,12 +15419,12 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
@@ -15442,12 +15446,12 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -15469,12 +15473,12 @@
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
@@ -15496,12 +15500,12 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D219" s="3" t="inlineStr">
@@ -15523,12 +15527,12 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
         </is>
       </c>
       <c r="D220" s="3" t="inlineStr">
@@ -15550,12 +15554,12 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D221" s="3" t="inlineStr">
@@ -15577,12 +15581,12 @@
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D222" s="3" t="inlineStr">
@@ -15604,12 +15608,12 @@
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D223" s="3" t="inlineStr">
@@ -15631,12 +15635,12 @@
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D224" s="3" t="inlineStr">
@@ -15658,12 +15662,12 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D225" s="3" t="inlineStr">
@@ -15685,12 +15689,12 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D226" s="3" t="inlineStr">
@@ -15712,12 +15716,12 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D227" s="3" t="inlineStr">
@@ -15739,12 +15743,12 @@
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D228" s="3" t="inlineStr">
@@ -15766,12 +15770,12 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
@@ -15793,12 +15797,12 @@
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D230" s="3" t="inlineStr">
@@ -15820,12 +15824,12 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D231" s="3" t="inlineStr">
@@ -15847,12 +15851,12 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D232" s="3" t="inlineStr">
@@ -15874,12 +15878,12 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D233" s="3" t="inlineStr">
@@ -15901,12 +15905,12 @@
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D234" s="3" t="inlineStr">
@@ -15928,12 +15932,12 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D235" s="3" t="inlineStr">
@@ -15955,12 +15959,12 @@
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D236" s="3" t="inlineStr">
@@ -15982,12 +15986,12 @@
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D237" s="3" t="inlineStr">
@@ -16009,12 +16013,12 @@
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D238" s="3" t="inlineStr">
@@ -16036,12 +16040,12 @@
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D239" s="3" t="inlineStr">
@@ -16063,12 +16067,12 @@
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D240" s="3" t="inlineStr">
@@ -16090,12 +16094,12 @@
       </c>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D241" s="3" t="inlineStr">
@@ -16117,12 +16121,12 @@
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D242" s="3" t="inlineStr">
@@ -16144,12 +16148,12 @@
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D243" s="3" t="inlineStr">
@@ -16171,12 +16175,12 @@
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D244" s="3" t="inlineStr">
@@ -16198,12 +16202,12 @@
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D245" s="3" t="inlineStr">
@@ -16225,12 +16229,12 @@
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D246" s="3" t="inlineStr">
@@ -16252,12 +16256,12 @@
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D247" s="3" t="inlineStr">
@@ -16279,12 +16283,12 @@
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
@@ -16306,12 +16310,12 @@
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D249" s="3" t="inlineStr">
@@ -16333,12 +16337,12 @@
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D250" s="3" t="inlineStr">
@@ -16360,12 +16364,12 @@
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D251" s="3" t="inlineStr">
@@ -16387,12 +16391,12 @@
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D252" s="3" t="inlineStr">
@@ -16414,12 +16418,12 @@
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D253" s="3" t="inlineStr">
@@ -16441,12 +16445,12 @@
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D254" s="3" t="inlineStr">
@@ -16468,12 +16472,12 @@
       </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D255" s="3" t="inlineStr">
@@ -16495,12 +16499,12 @@
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C256" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D256" s="3" t="inlineStr">
@@ -16522,12 +16526,12 @@
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D257" s="3" t="inlineStr">
@@ -16549,12 +16553,12 @@
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C258" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D258" s="3" t="inlineStr">
@@ -16576,12 +16580,12 @@
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D259" s="3" t="inlineStr">
@@ -16603,12 +16607,12 @@
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D260" s="3" t="inlineStr">
@@ -16630,12 +16634,12 @@
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D261" s="3" t="inlineStr">
@@ -16657,12 +16661,12 @@
       </c>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-11</t>
         </is>
       </c>
       <c r="C262" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
         </is>
       </c>
       <c r="D262" s="3" t="inlineStr">
@@ -16684,12 +16688,12 @@
       </c>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R4-ISO</t>
         </is>
       </c>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
         </is>
       </c>
       <c r="D263" s="3" t="inlineStr">
@@ -16711,12 +16715,12 @@
       </c>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R5-01</t>
         </is>
       </c>
       <c r="C264" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
         </is>
       </c>
       <c r="D264" s="3" t="inlineStr">
@@ -16738,12 +16742,12 @@
       </c>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R5-02</t>
         </is>
       </c>
       <c r="C265" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
         </is>
       </c>
       <c r="D265" s="3" t="inlineStr">
@@ -16765,12 +16769,12 @@
       </c>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R5-03</t>
         </is>
       </c>
       <c r="C266" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
         </is>
       </c>
       <c r="D266" s="3" t="inlineStr">
@@ -16792,12 +16796,12 @@
       </c>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R5-04</t>
         </is>
       </c>
       <c r="C267" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
         </is>
       </c>
       <c r="D267" s="3" t="inlineStr">
@@ -16819,12 +16823,12 @@
       </c>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R5-05</t>
         </is>
       </c>
       <c r="C268" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
         </is>
       </c>
       <c r="D268" s="3" t="inlineStr">
@@ -16846,12 +16850,12 @@
       </c>
       <c r="B269" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R5-06</t>
         </is>
       </c>
       <c r="C269" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
         </is>
       </c>
       <c r="D269" s="3" t="inlineStr">
@@ -16873,12 +16877,12 @@
       </c>
       <c r="B270" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R5-07</t>
         </is>
       </c>
       <c r="C270" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
         </is>
       </c>
       <c r="D270" s="3" t="inlineStr">
@@ -16900,12 +16904,12 @@
       </c>
       <c r="B271" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R5-08</t>
         </is>
       </c>
       <c r="C271" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
         </is>
       </c>
       <c r="D271" s="3" t="inlineStr">
@@ -16927,20 +16931,74 @@
       </c>
       <c r="B272" s="3" t="inlineStr">
         <is>
+          <t>E2E-R5-09</t>
+        </is>
+      </c>
+      <c r="C272" s="3" t="inlineStr">
+        <is>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+        </is>
+      </c>
+      <c r="D272" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E272" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B273" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C273" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D273" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E273" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B274" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C272" s="3" t="inlineStr">
+      <c r="C274" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D272" s="3" t="inlineStr">
+      <c r="D274" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E272" s="3" t="inlineStr">
+      <c r="E274" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
docs: library API and E2E plan; tracker marks BPMS-040 done
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E274" headerRowCount="1">
-  <autoFilter ref="A1:E274"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E279" headerRowCount="1">
+  <autoFilter ref="A1:E279"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -4795,13 +4795,17 @@
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L31" s="3" t="inlineStr"/>
       <c r="M31" s="3" t="inlineStr"/>
       <c r="N31" s="3" t="inlineStr"/>
-      <c r="O31" s="3" t="inlineStr"/>
+      <c r="O31" s="3" t="inlineStr">
+        <is>
+          <t>procera-library (migration 0012): artifacts + versions for SOPs and policies; lifecycle draft → in_review → approved → scheduled/published → deprecated → retired with guarded transitions; one open draft per artifact; reviews in numbered rounds, approvals from governance.review.* settings, author never reviews own version, distinct approvers, comment required to reject; content_hash = SHA-256(JCS) frozen at approval and a trigger forbids changing approved content or moving back (T07); publish supersedes, future effective_at schedules (worker + drain), reason for change on later versions, retire; step-up for controlled approve/publish; outbox artifact.published.v1; every transition audited. E2E-R1-LIB-01..05. Process artifacts arrive with the designer/compiler</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -9596,7 +9600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E274"/>
+  <dimension ref="A1:E279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -15014,12 +15018,12 @@
       </c>
       <c r="B201" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-LIB-01</t>
         </is>
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>SOP draft → edit with `If-Match` (stale → 412) → submit (no review needed: approved, content hash frozen) → published; editing an approved version 409; content and hash identical on retrieval; one open draft per artifact | FR-G04, FR-G05, T07</t>
         </is>
       </c>
       <c r="D201" s="3" t="inlineStr">
@@ -15041,12 +15045,12 @@
       </c>
       <c r="B202" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-LIB-02</t>
         </is>
       </c>
       <c r="C202" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>Controlled policy needs a review: the author's own approval is refused (403 `sod_violation`); a reviewer cannot publish; a reviewer approves; the owner publishes | FR-G04 SoD, docs/12 §6</t>
         </is>
       </c>
       <c r="D202" s="3" t="inlineStr">
@@ -15068,12 +15072,12 @@
       </c>
       <c r="B203" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-LIB-03</t>
         </is>
       </c>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>Changes requested needs a comment and returns the draft; withdraw; later versions need a reason for change; publishing supersedes (previous → deprecated) | FR-G04, docs/20 §2.6</t>
         </is>
       </c>
       <c r="D203" s="3" t="inlineStr">
@@ -15095,12 +15099,12 @@
       </c>
       <c r="B204" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-LIB-04</t>
         </is>
       </c>
       <c r="C204" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>A scheduled version goes live when its effective time passes (test clock + drain) and supersedes the live one; retire | FR-G05, FR-PL01</t>
         </is>
       </c>
       <c r="D204" s="3" t="inlineStr">
@@ -15122,12 +15126,12 @@
       </c>
       <c r="B205" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-LIB-05</t>
         </is>
       </c>
       <c r="C205" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>Members read published policies but cannot author; lists contain only kinds the member may view | docs/12 §5</t>
         </is>
       </c>
       <c r="D205" s="3" t="inlineStr">
@@ -15149,12 +15153,12 @@
       </c>
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
         </is>
       </c>
       <c r="D206" s="3" t="inlineStr">
@@ -15176,12 +15180,12 @@
       </c>
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D207" s="3" t="inlineStr">
@@ -15203,12 +15207,12 @@
       </c>
       <c r="B208" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D208" s="3" t="inlineStr">
@@ -15230,12 +15234,12 @@
       </c>
       <c r="B209" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
         </is>
       </c>
       <c r="D209" s="3" t="inlineStr">
@@ -15257,12 +15261,12 @@
       </c>
       <c r="B210" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
         </is>
       </c>
       <c r="D210" s="3" t="inlineStr">
@@ -15284,12 +15288,12 @@
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D211" s="3" t="inlineStr">
@@ -15311,12 +15315,12 @@
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D212" s="3" t="inlineStr">
@@ -15338,12 +15342,12 @@
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
         </is>
       </c>
       <c r="D213" s="3" t="inlineStr">
@@ -15365,12 +15369,12 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D214" s="3" t="inlineStr">
@@ -15392,12 +15396,12 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D215" s="3" t="inlineStr">
@@ -15419,12 +15423,12 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
@@ -15446,12 +15450,12 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -15473,12 +15477,12 @@
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
@@ -15500,12 +15504,12 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
         </is>
       </c>
       <c r="D219" s="3" t="inlineStr">
@@ -15527,12 +15531,12 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
         </is>
       </c>
       <c r="D220" s="3" t="inlineStr">
@@ -15554,12 +15558,12 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D221" s="3" t="inlineStr">
@@ -15581,12 +15585,12 @@
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
         </is>
       </c>
       <c r="D222" s="3" t="inlineStr">
@@ -15608,12 +15612,12 @@
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
         </is>
       </c>
       <c r="D223" s="3" t="inlineStr">
@@ -15635,12 +15639,12 @@
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D224" s="3" t="inlineStr">
@@ -15662,12 +15666,12 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
         </is>
       </c>
       <c r="D225" s="3" t="inlineStr">
@@ -15689,12 +15693,12 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D226" s="3" t="inlineStr">
@@ -15716,12 +15720,12 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D227" s="3" t="inlineStr">
@@ -15743,12 +15747,12 @@
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D228" s="3" t="inlineStr">
@@ -15770,12 +15774,12 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
@@ -15797,12 +15801,12 @@
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D230" s="3" t="inlineStr">
@@ -15824,12 +15828,12 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D231" s="3" t="inlineStr">
@@ -15851,12 +15855,12 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D232" s="3" t="inlineStr">
@@ -15878,12 +15882,12 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D233" s="3" t="inlineStr">
@@ -15905,12 +15909,12 @@
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D234" s="3" t="inlineStr">
@@ -15932,12 +15936,12 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D235" s="3" t="inlineStr">
@@ -15959,12 +15963,12 @@
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D236" s="3" t="inlineStr">
@@ -15986,12 +15990,12 @@
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D237" s="3" t="inlineStr">
@@ -16013,12 +16017,12 @@
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D238" s="3" t="inlineStr">
@@ -16040,12 +16044,12 @@
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D239" s="3" t="inlineStr">
@@ -16067,12 +16071,12 @@
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D240" s="3" t="inlineStr">
@@ -16094,12 +16098,12 @@
       </c>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D241" s="3" t="inlineStr">
@@ -16121,12 +16125,12 @@
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D242" s="3" t="inlineStr">
@@ -16148,12 +16152,12 @@
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D243" s="3" t="inlineStr">
@@ -16175,12 +16179,12 @@
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D244" s="3" t="inlineStr">
@@ -16202,12 +16206,12 @@
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D245" s="3" t="inlineStr">
@@ -16229,12 +16233,12 @@
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D246" s="3" t="inlineStr">
@@ -16256,12 +16260,12 @@
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D247" s="3" t="inlineStr">
@@ -16283,12 +16287,12 @@
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
@@ -16310,12 +16314,12 @@
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D249" s="3" t="inlineStr">
@@ -16337,12 +16341,12 @@
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D250" s="3" t="inlineStr">
@@ -16364,12 +16368,12 @@
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D251" s="3" t="inlineStr">
@@ -16391,12 +16395,12 @@
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D252" s="3" t="inlineStr">
@@ -16418,12 +16422,12 @@
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D253" s="3" t="inlineStr">
@@ -16445,12 +16449,12 @@
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D254" s="3" t="inlineStr">
@@ -16472,12 +16476,12 @@
       </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D255" s="3" t="inlineStr">
@@ -16499,12 +16503,12 @@
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C256" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D256" s="3" t="inlineStr">
@@ -16526,12 +16530,12 @@
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D257" s="3" t="inlineStr">
@@ -16553,12 +16557,12 @@
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C258" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D258" s="3" t="inlineStr">
@@ -16580,12 +16584,12 @@
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D259" s="3" t="inlineStr">
@@ -16607,12 +16611,12 @@
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D260" s="3" t="inlineStr">
@@ -16634,12 +16638,12 @@
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D261" s="3" t="inlineStr">
@@ -16661,12 +16665,12 @@
       </c>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C262" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D262" s="3" t="inlineStr">
@@ -16688,12 +16692,12 @@
       </c>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D263" s="3" t="inlineStr">
@@ -16715,12 +16719,12 @@
       </c>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C264" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D264" s="3" t="inlineStr">
@@ -16742,12 +16746,12 @@
       </c>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C265" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D265" s="3" t="inlineStr">
@@ -16769,12 +16773,12 @@
       </c>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C266" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D266" s="3" t="inlineStr">
@@ -16796,12 +16800,12 @@
       </c>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R4-11</t>
         </is>
       </c>
       <c r="C267" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
         </is>
       </c>
       <c r="D267" s="3" t="inlineStr">
@@ -16823,12 +16827,12 @@
       </c>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R4-ISO</t>
         </is>
       </c>
       <c r="C268" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
         </is>
       </c>
       <c r="D268" s="3" t="inlineStr">
@@ -16850,12 +16854,12 @@
       </c>
       <c r="B269" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R5-01</t>
         </is>
       </c>
       <c r="C269" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
         </is>
       </c>
       <c r="D269" s="3" t="inlineStr">
@@ -16877,12 +16881,12 @@
       </c>
       <c r="B270" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R5-02</t>
         </is>
       </c>
       <c r="C270" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
         </is>
       </c>
       <c r="D270" s="3" t="inlineStr">
@@ -16904,12 +16908,12 @@
       </c>
       <c r="B271" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R5-03</t>
         </is>
       </c>
       <c r="C271" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
         </is>
       </c>
       <c r="D271" s="3" t="inlineStr">
@@ -16931,12 +16935,12 @@
       </c>
       <c r="B272" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R5-04</t>
         </is>
       </c>
       <c r="C272" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
         </is>
       </c>
       <c r="D272" s="3" t="inlineStr">
@@ -16958,12 +16962,12 @@
       </c>
       <c r="B273" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R5-05</t>
         </is>
       </c>
       <c r="C273" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
         </is>
       </c>
       <c r="D273" s="3" t="inlineStr">
@@ -16985,20 +16989,155 @@
       </c>
       <c r="B274" s="3" t="inlineStr">
         <is>
+          <t>E2E-R5-06</t>
+        </is>
+      </c>
+      <c r="C274" s="3" t="inlineStr">
+        <is>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+        </is>
+      </c>
+      <c r="D274" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E274" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B275" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-07</t>
+        </is>
+      </c>
+      <c r="C275" s="3" t="inlineStr">
+        <is>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+        </is>
+      </c>
+      <c r="D275" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E275" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B276" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-08</t>
+        </is>
+      </c>
+      <c r="C276" s="3" t="inlineStr">
+        <is>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+        </is>
+      </c>
+      <c r="D276" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E276" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B277" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-09</t>
+        </is>
+      </c>
+      <c r="C277" s="3" t="inlineStr">
+        <is>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+        </is>
+      </c>
+      <c r="D277" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E277" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B278" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C278" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D278" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E278" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B279" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C274" s="3" t="inlineStr">
+      <c r="C279" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D274" s="3" t="inlineStr">
+      <c r="D279" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E274" s="3" t="inlineStr">
+      <c r="E279" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
docs: browser E2E scenarios; tracker BPMS-031 in progress
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E279" headerRowCount="1">
-  <autoFilter ref="A1:E279"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E284" headerRowCount="1">
+  <autoFilter ref="A1:E284"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -4547,13 +4547,17 @@
       </c>
       <c r="K27" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L27" s="3" t="inlineStr"/>
       <c r="M27" s="3" t="inlineStr"/>
       <c r="N27" s="3" t="inlineStr"/>
-      <c r="O27" s="3" t="inlineStr"/>
+      <c r="O27" s="3" t="inlineStr">
+        <is>
+          <t>Web app slice 1: history router, API client (in-memory access token, silent refresh via HttpOnly cookie, RFC 9457 errors), session provider, Vite proxy (same-origin), sign-in with MFA (TOTP or recovery code), workspace chooser, app shell with workspace switcher menu, notification bell with unread count, permission-shaped navigation, Home, notifications inbox; design gallery moved to /design. E2E-R1-UI-01..05 (axe on every screen). Remaining: system console shell, ⌘K command palette, mobile bottom bar</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -9600,7 +9604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E279"/>
+  <dimension ref="A1:E284"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -15153,12 +15157,12 @@
       </c>
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-UI-01</t>
         </is>
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>Sign in through the browser (password + recovery code) lands on Home; navigation is permission-shaped with the current page marked; axe clean on sign-in and Home; reload keeps the session | docs/05 §2.1, §3.1, WCAG 2.2 AA</t>
         </is>
       </c>
       <c r="D206" s="3" t="inlineStr">
@@ -15180,12 +15184,12 @@
       </c>
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-UI-02</t>
         </is>
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>Wrong password and wrong code produce clear, non-revealing messages (role=alert); axe clean | docs/06 §3, WCAG 3.3.1</t>
         </is>
       </c>
       <c r="D207" s="3" t="inlineStr">
@@ -15207,12 +15211,12 @@
       </c>
       <c r="B208" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-UI-03</t>
         </is>
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>With several workspaces the chooser appears; choosing one and switching from the header changes the context and the navigation (no Admin for a plain member) | docs/05 §2.1 workspace switcher</t>
         </is>
       </c>
       <c r="D208" s="3" t="inlineStr">
@@ -15234,12 +15238,12 @@
       </c>
       <c r="B209" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-UI-04</t>
         </is>
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>The bell announces the unread count; the inbox lists the "joined" notification; mark all as read | FR-N01</t>
         </is>
       </c>
       <c r="D209" s="3" t="inlineStr">
@@ -15261,12 +15265,12 @@
       </c>
       <c r="B210" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-UI-05</t>
         </is>
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>Sign out returns to sign-in; reloading stays signed out | docs/06 §3</t>
         </is>
       </c>
       <c r="D210" s="3" t="inlineStr">
@@ -15288,12 +15292,12 @@
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
         </is>
       </c>
       <c r="D211" s="3" t="inlineStr">
@@ -15315,12 +15319,12 @@
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D212" s="3" t="inlineStr">
@@ -15342,12 +15346,12 @@
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D213" s="3" t="inlineStr">
@@ -15369,12 +15373,12 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
         </is>
       </c>
       <c r="D214" s="3" t="inlineStr">
@@ -15396,12 +15400,12 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
         </is>
       </c>
       <c r="D215" s="3" t="inlineStr">
@@ -15423,12 +15427,12 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
@@ -15450,12 +15454,12 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -15477,12 +15481,12 @@
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
@@ -15504,12 +15508,12 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D219" s="3" t="inlineStr">
@@ -15531,12 +15535,12 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D220" s="3" t="inlineStr">
@@ -15558,12 +15562,12 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D221" s="3" t="inlineStr">
@@ -15585,12 +15589,12 @@
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D222" s="3" t="inlineStr">
@@ -15612,12 +15616,12 @@
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
         </is>
       </c>
       <c r="D223" s="3" t="inlineStr">
@@ -15639,12 +15643,12 @@
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
         </is>
       </c>
       <c r="D224" s="3" t="inlineStr">
@@ -15666,12 +15670,12 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
         </is>
       </c>
       <c r="D225" s="3" t="inlineStr">
@@ -15693,12 +15697,12 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D226" s="3" t="inlineStr">
@@ -15720,12 +15724,12 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
         </is>
       </c>
       <c r="D227" s="3" t="inlineStr">
@@ -15747,12 +15751,12 @@
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
         </is>
       </c>
       <c r="D228" s="3" t="inlineStr">
@@ -15774,12 +15778,12 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
@@ -15801,12 +15805,12 @@
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
         </is>
       </c>
       <c r="D230" s="3" t="inlineStr">
@@ -15828,12 +15832,12 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D231" s="3" t="inlineStr">
@@ -15855,12 +15859,12 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D232" s="3" t="inlineStr">
@@ -15882,12 +15886,12 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D233" s="3" t="inlineStr">
@@ -15909,12 +15913,12 @@
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D234" s="3" t="inlineStr">
@@ -15936,12 +15940,12 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D235" s="3" t="inlineStr">
@@ -15963,12 +15967,12 @@
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D236" s="3" t="inlineStr">
@@ -15990,12 +15994,12 @@
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D237" s="3" t="inlineStr">
@@ -16017,12 +16021,12 @@
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D238" s="3" t="inlineStr">
@@ -16044,12 +16048,12 @@
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D239" s="3" t="inlineStr">
@@ -16071,12 +16075,12 @@
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D240" s="3" t="inlineStr">
@@ -16098,12 +16102,12 @@
       </c>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D241" s="3" t="inlineStr">
@@ -16125,12 +16129,12 @@
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D242" s="3" t="inlineStr">
@@ -16152,12 +16156,12 @@
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D243" s="3" t="inlineStr">
@@ -16179,12 +16183,12 @@
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D244" s="3" t="inlineStr">
@@ -16206,12 +16210,12 @@
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D245" s="3" t="inlineStr">
@@ -16233,12 +16237,12 @@
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D246" s="3" t="inlineStr">
@@ -16260,12 +16264,12 @@
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D247" s="3" t="inlineStr">
@@ -16287,12 +16291,12 @@
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
@@ -16314,12 +16318,12 @@
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D249" s="3" t="inlineStr">
@@ -16341,12 +16345,12 @@
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D250" s="3" t="inlineStr">
@@ -16368,12 +16372,12 @@
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D251" s="3" t="inlineStr">
@@ -16395,12 +16399,12 @@
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D252" s="3" t="inlineStr">
@@ -16422,12 +16426,12 @@
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D253" s="3" t="inlineStr">
@@ -16449,12 +16453,12 @@
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D254" s="3" t="inlineStr">
@@ -16476,12 +16480,12 @@
       </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D255" s="3" t="inlineStr">
@@ -16503,12 +16507,12 @@
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C256" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D256" s="3" t="inlineStr">
@@ -16530,12 +16534,12 @@
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D257" s="3" t="inlineStr">
@@ -16557,12 +16561,12 @@
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C258" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D258" s="3" t="inlineStr">
@@ -16584,12 +16588,12 @@
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D259" s="3" t="inlineStr">
@@ -16611,12 +16615,12 @@
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D260" s="3" t="inlineStr">
@@ -16638,12 +16642,12 @@
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D261" s="3" t="inlineStr">
@@ -16665,12 +16669,12 @@
       </c>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C262" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D262" s="3" t="inlineStr">
@@ -16692,12 +16696,12 @@
       </c>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D263" s="3" t="inlineStr">
@@ -16719,12 +16723,12 @@
       </c>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C264" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D264" s="3" t="inlineStr">
@@ -16746,12 +16750,12 @@
       </c>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C265" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D265" s="3" t="inlineStr">
@@ -16773,12 +16777,12 @@
       </c>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C266" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D266" s="3" t="inlineStr">
@@ -16800,12 +16804,12 @@
       </c>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C267" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D267" s="3" t="inlineStr">
@@ -16827,12 +16831,12 @@
       </c>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C268" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D268" s="3" t="inlineStr">
@@ -16854,12 +16858,12 @@
       </c>
       <c r="B269" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C269" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D269" s="3" t="inlineStr">
@@ -16881,12 +16885,12 @@
       </c>
       <c r="B270" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C270" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D270" s="3" t="inlineStr">
@@ -16908,12 +16912,12 @@
       </c>
       <c r="B271" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C271" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D271" s="3" t="inlineStr">
@@ -16935,12 +16939,12 @@
       </c>
       <c r="B272" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R4-11</t>
         </is>
       </c>
       <c r="C272" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
         </is>
       </c>
       <c r="D272" s="3" t="inlineStr">
@@ -16962,12 +16966,12 @@
       </c>
       <c r="B273" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R4-ISO</t>
         </is>
       </c>
       <c r="C273" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
         </is>
       </c>
       <c r="D273" s="3" t="inlineStr">
@@ -16989,12 +16993,12 @@
       </c>
       <c r="B274" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R5-01</t>
         </is>
       </c>
       <c r="C274" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
         </is>
       </c>
       <c r="D274" s="3" t="inlineStr">
@@ -17016,12 +17020,12 @@
       </c>
       <c r="B275" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R5-02</t>
         </is>
       </c>
       <c r="C275" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
         </is>
       </c>
       <c r="D275" s="3" t="inlineStr">
@@ -17043,12 +17047,12 @@
       </c>
       <c r="B276" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R5-03</t>
         </is>
       </c>
       <c r="C276" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
         </is>
       </c>
       <c r="D276" s="3" t="inlineStr">
@@ -17070,12 +17074,12 @@
       </c>
       <c r="B277" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R5-04</t>
         </is>
       </c>
       <c r="C277" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
         </is>
       </c>
       <c r="D277" s="3" t="inlineStr">
@@ -17097,12 +17101,12 @@
       </c>
       <c r="B278" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R5-05</t>
         </is>
       </c>
       <c r="C278" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
         </is>
       </c>
       <c r="D278" s="3" t="inlineStr">
@@ -17124,20 +17128,155 @@
       </c>
       <c r="B279" s="3" t="inlineStr">
         <is>
+          <t>E2E-R5-06</t>
+        </is>
+      </c>
+      <c r="C279" s="3" t="inlineStr">
+        <is>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+        </is>
+      </c>
+      <c r="D279" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E279" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B280" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-07</t>
+        </is>
+      </c>
+      <c r="C280" s="3" t="inlineStr">
+        <is>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+        </is>
+      </c>
+      <c r="D280" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E280" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B281" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-08</t>
+        </is>
+      </c>
+      <c r="C281" s="3" t="inlineStr">
+        <is>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+        </is>
+      </c>
+      <c r="D281" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E281" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B282" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-09</t>
+        </is>
+      </c>
+      <c r="C282" s="3" t="inlineStr">
+        <is>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+        </is>
+      </c>
+      <c r="D282" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E282" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B283" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C283" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D283" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E283" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B284" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C279" s="3" t="inlineStr">
+      <c r="C284" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D279" s="3" t="inlineStr">
+      <c r="D284" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E279" s="3" t="inlineStr">
+      <c r="E284" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
feat(web): Notion/Attio-style redesign with Library, document view, Announcements and Members; browser journeys E2E-R1-UI-07..10 (BPMS-031)
Owner-chosen direction: warm paper neutrals, full-bleed pages with a warm
icon sidebar, pastel tags and avatars, larger readable titles. Home is
action-first (acknowledgements, reviews and announcements with inline
buttons, a library table, activity, people). The Library has filters, an
Attio-style table and a New document dialog; documents render as a
readable page with properties, lifecycle actions (with step-up), version
history and an acknowledgement callout. Announcements and Members pages
are added. Token refresh is single-flight so concurrent callers no longer
trip refresh-reuse revocation. The sign-in page no longer scrolls.

Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E307" headerRowCount="1">
-  <autoFilter ref="A1:E307"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E311" headerRowCount="1">
+  <autoFilter ref="A1:E311"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -4582,7 +4582,7 @@
       <c r="N27" s="3" t="inlineStr"/>
       <c r="O27" s="3" t="inlineStr">
         <is>
-          <t>Web app slice 1: history router, API client (in-memory access token, silent refresh via HttpOnly cookie, RFC 9457 errors), session provider, Vite proxy (same-origin), sign-in with MFA (TOTP or recovery code), workspace chooser, app shell with workspace switcher menu, notification bell with unread count, permission-shaped navigation, Home, notifications inbox; design gallery moved to /design. E2E-R1-UI-01..05 (axe on every screen). Remaining: system console shell, ⌘K command palette, mobile bottom bar</t>
+          <t>Web app on the Notion/Attio direction (owner choice): warm paper palette in tokens (contrast-checked), full-bleed pages with a warm icon sidebar, workspace + account menus (persisted theme), action-first Home (acknowledgements, reviews, announcements with inline actions, library table, activity, people), Library (filters, Attio-style table, New document dialog), document reading view with properties, lifecycle actions (edit, submit, approve, request changes, publish with step-up, new version), acknowledgement callout, Announcements feed with read/ack, Members with invite dialog; split sign-in with product preview; single-flight token refresh. E2E-R1-UI-01..10 with axe. Remaining: ⌘K command palette (search API is ready), system console shell, mobile bottom bar</t>
         </is>
       </c>
     </row>
@@ -9647,7 +9647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E307"/>
+  <dimension ref="A1:E311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -15362,12 +15362,12 @@
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-01</t>
+          <t>E2E-R1-UI-07</t>
         </is>
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
+          <t>Author a policy in the browser: New document dialog → write content (headings, lists) → save → submit → publish; the library row shows Published; axe clean | FR-G04, docs/05 §3.2/§3.21</t>
         </is>
       </c>
       <c r="D212" s="3" t="inlineStr">
@@ -15389,12 +15389,12 @@
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-02</t>
+          <t>E2E-R1-UI-08</t>
         </is>
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
+          <t>A campaign task on Home leads to the document; “I acknowledge” records the acknowledgement (campaign progress +1) and the callout disappears | FR-AK01, docs/05 §3.1</t>
         </is>
       </c>
       <c r="D213" s="3" t="inlineStr">
@@ -15416,12 +15416,12 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-03</t>
+          <t>E2E-R1-UI-09</t>
         </is>
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
+          <t>Invite a colleague from Members with a role; the invitation appears in the table as Invited | FR-W01, docs/05 §3.14</t>
         </is>
       </c>
       <c r="D214" s="3" t="inlineStr">
@@ -15443,12 +15443,12 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-04</t>
+          <t>E2E-R1-UI-10</t>
         </is>
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
+          <t>Read and acknowledge a critical, pinned announcement in the feed | FR-AN04, docs/05 §3.23</t>
         </is>
       </c>
       <c r="D215" s="3" t="inlineStr">
@@ -15470,12 +15470,12 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-05</t>
+          <t>E2E-R1-CMP-01</t>
         </is>
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
+          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
@@ -15497,12 +15497,12 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-06</t>
+          <t>E2E-R1-CMP-02</t>
         </is>
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
+          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -15524,12 +15524,12 @@
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-07</t>
+          <t>E2E-R1-CMP-03</t>
         </is>
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
+          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
@@ -15551,12 +15551,12 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-01</t>
+          <t>E2E-R1-CMP-04</t>
         </is>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
+          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
         </is>
       </c>
       <c r="D219" s="3" t="inlineStr">
@@ -15578,12 +15578,12 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-02</t>
+          <t>E2E-R1-CMP-05</t>
         </is>
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
+          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
         </is>
       </c>
       <c r="D220" s="3" t="inlineStr">
@@ -15605,12 +15605,12 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-03</t>
+          <t>E2E-R1-CMP-06</t>
         </is>
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
+          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
         </is>
       </c>
       <c r="D221" s="3" t="inlineStr">
@@ -15632,12 +15632,12 @@
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-04</t>
+          <t>E2E-R1-CMP-07</t>
         </is>
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
+          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D222" s="3" t="inlineStr">
@@ -15659,12 +15659,12 @@
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-05</t>
+          <t>E2E-R1-ANN-01</t>
         </is>
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
+          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
         </is>
       </c>
       <c r="D223" s="3" t="inlineStr">
@@ -15686,12 +15686,12 @@
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-06</t>
+          <t>E2E-R1-ANN-02</t>
         </is>
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
+          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
         </is>
       </c>
       <c r="D224" s="3" t="inlineStr">
@@ -15713,12 +15713,12 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-01</t>
+          <t>E2E-R1-ANN-03</t>
         </is>
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
+          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
         </is>
       </c>
       <c r="D225" s="3" t="inlineStr">
@@ -15740,12 +15740,12 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-02</t>
+          <t>E2E-R1-ANN-04</t>
         </is>
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
+          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
         </is>
       </c>
       <c r="D226" s="3" t="inlineStr">
@@ -15767,12 +15767,12 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-03</t>
+          <t>E2E-R1-ANN-05</t>
         </is>
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
+          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D227" s="3" t="inlineStr">
@@ -15794,12 +15794,12 @@
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-01</t>
+          <t>E2E-R1-ANN-06</t>
         </is>
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
+          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
         </is>
       </c>
       <c r="D228" s="3" t="inlineStr">
@@ -15821,12 +15821,12 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-02</t>
+          <t>E2E-R1-SRCH-01</t>
         </is>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
+          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
@@ -15848,12 +15848,12 @@
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-03</t>
+          <t>E2E-R1-SRCH-02</t>
         </is>
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
+          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
         </is>
       </c>
       <c r="D230" s="3" t="inlineStr">
@@ -15875,12 +15875,12 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-04</t>
+          <t>E2E-R1-SRCH-03</t>
         </is>
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>Chain verify reports intact | FR-T02</t>
+          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
         </is>
       </c>
       <c r="D231" s="3" t="inlineStr">
@@ -15902,12 +15902,12 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-05</t>
+          <t>E2E-R1-AUDX-01</t>
         </is>
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
+          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
         </is>
       </c>
       <c r="D232" s="3" t="inlineStr">
@@ -15929,12 +15929,12 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-06</t>
+          <t>E2E-R1-AUDX-02</t>
         </is>
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
+          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
         </is>
       </c>
       <c r="D233" s="3" t="inlineStr">
@@ -15956,12 +15956,12 @@
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-AUDX-03</t>
         </is>
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
         </is>
       </c>
       <c r="D234" s="3" t="inlineStr">
@@ -15983,12 +15983,12 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-AUDX-04</t>
         </is>
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>Chain verify reports intact | FR-T02</t>
         </is>
       </c>
       <c r="D235" s="3" t="inlineStr">
@@ -16010,12 +16010,12 @@
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-AUDX-05</t>
         </is>
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
         </is>
       </c>
       <c r="D236" s="3" t="inlineStr">
@@ -16037,12 +16037,12 @@
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-AUDX-06</t>
         </is>
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
         </is>
       </c>
       <c r="D237" s="3" t="inlineStr">
@@ -16064,12 +16064,12 @@
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
         </is>
       </c>
       <c r="D238" s="3" t="inlineStr">
@@ -16091,12 +16091,12 @@
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D239" s="3" t="inlineStr">
@@ -16118,12 +16118,12 @@
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D240" s="3" t="inlineStr">
@@ -16145,12 +16145,12 @@
       </c>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
         </is>
       </c>
       <c r="D241" s="3" t="inlineStr">
@@ -16172,12 +16172,12 @@
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
         </is>
       </c>
       <c r="D242" s="3" t="inlineStr">
@@ -16199,12 +16199,12 @@
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D243" s="3" t="inlineStr">
@@ -16226,12 +16226,12 @@
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D244" s="3" t="inlineStr">
@@ -16253,12 +16253,12 @@
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
         </is>
       </c>
       <c r="D245" s="3" t="inlineStr">
@@ -16280,12 +16280,12 @@
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D246" s="3" t="inlineStr">
@@ -16307,12 +16307,12 @@
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D247" s="3" t="inlineStr">
@@ -16334,12 +16334,12 @@
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
@@ -16361,12 +16361,12 @@
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D249" s="3" t="inlineStr">
@@ -16388,12 +16388,12 @@
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
         </is>
       </c>
       <c r="D250" s="3" t="inlineStr">
@@ -16415,12 +16415,12 @@
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
         </is>
       </c>
       <c r="D251" s="3" t="inlineStr">
@@ -16442,12 +16442,12 @@
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
         </is>
       </c>
       <c r="D252" s="3" t="inlineStr">
@@ -16469,12 +16469,12 @@
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D253" s="3" t="inlineStr">
@@ -16496,12 +16496,12 @@
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
         </is>
       </c>
       <c r="D254" s="3" t="inlineStr">
@@ -16523,12 +16523,12 @@
       </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
         </is>
       </c>
       <c r="D255" s="3" t="inlineStr">
@@ -16550,12 +16550,12 @@
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C256" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D256" s="3" t="inlineStr">
@@ -16577,12 +16577,12 @@
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
         </is>
       </c>
       <c r="D257" s="3" t="inlineStr">
@@ -16604,12 +16604,12 @@
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C258" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D258" s="3" t="inlineStr">
@@ -16631,12 +16631,12 @@
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D259" s="3" t="inlineStr">
@@ -16658,12 +16658,12 @@
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D260" s="3" t="inlineStr">
@@ -16685,12 +16685,12 @@
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D261" s="3" t="inlineStr">
@@ -16712,12 +16712,12 @@
       </c>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C262" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D262" s="3" t="inlineStr">
@@ -16739,12 +16739,12 @@
       </c>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D263" s="3" t="inlineStr">
@@ -16766,12 +16766,12 @@
       </c>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C264" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D264" s="3" t="inlineStr">
@@ -16793,12 +16793,12 @@
       </c>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C265" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D265" s="3" t="inlineStr">
@@ -16820,12 +16820,12 @@
       </c>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C266" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D266" s="3" t="inlineStr">
@@ -16847,12 +16847,12 @@
       </c>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C267" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D267" s="3" t="inlineStr">
@@ -16874,12 +16874,12 @@
       </c>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C268" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D268" s="3" t="inlineStr">
@@ -16901,12 +16901,12 @@
       </c>
       <c r="B269" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C269" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D269" s="3" t="inlineStr">
@@ -16928,12 +16928,12 @@
       </c>
       <c r="B270" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C270" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D270" s="3" t="inlineStr">
@@ -16955,12 +16955,12 @@
       </c>
       <c r="B271" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C271" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D271" s="3" t="inlineStr">
@@ -16982,12 +16982,12 @@
       </c>
       <c r="B272" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C272" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D272" s="3" t="inlineStr">
@@ -17009,12 +17009,12 @@
       </c>
       <c r="B273" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C273" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D273" s="3" t="inlineStr">
@@ -17036,12 +17036,12 @@
       </c>
       <c r="B274" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C274" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D274" s="3" t="inlineStr">
@@ -17063,12 +17063,12 @@
       </c>
       <c r="B275" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C275" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D275" s="3" t="inlineStr">
@@ -17090,12 +17090,12 @@
       </c>
       <c r="B276" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C276" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D276" s="3" t="inlineStr">
@@ -17117,12 +17117,12 @@
       </c>
       <c r="B277" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C277" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D277" s="3" t="inlineStr">
@@ -17144,12 +17144,12 @@
       </c>
       <c r="B278" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C278" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D278" s="3" t="inlineStr">
@@ -17171,12 +17171,12 @@
       </c>
       <c r="B279" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C279" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D279" s="3" t="inlineStr">
@@ -17198,12 +17198,12 @@
       </c>
       <c r="B280" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C280" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D280" s="3" t="inlineStr">
@@ -17225,12 +17225,12 @@
       </c>
       <c r="B281" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C281" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D281" s="3" t="inlineStr">
@@ -17252,12 +17252,12 @@
       </c>
       <c r="B282" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C282" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D282" s="3" t="inlineStr">
@@ -17279,12 +17279,12 @@
       </c>
       <c r="B283" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C283" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D283" s="3" t="inlineStr">
@@ -17306,12 +17306,12 @@
       </c>
       <c r="B284" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C284" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D284" s="3" t="inlineStr">
@@ -17333,12 +17333,12 @@
       </c>
       <c r="B285" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C285" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D285" s="3" t="inlineStr">
@@ -17360,12 +17360,12 @@
       </c>
       <c r="B286" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C286" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D286" s="3" t="inlineStr">
@@ -17387,12 +17387,12 @@
       </c>
       <c r="B287" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C287" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D287" s="3" t="inlineStr">
@@ -17414,12 +17414,12 @@
       </c>
       <c r="B288" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C288" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D288" s="3" t="inlineStr">
@@ -17441,12 +17441,12 @@
       </c>
       <c r="B289" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C289" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D289" s="3" t="inlineStr">
@@ -17468,12 +17468,12 @@
       </c>
       <c r="B290" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C290" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D290" s="3" t="inlineStr">
@@ -17495,12 +17495,12 @@
       </c>
       <c r="B291" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C291" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D291" s="3" t="inlineStr">
@@ -17522,12 +17522,12 @@
       </c>
       <c r="B292" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C292" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D292" s="3" t="inlineStr">
@@ -17549,12 +17549,12 @@
       </c>
       <c r="B293" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C293" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D293" s="3" t="inlineStr">
@@ -17576,12 +17576,12 @@
       </c>
       <c r="B294" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C294" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D294" s="3" t="inlineStr">
@@ -17603,12 +17603,12 @@
       </c>
       <c r="B295" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C295" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D295" s="3" t="inlineStr">
@@ -17630,12 +17630,12 @@
       </c>
       <c r="B296" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C296" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D296" s="3" t="inlineStr">
@@ -17657,12 +17657,12 @@
       </c>
       <c r="B297" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C297" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D297" s="3" t="inlineStr">
@@ -17684,12 +17684,12 @@
       </c>
       <c r="B298" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C298" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D298" s="3" t="inlineStr">
@@ -17711,12 +17711,12 @@
       </c>
       <c r="B299" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R4-11</t>
         </is>
       </c>
       <c r="C299" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
         </is>
       </c>
       <c r="D299" s="3" t="inlineStr">
@@ -17738,12 +17738,12 @@
       </c>
       <c r="B300" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R4-ISO</t>
         </is>
       </c>
       <c r="C300" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
         </is>
       </c>
       <c r="D300" s="3" t="inlineStr">
@@ -17765,12 +17765,12 @@
       </c>
       <c r="B301" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R5-01</t>
         </is>
       </c>
       <c r="C301" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
         </is>
       </c>
       <c r="D301" s="3" t="inlineStr">
@@ -17792,12 +17792,12 @@
       </c>
       <c r="B302" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R5-02</t>
         </is>
       </c>
       <c r="C302" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
         </is>
       </c>
       <c r="D302" s="3" t="inlineStr">
@@ -17819,12 +17819,12 @@
       </c>
       <c r="B303" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R5-03</t>
         </is>
       </c>
       <c r="C303" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
         </is>
       </c>
       <c r="D303" s="3" t="inlineStr">
@@ -17846,12 +17846,12 @@
       </c>
       <c r="B304" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R5-04</t>
         </is>
       </c>
       <c r="C304" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
         </is>
       </c>
       <c r="D304" s="3" t="inlineStr">
@@ -17873,12 +17873,12 @@
       </c>
       <c r="B305" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R5-05</t>
         </is>
       </c>
       <c r="C305" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
         </is>
       </c>
       <c r="D305" s="3" t="inlineStr">
@@ -17900,12 +17900,12 @@
       </c>
       <c r="B306" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R5-06</t>
         </is>
       </c>
       <c r="C306" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
         </is>
       </c>
       <c r="D306" s="3" t="inlineStr">
@@ -17927,20 +17927,128 @@
       </c>
       <c r="B307" s="3" t="inlineStr">
         <is>
+          <t>E2E-R5-07</t>
+        </is>
+      </c>
+      <c r="C307" s="3" t="inlineStr">
+        <is>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+        </is>
+      </c>
+      <c r="D307" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E307" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B308" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-08</t>
+        </is>
+      </c>
+      <c r="C308" s="3" t="inlineStr">
+        <is>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+        </is>
+      </c>
+      <c r="D308" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E308" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B309" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-09</t>
+        </is>
+      </c>
+      <c r="C309" s="3" t="inlineStr">
+        <is>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+        </is>
+      </c>
+      <c r="D309" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E309" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B310" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C310" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D310" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E310" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B311" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C307" s="3" t="inlineStr">
+      <c r="C311" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D307" s="3" t="inlineStr">
+      <c r="D311" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E307" s="3" t="inlineStr">
+      <c r="E311" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
docs: library governance API, settings, E2E rows; tracker BPMS-043/044 done
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E311" headerRowCount="1">
-  <autoFilter ref="A1:E311"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E317" headerRowCount="1">
+  <autoFilter ref="A1:E317"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -5013,13 +5013,17 @@
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L34" s="3" t="inlineStr"/>
       <c r="M34" s="3" t="inlineStr"/>
       <c r="N34" s="3" t="inlineStr"/>
-      <c r="O34" s="3" t="inlineStr"/>
+      <c r="O34" s="3" t="inlineStr">
+        <is>
+          <t>procera-library diff module: block-level LCS alignment of SOP/policy content with word-level diffs inside changed blocks (removals and additions paired by position within an unmatched run, same block type → changed); GET /versions/{a}/diff/{b} (same artifact only); unit + property test (applying a diff always rebuilds the target) + E2E-R1-LIB-06. Process/form/rule bundle artifacts diff once their editors land (BPMS-050+).</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -5074,13 +5078,17 @@
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L35" s="3" t="inlineStr"/>
       <c r="M35" s="3" t="inlineStr"/>
       <c r="N35" s="3" t="inlineStr"/>
-      <c r="O35" s="3" t="inlineStr"/>
+      <c r="O35" s="3" t="inlineStr">
+        <is>
+          <t>Migration 0016: review cadence (per-artifact override or governance.review_cadence.default/.controlled), next_review_at set on every publish, recertification, worker flag of passed review dates (once; artifact.review_overdue.v1 → owner in-app notification), verification badge with governance.verification.validity expiry, change requests (open → accepted/declined/implemented, linked to the implementing version); all audited and in the audit contract; E2E-R1-LIB-07..10. Effective-date scheduling shipped with BPMS-040.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -9647,7 +9655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E311"/>
+  <dimension ref="A1:E317"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -15200,12 +15208,12 @@
       </c>
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-01</t>
+          <t>E2E-R1-LIB-06</t>
         </is>
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>Sign in through the browser (password + recovery code) lands on Home; navigation is permission-shaped with the current page marked; axe clean on sign-in and Home; reload keeps the session | docs/05 §2.1, §3.1, WCAG 2.2 AA</t>
+          <t>Semantic diff between two versions: one changed block with word-level detail, one added list, unchanged blocks kept; the reverse direction mirrors it; versions of different artifacts → 422; members may compare; another workspace gets 404 | BPMS-043, FR-G05</t>
         </is>
       </c>
       <c r="D206" s="3" t="inlineStr">
@@ -15227,12 +15235,12 @@
       </c>
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-02</t>
+          <t>E2E-R1-LIB-07</t>
         </is>
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>Wrong password and wrong code produce clear, non-revealing messages (role=alert); axe clean | docs/06 §3, WCAG 3.3.1</t>
+          <t>Publishing sets `next_review_at = published + 365 d` (standard); a per-artifact cadence of 20 days moves it and makes it `due_soon`; 0 → 422; `null` restores the default; an unpublished artifact cannot be recertified (409) | BPMS-044, FR-G07, FX-G01</t>
         </is>
       </c>
       <c r="D207" s="3" t="inlineStr">
@@ -15254,12 +15262,12 @@
       </c>
       <c r="B208" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-03</t>
+          <t>E2E-R1-LIB-08</t>
         </is>
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>With several workspaces the chooser appears; choosing one and switching from the header changes the context and the navigation (no Admin for a plain member) | docs/05 §2.1 workspace switcher</t>
+          <t>A passed review date reads `overdue` immediately; the worker flags it once (two drains) and the owner receives one `review_overdue` notification linking the document; recertifying clears the flag and starts a new period; both are audited | BPMS-044, FR-G07, FX-G01</t>
         </is>
       </c>
       <c r="D208" s="3" t="inlineStr">
@@ -15281,12 +15289,12 @@
       </c>
       <c r="B209" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-04</t>
+          <t>E2E-R1-LIB-09</t>
         </is>
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>The bell announces the unread count; the inbox lists the "joined" notification; mark all as read | FR-N01</t>
+          <t>Verification lasts `governance.verification.validity` (90 d) and expires on its own; members cannot verify (403); removing it twice → 409 | BPMS-044, FX-G02</t>
         </is>
       </c>
       <c r="D209" s="3" t="inlineStr">
@@ -15308,12 +15316,12 @@
       </c>
       <c r="B210" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-05</t>
+          <t>E2E-R1-LIB-10</t>
         </is>
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>Sign out returns to sign-in; reloading stays signed out | docs/06 §3</t>
+          <t>Change requests: a member proposes (blank title 422) but cannot resolve (403); declining needs a reason; accepted → implemented by a version of the same artifact (another artifact's version 422); resolved requests are final (409); list filters by state | BPMS-044, FR-G05</t>
         </is>
       </c>
       <c r="D210" s="3" t="inlineStr">
@@ -15335,12 +15343,12 @@
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-06</t>
+          <t>E2E-R1-UI-01</t>
         </is>
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>Theme switched from the account menu persists across reload; dark theme passes axe | docs/05 §7, WCAG 2.2 AA</t>
+          <t>Sign in through the browser (password + recovery code) lands on Home; navigation is permission-shaped with the current page marked; axe clean on sign-in and Home; reload keeps the session | docs/05 §2.1, §3.1, WCAG 2.2 AA</t>
         </is>
       </c>
       <c r="D211" s="3" t="inlineStr">
@@ -15362,12 +15370,12 @@
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-07</t>
+          <t>E2E-R1-UI-02</t>
         </is>
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>Author a policy in the browser: New document dialog → write content (headings, lists) → save → submit → publish; the library row shows Published; axe clean | FR-G04, docs/05 §3.2/§3.21</t>
+          <t>Wrong password and wrong code produce clear, non-revealing messages (role=alert); axe clean | docs/06 §3, WCAG 3.3.1</t>
         </is>
       </c>
       <c r="D212" s="3" t="inlineStr">
@@ -15389,12 +15397,12 @@
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-08</t>
+          <t>E2E-R1-UI-03</t>
         </is>
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>A campaign task on Home leads to the document; “I acknowledge” records the acknowledgement (campaign progress +1) and the callout disappears | FR-AK01, docs/05 §3.1</t>
+          <t>With several workspaces the chooser appears; choosing one and switching from the header changes the context and the navigation (no Admin for a plain member) | docs/05 §2.1 workspace switcher</t>
         </is>
       </c>
       <c r="D213" s="3" t="inlineStr">
@@ -15416,12 +15424,12 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-09</t>
+          <t>E2E-R1-UI-04</t>
         </is>
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>Invite a colleague from Members with a role; the invitation appears in the table as Invited | FR-W01, docs/05 §3.14</t>
+          <t>The bell announces the unread count; the inbox lists the "joined" notification; mark all as read | FR-N01</t>
         </is>
       </c>
       <c r="D214" s="3" t="inlineStr">
@@ -15443,12 +15451,12 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-10</t>
+          <t>E2E-R1-UI-05</t>
         </is>
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>Read and acknowledge a critical, pinned announcement in the feed | FR-AN04, docs/05 §3.23</t>
+          <t>Sign out returns to sign-in; reloading stays signed out | docs/06 §3</t>
         </is>
       </c>
       <c r="D215" s="3" t="inlineStr">
@@ -15470,12 +15478,12 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-01</t>
+          <t>E2E-R1-UI-06</t>
         </is>
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
+          <t>Theme switched from the account menu persists across reload; dark theme passes axe | docs/05 §7, WCAG 2.2 AA</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
@@ -15497,12 +15505,12 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-02</t>
+          <t>E2E-R1-UI-07</t>
         </is>
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
+          <t>Author a policy in the browser: New document dialog → write content (headings, lists) → save → submit → publish; the library row shows Published; axe clean | FR-G04, docs/05 §3.2/§3.21</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -15524,12 +15532,12 @@
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-03</t>
+          <t>E2E-R1-UI-08</t>
         </is>
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
+          <t>A campaign task on Home leads to the document; “I acknowledge” records the acknowledgement (campaign progress +1) and the callout disappears | FR-AK01, docs/05 §3.1</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
@@ -15551,12 +15559,12 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-04</t>
+          <t>E2E-R1-UI-09</t>
         </is>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
+          <t>Invite a colleague from Members with a role; the invitation appears in the table as Invited | FR-W01, docs/05 §3.14</t>
         </is>
       </c>
       <c r="D219" s="3" t="inlineStr">
@@ -15578,12 +15586,12 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-05</t>
+          <t>E2E-R1-UI-10</t>
         </is>
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
+          <t>Read and acknowledge a critical, pinned announcement in the feed | FR-AN04, docs/05 §3.23</t>
         </is>
       </c>
       <c r="D220" s="3" t="inlineStr">
@@ -15605,12 +15613,12 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-06</t>
+          <t>E2E-R1-UI-11</t>
         </is>
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
+          <t>An admin without two-step verification is guided through setup (QR + key, confirm a code, recovery codes) and then signs in with MFA and lands on Home | docs/06 §3, docs/20 §2.3</t>
         </is>
       </c>
       <c r="D221" s="3" t="inlineStr">
@@ -15632,12 +15640,12 @@
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-07</t>
+          <t>E2E-R1-CMP-01</t>
         </is>
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
+          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
         </is>
       </c>
       <c r="D222" s="3" t="inlineStr">
@@ -15659,12 +15667,12 @@
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-01</t>
+          <t>E2E-R1-CMP-02</t>
         </is>
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
+          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
         </is>
       </c>
       <c r="D223" s="3" t="inlineStr">
@@ -15686,12 +15694,12 @@
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-02</t>
+          <t>E2E-R1-CMP-03</t>
         </is>
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
+          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
         </is>
       </c>
       <c r="D224" s="3" t="inlineStr">
@@ -15713,12 +15721,12 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-03</t>
+          <t>E2E-R1-CMP-04</t>
         </is>
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
+          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
         </is>
       </c>
       <c r="D225" s="3" t="inlineStr">
@@ -15740,12 +15748,12 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-04</t>
+          <t>E2E-R1-CMP-05</t>
         </is>
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
+          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
         </is>
       </c>
       <c r="D226" s="3" t="inlineStr">
@@ -15767,12 +15775,12 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-05</t>
+          <t>E2E-R1-CMP-06</t>
         </is>
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
+          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
         </is>
       </c>
       <c r="D227" s="3" t="inlineStr">
@@ -15794,12 +15802,12 @@
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-06</t>
+          <t>E2E-R1-CMP-07</t>
         </is>
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
+          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D228" s="3" t="inlineStr">
@@ -15821,12 +15829,12 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-01</t>
+          <t>E2E-R1-ANN-01</t>
         </is>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
+          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
@@ -15848,12 +15856,12 @@
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-02</t>
+          <t>E2E-R1-ANN-02</t>
         </is>
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
+          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
         </is>
       </c>
       <c r="D230" s="3" t="inlineStr">
@@ -15875,12 +15883,12 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-03</t>
+          <t>E2E-R1-ANN-03</t>
         </is>
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
+          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
         </is>
       </c>
       <c r="D231" s="3" t="inlineStr">
@@ -15902,12 +15910,12 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-01</t>
+          <t>E2E-R1-ANN-04</t>
         </is>
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
+          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
         </is>
       </c>
       <c r="D232" s="3" t="inlineStr">
@@ -15929,12 +15937,12 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-02</t>
+          <t>E2E-R1-ANN-05</t>
         </is>
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
+          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D233" s="3" t="inlineStr">
@@ -15956,12 +15964,12 @@
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-03</t>
+          <t>E2E-R1-ANN-06</t>
         </is>
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
+          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
         </is>
       </c>
       <c r="D234" s="3" t="inlineStr">
@@ -15983,12 +15991,12 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-04</t>
+          <t>E2E-R1-SRCH-01</t>
         </is>
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>Chain verify reports intact | FR-T02</t>
+          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
         </is>
       </c>
       <c r="D235" s="3" t="inlineStr">
@@ -16010,12 +16018,12 @@
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-05</t>
+          <t>E2E-R1-SRCH-02</t>
         </is>
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
+          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
         </is>
       </c>
       <c r="D236" s="3" t="inlineStr">
@@ -16037,12 +16045,12 @@
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-06</t>
+          <t>E2E-R1-SRCH-03</t>
         </is>
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
+          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
         </is>
       </c>
       <c r="D237" s="3" t="inlineStr">
@@ -16064,12 +16072,12 @@
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-AUDX-01</t>
         </is>
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
         </is>
       </c>
       <c r="D238" s="3" t="inlineStr">
@@ -16091,12 +16099,12 @@
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-AUDX-02</t>
         </is>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
         </is>
       </c>
       <c r="D239" s="3" t="inlineStr">
@@ -16118,12 +16126,12 @@
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-AUDX-03</t>
         </is>
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
         </is>
       </c>
       <c r="D240" s="3" t="inlineStr">
@@ -16145,12 +16153,12 @@
       </c>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-AUDX-04</t>
         </is>
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>Chain verify reports intact | FR-T02</t>
         </is>
       </c>
       <c r="D241" s="3" t="inlineStr">
@@ -16172,12 +16180,12 @@
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-AUDX-05</t>
         </is>
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
         </is>
       </c>
       <c r="D242" s="3" t="inlineStr">
@@ -16199,12 +16207,12 @@
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-AUDX-06</t>
         </is>
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
         </is>
       </c>
       <c r="D243" s="3" t="inlineStr">
@@ -16226,12 +16234,12 @@
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
         </is>
       </c>
       <c r="D244" s="3" t="inlineStr">
@@ -16253,12 +16261,12 @@
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D245" s="3" t="inlineStr">
@@ -16280,12 +16288,12 @@
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D246" s="3" t="inlineStr">
@@ -16307,12 +16315,12 @@
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
         </is>
       </c>
       <c r="D247" s="3" t="inlineStr">
@@ -16334,12 +16342,12 @@
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
@@ -16361,12 +16369,12 @@
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D249" s="3" t="inlineStr">
@@ -16388,12 +16396,12 @@
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D250" s="3" t="inlineStr">
@@ -16415,12 +16423,12 @@
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
         </is>
       </c>
       <c r="D251" s="3" t="inlineStr">
@@ -16442,12 +16450,12 @@
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D252" s="3" t="inlineStr">
@@ -16469,12 +16477,12 @@
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D253" s="3" t="inlineStr">
@@ -16496,12 +16504,12 @@
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D254" s="3" t="inlineStr">
@@ -16523,12 +16531,12 @@
       </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D255" s="3" t="inlineStr">
@@ -16550,12 +16558,12 @@
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C256" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
         </is>
       </c>
       <c r="D256" s="3" t="inlineStr">
@@ -16577,12 +16585,12 @@
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
         </is>
       </c>
       <c r="D257" s="3" t="inlineStr">
@@ -16604,12 +16612,12 @@
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C258" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
         </is>
       </c>
       <c r="D258" s="3" t="inlineStr">
@@ -16631,12 +16639,12 @@
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D259" s="3" t="inlineStr">
@@ -16658,12 +16666,12 @@
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
         </is>
       </c>
       <c r="D260" s="3" t="inlineStr">
@@ -16685,12 +16693,12 @@
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
         </is>
       </c>
       <c r="D261" s="3" t="inlineStr">
@@ -16712,12 +16720,12 @@
       </c>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C262" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D262" s="3" t="inlineStr">
@@ -16739,12 +16747,12 @@
       </c>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
         </is>
       </c>
       <c r="D263" s="3" t="inlineStr">
@@ -16766,12 +16774,12 @@
       </c>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C264" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D264" s="3" t="inlineStr">
@@ -16793,12 +16801,12 @@
       </c>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C265" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D265" s="3" t="inlineStr">
@@ -16820,12 +16828,12 @@
       </c>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C266" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D266" s="3" t="inlineStr">
@@ -16847,12 +16855,12 @@
       </c>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C267" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D267" s="3" t="inlineStr">
@@ -16874,12 +16882,12 @@
       </c>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C268" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D268" s="3" t="inlineStr">
@@ -16901,12 +16909,12 @@
       </c>
       <c r="B269" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C269" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D269" s="3" t="inlineStr">
@@ -16928,12 +16936,12 @@
       </c>
       <c r="B270" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C270" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D270" s="3" t="inlineStr">
@@ -16955,12 +16963,12 @@
       </c>
       <c r="B271" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C271" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D271" s="3" t="inlineStr">
@@ -16982,12 +16990,12 @@
       </c>
       <c r="B272" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C272" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D272" s="3" t="inlineStr">
@@ -17009,12 +17017,12 @@
       </c>
       <c r="B273" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C273" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D273" s="3" t="inlineStr">
@@ -17036,12 +17044,12 @@
       </c>
       <c r="B274" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C274" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D274" s="3" t="inlineStr">
@@ -17063,12 +17071,12 @@
       </c>
       <c r="B275" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C275" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D275" s="3" t="inlineStr">
@@ -17090,12 +17098,12 @@
       </c>
       <c r="B276" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C276" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D276" s="3" t="inlineStr">
@@ -17117,12 +17125,12 @@
       </c>
       <c r="B277" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C277" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D277" s="3" t="inlineStr">
@@ -17144,12 +17152,12 @@
       </c>
       <c r="B278" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C278" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D278" s="3" t="inlineStr">
@@ -17171,12 +17179,12 @@
       </c>
       <c r="B279" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C279" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D279" s="3" t="inlineStr">
@@ -17198,12 +17206,12 @@
       </c>
       <c r="B280" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C280" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D280" s="3" t="inlineStr">
@@ -17225,12 +17233,12 @@
       </c>
       <c r="B281" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C281" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D281" s="3" t="inlineStr">
@@ -17252,12 +17260,12 @@
       </c>
       <c r="B282" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C282" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D282" s="3" t="inlineStr">
@@ -17279,12 +17287,12 @@
       </c>
       <c r="B283" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C283" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D283" s="3" t="inlineStr">
@@ -17306,12 +17314,12 @@
       </c>
       <c r="B284" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C284" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D284" s="3" t="inlineStr">
@@ -17333,12 +17341,12 @@
       </c>
       <c r="B285" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C285" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D285" s="3" t="inlineStr">
@@ -17360,12 +17368,12 @@
       </c>
       <c r="B286" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C286" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D286" s="3" t="inlineStr">
@@ -17387,12 +17395,12 @@
       </c>
       <c r="B287" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C287" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D287" s="3" t="inlineStr">
@@ -17414,12 +17422,12 @@
       </c>
       <c r="B288" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C288" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D288" s="3" t="inlineStr">
@@ -17441,12 +17449,12 @@
       </c>
       <c r="B289" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C289" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D289" s="3" t="inlineStr">
@@ -17468,12 +17476,12 @@
       </c>
       <c r="B290" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C290" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D290" s="3" t="inlineStr">
@@ -17495,12 +17503,12 @@
       </c>
       <c r="B291" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C291" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D291" s="3" t="inlineStr">
@@ -17522,12 +17530,12 @@
       </c>
       <c r="B292" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C292" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D292" s="3" t="inlineStr">
@@ -17549,12 +17557,12 @@
       </c>
       <c r="B293" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C293" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D293" s="3" t="inlineStr">
@@ -17576,12 +17584,12 @@
       </c>
       <c r="B294" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C294" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D294" s="3" t="inlineStr">
@@ -17603,12 +17611,12 @@
       </c>
       <c r="B295" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C295" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D295" s="3" t="inlineStr">
@@ -17630,12 +17638,12 @@
       </c>
       <c r="B296" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C296" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D296" s="3" t="inlineStr">
@@ -17657,12 +17665,12 @@
       </c>
       <c r="B297" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C297" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D297" s="3" t="inlineStr">
@@ -17684,12 +17692,12 @@
       </c>
       <c r="B298" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C298" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D298" s="3" t="inlineStr">
@@ -17711,12 +17719,12 @@
       </c>
       <c r="B299" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C299" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D299" s="3" t="inlineStr">
@@ -17738,12 +17746,12 @@
       </c>
       <c r="B300" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C300" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D300" s="3" t="inlineStr">
@@ -17765,12 +17773,12 @@
       </c>
       <c r="B301" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C301" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D301" s="3" t="inlineStr">
@@ -17792,12 +17800,12 @@
       </c>
       <c r="B302" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C302" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D302" s="3" t="inlineStr">
@@ -17819,12 +17827,12 @@
       </c>
       <c r="B303" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C303" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D303" s="3" t="inlineStr">
@@ -17846,12 +17854,12 @@
       </c>
       <c r="B304" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C304" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D304" s="3" t="inlineStr">
@@ -17873,12 +17881,12 @@
       </c>
       <c r="B305" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R4-11</t>
         </is>
       </c>
       <c r="C305" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
         </is>
       </c>
       <c r="D305" s="3" t="inlineStr">
@@ -17900,12 +17908,12 @@
       </c>
       <c r="B306" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R4-ISO</t>
         </is>
       </c>
       <c r="C306" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
         </is>
       </c>
       <c r="D306" s="3" t="inlineStr">
@@ -17927,12 +17935,12 @@
       </c>
       <c r="B307" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R5-01</t>
         </is>
       </c>
       <c r="C307" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
         </is>
       </c>
       <c r="D307" s="3" t="inlineStr">
@@ -17954,12 +17962,12 @@
       </c>
       <c r="B308" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R5-02</t>
         </is>
       </c>
       <c r="C308" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
         </is>
       </c>
       <c r="D308" s="3" t="inlineStr">
@@ -17981,12 +17989,12 @@
       </c>
       <c r="B309" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R5-03</t>
         </is>
       </c>
       <c r="C309" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
         </is>
       </c>
       <c r="D309" s="3" t="inlineStr">
@@ -18008,12 +18016,12 @@
       </c>
       <c r="B310" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R5-04</t>
         </is>
       </c>
       <c r="C310" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
         </is>
       </c>
       <c r="D310" s="3" t="inlineStr">
@@ -18035,20 +18043,182 @@
       </c>
       <c r="B311" s="3" t="inlineStr">
         <is>
+          <t>E2E-R5-05</t>
+        </is>
+      </c>
+      <c r="C311" s="3" t="inlineStr">
+        <is>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+        </is>
+      </c>
+      <c r="D311" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E311" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B312" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-06</t>
+        </is>
+      </c>
+      <c r="C312" s="3" t="inlineStr">
+        <is>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+        </is>
+      </c>
+      <c r="D312" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E312" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B313" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-07</t>
+        </is>
+      </c>
+      <c r="C313" s="3" t="inlineStr">
+        <is>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+        </is>
+      </c>
+      <c r="D313" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E313" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B314" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-08</t>
+        </is>
+      </c>
+      <c r="C314" s="3" t="inlineStr">
+        <is>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+        </is>
+      </c>
+      <c r="D314" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E314" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B315" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-09</t>
+        </is>
+      </c>
+      <c r="C315" s="3" t="inlineStr">
+        <is>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+        </is>
+      </c>
+      <c r="D315" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E315" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B316" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C316" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D316" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E316" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B317" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C311" s="3" t="inlineStr">
+      <c r="C317" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D311" s="3" t="inlineStr">
+      <c r="D317" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E311" s="3" t="inlineStr">
+      <c r="E317" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
docs: policy portal API, A-14 visibility, E2E rows; tracker 043-045 in progress until UI E2E ships
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -197,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E14" headerRowCount="1">
-  <autoFilter ref="A1:E14"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E15" headerRowCount="1">
+  <autoFilter ref="A1:E15"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Source"/>
     <tableColumn id="2" name="ID"/>
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E317" headerRowCount="1">
-  <autoFilter ref="A1:E317"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E320" headerRowCount="1">
+  <autoFilter ref="A1:E320"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -1393,7 +1393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1778,6 +1778,33 @@
       <c r="E14" s="3" t="inlineStr">
         <is>
           <t>Count escalation from the due date; add `policy:acknowledge` to docs/12 §5</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>A-14</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Library visibility (BPMS-045): members who can only `view` a kind (no `create`/`edit_draft`/`review`/`approve`/`publish`) see an artifact only once it has a published version, and only its published history (published, deprecated, retired), never drafts, reviews or scheduled versions. This matches the UI promise "Nobody else sees it until it's published". A `restricted` policy is additionally hidden (404, also in search) from readers outside its applicability. Authors and admins see everything</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Product-owner review; pilot feedback</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Show drafts to readers through explicit visibility settings (docs/12 §8)</t>
         </is>
       </c>
     </row>
@@ -5013,7 +5040,7 @@
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L34" s="3" t="inlineStr"/>
@@ -5021,7 +5048,7 @@
       <c r="N34" s="3" t="inlineStr"/>
       <c r="O34" s="3" t="inlineStr">
         <is>
-          <t>procera-library diff module: block-level LCS alignment of SOP/policy content with word-level diffs inside changed blocks (removals and additions paired by position within an unmatched run, same block type → changed); GET /versions/{a}/diff/{b} (same artifact only); unit + property test (applying a diff always rebuilds the target) + E2E-R1-LIB-06. Process/form/rule bundle artifacts diff once their editors land (BPMS-050+).</t>
+          <t>API done (UI pending: compare view + UI E2E). procera-library diff module: block-level LCS alignment of SOP/policy content with word-level diffs inside changed blocks (removals and additions paired by position within an unmatched run, same block type → changed); GET /versions/{a}/diff/{b} (same artifact only); unit + property test (applying a diff always rebuilds the target) + E2E-R1-LIB-06. Process/form/rule bundle artifacts diff once their editors land (BPMS-050+).</t>
         </is>
       </c>
     </row>
@@ -5078,7 +5105,7 @@
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L35" s="3" t="inlineStr"/>
@@ -5086,7 +5113,7 @@
       <c r="N35" s="3" t="inlineStr"/>
       <c r="O35" s="3" t="inlineStr">
         <is>
-          <t>Migration 0016: review cadence (per-artifact override or governance.review_cadence.default/.controlled), next_review_at set on every publish, recertification, worker flag of passed review dates (once; artifact.review_overdue.v1 → owner in-app notification), verification badge with governance.verification.validity expiry, change requests (open → accepted/declined/implemented, linked to the implementing version); all audited and in the audit contract; E2E-R1-LIB-07..10. Effective-date scheduling shipped with BPMS-040.</t>
+          <t>API done (UI pending: governance panel, change requests + UI E2E). Migration 0016: review cadence (per-artifact override or governance.review_cadence.default/.controlled), next_review_at set on every publish, recertification, worker flag of passed review dates (once; artifact.review_overdue.v1 → owner in-app notification), verification badge with governance.verification.validity expiry, change requests (open → accepted/declined/implemented, linked to the implementing version); all audited and in the audit contract; E2E-R1-LIB-07..10. Effective-date scheduling shipped with BPMS-040.</t>
         </is>
       </c>
     </row>
@@ -5143,13 +5170,17 @@
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L36" s="3" t="inlineStr"/>
       <c r="M36" s="3" t="inlineStr"/>
       <c r="N36" s="3" t="inlineStr"/>
-      <c r="O36" s="3" t="inlineStr"/>
+      <c r="O36" s="3" t="inlineStr">
+        <is>
+          <t>API done (UI pending: Policies portal page, applicability control + UI E2E). Migration 0017: policy category, applicability (audience; NULL = everyone) and restricted flag; procera_audience_contains SQL twin of the audience resolver; reader visibility (A-14): view-only readers see published history only, restricted policies hidden outside their applicability in lists, reads, diff, change requests and search; PUT /artifacts/{id}/applicability (audited); GET /me/policies portal with what-changed summaries vs the previous published version, text + category filters; E2E-R1-POL-01..03. Remaining: re-acknowledgement on major publish (FR-PL03), superseded watermark in exports.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -9655,7 +9686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E317"/>
+  <dimension ref="A1:E320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -15343,12 +15374,12 @@
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-01</t>
+          <t>E2E-R1-POL-01</t>
         </is>
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>Sign in through the browser (password + recovery code) lands on Home; navigation is permission-shaped with the current page marked; axe clean on sign-in and Home; reload keeps the session | docs/05 §2.1, §3.1, WCAG 2.2 AA</t>
+          <t>Readers never see drafts: absent from lists, reads and search until published; a later draft stays hidden (version 404, diff 404, versions list shows v1 only); authors see drafts in search | BPMS-045, A-14</t>
         </is>
       </c>
       <c r="D211" s="3" t="inlineStr">
@@ -15370,12 +15401,12 @@
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-02</t>
+          <t>E2E-R1-POL-02</t>
         </is>
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>Wrong password and wrong code produce clear, non-revealing messages (role=alert); axe clean | docs/06 §3, WCAG 3.3.1</t>
+          <t>Applicability: empty audience or restricted without one → 422; members cannot set it (403); a restricted policy is hidden from members outside its group in lists, reads, search, the portal and change requests (404), and shown to those inside; an unrestricted one is listed for everyone but only "applicable" to its audience | BPMS-045, FR-PL01/PL02</t>
         </is>
       </c>
       <c r="D212" s="3" t="inlineStr">
@@ -15397,12 +15428,12 @@
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-03</t>
+          <t>E2E-R1-POL-03</t>
         </is>
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>With several workspaces the chooser appears; choosing one and switching from the header changes the context and the navigation (no Admin for a plain member) | docs/05 §2.1 workspace switcher</t>
+          <t>The portal lists published policies that apply to the member (no drafts), ordered by category, with what changed since the previous version (added/changed counts, reason) and text/category filters | BPMS-045, FR-PL02</t>
         </is>
       </c>
       <c r="D213" s="3" t="inlineStr">
@@ -15424,12 +15455,12 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-04</t>
+          <t>E2E-R1-UI-01</t>
         </is>
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>The bell announces the unread count; the inbox lists the "joined" notification; mark all as read | FR-N01</t>
+          <t>Sign in through the browser (password + recovery code) lands on Home; navigation is permission-shaped with the current page marked; axe clean on sign-in and Home; reload keeps the session | docs/05 §2.1, §3.1, WCAG 2.2 AA</t>
         </is>
       </c>
       <c r="D214" s="3" t="inlineStr">
@@ -15451,12 +15482,12 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-05</t>
+          <t>E2E-R1-UI-02</t>
         </is>
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>Sign out returns to sign-in; reloading stays signed out | docs/06 §3</t>
+          <t>Wrong password and wrong code produce clear, non-revealing messages (role=alert); axe clean | docs/06 §3, WCAG 3.3.1</t>
         </is>
       </c>
       <c r="D215" s="3" t="inlineStr">
@@ -15478,12 +15509,12 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-06</t>
+          <t>E2E-R1-UI-03</t>
         </is>
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>Theme switched from the account menu persists across reload; dark theme passes axe | docs/05 §7, WCAG 2.2 AA</t>
+          <t>With several workspaces the chooser appears; choosing one and switching from the header changes the context and the navigation (no Admin for a plain member) | docs/05 §2.1 workspace switcher</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
@@ -15505,12 +15536,12 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-07</t>
+          <t>E2E-R1-UI-04</t>
         </is>
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Author a policy in the browser: New document dialog → write content (headings, lists) → save → submit → publish; the library row shows Published; axe clean | FR-G04, docs/05 §3.2/§3.21</t>
+          <t>The bell announces the unread count; the inbox lists the "joined" notification; mark all as read | FR-N01</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -15532,12 +15563,12 @@
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-08</t>
+          <t>E2E-R1-UI-05</t>
         </is>
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>A campaign task on Home leads to the document; “I acknowledge” records the acknowledgement (campaign progress +1) and the callout disappears | FR-AK01, docs/05 §3.1</t>
+          <t>Sign out returns to sign-in; reloading stays signed out | docs/06 §3</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
@@ -15559,12 +15590,12 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-09</t>
+          <t>E2E-R1-UI-06</t>
         </is>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Invite a colleague from Members with a role; the invitation appears in the table as Invited | FR-W01, docs/05 §3.14</t>
+          <t>Theme switched from the account menu persists across reload; dark theme passes axe | docs/05 §7, WCAG 2.2 AA</t>
         </is>
       </c>
       <c r="D219" s="3" t="inlineStr">
@@ -15586,12 +15617,12 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-10</t>
+          <t>E2E-R1-UI-07</t>
         </is>
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Read and acknowledge a critical, pinned announcement in the feed | FR-AN04, docs/05 §3.23</t>
+          <t>Author a policy in the browser: New document dialog → write content (headings, lists) → save → submit → publish; the library row shows Published; axe clean | FR-G04, docs/05 §3.2/§3.21</t>
         </is>
       </c>
       <c r="D220" s="3" t="inlineStr">
@@ -15613,12 +15644,12 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-11</t>
+          <t>E2E-R1-UI-08</t>
         </is>
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>An admin without two-step verification is guided through setup (QR + key, confirm a code, recovery codes) and then signs in with MFA and lands on Home | docs/06 §3, docs/20 §2.3</t>
+          <t>A campaign task on Home leads to the document; “I acknowledge” records the acknowledgement (campaign progress +1) and the callout disappears | FR-AK01, docs/05 §3.1</t>
         </is>
       </c>
       <c r="D221" s="3" t="inlineStr">
@@ -15640,12 +15671,12 @@
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-01</t>
+          <t>E2E-R1-UI-09</t>
         </is>
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
+          <t>Invite a colleague from Members with a role; the invitation appears in the table as Invited | FR-W01, docs/05 §3.14</t>
         </is>
       </c>
       <c r="D222" s="3" t="inlineStr">
@@ -15667,12 +15698,12 @@
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-02</t>
+          <t>E2E-R1-UI-10</t>
         </is>
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
+          <t>Read and acknowledge a critical, pinned announcement in the feed | FR-AN04, docs/05 §3.23</t>
         </is>
       </c>
       <c r="D223" s="3" t="inlineStr">
@@ -15694,12 +15725,12 @@
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-03</t>
+          <t>E2E-R1-UI-11</t>
         </is>
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
+          <t>An admin without two-step verification is guided through setup (QR + key, confirm a code, recovery codes) and then signs in with MFA and lands on Home | docs/06 §3, docs/20 §2.3</t>
         </is>
       </c>
       <c r="D224" s="3" t="inlineStr">
@@ -15721,12 +15752,12 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-04</t>
+          <t>E2E-R1-CMP-01</t>
         </is>
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
+          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
         </is>
       </c>
       <c r="D225" s="3" t="inlineStr">
@@ -15748,12 +15779,12 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-05</t>
+          <t>E2E-R1-CMP-02</t>
         </is>
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
+          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
         </is>
       </c>
       <c r="D226" s="3" t="inlineStr">
@@ -15775,12 +15806,12 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-06</t>
+          <t>E2E-R1-CMP-03</t>
         </is>
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
+          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
         </is>
       </c>
       <c r="D227" s="3" t="inlineStr">
@@ -15802,12 +15833,12 @@
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-07</t>
+          <t>E2E-R1-CMP-04</t>
         </is>
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
+          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
         </is>
       </c>
       <c r="D228" s="3" t="inlineStr">
@@ -15829,12 +15860,12 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-01</t>
+          <t>E2E-R1-CMP-05</t>
         </is>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
+          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
@@ -15856,12 +15887,12 @@
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-02</t>
+          <t>E2E-R1-CMP-06</t>
         </is>
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
+          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
         </is>
       </c>
       <c r="D230" s="3" t="inlineStr">
@@ -15883,12 +15914,12 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-03</t>
+          <t>E2E-R1-CMP-07</t>
         </is>
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
+          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D231" s="3" t="inlineStr">
@@ -15910,12 +15941,12 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-04</t>
+          <t>E2E-R1-ANN-01</t>
         </is>
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
+          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
         </is>
       </c>
       <c r="D232" s="3" t="inlineStr">
@@ -15937,12 +15968,12 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-05</t>
+          <t>E2E-R1-ANN-02</t>
         </is>
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
+          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
         </is>
       </c>
       <c r="D233" s="3" t="inlineStr">
@@ -15964,12 +15995,12 @@
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-06</t>
+          <t>E2E-R1-ANN-03</t>
         </is>
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
+          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
         </is>
       </c>
       <c r="D234" s="3" t="inlineStr">
@@ -15991,12 +16022,12 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-01</t>
+          <t>E2E-R1-ANN-04</t>
         </is>
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
+          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
         </is>
       </c>
       <c r="D235" s="3" t="inlineStr">
@@ -16018,12 +16049,12 @@
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-02</t>
+          <t>E2E-R1-ANN-05</t>
         </is>
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
+          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D236" s="3" t="inlineStr">
@@ -16045,12 +16076,12 @@
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-03</t>
+          <t>E2E-R1-ANN-06</t>
         </is>
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
+          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
         </is>
       </c>
       <c r="D237" s="3" t="inlineStr">
@@ -16072,12 +16103,12 @@
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-01</t>
+          <t>E2E-R1-SRCH-01</t>
         </is>
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
+          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
         </is>
       </c>
       <c r="D238" s="3" t="inlineStr">
@@ -16099,12 +16130,12 @@
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-02</t>
+          <t>E2E-R1-SRCH-02</t>
         </is>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
+          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
         </is>
       </c>
       <c r="D239" s="3" t="inlineStr">
@@ -16126,12 +16157,12 @@
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-03</t>
+          <t>E2E-R1-SRCH-03</t>
         </is>
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
+          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
         </is>
       </c>
       <c r="D240" s="3" t="inlineStr">
@@ -16153,12 +16184,12 @@
       </c>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-04</t>
+          <t>E2E-R1-AUDX-01</t>
         </is>
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>Chain verify reports intact | FR-T02</t>
+          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
         </is>
       </c>
       <c r="D241" s="3" t="inlineStr">
@@ -16180,12 +16211,12 @@
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-05</t>
+          <t>E2E-R1-AUDX-02</t>
         </is>
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
+          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
         </is>
       </c>
       <c r="D242" s="3" t="inlineStr">
@@ -16207,12 +16238,12 @@
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-06</t>
+          <t>E2E-R1-AUDX-03</t>
         </is>
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
+          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
         </is>
       </c>
       <c r="D243" s="3" t="inlineStr">
@@ -16234,12 +16265,12 @@
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-AUDX-04</t>
         </is>
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>Chain verify reports intact | FR-T02</t>
         </is>
       </c>
       <c r="D244" s="3" t="inlineStr">
@@ -16261,12 +16292,12 @@
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-AUDX-05</t>
         </is>
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
         </is>
       </c>
       <c r="D245" s="3" t="inlineStr">
@@ -16288,12 +16319,12 @@
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-AUDX-06</t>
         </is>
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
         </is>
       </c>
       <c r="D246" s="3" t="inlineStr">
@@ -16315,12 +16346,12 @@
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
         </is>
       </c>
       <c r="D247" s="3" t="inlineStr">
@@ -16342,12 +16373,12 @@
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
@@ -16369,12 +16400,12 @@
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D249" s="3" t="inlineStr">
@@ -16396,12 +16427,12 @@
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
         </is>
       </c>
       <c r="D250" s="3" t="inlineStr">
@@ -16423,12 +16454,12 @@
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
         </is>
       </c>
       <c r="D251" s="3" t="inlineStr">
@@ -16450,12 +16481,12 @@
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D252" s="3" t="inlineStr">
@@ -16477,12 +16508,12 @@
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D253" s="3" t="inlineStr">
@@ -16504,12 +16535,12 @@
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
         </is>
       </c>
       <c r="D254" s="3" t="inlineStr">
@@ -16531,12 +16562,12 @@
       </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D255" s="3" t="inlineStr">
@@ -16558,12 +16589,12 @@
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C256" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D256" s="3" t="inlineStr">
@@ -16585,12 +16616,12 @@
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D257" s="3" t="inlineStr">
@@ -16612,12 +16643,12 @@
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C258" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D258" s="3" t="inlineStr">
@@ -16639,12 +16670,12 @@
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
         </is>
       </c>
       <c r="D259" s="3" t="inlineStr">
@@ -16666,12 +16697,12 @@
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
         </is>
       </c>
       <c r="D260" s="3" t="inlineStr">
@@ -16693,12 +16724,12 @@
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
         </is>
       </c>
       <c r="D261" s="3" t="inlineStr">
@@ -16720,12 +16751,12 @@
       </c>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C262" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D262" s="3" t="inlineStr">
@@ -16747,12 +16778,12 @@
       </c>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
         </is>
       </c>
       <c r="D263" s="3" t="inlineStr">
@@ -16774,12 +16805,12 @@
       </c>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C264" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
         </is>
       </c>
       <c r="D264" s="3" t="inlineStr">
@@ -16801,12 +16832,12 @@
       </c>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C265" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D265" s="3" t="inlineStr">
@@ -16828,12 +16859,12 @@
       </c>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C266" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
         </is>
       </c>
       <c r="D266" s="3" t="inlineStr">
@@ -16855,12 +16886,12 @@
       </c>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C267" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D267" s="3" t="inlineStr">
@@ -16882,12 +16913,12 @@
       </c>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C268" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D268" s="3" t="inlineStr">
@@ -16909,12 +16940,12 @@
       </c>
       <c r="B269" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C269" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D269" s="3" t="inlineStr">
@@ -16936,12 +16967,12 @@
       </c>
       <c r="B270" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C270" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D270" s="3" t="inlineStr">
@@ -16963,12 +16994,12 @@
       </c>
       <c r="B271" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C271" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D271" s="3" t="inlineStr">
@@ -16990,12 +17021,12 @@
       </c>
       <c r="B272" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C272" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D272" s="3" t="inlineStr">
@@ -17017,12 +17048,12 @@
       </c>
       <c r="B273" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C273" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D273" s="3" t="inlineStr">
@@ -17044,12 +17075,12 @@
       </c>
       <c r="B274" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C274" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D274" s="3" t="inlineStr">
@@ -17071,12 +17102,12 @@
       </c>
       <c r="B275" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C275" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D275" s="3" t="inlineStr">
@@ -17098,12 +17129,12 @@
       </c>
       <c r="B276" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C276" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D276" s="3" t="inlineStr">
@@ -17125,12 +17156,12 @@
       </c>
       <c r="B277" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C277" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D277" s="3" t="inlineStr">
@@ -17152,12 +17183,12 @@
       </c>
       <c r="B278" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C278" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D278" s="3" t="inlineStr">
@@ -17179,12 +17210,12 @@
       </c>
       <c r="B279" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C279" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D279" s="3" t="inlineStr">
@@ -17206,12 +17237,12 @@
       </c>
       <c r="B280" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C280" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D280" s="3" t="inlineStr">
@@ -17233,12 +17264,12 @@
       </c>
       <c r="B281" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C281" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D281" s="3" t="inlineStr">
@@ -17260,12 +17291,12 @@
       </c>
       <c r="B282" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C282" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D282" s="3" t="inlineStr">
@@ -17287,12 +17318,12 @@
       </c>
       <c r="B283" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C283" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D283" s="3" t="inlineStr">
@@ -17314,12 +17345,12 @@
       </c>
       <c r="B284" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C284" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D284" s="3" t="inlineStr">
@@ -17341,12 +17372,12 @@
       </c>
       <c r="B285" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C285" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D285" s="3" t="inlineStr">
@@ -17368,12 +17399,12 @@
       </c>
       <c r="B286" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C286" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D286" s="3" t="inlineStr">
@@ -17395,12 +17426,12 @@
       </c>
       <c r="B287" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C287" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D287" s="3" t="inlineStr">
@@ -17422,12 +17453,12 @@
       </c>
       <c r="B288" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C288" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D288" s="3" t="inlineStr">
@@ -17449,12 +17480,12 @@
       </c>
       <c r="B289" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C289" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D289" s="3" t="inlineStr">
@@ -17476,12 +17507,12 @@
       </c>
       <c r="B290" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C290" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D290" s="3" t="inlineStr">
@@ -17503,12 +17534,12 @@
       </c>
       <c r="B291" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C291" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D291" s="3" t="inlineStr">
@@ -17530,12 +17561,12 @@
       </c>
       <c r="B292" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C292" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D292" s="3" t="inlineStr">
@@ -17557,12 +17588,12 @@
       </c>
       <c r="B293" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C293" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D293" s="3" t="inlineStr">
@@ -17584,12 +17615,12 @@
       </c>
       <c r="B294" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C294" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D294" s="3" t="inlineStr">
@@ -17611,12 +17642,12 @@
       </c>
       <c r="B295" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C295" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D295" s="3" t="inlineStr">
@@ -17638,12 +17669,12 @@
       </c>
       <c r="B296" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C296" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D296" s="3" t="inlineStr">
@@ -17665,12 +17696,12 @@
       </c>
       <c r="B297" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C297" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D297" s="3" t="inlineStr">
@@ -17692,12 +17723,12 @@
       </c>
       <c r="B298" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C298" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D298" s="3" t="inlineStr">
@@ -17719,12 +17750,12 @@
       </c>
       <c r="B299" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C299" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D299" s="3" t="inlineStr">
@@ -17746,12 +17777,12 @@
       </c>
       <c r="B300" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C300" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D300" s="3" t="inlineStr">
@@ -17773,12 +17804,12 @@
       </c>
       <c r="B301" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C301" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D301" s="3" t="inlineStr">
@@ -17800,12 +17831,12 @@
       </c>
       <c r="B302" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C302" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D302" s="3" t="inlineStr">
@@ -17827,12 +17858,12 @@
       </c>
       <c r="B303" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C303" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D303" s="3" t="inlineStr">
@@ -17854,12 +17885,12 @@
       </c>
       <c r="B304" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C304" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D304" s="3" t="inlineStr">
@@ -17881,12 +17912,12 @@
       </c>
       <c r="B305" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C305" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D305" s="3" t="inlineStr">
@@ -17908,12 +17939,12 @@
       </c>
       <c r="B306" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C306" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D306" s="3" t="inlineStr">
@@ -17935,12 +17966,12 @@
       </c>
       <c r="B307" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C307" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D307" s="3" t="inlineStr">
@@ -17962,12 +17993,12 @@
       </c>
       <c r="B308" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R4-11</t>
         </is>
       </c>
       <c r="C308" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
         </is>
       </c>
       <c r="D308" s="3" t="inlineStr">
@@ -17989,12 +18020,12 @@
       </c>
       <c r="B309" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R4-ISO</t>
         </is>
       </c>
       <c r="C309" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
         </is>
       </c>
       <c r="D309" s="3" t="inlineStr">
@@ -18016,12 +18047,12 @@
       </c>
       <c r="B310" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R5-01</t>
         </is>
       </c>
       <c r="C310" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
         </is>
       </c>
       <c r="D310" s="3" t="inlineStr">
@@ -18043,12 +18074,12 @@
       </c>
       <c r="B311" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R5-02</t>
         </is>
       </c>
       <c r="C311" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
         </is>
       </c>
       <c r="D311" s="3" t="inlineStr">
@@ -18070,12 +18101,12 @@
       </c>
       <c r="B312" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R5-03</t>
         </is>
       </c>
       <c r="C312" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
         </is>
       </c>
       <c r="D312" s="3" t="inlineStr">
@@ -18097,12 +18128,12 @@
       </c>
       <c r="B313" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R5-04</t>
         </is>
       </c>
       <c r="C313" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
         </is>
       </c>
       <c r="D313" s="3" t="inlineStr">
@@ -18124,12 +18155,12 @@
       </c>
       <c r="B314" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R5-05</t>
         </is>
       </c>
       <c r="C314" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
         </is>
       </c>
       <c r="D314" s="3" t="inlineStr">
@@ -18151,12 +18182,12 @@
       </c>
       <c r="B315" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R5-06</t>
         </is>
       </c>
       <c r="C315" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
         </is>
       </c>
       <c r="D315" s="3" t="inlineStr">
@@ -18178,12 +18209,12 @@
       </c>
       <c r="B316" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R5-07</t>
         </is>
       </c>
       <c r="C316" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
         </is>
       </c>
       <c r="D316" s="3" t="inlineStr">
@@ -18205,20 +18236,101 @@
       </c>
       <c r="B317" s="3" t="inlineStr">
         <is>
+          <t>E2E-R5-08</t>
+        </is>
+      </c>
+      <c r="C317" s="3" t="inlineStr">
+        <is>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+        </is>
+      </c>
+      <c r="D317" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E317" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B318" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-09</t>
+        </is>
+      </c>
+      <c r="C318" s="3" t="inlineStr">
+        <is>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+        </is>
+      </c>
+      <c r="D318" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E318" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B319" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C319" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D319" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E319" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B320" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C317" s="3" t="inlineStr">
+      <c r="C320" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D317" s="3" t="inlineStr">
+      <c r="D320" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E317" s="3" t="inlineStr">
+      <c r="E320" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
docs: E2E rows UI-12..23 and ADM-01..02; tracker 043/044/063 done, 031/045/064 progress
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E320" headerRowCount="1">
-  <autoFilter ref="A1:E320"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E334" headerRowCount="1">
+  <autoFilter ref="A1:E334"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -4609,7 +4609,7 @@
       <c r="N27" s="3" t="inlineStr"/>
       <c r="O27" s="3" t="inlineStr">
         <is>
-          <t>Web app on the Notion/Attio direction (owner choice): warm paper palette in tokens (contrast-checked), full-bleed pages with a warm icon sidebar, workspace + account menus (persisted theme), action-first Home (acknowledgements, reviews, announcements with inline actions, library table, activity, people), Library (filters, Attio-style table, New document dialog), document reading view with properties, lifecycle actions (edit, submit, approve, request changes, publish with step-up, new version), acknowledgement callout, Announcements feed with read/ack, Members with invite dialog; split sign-in with product preview; single-flight token refresh. E2E-R1-UI-01..10 with axe. Remaining: ⌘K command palette (search API is ready), system console shell, mobile bottom bar</t>
+          <t>Web app on the Notion/Attio direction (owner choice): warm paper palette in tokens (contrast-checked), full-bleed pages with a warm icon sidebar, workspace + account menus (persisted theme), action-first Home (acknowledgements, reviews, announcements with inline actions, library table, activity, people), Library (filters, Attio-style table, New document dialog), document reading view with properties, lifecycle actions (edit, submit, approve, request changes, publish with step-up, new version), acknowledgement callout, Announcements feed with read/ack, Members with invite dialog; split sign-in with product preview; single-flight token refresh. E2E-R1-UI-01..10 with axe. Remaining: ⌘K command palette (search API is ready), system console shell, mobile bottom bar Second UI pass: Geist type, state kit (skeletons, empty states, load errors with retry), ⌘K palette over search + commands (E2E-R1-UI-12..13), admin screens: Manage announcements, Campaigns, Settings, Audit log, Overview, People &amp; access (E2E-R1-UI-14..17, 23); Policies portal and document governance (E2E-R1-UI-18..22). Remaining: system console shell, keyboard nav audit</t>
         </is>
       </c>
     </row>
@@ -5040,7 +5040,7 @@
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L34" s="3" t="inlineStr"/>
@@ -5048,7 +5048,7 @@
       <c r="N34" s="3" t="inlineStr"/>
       <c r="O34" s="3" t="inlineStr">
         <is>
-          <t>API done (UI pending: compare view + UI E2E). procera-library diff module: block-level LCS alignment of SOP/policy content with word-level diffs inside changed blocks (removals and additions paired by position within an unmatched run, same block type → changed); GET /versions/{a}/diff/{b} (same artifact only); unit + property test (applying a diff always rebuilds the target) + E2E-R1-LIB-06. Process/form/rule bundle artifacts diff once their editors land (BPMS-050+).</t>
+          <t>UI: Compare page (/library/:id/compare) with word-level ins/del, version pickers, E2E-R1-UI-20. procera-library diff module: block-level LCS alignment of SOP/policy content with word-level diffs inside changed blocks (removals and additions paired by position within an unmatched run, same block type → changed); GET /versions/{a}/diff/{b} (same artifact only); unit + property test (applying a diff always rebuilds the target) + E2E-R1-LIB-06. Process/form/rule bundle artifacts diff once their editors land (BPMS-050+).</t>
         </is>
       </c>
     </row>
@@ -5105,7 +5105,7 @@
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L35" s="3" t="inlineStr"/>
@@ -5113,7 +5113,7 @@
       <c r="N35" s="3" t="inlineStr"/>
       <c r="O35" s="3" t="inlineStr">
         <is>
-          <t>API done (UI pending: governance panel, change requests + UI E2E). Migration 0016: review cadence (per-artifact override or governance.review_cadence.default/.controlled), next_review_at set on every publish, recertification, worker flag of passed review dates (once; artifact.review_overdue.v1 → owner in-app notification), verification badge with governance.verification.validity expiry, change requests (open → accepted/declined/implemented, linked to the implementing version); all audited and in the audit contract; E2E-R1-LIB-07..10. Effective-date scheduling shipped with BPMS-040.</t>
+          <t>UI: document governance panel (review status, recertify, schedule, verify with step-up, suggested changes with accept/decline/implemented), E2E-R1-UI-18..19. Migration 0016: review cadence (per-artifact override or governance.review_cadence.default/.controlled), next_review_at set on every publish, recertification, worker flag of passed review dates (once; artifact.review_overdue.v1 → owner in-app notification), verification badge with governance.verification.validity expiry, change requests (open → accepted/declined/implemented, linked to the implementing version); all audited and in the audit contract; E2E-R1-LIB-07..10. Effective-date scheduling shipped with BPMS-040.</t>
         </is>
       </c>
     </row>
@@ -5178,7 +5178,7 @@
       <c r="N36" s="3" t="inlineStr"/>
       <c r="O36" s="3" t="inlineStr">
         <is>
-          <t>API done (UI pending: Policies portal page, applicability control + UI E2E). Migration 0017: policy category, applicability (audience; NULL = everyone) and restricted flag; procera_audience_contains SQL twin of the audience resolver; reader visibility (A-14): view-only readers see published history only, restricted policies hidden outside their applicability in lists, reads, diff, change requests and search; PUT /artifacts/{id}/applicability (audited); GET /me/policies portal with what-changed summaries vs the previous published version, text + category filters; E2E-R1-POL-01..03. Remaining: re-acknowledgement on major publish (FR-PL03), superseded watermark in exports.</t>
+          <t>UI: Policies portal (search, category chips, what changed → compare) and applicability control on the document page, E2E-R1-UI-21..22. Migration 0017: policy category, applicability (audience; NULL = everyone) and restricted flag; procera_audience_contains SQL twin of the audience resolver; reader visibility (A-14): view-only readers see published history only, restricted policies hidden outside their applicability in lists, reads, diff, change requests and search; PUT /artifacts/{id}/applicability (audited); GET /me/policies portal with what-changed summaries vs the previous published version, text + category filters; E2E-R1-POL-01..03. Remaining: re-acknowledgement on major publish (FR-PL03), superseded watermark in exports.</t>
         </is>
       </c>
     </row>
@@ -5678,13 +5678,17 @@
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L44" s="3" t="inlineStr"/>
       <c r="M44" s="3" t="inlineStr"/>
       <c r="N44" s="3" t="inlineStr"/>
-      <c r="O44" s="3" t="inlineStr"/>
+      <c r="O44" s="3" t="inlineStr">
+        <is>
+          <t>API: GET /admin/overview (needs-attention ranking: overdue acknowledgements, admins without MFA, documents past review, drafts in review, announcements to approve; acknowledgement metrics, published-versions series, security strip from the audit chain, departments; requests/storage reported as null with guidance until those modules ship) and GET /admin/people (MFA, last active, roles, dormant, privileged, expiring grants, pending invites, filters); migration 0018 discovery.member_login_failures. UI: Overview (typographic summary, ranked list, metric rows, security strip; time range + department in the URL) and People &amp; access (filter chips). E2E-R1-ADM-01..02, E2E-R1-UI-23.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -5747,7 +5751,7 @@
       <c r="N45" s="3" t="inlineStr"/>
       <c r="O45" s="3" t="inlineStr">
         <is>
-          <t>API done: procera_audit::explorer — filtered newest-first keyset paging, view-own scope, member names, artifact-aware object timelines, chain verify, private audited saved queries, capped CSV/JSONL exports with step-up that are themselves audited; E2E-R1-AUDX-01..06. Remaining: explorer UI (docs/05 §3.19), async export job, POST /audit/query</t>
+          <t>API done: procera_audit::explorer — filtered newest-first keyset paging, view-own scope, member names, artifact-aware object timelines, chain verify, private audited saved queries, capped CSV/JSONL exports with step-up that are themselves audited; E2E-R1-AUDX-01..06. UI: Audit log screen (chain-verified badge, filters, keyset paging, expandable records, object timelines in a drawer; E2E-R1-UI-17). Remaining: async export job, POST /audit/query</t>
         </is>
       </c>
     </row>
@@ -9686,7 +9690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E320"/>
+  <dimension ref="A1:E334"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -15455,12 +15459,12 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-01</t>
+          <t>E2E-R1-ADM-01</t>
         </is>
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>Sign in through the browser (password + recovery code) lands on Home; navigation is permission-shaped with the current page marked; axe clean on sign-in and Home; reload keeps the session | docs/05 §2.1, §3.1, WCAG 2.2 AA</t>
+          <t>Overview: overdue acknowledgements rank first in "needs attention", followed by an admin without two-step verification; acknowledgement metrics and a daily published series; the security strip counts a failed sign-in, members without MFA and the new admin grant; requests/storage are null; members get 403; an inverted range → 422 | BPMS-063, FR-A01</t>
         </is>
       </c>
       <c r="D214" s="3" t="inlineStr">
@@ -15482,12 +15486,12 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-02</t>
+          <t>E2E-R1-ADM-02</t>
         </is>
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>Wrong password and wrong code produce clear, non-revealing messages (role=alert); axe clean | docs/06 §3, WCAG 3.3.1</t>
+          <t>People &amp; access: counts (members, no MFA, privileged, pending invites), member row (MFA off, last active set, not dormant), no-MFA and admin filters; unknown filter → 422; members get 403 | BPMS-063, FR-A06</t>
         </is>
       </c>
       <c r="D215" s="3" t="inlineStr">
@@ -15509,12 +15513,12 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-03</t>
+          <t>E2E-R1-UI-01</t>
         </is>
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>With several workspaces the chooser appears; choosing one and switching from the header changes the context and the navigation (no Admin for a plain member) | docs/05 §2.1 workspace switcher</t>
+          <t>Sign in through the browser (password + recovery code) lands on Home; navigation is permission-shaped with the current page marked; axe clean on sign-in and Home; reload keeps the session | docs/05 §2.1, §3.1, WCAG 2.2 AA</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
@@ -15536,12 +15540,12 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-04</t>
+          <t>E2E-R1-UI-02</t>
         </is>
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>The bell announces the unread count; the inbox lists the "joined" notification; mark all as read | FR-N01</t>
+          <t>Wrong password and wrong code produce clear, non-revealing messages (role=alert); axe clean | docs/06 §3, WCAG 3.3.1</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -15563,12 +15567,12 @@
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-05</t>
+          <t>E2E-R1-UI-03</t>
         </is>
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>Sign out returns to sign-in; reloading stays signed out | docs/06 §3</t>
+          <t>With several workspaces the chooser appears; choosing one and switching from the header changes the context and the navigation (no Admin for a plain member) | docs/05 §2.1 workspace switcher</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
@@ -15590,12 +15594,12 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-06</t>
+          <t>E2E-R1-UI-04</t>
         </is>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Theme switched from the account menu persists across reload; dark theme passes axe | docs/05 §7, WCAG 2.2 AA</t>
+          <t>The bell announces the unread count; the inbox lists the "joined" notification; mark all as read | FR-N01</t>
         </is>
       </c>
       <c r="D219" s="3" t="inlineStr">
@@ -15617,12 +15621,12 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-07</t>
+          <t>E2E-R1-UI-05</t>
         </is>
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Author a policy in the browser: New document dialog → write content (headings, lists) → save → submit → publish; the library row shows Published; axe clean | FR-G04, docs/05 §3.2/§3.21</t>
+          <t>Sign out returns to sign-in; reloading stays signed out | docs/06 §3</t>
         </is>
       </c>
       <c r="D220" s="3" t="inlineStr">
@@ -15644,12 +15648,12 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-08</t>
+          <t>E2E-R1-UI-06</t>
         </is>
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>A campaign task on Home leads to the document; “I acknowledge” records the acknowledgement (campaign progress +1) and the callout disappears | FR-AK01, docs/05 §3.1</t>
+          <t>Theme switched from the account menu persists across reload; dark theme passes axe | docs/05 §7, WCAG 2.2 AA</t>
         </is>
       </c>
       <c r="D221" s="3" t="inlineStr">
@@ -15671,12 +15675,12 @@
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-09</t>
+          <t>E2E-R1-UI-07</t>
         </is>
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>Invite a colleague from Members with a role; the invitation appears in the table as Invited | FR-W01, docs/05 §3.14</t>
+          <t>Author a policy in the browser: New document dialog → write content (headings, lists) → save → submit → publish; the library row shows Published; axe clean | FR-G04, docs/05 §3.2/§3.21</t>
         </is>
       </c>
       <c r="D222" s="3" t="inlineStr">
@@ -15698,12 +15702,12 @@
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-10</t>
+          <t>E2E-R1-UI-08</t>
         </is>
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Read and acknowledge a critical, pinned announcement in the feed | FR-AN04, docs/05 §3.23</t>
+          <t>A campaign task on Home leads to the document; “I acknowledge” records the acknowledgement (campaign progress +1) and the callout disappears | FR-AK01, docs/05 §3.1</t>
         </is>
       </c>
       <c r="D223" s="3" t="inlineStr">
@@ -15725,12 +15729,12 @@
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-11</t>
+          <t>E2E-R1-UI-09</t>
         </is>
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>An admin without two-step verification is guided through setup (QR + key, confirm a code, recovery codes) and then signs in with MFA and lands on Home | docs/06 §3, docs/20 §2.3</t>
+          <t>Invite a colleague from Members with a role; the invitation appears in the table as Invited | FR-W01, docs/05 §3.14</t>
         </is>
       </c>
       <c r="D224" s="3" t="inlineStr">
@@ -15752,12 +15756,12 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-01</t>
+          <t>E2E-R1-UI-10</t>
         </is>
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
+          <t>Read and acknowledge a critical, pinned announcement in the feed | FR-AN04, docs/05 §3.23</t>
         </is>
       </c>
       <c r="D225" s="3" t="inlineStr">
@@ -15779,12 +15783,12 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-02</t>
+          <t>E2E-R1-UI-11</t>
         </is>
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
+          <t>An admin without two-step verification is guided through setup (QR + key, confirm a code, recovery codes) and then signs in with MFA and lands on Home | docs/06 §3, docs/20 §2.3</t>
         </is>
       </c>
       <c r="D226" s="3" t="inlineStr">
@@ -15806,12 +15810,12 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-03</t>
+          <t>E2E-R1-UI-12</t>
         </is>
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
+          <t>⌘K finds a document by its content and opens it; commands navigate; recent items are offered; keyboard only | BPMS-031, BPMS-049</t>
         </is>
       </c>
       <c r="D227" s="3" t="inlineStr">
@@ -15833,12 +15837,12 @@
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-04</t>
+          <t>E2E-R1-UI-13</t>
         </is>
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
+          <t>A new workspace shows composed empty states; an unknown page offers a way back; a failed load shows the error with a retry | BPMS-031 (UX-005)</t>
         </is>
       </c>
       <c r="D228" s="3" t="inlineStr">
@@ -15860,12 +15864,12 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-05</t>
+          <t>E2E-R1-UI-14</t>
         </is>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
+          <t>Manage announcements: compose a draft; a workspace-wide post is sent for approval; a targeted draft is published and shows receipts | BPMS-031, BPMS-047</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
@@ -15887,12 +15891,12 @@
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-06</t>
+          <t>E2E-R1-UI-15</t>
         </is>
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
+          <t>Campaigns: create from a published document with an audience, check the reach, launch, follow progress, download the evidence CSV | BPMS-031, BPMS-046</t>
         </is>
       </c>
       <c r="D230" s="3" t="inlineStr">
@@ -15914,12 +15918,12 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-07</t>
+          <t>E2E-R1-UI-16</t>
         </is>
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
+          <t>Settings: change a value in place with a reason and see why it applies; a step-up key asks to confirm identity | BPMS-031, BPMS-027</t>
         </is>
       </c>
       <c r="D231" s="3" t="inlineStr">
@@ -15941,12 +15945,12 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-01</t>
+          <t>E2E-R1-UI-17</t>
         </is>
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
+          <t>Audit log: chain verified; filter by category; expand a record; open an object timeline; no-match state | BPMS-031, BPMS-064</t>
         </is>
       </c>
       <c r="D232" s="3" t="inlineStr">
@@ -15968,12 +15972,12 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-02</t>
+          <t>E2E-R1-UI-18</t>
         </is>
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
+          <t>The owner sets a review schedule, recertifies when it falls due, verifies and removes verification | BPMS-044</t>
         </is>
       </c>
       <c r="D233" s="3" t="inlineStr">
@@ -15995,12 +15999,12 @@
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-03</t>
+          <t>E2E-R1-UI-19</t>
         </is>
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
+          <t>A member suggests a change; the owner accepts it and marks it implemented in v2 | BPMS-044</t>
         </is>
       </c>
       <c r="D234" s="3" t="inlineStr">
@@ -16022,12 +16026,12 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-04</t>
+          <t>E2E-R1-UI-20</t>
         </is>
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
+          <t>Compare v1 and v2 from the version history: word-level changes and the summary | BPMS-043</t>
         </is>
       </c>
       <c r="D235" s="3" t="inlineStr">
@@ -16049,12 +16053,12 @@
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-05</t>
+          <t>E2E-R1-UI-21</t>
         </is>
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
+          <t>A member opens Policies, filters by category and follows "what changed" to the comparison | BPMS-045</t>
         </is>
       </c>
       <c r="D236" s="3" t="inlineStr">
@@ -16076,12 +16080,12 @@
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-06</t>
+          <t>E2E-R1-UI-22</t>
         </is>
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
+          <t>A publisher restricts a policy to a role; a member outside it can't find it in Policies or open it | BPMS-045, A-14</t>
         </is>
       </c>
       <c r="D237" s="3" t="inlineStr">
@@ -16103,12 +16107,12 @@
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-01</t>
+          <t>E2E-R1-UI-23</t>
         </is>
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
+          <t>An admin opens Overview: the summary and "Needs attention" show overdue acknowledgements, and the security strip shows one member without two-step verification; drilling in opens People &amp; access filtered to them; the Admins filter shows the owner | BPMS-063</t>
         </is>
       </c>
       <c r="D238" s="3" t="inlineStr">
@@ -16130,12 +16134,12 @@
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-02</t>
+          <t>E2E-R1-CMP-01</t>
         </is>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
+          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
         </is>
       </c>
       <c r="D239" s="3" t="inlineStr">
@@ -16157,12 +16161,12 @@
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-03</t>
+          <t>E2E-R1-CMP-02</t>
         </is>
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
+          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
         </is>
       </c>
       <c r="D240" s="3" t="inlineStr">
@@ -16184,12 +16188,12 @@
       </c>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-01</t>
+          <t>E2E-R1-CMP-03</t>
         </is>
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
+          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
         </is>
       </c>
       <c r="D241" s="3" t="inlineStr">
@@ -16211,12 +16215,12 @@
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-02</t>
+          <t>E2E-R1-CMP-04</t>
         </is>
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
+          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
         </is>
       </c>
       <c r="D242" s="3" t="inlineStr">
@@ -16238,12 +16242,12 @@
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-03</t>
+          <t>E2E-R1-CMP-05</t>
         </is>
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
+          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
         </is>
       </c>
       <c r="D243" s="3" t="inlineStr">
@@ -16265,12 +16269,12 @@
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-04</t>
+          <t>E2E-R1-CMP-06</t>
         </is>
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>Chain verify reports intact | FR-T02</t>
+          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
         </is>
       </c>
       <c r="D244" s="3" t="inlineStr">
@@ -16292,12 +16296,12 @@
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-05</t>
+          <t>E2E-R1-CMP-07</t>
         </is>
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
+          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D245" s="3" t="inlineStr">
@@ -16319,12 +16323,12 @@
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-06</t>
+          <t>E2E-R1-ANN-01</t>
         </is>
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
+          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
         </is>
       </c>
       <c r="D246" s="3" t="inlineStr">
@@ -16346,12 +16350,12 @@
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-ANN-02</t>
         </is>
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
         </is>
       </c>
       <c r="D247" s="3" t="inlineStr">
@@ -16373,12 +16377,12 @@
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-ANN-03</t>
         </is>
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
@@ -16400,12 +16404,12 @@
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-ANN-04</t>
         </is>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
         </is>
       </c>
       <c r="D249" s="3" t="inlineStr">
@@ -16427,12 +16431,12 @@
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-ANN-05</t>
         </is>
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D250" s="3" t="inlineStr">
@@ -16454,12 +16458,12 @@
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-ANN-06</t>
         </is>
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
         </is>
       </c>
       <c r="D251" s="3" t="inlineStr">
@@ -16481,12 +16485,12 @@
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-SRCH-01</t>
         </is>
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
         </is>
       </c>
       <c r="D252" s="3" t="inlineStr">
@@ -16508,12 +16512,12 @@
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-SRCH-02</t>
         </is>
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
         </is>
       </c>
       <c r="D253" s="3" t="inlineStr">
@@ -16535,12 +16539,12 @@
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-SRCH-03</t>
         </is>
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
         </is>
       </c>
       <c r="D254" s="3" t="inlineStr">
@@ -16562,12 +16566,12 @@
       </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-AUDX-01</t>
         </is>
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
         </is>
       </c>
       <c r="D255" s="3" t="inlineStr">
@@ -16589,12 +16593,12 @@
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-AUDX-02</t>
         </is>
       </c>
       <c r="C256" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
         </is>
       </c>
       <c r="D256" s="3" t="inlineStr">
@@ -16616,12 +16620,12 @@
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-AUDX-03</t>
         </is>
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
         </is>
       </c>
       <c r="D257" s="3" t="inlineStr">
@@ -16643,12 +16647,12 @@
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-AUDX-04</t>
         </is>
       </c>
       <c r="C258" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>Chain verify reports intact | FR-T02</t>
         </is>
       </c>
       <c r="D258" s="3" t="inlineStr">
@@ -16670,12 +16674,12 @@
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-AUDX-05</t>
         </is>
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
         </is>
       </c>
       <c r="D259" s="3" t="inlineStr">
@@ -16697,12 +16701,12 @@
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-AUDX-06</t>
         </is>
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
         </is>
       </c>
       <c r="D260" s="3" t="inlineStr">
@@ -16724,12 +16728,12 @@
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
         </is>
       </c>
       <c r="D261" s="3" t="inlineStr">
@@ -16751,12 +16755,12 @@
       </c>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C262" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D262" s="3" t="inlineStr">
@@ -16778,12 +16782,12 @@
       </c>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D263" s="3" t="inlineStr">
@@ -16805,12 +16809,12 @@
       </c>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C264" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
         </is>
       </c>
       <c r="D264" s="3" t="inlineStr">
@@ -16832,12 +16836,12 @@
       </c>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C265" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
         </is>
       </c>
       <c r="D265" s="3" t="inlineStr">
@@ -16859,12 +16863,12 @@
       </c>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C266" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D266" s="3" t="inlineStr">
@@ -16886,12 +16890,12 @@
       </c>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C267" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D267" s="3" t="inlineStr">
@@ -16913,12 +16917,12 @@
       </c>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C268" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
         </is>
       </c>
       <c r="D268" s="3" t="inlineStr">
@@ -16940,12 +16944,12 @@
       </c>
       <c r="B269" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C269" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D269" s="3" t="inlineStr">
@@ -16967,12 +16971,12 @@
       </c>
       <c r="B270" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C270" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D270" s="3" t="inlineStr">
@@ -16994,12 +16998,12 @@
       </c>
       <c r="B271" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C271" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D271" s="3" t="inlineStr">
@@ -17021,12 +17025,12 @@
       </c>
       <c r="B272" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C272" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D272" s="3" t="inlineStr">
@@ -17048,12 +17052,12 @@
       </c>
       <c r="B273" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C273" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
         </is>
       </c>
       <c r="D273" s="3" t="inlineStr">
@@ -17075,12 +17079,12 @@
       </c>
       <c r="B274" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C274" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
         </is>
       </c>
       <c r="D274" s="3" t="inlineStr">
@@ -17102,12 +17106,12 @@
       </c>
       <c r="B275" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C275" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
         </is>
       </c>
       <c r="D275" s="3" t="inlineStr">
@@ -17129,12 +17133,12 @@
       </c>
       <c r="B276" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C276" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D276" s="3" t="inlineStr">
@@ -17156,12 +17160,12 @@
       </c>
       <c r="B277" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C277" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
         </is>
       </c>
       <c r="D277" s="3" t="inlineStr">
@@ -17183,12 +17187,12 @@
       </c>
       <c r="B278" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C278" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
         </is>
       </c>
       <c r="D278" s="3" t="inlineStr">
@@ -17210,12 +17214,12 @@
       </c>
       <c r="B279" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C279" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D279" s="3" t="inlineStr">
@@ -17237,12 +17241,12 @@
       </c>
       <c r="B280" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C280" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
         </is>
       </c>
       <c r="D280" s="3" t="inlineStr">
@@ -17264,12 +17268,12 @@
       </c>
       <c r="B281" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C281" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D281" s="3" t="inlineStr">
@@ -17291,12 +17295,12 @@
       </c>
       <c r="B282" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C282" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D282" s="3" t="inlineStr">
@@ -17318,12 +17322,12 @@
       </c>
       <c r="B283" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C283" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D283" s="3" t="inlineStr">
@@ -17345,12 +17349,12 @@
       </c>
       <c r="B284" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C284" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D284" s="3" t="inlineStr">
@@ -17372,12 +17376,12 @@
       </c>
       <c r="B285" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C285" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D285" s="3" t="inlineStr">
@@ -17399,12 +17403,12 @@
       </c>
       <c r="B286" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C286" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D286" s="3" t="inlineStr">
@@ -17426,12 +17430,12 @@
       </c>
       <c r="B287" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C287" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D287" s="3" t="inlineStr">
@@ -17453,12 +17457,12 @@
       </c>
       <c r="B288" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C288" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D288" s="3" t="inlineStr">
@@ -17480,12 +17484,12 @@
       </c>
       <c r="B289" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C289" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D289" s="3" t="inlineStr">
@@ -17507,12 +17511,12 @@
       </c>
       <c r="B290" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C290" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D290" s="3" t="inlineStr">
@@ -17534,12 +17538,12 @@
       </c>
       <c r="B291" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C291" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D291" s="3" t="inlineStr">
@@ -17561,12 +17565,12 @@
       </c>
       <c r="B292" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C292" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D292" s="3" t="inlineStr">
@@ -17588,12 +17592,12 @@
       </c>
       <c r="B293" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C293" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D293" s="3" t="inlineStr">
@@ -17615,12 +17619,12 @@
       </c>
       <c r="B294" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C294" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D294" s="3" t="inlineStr">
@@ -17642,12 +17646,12 @@
       </c>
       <c r="B295" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C295" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D295" s="3" t="inlineStr">
@@ -17669,12 +17673,12 @@
       </c>
       <c r="B296" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C296" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D296" s="3" t="inlineStr">
@@ -17696,12 +17700,12 @@
       </c>
       <c r="B297" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C297" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D297" s="3" t="inlineStr">
@@ -17723,12 +17727,12 @@
       </c>
       <c r="B298" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C298" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D298" s="3" t="inlineStr">
@@ -17750,12 +17754,12 @@
       </c>
       <c r="B299" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C299" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D299" s="3" t="inlineStr">
@@ -17777,12 +17781,12 @@
       </c>
       <c r="B300" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C300" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D300" s="3" t="inlineStr">
@@ -17804,12 +17808,12 @@
       </c>
       <c r="B301" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C301" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D301" s="3" t="inlineStr">
@@ -17831,12 +17835,12 @@
       </c>
       <c r="B302" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C302" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D302" s="3" t="inlineStr">
@@ -17858,12 +17862,12 @@
       </c>
       <c r="B303" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C303" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D303" s="3" t="inlineStr">
@@ -17885,12 +17889,12 @@
       </c>
       <c r="B304" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C304" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D304" s="3" t="inlineStr">
@@ -17912,12 +17916,12 @@
       </c>
       <c r="B305" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C305" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D305" s="3" t="inlineStr">
@@ -17939,12 +17943,12 @@
       </c>
       <c r="B306" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C306" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D306" s="3" t="inlineStr">
@@ -17966,12 +17970,12 @@
       </c>
       <c r="B307" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C307" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D307" s="3" t="inlineStr">
@@ -17993,12 +17997,12 @@
       </c>
       <c r="B308" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C308" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D308" s="3" t="inlineStr">
@@ -18020,12 +18024,12 @@
       </c>
       <c r="B309" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C309" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D309" s="3" t="inlineStr">
@@ -18047,12 +18051,12 @@
       </c>
       <c r="B310" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C310" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D310" s="3" t="inlineStr">
@@ -18074,12 +18078,12 @@
       </c>
       <c r="B311" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C311" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D311" s="3" t="inlineStr">
@@ -18101,12 +18105,12 @@
       </c>
       <c r="B312" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C312" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D312" s="3" t="inlineStr">
@@ -18128,12 +18132,12 @@
       </c>
       <c r="B313" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C313" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D313" s="3" t="inlineStr">
@@ -18155,12 +18159,12 @@
       </c>
       <c r="B314" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C314" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D314" s="3" t="inlineStr">
@@ -18182,12 +18186,12 @@
       </c>
       <c r="B315" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C315" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D315" s="3" t="inlineStr">
@@ -18209,12 +18213,12 @@
       </c>
       <c r="B316" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C316" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D316" s="3" t="inlineStr">
@@ -18236,12 +18240,12 @@
       </c>
       <c r="B317" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C317" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D317" s="3" t="inlineStr">
@@ -18263,12 +18267,12 @@
       </c>
       <c r="B318" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C318" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D318" s="3" t="inlineStr">
@@ -18290,12 +18294,12 @@
       </c>
       <c r="B319" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C319" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D319" s="3" t="inlineStr">
@@ -18317,20 +18321,398 @@
       </c>
       <c r="B320" s="3" t="inlineStr">
         <is>
+          <t>E2E-R4-09</t>
+        </is>
+      </c>
+      <c r="C320" s="3" t="inlineStr">
+        <is>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+        </is>
+      </c>
+      <c r="D320" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E320" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B321" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-10</t>
+        </is>
+      </c>
+      <c r="C321" s="3" t="inlineStr">
+        <is>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+        </is>
+      </c>
+      <c r="D321" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E321" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B322" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-11</t>
+        </is>
+      </c>
+      <c r="C322" s="3" t="inlineStr">
+        <is>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+        </is>
+      </c>
+      <c r="D322" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E322" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B323" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-ISO</t>
+        </is>
+      </c>
+      <c r="C323" s="3" t="inlineStr">
+        <is>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+        </is>
+      </c>
+      <c r="D323" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E323" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B324" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-01</t>
+        </is>
+      </c>
+      <c r="C324" s="3" t="inlineStr">
+        <is>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+        </is>
+      </c>
+      <c r="D324" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E324" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B325" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-02</t>
+        </is>
+      </c>
+      <c r="C325" s="3" t="inlineStr">
+        <is>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+        </is>
+      </c>
+      <c r="D325" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E325" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B326" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-03</t>
+        </is>
+      </c>
+      <c r="C326" s="3" t="inlineStr">
+        <is>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+        </is>
+      </c>
+      <c r="D326" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E326" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B327" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-04</t>
+        </is>
+      </c>
+      <c r="C327" s="3" t="inlineStr">
+        <is>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+        </is>
+      </c>
+      <c r="D327" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E327" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B328" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-05</t>
+        </is>
+      </c>
+      <c r="C328" s="3" t="inlineStr">
+        <is>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+        </is>
+      </c>
+      <c r="D328" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E328" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B329" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-06</t>
+        </is>
+      </c>
+      <c r="C329" s="3" t="inlineStr">
+        <is>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+        </is>
+      </c>
+      <c r="D329" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E329" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B330" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-07</t>
+        </is>
+      </c>
+      <c r="C330" s="3" t="inlineStr">
+        <is>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+        </is>
+      </c>
+      <c r="D330" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E330" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B331" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-08</t>
+        </is>
+      </c>
+      <c r="C331" s="3" t="inlineStr">
+        <is>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+        </is>
+      </c>
+      <c r="D331" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E331" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B332" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-09</t>
+        </is>
+      </c>
+      <c r="C332" s="3" t="inlineStr">
+        <is>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+        </is>
+      </c>
+      <c r="D332" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E332" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B333" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C333" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D333" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E333" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B334" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C320" s="3" t="inlineStr">
+      <c r="C334" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D320" s="3" t="inlineStr">
+      <c r="D334" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E320" s="3" t="inlineStr">
+      <c r="E334" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
docs: tracker BPMS-022/027/045/065 done (30/109); E2E rows for passkeys, settings layers, re-ack, system console
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -197,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E15" headerRowCount="1">
-  <autoFilter ref="A1:E15"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E20" headerRowCount="1">
+  <autoFilter ref="A1:E20"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Source"/>
     <tableColumn id="2" name="ID"/>
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E334" headerRowCount="1">
-  <autoFilter ref="A1:E334"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E359" headerRowCount="1">
+  <autoFilter ref="A1:E359"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -1393,7 +1393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1789,22 +1789,157 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
+          <t>A-18 (BPMS-065)</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>System console: (1) the member quota counts active members plus open invitations, checked when inviting (accepting a reserved seat is never refused; lowering a quota below current use blocks new invitations only); (2) quota defaults are per configuration profile and apply to new workspaces only; (3) the system plane's step-up window is the docs/12 §11 default of 5 minutes (it has no workspace settings) and covers suspend, reactivate, schedule deletion, workspace quotas and quota defaults; (4) scheduling deletion requires a reason, stored as the workspace's state reason; (5) health is "degraded" when the oldest pending event or queued email is older than 5 minutes, any email has failed, the cache is degraded, no dispatcher runs, or migrations are missing; (6) "last activity" is the newest event on the workspace's own audit chain; (7) the system audit names system administrators only, other actors stay pseudonymous</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Product-owner review of docs/05 §3.20 and docs/20 §3 "As built"; operator feedback</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Count invitations separately; per-plan defaults; a platform setting for the system step-up window</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
           <t>A-14</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Library visibility (BPMS-045): members who can only `view` a kind (no `create`/`edit_draft`/`review`/`approve`/`publish`) see an artifact only once it has a published version, and only its published history (published, deprecated, retired), never drafts, reviews or scheduled versions. This matches the UI promise "Nobody else sees it until it's published". A `restricted` policy is additionally hidden (404, also in search) from readers outside its applicability. Authors and admins see everything</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>Product-owner review; pilot feedback</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>Show drafts to readers through explicit visibility settings (docs/12 §8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>A-15 (BPMS-048)</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Quiet hours apply every day (no per-day selection yet); digest and quiet-hour times use whole hours in the member's time zone; which emails are "urgent" is fixed per kind (campaign actions and acknowledgement requests urgent, plain announcements normal, critical announcements critical)</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Pilot feedback</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Per-day quiet hours; per-kind member choices (CFG)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>A-16 (BPMS-045)</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Re-acknowledgement on publish: the publisher picks major (default) or minor; v1 is `1.0` and never asks; the decision is fixed when the version is published or scheduled. One `governance.reack.policy` covers SOPs and policies (no separate `policies.reack.policy` key). The campaign goes to the artifact's applicability (everyone when unset), starts automatically with the workspace campaign defaults and `governance.reack.window`, and needs no `campaign:manage` from the publisher (the policy setting authorises it). Earlier campaigns on older versions keep running and are not closed. An audience with no active members starts no campaign</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Product-owner review of docs/04 §2.7 "As built (0019)"; pilot feedback</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Close superseded campaigns automatically; let the publisher edit the audience or due date before it launches; a per-artifact acknowledgement requirement (docs/05 §3.22 "none / on publish / on major / annual")</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>A-17 (BPMS-027)</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Settings layers: (1) department overrides are inherited down the department tree and the nearest department wins; (2) department-scopable keys are the §2 Ovr ✓ / ✓ (dept) keys, never collection-only or ⚡ keys, and features keep reading workspace-level values until they carry a department context; (3) a profile switch resets every key any profile sets to the target profile's value (or the code default), replacing admin-set values (flagged in the plan), raising looser values to the floor, with a reason and step-up; (4) the effective-settings cache is used only with a shared Valkey cache, and only by the settings read API; (5) clearing a department override needs no reason</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Product-owner review of docs/20 §0-§1 "As built"; pilot feedback</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Keep admin-set values on a switch; let features resolve per department; cache with the in-process backend for single-node installs</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>A-19 (BPMS-022)</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Passkeys at P0 (WebAuthn L3, docs/06 §3.6): (1) a passkey is a **second factor** after the password and a step-up method; passkey-only sign-in stays P1 (docs/12 §3). (2) Attestation is requested as `none` and not verified, so any authenticator is accepted (no AAGUID allow list). (3) User verification is `preferred`, not required; user presence is required. The UV flag is stored per passkey so "UV required for admins" can be enforced later. (4) Accepted algorithms: ES256, EdDSA, RS256 (≥ 2048 bits). (5) Verification uses `ring` + `ciborium` (Apache-2.0/ISC, Apache-2.0) because `webauthn-rs` is MPL-2.0, which is not on the ADR-0014 allow list. (6) The first second factor (passkey or TOTP) issues 10 recovery codes; removing the last one removes them. (7) Account-level step-up (removing a passkey) uses the platform default window of 5 minutes, since the account is not tied to one workspace. Adding a passkey needs only a valid session, like TOTP enrolment. (8) The RP ID is the public URL's host (override: `PROCERA_WEBAUTHN_RP_ID`); a loopback IP maps to `localhost`, because browsers reject IP addresses as RP IDs. (9) A signature counter that does not increase is rejected as a possible clone. (10) The access token's `amr` gets `hwk` for a passkey (RFC 8176)</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Security review of BPMS-022; pilot feedback from admins with hardware keys</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Add an attestation/AAGUID policy setting; require UV for admin roles; move passkey-only sign-in earlier</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4155,7 @@
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L18" s="3" t="inlineStr"/>
@@ -4028,7 +4163,7 @@
       <c r="N18" s="3" t="inlineStr"/>
       <c r="O18" s="3" t="inlineStr">
         <is>
-          <t>TOTP (RFC 6238, replay-protected, sealed secrets) + 10 recovery codes + MFA login (E2E-R1-AUTH-06). Step-up: POST /session/step-up (TOTP code, or password without MFA) re-issues the token with a fresh auth_time; enforced against auth.stepup.window (401 step_up_required) for step-up settings, role create/edit and grant/revoke (E2E-R1-CFG-03). MFA required by role (auth.mfa.required_roles) enforced at workspace entry, 403 mfa_required (E2E-R1-MEM-10). Remaining: WebAuthn/passkeys</t>
+          <t>TOTP + recovery codes + step-up + MFA by role (earlier); passkeys (WebAuthn L3, migration 0020): registration, sign-in second factor and step-up, list/rename/remove with step-up, phishing-origin and replay protection, Account › Security page, Use a passkey at sign-in and in step-up. E2E-R1-AUTH-06, 20..23, E2E-R1-UI-30..31. Passkey-only sign-in is P1 (A-19)</t>
         </is>
       </c>
     </row>
@@ -4345,7 +4480,7 @@
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L23" s="3" t="inlineStr"/>
@@ -4353,7 +4488,7 @@
       <c r="N23" s="3" t="inlineStr"/>
       <c r="O23" s="3" t="inlineStr">
         <is>
-          <t>procera-settings: catalogue in code (P0 subset, 38 keys) with comparators; platform floors + workspace values + append-only revisions (migration 0007, RLS); 4 configuration profiles applied at workspace creation; resolution with clamping when a floor is raised; explainer; /api/v1/settings (list, explainer, PUT per key with If-Match, history) and /sysapi/v1/settings floors; reasons for ⚡ keys, step-up = MFA session (interim); audited (setting.changed, platform.floor_changed); property test (512 cases, never looser than floor); E2E-R1-CFG-01..05. Remaining: department/collection overrides (needs directory), profile switch plan/apply (CFG-017), settings cache invalidation (CFG-004)</t>
+          <t>Catalogue, floors, profiles, explainer (earlier); department overrides as layer 4 with tree inheritance (0021), profile switch plan/apply with If-Match, reason and step-up (CFG-017), effective-settings cache with generation invalidation over Valkey, never authoritative (CFG-004); Settings tabs for departments and profile. E2E-R1-CFG-01..08, E2E-R1-UI-16, 35..36 (A-17)</t>
         </is>
       </c>
     </row>
@@ -5170,7 +5305,7 @@
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L36" s="3" t="inlineStr"/>
@@ -5178,7 +5313,7 @@
       <c r="N36" s="3" t="inlineStr"/>
       <c r="O36" s="3" t="inlineStr">
         <is>
-          <t>UI: Policies portal (search, category chips, what changed → compare) and applicability control on the document page, E2E-R1-UI-21..22. Migration 0017: policy category, applicability (audience; NULL = everyone) and restricted flag; procera_audience_contains SQL twin of the audience resolver; reader visibility (A-14): view-only readers see published history only, restricted policies hidden outside their applicability in lists, reads, diff, change requests and search; PUT /artifacts/{id}/applicability (audited); GET /me/policies portal with what-changed summaries vs the previous published version, text + category filters; E2E-R1-POL-01..03. Remaining: re-acknowledgement on major publish (FR-PL03), superseded watermark in exports.</t>
+          <t>Category, applicability and restricted policies; Policies portal with what changed (migration 0017, A-14); re-acknowledgement on publish (0019): major/minor semver fixed at publish or scheduling, governance.reack.policy/window, campaign to the applicable audience bound to the exact version hash (immediate in the publish transaction, scheduled on go-live via the bus), publish preview and dialog. E2E-R1-POL-01..05, E2E-R1-UI-21..22, 24. Later: per-artifact acknowledgement requirement (docs/05), closing older campaigns (A-16)</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5500,7 @@
       </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L39" s="3" t="inlineStr"/>
@@ -5373,7 +5508,7 @@
       <c r="N39" s="3" t="inlineStr"/>
       <c r="O39" s="3" t="inlineStr">
         <is>
-          <t>procera-notify (migration 0011): templates in code (minijinja, strict, HTML auto-escaped), in-app inbox (list/unread/read/read-all), email queue with sealed bodies and dedupe, SMTP delivery via lettre (STARTTLS/TLS) with backoff (max 1 h, 12 tries), workspace sender name; outbox consumers: invitation email with accept link, member-joined in-app to the inviter. Flags --public-url, --smtp-url, --mail-from. E2E-R1-NOT-01..02. Remaining: digests + quiet hours (FR-N04), localisation + terminology (CFG-008), more event kinds as features land</t>
+          <t>procera-notify (migrations 0011, 0023): templates in code (minijinja, strict, HTML auto-escaped), in-app inbox, sealed email queue with dedupe, SMTP delivery via lettre with backoff; digests (daily/weekly at the member's hour and time zone; only normal emails are digested), quiet hours (emails held until the window ends; critical override), bounce suppression on permanent SMTP rejection (global email_suppressions); member preferences with workspace defaults (notify.digest.*, notify.quiet_hours.*); Notification preferences page. E2E-R1-NOT-01..05, E2E-R1-UI-25. Later: localisation + terminology (CFG-008), per-day quiet hours (A-15), more event kinds as features land</t>
         </is>
       </c>
     </row>
@@ -5808,13 +5943,17 @@
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L46" s="3" t="inlineStr"/>
       <c r="M46" s="3" t="inlineStr"/>
       <c r="N46" s="3" t="inlineStr"/>
-      <c r="O46" s="3" t="inlineStr"/>
+      <c r="O46" s="3" t="inlineStr">
+        <is>
+          <t>System console (0022): workspaces grid with usage and quotas, suspend/reactivate/schedule deletion with step-up on the system chain, quota defaults per profile with the member quota enforced at invite, platform health, system audit explorer; console shell for system admins (metadata only, never workspace content). E2E-R1-SYS-01..09, E2E-R1-UI-40..41 (A-18)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -9690,7 +9829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E334"/>
+  <dimension ref="A1:E359"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14087,7 +14226,7 @@
       </c>
       <c r="C163" s="3" t="inlineStr">
         <is>
-          <t>Confirm dialog: Cancel focused first, focus trapped, axe-clean, Esc closes and restores focus to the trigger; confirm performs the action | WCAG 2.4.3, 2.1.2; docs/05 §7.1.1</t>
+          <t>The root size follows the display width, not the window: 16px on displays up to 1440 wide and on small screens, about 17.7px at 1920, 20px at 2560 (also in a half-width window) | docs/05 §7.1.0</t>
         </is>
       </c>
       <c r="D163" s="3" t="inlineStr">
@@ -14109,12 +14248,12 @@
       </c>
       <c r="B164" s="3" t="inlineStr">
         <is>
-          <t>E2E-P0-11</t>
+          <t>E2E-P0-10</t>
         </is>
       </c>
       <c r="C164" s="3" t="inlineStr">
         <is>
-          <t>Data grid: `aria-sort` none→ascending→descending, filter result count announced in a live region, select-all count | FR-V01/V02/V06/V08</t>
+          <t>Confirm dialog: Cancel focused first, focus trapped, axe-clean, Esc closes and restores focus to the trigger; confirm performs the action | WCAG 2.4.3, 2.1.2; docs/05 §7.1.1</t>
         </is>
       </c>
       <c r="D164" s="3" t="inlineStr">
@@ -14136,12 +14275,12 @@
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>E2E-P0-12</t>
+          <t>E2E-P0-11</t>
         </is>
       </c>
       <c r="C165" s="3" t="inlineStr">
         <is>
-          <t>Select operable by keyboard only (open, move, choose) | WCAG 2.1.1</t>
+          <t>Data grid: `aria-sort` none→ascending→descending, filter result count announced in a live region, select-all count | FR-V01/V02/V06/V08</t>
         </is>
       </c>
       <c r="D165" s="3" t="inlineStr">
@@ -14163,12 +14302,12 @@
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>E2E-P0-13</t>
+          <t>E2E-P0-12</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
         <is>
-          <t>Tabs: arrow keys move focus and selection; the panel follows | WAI-ARIA tabs pattern</t>
+          <t>Select operable by keyboard only (open, move, choose) | WCAG 2.1.1</t>
         </is>
       </c>
       <c r="D166" s="3" t="inlineStr">
@@ -14190,12 +14329,12 @@
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUTH-01</t>
+          <t>E2E-P0-13</t>
         </is>
       </c>
       <c r="C167" s="3" t="inlineStr">
         <is>
-          <t>Login returns a ≤ 15 min Bearer JWT + HttpOnly/SameSite=Strict refresh cookie, `Cache-Control: no-store`; `/me` works only with a valid token; forged token → 401 problem+json | §3.2</t>
+          <t>Tabs: arrow keys move focus and selection; the panel follows | WAI-ARIA tabs pattern</t>
         </is>
       </c>
       <c r="D167" s="3" t="inlineStr">
@@ -14217,12 +14356,12 @@
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUTH-02</t>
+          <t>E2E-R1-AUTH-01</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
         <is>
-          <t>Wrong password and unknown account return the same error code | enumeration resistance</t>
+          <t>Login returns a ≤ 15 min Bearer JWT + HttpOnly/SameSite=Strict refresh cookie, `Cache-Control: no-store`; `/me` works only with a valid token; forged token → 401 problem+json | §3.2</t>
         </is>
       </c>
       <c r="D168" s="3" t="inlineStr">
@@ -14244,12 +14383,12 @@
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUTH-03</t>
+          <t>E2E-R1-AUTH-02</t>
         </is>
       </c>
       <c r="C169" s="3" t="inlineStr">
         <is>
-          <t>Refresh rotates the cookie; replaying the old refresh token → `token_reused` and the legitimate session is revoked too | SEC-14</t>
+          <t>Wrong password and unknown account return the same error code | enumeration resistance</t>
         </is>
       </c>
       <c r="D169" s="3" t="inlineStr">
@@ -14271,12 +14410,12 @@
       </c>
       <c r="B170" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUTH-04</t>
+          <t>E2E-R1-AUTH-03</t>
         </is>
       </c>
       <c r="C170" s="3" t="inlineStr">
         <is>
-          <t>Cookie endpoints without `X-Requested-With: procera` → 403 `csrf` | CSRF</t>
+          <t>Refresh rotates the cookie; replaying the old refresh token → `token_reused` and the legitimate session is revoked too | SEC-14</t>
         </is>
       </c>
       <c r="D170" s="3" t="inlineStr">
@@ -14298,12 +14437,12 @@
       </c>
       <c r="B171" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUTH-05</t>
+          <t>E2E-R1-AUTH-04</t>
         </is>
       </c>
       <c r="C171" s="3" t="inlineStr">
         <is>
-          <t>Logout revokes the family and clears the cookie | §3.2</t>
+          <t>Cookie endpoints without `X-Requested-With: procera` → 403 `csrf` | CSRF</t>
         </is>
       </c>
       <c r="D171" s="3" t="inlineStr">
@@ -14325,12 +14464,12 @@
       </c>
       <c r="B172" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUTH-06</t>
+          <t>E2E-R1-AUTH-05</t>
         </is>
       </c>
       <c r="C172" s="3" t="inlineStr">
         <is>
-          <t>TOTP enrolment (otpauth URI), MFA login (`amr=[pwd,otp]`), MFA token rejected as access token, TOTP replay rejected, recovery code single-use | §3.6</t>
+          <t>Logout revokes the family and clears the cookie | §3.2</t>
         </is>
       </c>
       <c r="D172" s="3" t="inlineStr">
@@ -14352,12 +14491,12 @@
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUTH-07</t>
+          <t>E2E-R1-AUTH-06</t>
         </is>
       </c>
       <c r="C173" s="3" t="inlineStr">
         <is>
-          <t>Sign-out-everywhere rejects another device's unexpired JWT and refresh; system audit chain verifies | SEC-04, AUD-01</t>
+          <t>TOTP enrolment (otpauth URI), MFA login (`amr=[pwd,otp]`), MFA token rejected as access token, TOTP replay rejected, recovery code single-use | §3.6</t>
         </is>
       </c>
       <c r="D173" s="3" t="inlineStr">
@@ -14379,12 +14518,12 @@
       </c>
       <c r="B174" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SYS-01</t>
+          <t>E2E-R1-AUTH-07</t>
         </is>
       </c>
       <c r="C174" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: wrong token 401; one-time token creates `system.owner`; reuse 409; no further tokens | FR-S01 (= E2E-R1-01)</t>
+          <t>Sign-out-everywhere rejects another device's unexpired JWT and refresh; system audit chain verifies | SEC-04, AUD-01</t>
         </is>
       </c>
       <c r="D174" s="3" t="inlineStr">
@@ -14406,12 +14545,12 @@
       </c>
       <c r="B175" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SYS-02</t>
+          <t>E2E-R1-AUTH-20</t>
         </is>
       </c>
       <c r="C175" s="3" t="inlineStr">
         <is>
-          <t>System API returns 404 to non-system users and 403 `mfa_required` to system users without MFA | docs/12 §1, docs/06 §3.6</t>
+          <t>Register a passkey: options, single-use challenge, recovery codes once, duplicates refused | BPMS-022</t>
         </is>
       </c>
       <c r="D175" s="3" t="inlineStr">
@@ -14433,12 +14572,12 @@
       </c>
       <c r="B176" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SYS-03</t>
+          <t>E2E-R1-AUTH-21</t>
         </is>
       </c>
       <c r="C176" s="3" t="inlineStr">
         <is>
-          <t>Create workspaces A (starter) and B (enterprise): 201 + Location + ETag, profile quotas, duplicate slug 409, invalid slug 422, listing | FR-S02/S04 (= E2E-R1-02)</t>
+          <t>Sign in with password + passkey; phishing origin and replayed assertions fail | BPMS-022</t>
         </is>
       </c>
       <c r="D176" s="3" t="inlineStr">
@@ -14460,12 +14599,12 @@
       </c>
       <c r="B177" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SYS-04</t>
+          <t>E2E-R1-AUTH-22</t>
         </is>
       </c>
       <c r="C177" s="3" t="inlineStr">
         <is>
-          <t>Suspend read-only with reason; stale `If-Match` → 412; restore with current ETag; invalid transition 409; schedule deletion (grace validated) | FR-S02 (= E2E-R1-17)</t>
+          <t>Step up with a passkey; a sign-in challenge cannot be reused for step-up | BPMS-022</t>
         </is>
       </c>
       <c r="D177" s="3" t="inlineStr">
@@ -14487,12 +14626,12 @@
       </c>
       <c r="B178" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SYS-05</t>
+          <t>E2E-R1-AUTH-23</t>
         </is>
       </c>
       <c r="C178" s="3" t="inlineStr">
         <is>
-          <t>`system.operator` can read but not write; system audit chain verifies | docs/12 §4.1, FR-S09</t>
+          <t>Removing a passkey needs step-up; another user’s passkey is 404; the last one turns MFA off | BPMS-022</t>
         </is>
       </c>
       <c r="D178" s="3" t="inlineStr">
@@ -14514,12 +14653,12 @@
       </c>
       <c r="B179" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-MEM-01</t>
+          <t>E2E-R1-SYS-01</t>
         </is>
       </c>
       <c r="C179" s="3" t="inlineStr">
         <is>
-          <t>Owner registers through the system-created invitation; workspace becomes `active`; owner holds owner permissions; invitation is single-use | FR-S01, FR-W01</t>
+          <t>Bootstrap: wrong token 401; one-time token creates `system.owner`; reuse 409; no further tokens | FR-S01 (= E2E-R1-01)</t>
         </is>
       </c>
       <c r="D179" s="3" t="inlineStr">
@@ -14541,12 +14680,12 @@
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-MEM-02</t>
+          <t>E2E-R1-SYS-02</t>
         </is>
       </c>
       <c r="C180" s="3" t="inlineStr">
         <is>
-          <t>Invite → accept only by the invited email; the token is never returned to the inviter; member appears in the list | FR-W01, docs/06 §3</t>
+          <t>System API returns 404 to non-system users and 403 `mfa_required` to system users without MFA | docs/12 §1, docs/06 §3.6</t>
         </is>
       </c>
       <c r="D180" s="3" t="inlineStr">
@@ -14568,12 +14707,12 @@
       </c>
       <c r="B181" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-MEM-03</t>
+          <t>E2E-R1-SYS-03</t>
         </is>
       </c>
       <c r="C181" s="3" t="inlineStr">
         <is>
-          <t>A non-member cannot switch into another workspace (404); workspace APIs need a selected workspace | docs/12 §1, SEC-01</t>
+          <t>Create workspaces A (starter) and B (enterprise): 201 + Location + ETag, profile quotas, duplicate slug 409, invalid slug 422, listing | FR-S02/S04 (= E2E-R1-02)</t>
         </is>
       </c>
       <c r="D181" s="3" t="inlineStr">
@@ -14595,12 +14734,12 @@
       </c>
       <c r="B182" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-MEM-04</t>
+          <t>E2E-R1-SYS-04</t>
         </is>
       </c>
       <c r="C182" s="3" t="inlineStr">
         <is>
-          <t>Custom role: no escalation, built-ins immutable, grant/revoke takes effect on the next request | FR-W03, ADR-0011</t>
+          <t>Suspend read-only with reason; stale `If-Match` → 412; restore with current ETag; invalid transition 409; schedule deletion (grace validated) | FR-S02 (= E2E-R1-17)</t>
         </is>
       </c>
       <c r="D182" s="3" t="inlineStr">
@@ -14622,12 +14761,12 @@
       </c>
       <c r="B183" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-MEM-05</t>
+          <t>E2E-R1-SYS-05</t>
         </is>
       </c>
       <c r="C183" s="3" t="inlineStr">
         <is>
-          <t>Admin cannot invite an owner, cannot remove the last owner or themselves; a deactivated member loses access at once | FR-W01, docs/12 §6</t>
+          <t>`system.operator` can read but not write; system audit chain verifies | docs/12 §4.1, FR-S09</t>
         </is>
       </c>
       <c r="D183" s="3" t="inlineStr">
@@ -14649,12 +14788,12 @@
       </c>
       <c r="B184" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-MEM-06</t>
+          <t>E2E-R1-SYS-06</t>
         </is>
       </c>
       <c r="C184" s="3" t="inlineStr">
         <is>
-          <t>Read-only suspension blocks workspace writes with 423, reads still work; restore re-enables writes | FR-S02</t>
+          <t>Workspaces grid lists metadata, quotas and usage counts with filters | BPMS-065</t>
         </is>
       </c>
       <c r="D184" s="3" t="inlineStr">
@@ -14676,12 +14815,12 @@
       </c>
       <c r="B185" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-MEM-07</t>
+          <t>E2E-R1-SYS-07</t>
         </is>
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>Pending invitations listed; revoking kills the token (404); resend issues a new working token; `/__test/drain` dispatches the outbox to idle | FR-W01, docs/04 §2.11</t>
+          <t>Suspend, reactivate and schedule deletion need step-up and land on the system chain | BPMS-065</t>
         </is>
       </c>
       <c r="D185" s="3" t="inlineStr">
@@ -14703,12 +14842,12 @@
       </c>
       <c r="B186" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-MEM-08</t>
+          <t>E2E-R1-SYS-08</t>
         </is>
       </c>
       <c r="C186" s="3" t="inlineStr">
         <is>
-          <t>An admin cannot revoke the owner's grant (escalation); the last owner keeps the role; role preview shows added/removed/affected members; role and grant changes are on the verified audit chain | FR-W03, docs/12 §5, FR-T01</t>
+          <t>Quota defaults per profile and the member quota enforced at invite time | BPMS-065</t>
         </is>
       </c>
       <c r="D186" s="3" t="inlineStr">
@@ -14730,12 +14869,12 @@
       </c>
       <c r="B187" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-MEM-09</t>
+          <t>E2E-R1-SYS-09</t>
         </is>
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>A role granted to a group applies while the member is in it and stops when removed; owner role cannot go to groups; a department-scoped admin reaches members in the subtree only | docs/12 §5, FR-W03</t>
+          <t>Platform health and the system audit explorer; auditors read, never change | BPMS-065</t>
         </is>
       </c>
       <c r="D187" s="3" t="inlineStr">
@@ -14757,12 +14896,12 @@
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-MEM-10</t>
+          <t>E2E-R1-MEM-01</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
         <is>
-          <t>MFA by role: in a Standard workspace an admin signed in without MFA is refused at workspace entry (403 `mfa_required`); a plain member is not | docs/20 §2.3 `auth.mfa.required_roles`, FR-W06</t>
+          <t>Owner registers through the system-created invitation; workspace becomes `active`; owner holds owner permissions; invitation is single-use | FR-S01, FR-W01</t>
         </is>
       </c>
       <c r="D188" s="3" t="inlineStr">
@@ -14784,12 +14923,12 @@
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUD-01</t>
+          <t>E2E-R1-MEM-02</t>
         </is>
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>Every mutating route is called once and appends exactly the audit actions in its route contract (`/__test/audit/contract`); exempt routes append nothing; no route goes unexercised (bootstrap is one-shot and checked by the platform integration test) | FR-T01, docs/24 §3.5</t>
+          <t>Invite → accept only by the invited email; the token is never returned to the inviter; member appears in the list | FR-W01, docs/06 §3</t>
         </is>
       </c>
       <c r="D189" s="3" t="inlineStr">
@@ -14811,12 +14950,12 @@
       </c>
       <c r="B190" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CFG-01</t>
+          <t>E2E-R1-MEM-03</t>
         </is>
       </c>
       <c r="C190" s="3" t="inlineStr">
         <is>
-          <t>The creation profile seeds values (Starter: 8 h idle); the explainer lists default → platform floor → profile; unknown keys 404 | FR-W04, docs/20 §0-1</t>
+          <t>A non-member cannot switch into another workspace (404); workspace APIs need a selected workspace | docs/12 §1, SEC-01</t>
         </is>
       </c>
       <c r="D190" s="3" t="inlineStr">
@@ -14838,12 +14977,12 @@
       </c>
       <c r="B191" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CFG-02</t>
+          <t>E2E-R1-MEM-04</t>
         </is>
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>Looser than a floor → 422 `setting_below_floor`; ⚡ keys need a reason; stricter value saved with `ETag`/`If-Match` (stale → 412); floor-locked key 403; invalid value 422; history records the change | FR-S05, FR-W06</t>
+          <t>Custom role: no escalation, built-ins immutable, grant/revoke takes effect on the next request | FR-W03, ADR-0011</t>
         </is>
       </c>
       <c r="D191" s="3" t="inlineStr">
@@ -14865,12 +15004,12 @@
       </c>
       <c r="B192" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CFG-03</t>
+          <t>E2E-R1-MEM-05</t>
         </is>
       </c>
       <c r="C192" s="3" t="inlineStr">
         <is>
-          <t>Step-up keys need a recent authentication: a 10-minute-old sign-in gets 401 `step_up_required`; a wrong code fails; `POST /session/step-up` with a current TOTP code issues a fresh token that succeeds | docs/12 §11, SEC-17</t>
+          <t>Admin cannot invite an owner, cannot remove the last owner or themselves; a deactivated member loses access at once | FR-W01, docs/12 §6</t>
         </is>
       </c>
       <c r="D192" s="3" t="inlineStr">
@@ -14892,12 +15031,12 @@
       </c>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CFG-04</t>
+          <t>E2E-R1-MEM-06</t>
         </is>
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>A member without settings permissions can neither view nor change settings | docs/12 §5</t>
+          <t>Read-only suspension blocks workspace writes with 423, reads still work; restore re-enables writes | FR-S02</t>
         </is>
       </c>
       <c r="D193" s="3" t="inlineStr">
@@ -14919,12 +15058,12 @@
       </c>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CFG-05</t>
+          <t>E2E-R1-MEM-07</t>
         </is>
       </c>
       <c r="C194" s="3" t="inlineStr">
         <is>
-          <t>Raising a platform floor clamps a looser workspace value at resolution (stored value kept, `clamped: true`); floors need a reason; keys without floors are rejected | docs/20 §1 rules 4-5</t>
+          <t>Pending invitations listed; revoking kills the token (404); resend issues a new working token; `/__test/drain` dispatches the outbox to idle | FR-W01, docs/04 §2.11</t>
         </is>
       </c>
       <c r="D194" s="3" t="inlineStr">
@@ -14946,12 +15085,12 @@
       </c>
       <c r="B195" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-DIR-01</t>
+          <t>E2E-R1-MEM-08</t>
         </is>
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>Department tree: sibling names unique (409), moving under a descendant rejected (422 `cycle`), deleting a non-empty department refused | FR-W02</t>
+          <t>An admin cannot revoke the owner's grant (escalation); the last owner keeps the role; role preview shows added/removed/affected members; role and grant changes are on the verified audit chain | FR-W03, docs/12 §5, FR-T01</t>
         </is>
       </c>
       <c r="D195" s="3" t="inlineStr">
@@ -14973,12 +15112,12 @@
       </c>
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-DIR-02</t>
+          <t>E2E-R1-MEM-09</t>
         </is>
       </c>
       <c r="C196" s="3" t="inlineStr">
         <is>
-          <t>Manager cycles rejected; resolution is the explicit manager, else the nearest department head that is not the member; field sources recorded | FR-W02 (deterministic resolution)</t>
+          <t>A role granted to a group applies while the member is in it and stops when removed; owner role cannot go to groups; a department-scoped admin reaches members in the subtree only | docs/12 §5, FR-W03</t>
         </is>
       </c>
       <c r="D196" s="3" t="inlineStr">
@@ -15000,12 +15139,12 @@
       </c>
       <c r="B197" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-DIR-03</t>
+          <t>E2E-R1-MEM-10</t>
         </is>
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>Static groups (duplicate member 409); positions blocked until `directory.positions.enabled`; members read the directory but cannot change it | FR-W02, docs/20 §2.5</t>
+          <t>MFA by role: in a Standard workspace an admin signed in without MFA is refused at workspace entry (403 `mfa_required`); a plain member is not | docs/20 §2.3 `auth.mfa.required_roles`, FR-W06</t>
         </is>
       </c>
       <c r="D197" s="3" t="inlineStr">
@@ -15027,12 +15166,12 @@
       </c>
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-DIR-04</t>
+          <t>E2E-R1-AUD-01</t>
         </is>
       </c>
       <c r="C198" s="3" t="inlineStr">
         <is>
-          <t>CSV import: `mode=plan` changes nothing; `mode=apply` creates departments by path and links managers listed later in the file; unknown members reported per row; unknown columns 422 | FR-W02</t>
+          <t>Every mutating route is called once and appends exactly the audit actions in its route contract (`/__test/audit/contract`); exempt routes append nothing; no route goes unexercised (bootstrap is one-shot and checked by the platform integration test) | FR-T01, docs/24 §3.5</t>
         </is>
       </c>
       <c r="D198" s="3" t="inlineStr">
@@ -15054,12 +15193,12 @@
       </c>
       <c r="B199" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-NOT-01</t>
+          <t>E2E-R1-CFG-01</t>
         </is>
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>An invitation queues an email (subject, HTML button, link); the link's token registers the invitee; the inviter gets an in-app "joined" notification; read / unread / read-all work | FR-N01, FR-N02, FR-W01</t>
+          <t>The creation profile seeds values (Starter: 8 h idle); the explainer lists default → platform floor → profile; unknown keys 404 | FR-W04, docs/20 §0-1</t>
         </is>
       </c>
       <c r="D199" s="3" t="inlineStr">
@@ -15081,12 +15220,12 @@
       </c>
       <c r="B200" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-NOT-02</t>
+          <t>E2E-R1-CFG-02</t>
         </is>
       </c>
       <c r="C200" s="3" t="inlineStr">
         <is>
-          <t>A member cannot mark another member's notification (404) | FR-N01, SEC-01</t>
+          <t>Looser than a floor → 422 `setting_below_floor`; ⚡ keys need a reason; stricter value saved with `ETag`/`If-Match` (stale → 412); floor-locked key 403; invalid value 422; history records the change | FR-S05, FR-W06</t>
         </is>
       </c>
       <c r="D200" s="3" t="inlineStr">
@@ -15108,12 +15247,12 @@
       </c>
       <c r="B201" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-LIB-01</t>
+          <t>E2E-R1-CFG-03</t>
         </is>
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>SOP draft → edit with `If-Match` (stale → 412) → submit (no review needed: approved, content hash frozen) → published; editing an approved version 409; content and hash identical on retrieval; one open draft per artifact | FR-G04, FR-G05, T07</t>
+          <t>Step-up keys need a recent authentication: a 10-minute-old sign-in gets 401 `step_up_required`; a wrong code fails; `POST /session/step-up` with a current TOTP code issues a fresh token that succeeds | docs/12 §11, SEC-17</t>
         </is>
       </c>
       <c r="D201" s="3" t="inlineStr">
@@ -15135,12 +15274,12 @@
       </c>
       <c r="B202" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-LIB-02</t>
+          <t>E2E-R1-CFG-04</t>
         </is>
       </c>
       <c r="C202" s="3" t="inlineStr">
         <is>
-          <t>Controlled policy needs a review: the author's own approval is refused (403 `sod_violation`); a reviewer cannot publish; a reviewer approves; the owner publishes | FR-G04 SoD, docs/12 §6</t>
+          <t>A member without settings permissions can neither view nor change settings | docs/12 §5</t>
         </is>
       </c>
       <c r="D202" s="3" t="inlineStr">
@@ -15162,12 +15301,12 @@
       </c>
       <c r="B203" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-LIB-03</t>
+          <t>E2E-R1-CFG-05</t>
         </is>
       </c>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>Changes requested needs a comment and returns the draft; withdraw; later versions need a reason for change; publishing supersedes (previous → deprecated) | FR-G04, docs/20 §2.6</t>
+          <t>Raising a platform floor clamps a looser workspace value at resolution (stored value kept, `clamped: true`); floors need a reason; keys without floors are rejected | docs/20 §1 rules 4-5</t>
         </is>
       </c>
       <c r="D203" s="3" t="inlineStr">
@@ -15189,12 +15328,12 @@
       </c>
       <c r="B204" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-LIB-04</t>
+          <t>E2E-R1-CFG-06</t>
         </is>
       </c>
       <c r="C204" s="3" t="inlineStr">
         <is>
-          <t>A scheduled version goes live when its effective time passes (test clock + drain) and supersedes the live one; retire | FR-G05, FR-PL01</t>
+          <t>Department overrides: set on a parent, inherited by a child, explained, cleared; catalogue and workspace isolation enforced | BPMS-027</t>
         </is>
       </c>
       <c r="D204" s="3" t="inlineStr">
@@ -15216,12 +15355,12 @@
       </c>
       <c r="B205" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-LIB-05</t>
+          <t>E2E-R1-CFG-07</t>
         </is>
       </c>
       <c r="C205" s="3" t="inlineStr">
         <is>
-          <t>Members read published policies but cannot author; lists contain only kinds the member may view | docs/12 §5</t>
+          <t>Profile switch: the plan shows current, new and floor values; apply needs If-Match, a reason and step-up; then nothing is left to change | BPMS-027, CFG-017</t>
         </is>
       </c>
       <c r="D205" s="3" t="inlineStr">
@@ -15243,12 +15382,12 @@
       </c>
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-LIB-06</t>
+          <t>E2E-R1-CFG-08</t>
         </is>
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>Semantic diff between two versions: one changed block with word-level detail, one added list, unchanged blocks kept; the reverse direction mirrors it; versions of different artifacts → 422; members may compare; another workspace gets 404 | BPMS-043, FR-G05</t>
+          <t>A settings change is visible on the very next read, through the cache when one is configured | BPMS-027, CFG-004</t>
         </is>
       </c>
       <c r="D206" s="3" t="inlineStr">
@@ -15270,12 +15409,12 @@
       </c>
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-LIB-07</t>
+          <t>E2E-R1-DIR-01</t>
         </is>
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>Publishing sets `next_review_at = published + 365 d` (standard); a per-artifact cadence of 20 days moves it and makes it `due_soon`; 0 → 422; `null` restores the default; an unpublished artifact cannot be recertified (409) | BPMS-044, FR-G07, FX-G01</t>
+          <t>Department tree: sibling names unique (409), moving under a descendant rejected (422 `cycle`), deleting a non-empty department refused | FR-W02</t>
         </is>
       </c>
       <c r="D207" s="3" t="inlineStr">
@@ -15297,12 +15436,12 @@
       </c>
       <c r="B208" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-LIB-08</t>
+          <t>E2E-R1-DIR-02</t>
         </is>
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>A passed review date reads `overdue` immediately; the worker flags it once (two drains) and the owner receives one `review_overdue` notification linking the document; recertifying clears the flag and starts a new period; both are audited | BPMS-044, FR-G07, FX-G01</t>
+          <t>Manager cycles rejected; resolution is the explicit manager, else the nearest department head that is not the member; field sources recorded | FR-W02 (deterministic resolution)</t>
         </is>
       </c>
       <c r="D208" s="3" t="inlineStr">
@@ -15324,12 +15463,12 @@
       </c>
       <c r="B209" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-LIB-09</t>
+          <t>E2E-R1-DIR-03</t>
         </is>
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>Verification lasts `governance.verification.validity` (90 d) and expires on its own; members cannot verify (403); removing it twice → 409 | BPMS-044, FX-G02</t>
+          <t>Static groups (duplicate member 409); positions blocked until `directory.positions.enabled`; members read the directory but cannot change it | FR-W02, docs/20 §2.5</t>
         </is>
       </c>
       <c r="D209" s="3" t="inlineStr">
@@ -15351,12 +15490,12 @@
       </c>
       <c r="B210" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-LIB-10</t>
+          <t>E2E-R1-DIR-04</t>
         </is>
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>Change requests: a member proposes (blank title 422) but cannot resolve (403); declining needs a reason; accepted → implemented by a version of the same artifact (another artifact's version 422); resolved requests are final (409); list filters by state | BPMS-044, FR-G05</t>
+          <t>CSV import: `mode=plan` changes nothing; `mode=apply` creates departments by path and links managers listed later in the file; unknown members reported per row; unknown columns 422 | FR-W02</t>
         </is>
       </c>
       <c r="D210" s="3" t="inlineStr">
@@ -15378,12 +15517,12 @@
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-POL-01</t>
+          <t>E2E-R1-NOT-01</t>
         </is>
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>Readers never see drafts: absent from lists, reads and search until published; a later draft stays hidden (version 404, diff 404, versions list shows v1 only); authors see drafts in search | BPMS-045, A-14</t>
+          <t>An invitation queues an email (subject, HTML button, link); the link's token registers the invitee; the inviter gets an in-app "joined" notification; read / unread / read-all work | FR-N01, FR-N02, FR-W01</t>
         </is>
       </c>
       <c r="D211" s="3" t="inlineStr">
@@ -15405,12 +15544,12 @@
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-POL-02</t>
+          <t>E2E-R1-NOT-02</t>
         </is>
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>Applicability: empty audience or restricted without one → 422; members cannot set it (403); a restricted policy is hidden from members outside its group in lists, reads, search, the portal and change requests (404), and shown to those inside; an unrestricted one is listed for everyone but only "applicable" to its audience | BPMS-045, FR-PL01/PL02</t>
+          <t>A member cannot mark another member's notification (404) | FR-N01, SEC-01</t>
         </is>
       </c>
       <c r="D212" s="3" t="inlineStr">
@@ -15432,12 +15571,12 @@
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-POL-03</t>
+          <t>E2E-R1-NOT-03</t>
         </is>
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>The portal lists published policies that apply to the member (no drafts), ordered by category, with what changed since the previous version (added/changed counts, reason) and text/category filters | BPMS-045, FR-PL02</t>
+          <t>Preferences fall back to the workspace defaults; a member's overrides apply to them only; invalid digest/hour → 422; null resets | BPMS-048, FR-N04</t>
         </is>
       </c>
       <c r="D213" s="3" t="inlineStr">
@@ -15459,12 +15598,12 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ADM-01</t>
+          <t>E2E-R1-NOT-04</t>
         </is>
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>Overview: overdue acknowledgements rank first in "needs attention", followed by an admin without two-step verification; acknowledgement metrics and a daily published series; the security strip counts a failed sign-in, members without MFA and the new admin grant; requests/storage are null; members get 403; an inverted range → 422 | BPMS-063, FR-A01</t>
+          <t>With a daily digest due now, two plain announcements produce no individual emails and exactly one digest listing both (a second drain sends nothing more); in-app notifications still arrive | BPMS-048, FR-N04</t>
         </is>
       </c>
       <c r="D214" s="3" t="inlineStr">
@@ -15486,12 +15625,12 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ADM-02</t>
+          <t>E2E-R1-NOT-05</t>
         </is>
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>People &amp; access: counts (members, no MFA, privileged, pending invites), member row (MFA off, last active set, not dormant), no-MFA and admin filters; unknown filter → 422; members get 403 | BPMS-063, FR-A06</t>
+          <t>During quiet hours a plain announcement email is held until the window ends; a critical one is not held | BPMS-048, FR-N04</t>
         </is>
       </c>
       <c r="D215" s="3" t="inlineStr">
@@ -15513,12 +15652,12 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-01</t>
+          <t>E2E-R1-LIB-01</t>
         </is>
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>Sign in through the browser (password + recovery code) lands on Home; navigation is permission-shaped with the current page marked; axe clean on sign-in and Home; reload keeps the session | docs/05 §2.1, §3.1, WCAG 2.2 AA</t>
+          <t>SOP draft → edit with `If-Match` (stale → 412) → submit (no review needed: approved, content hash frozen) → published; editing an approved version 409; content and hash identical on retrieval; one open draft per artifact | FR-G04, FR-G05, T07</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
@@ -15540,12 +15679,12 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-02</t>
+          <t>E2E-R1-LIB-02</t>
         </is>
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Wrong password and wrong code produce clear, non-revealing messages (role=alert); axe clean | docs/06 §3, WCAG 3.3.1</t>
+          <t>Controlled policy needs a review: the author's own approval is refused (403 `sod_violation`); a reviewer cannot publish; a reviewer approves; the owner publishes | FR-G04 SoD, docs/12 §6</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -15567,12 +15706,12 @@
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-03</t>
+          <t>E2E-R1-LIB-03</t>
         </is>
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>With several workspaces the chooser appears; choosing one and switching from the header changes the context and the navigation (no Admin for a plain member) | docs/05 §2.1 workspace switcher</t>
+          <t>Changes requested needs a comment and returns the draft; withdraw; later versions need a reason for change; publishing supersedes (previous → deprecated) | FR-G04, docs/20 §2.6</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
@@ -15594,12 +15733,12 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-04</t>
+          <t>E2E-R1-LIB-04</t>
         </is>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>The bell announces the unread count; the inbox lists the "joined" notification; mark all as read | FR-N01</t>
+          <t>A scheduled version goes live when its effective time passes (test clock + drain) and supersedes the live one; retire | FR-G05, FR-PL01</t>
         </is>
       </c>
       <c r="D219" s="3" t="inlineStr">
@@ -15621,12 +15760,12 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-05</t>
+          <t>E2E-R1-LIB-05</t>
         </is>
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>Sign out returns to sign-in; reloading stays signed out | docs/06 §3</t>
+          <t>Members read published policies but cannot author; lists contain only kinds the member may view | docs/12 §5</t>
         </is>
       </c>
       <c r="D220" s="3" t="inlineStr">
@@ -15648,12 +15787,12 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-06</t>
+          <t>E2E-R1-LIB-06</t>
         </is>
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Theme switched from the account menu persists across reload; dark theme passes axe | docs/05 §7, WCAG 2.2 AA</t>
+          <t>Semantic diff between two versions: one changed block with word-level detail, one added list, unchanged blocks kept; the reverse direction mirrors it; versions of different artifacts → 422; members may compare; another workspace gets 404 | BPMS-043, FR-G05</t>
         </is>
       </c>
       <c r="D221" s="3" t="inlineStr">
@@ -15675,12 +15814,12 @@
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-07</t>
+          <t>E2E-R1-LIB-07</t>
         </is>
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>Author a policy in the browser: New document dialog → write content (headings, lists) → save → submit → publish; the library row shows Published; axe clean | FR-G04, docs/05 §3.2/§3.21</t>
+          <t>Publishing sets `next_review_at = published + 365 d` (standard); a per-artifact cadence of 20 days moves it and makes it `due_soon`; 0 → 422; `null` restores the default; an unpublished artifact cannot be recertified (409) | BPMS-044, FR-G07, FX-G01</t>
         </is>
       </c>
       <c r="D222" s="3" t="inlineStr">
@@ -15702,12 +15841,12 @@
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-08</t>
+          <t>E2E-R1-LIB-08</t>
         </is>
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>A campaign task on Home leads to the document; “I acknowledge” records the acknowledgement (campaign progress +1) and the callout disappears | FR-AK01, docs/05 §3.1</t>
+          <t>A passed review date reads `overdue` immediately; the worker flags it once (two drains) and the owner receives one `review_overdue` notification linking the document; recertifying clears the flag and starts a new period; both are audited | BPMS-044, FR-G07, FX-G01</t>
         </is>
       </c>
       <c r="D223" s="3" t="inlineStr">
@@ -15729,12 +15868,12 @@
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-09</t>
+          <t>E2E-R1-LIB-09</t>
         </is>
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>Invite a colleague from Members with a role; the invitation appears in the table as Invited | FR-W01, docs/05 §3.14</t>
+          <t>Verification lasts `governance.verification.validity` (90 d) and expires on its own; members cannot verify (403); removing it twice → 409 | BPMS-044, FX-G02</t>
         </is>
       </c>
       <c r="D224" s="3" t="inlineStr">
@@ -15756,12 +15895,12 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-10</t>
+          <t>E2E-R1-LIB-10</t>
         </is>
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Read and acknowledge a critical, pinned announcement in the feed | FR-AN04, docs/05 §3.23</t>
+          <t>Change requests: a member proposes (blank title 422) but cannot resolve (403); declining needs a reason; accepted → implemented by a version of the same artifact (another artifact's version 422); resolved requests are final (409); list filters by state | BPMS-044, FR-G05</t>
         </is>
       </c>
       <c r="D225" s="3" t="inlineStr">
@@ -15783,12 +15922,12 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-11</t>
+          <t>E2E-R1-POL-01</t>
         </is>
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>An admin without two-step verification is guided through setup (QR + key, confirm a code, recovery codes) and then signs in with MFA and lands on Home | docs/06 §3, docs/20 §2.3</t>
+          <t>Readers never see drafts: absent from lists, reads and search until published; a later draft stays hidden (version 404, diff 404, versions list shows v1 only); authors see drafts in search | BPMS-045, A-14</t>
         </is>
       </c>
       <c r="D226" s="3" t="inlineStr">
@@ -15810,12 +15949,12 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-12</t>
+          <t>E2E-R1-POL-02</t>
         </is>
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>⌘K finds a document by its content and opens it; commands navigate; recent items are offered; keyboard only | BPMS-031, BPMS-049</t>
+          <t>Applicability: empty audience or restricted without one → 422; members cannot set it (403); a restricted policy is hidden from members outside its group in lists, reads, search, the portal and change requests (404), and shown to those inside; an unrestricted one is listed for everyone but only "applicable" to its audience | BPMS-045, FR-PL01/PL02</t>
         </is>
       </c>
       <c r="D227" s="3" t="inlineStr">
@@ -15837,12 +15976,12 @@
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-13</t>
+          <t>E2E-R1-POL-03</t>
         </is>
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>A new workspace shows composed empty states; an unknown page offers a way back; a failed load shows the error with a retry | BPMS-031 (UX-005)</t>
+          <t>The portal lists published policies that apply to the member (no drafts), ordered by category, with what changed since the previous version (added/changed counts, reason) and text/category filters | BPMS-045, FR-PL02</t>
         </is>
       </c>
       <c r="D228" s="3" t="inlineStr">
@@ -15864,12 +16003,12 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-14</t>
+          <t>E2E-R1-POL-04</t>
         </is>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>Manage announcements: compose a draft; a workspace-wide post is sent for approval; a targeted draft is published and shows receipts | BPMS-031, BPMS-047</t>
+          <t>A major version asks the applicable audience to re-acknowledge that exact version; a minor one does not (major_only) | BPMS-045, FR-PL03</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
@@ -15891,12 +16030,12 @@
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-15</t>
+          <t>E2E-R1-POL-05</t>
         </is>
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>Campaigns: create from a published document with an audience, check the reach, launch, follow progress, download the evidence CSV | BPMS-031, BPMS-046</t>
+          <t>Every_publish asks on minors, none never asks, and a scheduled major asks when it goes live | BPMS-045, FR-PL03</t>
         </is>
       </c>
       <c r="D230" s="3" t="inlineStr">
@@ -15918,12 +16057,12 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-16</t>
+          <t>E2E-R1-ADM-01</t>
         </is>
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>Settings: change a value in place with a reason and see why it applies; a step-up key asks to confirm identity | BPMS-031, BPMS-027</t>
+          <t>Overview: overdue acknowledgements rank first in "needs attention", followed by an admin without two-step verification; acknowledgement metrics and a daily published series; the security strip counts a failed sign-in, members without MFA and the new admin grant; requests/storage are null; members get 403; an inverted range → 422 | BPMS-063, FR-A01</t>
         </is>
       </c>
       <c r="D231" s="3" t="inlineStr">
@@ -15945,12 +16084,12 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-17</t>
+          <t>E2E-R1-ADM-02</t>
         </is>
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>Audit log: chain verified; filter by category; expand a record; open an object timeline; no-match state | BPMS-031, BPMS-064</t>
+          <t>People &amp; access: counts (members, no MFA, privileged, pending invites), member row (MFA off, last active set, not dormant), no-MFA and admin filters; unknown filter → 422; members get 403 | BPMS-063, FR-A06</t>
         </is>
       </c>
       <c r="D232" s="3" t="inlineStr">
@@ -15972,12 +16111,12 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-18</t>
+          <t>E2E-R1-UI-01</t>
         </is>
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>The owner sets a review schedule, recertifies when it falls due, verifies and removes verification | BPMS-044</t>
+          <t>Sign in through the browser (password + recovery code) lands on Home; navigation is permission-shaped with the current page marked; axe clean on sign-in and Home; reload keeps the session | docs/05 §2.1, §3.1, WCAG 2.2 AA</t>
         </is>
       </c>
       <c r="D233" s="3" t="inlineStr">
@@ -15999,12 +16138,12 @@
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-19</t>
+          <t>E2E-R1-UI-02</t>
         </is>
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>A member suggests a change; the owner accepts it and marks it implemented in v2 | BPMS-044</t>
+          <t>Wrong password and wrong code produce clear, non-revealing messages (role=alert); axe clean | docs/06 §3, WCAG 3.3.1</t>
         </is>
       </c>
       <c r="D234" s="3" t="inlineStr">
@@ -16026,12 +16165,12 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-20</t>
+          <t>E2E-R1-UI-03</t>
         </is>
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>Compare v1 and v2 from the version history: word-level changes and the summary | BPMS-043</t>
+          <t>With several workspaces the chooser appears; choosing one and switching from the header changes the context and the navigation (no Admin for a plain member) | docs/05 §2.1 workspace switcher</t>
         </is>
       </c>
       <c r="D235" s="3" t="inlineStr">
@@ -16053,12 +16192,12 @@
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-21</t>
+          <t>E2E-R1-UI-04</t>
         </is>
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>A member opens Policies, filters by category and follows "what changed" to the comparison | BPMS-045</t>
+          <t>The bell announces the unread count; the inbox lists the "joined" notification; mark all as read | FR-N01</t>
         </is>
       </c>
       <c r="D236" s="3" t="inlineStr">
@@ -16080,12 +16219,12 @@
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-22</t>
+          <t>E2E-R1-UI-05</t>
         </is>
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>A publisher restricts a policy to a role; a member outside it can't find it in Policies or open it | BPMS-045, A-14</t>
+          <t>Sign out returns to sign-in; reloading stays signed out | docs/06 §3</t>
         </is>
       </c>
       <c r="D237" s="3" t="inlineStr">
@@ -16107,12 +16246,12 @@
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-23</t>
+          <t>E2E-R1-UI-06</t>
         </is>
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>An admin opens Overview: the summary and "Needs attention" show overdue acknowledgements, and the security strip shows one member without two-step verification; drilling in opens People &amp; access filtered to them; the Admins filter shows the owner | BPMS-063</t>
+          <t>Theme switched from the account menu persists across reload; dark theme passes axe | docs/05 §7, WCAG 2.2 AA</t>
         </is>
       </c>
       <c r="D238" s="3" t="inlineStr">
@@ -16134,12 +16273,12 @@
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-01</t>
+          <t>E2E-R1-UI-07</t>
         </is>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
+          <t>Author a policy in the browser: New document dialog → write content (headings, lists) → save → submit → publish; the library row shows Published; axe clean | FR-G04, docs/05 §3.2/§3.21</t>
         </is>
       </c>
       <c r="D239" s="3" t="inlineStr">
@@ -16161,12 +16300,12 @@
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-02</t>
+          <t>E2E-R1-UI-08</t>
         </is>
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
+          <t>A campaign task on Home leads to the document; “I acknowledge” records the acknowledgement (campaign progress +1) and the callout disappears | FR-AK01, docs/05 §3.1</t>
         </is>
       </c>
       <c r="D240" s="3" t="inlineStr">
@@ -16188,12 +16327,12 @@
       </c>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-03</t>
+          <t>E2E-R1-UI-09</t>
         </is>
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
+          <t>Invite a colleague from Members with a role; the invitation appears in the table as Invited | FR-W01, docs/05 §3.14</t>
         </is>
       </c>
       <c r="D241" s="3" t="inlineStr">
@@ -16215,12 +16354,12 @@
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-04</t>
+          <t>E2E-R1-UI-10</t>
         </is>
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
+          <t>Read and acknowledge a critical, pinned announcement in the feed | FR-AN04, docs/05 §3.23</t>
         </is>
       </c>
       <c r="D242" s="3" t="inlineStr">
@@ -16242,12 +16381,12 @@
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-05</t>
+          <t>E2E-R1-UI-11</t>
         </is>
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
+          <t>An admin without two-step verification is guided through setup (QR + key, confirm a code, recovery codes) and then signs in with MFA and lands on Home | docs/06 §3, docs/20 §2.3</t>
         </is>
       </c>
       <c r="D243" s="3" t="inlineStr">
@@ -16269,12 +16408,12 @@
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-06</t>
+          <t>E2E-R1-UI-12</t>
         </is>
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
+          <t>⌘K finds a document by its content and opens it; commands navigate; recent items are offered; keyboard only | BPMS-031, BPMS-049</t>
         </is>
       </c>
       <c r="D244" s="3" t="inlineStr">
@@ -16296,12 +16435,12 @@
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-07</t>
+          <t>E2E-R1-UI-13</t>
         </is>
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
+          <t>A new workspace shows composed empty states; an unknown page offers a way back; a failed load shows the error with a retry | BPMS-031 (UX-005)</t>
         </is>
       </c>
       <c r="D245" s="3" t="inlineStr">
@@ -16323,12 +16462,12 @@
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-01</t>
+          <t>E2E-R1-UI-14</t>
         </is>
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
+          <t>Manage announcements: compose a draft; a workspace-wide post is sent for approval; a targeted draft is published and shows receipts | BPMS-031, BPMS-047</t>
         </is>
       </c>
       <c r="D246" s="3" t="inlineStr">
@@ -16350,12 +16489,12 @@
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-02</t>
+          <t>E2E-R1-UI-15</t>
         </is>
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
+          <t>Campaigns: create from a published document with an audience, check the reach, launch, follow progress, download the evidence CSV | BPMS-031, BPMS-046</t>
         </is>
       </c>
       <c r="D247" s="3" t="inlineStr">
@@ -16377,12 +16516,12 @@
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-03</t>
+          <t>E2E-R1-UI-16</t>
         </is>
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
+          <t>Settings: change a value in place with a reason and see why it applies; a step-up key asks to confirm identity | BPMS-031, BPMS-027</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
@@ -16404,12 +16543,12 @@
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-04</t>
+          <t>E2E-R1-UI-17</t>
         </is>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
+          <t>Audit log: chain verified; filter by category; expand a record; open an object timeline; no-match state | BPMS-031, BPMS-064</t>
         </is>
       </c>
       <c r="D249" s="3" t="inlineStr">
@@ -16431,12 +16570,12 @@
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-05</t>
+          <t>E2E-R1-UI-18</t>
         </is>
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
+          <t>The owner sets a review schedule, recertifies when it falls due, verifies and removes verification | BPMS-044</t>
         </is>
       </c>
       <c r="D250" s="3" t="inlineStr">
@@ -16458,12 +16597,12 @@
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-06</t>
+          <t>E2E-R1-UI-19</t>
         </is>
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
+          <t>A member suggests a change; the owner accepts it and marks it implemented in v2 | BPMS-044</t>
         </is>
       </c>
       <c r="D251" s="3" t="inlineStr">
@@ -16485,12 +16624,12 @@
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-01</t>
+          <t>E2E-R1-UI-20</t>
         </is>
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
+          <t>Compare v1 and v2 from the version history: word-level changes and the summary | BPMS-043</t>
         </is>
       </c>
       <c r="D252" s="3" t="inlineStr">
@@ -16512,12 +16651,12 @@
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-02</t>
+          <t>E2E-R1-UI-21</t>
         </is>
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
+          <t>A member opens Policies, filters by category and follows "what changed" to the comparison | BPMS-045</t>
         </is>
       </c>
       <c r="D253" s="3" t="inlineStr">
@@ -16539,12 +16678,12 @@
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-03</t>
+          <t>E2E-R1-UI-22</t>
         </is>
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
+          <t>A publisher restricts a policy to a role; a member outside it can't find it in Policies or open it | BPMS-045, A-14</t>
         </is>
       </c>
       <c r="D254" s="3" t="inlineStr">
@@ -16566,12 +16705,12 @@
       </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-01</t>
+          <t>E2E-R1-UI-23</t>
         </is>
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
+          <t>An admin opens Overview: the summary and "Needs attention" show overdue acknowledgements, and the security strip shows one member without two-step verification; drilling in opens People &amp; access filtered to them; the Admins filter shows the owner | BPMS-063</t>
         </is>
       </c>
       <c r="D255" s="3" t="inlineStr">
@@ -16593,12 +16732,12 @@
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-02</t>
+          <t>E2E-R1-UI-24</t>
         </is>
       </c>
       <c r="C256" s="3" t="inlineStr">
         <is>
-          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
+          <t>An owner publishes v2 as a major change, sees who will be asked, then finds the campaign | BPMS-045</t>
         </is>
       </c>
       <c r="D256" s="3" t="inlineStr">
@@ -16620,12 +16759,12 @@
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-03</t>
+          <t>E2E-R1-UI-25</t>
         </is>
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
+          <t>A member opens Notifications → Preferences, picks a daily digest and quiet hours, saves, sees them after a reload, and resets to the workspace defaults | BPMS-048</t>
         </is>
       </c>
       <c r="D257" s="3" t="inlineStr">
@@ -16647,12 +16786,12 @@
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-04</t>
+          <t>E2E-R1-UI-30</t>
         </is>
       </c>
       <c r="C258" s="3" t="inlineStr">
         <is>
-          <t>Chain verify reports intact | FR-T02</t>
+          <t>Add a passkey from Account › Security, sign out, sign in with password + passkey | BPMS-022</t>
         </is>
       </c>
       <c r="D258" s="3" t="inlineStr">
@@ -16674,12 +16813,12 @@
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-05</t>
+          <t>E2E-R1-UI-31</t>
         </is>
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
+          <t>Removing a passkey asks to confirm it’s you; the passkey itself passes step-up | BPMS-022</t>
         </is>
       </c>
       <c r="D259" s="3" t="inlineStr">
@@ -16701,12 +16840,12 @@
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-06</t>
+          <t>E2E-R1-UI-35</t>
         </is>
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
-          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
+          <t>Departments: override a setting for a parent department, see a child inherit it, then clear it | BPMS-027</t>
         </is>
       </c>
       <c r="D260" s="3" t="inlineStr">
@@ -16728,12 +16867,12 @@
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-UI-36</t>
         </is>
       </c>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>Configuration profile: preview a switch with every change, then switch with a reason | BPMS-027, CFG-017</t>
         </is>
       </c>
       <c r="D261" s="3" t="inlineStr">
@@ -16755,12 +16894,12 @@
       </c>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-UI-40</t>
         </is>
       </c>
       <c r="C262" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>A system admin finds a workspace, makes it read-only with a reason, and reactivates it | BPMS-065</t>
         </is>
       </c>
       <c r="D262" s="3" t="inlineStr">
@@ -16782,12 +16921,12 @@
       </c>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-UI-41</t>
         </is>
       </c>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>Quotas, platform health and the system audit; non-system users never see the console | BPMS-065</t>
         </is>
       </c>
       <c r="D263" s="3" t="inlineStr">
@@ -16809,12 +16948,12 @@
       </c>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-CMP-01</t>
         </is>
       </c>
       <c r="C264" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
         </is>
       </c>
       <c r="D264" s="3" t="inlineStr">
@@ -16836,12 +16975,12 @@
       </c>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-CMP-02</t>
         </is>
       </c>
       <c r="C265" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
         </is>
       </c>
       <c r="D265" s="3" t="inlineStr">
@@ -16863,12 +17002,12 @@
       </c>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-CMP-03</t>
         </is>
       </c>
       <c r="C266" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
         </is>
       </c>
       <c r="D266" s="3" t="inlineStr">
@@ -16890,12 +17029,12 @@
       </c>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-CMP-04</t>
         </is>
       </c>
       <c r="C267" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
         </is>
       </c>
       <c r="D267" s="3" t="inlineStr">
@@ -16917,12 +17056,12 @@
       </c>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-CMP-05</t>
         </is>
       </c>
       <c r="C268" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
         </is>
       </c>
       <c r="D268" s="3" t="inlineStr">
@@ -16944,12 +17083,12 @@
       </c>
       <c r="B269" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-CMP-06</t>
         </is>
       </c>
       <c r="C269" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
         </is>
       </c>
       <c r="D269" s="3" t="inlineStr">
@@ -16971,12 +17110,12 @@
       </c>
       <c r="B270" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-CMP-07</t>
         </is>
       </c>
       <c r="C270" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D270" s="3" t="inlineStr">
@@ -16998,12 +17137,12 @@
       </c>
       <c r="B271" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-ANN-01</t>
         </is>
       </c>
       <c r="C271" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
         </is>
       </c>
       <c r="D271" s="3" t="inlineStr">
@@ -17025,12 +17164,12 @@
       </c>
       <c r="B272" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-ANN-02</t>
         </is>
       </c>
       <c r="C272" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
         </is>
       </c>
       <c r="D272" s="3" t="inlineStr">
@@ -17052,12 +17191,12 @@
       </c>
       <c r="B273" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-ANN-03</t>
         </is>
       </c>
       <c r="C273" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
         </is>
       </c>
       <c r="D273" s="3" t="inlineStr">
@@ -17079,12 +17218,12 @@
       </c>
       <c r="B274" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-ANN-04</t>
         </is>
       </c>
       <c r="C274" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
         </is>
       </c>
       <c r="D274" s="3" t="inlineStr">
@@ -17106,12 +17245,12 @@
       </c>
       <c r="B275" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-ANN-05</t>
         </is>
       </c>
       <c r="C275" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D275" s="3" t="inlineStr">
@@ -17133,12 +17272,12 @@
       </c>
       <c r="B276" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-ANN-06</t>
         </is>
       </c>
       <c r="C276" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
         </is>
       </c>
       <c r="D276" s="3" t="inlineStr">
@@ -17160,12 +17299,12 @@
       </c>
       <c r="B277" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-SRCH-01</t>
         </is>
       </c>
       <c r="C277" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
         </is>
       </c>
       <c r="D277" s="3" t="inlineStr">
@@ -17187,12 +17326,12 @@
       </c>
       <c r="B278" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-SRCH-02</t>
         </is>
       </c>
       <c r="C278" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
         </is>
       </c>
       <c r="D278" s="3" t="inlineStr">
@@ -17214,12 +17353,12 @@
       </c>
       <c r="B279" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-SRCH-03</t>
         </is>
       </c>
       <c r="C279" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
         </is>
       </c>
       <c r="D279" s="3" t="inlineStr">
@@ -17241,12 +17380,12 @@
       </c>
       <c r="B280" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-AUDX-01</t>
         </is>
       </c>
       <c r="C280" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
         </is>
       </c>
       <c r="D280" s="3" t="inlineStr">
@@ -17268,12 +17407,12 @@
       </c>
       <c r="B281" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-AUDX-02</t>
         </is>
       </c>
       <c r="C281" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
         </is>
       </c>
       <c r="D281" s="3" t="inlineStr">
@@ -17295,12 +17434,12 @@
       </c>
       <c r="B282" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R1-AUDX-03</t>
         </is>
       </c>
       <c r="C282" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
         </is>
       </c>
       <c r="D282" s="3" t="inlineStr">
@@ -17322,12 +17461,12 @@
       </c>
       <c r="B283" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R1-AUDX-04</t>
         </is>
       </c>
       <c r="C283" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>Chain verify reports intact | FR-T02</t>
         </is>
       </c>
       <c r="D283" s="3" t="inlineStr">
@@ -17349,12 +17488,12 @@
       </c>
       <c r="B284" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R1-AUDX-05</t>
         </is>
       </c>
       <c r="C284" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
         </is>
       </c>
       <c r="D284" s="3" t="inlineStr">
@@ -17376,12 +17515,12 @@
       </c>
       <c r="B285" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R1-AUDX-06</t>
         </is>
       </c>
       <c r="C285" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
         </is>
       </c>
       <c r="D285" s="3" t="inlineStr">
@@ -17403,12 +17542,12 @@
       </c>
       <c r="B286" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C286" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
         </is>
       </c>
       <c r="D286" s="3" t="inlineStr">
@@ -17430,12 +17569,12 @@
       </c>
       <c r="B287" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C287" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D287" s="3" t="inlineStr">
@@ -17457,12 +17596,12 @@
       </c>
       <c r="B288" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C288" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D288" s="3" t="inlineStr">
@@ -17484,12 +17623,12 @@
       </c>
       <c r="B289" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C289" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
         </is>
       </c>
       <c r="D289" s="3" t="inlineStr">
@@ -17511,12 +17650,12 @@
       </c>
       <c r="B290" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C290" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
         </is>
       </c>
       <c r="D290" s="3" t="inlineStr">
@@ -17538,12 +17677,12 @@
       </c>
       <c r="B291" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C291" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D291" s="3" t="inlineStr">
@@ -17565,12 +17704,12 @@
       </c>
       <c r="B292" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C292" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D292" s="3" t="inlineStr">
@@ -17592,12 +17731,12 @@
       </c>
       <c r="B293" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C293" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
         </is>
       </c>
       <c r="D293" s="3" t="inlineStr">
@@ -17619,12 +17758,12 @@
       </c>
       <c r="B294" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C294" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D294" s="3" t="inlineStr">
@@ -17646,12 +17785,12 @@
       </c>
       <c r="B295" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C295" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D295" s="3" t="inlineStr">
@@ -17673,12 +17812,12 @@
       </c>
       <c r="B296" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C296" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D296" s="3" t="inlineStr">
@@ -17700,12 +17839,12 @@
       </c>
       <c r="B297" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C297" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D297" s="3" t="inlineStr">
@@ -17727,12 +17866,12 @@
       </c>
       <c r="B298" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C298" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
         </is>
       </c>
       <c r="D298" s="3" t="inlineStr">
@@ -17754,12 +17893,12 @@
       </c>
       <c r="B299" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C299" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
         </is>
       </c>
       <c r="D299" s="3" t="inlineStr">
@@ -17781,12 +17920,12 @@
       </c>
       <c r="B300" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C300" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
         </is>
       </c>
       <c r="D300" s="3" t="inlineStr">
@@ -17808,12 +17947,12 @@
       </c>
       <c r="B301" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C301" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D301" s="3" t="inlineStr">
@@ -17835,12 +17974,12 @@
       </c>
       <c r="B302" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C302" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
         </is>
       </c>
       <c r="D302" s="3" t="inlineStr">
@@ -17862,12 +18001,12 @@
       </c>
       <c r="B303" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C303" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
         </is>
       </c>
       <c r="D303" s="3" t="inlineStr">
@@ -17889,12 +18028,12 @@
       </c>
       <c r="B304" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C304" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D304" s="3" t="inlineStr">
@@ -17916,12 +18055,12 @@
       </c>
       <c r="B305" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C305" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
         </is>
       </c>
       <c r="D305" s="3" t="inlineStr">
@@ -17943,12 +18082,12 @@
       </c>
       <c r="B306" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C306" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D306" s="3" t="inlineStr">
@@ -17970,12 +18109,12 @@
       </c>
       <c r="B307" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C307" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D307" s="3" t="inlineStr">
@@ -17997,12 +18136,12 @@
       </c>
       <c r="B308" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C308" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D308" s="3" t="inlineStr">
@@ -18024,12 +18163,12 @@
       </c>
       <c r="B309" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C309" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D309" s="3" t="inlineStr">
@@ -18051,12 +18190,12 @@
       </c>
       <c r="B310" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C310" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D310" s="3" t="inlineStr">
@@ -18078,12 +18217,12 @@
       </c>
       <c r="B311" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C311" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D311" s="3" t="inlineStr">
@@ -18105,12 +18244,12 @@
       </c>
       <c r="B312" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C312" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D312" s="3" t="inlineStr">
@@ -18132,12 +18271,12 @@
       </c>
       <c r="B313" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C313" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D313" s="3" t="inlineStr">
@@ -18159,12 +18298,12 @@
       </c>
       <c r="B314" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C314" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D314" s="3" t="inlineStr">
@@ -18186,12 +18325,12 @@
       </c>
       <c r="B315" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C315" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D315" s="3" t="inlineStr">
@@ -18213,12 +18352,12 @@
       </c>
       <c r="B316" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C316" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D316" s="3" t="inlineStr">
@@ -18240,12 +18379,12 @@
       </c>
       <c r="B317" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C317" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D317" s="3" t="inlineStr">
@@ -18267,12 +18406,12 @@
       </c>
       <c r="B318" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C318" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D318" s="3" t="inlineStr">
@@ -18294,12 +18433,12 @@
       </c>
       <c r="B319" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C319" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D319" s="3" t="inlineStr">
@@ -18321,12 +18460,12 @@
       </c>
       <c r="B320" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C320" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D320" s="3" t="inlineStr">
@@ -18348,12 +18487,12 @@
       </c>
       <c r="B321" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C321" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D321" s="3" t="inlineStr">
@@ -18375,12 +18514,12 @@
       </c>
       <c r="B322" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C322" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D322" s="3" t="inlineStr">
@@ -18402,12 +18541,12 @@
       </c>
       <c r="B323" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C323" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D323" s="3" t="inlineStr">
@@ -18429,12 +18568,12 @@
       </c>
       <c r="B324" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C324" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D324" s="3" t="inlineStr">
@@ -18456,12 +18595,12 @@
       </c>
       <c r="B325" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C325" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D325" s="3" t="inlineStr">
@@ -18483,12 +18622,12 @@
       </c>
       <c r="B326" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C326" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D326" s="3" t="inlineStr">
@@ -18510,12 +18649,12 @@
       </c>
       <c r="B327" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C327" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D327" s="3" t="inlineStr">
@@ -18537,12 +18676,12 @@
       </c>
       <c r="B328" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C328" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D328" s="3" t="inlineStr">
@@ -18564,12 +18703,12 @@
       </c>
       <c r="B329" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C329" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D329" s="3" t="inlineStr">
@@ -18591,12 +18730,12 @@
       </c>
       <c r="B330" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C330" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D330" s="3" t="inlineStr">
@@ -18618,12 +18757,12 @@
       </c>
       <c r="B331" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C331" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D331" s="3" t="inlineStr">
@@ -18645,12 +18784,12 @@
       </c>
       <c r="B332" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C332" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D332" s="3" t="inlineStr">
@@ -18672,12 +18811,12 @@
       </c>
       <c r="B333" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C333" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D333" s="3" t="inlineStr">
@@ -18699,20 +18838,695 @@
       </c>
       <c r="B334" s="3" t="inlineStr">
         <is>
+          <t>E2E-R3-12</t>
+        </is>
+      </c>
+      <c r="C334" s="3" t="inlineStr">
+        <is>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+        </is>
+      </c>
+      <c r="D334" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E334" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B335" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R3-MOB</t>
+        </is>
+      </c>
+      <c r="C335" s="3" t="inlineStr">
+        <is>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+        </is>
+      </c>
+      <c r="D335" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E335" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B336" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R3-ISO</t>
+        </is>
+      </c>
+      <c r="C336" s="3" t="inlineStr">
+        <is>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+        </is>
+      </c>
+      <c r="D336" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E336" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B337" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-01</t>
+        </is>
+      </c>
+      <c r="C337" s="3" t="inlineStr">
+        <is>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+        </is>
+      </c>
+      <c r="D337" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E337" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B338" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-02</t>
+        </is>
+      </c>
+      <c r="C338" s="3" t="inlineStr">
+        <is>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+        </is>
+      </c>
+      <c r="D338" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E338" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B339" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-03</t>
+        </is>
+      </c>
+      <c r="C339" s="3" t="inlineStr">
+        <is>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+        </is>
+      </c>
+      <c r="D339" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E339" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B340" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-04</t>
+        </is>
+      </c>
+      <c r="C340" s="3" t="inlineStr">
+        <is>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+        </is>
+      </c>
+      <c r="D340" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E340" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B341" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-05</t>
+        </is>
+      </c>
+      <c r="C341" s="3" t="inlineStr">
+        <is>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+        </is>
+      </c>
+      <c r="D341" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E341" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B342" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-06</t>
+        </is>
+      </c>
+      <c r="C342" s="3" t="inlineStr">
+        <is>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+        </is>
+      </c>
+      <c r="D342" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E342" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B343" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-07</t>
+        </is>
+      </c>
+      <c r="C343" s="3" t="inlineStr">
+        <is>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+        </is>
+      </c>
+      <c r="D343" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E343" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B344" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-08</t>
+        </is>
+      </c>
+      <c r="C344" s="3" t="inlineStr">
+        <is>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+        </is>
+      </c>
+      <c r="D344" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E344" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B345" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-09</t>
+        </is>
+      </c>
+      <c r="C345" s="3" t="inlineStr">
+        <is>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+        </is>
+      </c>
+      <c r="D345" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E345" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B346" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-10</t>
+        </is>
+      </c>
+      <c r="C346" s="3" t="inlineStr">
+        <is>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+        </is>
+      </c>
+      <c r="D346" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E346" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B347" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-11</t>
+        </is>
+      </c>
+      <c r="C347" s="3" t="inlineStr">
+        <is>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+        </is>
+      </c>
+      <c r="D347" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E347" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B348" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-ISO</t>
+        </is>
+      </c>
+      <c r="C348" s="3" t="inlineStr">
+        <is>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+        </is>
+      </c>
+      <c r="D348" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E348" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B349" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-01</t>
+        </is>
+      </c>
+      <c r="C349" s="3" t="inlineStr">
+        <is>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+        </is>
+      </c>
+      <c r="D349" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E349" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B350" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-02</t>
+        </is>
+      </c>
+      <c r="C350" s="3" t="inlineStr">
+        <is>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+        </is>
+      </c>
+      <c r="D350" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E350" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B351" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-03</t>
+        </is>
+      </c>
+      <c r="C351" s="3" t="inlineStr">
+        <is>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+        </is>
+      </c>
+      <c r="D351" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E351" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B352" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-04</t>
+        </is>
+      </c>
+      <c r="C352" s="3" t="inlineStr">
+        <is>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+        </is>
+      </c>
+      <c r="D352" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E352" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B353" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-05</t>
+        </is>
+      </c>
+      <c r="C353" s="3" t="inlineStr">
+        <is>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+        </is>
+      </c>
+      <c r="D353" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E353" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B354" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-06</t>
+        </is>
+      </c>
+      <c r="C354" s="3" t="inlineStr">
+        <is>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+        </is>
+      </c>
+      <c r="D354" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E354" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B355" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-07</t>
+        </is>
+      </c>
+      <c r="C355" s="3" t="inlineStr">
+        <is>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+        </is>
+      </c>
+      <c r="D355" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E355" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B356" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-08</t>
+        </is>
+      </c>
+      <c r="C356" s="3" t="inlineStr">
+        <is>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+        </is>
+      </c>
+      <c r="D356" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E356" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B357" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-09</t>
+        </is>
+      </c>
+      <c r="C357" s="3" t="inlineStr">
+        <is>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+        </is>
+      </c>
+      <c r="D357" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E357" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B358" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C358" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D358" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E358" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B359" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C334" s="3" t="inlineStr">
+      <c r="C359" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D334" s="3" t="inlineStr">
+      <c r="D359" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E334" s="3" t="inlineStr">
+      <c r="E359" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
docs: tracker for flows, review/approval notifications, BPMS-062 files view, BPMS-081/082 merged
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -197,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E20" headerRowCount="1">
-  <autoFilter ref="A1:E20"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E26" headerRowCount="1">
+  <autoFilter ref="A1:E26"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Source"/>
     <tableColumn id="2" name="ID"/>
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E359" headerRowCount="1">
-  <autoFilter ref="A1:E359"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E390" headerRowCount="1">
+  <autoFilter ref="A1:E390"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -324,8 +324,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="OpenQuestionsT" displayName="OpenQuestionsT" ref="A1:G15" headerRowCount="1">
-  <autoFilter ref="A1:G15"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="OpenQuestionsT" displayName="OpenQuestionsT" ref="A1:G16" headerRowCount="1">
+  <autoFilter ref="A1:G16"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Source"/>
     <tableColumn id="2" name="ID"/>
@@ -1393,7 +1393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1942,6 +1942,156 @@
           <t>Add an attestation/AAGUID policy setting; require UV for admin roles; move passkey-only sign-in earlier</t>
         </is>
       </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>A-20 (BPMS-041)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Collection visibility applies to view-only readers like A-14: a document is hidden when any collection on its path restricts visibility to an audience the reader is outside of; authors (create/edit/review/approve/publish on the kind) and collection managers see everything. Collection-scoped role grants (docs/12 §5 scope `collection`) do not yet narrow document permissions; checks stay workspace-wide</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Product-owner review</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Honour collection-scoped grants in document permission checks (resource-scoped evaluation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>A-21 (BPMS-080)</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>IR compiler (docs/11 §14): (1) the input is an IR v1 document as authored, not yet normalised; each editor maps its canvas JSON to that shape. (2) The normal form fills `on: next`, sorts nodes and edges by id, variables by name and SLAs by id, and sets `meta.compilerVersion`, which is hashed with the rest. (3) An outcome handled by two edges is an error (IR-E017), because it would be an implicit fork. (4) For the `restricted` rule, the event-facing fields are every `notify` field, `correlation` and `idempotencyKey`. (5) In a `controlled` process every `outcome` escalation is rejected, not only auto-approval. (6) Zero-length durations are rejected. (7) `subject` names `policy`, `sop` or a `refs.documents` key; `document` names a `refs.documents` key or a `file` variable; `quiz` names a `refs.forms` key. (8) SLA `pauseWhile` entries are node ids, optionally prefixed with the node kind (`wait.signal:vendor-quote`). (9) A variable with no classification counts as not restricted, and the compiler adds no default. (10) With no workspace environment, checks 8–10 are skipped and IR-I001 is reported</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Runtime-lead review of docs/11 §14; feedback from the designer (BPMS-05x) and publish integration (BPMS-084)</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Change the normal form (and bump `COMPILER_VERSION`); allow selected auto-outcomes in controlled processes; widen or narrow the event-facing field list</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>A-22 (BPMS-081)</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Expression engine, as built (docs/11 §6.1). (1) **Our own CEL-subset implementation** (parser, type checker, evaluator) instead of `cel-rust`. `cel-rust` has no step budget (only the non-deterministic wall-clock guard SP-08 suggested, and `wasm32` has no clock), uses IEEE doubles, and has no static checker. Our implementation follows CEL syntax and precedence, so it is a CEL subset, not the custom DSL ADR-0010 rejects. (2) There is no floating point: `1.5` is an exact decimal, and an integer is accepted wherever a decimal is. (3) `&amp;&amp;`/`</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>` short-circuit left to right; CEL's commutative error absorption is not implemented. (4) Fields of inline `record` types are required. The built-in shapes are principal (`id`, `manager?`, `department?`, `email?`), group (`id`, `name?`), file (`name`, `hash`, `size`, `content_type?`) and instance (`id`, `display_id`, `started_at`). (5) `today()` and date parts use a fixed UTC offset that the caller injects, resolved from the process calendar at `now`; there is no IANA zone database in the engine. (6) Rounding is half away from zero. (7) Event-facing contexts (notify templates, values copied into events, idempotency keys) reject `restricted` reads; confidential reads are allowed and the result carries the classification. (8) Budget defaults: 10 000 steps, 1 MiB allocation, 64 KiB strings, 10 000-element lists, evaluator depth 64. The step budget replaces SP-08's 10 ms wall-clock guard</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>A-23 (BPMS-082)</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Native interpreter (docs/11 §15): (1) `set` evaluates every expression against the variables as they were before the node (parallel assignment). (2) A rule-table decision whose output is null or names no branch takes `default`; an expression branch whose condition is not a boolean raises incident IR-R002 (docs/11 §6). (3) Runtime incident codes besides IR-R010: IR-R001 expression failed, IR-R002 non-boolean condition, IR-R003 no edge for an outcome without `unhandled: fail`, IR-R004 loop guard, IR-R005 join outside its split, IR-R006 bad value (timer instant, idempotency key). An incident parks the token; the instance keeps running (docs/04 §4.1 default policy). (4) Loop guard: a node is entered at most `maxIterations` times when it declares one, else 1,000 times per instance; the next entry raises IR-R004. (5) A boundary without `interrupting` interrupts (BPMN default). A non-interrupting boundary token keeps its parent's branch frames; a join counts each branch once. (6) A typed connector error `error:&lt;CODE&gt;` goes to the matching `error:&lt;CODE&gt;` boundary, else to the `error` outcome. (7) Cancelling or terminating withdraws work items, timers, subscriptions and child instances; in-flight connector calls and opened cases are not cancelled, and a late connector result is refused as an unknown key. (8) An outcome produced with no edge and `unhandled: fail` fails the instance. (9) Instance status `terminated` covers both `end{result: terminated}` and an instance cancel (docs/04 stores `cancelled`). (10) Activation and command keys are `&lt;instance&gt;/&lt;node&gt;/&lt;n&gt;` with `n` from the instance's own counter; the connector receives the evaluated `idempotencyKey` separately. (11) Runtime conformance fixtures live in `conformance/runtime/&lt;group&gt;/&lt;case&gt;/` (the repository's conformance crate, docs/04 §1) rather than `crates/runtime/conformance/fixtures/` (docs/15 §4), and the script is `script.json`, not `script.yaml`, to avoid a YAML dependency. Traces are compared in total order, since the native interpreter is deterministic</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Runtime-lead review of docs/11 §15; BPMS-083/085/088 integration</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Change the parallel-assignment rule; make the loop default 50 (docs/11 §4) for every node; cancel in-flight connector calls; move the fixtures and adopt YAML</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>A-24 (BPMS-023)</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Invitation page: whoever holds the link (the token is the credential, 7-day single use) may see the invited email, the workspace name, the inviter's name, the expiry and whether that email already has an account, so the page can offer "create account" or "sign in to accept" (`GET /invitations/preview`, public, read-only, not audited). Signed in as a different email, the page says so and offers sign-out; it never accepts for another address. After sign-in, any same-origin `next` path is restored (deep links from emails survive sign-in); a deliberate sign-out drops it.</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>A-25 (BPMS-040)</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Review notifications: on submit (when a review is required) every active member holding `{kind}:review` or `{kind}:approve` through a live grant at any scope, except the author, gets an in-app notice and an urgent email; scoped grants are not narrowed to the document's collection yet. The author gets the outcome (approved and ready to publish, changes requested or rejected, with the reviewer's comment) in-app and as a normal email (digest rules apply). A partial approval (more approvals still needed) notifies nobody. Announcements follow the same rule: on submit when approval applies, holders of `announcement:publish` or `announcement:manage` except the author are told (urgent); the author hears approved or sent back with the note.</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4228,7 +4378,7 @@
       <c r="N19" s="3" t="inlineStr"/>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>procera-members + /api/v1: memberships, invitations (hashed + sealed tokens, 7-day expiry, email-bound, single use; list, revoke, resend), register-by-invite, owner onboarding activates the workspace, workspace switch (ws-scoped JWT), deactivation guards, state gate (423). Directory (migration 0008): department tree (uuid[] paths, sibling-unique names, no moves under descendants), static groups, positions (behind directory.positions.enabled), manager links with cycle rejection, deterministic manager resolution (explicit → nearest department head), per-field source attribution, CSV import with plan/apply. All audited; E2E-R1-MEM-01..03,05..07, E2E-R1-DIR-01..04</t>
+          <t>procera-members + /api/v1: memberships, invitations (hashed + sealed tokens, 7-day expiry, email-bound, single use; list, revoke, resend), register-by-invite, owner onboarding activates the workspace, workspace switch (ws-scoped JWT), deactivation guards, state gate (423). Directory (migration 0008): department tree (uuid[] paths, sibling-unique names, no moves under descendants), static groups, positions (behind directory.positions.enabled), manager links with cycle rejection, deterministic manager resolution (explicit → nearest department head), per-field source attribution, CSV import with plan/apply. All audited; E2E-R1-MEM-01..03,05..07, E2E-R1-DIR-01..04 Invitation page /invite (GET /invitations/preview, A-24): create account and join, or sign in and join; deep links survive sign-in. E2E-R1-FLOW-01, 02.</t>
         </is>
       </c>
     </row>
@@ -4545,13 +4695,17 @@
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L24" s="3" t="inlineStr"/>
       <c r="M24" s="3" t="inlineStr"/>
       <c r="N24" s="3" t="inlineStr"/>
-      <c r="O24" s="3" t="inlineStr"/>
+      <c r="O24" s="3" t="inlineStr">
+        <is>
+          <t>DataGrid v1 (web/src/ui/components/DataGrid.tsx): quick search, typed filter builder with chips and plain-language summary, multi-sort with order numbers, columns chooser, density, formula-safe CSV export audited via POST /exports, saved views per list (personal/shared, default, modified marker; migration 0028; /views API) with URL state, selection with shift-range and bulk actions, Enter/Space keyboard, live count, cards below 40rem; adopted by Library and Members. E2E-R1-VIEW-01, E2E-R1-UI-38, E2E-P0-10. Later: server-driven query + cursor paging, XLSX/async export, AND/OR groups, column resize.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -4679,7 +4833,7 @@
       <c r="N26" s="3" t="inlineStr"/>
       <c r="O26" s="3" t="inlineStr">
         <is>
-          <t>procera-crypto: LocalKey (env root key, HMAC-derived purpose keys), AES-256-GCM seal/open bound to context, token helpers, procera keygen. Remaining: KMS/OpenBao adapters, per-workspace KEKs, rotation</t>
+          <t>procera-crypto: LocalKey root, AES-256-GCM seal/open, envelope_* (per-value DEK wrapped by a versioned KEK; rewrap without re-encryption). procera-keys (migration 0026): per-workspace versioned KEKs root-sealed, lazy v1, rotation (reason + step-up, audited), background rewrap of registered envelope columns, unused retired keys destroyed, crypto-shred; email bodies moved to workspace envelopes (legacy still opens); Encryption admin page. E2E-R1-KEY-01, E2E-R1-UI-29, keys integration test. Remaining: KMS / OpenBao root adapters, yearly auto-rotation, files and restricted fields on envelopes as they land</t>
         </is>
       </c>
     </row>
@@ -4996,7 +5150,7 @@
       <c r="N31" s="3" t="inlineStr"/>
       <c r="O31" s="3" t="inlineStr">
         <is>
-          <t>procera-library (migration 0012): artifacts + versions for SOPs and policies; lifecycle draft → in_review → approved → scheduled/published → deprecated → retired with guarded transitions; one open draft per artifact; reviews in numbered rounds, approvals from governance.review.* settings, author never reviews own version, distinct approvers, comment required to reject; content_hash = SHA-256(JCS) frozen at approval and a trigger forbids changing approved content or moving back (T07); publish supersedes, future effective_at schedules (worker + drain), reason for change on later versions, retire; step-up for controlled approve/publish; outbox artifact.published.v1; every transition audited. E2E-R1-LIB-01..05. Process artifacts arrive with the designer/compiler</t>
+          <t>procera-library (migration 0012): artifacts + versions for SOPs and policies; lifecycle draft → in_review → approved → scheduled/published → deprecated → retired with guarded transitions; one open draft per artifact; reviews in numbered rounds, approvals from governance.review.* settings, author never reviews own version, distinct approvers, comment required to reject; content_hash = SHA-256(JCS) frozen at approval and a trigger forbids changing approved content or moving back (T07); publish supersedes, future effective_at schedules (worker + drain), reason for change on later versions, retire; step-up for controlled approve/publish; outbox artifact.published.v1; every transition audited. E2E-R1-LIB-01..05. Process artifacts arrive with the designer/compiler Review notifications (A-25): reviewers told on submit (in-app + email), author told the outcome with the comment. E2E-R1-FLOW-03, 05.</t>
         </is>
       </c>
     </row>
@@ -5053,13 +5207,17 @@
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L32" s="3" t="inlineStr"/>
       <c r="M32" s="3" t="inlineStr"/>
       <c r="N32" s="3" t="inlineStr"/>
-      <c r="O32" s="3" t="inlineStr"/>
+      <c r="O32" s="3" t="inlineStr">
+        <is>
+          <t>Collections (migration 0025): a tree with uuid[] paths, sibling-unique names, moves that rewrite the subtree, empty-only deletion; per-collection visibility (audience) hiding filed documents from view-only readers in lists, reads, search, the policy portal and the tree (A-20); document owner hand-over; RACI per document (members or groups, one accountable) with formula-safe CSV export (audited); Library collection rail with filtering and management, document-page Collection/Owner/RACI rows. E2E-R1-LIB-11..13, E2E-R1-UI-27. Later: landscape for processes (domain › capability › process) with the designer, collection-scoped grants (A-20).</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -5114,13 +5272,17 @@
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L33" s="3" t="inlineStr"/>
       <c r="M33" s="3" t="inlineStr"/>
       <c r="N33" s="3" t="inlineStr"/>
-      <c r="O33" s="3" t="inlineStr"/>
+      <c r="O33" s="3" t="inlineStr">
+        <is>
+          <t>Block editor (TipTap core, MIT; U-10 closed): headings, bold/italic/links, bullet and numbered lists, callouts, tables, accessible single-tab-stop toolbar, markdown shortcuts; block model validated server-side (ADR-0013 as built); shared renderer; HTML (print to tagged PDF in the browser) and Markdown export with a superseded banner, audited. E2E-R1-LIB-14, E2E-R1-UI-07, 28. Remaining: deterministic server-side tagged PDF, DOCX export/import, images and variables blocks.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -5443,7 +5605,7 @@
       <c r="N38" s="3" t="inlineStr"/>
       <c r="O38" s="3" t="inlineStr">
         <is>
-          <t>procera-announcements (migration 0014): drafts with block content, audience snapshot, approval per announcements.approval_required with SoD, scheduling + derived expiry, pinned/critical, channels from settings, in-app + email delivery via the outbox, read and acknowledgement receipts, analytics, archive; settings announcements.*; E2E-R1-ANN-01..06. Later: poster scoping, reminders/escalation for unacked, comments/reactions, reach preview</t>
+          <t>procera-announcements (migration 0014): drafts with block content, audience snapshot, approval per announcements.approval_required with SoD, scheduling + derived expiry, pinned/critical, channels from settings, in-app + email delivery via the outbox, read and acknowledgement receipts, analytics, archive; settings announcements.*; E2E-R1-ANN-01..06. Later: poster scoping, reminders/escalation for unacked, comments/reactions, reach preview Approval loop notifications (A-25): approvers told on submit, author told approved or sent back. E2E-R1-FLOW-04, 06.</t>
         </is>
       </c>
     </row>
@@ -5630,13 +5792,17 @@
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L41" s="3" t="inlineStr"/>
       <c r="M41" s="3" t="inlineStr"/>
       <c r="N41" s="3" t="inlineStr"/>
-      <c r="O41" s="3" t="inlineStr"/>
+      <c r="O41" s="3" t="inlineStr">
+        <is>
+          <t>procera-files (migration 0027): resumable chunked upload (offset-checked, resume from received), size limit and storage quota, SHA-256, magic-byte type with a platform deny list (executables, scripts, HTML, SVG), clamd INSTREAM scanner (built-in EICAR-only fallback, warned), quarantine and rejection, per-file DEK under the workspace KEK (rotated and shredded with it), local storage port, 5-minute signed download links re-authorized per request (nosniff, CSP sandbox), audited; attachments on draft versions fixed once past draft. E2E-R1-FILE-01..03, E2E-R1-UI-32..33. Remaining: S3-compatible storage backend, EXIF stripping at upload (previews done in BPMS-061), attachments elsewhere (forms, cases).</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -5691,13 +5857,17 @@
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L42" s="3" t="inlineStr"/>
       <c r="M42" s="3" t="inlineStr"/>
       <c r="N42" s="3" t="inlineStr"/>
-      <c r="O42" s="3" t="inlineStr"/>
+      <c r="O42" s="3" t="inlineStr">
+        <is>
+          <t>Image/PDF previews: GET /files/{id}/preview-url (kind image|pdf|none) and GET /files/preview/{token} (own preview HMAC purpose, 2-minute TTL, re-authorized per request; clean PNG/JPEG/GIF/WebP/PDF only by recorded type plus fresh sniff, else 415; inline under CSP sandbox, nosniff, CORP same-origin, no-store; audited file.previewed); JPEG Exif/XMP/IPTC stripped from previews (files.exif_strip); Preview dialog on attachments. E2E-R1-FILE-04, E2E-R1-UI-34. Remaining: separate preview origin, EXIF strip at upload, Office preview (P1).</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -5752,13 +5922,17 @@
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L43" s="3" t="inlineStr"/>
       <c r="M43" s="3" t="inlineStr"/>
       <c r="N43" s="3" t="inlineStr"/>
-      <c r="O43" s="3" t="inlineStr"/>
+      <c r="O43" s="3" t="inlineStr">
+        <is>
+          <t>Files admin view: usage against the storage quota, scan states, every file with uploader, use and scan result, delete (blocked while held by a version past draft), orphan report and purge (files.orphan_purge_after). E2E-R1-FILE-03, E2E-R1-UI-33. Files view on the DataGrid: retention class per file (from what holds it), last accessed (migration 0030, set on download/preview), bulk delete; audit-export files held by their job. E2E-R1-UI-43. Remaining: legal hold column (holds engine is BPMS-164).</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -5878,7 +6052,7 @@
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L45" s="3" t="inlineStr"/>
@@ -5886,7 +6060,7 @@
       <c r="N45" s="3" t="inlineStr"/>
       <c r="O45" s="3" t="inlineStr">
         <is>
-          <t>API done: procera_audit::explorer — filtered newest-first keyset paging, view-own scope, member names, artifact-aware object timelines, chain verify, private audited saved queries, capped CSV/JSONL exports with step-up that are themselves audited; E2E-R1-AUDX-01..06. UI: Audit log screen (chain-verified badge, filters, keyset paging, expandable records, object timelines in a drawer; E2E-R1-UI-17). Remaining: async export job, POST /audit/query</t>
+          <t>procera_audit::explorer and query: filtered newest-first keyset paging, view-own scope, member names, artifact timelines (own and version events), chain verify, saved queries, capped synchronous CSV/JSONL exports with step-up; POST /audit/query (AND/OR tree, allow-listed fields, depth 2); background export jobs (migration 0029) stored as the requester's encrypted file with notification; Audit log UI with filters, timelines and background exports. E2E-R1-AUDX-01..08, E2E-R1-AUD-01, E2E-R1-UI-17, 39. Later: verify-proof per sequence, the P95 &lt; 2 s at 10 M events benchmark</t>
         </is>
       </c>
     </row>
@@ -6069,13 +6243,17 @@
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L48" s="3" t="inlineStr"/>
       <c r="M48" s="3" t="inlineStr"/>
       <c r="N48" s="3" t="inlineStr"/>
-      <c r="O48" s="3" t="inlineStr"/>
+      <c r="O48" s="3" t="inlineStr">
+        <is>
+          <t>procera-ir crate: IR v1 model, compiler with the docs/11 §11 checks (IR-E001..E034, E100, W001-W002, I001; JSON-pointer diagnostics), JCS canonical form + sha256 checksum, semantic diff with apply; a test per code, property tests, conformance/compiler fixtures, golden checksums for the reference processes (A-21). Remaining: type checking with the BPMS-081 engine, environment wiring at publish (BPMS-084), declared perpetual waits.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -6130,13 +6308,17 @@
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L49" s="3" t="inlineStr"/>
       <c r="M49" s="3" t="inlineStr"/>
       <c r="N49" s="3" t="inlineStr"/>
-      <c r="O49" s="3" t="inlineStr"/>
+      <c r="O49" s="3" t="inlineStr">
+        <is>
+          <t>procera-expr: a typed CEL subset of our own (A-22): static checker with null policy and exact decimal/money, budgeted pure evaluator (10k steps, 1 MiB, 64 KiB strings, 10k lists; exhaustion is IR-R010), stdlib, read sets with the restricted-in-event-facing check; wasm32 build checked; unit + property tests; docs/11 §6.1. Remaining: wiring into the IR compiler (BPMS-080) and runtime (BPMS-082), business-time functions with calendars (BPMS-083).</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -6191,13 +6373,17 @@
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L50" s="3" t="inlineStr"/>
       <c r="M50" s="3" t="inlineStr"/>
       <c r="N50" s="3" t="inlineStr"/>
-      <c r="O50" s="3" t="inlineStr"/>
+      <c r="O50" s="3" t="inlineStr">
+        <is>
+          <t>procera-runtime: pure deterministic interpreter (Program, InstanceState, Stimulus) -&gt; (state, commands) with injected Clock/IdGen; advance loop with a step budget (ContinueAdvance) and loop guard (IR-R004); start/end/terminate, set, decision (+rule tables via the Evaluator port), parallel split/join released exactly once, human.* work items, wait.timer/signal, service.call with typed error boundaries, notify, subprocess.call, case.open, timeout boundaries, cancel; commands with deterministic idempotency keys; unit tests per node kind, the five reference processes end to end, 22 conformance/runtime fixtures, property tests (replay, budgets, joins, terminate); docs/11 §15, A-23. Remaining: the CEL engine behind the port, persistence and timers (BPMS-083), work items (BPMS-085), incidents (BPMS-088), E2E once wired to the API.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -7106,13 +7292,17 @@
       </c>
       <c r="K65" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L65" s="3" t="inlineStr"/>
       <c r="M65" s="3" t="inlineStr"/>
       <c r="N65" s="3" t="inlineStr"/>
-      <c r="O65" s="3" t="inlineStr"/>
+      <c r="O65" s="3" t="inlineStr">
+        <is>
+          <t>Retention classes honoured by jobs (migration 0024, docs/14 §4): draft (deleted after retention.draft.inactive_after without edits; authors notified retention.draft.notice_before ahead; a never-published artifact goes with its only draft; drafts linked to change requests kept), operational (sent/failed emails, read notifications, sent digest items after retention.operational.keep_for), governance_record and audit never deleted by the app (disposition with certificates is P1); hourly in the scheduler, every run recorded and audited (retention.purged); Retention admin page with due drafts and period changes (reason + step-up). E2E-R1-RET-01..02, E2E-R1-UI-26.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
@@ -9829,7 +10019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E359"/>
+  <dimension ref="A1:E390"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -15922,12 +16112,12 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-POL-01</t>
+          <t>E2E-R1-LIB-11</t>
         </is>
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>Readers never see drafts: absent from lists, reads and search until published; a later draft stays hidden (version 404, diff 404, versions list shows v1 only); authors see drafts in search | BPMS-045, A-14</t>
+          <t>Collection tree: sibling names unique (409), moving rewrites paths, no move under itself (422), lists filter by subtree, only empty collections delete (409/204) | BPMS-041, FR-G01</t>
         </is>
       </c>
       <c r="D226" s="3" t="inlineStr">
@@ -15949,12 +16139,12 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-POL-02</t>
+          <t>E2E-R1-LIB-12</t>
         </is>
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>Applicability: empty audience or restricted without one → 422; members cannot set it (403); a restricted policy is hidden from members outside its group in lists, reads, search, the portal and change requests (404), and shown to those inside; an unrestricted one is listed for everyone but only "applicable" to its audience | BPMS-045, FR-PL01/PL02</t>
+          <t>A restricted collection hides the documents filed under it (also in sub-collections) from readers outside its audience in lists, reads, search and the tree; members cannot manage collections | BPMS-041, FR-G01 "search authorized-only", A-20</t>
         </is>
       </c>
       <c r="D227" s="3" t="inlineStr">
@@ -15976,12 +16166,12 @@
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-POL-03</t>
+          <t>E2E-R1-LIB-13</t>
         </is>
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>The portal lists published policies that apply to the member (no drafts), ordered by category, with what changed since the previous version (added/changed counts, reason) and text/category filters | BPMS-045, FR-PL02</t>
+          <t>Owner hand-over (publishers only); RACI with at most one accountable, readable by readers; CSV export with the exact row and an audit event | BPMS-041, FR-G01 "RACI exportable"</t>
         </is>
       </c>
       <c r="D228" s="3" t="inlineStr">
@@ -16003,12 +16193,12 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-POL-04</t>
+          <t>E2E-R1-LIB-14</t>
         </is>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>A major version asks the applicable audience to re-acknowledge that exact version; a minor one does not (major_only) | BPMS-045, FR-PL03</t>
+          <t>Rich blocks (heading, formatted paragraph with an in-app link, numbered list, warning callout, table) save; unknown blocks, `javascript:` links and runs that don't add up to the text → 422; HTML export is faithful and escaped, Markdown export exact, unknown format 422; a superseded version's export says so; exports are audited | BPMS-042, ADR-0013</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
@@ -16030,12 +16220,12 @@
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-POL-05</t>
+          <t>E2E-R1-POL-01</t>
         </is>
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>Every_publish asks on minors, none never asks, and a scheduled major asks when it goes live | BPMS-045, FR-PL03</t>
+          <t>Readers never see drafts: absent from lists, reads and search until published; a later draft stays hidden (version 404, diff 404, versions list shows v1 only); authors see drafts in search | BPMS-045, A-14</t>
         </is>
       </c>
       <c r="D230" s="3" t="inlineStr">
@@ -16057,12 +16247,12 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ADM-01</t>
+          <t>E2E-R1-POL-02</t>
         </is>
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>Overview: overdue acknowledgements rank first in "needs attention", followed by an admin without two-step verification; acknowledgement metrics and a daily published series; the security strip counts a failed sign-in, members without MFA and the new admin grant; requests/storage are null; members get 403; an inverted range → 422 | BPMS-063, FR-A01</t>
+          <t>Applicability: empty audience or restricted without one → 422; members cannot set it (403); a restricted policy is hidden from members outside its group in lists, reads, search, the portal and change requests (404), and shown to those inside; an unrestricted one is listed for everyone but only "applicable" to its audience | BPMS-045, FR-PL01/PL02</t>
         </is>
       </c>
       <c r="D231" s="3" t="inlineStr">
@@ -16084,12 +16274,12 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ADM-02</t>
+          <t>E2E-R1-POL-03</t>
         </is>
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>People &amp; access: counts (members, no MFA, privileged, pending invites), member row (MFA off, last active set, not dormant), no-MFA and admin filters; unknown filter → 422; members get 403 | BPMS-063, FR-A06</t>
+          <t>The portal lists published policies that apply to the member (no drafts), ordered by category, with what changed since the previous version (added/changed counts, reason) and text/category filters | BPMS-045, FR-PL02</t>
         </is>
       </c>
       <c r="D232" s="3" t="inlineStr">
@@ -16111,12 +16301,12 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-01</t>
+          <t>E2E-R1-POL-04</t>
         </is>
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>Sign in through the browser (password + recovery code) lands on Home; navigation is permission-shaped with the current page marked; axe clean on sign-in and Home; reload keeps the session | docs/05 §2.1, §3.1, WCAG 2.2 AA</t>
+          <t>A major version asks the applicable audience to re-acknowledge that exact version; a minor one does not (major_only) | BPMS-045, FR-PL03</t>
         </is>
       </c>
       <c r="D233" s="3" t="inlineStr">
@@ -16138,12 +16328,12 @@
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-02</t>
+          <t>E2E-R1-POL-05</t>
         </is>
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Wrong password and wrong code produce clear, non-revealing messages (role=alert); axe clean | docs/06 §3, WCAG 3.3.1</t>
+          <t>Every_publish asks on minors, none never asks, and a scheduled major asks when it goes live | BPMS-045, FR-PL03</t>
         </is>
       </c>
       <c r="D234" s="3" t="inlineStr">
@@ -16165,12 +16355,12 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-03</t>
+          <t>E2E-R1-ADM-01</t>
         </is>
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>With several workspaces the chooser appears; choosing one and switching from the header changes the context and the navigation (no Admin for a plain member) | docs/05 §2.1 workspace switcher</t>
+          <t>Overview: overdue acknowledgements rank first in "needs attention", followed by an admin without two-step verification; acknowledgement metrics and a daily published series; the security strip counts a failed sign-in, members without MFA and the new admin grant; requests/storage are null; members get 403; an inverted range → 422 | BPMS-063, FR-A01</t>
         </is>
       </c>
       <c r="D235" s="3" t="inlineStr">
@@ -16192,12 +16382,12 @@
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-04</t>
+          <t>E2E-R1-ADM-02</t>
         </is>
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>The bell announces the unread count; the inbox lists the "joined" notification; mark all as read | FR-N01</t>
+          <t>People &amp; access: counts (members, no MFA, privileged, pending invites), member row (MFA off, last active set, not dormant), no-MFA and admin filters; unknown filter → 422; members get 403 | BPMS-063, FR-A06</t>
         </is>
       </c>
       <c r="D236" s="3" t="inlineStr">
@@ -16219,12 +16409,12 @@
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-05</t>
+          <t>E2E-R1-RET-01</t>
         </is>
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>Sign out returns to sign-in; reloading stays signed out | docs/06 §3</t>
+          <t>Retention classes are listed (draft and operational automatic; governance records and audit never). Drafts untouched for 170 of 180 days are due and their author is notified once; editing one resets its clock; 11 days later the untouched drafts are deleted (a never-published artifact with its draft, a v2 draft beside a published v1 that stays); the run is recorded and audited (`retention.purged`) | BPMS-066, PRV-04</t>
         </is>
       </c>
       <c r="D237" s="3" t="inlineStr">
@@ -16246,12 +16436,12 @@
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-06</t>
+          <t>E2E-R1-RET-02</t>
         </is>
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>Theme switched from the account menu persists across reload; dark theme passes axe | docs/05 §7, WCAG 2.2 AA</t>
+          <t>A read notification older than the operational period is removed by the job; members cannot see retention (403) | BPMS-066, PRV-04</t>
         </is>
       </c>
       <c r="D238" s="3" t="inlineStr">
@@ -16273,12 +16463,12 @@
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-07</t>
+          <t>E2E-R1-KEY-01</t>
         </is>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>Author a policy in the browser: New document dialog → write content (headings, lists) → save → submit → publish; the library row shows Published; axe clean | FR-G04, docs/05 §3.2/§3.21</t>
+          <t>An invitation email is envelope-encrypted under the workspace KEK; rotation needs a reason (422) and is audited; the email stays readable right after rotation and after the background rewrap moves it to v2; the unused v1 is destroyed; members cannot see or rotate keys (403). Crypto-shredding is proven in the `procera-keys` integration test | BPMS-030</t>
         </is>
       </c>
       <c r="D239" s="3" t="inlineStr">
@@ -16300,12 +16490,12 @@
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-08</t>
+          <t>E2E-R1-FILE-01</t>
         </is>
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>A campaign task on Home leads to the document; “I acknowledge” records the acknowledgement (campaign progress +1) and the callout disappears | FR-AK01, docs/05 §3.1</t>
+          <t>A chunked upload refuses a wrong offset (409) and resumes from `received`; completion before all bytes 409; the file is hashed (SHA-256 matches), typed by content (PDF despite a .txt name and text/plain declared) and clean; the signed link downloads without a bearer with nosniff and the exact bytes; a tampered link 403; another member gets 404; upload and download are audited | BPMS-060, FR-F01–F03</t>
         </is>
       </c>
       <c r="D240" s="3" t="inlineStr">
@@ -16327,12 +16517,12 @@
       </c>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-09</t>
+          <t>E2E-R1-FILE-02</t>
         </is>
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>Invite a colleague from Members with a role; the invitation appears in the table as Invited | FR-W01, docs/05 §3.14</t>
+          <t>EICAR is quarantined and its download link refused (409); an executable named .pdf and an HTML file named .txt are rejected by content; 500 MB → 413; empty → 422; usage counts states | BPMS-060, FR-F02</t>
         </is>
       </c>
       <c r="D241" s="3" t="inlineStr">
@@ -16354,12 +16544,12 @@
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-10</t>
+          <t>E2E-R1-FILE-03</t>
         </is>
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>Read and acknowledge a critical, pinned announcement in the feed | FR-AN04, docs/05 §3.23</t>
+          <t>A draft takes an attachment; after publishing it can't be unlinked or the file deleted (409); a member reading the published SOP downloads it; an unattached file past the orphan period is listed, members can't purge (403), the owner purges it | BPMS-060/062, FR-F05/F07</t>
         </is>
       </c>
       <c r="D242" s="3" t="inlineStr">
@@ -16381,12 +16571,12 @@
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-11</t>
+          <t>E2E-R1-FILE-04</t>
         </is>
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>An admin without two-step verification is guided through setup (QR + key, confirm a code, recovery codes) and then signs in with MFA and lands on Home | docs/06 §3, docs/20 §2.3</t>
+          <t>A PNG, a PDF and a JPEG get preview links that serve inline with the strict headers (CSP sandbox, nosniff, CORP same-origin, no-store) and a ≤ 2-minute expiry; the JPEG's Exif is removed; a text file gets kind none and no URL; a tampered token and a download token on the preview route are 403; another member gets 404; previews are audited | BPMS-061, FR-F04/F02</t>
         </is>
       </c>
       <c r="D243" s="3" t="inlineStr">
@@ -16408,12 +16598,12 @@
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-12</t>
+          <t>E2E-R1-VIEW-01</t>
         </is>
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>⌘K finds a document by its content and opens it; commands navigate; recent items are offered; keyboard only | BPMS-031, BPMS-049</t>
+          <t>Saved views: personal and shared, one default per member (setting a new default clears the old), invalid list or name 422; another member sees only shared views and can't edit or delete them (403) or touch personal ones (404); unsharing hides it; exports are recorded (`data.exported`), unknown format 422 | BPMS-028, FR-V05/V06</t>
         </is>
       </c>
       <c r="D244" s="3" t="inlineStr">
@@ -16435,12 +16625,12 @@
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-13</t>
+          <t>E2E-R1-UI-01</t>
         </is>
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>A new workspace shows composed empty states; an unknown page offers a way back; a failed load shows the error with a retry | BPMS-031 (UX-005)</t>
+          <t>Sign in through the browser (password + recovery code) lands on Home; navigation is permission-shaped with the current page marked; axe clean on sign-in and Home; reload keeps the session | docs/05 §2.1, §3.1, WCAG 2.2 AA</t>
         </is>
       </c>
       <c r="D245" s="3" t="inlineStr">
@@ -16462,12 +16652,12 @@
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-14</t>
+          <t>E2E-R1-UI-02</t>
         </is>
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>Manage announcements: compose a draft; a workspace-wide post is sent for approval; a targeted draft is published and shows receipts | BPMS-031, BPMS-047</t>
+          <t>Wrong password and wrong code produce clear, non-revealing messages (role=alert); axe clean | docs/06 §3, WCAG 3.3.1</t>
         </is>
       </c>
       <c r="D246" s="3" t="inlineStr">
@@ -16489,12 +16679,12 @@
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-15</t>
+          <t>E2E-R1-UI-03</t>
         </is>
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>Campaigns: create from a published document with an audience, check the reach, launch, follow progress, download the evidence CSV | BPMS-031, BPMS-046</t>
+          <t>With several workspaces the chooser appears; choosing one and switching from the header changes the context and the navigation (no Admin for a plain member) | docs/05 §2.1 workspace switcher</t>
         </is>
       </c>
       <c r="D247" s="3" t="inlineStr">
@@ -16516,12 +16706,12 @@
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-16</t>
+          <t>E2E-R1-UI-04</t>
         </is>
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>Settings: change a value in place with a reason and see why it applies; a step-up key asks to confirm identity | BPMS-031, BPMS-027</t>
+          <t>The bell announces the unread count; the inbox lists the "joined" notification; mark all as read | FR-N01</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
@@ -16543,12 +16733,12 @@
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-17</t>
+          <t>E2E-R1-UI-05</t>
         </is>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>Audit log: chain verified; filter by category; expand a record; open an object timeline; no-match state | BPMS-031, BPMS-064</t>
+          <t>Sign out returns to sign-in; reloading stays signed out | docs/06 §3</t>
         </is>
       </c>
       <c r="D249" s="3" t="inlineStr">
@@ -16570,12 +16760,12 @@
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-18</t>
+          <t>E2E-R1-UI-06</t>
         </is>
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>The owner sets a review schedule, recertifies when it falls due, verifies and removes verification | BPMS-044</t>
+          <t>Theme switched from the account menu persists across reload; dark theme passes axe | docs/05 §7, WCAG 2.2 AA</t>
         </is>
       </c>
       <c r="D250" s="3" t="inlineStr">
@@ -16597,12 +16787,12 @@
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-19</t>
+          <t>E2E-R1-UI-07</t>
         </is>
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>A member suggests a change; the owner accepts it and marks it implemented in v2 | BPMS-044</t>
+          <t>Author a policy in the browser: New document dialog → write content (headings, lists) → save → submit → publish; the library row shows Published; axe clean | FR-G04, docs/05 §3.2/§3.21</t>
         </is>
       </c>
       <c r="D251" s="3" t="inlineStr">
@@ -16624,12 +16814,12 @@
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-20</t>
+          <t>E2E-R1-UI-08</t>
         </is>
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>Compare v1 and v2 from the version history: word-level changes and the summary | BPMS-043</t>
+          <t>A campaign task on Home leads to the document; “I acknowledge” records the acknowledgement (campaign progress +1) and the callout disappears | FR-AK01, docs/05 §3.1</t>
         </is>
       </c>
       <c r="D252" s="3" t="inlineStr">
@@ -16651,12 +16841,12 @@
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-21</t>
+          <t>E2E-R1-UI-09</t>
         </is>
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>A member opens Policies, filters by category and follows "what changed" to the comparison | BPMS-045</t>
+          <t>Invite a colleague from Members with a role; the invitation appears in the table as Invited | FR-W01, docs/05 §3.14</t>
         </is>
       </c>
       <c r="D253" s="3" t="inlineStr">
@@ -16678,12 +16868,12 @@
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-22</t>
+          <t>E2E-R1-UI-10</t>
         </is>
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>A publisher restricts a policy to a role; a member outside it can't find it in Policies or open it | BPMS-045, A-14</t>
+          <t>Read and acknowledge a critical, pinned announcement in the feed | FR-AN04, docs/05 §3.23</t>
         </is>
       </c>
       <c r="D254" s="3" t="inlineStr">
@@ -16705,12 +16895,12 @@
       </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-23</t>
+          <t>E2E-R1-UI-11</t>
         </is>
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>An admin opens Overview: the summary and "Needs attention" show overdue acknowledgements, and the security strip shows one member without two-step verification; drilling in opens People &amp; access filtered to them; the Admins filter shows the owner | BPMS-063</t>
+          <t>An admin without two-step verification is guided through setup (QR + key, confirm a code, recovery codes) and then signs in with MFA and lands on Home | docs/06 §3, docs/20 §2.3</t>
         </is>
       </c>
       <c r="D255" s="3" t="inlineStr">
@@ -16732,12 +16922,12 @@
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-24</t>
+          <t>E2E-R1-UI-12</t>
         </is>
       </c>
       <c r="C256" s="3" t="inlineStr">
         <is>
-          <t>An owner publishes v2 as a major change, sees who will be asked, then finds the campaign | BPMS-045</t>
+          <t>⌘K finds a document by its content and opens it; commands navigate; recent items are offered; keyboard only | BPMS-031, BPMS-049</t>
         </is>
       </c>
       <c r="D256" s="3" t="inlineStr">
@@ -16759,12 +16949,12 @@
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-25</t>
+          <t>E2E-R1-UI-13</t>
         </is>
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>A member opens Notifications → Preferences, picks a daily digest and quiet hours, saves, sees them after a reload, and resets to the workspace defaults | BPMS-048</t>
+          <t>A new workspace shows composed empty states; an unknown page offers a way back; a failed load shows the error with a retry | BPMS-031 (UX-005)</t>
         </is>
       </c>
       <c r="D257" s="3" t="inlineStr">
@@ -16786,12 +16976,12 @@
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-30</t>
+          <t>E2E-R1-UI-14</t>
         </is>
       </c>
       <c r="C258" s="3" t="inlineStr">
         <is>
-          <t>Add a passkey from Account › Security, sign out, sign in with password + passkey | BPMS-022</t>
+          <t>Manage announcements: compose a draft; a workspace-wide post is sent for approval; a targeted draft is published and shows receipts | BPMS-031, BPMS-047</t>
         </is>
       </c>
       <c r="D258" s="3" t="inlineStr">
@@ -16813,12 +17003,12 @@
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-31</t>
+          <t>E2E-R1-UI-15</t>
         </is>
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>Removing a passkey asks to confirm it’s you; the passkey itself passes step-up | BPMS-022</t>
+          <t>Campaigns: create from a published document with an audience, check the reach, launch, follow progress, download the evidence CSV | BPMS-031, BPMS-046</t>
         </is>
       </c>
       <c r="D259" s="3" t="inlineStr">
@@ -16840,12 +17030,12 @@
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-35</t>
+          <t>E2E-R1-UI-16</t>
         </is>
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
-          <t>Departments: override a setting for a parent department, see a child inherit it, then clear it | BPMS-027</t>
+          <t>Settings: change a value in place with a reason and see why it applies; a step-up key asks to confirm identity | BPMS-031, BPMS-027</t>
         </is>
       </c>
       <c r="D260" s="3" t="inlineStr">
@@ -16867,12 +17057,12 @@
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-36</t>
+          <t>E2E-R1-UI-17</t>
         </is>
       </c>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>Configuration profile: preview a switch with every change, then switch with a reason | BPMS-027, CFG-017</t>
+          <t>Audit log: chain verified; filter by category; expand a record; open an object timeline; no-match state | BPMS-031, BPMS-064</t>
         </is>
       </c>
       <c r="D261" s="3" t="inlineStr">
@@ -16894,12 +17084,12 @@
       </c>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-40</t>
+          <t>E2E-R1-UI-18</t>
         </is>
       </c>
       <c r="C262" s="3" t="inlineStr">
         <is>
-          <t>A system admin finds a workspace, makes it read-only with a reason, and reactivates it | BPMS-065</t>
+          <t>The owner sets a review schedule, recertifies when it falls due, verifies and removes verification | BPMS-044</t>
         </is>
       </c>
       <c r="D262" s="3" t="inlineStr">
@@ -16921,12 +17111,12 @@
       </c>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-41</t>
+          <t>E2E-R1-UI-19</t>
         </is>
       </c>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>Quotas, platform health and the system audit; non-system users never see the console | BPMS-065</t>
+          <t>A member suggests a change; the owner accepts it and marks it implemented in v2 | BPMS-044</t>
         </is>
       </c>
       <c r="D263" s="3" t="inlineStr">
@@ -16948,12 +17138,12 @@
       </c>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-01</t>
+          <t>E2E-R1-UI-20</t>
         </is>
       </c>
       <c r="C264" s="3" t="inlineStr">
         <is>
-          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
+          <t>Compare v1 and v2 from the version history: word-level changes and the summary | BPMS-043</t>
         </is>
       </c>
       <c r="D264" s="3" t="inlineStr">
@@ -16975,12 +17165,12 @@
       </c>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-02</t>
+          <t>E2E-R1-UI-21</t>
         </is>
       </c>
       <c r="C265" s="3" t="inlineStr">
         <is>
-          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
+          <t>A member opens Policies, filters by category and follows "what changed" to the comparison | BPMS-045</t>
         </is>
       </c>
       <c r="D265" s="3" t="inlineStr">
@@ -17002,12 +17192,12 @@
       </c>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-03</t>
+          <t>E2E-R1-UI-22</t>
         </is>
       </c>
       <c r="C266" s="3" t="inlineStr">
         <is>
-          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
+          <t>A publisher restricts a policy to a role; a member outside it can't find it in Policies or open it | BPMS-045, A-14</t>
         </is>
       </c>
       <c r="D266" s="3" t="inlineStr">
@@ -17029,12 +17219,12 @@
       </c>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-04</t>
+          <t>E2E-R1-UI-23</t>
         </is>
       </c>
       <c r="C267" s="3" t="inlineStr">
         <is>
-          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
+          <t>An admin opens Overview: the summary and "Needs attention" show overdue acknowledgements, and the security strip shows one member without two-step verification; drilling in opens People &amp; access filtered to them; the Admins filter shows the owner | BPMS-063</t>
         </is>
       </c>
       <c r="D267" s="3" t="inlineStr">
@@ -17056,12 +17246,12 @@
       </c>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-05</t>
+          <t>E2E-R1-UI-24</t>
         </is>
       </c>
       <c r="C268" s="3" t="inlineStr">
         <is>
-          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
+          <t>An owner publishes v2 as a major change, sees who will be asked, then finds the campaign | BPMS-045</t>
         </is>
       </c>
       <c r="D268" s="3" t="inlineStr">
@@ -17083,12 +17273,12 @@
       </c>
       <c r="B269" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-06</t>
+          <t>E2E-R1-UI-25</t>
         </is>
       </c>
       <c r="C269" s="3" t="inlineStr">
         <is>
-          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
+          <t>A member opens Notifications → Preferences, picks a daily digest and quiet hours, saves, sees them after a reload, and resets to the workspace defaults | BPMS-048</t>
         </is>
       </c>
       <c r="D269" s="3" t="inlineStr">
@@ -17110,12 +17300,12 @@
       </c>
       <c r="B270" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-07</t>
+          <t>E2E-R1-UI-26</t>
         </is>
       </c>
       <c r="C270" s="3" t="inlineStr">
         <is>
-          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
+          <t>An admin opens Retention, sees each record class and a draft due for deletion, and shortens the draft period with a reason | BPMS-066</t>
         </is>
       </c>
       <c r="D270" s="3" t="inlineStr">
@@ -17137,12 +17327,12 @@
       </c>
       <c r="B271" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-01</t>
+          <t>E2E-R1-UI-27</t>
         </is>
       </c>
       <c r="C271" s="3" t="inlineStr">
         <is>
-          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
+          <t>An admin creates a collection from the Library rail, files a document in it from the document page, sets the accountable person in RACI, and filters the Library by the collection | BPMS-041</t>
         </is>
       </c>
       <c r="D271" s="3" t="inlineStr">
@@ -17164,12 +17354,12 @@
       </c>
       <c r="B272" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-02</t>
+          <t>E2E-R1-UI-28</t>
         </is>
       </c>
       <c r="C272" s="3" t="inlineStr">
         <is>
-          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
+          <t>An author uses the editor toolbar (bold, numbered steps, callout, table), saves, and the document renders them; the stored blocks match; axe on the editor and the result. UI-07 types markdown shortcuts into the editor | BPMS-042</t>
         </is>
       </c>
       <c r="D272" s="3" t="inlineStr">
@@ -17191,12 +17381,12 @@
       </c>
       <c r="B273" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-03</t>
+          <t>E2E-R1-UI-29</t>
         </is>
       </c>
       <c r="C273" s="3" t="inlineStr">
         <is>
-          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
+          <t>An admin opens Encryption, sees version 1 in use, rotates the key with a reason, and sees version 2 in use | BPMS-030</t>
         </is>
       </c>
       <c r="D273" s="3" t="inlineStr">
@@ -17218,12 +17408,12 @@
       </c>
       <c r="B274" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-04</t>
+          <t>E2E-R1-UI-32</t>
         </is>
       </c>
       <c r="C274" s="3" t="inlineStr">
         <is>
-          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
+          <t>An author attaches a file to a draft from the document page, sees it clean, and downloads it | BPMS-060</t>
         </is>
       </c>
       <c r="D274" s="3" t="inlineStr">
@@ -17245,12 +17435,12 @@
       </c>
       <c r="B275" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-05</t>
+          <t>E2E-R1-UI-33</t>
         </is>
       </c>
       <c r="C275" s="3" t="inlineStr">
         <is>
-          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
+          <t>An EICAR upload on a document is refused with a quarantine message and shows as Quarantined (no download) in the Files view | BPMS-060/062</t>
         </is>
       </c>
       <c r="D275" s="3" t="inlineStr">
@@ -17272,12 +17462,12 @@
       </c>
       <c r="B276" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-06</t>
+          <t>E2E-R1-UI-34</t>
         </is>
       </c>
       <c r="C276" s="3" t="inlineStr">
         <is>
-          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
+          <t>An author opens Preview on an image attachment: a dialog named after the file shows the image (axe clean); a text attachment offers no Preview; Escape closes it and focus returns | BPMS-061</t>
         </is>
       </c>
       <c r="D276" s="3" t="inlineStr">
@@ -17299,12 +17489,12 @@
       </c>
       <c r="B277" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-01</t>
+          <t>E2E-R1-UI-38</t>
         </is>
       </c>
       <c r="C277" s="3" t="inlineStr">
         <is>
-          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
+          <t>On the Library grid: build a Status filter (chip + count), sort by name descending, save the view, reload and get the same filter and order back with no modified marker, export a CSV with exactly the visible columns and rows | BPMS-028</t>
         </is>
       </c>
       <c r="D277" s="3" t="inlineStr">
@@ -17326,12 +17516,12 @@
       </c>
       <c r="B278" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-02</t>
+          <t>E2E-R1-UI-39</t>
         </is>
       </c>
       <c r="C278" s="3" t="inlineStr">
         <is>
-          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
+          <t>An admin filters the Audit log to content events, starts a background export (dialog says it uses the current filters), sees it become Ready in Your exports, and downloads the CSV | BPMS-064</t>
         </is>
       </c>
       <c r="D278" s="3" t="inlineStr">
@@ -17353,12 +17543,12 @@
       </c>
       <c r="B279" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-03</t>
+          <t>E2E-R1-UI-30</t>
         </is>
       </c>
       <c r="C279" s="3" t="inlineStr">
         <is>
-          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
+          <t>Add a passkey from Account › Security, sign out, sign in with password + passkey | BPMS-022</t>
         </is>
       </c>
       <c r="D279" s="3" t="inlineStr">
@@ -17380,12 +17570,12 @@
       </c>
       <c r="B280" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-01</t>
+          <t>E2E-R1-UI-31</t>
         </is>
       </c>
       <c r="C280" s="3" t="inlineStr">
         <is>
-          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
+          <t>Removing a passkey asks to confirm it’s you; the passkey itself passes step-up | BPMS-022</t>
         </is>
       </c>
       <c r="D280" s="3" t="inlineStr">
@@ -17407,12 +17597,12 @@
       </c>
       <c r="B281" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-02</t>
+          <t>E2E-R1-UI-35</t>
         </is>
       </c>
       <c r="C281" s="3" t="inlineStr">
         <is>
-          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
+          <t>Departments: override a setting for a parent department, see a child inherit it, then clear it | BPMS-027</t>
         </is>
       </c>
       <c r="D281" s="3" t="inlineStr">
@@ -17434,12 +17624,12 @@
       </c>
       <c r="B282" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-03</t>
+          <t>E2E-R1-UI-36</t>
         </is>
       </c>
       <c r="C282" s="3" t="inlineStr">
         <is>
-          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
+          <t>Configuration profile: preview a switch with every change, then switch with a reason | BPMS-027, CFG-017</t>
         </is>
       </c>
       <c r="D282" s="3" t="inlineStr">
@@ -17461,12 +17651,12 @@
       </c>
       <c r="B283" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-04</t>
+          <t>E2E-R1-UI-40</t>
         </is>
       </c>
       <c r="C283" s="3" t="inlineStr">
         <is>
-          <t>Chain verify reports intact | FR-T02</t>
+          <t>A system admin finds a workspace, makes it read-only with a reason, and reactivates it | BPMS-065</t>
         </is>
       </c>
       <c r="D283" s="3" t="inlineStr">
@@ -17488,12 +17678,12 @@
       </c>
       <c r="B284" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-05</t>
+          <t>E2E-R1-UI-41</t>
         </is>
       </c>
       <c r="C284" s="3" t="inlineStr">
         <is>
-          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
+          <t>Quotas, platform health and the system audit; non-system users never see the console | BPMS-065</t>
         </is>
       </c>
       <c r="D284" s="3" t="inlineStr">
@@ -17515,12 +17705,12 @@
       </c>
       <c r="B285" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-06</t>
+          <t>E2E-R1-UI-42</t>
         </is>
       </c>
       <c r="C285" s="3" t="inlineStr">
         <is>
-          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
+          <t>With the API slowed down, every main page (Home, Library, Members, Campaigns, Manage announcements, Overview, People &amp; access, Settings, Audit log, Notifications) shows a content-shaped skeleton, then its content; a reload shows the app frame, never a blank page | UX-005</t>
         </is>
       </c>
       <c r="D285" s="3" t="inlineStr">
@@ -17542,12 +17732,12 @@
       </c>
       <c r="B286" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-UI-43</t>
         </is>
       </c>
       <c r="C286" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>Files: a draft attachment shows retention class Draft and last accessed Never; downloading it updates last accessed; two unattached files are selected and deleted in bulk | BPMS-062</t>
         </is>
       </c>
       <c r="D286" s="3" t="inlineStr">
@@ -17569,12 +17759,12 @@
       </c>
       <c r="B287" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-FLOW-01</t>
         </is>
       </c>
       <c r="C287" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>Onboarding start to finish: the owner invites from Members; the invitee opens the link from the email, creates an account (password confirmation checked) and lands on Home in the workspace; the link then no longer works; the owner sees them Active and opens their person page | BPMS-023</t>
         </is>
       </c>
       <c r="D287" s="3" t="inlineStr">
@@ -17596,12 +17786,12 @@
       </c>
       <c r="B288" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-FLOW-02</t>
         </is>
       </c>
       <c r="C288" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>Someone with an account opens the invitation email, signs in from the page, comes back to it and joins with one click; an unknown link explains itself | BPMS-023</t>
         </is>
       </c>
       <c r="D288" s="3" t="inlineStr">
@@ -17623,12 +17813,12 @@
       </c>
       <c r="B289" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-FLOW-03</t>
         </is>
       </c>
       <c r="C289" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>Policy to evidence: the owner writes and publishes a policy and launches a campaign; a colleague (invited the same way) sees the task on Home, opens the acknowledgement email link, acknowledges on the document; the owner sees them Done, 1 of 2, and downloads the evidence CSV | BPMS-040, 046</t>
         </is>
       </c>
       <c r="D289" s="3" t="inlineStr">
@@ -17650,12 +17840,12 @@
       </c>
       <c r="B290" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-FLOW-04</t>
         </is>
       </c>
       <c r="C290" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>Announcement: the owner composes a critical post that needs acknowledgement and publishes it; a colleague opens the email link while signed out, signs in, lands on the open post and confirms; the owner sees the receipt | BPMS-047</t>
         </is>
       </c>
       <c r="D290" s="3" t="inlineStr">
@@ -17677,12 +17867,12 @@
       </c>
       <c r="B291" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-FLOW-05</t>
         </is>
       </c>
       <c r="C291" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>Review loop: the owner submits a controlled policy; the reviewer (invited as Reviewer) gets the review email, opens it and requests changes with a comment; the owner gets a notification quoting it, edits and resubmits; the reviewer approves from Home; the owner is told it is approved and publishes | BPMS-040</t>
         </is>
       </c>
       <c r="D291" s="3" t="inlineStr">
@@ -17704,12 +17894,12 @@
       </c>
       <c r="B292" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-FLOW-06</t>
         </is>
       </c>
       <c r="C292" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>Announcement approval: a second admin joins from the invitation and turns on two-step verification; the owner sends a workspace-wide post for approval; the admin gets the approval email, opens it and sends it back with a note; the owner gets a notification with the note, edits and resubmits; the admin approves and publishes; the owner is told; the post is in the feed | BPMS-047</t>
         </is>
       </c>
       <c r="D292" s="3" t="inlineStr">
@@ -17731,12 +17921,12 @@
       </c>
       <c r="B293" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-CMP-01</t>
         </is>
       </c>
       <c r="C293" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
         </is>
       </c>
       <c r="D293" s="3" t="inlineStr">
@@ -17758,12 +17948,12 @@
       </c>
       <c r="B294" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-CMP-02</t>
         </is>
       </c>
       <c r="C294" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
         </is>
       </c>
       <c r="D294" s="3" t="inlineStr">
@@ -17785,12 +17975,12 @@
       </c>
       <c r="B295" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-CMP-03</t>
         </is>
       </c>
       <c r="C295" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
         </is>
       </c>
       <c r="D295" s="3" t="inlineStr">
@@ -17812,12 +18002,12 @@
       </c>
       <c r="B296" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-CMP-04</t>
         </is>
       </c>
       <c r="C296" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
         </is>
       </c>
       <c r="D296" s="3" t="inlineStr">
@@ -17839,12 +18029,12 @@
       </c>
       <c r="B297" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-CMP-05</t>
         </is>
       </c>
       <c r="C297" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
         </is>
       </c>
       <c r="D297" s="3" t="inlineStr">
@@ -17866,12 +18056,12 @@
       </c>
       <c r="B298" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-CMP-06</t>
         </is>
       </c>
       <c r="C298" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
         </is>
       </c>
       <c r="D298" s="3" t="inlineStr">
@@ -17893,12 +18083,12 @@
       </c>
       <c r="B299" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-CMP-07</t>
         </is>
       </c>
       <c r="C299" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D299" s="3" t="inlineStr">
@@ -17920,12 +18110,12 @@
       </c>
       <c r="B300" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-ANN-01</t>
         </is>
       </c>
       <c r="C300" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
         </is>
       </c>
       <c r="D300" s="3" t="inlineStr">
@@ -17947,12 +18137,12 @@
       </c>
       <c r="B301" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-ANN-02</t>
         </is>
       </c>
       <c r="C301" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
         </is>
       </c>
       <c r="D301" s="3" t="inlineStr">
@@ -17974,12 +18164,12 @@
       </c>
       <c r="B302" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-ANN-03</t>
         </is>
       </c>
       <c r="C302" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
         </is>
       </c>
       <c r="D302" s="3" t="inlineStr">
@@ -18001,12 +18191,12 @@
       </c>
       <c r="B303" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-ANN-04</t>
         </is>
       </c>
       <c r="C303" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
         </is>
       </c>
       <c r="D303" s="3" t="inlineStr">
@@ -18028,12 +18218,12 @@
       </c>
       <c r="B304" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-ANN-05</t>
         </is>
       </c>
       <c r="C304" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D304" s="3" t="inlineStr">
@@ -18055,12 +18245,12 @@
       </c>
       <c r="B305" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-ANN-06</t>
         </is>
       </c>
       <c r="C305" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
         </is>
       </c>
       <c r="D305" s="3" t="inlineStr">
@@ -18082,12 +18272,12 @@
       </c>
       <c r="B306" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-SRCH-01</t>
         </is>
       </c>
       <c r="C306" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
         </is>
       </c>
       <c r="D306" s="3" t="inlineStr">
@@ -18109,12 +18299,12 @@
       </c>
       <c r="B307" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R1-SRCH-02</t>
         </is>
       </c>
       <c r="C307" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
         </is>
       </c>
       <c r="D307" s="3" t="inlineStr">
@@ -18136,12 +18326,12 @@
       </c>
       <c r="B308" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R1-SRCH-03</t>
         </is>
       </c>
       <c r="C308" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
         </is>
       </c>
       <c r="D308" s="3" t="inlineStr">
@@ -18163,12 +18353,12 @@
       </c>
       <c r="B309" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R1-AUDX-01</t>
         </is>
       </c>
       <c r="C309" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
         </is>
       </c>
       <c r="D309" s="3" t="inlineStr">
@@ -18190,12 +18380,12 @@
       </c>
       <c r="B310" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R1-AUDX-02</t>
         </is>
       </c>
       <c r="C310" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
         </is>
       </c>
       <c r="D310" s="3" t="inlineStr">
@@ -18217,12 +18407,12 @@
       </c>
       <c r="B311" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R1-AUDX-03</t>
         </is>
       </c>
       <c r="C311" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
         </is>
       </c>
       <c r="D311" s="3" t="inlineStr">
@@ -18244,12 +18434,12 @@
       </c>
       <c r="B312" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R1-AUDX-04</t>
         </is>
       </c>
       <c r="C312" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>Chain verify reports intact | FR-T02</t>
         </is>
       </c>
       <c r="D312" s="3" t="inlineStr">
@@ -18271,12 +18461,12 @@
       </c>
       <c r="B313" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R1-AUDX-05</t>
         </is>
       </c>
       <c r="C313" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
         </is>
       </c>
       <c r="D313" s="3" t="inlineStr">
@@ -18298,12 +18488,12 @@
       </c>
       <c r="B314" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R1-AUDX-06</t>
         </is>
       </c>
       <c r="C314" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
         </is>
       </c>
       <c r="D314" s="3" t="inlineStr">
@@ -18325,12 +18515,12 @@
       </c>
       <c r="B315" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R1-AUDX-07</t>
         </is>
       </c>
       <c r="C315" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>`POST /audit/query`: an AND group (category, action prefix, within P30D) sorted ascending pages by cursor; an OR group returns only matching events; unknown fields or values, bad durations, nesting deeper than 2 and unsupported sorts → 422 | BPMS-064, docs/08 §7.5</t>
         </is>
       </c>
       <c r="D315" s="3" t="inlineStr">
@@ -18352,12 +18542,12 @@
       </c>
       <c r="B316" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R1-AUDX-08</t>
         </is>
       </c>
       <c r="C316" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>A background export (202) runs as a job, finishes `done` with rows, its CSV downloads through the requester's signed file link, the requester is notified, and both `audit.export_requested` and `audit.exported` are recorded | BPMS-064, FR-T04</t>
         </is>
       </c>
       <c r="D316" s="3" t="inlineStr">
@@ -18379,12 +18569,12 @@
       </c>
       <c r="B317" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C317" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
         </is>
       </c>
       <c r="D317" s="3" t="inlineStr">
@@ -18406,12 +18596,12 @@
       </c>
       <c r="B318" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C318" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D318" s="3" t="inlineStr">
@@ -18433,12 +18623,12 @@
       </c>
       <c r="B319" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C319" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D319" s="3" t="inlineStr">
@@ -18460,12 +18650,12 @@
       </c>
       <c r="B320" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C320" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
         </is>
       </c>
       <c r="D320" s="3" t="inlineStr">
@@ -18487,12 +18677,12 @@
       </c>
       <c r="B321" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C321" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
         </is>
       </c>
       <c r="D321" s="3" t="inlineStr">
@@ -18514,12 +18704,12 @@
       </c>
       <c r="B322" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C322" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D322" s="3" t="inlineStr">
@@ -18541,12 +18731,12 @@
       </c>
       <c r="B323" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C323" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D323" s="3" t="inlineStr">
@@ -18568,12 +18758,12 @@
       </c>
       <c r="B324" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C324" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
         </is>
       </c>
       <c r="D324" s="3" t="inlineStr">
@@ -18595,12 +18785,12 @@
       </c>
       <c r="B325" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C325" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D325" s="3" t="inlineStr">
@@ -18622,12 +18812,12 @@
       </c>
       <c r="B326" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C326" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D326" s="3" t="inlineStr">
@@ -18649,12 +18839,12 @@
       </c>
       <c r="B327" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C327" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D327" s="3" t="inlineStr">
@@ -18676,12 +18866,12 @@
       </c>
       <c r="B328" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C328" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D328" s="3" t="inlineStr">
@@ -18703,12 +18893,12 @@
       </c>
       <c r="B329" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C329" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
         </is>
       </c>
       <c r="D329" s="3" t="inlineStr">
@@ -18730,12 +18920,12 @@
       </c>
       <c r="B330" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C330" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
         </is>
       </c>
       <c r="D330" s="3" t="inlineStr">
@@ -18757,12 +18947,12 @@
       </c>
       <c r="B331" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C331" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
         </is>
       </c>
       <c r="D331" s="3" t="inlineStr">
@@ -18784,12 +18974,12 @@
       </c>
       <c r="B332" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C332" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D332" s="3" t="inlineStr">
@@ -18811,12 +19001,12 @@
       </c>
       <c r="B333" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C333" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
         </is>
       </c>
       <c r="D333" s="3" t="inlineStr">
@@ -18838,12 +19028,12 @@
       </c>
       <c r="B334" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C334" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
         </is>
       </c>
       <c r="D334" s="3" t="inlineStr">
@@ -18865,12 +19055,12 @@
       </c>
       <c r="B335" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C335" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D335" s="3" t="inlineStr">
@@ -18892,12 +19082,12 @@
       </c>
       <c r="B336" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C336" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
         </is>
       </c>
       <c r="D336" s="3" t="inlineStr">
@@ -18919,12 +19109,12 @@
       </c>
       <c r="B337" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C337" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D337" s="3" t="inlineStr">
@@ -18946,12 +19136,12 @@
       </c>
       <c r="B338" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C338" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D338" s="3" t="inlineStr">
@@ -18973,12 +19163,12 @@
       </c>
       <c r="B339" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C339" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D339" s="3" t="inlineStr">
@@ -19000,12 +19190,12 @@
       </c>
       <c r="B340" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C340" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D340" s="3" t="inlineStr">
@@ -19027,12 +19217,12 @@
       </c>
       <c r="B341" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C341" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D341" s="3" t="inlineStr">
@@ -19054,12 +19244,12 @@
       </c>
       <c r="B342" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C342" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D342" s="3" t="inlineStr">
@@ -19081,12 +19271,12 @@
       </c>
       <c r="B343" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C343" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D343" s="3" t="inlineStr">
@@ -19108,12 +19298,12 @@
       </c>
       <c r="B344" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C344" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D344" s="3" t="inlineStr">
@@ -19135,12 +19325,12 @@
       </c>
       <c r="B345" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C345" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D345" s="3" t="inlineStr">
@@ -19162,12 +19352,12 @@
       </c>
       <c r="B346" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C346" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D346" s="3" t="inlineStr">
@@ -19189,12 +19379,12 @@
       </c>
       <c r="B347" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C347" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D347" s="3" t="inlineStr">
@@ -19216,12 +19406,12 @@
       </c>
       <c r="B348" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C348" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D348" s="3" t="inlineStr">
@@ -19243,12 +19433,12 @@
       </c>
       <c r="B349" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C349" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D349" s="3" t="inlineStr">
@@ -19270,12 +19460,12 @@
       </c>
       <c r="B350" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C350" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D350" s="3" t="inlineStr">
@@ -19297,12 +19487,12 @@
       </c>
       <c r="B351" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C351" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D351" s="3" t="inlineStr">
@@ -19324,12 +19514,12 @@
       </c>
       <c r="B352" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C352" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D352" s="3" t="inlineStr">
@@ -19351,12 +19541,12 @@
       </c>
       <c r="B353" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C353" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D353" s="3" t="inlineStr">
@@ -19378,12 +19568,12 @@
       </c>
       <c r="B354" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C354" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D354" s="3" t="inlineStr">
@@ -19405,12 +19595,12 @@
       </c>
       <c r="B355" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C355" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D355" s="3" t="inlineStr">
@@ -19432,12 +19622,12 @@
       </c>
       <c r="B356" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C356" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D356" s="3" t="inlineStr">
@@ -19459,12 +19649,12 @@
       </c>
       <c r="B357" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C357" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D357" s="3" t="inlineStr">
@@ -19486,12 +19676,12 @@
       </c>
       <c r="B358" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C358" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D358" s="3" t="inlineStr">
@@ -19513,20 +19703,857 @@
       </c>
       <c r="B359" s="3" t="inlineStr">
         <is>
+          <t>E2E-R3-06</t>
+        </is>
+      </c>
+      <c r="C359" s="3" t="inlineStr">
+        <is>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+        </is>
+      </c>
+      <c r="D359" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E359" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B360" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R3-07</t>
+        </is>
+      </c>
+      <c r="C360" s="3" t="inlineStr">
+        <is>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+        </is>
+      </c>
+      <c r="D360" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E360" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B361" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R3-08</t>
+        </is>
+      </c>
+      <c r="C361" s="3" t="inlineStr">
+        <is>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+        </is>
+      </c>
+      <c r="D361" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E361" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B362" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R3-09</t>
+        </is>
+      </c>
+      <c r="C362" s="3" t="inlineStr">
+        <is>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+        </is>
+      </c>
+      <c r="D362" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E362" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B363" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R3-10</t>
+        </is>
+      </c>
+      <c r="C363" s="3" t="inlineStr">
+        <is>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+        </is>
+      </c>
+      <c r="D363" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E363" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B364" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R3-11</t>
+        </is>
+      </c>
+      <c r="C364" s="3" t="inlineStr">
+        <is>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+        </is>
+      </c>
+      <c r="D364" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E364" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B365" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R3-12</t>
+        </is>
+      </c>
+      <c r="C365" s="3" t="inlineStr">
+        <is>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+        </is>
+      </c>
+      <c r="D365" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E365" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B366" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R3-MOB</t>
+        </is>
+      </c>
+      <c r="C366" s="3" t="inlineStr">
+        <is>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+        </is>
+      </c>
+      <c r="D366" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E366" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B367" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R3-ISO</t>
+        </is>
+      </c>
+      <c r="C367" s="3" t="inlineStr">
+        <is>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+        </is>
+      </c>
+      <c r="D367" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E367" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B368" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-01</t>
+        </is>
+      </c>
+      <c r="C368" s="3" t="inlineStr">
+        <is>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+        </is>
+      </c>
+      <c r="D368" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E368" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B369" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-02</t>
+        </is>
+      </c>
+      <c r="C369" s="3" t="inlineStr">
+        <is>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+        </is>
+      </c>
+      <c r="D369" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E369" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B370" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-03</t>
+        </is>
+      </c>
+      <c r="C370" s="3" t="inlineStr">
+        <is>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+        </is>
+      </c>
+      <c r="D370" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E370" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B371" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-04</t>
+        </is>
+      </c>
+      <c r="C371" s="3" t="inlineStr">
+        <is>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+        </is>
+      </c>
+      <c r="D371" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E371" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B372" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-05</t>
+        </is>
+      </c>
+      <c r="C372" s="3" t="inlineStr">
+        <is>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+        </is>
+      </c>
+      <c r="D372" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E372" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B373" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-06</t>
+        </is>
+      </c>
+      <c r="C373" s="3" t="inlineStr">
+        <is>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+        </is>
+      </c>
+      <c r="D373" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E373" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B374" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-07</t>
+        </is>
+      </c>
+      <c r="C374" s="3" t="inlineStr">
+        <is>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+        </is>
+      </c>
+      <c r="D374" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E374" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B375" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-08</t>
+        </is>
+      </c>
+      <c r="C375" s="3" t="inlineStr">
+        <is>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+        </is>
+      </c>
+      <c r="D375" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E375" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B376" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-09</t>
+        </is>
+      </c>
+      <c r="C376" s="3" t="inlineStr">
+        <is>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+        </is>
+      </c>
+      <c r="D376" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E376" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B377" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-10</t>
+        </is>
+      </c>
+      <c r="C377" s="3" t="inlineStr">
+        <is>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+        </is>
+      </c>
+      <c r="D377" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E377" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B378" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-11</t>
+        </is>
+      </c>
+      <c r="C378" s="3" t="inlineStr">
+        <is>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+        </is>
+      </c>
+      <c r="D378" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E378" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B379" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R4-ISO</t>
+        </is>
+      </c>
+      <c r="C379" s="3" t="inlineStr">
+        <is>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+        </is>
+      </c>
+      <c r="D379" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E379" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B380" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-01</t>
+        </is>
+      </c>
+      <c r="C380" s="3" t="inlineStr">
+        <is>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+        </is>
+      </c>
+      <c r="D380" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E380" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B381" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-02</t>
+        </is>
+      </c>
+      <c r="C381" s="3" t="inlineStr">
+        <is>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+        </is>
+      </c>
+      <c r="D381" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E381" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B382" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-03</t>
+        </is>
+      </c>
+      <c r="C382" s="3" t="inlineStr">
+        <is>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+        </is>
+      </c>
+      <c r="D382" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E382" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B383" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-04</t>
+        </is>
+      </c>
+      <c r="C383" s="3" t="inlineStr">
+        <is>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+        </is>
+      </c>
+      <c r="D383" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E383" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B384" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-05</t>
+        </is>
+      </c>
+      <c r="C384" s="3" t="inlineStr">
+        <is>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+        </is>
+      </c>
+      <c r="D384" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E384" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B385" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-06</t>
+        </is>
+      </c>
+      <c r="C385" s="3" t="inlineStr">
+        <is>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+        </is>
+      </c>
+      <c r="D385" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E385" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B386" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-07</t>
+        </is>
+      </c>
+      <c r="C386" s="3" t="inlineStr">
+        <is>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+        </is>
+      </c>
+      <c r="D386" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E386" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B387" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-08</t>
+        </is>
+      </c>
+      <c r="C387" s="3" t="inlineStr">
+        <is>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+        </is>
+      </c>
+      <c r="D387" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E387" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B388" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-09</t>
+        </is>
+      </c>
+      <c r="C388" s="3" t="inlineStr">
+        <is>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+        </is>
+      </c>
+      <c r="D388" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E388" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B389" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C389" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D389" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E389" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B390" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C359" s="3" t="inlineStr">
+      <c r="C390" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D359" s="3" t="inlineStr">
+      <c r="D390" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E359" s="3" t="inlineStr">
+      <c r="E390" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
@@ -23199,7 +24226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -23710,6 +24737,39 @@
       </c>
       <c r="G15" s="3" t="inlineStr"/>
     </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>OQ-15</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Forgotten passwords.** Self-service reset by email link, or admin-initiated reset only (the sign-in page today says "Lost access? Ask your workspace admin", and there is no reset flow at all)? What happens to MFA on reset?</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Self-service email reset (single-use 30-minute link, signs out all sessions, keeps MFA so a mailbox alone can't take the account) plus an admin "send reset link" on Members; lost second factor stays admin-assisted with step-up and audit</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Product owner</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
docs: tracker for DOCX export and the CEL wiring
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -197,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E26" headerRowCount="1">
-  <autoFilter ref="A1:E26"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E27" headerRowCount="1">
+  <autoFilter ref="A1:E27"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Source"/>
     <tableColumn id="2" name="ID"/>
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E390" headerRowCount="1">
-  <autoFilter ref="A1:E390"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E391" headerRowCount="1">
+  <autoFilter ref="A1:E391"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -1393,7 +1393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2092,6 +2092,33 @@
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>A-26 (BPMS-080/081/082)</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Expression wiring (docs/11 §14 *Expressions*, §15). (1) What each field must produce: a decision `when` is a non-null boolean; a `set` assignment has its variable's declared type; a timer `at` is a `datetime`; an `idempotencyKey` is a `string`; an assignee `ref` is a principal, a group or a string id (or a list of them, possibly null, when the fallback applies); `correlation` and connector `input` values may have any type. (2) Expression diagnostics map onto IR codes: syntax and limits to IR-E019, unknown variables to IR-E020, restricted reads in event-facing fields to IR-E021, null misuse to the new IR-E036, every other type error to the new IR-E035. A variable type with no expression type (`money` without a currency) is IR-E035 at the variable. (3) `expr:feel:` is rejected (IR-E019); the reference fixtures moved to CEL. (4) At run time a principal or group given as a bare string is read as `{ id }`; fields the built-in principal, group, file and instance shapes do not expose are dropped; `instance.display_id` is the instance id until display ids exist (BPMS-083). (5) A rule-table decision whose rule the evaluator cannot provide raises incident IR-R001 instead of taking `default`; until BPMS-087 a CEL stand-in per rule can be configured. (6) The time-zone offset for `today()` is injected into the evaluator, UTC by default, until calendars resolve it (BPMS-083)</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Runtime-lead review of docs/11 §14-§15; designer feedback (BPMS-100/101)</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Narrow or widen the per-field types (for example, allow string instants for `at`); split IR-E035 into finer codes; carry display ids on `start`</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5280,7 +5307,7 @@
       <c r="N33" s="3" t="inlineStr"/>
       <c r="O33" s="3" t="inlineStr">
         <is>
-          <t>Block editor (TipTap core, MIT; U-10 closed): headings, bold/italic/links, bullet and numbered lists, callouts, tables, accessible single-tab-stop toolbar, markdown shortcuts; block model validated server-side (ADR-0013 as built); shared renderer; HTML (print to tagged PDF in the browser) and Markdown export with a superseded banner, audited. E2E-R1-LIB-14, E2E-R1-UI-07, 28. Remaining: deterministic server-side tagged PDF, DOCX export/import, images and variables blocks.</t>
+          <t>Block editor (TipTap core, MIT; U-10 closed): headings, bold/italic/links, bullet and numbered lists, callouts, tables, accessible single-tab-stop toolbar, markdown shortcuts; block model validated server-side (ADR-0013 as built); shared renderer; HTML (print to tagged PDF in the browser) and Markdown export with a superseded banner, audited. E2E-R1-LIB-14, E2E-R1-UI-07, 28. Word (.docx) export with heading styles, numbering, tables and links, reproducible bytes; Export menu. E2E-R1-UI-44. Remaining: deterministic server-side tagged PDF, DOCX import, images and variables blocks.</t>
         </is>
       </c>
     </row>
@@ -6251,7 +6278,7 @@
       <c r="N48" s="3" t="inlineStr"/>
       <c r="O48" s="3" t="inlineStr">
         <is>
-          <t>procera-ir crate: IR v1 model, compiler with the docs/11 §11 checks (IR-E001..E034, E100, W001-W002, I001; JSON-pointer diagnostics), JCS canonical form + sha256 checksum, semantic diff with apply; a test per code, property tests, conformance/compiler fixtures, golden checksums for the reference processes (A-21). Remaining: type checking with the BPMS-081 engine, environment wiring at publish (BPMS-084), declared perpetual waits.</t>
+          <t>procera-ir crate: IR v1 model, compiler with the docs/11 §11 checks (IR-E001..E034, E100, W001-W002, I001; JSON-pointer diagnostics), JCS canonical form + sha256 checksum, semantic diff with apply; a test per code, property tests, conformance/compiler fixtures, golden checksums for the reference processes (A-21). Expressions type-checked with procera-expr (check 7 complete; IR-E035/E036, A-26); checked forms in Compiled::expressions; reference fixtures in CEL with regenerated checksums. Remaining: type checking with the BPMS-081 engine, environment wiring at publish (BPMS-084), declared perpetual waits.</t>
         </is>
       </c>
     </row>
@@ -6316,7 +6343,7 @@
       <c r="N49" s="3" t="inlineStr"/>
       <c r="O49" s="3" t="inlineStr">
         <is>
-          <t>procera-expr: a typed CEL subset of our own (A-22): static checker with null policy and exact decimal/money, budgeted pure evaluator (10k steps, 1 MiB, 64 KiB strings, 10k lists; exhaustion is IR-R010), stdlib, read sets with the restricted-in-event-facing check; wasm32 build checked; unit + property tests; docs/11 §6.1. Remaining: wiring into the IR compiler (BPMS-080) and runtime (BPMS-082), business-time functions with calendars (BPMS-083).</t>
+          <t>procera-expr: a typed CEL subset of our own (A-22): static checker with null policy and exact decimal/money, budgeted pure evaluator (10k steps, 1 MiB, 64 KiB strings, 10k lists; exhaustion is IR-R010), stdlib, read sets with the restricted-in-event-facing check; wasm32 build checked; unit + property tests; docs/11 §6.1. Wired end to end: the IR compiler type-checks with it and the runtime CelEvaluator runs stored checked expressions (injected now/tz, budget → IR-R010). Remaining: business-time functions with calendars (BPMS-083).</t>
         </is>
       </c>
     </row>
@@ -6381,7 +6408,7 @@
       <c r="N50" s="3" t="inlineStr"/>
       <c r="O50" s="3" t="inlineStr">
         <is>
-          <t>procera-runtime: pure deterministic interpreter (Program, InstanceState, Stimulus) -&gt; (state, commands) with injected Clock/IdGen; advance loop with a step budget (ContinueAdvance) and loop guard (IR-R004); start/end/terminate, set, decision (+rule tables via the Evaluator port), parallel split/join released exactly once, human.* work items, wait.timer/signal, service.call with typed error boundaries, notify, subprocess.call, case.open, timeout boundaries, cancel; commands with deterministic idempotency keys; unit tests per node kind, the five reference processes end to end, 22 conformance/runtime fixtures, property tests (replay, budgets, joins, terminate); docs/11 §15, A-23. Remaining: the CEL engine behind the port, persistence and timers (BPMS-083), work items (BPMS-085), incidents (BPMS-088), E2E once wired to the API.</t>
+          <t>procera-runtime: pure deterministic interpreter (Program, InstanceState, Stimulus) -&gt; (state, commands) with injected Clock/IdGen; advance loop with a step budget (ContinueAdvance) and loop guard (IR-R004); start/end/terminate, set, decision (+rule tables via the Evaluator port), parallel split/join released exactly once, human.* work items, wait.timer/signal, service.call with typed error boundaries, notify, subprocess.call, case.open, timeout boundaries, cancel; commands with deterministic idempotency keys; unit tests per node kind, the five reference processes end to end, 22 conformance/runtime fixtures, property tests (replay, budgets, joins, terminate); docs/11 §15, A-23. Runs real CEL via CelEvaluator; conformance (24 cases) green on CEL and the stand-in; determinism property over compiled CEL. Remaining: persistence and timers (BPMS-083), work items (BPMS-085), incidents (BPMS-088), E2E once wired to the API.</t>
         </is>
       </c>
     </row>
@@ -10019,7 +10046,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E390"/>
+  <dimension ref="A1:E391"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -17759,12 +17786,12 @@
       </c>
       <c r="B287" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-01</t>
+          <t>E2E-R1-UI-44</t>
         </is>
       </c>
       <c r="C287" s="3" t="inlineStr">
         <is>
-          <t>Onboarding start to finish: the owner invites from Members; the invitee opens the link from the email, creates an account (password confirmation checked) and lands on Home in the workspace; the link then no longer works; the owner sees them Active and opens their person page | BPMS-023</t>
+          <t>A reader opens Export on a published SOP (Print or PDF, Word, Markdown) and downloads a .docx | BPMS-042</t>
         </is>
       </c>
       <c r="D287" s="3" t="inlineStr">
@@ -17786,12 +17813,12 @@
       </c>
       <c r="B288" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-02</t>
+          <t>E2E-R1-FLOW-01</t>
         </is>
       </c>
       <c r="C288" s="3" t="inlineStr">
         <is>
-          <t>Someone with an account opens the invitation email, signs in from the page, comes back to it and joins with one click; an unknown link explains itself | BPMS-023</t>
+          <t>Onboarding start to finish: the owner invites from Members; the invitee opens the link from the email, creates an account (password confirmation checked) and lands on Home in the workspace; the link then no longer works; the owner sees them Active and opens their person page | BPMS-023</t>
         </is>
       </c>
       <c r="D288" s="3" t="inlineStr">
@@ -17813,12 +17840,12 @@
       </c>
       <c r="B289" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-03</t>
+          <t>E2E-R1-FLOW-02</t>
         </is>
       </c>
       <c r="C289" s="3" t="inlineStr">
         <is>
-          <t>Policy to evidence: the owner writes and publishes a policy and launches a campaign; a colleague (invited the same way) sees the task on Home, opens the acknowledgement email link, acknowledges on the document; the owner sees them Done, 1 of 2, and downloads the evidence CSV | BPMS-040, 046</t>
+          <t>Someone with an account opens the invitation email, signs in from the page, comes back to it and joins with one click; an unknown link explains itself | BPMS-023</t>
         </is>
       </c>
       <c r="D289" s="3" t="inlineStr">
@@ -17840,12 +17867,12 @@
       </c>
       <c r="B290" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-04</t>
+          <t>E2E-R1-FLOW-03</t>
         </is>
       </c>
       <c r="C290" s="3" t="inlineStr">
         <is>
-          <t>Announcement: the owner composes a critical post that needs acknowledgement and publishes it; a colleague opens the email link while signed out, signs in, lands on the open post and confirms; the owner sees the receipt | BPMS-047</t>
+          <t>Policy to evidence: the owner writes and publishes a policy and launches a campaign; a colleague (invited the same way) sees the task on Home, opens the acknowledgement email link, acknowledges on the document; the owner sees them Done, 1 of 2, and downloads the evidence CSV | BPMS-040, 046</t>
         </is>
       </c>
       <c r="D290" s="3" t="inlineStr">
@@ -17867,12 +17894,12 @@
       </c>
       <c r="B291" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-05</t>
+          <t>E2E-R1-FLOW-04</t>
         </is>
       </c>
       <c r="C291" s="3" t="inlineStr">
         <is>
-          <t>Review loop: the owner submits a controlled policy; the reviewer (invited as Reviewer) gets the review email, opens it and requests changes with a comment; the owner gets a notification quoting it, edits and resubmits; the reviewer approves from Home; the owner is told it is approved and publishes | BPMS-040</t>
+          <t>Announcement: the owner composes a critical post that needs acknowledgement and publishes it; a colleague opens the email link while signed out, signs in, lands on the open post and confirms; the owner sees the receipt | BPMS-047</t>
         </is>
       </c>
       <c r="D291" s="3" t="inlineStr">
@@ -17894,12 +17921,12 @@
       </c>
       <c r="B292" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-06</t>
+          <t>E2E-R1-FLOW-05</t>
         </is>
       </c>
       <c r="C292" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval: a second admin joins from the invitation and turns on two-step verification; the owner sends a workspace-wide post for approval; the admin gets the approval email, opens it and sends it back with a note; the owner gets a notification with the note, edits and resubmits; the admin approves and publishes; the owner is told; the post is in the feed | BPMS-047</t>
+          <t>Review loop: the owner submits a controlled policy; the reviewer (invited as Reviewer) gets the review email, opens it and requests changes with a comment; the owner gets a notification quoting it, edits and resubmits; the reviewer approves from Home; the owner is told it is approved and publishes | BPMS-040</t>
         </is>
       </c>
       <c r="D292" s="3" t="inlineStr">
@@ -17921,12 +17948,12 @@
       </c>
       <c r="B293" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-01</t>
+          <t>E2E-R1-FLOW-06</t>
         </is>
       </c>
       <c r="C293" s="3" t="inlineStr">
         <is>
-          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
+          <t>Announcement approval: a second admin joins from the invitation and turns on two-step verification; the owner sends a workspace-wide post for approval; the admin gets the approval email, opens it and sends it back with a note; the owner gets a notification with the note, edits and resubmits; the admin approves and publishes; the owner is told; the post is in the feed | BPMS-047</t>
         </is>
       </c>
       <c r="D293" s="3" t="inlineStr">
@@ -17948,12 +17975,12 @@
       </c>
       <c r="B294" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-02</t>
+          <t>E2E-R1-CMP-01</t>
         </is>
       </c>
       <c r="C294" s="3" t="inlineStr">
         <is>
-          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
+          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
         </is>
       </c>
       <c r="D294" s="3" t="inlineStr">
@@ -17975,12 +18002,12 @@
       </c>
       <c r="B295" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-03</t>
+          <t>E2E-R1-CMP-02</t>
         </is>
       </c>
       <c r="C295" s="3" t="inlineStr">
         <is>
-          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
+          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
         </is>
       </c>
       <c r="D295" s="3" t="inlineStr">
@@ -18002,12 +18029,12 @@
       </c>
       <c r="B296" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-04</t>
+          <t>E2E-R1-CMP-03</t>
         </is>
       </c>
       <c r="C296" s="3" t="inlineStr">
         <is>
-          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
+          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
         </is>
       </c>
       <c r="D296" s="3" t="inlineStr">
@@ -18029,12 +18056,12 @@
       </c>
       <c r="B297" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-05</t>
+          <t>E2E-R1-CMP-04</t>
         </is>
       </c>
       <c r="C297" s="3" t="inlineStr">
         <is>
-          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
+          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
         </is>
       </c>
       <c r="D297" s="3" t="inlineStr">
@@ -18056,12 +18083,12 @@
       </c>
       <c r="B298" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-06</t>
+          <t>E2E-R1-CMP-05</t>
         </is>
       </c>
       <c r="C298" s="3" t="inlineStr">
         <is>
-          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
+          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
         </is>
       </c>
       <c r="D298" s="3" t="inlineStr">
@@ -18083,12 +18110,12 @@
       </c>
       <c r="B299" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-07</t>
+          <t>E2E-R1-CMP-06</t>
         </is>
       </c>
       <c r="C299" s="3" t="inlineStr">
         <is>
-          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
+          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
         </is>
       </c>
       <c r="D299" s="3" t="inlineStr">
@@ -18110,12 +18137,12 @@
       </c>
       <c r="B300" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-01</t>
+          <t>E2E-R1-CMP-07</t>
         </is>
       </c>
       <c r="C300" s="3" t="inlineStr">
         <is>
-          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
+          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D300" s="3" t="inlineStr">
@@ -18137,12 +18164,12 @@
       </c>
       <c r="B301" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-02</t>
+          <t>E2E-R1-ANN-01</t>
         </is>
       </c>
       <c r="C301" s="3" t="inlineStr">
         <is>
-          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
+          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
         </is>
       </c>
       <c r="D301" s="3" t="inlineStr">
@@ -18164,12 +18191,12 @@
       </c>
       <c r="B302" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-03</t>
+          <t>E2E-R1-ANN-02</t>
         </is>
       </c>
       <c r="C302" s="3" t="inlineStr">
         <is>
-          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
+          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
         </is>
       </c>
       <c r="D302" s="3" t="inlineStr">
@@ -18191,12 +18218,12 @@
       </c>
       <c r="B303" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-04</t>
+          <t>E2E-R1-ANN-03</t>
         </is>
       </c>
       <c r="C303" s="3" t="inlineStr">
         <is>
-          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
+          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
         </is>
       </c>
       <c r="D303" s="3" t="inlineStr">
@@ -18218,12 +18245,12 @@
       </c>
       <c r="B304" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-05</t>
+          <t>E2E-R1-ANN-04</t>
         </is>
       </c>
       <c r="C304" s="3" t="inlineStr">
         <is>
-          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
+          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
         </is>
       </c>
       <c r="D304" s="3" t="inlineStr">
@@ -18245,12 +18272,12 @@
       </c>
       <c r="B305" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-06</t>
+          <t>E2E-R1-ANN-05</t>
         </is>
       </c>
       <c r="C305" s="3" t="inlineStr">
         <is>
-          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
+          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D305" s="3" t="inlineStr">
@@ -18272,12 +18299,12 @@
       </c>
       <c r="B306" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-01</t>
+          <t>E2E-R1-ANN-06</t>
         </is>
       </c>
       <c r="C306" s="3" t="inlineStr">
         <is>
-          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
+          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
         </is>
       </c>
       <c r="D306" s="3" t="inlineStr">
@@ -18299,12 +18326,12 @@
       </c>
       <c r="B307" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-02</t>
+          <t>E2E-R1-SRCH-01</t>
         </is>
       </c>
       <c r="C307" s="3" t="inlineStr">
         <is>
-          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
+          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
         </is>
       </c>
       <c r="D307" s="3" t="inlineStr">
@@ -18326,12 +18353,12 @@
       </c>
       <c r="B308" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-03</t>
+          <t>E2E-R1-SRCH-02</t>
         </is>
       </c>
       <c r="C308" s="3" t="inlineStr">
         <is>
-          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
+          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
         </is>
       </c>
       <c r="D308" s="3" t="inlineStr">
@@ -18353,12 +18380,12 @@
       </c>
       <c r="B309" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-01</t>
+          <t>E2E-R1-SRCH-03</t>
         </is>
       </c>
       <c r="C309" s="3" t="inlineStr">
         <is>
-          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
+          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
         </is>
       </c>
       <c r="D309" s="3" t="inlineStr">
@@ -18380,12 +18407,12 @@
       </c>
       <c r="B310" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-02</t>
+          <t>E2E-R1-AUDX-01</t>
         </is>
       </c>
       <c r="C310" s="3" t="inlineStr">
         <is>
-          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
+          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
         </is>
       </c>
       <c r="D310" s="3" t="inlineStr">
@@ -18407,12 +18434,12 @@
       </c>
       <c r="B311" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-03</t>
+          <t>E2E-R1-AUDX-02</t>
         </is>
       </c>
       <c r="C311" s="3" t="inlineStr">
         <is>
-          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
+          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
         </is>
       </c>
       <c r="D311" s="3" t="inlineStr">
@@ -18434,12 +18461,12 @@
       </c>
       <c r="B312" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-04</t>
+          <t>E2E-R1-AUDX-03</t>
         </is>
       </c>
       <c r="C312" s="3" t="inlineStr">
         <is>
-          <t>Chain verify reports intact | FR-T02</t>
+          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
         </is>
       </c>
       <c r="D312" s="3" t="inlineStr">
@@ -18461,12 +18488,12 @@
       </c>
       <c r="B313" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-05</t>
+          <t>E2E-R1-AUDX-04</t>
         </is>
       </c>
       <c r="C313" s="3" t="inlineStr">
         <is>
-          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
+          <t>Chain verify reports intact | FR-T02</t>
         </is>
       </c>
       <c r="D313" s="3" t="inlineStr">
@@ -18488,12 +18515,12 @@
       </c>
       <c r="B314" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-06</t>
+          <t>E2E-R1-AUDX-05</t>
         </is>
       </c>
       <c r="C314" s="3" t="inlineStr">
         <is>
-          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
+          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
         </is>
       </c>
       <c r="D314" s="3" t="inlineStr">
@@ -18515,12 +18542,12 @@
       </c>
       <c r="B315" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-07</t>
+          <t>E2E-R1-AUDX-06</t>
         </is>
       </c>
       <c r="C315" s="3" t="inlineStr">
         <is>
-          <t>`POST /audit/query`: an AND group (category, action prefix, within P30D) sorted ascending pages by cursor; an OR group returns only matching events; unknown fields or values, bad durations, nesting deeper than 2 and unsupported sorts → 422 | BPMS-064, docs/08 §7.5</t>
+          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
         </is>
       </c>
       <c r="D315" s="3" t="inlineStr">
@@ -18542,12 +18569,12 @@
       </c>
       <c r="B316" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-08</t>
+          <t>E2E-R1-AUDX-07</t>
         </is>
       </c>
       <c r="C316" s="3" t="inlineStr">
         <is>
-          <t>A background export (202) runs as a job, finishes `done` with rows, its CSV downloads through the requester's signed file link, the requester is notified, and both `audit.export_requested` and `audit.exported` are recorded | BPMS-064, FR-T04</t>
+          <t>`POST /audit/query`: an AND group (category, action prefix, within P30D) sorted ascending pages by cursor; an OR group returns only matching events; unknown fields or values, bad durations, nesting deeper than 2 and unsupported sorts → 422 | BPMS-064, docs/08 §7.5</t>
         </is>
       </c>
       <c r="D316" s="3" t="inlineStr">
@@ -18569,12 +18596,12 @@
       </c>
       <c r="B317" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-AUDX-08</t>
         </is>
       </c>
       <c r="C317" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>A background export (202) runs as a job, finishes `done` with rows, its CSV downloads through the requester's signed file link, the requester is notified, and both `audit.export_requested` and `audit.exported` are recorded | BPMS-064, FR-T04</t>
         </is>
       </c>
       <c r="D317" s="3" t="inlineStr">
@@ -18596,12 +18623,12 @@
       </c>
       <c r="B318" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C318" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
         </is>
       </c>
       <c r="D318" s="3" t="inlineStr">
@@ -18623,12 +18650,12 @@
       </c>
       <c r="B319" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C319" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D319" s="3" t="inlineStr">
@@ -18650,12 +18677,12 @@
       </c>
       <c r="B320" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C320" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D320" s="3" t="inlineStr">
@@ -18677,12 +18704,12 @@
       </c>
       <c r="B321" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C321" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
         </is>
       </c>
       <c r="D321" s="3" t="inlineStr">
@@ -18704,12 +18731,12 @@
       </c>
       <c r="B322" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C322" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
         </is>
       </c>
       <c r="D322" s="3" t="inlineStr">
@@ -18731,12 +18758,12 @@
       </c>
       <c r="B323" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C323" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D323" s="3" t="inlineStr">
@@ -18758,12 +18785,12 @@
       </c>
       <c r="B324" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C324" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D324" s="3" t="inlineStr">
@@ -18785,12 +18812,12 @@
       </c>
       <c r="B325" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C325" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
         </is>
       </c>
       <c r="D325" s="3" t="inlineStr">
@@ -18812,12 +18839,12 @@
       </c>
       <c r="B326" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C326" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D326" s="3" t="inlineStr">
@@ -18839,12 +18866,12 @@
       </c>
       <c r="B327" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C327" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D327" s="3" t="inlineStr">
@@ -18866,12 +18893,12 @@
       </c>
       <c r="B328" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C328" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D328" s="3" t="inlineStr">
@@ -18893,12 +18920,12 @@
       </c>
       <c r="B329" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C329" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D329" s="3" t="inlineStr">
@@ -18920,12 +18947,12 @@
       </c>
       <c r="B330" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C330" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
         </is>
       </c>
       <c r="D330" s="3" t="inlineStr">
@@ -18947,12 +18974,12 @@
       </c>
       <c r="B331" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C331" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
         </is>
       </c>
       <c r="D331" s="3" t="inlineStr">
@@ -18974,12 +19001,12 @@
       </c>
       <c r="B332" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C332" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
         </is>
       </c>
       <c r="D332" s="3" t="inlineStr">
@@ -19001,12 +19028,12 @@
       </c>
       <c r="B333" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C333" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D333" s="3" t="inlineStr">
@@ -19028,12 +19055,12 @@
       </c>
       <c r="B334" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C334" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
         </is>
       </c>
       <c r="D334" s="3" t="inlineStr">
@@ -19055,12 +19082,12 @@
       </c>
       <c r="B335" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C335" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
         </is>
       </c>
       <c r="D335" s="3" t="inlineStr">
@@ -19082,12 +19109,12 @@
       </c>
       <c r="B336" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C336" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D336" s="3" t="inlineStr">
@@ -19109,12 +19136,12 @@
       </c>
       <c r="B337" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C337" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
         </is>
       </c>
       <c r="D337" s="3" t="inlineStr">
@@ -19136,12 +19163,12 @@
       </c>
       <c r="B338" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C338" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D338" s="3" t="inlineStr">
@@ -19163,12 +19190,12 @@
       </c>
       <c r="B339" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C339" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D339" s="3" t="inlineStr">
@@ -19190,12 +19217,12 @@
       </c>
       <c r="B340" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C340" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D340" s="3" t="inlineStr">
@@ -19217,12 +19244,12 @@
       </c>
       <c r="B341" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C341" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D341" s="3" t="inlineStr">
@@ -19244,12 +19271,12 @@
       </c>
       <c r="B342" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C342" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D342" s="3" t="inlineStr">
@@ -19271,12 +19298,12 @@
       </c>
       <c r="B343" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C343" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D343" s="3" t="inlineStr">
@@ -19298,12 +19325,12 @@
       </c>
       <c r="B344" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C344" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D344" s="3" t="inlineStr">
@@ -19325,12 +19352,12 @@
       </c>
       <c r="B345" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C345" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D345" s="3" t="inlineStr">
@@ -19352,12 +19379,12 @@
       </c>
       <c r="B346" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C346" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D346" s="3" t="inlineStr">
@@ -19379,12 +19406,12 @@
       </c>
       <c r="B347" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C347" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D347" s="3" t="inlineStr">
@@ -19406,12 +19433,12 @@
       </c>
       <c r="B348" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C348" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D348" s="3" t="inlineStr">
@@ -19433,12 +19460,12 @@
       </c>
       <c r="B349" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C349" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D349" s="3" t="inlineStr">
@@ -19460,12 +19487,12 @@
       </c>
       <c r="B350" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C350" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D350" s="3" t="inlineStr">
@@ -19487,12 +19514,12 @@
       </c>
       <c r="B351" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C351" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D351" s="3" t="inlineStr">
@@ -19514,12 +19541,12 @@
       </c>
       <c r="B352" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C352" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D352" s="3" t="inlineStr">
@@ -19541,12 +19568,12 @@
       </c>
       <c r="B353" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C353" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D353" s="3" t="inlineStr">
@@ -19568,12 +19595,12 @@
       </c>
       <c r="B354" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C354" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D354" s="3" t="inlineStr">
@@ -19595,12 +19622,12 @@
       </c>
       <c r="B355" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C355" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D355" s="3" t="inlineStr">
@@ -19622,12 +19649,12 @@
       </c>
       <c r="B356" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C356" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D356" s="3" t="inlineStr">
@@ -19649,12 +19676,12 @@
       </c>
       <c r="B357" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C357" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D357" s="3" t="inlineStr">
@@ -19676,12 +19703,12 @@
       </c>
       <c r="B358" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C358" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D358" s="3" t="inlineStr">
@@ -19703,12 +19730,12 @@
       </c>
       <c r="B359" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C359" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D359" s="3" t="inlineStr">
@@ -19730,12 +19757,12 @@
       </c>
       <c r="B360" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C360" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D360" s="3" t="inlineStr">
@@ -19757,12 +19784,12 @@
       </c>
       <c r="B361" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C361" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D361" s="3" t="inlineStr">
@@ -19784,12 +19811,12 @@
       </c>
       <c r="B362" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C362" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D362" s="3" t="inlineStr">
@@ -19811,12 +19838,12 @@
       </c>
       <c r="B363" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C363" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D363" s="3" t="inlineStr">
@@ -19838,12 +19865,12 @@
       </c>
       <c r="B364" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C364" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D364" s="3" t="inlineStr">
@@ -19865,12 +19892,12 @@
       </c>
       <c r="B365" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C365" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D365" s="3" t="inlineStr">
@@ -19892,12 +19919,12 @@
       </c>
       <c r="B366" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C366" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D366" s="3" t="inlineStr">
@@ -19919,12 +19946,12 @@
       </c>
       <c r="B367" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C367" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D367" s="3" t="inlineStr">
@@ -19946,12 +19973,12 @@
       </c>
       <c r="B368" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C368" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D368" s="3" t="inlineStr">
@@ -19973,12 +20000,12 @@
       </c>
       <c r="B369" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C369" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D369" s="3" t="inlineStr">
@@ -20000,12 +20027,12 @@
       </c>
       <c r="B370" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C370" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D370" s="3" t="inlineStr">
@@ -20027,12 +20054,12 @@
       </c>
       <c r="B371" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C371" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D371" s="3" t="inlineStr">
@@ -20054,12 +20081,12 @@
       </c>
       <c r="B372" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C372" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D372" s="3" t="inlineStr">
@@ -20081,12 +20108,12 @@
       </c>
       <c r="B373" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C373" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D373" s="3" t="inlineStr">
@@ -20108,12 +20135,12 @@
       </c>
       <c r="B374" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C374" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D374" s="3" t="inlineStr">
@@ -20135,12 +20162,12 @@
       </c>
       <c r="B375" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C375" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D375" s="3" t="inlineStr">
@@ -20162,12 +20189,12 @@
       </c>
       <c r="B376" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C376" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D376" s="3" t="inlineStr">
@@ -20189,12 +20216,12 @@
       </c>
       <c r="B377" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C377" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D377" s="3" t="inlineStr">
@@ -20216,12 +20243,12 @@
       </c>
       <c r="B378" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C378" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D378" s="3" t="inlineStr">
@@ -20243,12 +20270,12 @@
       </c>
       <c r="B379" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R4-11</t>
         </is>
       </c>
       <c r="C379" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
         </is>
       </c>
       <c r="D379" s="3" t="inlineStr">
@@ -20270,12 +20297,12 @@
       </c>
       <c r="B380" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-ISO</t>
         </is>
       </c>
       <c r="C380" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
         </is>
       </c>
       <c r="D380" s="3" t="inlineStr">
@@ -20297,12 +20324,12 @@
       </c>
       <c r="B381" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R5-01</t>
         </is>
       </c>
       <c r="C381" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
         </is>
       </c>
       <c r="D381" s="3" t="inlineStr">
@@ -20324,12 +20351,12 @@
       </c>
       <c r="B382" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R5-02</t>
         </is>
       </c>
       <c r="C382" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
         </is>
       </c>
       <c r="D382" s="3" t="inlineStr">
@@ -20351,12 +20378,12 @@
       </c>
       <c r="B383" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R5-03</t>
         </is>
       </c>
       <c r="C383" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
         </is>
       </c>
       <c r="D383" s="3" t="inlineStr">
@@ -20378,12 +20405,12 @@
       </c>
       <c r="B384" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R5-04</t>
         </is>
       </c>
       <c r="C384" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
         </is>
       </c>
       <c r="D384" s="3" t="inlineStr">
@@ -20405,12 +20432,12 @@
       </c>
       <c r="B385" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R5-05</t>
         </is>
       </c>
       <c r="C385" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
         </is>
       </c>
       <c r="D385" s="3" t="inlineStr">
@@ -20432,12 +20459,12 @@
       </c>
       <c r="B386" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R5-06</t>
         </is>
       </c>
       <c r="C386" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
         </is>
       </c>
       <c r="D386" s="3" t="inlineStr">
@@ -20459,12 +20486,12 @@
       </c>
       <c r="B387" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R5-07</t>
         </is>
       </c>
       <c r="C387" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
         </is>
       </c>
       <c r="D387" s="3" t="inlineStr">
@@ -20486,12 +20513,12 @@
       </c>
       <c r="B388" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R5-08</t>
         </is>
       </c>
       <c r="C388" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
         </is>
       </c>
       <c r="D388" s="3" t="inlineStr">
@@ -20513,12 +20540,12 @@
       </c>
       <c r="B389" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R5-09</t>
         </is>
       </c>
       <c r="C389" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
         </is>
       </c>
       <c r="D389" s="3" t="inlineStr">
@@ -20540,20 +20567,47 @@
       </c>
       <c r="B390" s="3" t="inlineStr">
         <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C390" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D390" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E390" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B391" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C390" s="3" t="inlineStr">
+      <c r="C391" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D390" s="3" t="inlineStr">
+      <c r="D391" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E390" s="3" t="inlineStr">
+      <c r="E391" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
docs: tracker for image blocks
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -197,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E27" headerRowCount="1">
-  <autoFilter ref="A1:E27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E28" headerRowCount="1">
+  <autoFilter ref="A1:E28"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Source"/>
     <tableColumn id="2" name="ID"/>
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E391" headerRowCount="1">
-  <autoFilter ref="A1:E391"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E393" headerRowCount="1">
+  <autoFilter ref="A1:E393"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -1393,7 +1393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2119,6 +2119,29 @@
           <t>Narrow or widen the per-field types (for example, allow string instants for `at`); split IR-E035 into finer codes; carry display ids on `start`</t>
         </is>
       </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>A-28 (BPMS-042)</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Image blocks: the alt text is required (no decorative images yet) and is the block's `text`, so diffs, search and re-ack hashes see it; a swapped picture with the same text still diffs (the file id is part of the compared text). Images can only use files already attached to the same version (attach, then insert); creating an artifact with images is refused. Starting a new version copies the previous version's attachment links so its images and files carry over. DOCX shows `[Image: alt] caption` until pictures are embedded.</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5307,7 +5330,7 @@
       <c r="N33" s="3" t="inlineStr"/>
       <c r="O33" s="3" t="inlineStr">
         <is>
-          <t>Block editor (TipTap core, MIT; U-10 closed): headings, bold/italic/links, bullet and numbered lists, callouts, tables, accessible single-tab-stop toolbar, markdown shortcuts; block model validated server-side (ADR-0013 as built); shared renderer; HTML (print to tagged PDF in the browser) and Markdown export with a superseded banner, audited. E2E-R1-LIB-14, E2E-R1-UI-07, 28. Word (.docx) export with heading styles, numbering, tables and links, reproducible bytes; Export menu. E2E-R1-UI-44. Remaining: deterministic server-side tagged PDF, DOCX import, images and variables blocks.</t>
+          <t>Block editor (TipTap core, MIT; U-10 closed): headings, bold/italic/links, bullet and numbered lists, callouts, tables, accessible single-tab-stop toolbar, markdown shortcuts; block model validated server-side (ADR-0013 as built); shared renderer; HTML (print to tagged PDF in the browser) and Markdown export with a superseded banner, audited. E2E-R1-LIB-14, E2E-R1-UI-07, 28. Word (.docx) export with heading styles, numbering, tables and links, reproducible bytes; Export menu. E2E-R1-UI-44. Image blocks (alt text required, attached clean images only, embedded in print HTML; A-28) inserted from the editor. E2E-R1-LIB-15, UI-45. Remaining: deterministic server-side tagged PDF, DOCX import, pictures inside DOCX, variables blocks.</t>
         </is>
       </c>
     </row>
@@ -10046,7 +10069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E391"/>
+  <dimension ref="A1:E393"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -16247,12 +16270,12 @@
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-POL-01</t>
+          <t>E2E-R1-LIB-15</t>
         </is>
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>Readers never see drafts: absent from lists, reads and search until published; a later draft stays hidden (version 404, diff 404, versions list shows v1 only); authors see drafts in search | BPMS-045, A-14</t>
+          <t>Image blocks: refused unless a clean image attached to the draft with a description; HTML export embeds it, Markdown references it; a new version keeps the attachment | BPMS-042</t>
         </is>
       </c>
       <c r="D230" s="3" t="inlineStr">
@@ -16274,12 +16297,12 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-POL-02</t>
+          <t>E2E-R1-POL-01</t>
         </is>
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>Applicability: empty audience or restricted without one → 422; members cannot set it (403); a restricted policy is hidden from members outside its group in lists, reads, search, the portal and change requests (404), and shown to those inside; an unrestricted one is listed for everyone but only "applicable" to its audience | BPMS-045, FR-PL01/PL02</t>
+          <t>Readers never see drafts: absent from lists, reads and search until published; a later draft stays hidden (version 404, diff 404, versions list shows v1 only); authors see drafts in search | BPMS-045, A-14</t>
         </is>
       </c>
       <c r="D231" s="3" t="inlineStr">
@@ -16301,12 +16324,12 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-POL-03</t>
+          <t>E2E-R1-POL-02</t>
         </is>
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>The portal lists published policies that apply to the member (no drafts), ordered by category, with what changed since the previous version (added/changed counts, reason) and text/category filters | BPMS-045, FR-PL02</t>
+          <t>Applicability: empty audience or restricted without one → 422; members cannot set it (403); a restricted policy is hidden from members outside its group in lists, reads, search, the portal and change requests (404), and shown to those inside; an unrestricted one is listed for everyone but only "applicable" to its audience | BPMS-045, FR-PL01/PL02</t>
         </is>
       </c>
       <c r="D232" s="3" t="inlineStr">
@@ -16328,12 +16351,12 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-POL-04</t>
+          <t>E2E-R1-POL-03</t>
         </is>
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>A major version asks the applicable audience to re-acknowledge that exact version; a minor one does not (major_only) | BPMS-045, FR-PL03</t>
+          <t>The portal lists published policies that apply to the member (no drafts), ordered by category, with what changed since the previous version (added/changed counts, reason) and text/category filters | BPMS-045, FR-PL02</t>
         </is>
       </c>
       <c r="D233" s="3" t="inlineStr">
@@ -16355,12 +16378,12 @@
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-POL-05</t>
+          <t>E2E-R1-POL-04</t>
         </is>
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>Every_publish asks on minors, none never asks, and a scheduled major asks when it goes live | BPMS-045, FR-PL03</t>
+          <t>A major version asks the applicable audience to re-acknowledge that exact version; a minor one does not (major_only) | BPMS-045, FR-PL03</t>
         </is>
       </c>
       <c r="D234" s="3" t="inlineStr">
@@ -16382,12 +16405,12 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ADM-01</t>
+          <t>E2E-R1-POL-05</t>
         </is>
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>Overview: overdue acknowledgements rank first in "needs attention", followed by an admin without two-step verification; acknowledgement metrics and a daily published series; the security strip counts a failed sign-in, members without MFA and the new admin grant; requests/storage are null; members get 403; an inverted range → 422 | BPMS-063, FR-A01</t>
+          <t>Every_publish asks on minors, none never asks, and a scheduled major asks when it goes live | BPMS-045, FR-PL03</t>
         </is>
       </c>
       <c r="D235" s="3" t="inlineStr">
@@ -16409,12 +16432,12 @@
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ADM-02</t>
+          <t>E2E-R1-ADM-01</t>
         </is>
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>People &amp; access: counts (members, no MFA, privileged, pending invites), member row (MFA off, last active set, not dormant), no-MFA and admin filters; unknown filter → 422; members get 403 | BPMS-063, FR-A06</t>
+          <t>Overview: overdue acknowledgements rank first in "needs attention", followed by an admin without two-step verification; acknowledgement metrics and a daily published series; the security strip counts a failed sign-in, members without MFA and the new admin grant; requests/storage are null; members get 403; an inverted range → 422 | BPMS-063, FR-A01</t>
         </is>
       </c>
       <c r="D236" s="3" t="inlineStr">
@@ -16436,12 +16459,12 @@
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-RET-01</t>
+          <t>E2E-R1-ADM-02</t>
         </is>
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>Retention classes are listed (draft and operational automatic; governance records and audit never). Drafts untouched for 170 of 180 days are due and their author is notified once; editing one resets its clock; 11 days later the untouched drafts are deleted (a never-published artifact with its draft, a v2 draft beside a published v1 that stays); the run is recorded and audited (`retention.purged`) | BPMS-066, PRV-04</t>
+          <t>People &amp; access: counts (members, no MFA, privileged, pending invites), member row (MFA off, last active set, not dormant), no-MFA and admin filters; unknown filter → 422; members get 403 | BPMS-063, FR-A06</t>
         </is>
       </c>
       <c r="D237" s="3" t="inlineStr">
@@ -16463,12 +16486,12 @@
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-RET-02</t>
+          <t>E2E-R1-RET-01</t>
         </is>
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>A read notification older than the operational period is removed by the job; members cannot see retention (403) | BPMS-066, PRV-04</t>
+          <t>Retention classes are listed (draft and operational automatic; governance records and audit never). Drafts untouched for 170 of 180 days are due and their author is notified once; editing one resets its clock; 11 days later the untouched drafts are deleted (a never-published artifact with its draft, a v2 draft beside a published v1 that stays); the run is recorded and audited (`retention.purged`) | BPMS-066, PRV-04</t>
         </is>
       </c>
       <c r="D238" s="3" t="inlineStr">
@@ -16490,12 +16513,12 @@
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-KEY-01</t>
+          <t>E2E-R1-RET-02</t>
         </is>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>An invitation email is envelope-encrypted under the workspace KEK; rotation needs a reason (422) and is audited; the email stays readable right after rotation and after the background rewrap moves it to v2; the unused v1 is destroyed; members cannot see or rotate keys (403). Crypto-shredding is proven in the `procera-keys` integration test | BPMS-030</t>
+          <t>A read notification older than the operational period is removed by the job; members cannot see retention (403) | BPMS-066, PRV-04</t>
         </is>
       </c>
       <c r="D239" s="3" t="inlineStr">
@@ -16517,12 +16540,12 @@
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FILE-01</t>
+          <t>E2E-R1-KEY-01</t>
         </is>
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>A chunked upload refuses a wrong offset (409) and resumes from `received`; completion before all bytes 409; the file is hashed (SHA-256 matches), typed by content (PDF despite a .txt name and text/plain declared) and clean; the signed link downloads without a bearer with nosniff and the exact bytes; a tampered link 403; another member gets 404; upload and download are audited | BPMS-060, FR-F01–F03</t>
+          <t>An invitation email is envelope-encrypted under the workspace KEK; rotation needs a reason (422) and is audited; the email stays readable right after rotation and after the background rewrap moves it to v2; the unused v1 is destroyed; members cannot see or rotate keys (403). Crypto-shredding is proven in the `procera-keys` integration test | BPMS-030</t>
         </is>
       </c>
       <c r="D240" s="3" t="inlineStr">
@@ -16544,12 +16567,12 @@
       </c>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FILE-02</t>
+          <t>E2E-R1-FILE-01</t>
         </is>
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>EICAR is quarantined and its download link refused (409); an executable named .pdf and an HTML file named .txt are rejected by content; 500 MB → 413; empty → 422; usage counts states | BPMS-060, FR-F02</t>
+          <t>A chunked upload refuses a wrong offset (409) and resumes from `received`; completion before all bytes 409; the file is hashed (SHA-256 matches), typed by content (PDF despite a .txt name and text/plain declared) and clean; the signed link downloads without a bearer with nosniff and the exact bytes; a tampered link 403; another member gets 404; upload and download are audited | BPMS-060, FR-F01–F03</t>
         </is>
       </c>
       <c r="D241" s="3" t="inlineStr">
@@ -16571,12 +16594,12 @@
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FILE-03</t>
+          <t>E2E-R1-FILE-02</t>
         </is>
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>A draft takes an attachment; after publishing it can't be unlinked or the file deleted (409); a member reading the published SOP downloads it; an unattached file past the orphan period is listed, members can't purge (403), the owner purges it | BPMS-060/062, FR-F05/F07</t>
+          <t>EICAR is quarantined and its download link refused (409); an executable named .pdf and an HTML file named .txt are rejected by content; 500 MB → 413; empty → 422; usage counts states | BPMS-060, FR-F02</t>
         </is>
       </c>
       <c r="D242" s="3" t="inlineStr">
@@ -16598,12 +16621,12 @@
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FILE-04</t>
+          <t>E2E-R1-FILE-03</t>
         </is>
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>A PNG, a PDF and a JPEG get preview links that serve inline with the strict headers (CSP sandbox, nosniff, CORP same-origin, no-store) and a ≤ 2-minute expiry; the JPEG's Exif is removed; a text file gets kind none and no URL; a tampered token and a download token on the preview route are 403; another member gets 404; previews are audited | BPMS-061, FR-F04/F02</t>
+          <t>A draft takes an attachment; after publishing it can't be unlinked or the file deleted (409); a member reading the published SOP downloads it; an unattached file past the orphan period is listed, members can't purge (403), the owner purges it | BPMS-060/062, FR-F05/F07</t>
         </is>
       </c>
       <c r="D243" s="3" t="inlineStr">
@@ -16625,12 +16648,12 @@
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-VIEW-01</t>
+          <t>E2E-R1-FILE-04</t>
         </is>
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>Saved views: personal and shared, one default per member (setting a new default clears the old), invalid list or name 422; another member sees only shared views and can't edit or delete them (403) or touch personal ones (404); unsharing hides it; exports are recorded (`data.exported`), unknown format 422 | BPMS-028, FR-V05/V06</t>
+          <t>A PNG, a PDF and a JPEG get preview links that serve inline with the strict headers (CSP sandbox, nosniff, CORP same-origin, no-store) and a ≤ 2-minute expiry; the JPEG's Exif is removed; a text file gets kind none and no URL; a tampered token and a download token on the preview route are 403; another member gets 404; previews are audited | BPMS-061, FR-F04/F02</t>
         </is>
       </c>
       <c r="D244" s="3" t="inlineStr">
@@ -16652,12 +16675,12 @@
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-01</t>
+          <t>E2E-R1-VIEW-01</t>
         </is>
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>Sign in through the browser (password + recovery code) lands on Home; navigation is permission-shaped with the current page marked; axe clean on sign-in and Home; reload keeps the session | docs/05 §2.1, §3.1, WCAG 2.2 AA</t>
+          <t>Saved views: personal and shared, one default per member (setting a new default clears the old), invalid list or name 422; another member sees only shared views and can't edit or delete them (403) or touch personal ones (404); unsharing hides it; exports are recorded (`data.exported`), unknown format 422 | BPMS-028, FR-V05/V06</t>
         </is>
       </c>
       <c r="D245" s="3" t="inlineStr">
@@ -16679,12 +16702,12 @@
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-02</t>
+          <t>E2E-R1-UI-01</t>
         </is>
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>Wrong password and wrong code produce clear, non-revealing messages (role=alert); axe clean | docs/06 §3, WCAG 3.3.1</t>
+          <t>Sign in through the browser (password + recovery code) lands on Home; navigation is permission-shaped with the current page marked; axe clean on sign-in and Home; reload keeps the session | docs/05 §2.1, §3.1, WCAG 2.2 AA</t>
         </is>
       </c>
       <c r="D246" s="3" t="inlineStr">
@@ -16706,12 +16729,12 @@
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-03</t>
+          <t>E2E-R1-UI-02</t>
         </is>
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>With several workspaces the chooser appears; choosing one and switching from the header changes the context and the navigation (no Admin for a plain member) | docs/05 §2.1 workspace switcher</t>
+          <t>Wrong password and wrong code produce clear, non-revealing messages (role=alert); axe clean | docs/06 §3, WCAG 3.3.1</t>
         </is>
       </c>
       <c r="D247" s="3" t="inlineStr">
@@ -16733,12 +16756,12 @@
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-04</t>
+          <t>E2E-R1-UI-03</t>
         </is>
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>The bell announces the unread count; the inbox lists the "joined" notification; mark all as read | FR-N01</t>
+          <t>With several workspaces the chooser appears; choosing one and switching from the header changes the context and the navigation (no Admin for a plain member) | docs/05 §2.1 workspace switcher</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
@@ -16760,12 +16783,12 @@
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-05</t>
+          <t>E2E-R1-UI-04</t>
         </is>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>Sign out returns to sign-in; reloading stays signed out | docs/06 §3</t>
+          <t>The bell announces the unread count; the inbox lists the "joined" notification; mark all as read | FR-N01</t>
         </is>
       </c>
       <c r="D249" s="3" t="inlineStr">
@@ -16787,12 +16810,12 @@
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-06</t>
+          <t>E2E-R1-UI-05</t>
         </is>
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>Theme switched from the account menu persists across reload; dark theme passes axe | docs/05 §7, WCAG 2.2 AA</t>
+          <t>Sign out returns to sign-in; reloading stays signed out | docs/06 §3</t>
         </is>
       </c>
       <c r="D250" s="3" t="inlineStr">
@@ -16814,12 +16837,12 @@
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-07</t>
+          <t>E2E-R1-UI-06</t>
         </is>
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>Author a policy in the browser: New document dialog → write content (headings, lists) → save → submit → publish; the library row shows Published; axe clean | FR-G04, docs/05 §3.2/§3.21</t>
+          <t>Theme switched from the account menu persists across reload; dark theme passes axe | docs/05 §7, WCAG 2.2 AA</t>
         </is>
       </c>
       <c r="D251" s="3" t="inlineStr">
@@ -16841,12 +16864,12 @@
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-08</t>
+          <t>E2E-R1-UI-07</t>
         </is>
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>A campaign task on Home leads to the document; “I acknowledge” records the acknowledgement (campaign progress +1) and the callout disappears | FR-AK01, docs/05 §3.1</t>
+          <t>Author a policy in the browser: New document dialog → write content (headings, lists) → save → submit → publish; the library row shows Published; axe clean | FR-G04, docs/05 §3.2/§3.21</t>
         </is>
       </c>
       <c r="D252" s="3" t="inlineStr">
@@ -16868,12 +16891,12 @@
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-09</t>
+          <t>E2E-R1-UI-08</t>
         </is>
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>Invite a colleague from Members with a role; the invitation appears in the table as Invited | FR-W01, docs/05 §3.14</t>
+          <t>A campaign task on Home leads to the document; “I acknowledge” records the acknowledgement (campaign progress +1) and the callout disappears | FR-AK01, docs/05 §3.1</t>
         </is>
       </c>
       <c r="D253" s="3" t="inlineStr">
@@ -16895,12 +16918,12 @@
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-10</t>
+          <t>E2E-R1-UI-09</t>
         </is>
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>Read and acknowledge a critical, pinned announcement in the feed | FR-AN04, docs/05 §3.23</t>
+          <t>Invite a colleague from Members with a role; the invitation appears in the table as Invited | FR-W01, docs/05 §3.14</t>
         </is>
       </c>
       <c r="D254" s="3" t="inlineStr">
@@ -16922,12 +16945,12 @@
       </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-11</t>
+          <t>E2E-R1-UI-10</t>
         </is>
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>An admin without two-step verification is guided through setup (QR + key, confirm a code, recovery codes) and then signs in with MFA and lands on Home | docs/06 §3, docs/20 §2.3</t>
+          <t>Read and acknowledge a critical, pinned announcement in the feed | FR-AN04, docs/05 §3.23</t>
         </is>
       </c>
       <c r="D255" s="3" t="inlineStr">
@@ -16949,12 +16972,12 @@
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-12</t>
+          <t>E2E-R1-UI-11</t>
         </is>
       </c>
       <c r="C256" s="3" t="inlineStr">
         <is>
-          <t>⌘K finds a document by its content and opens it; commands navigate; recent items are offered; keyboard only | BPMS-031, BPMS-049</t>
+          <t>An admin without two-step verification is guided through setup (QR + key, confirm a code, recovery codes) and then signs in with MFA and lands on Home | docs/06 §3, docs/20 §2.3</t>
         </is>
       </c>
       <c r="D256" s="3" t="inlineStr">
@@ -16976,12 +16999,12 @@
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-13</t>
+          <t>E2E-R1-UI-12</t>
         </is>
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>A new workspace shows composed empty states; an unknown page offers a way back; a failed load shows the error with a retry | BPMS-031 (UX-005)</t>
+          <t>⌘K finds a document by its content and opens it; commands navigate; recent items are offered; keyboard only | BPMS-031, BPMS-049</t>
         </is>
       </c>
       <c r="D257" s="3" t="inlineStr">
@@ -17003,12 +17026,12 @@
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-14</t>
+          <t>E2E-R1-UI-13</t>
         </is>
       </c>
       <c r="C258" s="3" t="inlineStr">
         <is>
-          <t>Manage announcements: compose a draft; a workspace-wide post is sent for approval; a targeted draft is published and shows receipts | BPMS-031, BPMS-047</t>
+          <t>A new workspace shows composed empty states; an unknown page offers a way back; a failed load shows the error with a retry | BPMS-031 (UX-005)</t>
         </is>
       </c>
       <c r="D258" s="3" t="inlineStr">
@@ -17030,12 +17053,12 @@
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-15</t>
+          <t>E2E-R1-UI-14</t>
         </is>
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>Campaigns: create from a published document with an audience, check the reach, launch, follow progress, download the evidence CSV | BPMS-031, BPMS-046</t>
+          <t>Manage announcements: compose a draft; a workspace-wide post is sent for approval; a targeted draft is published and shows receipts | BPMS-031, BPMS-047</t>
         </is>
       </c>
       <c r="D259" s="3" t="inlineStr">
@@ -17057,12 +17080,12 @@
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-16</t>
+          <t>E2E-R1-UI-15</t>
         </is>
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
-          <t>Settings: change a value in place with a reason and see why it applies; a step-up key asks to confirm identity | BPMS-031, BPMS-027</t>
+          <t>Campaigns: create from a published document with an audience, check the reach, launch, follow progress, download the evidence CSV | BPMS-031, BPMS-046</t>
         </is>
       </c>
       <c r="D260" s="3" t="inlineStr">
@@ -17084,12 +17107,12 @@
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-17</t>
+          <t>E2E-R1-UI-16</t>
         </is>
       </c>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>Audit log: chain verified; filter by category; expand a record; open an object timeline; no-match state | BPMS-031, BPMS-064</t>
+          <t>Settings: change a value in place with a reason and see why it applies; a step-up key asks to confirm identity | BPMS-031, BPMS-027</t>
         </is>
       </c>
       <c r="D261" s="3" t="inlineStr">
@@ -17111,12 +17134,12 @@
       </c>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-18</t>
+          <t>E2E-R1-UI-17</t>
         </is>
       </c>
       <c r="C262" s="3" t="inlineStr">
         <is>
-          <t>The owner sets a review schedule, recertifies when it falls due, verifies and removes verification | BPMS-044</t>
+          <t>Audit log: chain verified; filter by category; expand a record; open an object timeline; no-match state | BPMS-031, BPMS-064</t>
         </is>
       </c>
       <c r="D262" s="3" t="inlineStr">
@@ -17138,12 +17161,12 @@
       </c>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-19</t>
+          <t>E2E-R1-UI-18</t>
         </is>
       </c>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>A member suggests a change; the owner accepts it and marks it implemented in v2 | BPMS-044</t>
+          <t>The owner sets a review schedule, recertifies when it falls due, verifies and removes verification | BPMS-044</t>
         </is>
       </c>
       <c r="D263" s="3" t="inlineStr">
@@ -17165,12 +17188,12 @@
       </c>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-20</t>
+          <t>E2E-R1-UI-19</t>
         </is>
       </c>
       <c r="C264" s="3" t="inlineStr">
         <is>
-          <t>Compare v1 and v2 from the version history: word-level changes and the summary | BPMS-043</t>
+          <t>A member suggests a change; the owner accepts it and marks it implemented in v2 | BPMS-044</t>
         </is>
       </c>
       <c r="D264" s="3" t="inlineStr">
@@ -17192,12 +17215,12 @@
       </c>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-21</t>
+          <t>E2E-R1-UI-20</t>
         </is>
       </c>
       <c r="C265" s="3" t="inlineStr">
         <is>
-          <t>A member opens Policies, filters by category and follows "what changed" to the comparison | BPMS-045</t>
+          <t>Compare v1 and v2 from the version history: word-level changes and the summary | BPMS-043</t>
         </is>
       </c>
       <c r="D265" s="3" t="inlineStr">
@@ -17219,12 +17242,12 @@
       </c>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-22</t>
+          <t>E2E-R1-UI-21</t>
         </is>
       </c>
       <c r="C266" s="3" t="inlineStr">
         <is>
-          <t>A publisher restricts a policy to a role; a member outside it can't find it in Policies or open it | BPMS-045, A-14</t>
+          <t>A member opens Policies, filters by category and follows "what changed" to the comparison | BPMS-045</t>
         </is>
       </c>
       <c r="D266" s="3" t="inlineStr">
@@ -17246,12 +17269,12 @@
       </c>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-23</t>
+          <t>E2E-R1-UI-22</t>
         </is>
       </c>
       <c r="C267" s="3" t="inlineStr">
         <is>
-          <t>An admin opens Overview: the summary and "Needs attention" show overdue acknowledgements, and the security strip shows one member without two-step verification; drilling in opens People &amp; access filtered to them; the Admins filter shows the owner | BPMS-063</t>
+          <t>A publisher restricts a policy to a role; a member outside it can't find it in Policies or open it | BPMS-045, A-14</t>
         </is>
       </c>
       <c r="D267" s="3" t="inlineStr">
@@ -17273,12 +17296,12 @@
       </c>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-24</t>
+          <t>E2E-R1-UI-23</t>
         </is>
       </c>
       <c r="C268" s="3" t="inlineStr">
         <is>
-          <t>An owner publishes v2 as a major change, sees who will be asked, then finds the campaign | BPMS-045</t>
+          <t>An admin opens Overview: the summary and "Needs attention" show overdue acknowledgements, and the security strip shows one member without two-step verification; drilling in opens People &amp; access filtered to them; the Admins filter shows the owner | BPMS-063</t>
         </is>
       </c>
       <c r="D268" s="3" t="inlineStr">
@@ -17300,12 +17323,12 @@
       </c>
       <c r="B269" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-25</t>
+          <t>E2E-R1-UI-24</t>
         </is>
       </c>
       <c r="C269" s="3" t="inlineStr">
         <is>
-          <t>A member opens Notifications → Preferences, picks a daily digest and quiet hours, saves, sees them after a reload, and resets to the workspace defaults | BPMS-048</t>
+          <t>An owner publishes v2 as a major change, sees who will be asked, then finds the campaign | BPMS-045</t>
         </is>
       </c>
       <c r="D269" s="3" t="inlineStr">
@@ -17327,12 +17350,12 @@
       </c>
       <c r="B270" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-26</t>
+          <t>E2E-R1-UI-25</t>
         </is>
       </c>
       <c r="C270" s="3" t="inlineStr">
         <is>
-          <t>An admin opens Retention, sees each record class and a draft due for deletion, and shortens the draft period with a reason | BPMS-066</t>
+          <t>A member opens Notifications → Preferences, picks a daily digest and quiet hours, saves, sees them after a reload, and resets to the workspace defaults | BPMS-048</t>
         </is>
       </c>
       <c r="D270" s="3" t="inlineStr">
@@ -17354,12 +17377,12 @@
       </c>
       <c r="B271" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-27</t>
+          <t>E2E-R1-UI-26</t>
         </is>
       </c>
       <c r="C271" s="3" t="inlineStr">
         <is>
-          <t>An admin creates a collection from the Library rail, files a document in it from the document page, sets the accountable person in RACI, and filters the Library by the collection | BPMS-041</t>
+          <t>An admin opens Retention, sees each record class and a draft due for deletion, and shortens the draft period with a reason | BPMS-066</t>
         </is>
       </c>
       <c r="D271" s="3" t="inlineStr">
@@ -17381,12 +17404,12 @@
       </c>
       <c r="B272" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-28</t>
+          <t>E2E-R1-UI-27</t>
         </is>
       </c>
       <c r="C272" s="3" t="inlineStr">
         <is>
-          <t>An author uses the editor toolbar (bold, numbered steps, callout, table), saves, and the document renders them; the stored blocks match; axe on the editor and the result. UI-07 types markdown shortcuts into the editor | BPMS-042</t>
+          <t>An admin creates a collection from the Library rail, files a document in it from the document page, sets the accountable person in RACI, and filters the Library by the collection | BPMS-041</t>
         </is>
       </c>
       <c r="D272" s="3" t="inlineStr">
@@ -17408,12 +17431,12 @@
       </c>
       <c r="B273" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-29</t>
+          <t>E2E-R1-UI-28</t>
         </is>
       </c>
       <c r="C273" s="3" t="inlineStr">
         <is>
-          <t>An admin opens Encryption, sees version 1 in use, rotates the key with a reason, and sees version 2 in use | BPMS-030</t>
+          <t>An author uses the editor toolbar (bold, numbered steps, callout, table), saves, and the document renders them; the stored blocks match; axe on the editor and the result. UI-07 types markdown shortcuts into the editor | BPMS-042</t>
         </is>
       </c>
       <c r="D273" s="3" t="inlineStr">
@@ -17435,12 +17458,12 @@
       </c>
       <c r="B274" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-32</t>
+          <t>E2E-R1-UI-29</t>
         </is>
       </c>
       <c r="C274" s="3" t="inlineStr">
         <is>
-          <t>An author attaches a file to a draft from the document page, sees it clean, and downloads it | BPMS-060</t>
+          <t>An admin opens Encryption, sees version 1 in use, rotates the key with a reason, and sees version 2 in use | BPMS-030</t>
         </is>
       </c>
       <c r="D274" s="3" t="inlineStr">
@@ -17462,12 +17485,12 @@
       </c>
       <c r="B275" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-33</t>
+          <t>E2E-R1-UI-32</t>
         </is>
       </c>
       <c r="C275" s="3" t="inlineStr">
         <is>
-          <t>An EICAR upload on a document is refused with a quarantine message and shows as Quarantined (no download) in the Files view | BPMS-060/062</t>
+          <t>An author attaches a file to a draft from the document page, sees it clean, and downloads it | BPMS-060</t>
         </is>
       </c>
       <c r="D275" s="3" t="inlineStr">
@@ -17489,12 +17512,12 @@
       </c>
       <c r="B276" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-34</t>
+          <t>E2E-R1-UI-33</t>
         </is>
       </c>
       <c r="C276" s="3" t="inlineStr">
         <is>
-          <t>An author opens Preview on an image attachment: a dialog named after the file shows the image (axe clean); a text attachment offers no Preview; Escape closes it and focus returns | BPMS-061</t>
+          <t>An EICAR upload on a document is refused with a quarantine message and shows as Quarantined (no download) in the Files view | BPMS-060/062</t>
         </is>
       </c>
       <c r="D276" s="3" t="inlineStr">
@@ -17516,12 +17539,12 @@
       </c>
       <c r="B277" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-38</t>
+          <t>E2E-R1-UI-34</t>
         </is>
       </c>
       <c r="C277" s="3" t="inlineStr">
         <is>
-          <t>On the Library grid: build a Status filter (chip + count), sort by name descending, save the view, reload and get the same filter and order back with no modified marker, export a CSV with exactly the visible columns and rows | BPMS-028</t>
+          <t>An author opens Preview on an image attachment: a dialog named after the file shows the image (axe clean); a text attachment offers no Preview; Escape closes it and focus returns | BPMS-061</t>
         </is>
       </c>
       <c r="D277" s="3" t="inlineStr">
@@ -17543,12 +17566,12 @@
       </c>
       <c r="B278" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-39</t>
+          <t>E2E-R1-UI-38</t>
         </is>
       </c>
       <c r="C278" s="3" t="inlineStr">
         <is>
-          <t>An admin filters the Audit log to content events, starts a background export (dialog says it uses the current filters), sees it become Ready in Your exports, and downloads the CSV | BPMS-064</t>
+          <t>On the Library grid: build a Status filter (chip + count), sort by name descending, save the view, reload and get the same filter and order back with no modified marker, export a CSV with exactly the visible columns and rows | BPMS-028</t>
         </is>
       </c>
       <c r="D278" s="3" t="inlineStr">
@@ -17570,12 +17593,12 @@
       </c>
       <c r="B279" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-30</t>
+          <t>E2E-R1-UI-39</t>
         </is>
       </c>
       <c r="C279" s="3" t="inlineStr">
         <is>
-          <t>Add a passkey from Account › Security, sign out, sign in with password + passkey | BPMS-022</t>
+          <t>An admin filters the Audit log to content events, starts a background export (dialog says it uses the current filters), sees it become Ready in Your exports, and downloads the CSV | BPMS-064</t>
         </is>
       </c>
       <c r="D279" s="3" t="inlineStr">
@@ -17597,12 +17620,12 @@
       </c>
       <c r="B280" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-31</t>
+          <t>E2E-R1-UI-30</t>
         </is>
       </c>
       <c r="C280" s="3" t="inlineStr">
         <is>
-          <t>Removing a passkey asks to confirm it’s you; the passkey itself passes step-up | BPMS-022</t>
+          <t>Add a passkey from Account › Security, sign out, sign in with password + passkey | BPMS-022</t>
         </is>
       </c>
       <c r="D280" s="3" t="inlineStr">
@@ -17624,12 +17647,12 @@
       </c>
       <c r="B281" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-35</t>
+          <t>E2E-R1-UI-31</t>
         </is>
       </c>
       <c r="C281" s="3" t="inlineStr">
         <is>
-          <t>Departments: override a setting for a parent department, see a child inherit it, then clear it | BPMS-027</t>
+          <t>Removing a passkey asks to confirm it’s you; the passkey itself passes step-up | BPMS-022</t>
         </is>
       </c>
       <c r="D281" s="3" t="inlineStr">
@@ -17651,12 +17674,12 @@
       </c>
       <c r="B282" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-36</t>
+          <t>E2E-R1-UI-35</t>
         </is>
       </c>
       <c r="C282" s="3" t="inlineStr">
         <is>
-          <t>Configuration profile: preview a switch with every change, then switch with a reason | BPMS-027, CFG-017</t>
+          <t>Departments: override a setting for a parent department, see a child inherit it, then clear it | BPMS-027</t>
         </is>
       </c>
       <c r="D282" s="3" t="inlineStr">
@@ -17678,12 +17701,12 @@
       </c>
       <c r="B283" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-40</t>
+          <t>E2E-R1-UI-36</t>
         </is>
       </c>
       <c r="C283" s="3" t="inlineStr">
         <is>
-          <t>A system admin finds a workspace, makes it read-only with a reason, and reactivates it | BPMS-065</t>
+          <t>Configuration profile: preview a switch with every change, then switch with a reason | BPMS-027, CFG-017</t>
         </is>
       </c>
       <c r="D283" s="3" t="inlineStr">
@@ -17705,12 +17728,12 @@
       </c>
       <c r="B284" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-41</t>
+          <t>E2E-R1-UI-40</t>
         </is>
       </c>
       <c r="C284" s="3" t="inlineStr">
         <is>
-          <t>Quotas, platform health and the system audit; non-system users never see the console | BPMS-065</t>
+          <t>A system admin finds a workspace, makes it read-only with a reason, and reactivates it | BPMS-065</t>
         </is>
       </c>
       <c r="D284" s="3" t="inlineStr">
@@ -17732,12 +17755,12 @@
       </c>
       <c r="B285" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-42</t>
+          <t>E2E-R1-UI-41</t>
         </is>
       </c>
       <c r="C285" s="3" t="inlineStr">
         <is>
-          <t>With the API slowed down, every main page (Home, Library, Members, Campaigns, Manage announcements, Overview, People &amp; access, Settings, Audit log, Notifications) shows a content-shaped skeleton, then its content; a reload shows the app frame, never a blank page | UX-005</t>
+          <t>Quotas, platform health and the system audit; non-system users never see the console | BPMS-065</t>
         </is>
       </c>
       <c r="D285" s="3" t="inlineStr">
@@ -17759,12 +17782,12 @@
       </c>
       <c r="B286" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-43</t>
+          <t>E2E-R1-UI-42</t>
         </is>
       </c>
       <c r="C286" s="3" t="inlineStr">
         <is>
-          <t>Files: a draft attachment shows retention class Draft and last accessed Never; downloading it updates last accessed; two unattached files are selected and deleted in bulk | BPMS-062</t>
+          <t>With the API slowed down, every main page (Home, Library, Members, Campaigns, Manage announcements, Overview, People &amp; access, Settings, Audit log, Notifications) shows a content-shaped skeleton, then its content; a reload shows the app frame, never a blank page | UX-005</t>
         </is>
       </c>
       <c r="D286" s="3" t="inlineStr">
@@ -17786,12 +17809,12 @@
       </c>
       <c r="B287" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-UI-44</t>
+          <t>E2E-R1-UI-43</t>
         </is>
       </c>
       <c r="C287" s="3" t="inlineStr">
         <is>
-          <t>A reader opens Export on a published SOP (Print or PDF, Word, Markdown) and downloads a .docx | BPMS-042</t>
+          <t>Files: a draft attachment shows retention class Draft and last accessed Never; downloading it updates last accessed; two unattached files are selected and deleted in bulk | BPMS-062</t>
         </is>
       </c>
       <c r="D287" s="3" t="inlineStr">
@@ -17813,12 +17836,12 @@
       </c>
       <c r="B288" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-01</t>
+          <t>E2E-R1-UI-44</t>
         </is>
       </c>
       <c r="C288" s="3" t="inlineStr">
         <is>
-          <t>Onboarding start to finish: the owner invites from Members; the invitee opens the link from the email, creates an account (password confirmation checked) and lands on Home in the workspace; the link then no longer works; the owner sees them Active and opens their person page | BPMS-023</t>
+          <t>A reader opens Export on a published SOP (Print or PDF, Word, Markdown) and downloads a .docx | BPMS-042</t>
         </is>
       </c>
       <c r="D288" s="3" t="inlineStr">
@@ -17840,12 +17863,12 @@
       </c>
       <c r="B289" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-02</t>
+          <t>E2E-R1-UI-45</t>
         </is>
       </c>
       <c r="C289" s="3" t="inlineStr">
         <is>
-          <t>Someone with an account opens the invitation email, signs in from the page, comes back to it and joins with one click; an unknown link explains itself | BPMS-023</t>
+          <t>An author inserts an image from the editor (upload, required description, caption), saves, and readers see it with its alt text after a reload | BPMS-042</t>
         </is>
       </c>
       <c r="D289" s="3" t="inlineStr">
@@ -17867,12 +17890,12 @@
       </c>
       <c r="B290" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-03</t>
+          <t>E2E-R1-FLOW-01</t>
         </is>
       </c>
       <c r="C290" s="3" t="inlineStr">
         <is>
-          <t>Policy to evidence: the owner writes and publishes a policy and launches a campaign; a colleague (invited the same way) sees the task on Home, opens the acknowledgement email link, acknowledges on the document; the owner sees them Done, 1 of 2, and downloads the evidence CSV | BPMS-040, 046</t>
+          <t>Onboarding start to finish: the owner invites from Members; the invitee opens the link from the email, creates an account (password confirmation checked) and lands on Home in the workspace; the link then no longer works; the owner sees them Active and opens their person page | BPMS-023</t>
         </is>
       </c>
       <c r="D290" s="3" t="inlineStr">
@@ -17894,12 +17917,12 @@
       </c>
       <c r="B291" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-04</t>
+          <t>E2E-R1-FLOW-02</t>
         </is>
       </c>
       <c r="C291" s="3" t="inlineStr">
         <is>
-          <t>Announcement: the owner composes a critical post that needs acknowledgement and publishes it; a colleague opens the email link while signed out, signs in, lands on the open post and confirms; the owner sees the receipt | BPMS-047</t>
+          <t>Someone with an account opens the invitation email, signs in from the page, comes back to it and joins with one click; an unknown link explains itself | BPMS-023</t>
         </is>
       </c>
       <c r="D291" s="3" t="inlineStr">
@@ -17921,12 +17944,12 @@
       </c>
       <c r="B292" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-05</t>
+          <t>E2E-R1-FLOW-03</t>
         </is>
       </c>
       <c r="C292" s="3" t="inlineStr">
         <is>
-          <t>Review loop: the owner submits a controlled policy; the reviewer (invited as Reviewer) gets the review email, opens it and requests changes with a comment; the owner gets a notification quoting it, edits and resubmits; the reviewer approves from Home; the owner is told it is approved and publishes | BPMS-040</t>
+          <t>Policy to evidence: the owner writes and publishes a policy and launches a campaign; a colleague (invited the same way) sees the task on Home, opens the acknowledgement email link, acknowledges on the document; the owner sees them Done, 1 of 2, and downloads the evidence CSV | BPMS-040, 046</t>
         </is>
       </c>
       <c r="D292" s="3" t="inlineStr">
@@ -17948,12 +17971,12 @@
       </c>
       <c r="B293" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-06</t>
+          <t>E2E-R1-FLOW-04</t>
         </is>
       </c>
       <c r="C293" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval: a second admin joins from the invitation and turns on two-step verification; the owner sends a workspace-wide post for approval; the admin gets the approval email, opens it and sends it back with a note; the owner gets a notification with the note, edits and resubmits; the admin approves and publishes; the owner is told; the post is in the feed | BPMS-047</t>
+          <t>Announcement: the owner composes a critical post that needs acknowledgement and publishes it; a colleague opens the email link while signed out, signs in, lands on the open post and confirms; the owner sees the receipt | BPMS-047</t>
         </is>
       </c>
       <c r="D293" s="3" t="inlineStr">
@@ -17975,12 +17998,12 @@
       </c>
       <c r="B294" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-01</t>
+          <t>E2E-R1-FLOW-05</t>
         </is>
       </c>
       <c r="C294" s="3" t="inlineStr">
         <is>
-          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
+          <t>Review loop: the owner submits a controlled policy; the reviewer (invited as Reviewer) gets the review email, opens it and requests changes with a comment; the owner gets a notification quoting it, edits and resubmits; the reviewer approves from Home; the owner is told it is approved and publishes | BPMS-040</t>
         </is>
       </c>
       <c r="D294" s="3" t="inlineStr">
@@ -18002,12 +18025,12 @@
       </c>
       <c r="B295" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-02</t>
+          <t>E2E-R1-FLOW-06</t>
         </is>
       </c>
       <c r="C295" s="3" t="inlineStr">
         <is>
-          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
+          <t>Announcement approval: a second admin joins from the invitation and turns on two-step verification; the owner sends a workspace-wide post for approval; the admin gets the approval email, opens it and sends it back with a note; the owner gets a notification with the note, edits and resubmits; the admin approves and publishes; the owner is told; the post is in the feed | BPMS-047</t>
         </is>
       </c>
       <c r="D295" s="3" t="inlineStr">
@@ -18029,12 +18052,12 @@
       </c>
       <c r="B296" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-03</t>
+          <t>E2E-R1-CMP-01</t>
         </is>
       </c>
       <c r="C296" s="3" t="inlineStr">
         <is>
-          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
+          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
         </is>
       </c>
       <c r="D296" s="3" t="inlineStr">
@@ -18056,12 +18079,12 @@
       </c>
       <c r="B297" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-04</t>
+          <t>E2E-R1-CMP-02</t>
         </is>
       </c>
       <c r="C297" s="3" t="inlineStr">
         <is>
-          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
+          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
         </is>
       </c>
       <c r="D297" s="3" t="inlineStr">
@@ -18083,12 +18106,12 @@
       </c>
       <c r="B298" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-05</t>
+          <t>E2E-R1-CMP-03</t>
         </is>
       </c>
       <c r="C298" s="3" t="inlineStr">
         <is>
-          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
+          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
         </is>
       </c>
       <c r="D298" s="3" t="inlineStr">
@@ -18110,12 +18133,12 @@
       </c>
       <c r="B299" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-06</t>
+          <t>E2E-R1-CMP-04</t>
         </is>
       </c>
       <c r="C299" s="3" t="inlineStr">
         <is>
-          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
+          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
         </is>
       </c>
       <c r="D299" s="3" t="inlineStr">
@@ -18137,12 +18160,12 @@
       </c>
       <c r="B300" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-07</t>
+          <t>E2E-R1-CMP-05</t>
         </is>
       </c>
       <c r="C300" s="3" t="inlineStr">
         <is>
-          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
+          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
         </is>
       </c>
       <c r="D300" s="3" t="inlineStr">
@@ -18164,12 +18187,12 @@
       </c>
       <c r="B301" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-01</t>
+          <t>E2E-R1-CMP-06</t>
         </is>
       </c>
       <c r="C301" s="3" t="inlineStr">
         <is>
-          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
+          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
         </is>
       </c>
       <c r="D301" s="3" t="inlineStr">
@@ -18191,12 +18214,12 @@
       </c>
       <c r="B302" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-02</t>
+          <t>E2E-R1-CMP-07</t>
         </is>
       </c>
       <c r="C302" s="3" t="inlineStr">
         <is>
-          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
+          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D302" s="3" t="inlineStr">
@@ -18218,12 +18241,12 @@
       </c>
       <c r="B303" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-03</t>
+          <t>E2E-R1-ANN-01</t>
         </is>
       </c>
       <c r="C303" s="3" t="inlineStr">
         <is>
-          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
+          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
         </is>
       </c>
       <c r="D303" s="3" t="inlineStr">
@@ -18245,12 +18268,12 @@
       </c>
       <c r="B304" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-04</t>
+          <t>E2E-R1-ANN-02</t>
         </is>
       </c>
       <c r="C304" s="3" t="inlineStr">
         <is>
-          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
+          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
         </is>
       </c>
       <c r="D304" s="3" t="inlineStr">
@@ -18272,12 +18295,12 @@
       </c>
       <c r="B305" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-05</t>
+          <t>E2E-R1-ANN-03</t>
         </is>
       </c>
       <c r="C305" s="3" t="inlineStr">
         <is>
-          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
+          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
         </is>
       </c>
       <c r="D305" s="3" t="inlineStr">
@@ -18299,12 +18322,12 @@
       </c>
       <c r="B306" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-06</t>
+          <t>E2E-R1-ANN-04</t>
         </is>
       </c>
       <c r="C306" s="3" t="inlineStr">
         <is>
-          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
+          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
         </is>
       </c>
       <c r="D306" s="3" t="inlineStr">
@@ -18326,12 +18349,12 @@
       </c>
       <c r="B307" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-01</t>
+          <t>E2E-R1-ANN-05</t>
         </is>
       </c>
       <c r="C307" s="3" t="inlineStr">
         <is>
-          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
+          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D307" s="3" t="inlineStr">
@@ -18353,12 +18376,12 @@
       </c>
       <c r="B308" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-02</t>
+          <t>E2E-R1-ANN-06</t>
         </is>
       </c>
       <c r="C308" s="3" t="inlineStr">
         <is>
-          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
+          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
         </is>
       </c>
       <c r="D308" s="3" t="inlineStr">
@@ -18380,12 +18403,12 @@
       </c>
       <c r="B309" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-03</t>
+          <t>E2E-R1-SRCH-01</t>
         </is>
       </c>
       <c r="C309" s="3" t="inlineStr">
         <is>
-          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
+          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
         </is>
       </c>
       <c r="D309" s="3" t="inlineStr">
@@ -18407,12 +18430,12 @@
       </c>
       <c r="B310" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-01</t>
+          <t>E2E-R1-SRCH-02</t>
         </is>
       </c>
       <c r="C310" s="3" t="inlineStr">
         <is>
-          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
+          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
         </is>
       </c>
       <c r="D310" s="3" t="inlineStr">
@@ -18434,12 +18457,12 @@
       </c>
       <c r="B311" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-02</t>
+          <t>E2E-R1-SRCH-03</t>
         </is>
       </c>
       <c r="C311" s="3" t="inlineStr">
         <is>
-          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
+          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
         </is>
       </c>
       <c r="D311" s="3" t="inlineStr">
@@ -18461,12 +18484,12 @@
       </c>
       <c r="B312" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-03</t>
+          <t>E2E-R1-AUDX-01</t>
         </is>
       </c>
       <c r="C312" s="3" t="inlineStr">
         <is>
-          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
+          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
         </is>
       </c>
       <c r="D312" s="3" t="inlineStr">
@@ -18488,12 +18511,12 @@
       </c>
       <c r="B313" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-04</t>
+          <t>E2E-R1-AUDX-02</t>
         </is>
       </c>
       <c r="C313" s="3" t="inlineStr">
         <is>
-          <t>Chain verify reports intact | FR-T02</t>
+          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
         </is>
       </c>
       <c r="D313" s="3" t="inlineStr">
@@ -18515,12 +18538,12 @@
       </c>
       <c r="B314" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-05</t>
+          <t>E2E-R1-AUDX-03</t>
         </is>
       </c>
       <c r="C314" s="3" t="inlineStr">
         <is>
-          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
+          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
         </is>
       </c>
       <c r="D314" s="3" t="inlineStr">
@@ -18542,12 +18565,12 @@
       </c>
       <c r="B315" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-06</t>
+          <t>E2E-R1-AUDX-04</t>
         </is>
       </c>
       <c r="C315" s="3" t="inlineStr">
         <is>
-          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
+          <t>Chain verify reports intact | FR-T02</t>
         </is>
       </c>
       <c r="D315" s="3" t="inlineStr">
@@ -18569,12 +18592,12 @@
       </c>
       <c r="B316" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-07</t>
+          <t>E2E-R1-AUDX-05</t>
         </is>
       </c>
       <c r="C316" s="3" t="inlineStr">
         <is>
-          <t>`POST /audit/query`: an AND group (category, action prefix, within P30D) sorted ascending pages by cursor; an OR group returns only matching events; unknown fields or values, bad durations, nesting deeper than 2 and unsupported sorts → 422 | BPMS-064, docs/08 §7.5</t>
+          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
         </is>
       </c>
       <c r="D316" s="3" t="inlineStr">
@@ -18596,12 +18619,12 @@
       </c>
       <c r="B317" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-08</t>
+          <t>E2E-R1-AUDX-06</t>
         </is>
       </c>
       <c r="C317" s="3" t="inlineStr">
         <is>
-          <t>A background export (202) runs as a job, finishes `done` with rows, its CSV downloads through the requester's signed file link, the requester is notified, and both `audit.export_requested` and `audit.exported` are recorded | BPMS-064, FR-T04</t>
+          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
         </is>
       </c>
       <c r="D317" s="3" t="inlineStr">
@@ -18623,12 +18646,12 @@
       </c>
       <c r="B318" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-AUDX-07</t>
         </is>
       </c>
       <c r="C318" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>`POST /audit/query`: an AND group (category, action prefix, within P30D) sorted ascending pages by cursor; an OR group returns only matching events; unknown fields or values, bad durations, nesting deeper than 2 and unsupported sorts → 422 | BPMS-064, docs/08 §7.5</t>
         </is>
       </c>
       <c r="D318" s="3" t="inlineStr">
@@ -18650,12 +18673,12 @@
       </c>
       <c r="B319" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-AUDX-08</t>
         </is>
       </c>
       <c r="C319" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>A background export (202) runs as a job, finishes `done` with rows, its CSV downloads through the requester's signed file link, the requester is notified, and both `audit.export_requested` and `audit.exported` are recorded | BPMS-064, FR-T04</t>
         </is>
       </c>
       <c r="D319" s="3" t="inlineStr">
@@ -18677,12 +18700,12 @@
       </c>
       <c r="B320" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C320" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
         </is>
       </c>
       <c r="D320" s="3" t="inlineStr">
@@ -18704,12 +18727,12 @@
       </c>
       <c r="B321" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C321" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D321" s="3" t="inlineStr">
@@ -18731,12 +18754,12 @@
       </c>
       <c r="B322" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C322" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D322" s="3" t="inlineStr">
@@ -18758,12 +18781,12 @@
       </c>
       <c r="B323" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C323" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
         </is>
       </c>
       <c r="D323" s="3" t="inlineStr">
@@ -18785,12 +18808,12 @@
       </c>
       <c r="B324" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C324" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
         </is>
       </c>
       <c r="D324" s="3" t="inlineStr">
@@ -18812,12 +18835,12 @@
       </c>
       <c r="B325" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C325" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D325" s="3" t="inlineStr">
@@ -18839,12 +18862,12 @@
       </c>
       <c r="B326" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C326" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D326" s="3" t="inlineStr">
@@ -18866,12 +18889,12 @@
       </c>
       <c r="B327" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C327" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
         </is>
       </c>
       <c r="D327" s="3" t="inlineStr">
@@ -18893,12 +18916,12 @@
       </c>
       <c r="B328" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C328" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D328" s="3" t="inlineStr">
@@ -18920,12 +18943,12 @@
       </c>
       <c r="B329" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C329" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D329" s="3" t="inlineStr">
@@ -18947,12 +18970,12 @@
       </c>
       <c r="B330" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C330" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D330" s="3" t="inlineStr">
@@ -18974,12 +18997,12 @@
       </c>
       <c r="B331" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C331" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D331" s="3" t="inlineStr">
@@ -19001,12 +19024,12 @@
       </c>
       <c r="B332" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C332" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
         </is>
       </c>
       <c r="D332" s="3" t="inlineStr">
@@ -19028,12 +19051,12 @@
       </c>
       <c r="B333" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C333" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
         </is>
       </c>
       <c r="D333" s="3" t="inlineStr">
@@ -19055,12 +19078,12 @@
       </c>
       <c r="B334" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C334" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
         </is>
       </c>
       <c r="D334" s="3" t="inlineStr">
@@ -19082,12 +19105,12 @@
       </c>
       <c r="B335" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C335" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D335" s="3" t="inlineStr">
@@ -19109,12 +19132,12 @@
       </c>
       <c r="B336" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C336" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
         </is>
       </c>
       <c r="D336" s="3" t="inlineStr">
@@ -19136,12 +19159,12 @@
       </c>
       <c r="B337" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C337" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
         </is>
       </c>
       <c r="D337" s="3" t="inlineStr">
@@ -19163,12 +19186,12 @@
       </c>
       <c r="B338" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C338" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D338" s="3" t="inlineStr">
@@ -19190,12 +19213,12 @@
       </c>
       <c r="B339" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C339" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
         </is>
       </c>
       <c r="D339" s="3" t="inlineStr">
@@ -19217,12 +19240,12 @@
       </c>
       <c r="B340" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C340" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D340" s="3" t="inlineStr">
@@ -19244,12 +19267,12 @@
       </c>
       <c r="B341" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C341" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D341" s="3" t="inlineStr">
@@ -19271,12 +19294,12 @@
       </c>
       <c r="B342" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C342" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D342" s="3" t="inlineStr">
@@ -19298,12 +19321,12 @@
       </c>
       <c r="B343" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C343" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D343" s="3" t="inlineStr">
@@ -19325,12 +19348,12 @@
       </c>
       <c r="B344" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C344" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D344" s="3" t="inlineStr">
@@ -19352,12 +19375,12 @@
       </c>
       <c r="B345" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C345" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D345" s="3" t="inlineStr">
@@ -19379,12 +19402,12 @@
       </c>
       <c r="B346" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C346" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D346" s="3" t="inlineStr">
@@ -19406,12 +19429,12 @@
       </c>
       <c r="B347" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C347" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D347" s="3" t="inlineStr">
@@ -19433,12 +19456,12 @@
       </c>
       <c r="B348" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C348" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D348" s="3" t="inlineStr">
@@ -19460,12 +19483,12 @@
       </c>
       <c r="B349" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C349" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D349" s="3" t="inlineStr">
@@ -19487,12 +19510,12 @@
       </c>
       <c r="B350" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C350" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D350" s="3" t="inlineStr">
@@ -19514,12 +19537,12 @@
       </c>
       <c r="B351" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C351" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D351" s="3" t="inlineStr">
@@ -19541,12 +19564,12 @@
       </c>
       <c r="B352" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C352" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D352" s="3" t="inlineStr">
@@ -19568,12 +19591,12 @@
       </c>
       <c r="B353" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C353" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D353" s="3" t="inlineStr">
@@ -19595,12 +19618,12 @@
       </c>
       <c r="B354" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C354" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D354" s="3" t="inlineStr">
@@ -19622,12 +19645,12 @@
       </c>
       <c r="B355" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C355" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D355" s="3" t="inlineStr">
@@ -19649,12 +19672,12 @@
       </c>
       <c r="B356" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C356" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D356" s="3" t="inlineStr">
@@ -19676,12 +19699,12 @@
       </c>
       <c r="B357" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C357" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D357" s="3" t="inlineStr">
@@ -19703,12 +19726,12 @@
       </c>
       <c r="B358" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C358" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D358" s="3" t="inlineStr">
@@ -19730,12 +19753,12 @@
       </c>
       <c r="B359" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C359" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D359" s="3" t="inlineStr">
@@ -19757,12 +19780,12 @@
       </c>
       <c r="B360" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C360" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D360" s="3" t="inlineStr">
@@ -19784,12 +19807,12 @@
       </c>
       <c r="B361" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C361" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D361" s="3" t="inlineStr">
@@ -19811,12 +19834,12 @@
       </c>
       <c r="B362" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C362" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D362" s="3" t="inlineStr">
@@ -19838,12 +19861,12 @@
       </c>
       <c r="B363" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C363" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D363" s="3" t="inlineStr">
@@ -19865,12 +19888,12 @@
       </c>
       <c r="B364" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C364" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D364" s="3" t="inlineStr">
@@ -19892,12 +19915,12 @@
       </c>
       <c r="B365" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C365" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D365" s="3" t="inlineStr">
@@ -19919,12 +19942,12 @@
       </c>
       <c r="B366" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C366" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D366" s="3" t="inlineStr">
@@ -19946,12 +19969,12 @@
       </c>
       <c r="B367" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C367" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D367" s="3" t="inlineStr">
@@ -19973,12 +19996,12 @@
       </c>
       <c r="B368" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C368" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D368" s="3" t="inlineStr">
@@ -20000,12 +20023,12 @@
       </c>
       <c r="B369" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C369" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D369" s="3" t="inlineStr">
@@ -20027,12 +20050,12 @@
       </c>
       <c r="B370" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C370" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D370" s="3" t="inlineStr">
@@ -20054,12 +20077,12 @@
       </c>
       <c r="B371" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C371" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D371" s="3" t="inlineStr">
@@ -20081,12 +20104,12 @@
       </c>
       <c r="B372" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C372" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D372" s="3" t="inlineStr">
@@ -20108,12 +20131,12 @@
       </c>
       <c r="B373" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C373" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D373" s="3" t="inlineStr">
@@ -20135,12 +20158,12 @@
       </c>
       <c r="B374" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C374" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D374" s="3" t="inlineStr">
@@ -20162,12 +20185,12 @@
       </c>
       <c r="B375" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C375" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D375" s="3" t="inlineStr">
@@ -20189,12 +20212,12 @@
       </c>
       <c r="B376" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C376" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D376" s="3" t="inlineStr">
@@ -20216,12 +20239,12 @@
       </c>
       <c r="B377" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C377" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D377" s="3" t="inlineStr">
@@ -20243,12 +20266,12 @@
       </c>
       <c r="B378" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C378" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D378" s="3" t="inlineStr">
@@ -20270,12 +20293,12 @@
       </c>
       <c r="B379" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C379" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D379" s="3" t="inlineStr">
@@ -20297,12 +20320,12 @@
       </c>
       <c r="B380" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C380" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D380" s="3" t="inlineStr">
@@ -20324,12 +20347,12 @@
       </c>
       <c r="B381" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-11</t>
         </is>
       </c>
       <c r="C381" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
         </is>
       </c>
       <c r="D381" s="3" t="inlineStr">
@@ -20351,12 +20374,12 @@
       </c>
       <c r="B382" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R4-ISO</t>
         </is>
       </c>
       <c r="C382" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
         </is>
       </c>
       <c r="D382" s="3" t="inlineStr">
@@ -20378,12 +20401,12 @@
       </c>
       <c r="B383" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R5-01</t>
         </is>
       </c>
       <c r="C383" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
         </is>
       </c>
       <c r="D383" s="3" t="inlineStr">
@@ -20405,12 +20428,12 @@
       </c>
       <c r="B384" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R5-02</t>
         </is>
       </c>
       <c r="C384" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
         </is>
       </c>
       <c r="D384" s="3" t="inlineStr">
@@ -20432,12 +20455,12 @@
       </c>
       <c r="B385" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R5-03</t>
         </is>
       </c>
       <c r="C385" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
         </is>
       </c>
       <c r="D385" s="3" t="inlineStr">
@@ -20459,12 +20482,12 @@
       </c>
       <c r="B386" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R5-04</t>
         </is>
       </c>
       <c r="C386" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
         </is>
       </c>
       <c r="D386" s="3" t="inlineStr">
@@ -20486,12 +20509,12 @@
       </c>
       <c r="B387" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R5-05</t>
         </is>
       </c>
       <c r="C387" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
         </is>
       </c>
       <c r="D387" s="3" t="inlineStr">
@@ -20513,12 +20536,12 @@
       </c>
       <c r="B388" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R5-06</t>
         </is>
       </c>
       <c r="C388" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
         </is>
       </c>
       <c r="D388" s="3" t="inlineStr">
@@ -20540,12 +20563,12 @@
       </c>
       <c r="B389" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R5-07</t>
         </is>
       </c>
       <c r="C389" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
         </is>
       </c>
       <c r="D389" s="3" t="inlineStr">
@@ -20567,12 +20590,12 @@
       </c>
       <c r="B390" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R5-08</t>
         </is>
       </c>
       <c r="C390" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
         </is>
       </c>
       <c r="D390" s="3" t="inlineStr">
@@ -20594,20 +20617,74 @@
       </c>
       <c r="B391" s="3" t="inlineStr">
         <is>
+          <t>E2E-R5-09</t>
+        </is>
+      </c>
+      <c r="C391" s="3" t="inlineStr">
+        <is>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+        </is>
+      </c>
+      <c r="D391" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E391" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B392" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C392" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D392" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E392" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B393" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C391" s="3" t="inlineStr">
+      <c r="C393" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D391" s="3" t="inlineStr">
+      <c r="D393" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E391" s="3" t="inlineStr">
+      <c r="E393" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
docs: image-block assumption renumbered to A-30 (A-27..A-29 belong to BPMS-083)
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -2128,7 +2128,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>A-28 (BPMS-042)</t>
+          <t>A-30 (BPMS-042)</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -5330,7 +5330,7 @@
       <c r="N33" s="3" t="inlineStr"/>
       <c r="O33" s="3" t="inlineStr">
         <is>
-          <t>Block editor (TipTap core, MIT; U-10 closed): headings, bold/italic/links, bullet and numbered lists, callouts, tables, accessible single-tab-stop toolbar, markdown shortcuts; block model validated server-side (ADR-0013 as built); shared renderer; HTML (print to tagged PDF in the browser) and Markdown export with a superseded banner, audited. E2E-R1-LIB-14, E2E-R1-UI-07, 28. Word (.docx) export with heading styles, numbering, tables and links, reproducible bytes; Export menu. E2E-R1-UI-44. Image blocks (alt text required, attached clean images only, embedded in print HTML; A-28) inserted from the editor. E2E-R1-LIB-15, UI-45. Remaining: deterministic server-side tagged PDF, DOCX import, pictures inside DOCX, variables blocks.</t>
+          <t>Block editor (TipTap core, MIT; U-10 closed): headings, bold/italic/links, bullet and numbered lists, callouts, tables, accessible single-tab-stop toolbar, markdown shortcuts; block model validated server-side (ADR-0013 as built); shared renderer; HTML (print to tagged PDF in the browser) and Markdown export with a superseded banner, audited. E2E-R1-LIB-14, E2E-R1-UI-07, 28. Word (.docx) export with heading styles, numbering, tables and links, reproducible bytes; Export menu. E2E-R1-UI-44. Image blocks (alt text required, attached clean images only, embedded in print HTML; A-30) inserted from the editor. E2E-R1-LIB-15, UI-45. Remaining: deterministic server-side tagged PDF, DOCX import, pictures inside DOCX, variables blocks.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: tracker for BPMS-083 and the R1 gate tests
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -197,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E28" headerRowCount="1">
-  <autoFilter ref="A1:E28"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E31" headerRowCount="1">
+  <autoFilter ref="A1:E31"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Source"/>
     <tableColumn id="2" name="ID"/>
@@ -1393,7 +1393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2128,20 +2128,101 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
+          <t>A-27 (BPMS-083)</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Business calendars and durations (docs/04 §4.4 *As built*). (1) A calendar version's time zone is a fixed UTC offset (`+05:30`); IANA zone names are rejected until a zone database is added behind the calendar (A-22 (5)), so a DST region needs one version per offset period. (2) Working hours are `[start, end)` ranges per weekday in local time (`HH:MM`, up to `24:00`), ordered and non-overlapping; holidays are whole local dates; a calendar with no working time is invalid. (3) In a business duration the date part counts **working days**: `nD` lands at the same local time on the n-th next working day, after rolling a start outside working time forward to the next working instant, and a time the target day does not work is clamped into that day's hours; `nW` is n × the calendar's working weekdays (`P1W` = one working week). The time part (`H`, `M`, `S`) counts working time only. A zero duration is the identity. (4) A business timer or SLA whose calendar reference is not stored fails the advance (`calendar not found`); publish (BPMS-084) is expected to guarantee the reference. (5) A `calendar` on a node names a `refs.calendars` key; anything else is read as a calendar reference</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Runtime-lead and product-owner review; pilot calendars (E2E-R2-10, IN holidays)</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Count business days as fixed working-hour blocks (e.g. `P1D` = 8 working hours); add an IANA zone database; fall back to a 24×7 calendar instead of failing</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>A-28 (BPMS-083)</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Runtime persistence (docs/04 §4.2 and §4.4 *As built*). (1) `instance_events` stores the **stimuli** (the replay log); the interpreter trace stays inside the stored state until analytics needs it as rows. The table is not partitioned yet (docs/04 §2.5 says monthly partitions); partitioning follows the SP-10 volume check. (2) Every command is recorded once in `instance_effects` by `(key, command)`; commands owned by later items (work items, connector calls, signals, subprocesses, cases, incidents, notifications, SLA breach actions) are left `pending` for those items to consume. (3) A program that declares a `restricted` variable cannot be started until instance data gets envelope encryption at rest (docs/11 §5); every other value is stored in the state JSONB. (4) One runtime audit record per accepted stimulus (`instance.started`, `instance.advanced`, `instance.completed`, `instance.cancelled`, `instance.failed`) with the system actor; user actors arrive with the stimuli that carry them (BPMS-085). (5) A stimulus the instance rejects (stale or duplicate) finishes its job as a no-op with the reason kept on the job. (6) A job whose last allowed attempt loses its lease is dead-lettered; jobs back off 2^n s up to 1 h, 10 attempts. (7) Timers fire when `due_at &lt;= now` (not `now + 1 s`) so `now` in the fired stimulus is never before the due time; a timer fires under a row lock in one transaction, so timers carry no lease or fence (the advance it enqueues is a leased job)</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Runtime-lead review of docs/04 §4 *As built*; SP-10</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Store trace rows; partition `instance_events`; encrypt restricted variables (lifts (3)); audit per command</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>A-29 (BPMS-083)</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>SLA clocks (docs/11 §9, FR-E12). (1) Clocks are level-triggered from the state after each stimulus: an `instance` SLA runs while the instance is not final; a node SLA runs while a live token (waiting or in incident) sits on its node; a running SLA is paused while a live token sits on a `pauseWhile` node. A node passed through within one advance takes no time and opens no clock; re-entering a node later opens a new clock. (2) Business SLAs use the process's default calendar. On resume, the due date moves by the paused working time (business) or the paused wall time (otherwise). (3) A breach fires once per clock, emits `sla.breached` and records the SLA's `breach` actions as a pending effect; delivering them (notify, escalate) waits for notification routing and assignment resolution (BPMS-085). The clock keeps running after a breach and `sla.stopped` reports `met: false`. (4) There is no `at-risk` state yet (E2E-R2-10 needs it; threshold unspecified)</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Product-owner review; E2E-R2-10</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Edge-triggered clocks from node entry/exit; an at-risk threshold setting; stop the clock at breach</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
           <t>A-30 (BPMS-042)</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>Image blocks: the alt text is required (no decorative images yet) and is the block's `text`, so diffs, search and re-ack hashes see it; a swapped picture with the same text still diffs (the file id is part of the compared text). Images can only use files already attached to the same version (attach, then insert); creating an artifact with images is refused. Starting a new version copies the previous version's attachment links so its images and files carry over. DOCX shows `[Image: alt] caption` until pictures are embedded.</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6488,13 +6569,17 @@
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L51" s="3" t="inlineStr"/>
       <c r="M51" s="3" t="inlineStr"/>
       <c r="N51" s="3" t="inlineStr"/>
-      <c r="O51" s="3" t="inlineStr"/>
+      <c r="O51" s="3" t="inlineStr">
+        <is>
+          <t>procera-engine + migration 0031: instances persisted (state JSONB, optimistic revision) with an append-only stimulus log and replay; advance = interpreter + state + log + effects (timers, advance jobs, outbox, pending effects) + SLA clocks + audit in one transaction; jobs with SKIP LOCKED claims, 30 s leases, fencing tokens checked on completion, backoff, dead letter, idempotency keys; scheduler run_once fires due timers once, lateness histogram for the 60 s SLO; business calendars (fixed offset, working days/hours, holidays) with property-tested arithmetic; SLA clocks start/pause/resume/stop/breach; unit, property and PostgreSQL integration tests; docs/04 §4.4, A-27..A-29. Remaining: wiring into the serve scheduler loop and /__test/drain, API/UI and E2E (BPMS-084/085+), encryption of restricted instance data, at-risk SLA state, IANA zones.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -19110,7 +19195,7 @@
       </c>
       <c r="C335" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act | SEC-04, FR-W01</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act (browser: owner deactivates from the person page; the member's open tab is sent to the chooser on the next page; signing in again offers no workspace; the API refuses entry) | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D335" s="3" t="inlineStr">
@@ -19191,7 +19276,7 @@
       </c>
       <c r="C338" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse | A11Y-01, T10</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse (browser: Tab/Enter/typing only, author from Library to Published, colleague from sign-in to Acknowledged) | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D338" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: tracker for the directory import and the R1 gate pack
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -4509,7 +4509,7 @@
       <c r="N19" s="3" t="inlineStr"/>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>procera-members + /api/v1: memberships, invitations (hashed + sealed tokens, 7-day expiry, email-bound, single use; list, revoke, resend), register-by-invite, owner onboarding activates the workspace, workspace switch (ws-scoped JWT), deactivation guards, state gate (423). Directory (migration 0008): department tree (uuid[] paths, sibling-unique names, no moves under descendants), static groups, positions (behind directory.positions.enabled), manager links with cycle rejection, deterministic manager resolution (explicit → nearest department head), per-field source attribution, CSV import with plan/apply. All audited; E2E-R1-MEM-01..03,05..07, E2E-R1-DIR-01..04 Invitation page /invite (GET /invitations/preview, A-24): create account and join, or sign in and join; deep links survive sign-in. E2E-R1-FLOW-01, 02.</t>
+          <t>procera-members + /api/v1: memberships, invitations (hashed + sealed tokens, 7-day expiry, email-bound, single use; list, revoke, resend), register-by-invite, owner onboarding activates the workspace, workspace switch (ws-scoped JWT), deactivation guards, state gate (423). Directory (migration 0008): department tree (uuid[] paths, sibling-unique names, no moves under descendants), static groups, positions (behind directory.positions.enabled), manager links with cycle rejection, deterministic manager resolution (explicit → nearest department head), per-field source attribution, CSV import with plan/apply. All audited; E2E-R1-MEM-01..03,05..07, E2E-R1-DIR-01..04 Invitation page /invite (GET /invitations/preview, A-24): create account and join, or sign in and join; deep links survive sign-in. E2E-R1-FLOW-01, 02. Directory import UI with a check step and per-row reasons (E2E-R1-04); deactivate from the person page with immediate session exit (E2E-R1-16); person page with department, manager and location.</t>
         </is>
       </c>
     </row>
@@ -5086,13 +5086,17 @@
       </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L28" s="3" t="inlineStr"/>
       <c r="M28" s="3" t="inlineStr"/>
       <c r="N28" s="3" t="inlineStr"/>
-      <c r="O28" s="3" t="inlineStr"/>
+      <c r="O28" s="3" t="inlineStr">
+        <is>
+          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-04 directory import, E2E-R1-16 deactivation, E2E-R1-19 keyboard only; plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01..03, 05..15, 17, 18, ISO (several need branding, terminology, template packs, location audiences).</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -18871,7 +18875,7 @@
       </c>
       <c r="C323" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error | FR-W02</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error (browser: Members › Import directory › Check shows each row; cycle and unknown member refused; Apply saves the rest; person pages show department, manager and location) | FR-W02</t>
         </is>
       </c>
       <c r="D323" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: tracker for E2E-R1-17
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -5094,7 +5094,7 @@
       <c r="N28" s="3" t="inlineStr"/>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-04 directory import, E2E-R1-16 deactivation, E2E-R1-19 keyboard only; plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01..03, 05..15, 17, 18, ISO (several need branding, terminology, template packs, location audiences).</t>
+          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-04 directory import, E2E-R1-16 deactivation, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only; plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01..03, 05..15, 18, ISO (several need branding, terminology, template packs, location audiences).</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       </c>
       <c r="C336" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore | FR-S02, J8</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore (browser: reads keep working; the first change is refused and a read-only banner appears on every page; after restore the banner is gone and changes work) | FR-S02, J8</t>
         </is>
       </c>
       <c r="D336" s="3" t="inlineStr">

</xml_diff>

<commit_message>
test(e2e): R1 gate E2E-R1-14 audit trail in the browser and E2E-R1-ISO isolation sweep (BPMS-032)
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -5094,7 +5094,7 @@
       <c r="N28" s="3" t="inlineStr"/>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-04 directory import, E2E-R1-16 deactivation, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only; plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01..03, 05..15, 18, ISO (several need branding, terminology, template packs, location audiences).</t>
+          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-04 directory import, E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO 404 sweep (21 probes); plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01..03, 05..13, 15, 18, and a `denied` audit record for cross-workspace probes (ISO) (several need branding, terminology, template packs, location audiences).</t>
         </is>
       </c>
     </row>
@@ -19145,7 +19145,7 @@
       </c>
       <c r="C333" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK | FR-T01–T04</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK (browser: Person filter shows only that person's events; a version's timeline is oldest first: three edits, submitted, published; the page shows Chain verified) | FR-T01–T04</t>
         </is>
       </c>
       <c r="D333" s="3" t="inlineStr">
@@ -19307,7 +19307,7 @@
       </c>
       <c r="C339" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` | SEC-01/02</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` (built: B's owner probes 21 reads and writes on A's documents, versions, exports, campaigns, announcements, collections, departments, views, files and members → all 404, A unchanged; not yet: the `denied` audit record for cross-workspace probes) | SEC-01/02</t>
         </is>
       </c>
       <c r="D339" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(audit): [protected] a 404 on an object id is recorded as access.denied in the caller's workspace (SEC-01/02)
Completes E2E-R1-ISO: every cross-workspace probe answers 404 and is on record in the
prober's audit log with the object id. A-31.

Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -197,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E31" headerRowCount="1">
-  <autoFilter ref="A1:E31"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E32" headerRowCount="1">
+  <autoFilter ref="A1:E32"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Source"/>
     <tableColumn id="2" name="ID"/>
@@ -1393,7 +1393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2223,6 +2223,29 @@
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>A-31 (SEC-01/02)</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Denied-access audit: any workspace-plane request from an authenticated member that names an object id in its path and answers 404 appends `access.denied` (category access, result denied, object = the first id in the path, reason = method and path) to the caller's own workspace chain. A probe of another workspace's id and a missing id look the same to the caller and are recorded the same way; the other workspace's chain is not written (it cannot be told without cross-tenant lookups). Not rate-limited or deduplicated yet.</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5094,7 +5117,7 @@
       <c r="N28" s="3" t="inlineStr"/>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-04 directory import, E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO 404 sweep (21 probes); plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01..03, 05..13, 15, 18, and a `denied` audit record for cross-workspace probes (ISO) (several need branding, terminology, template packs, location audiences).</t>
+          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-04 directory import, E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO sweep (21 probes → 404, each audited as access.denied, A-31); plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01..03, 05..13, 15, 18 (several need branding, terminology, template packs, location audiences).</t>
         </is>
       </c>
     </row>
@@ -19307,7 +19330,7 @@
       </c>
       <c r="C339" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` (built: B's owner probes 21 reads and writes on A's documents, versions, exports, campaigns, announcements, collections, departments, views, files and members → all 404, A unchanged; not yet: the `denied` audit record for cross-workspace probes) | SEC-01/02</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` (built: B's owner probes 21 reads and writes on A's documents, versions, exports, campaigns, announcements, collections, departments, views, files and members → all 404, each recorded in B's audit log as `access.denied` with the object id, B's chain verifies, A unchanged) | SEC-01/02</t>
         </is>
       </c>
       <c r="D339" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(campaigns): say and choose whether people who join later are asked; E2E-R1-08 (BPMS-046, BPMS-032)
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -5117,7 +5117,7 @@
       <c r="N28" s="3" t="inlineStr"/>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-04 directory import, E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO sweep (21 probes → 404, each audited as access.denied, A-31); plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01..03, 05..13, 15, 18 (several need branding, terminology, template packs, location audiences).</t>
+          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-04 directory import, E2E-R1-08 new joiner gets open campaigns, E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO sweep (21 probes → 404, each audited as access.denied, A-31); plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01..03, 05..07, 09..13, 15, 18 (several need branding, terminology, template packs, location audiences).</t>
         </is>
       </c>
     </row>
@@ -19006,7 +19006,7 @@
       </c>
       <c r="C327" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns | FR-AK03</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns (browser: a campaign created with "Also ask people who join later" on; a new hire who joins from the invitation email after launch finds the request on Home, acknowledges, and shows Done) | FR-AK03</t>
         </is>
       </c>
       <c r="D327" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(members): [protected] audiences can target directory locations; GET /locations (E2E-R1-09)
The audience union gains locations (trimmed, case-insensitive) in the resolver and its
SQL twin (migration 0032). Campaigns, announcements, applicability and collection
visibility all use it; the picker lists locations with member counts.

Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -5117,7 +5117,7 @@
       <c r="N28" s="3" t="inlineStr"/>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-04 directory import, E2E-R1-08 new joiner gets open campaigns, E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO sweep (21 probes → 404, each audited as access.denied, A-31); plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01..03, 05..07, 09..13, 15, 18 (several need branding, terminology, template packs, location audiences).</t>
+          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-04 directory import, E2E-R1-08 new joiner gets open campaigns, E2E-R1-09 location audience (reminders/escalation pending), E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO sweep (21 probes → 404, each audited as access.denied, A-31); plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01..03, 05..07, 10..13, 15, 18, announcement reminders and escalation (R1-09) (several need branding, terminology, template packs, location audiences).</t>
         </is>
       </c>
     </row>
@@ -19033,7 +19033,7 @@
       </c>
       <c r="C328" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct | FR-AN01–06, J14</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct (built: location audience from the directory, only Bangalore members receive it, the acknowledgement shows in receipts; not yet: announcement reminders and manager escalation) | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D328" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(settings): workspace accent painted with contrast-safe shades; live contrast note; GET /branding (FR-W04, E2E-R1-03)
The server moves the accent just far enough to read at 4.5:1 for text and labels and
3:1 for focus, in light and dark themes (property-tested); default is Procera red per
docs/05 §7 (A-33).

Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -197,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E32" headerRowCount="1">
-  <autoFilter ref="A1:E32"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E33" headerRowCount="1">
+  <autoFilter ref="A1:E33"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Source"/>
     <tableColumn id="2" name="ID"/>
@@ -1393,7 +1393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2246,6 +2246,29 @@
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>A-33 (FR-W04)</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Branding accent: docs/20 listed `#4F46E5` as the default while docs/05 §7 and the brand rules make Procera red the default; the default is now `#EE4136`. Any valid colour is accepted (never rejected); the server derives the shades the UI uses by moving it toward black (light theme) or white (dark theme) just enough to pass: links and filled-button labels 4.5:1 on every surface, focus ring 3:1. The logo and the brand mark stay Procera red; `GET /branding` is readable by every member.</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5117,7 +5140,7 @@
       <c r="N28" s="3" t="inlineStr"/>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-04 directory import, E2E-R1-08 new joiner gets open campaigns, E2E-R1-09 location audience (reminders/escalation pending), E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO sweep (21 probes → 404, each audited as access.denied, A-31); plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01..03, 05..07, 10..13, 15, 18, announcement reminders and escalation (R1-09) (several need branding, terminology, template packs, location audiences).</t>
+          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-03 accent branding with contrast-safe shades (logo and terminology pending), E2E-R1-04 directory import, E2E-R1-08 new joiner gets open campaigns, E2E-R1-09 location audience (reminders/escalation pending), E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO sweep (21 probes → 404, each audited as access.denied, A-31); plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01, 02, 05..07, 10..13, branding logo and terminology (R1-03), 15, 18, announcement reminders and escalation (R1-09) (several need branding, terminology, template packs, location audiences).</t>
         </is>
       </c>
     </row>
@@ -18871,7 +18894,7 @@
       </c>
       <c r="C322" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email | FR-W04, 05 §7</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email (built: a too-light accent shows a live contrast note with the shade text will use; the server derives 4.5:1 text and 3:1 focus shades; every member's app paints them; not yet: logo, terminology overrides) | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D322" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs(brand): update BPMS-034 vector asset progress
BPMS-034: record the SVG and favicon slice under docs/05 section 7.1.1. Trademark/domain clearance remains pending under OQ-01. Regenerated tracker outputs with python3 scripts/build_tracker.py.
Signed-off-by: Sachin Sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Milestones" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Backlog" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Domain Backlog" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Risks" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Decisions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Security Tests" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Test Matrix" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Open Questions" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Unknowns" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Assumptions" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="RACI" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Burndown" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Backlog" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Tests" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Questions" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unknowns" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RACI" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Burndown" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5243,7 +5243,7 @@
       <c r="N30" s="3" t="inlineStr"/>
       <c r="O30" s="3" t="inlineStr">
         <is>
-          <t>Raster assets + brand guide merged; SVG masters and trademark search pending</t>
+          <t>Geometric SVG masters, outlined Geist lockups, small-size favicons/PWA icons, marketing assets and theme-aware GitHub README prepared (brand/procera-identity-v2); trademark/domain clearance remains pending (OQ-01)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(web): announcement confirm-by date and campaign link; announcement subjects across Home, campaigns and links (BPMS-047, E2E-R1-09 J14)
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -197,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E33" headerRowCount="1">
-  <autoFilter ref="A1:E33"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E34" headerRowCount="1">
+  <autoFilter ref="A1:E34"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Source"/>
     <tableColumn id="2" name="ID"/>
@@ -1393,7 +1393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2255,20 +2255,47 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
+          <t>A-32 (BPMS-046/047)</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Announcement acknowledgements on the campaign engine (FR-AN04, FR-AK01; docs/04 §2.7 *As built (0033)*). (1) The deadline is the announcement's optional `ack_by` (require_ack only; after publication, no later than `expires_at`); without it the campaign uses going live + **`campaign.default_due`** (no new `announcements.ack.due` key), capped at `expires_at`. (2) Reminders use `campaign.reminders.cadence` and escalation `campaign.escalation.to_manager_after` (0 = off); the escalation offset is `max(that value, the ack window)` so it never fires before the deadline (FR-AN04 "after the deadline"). docs/20 §2.17 `announcements.escalate_unacked_to_manager` is not built; the campaign keys apply. (3) Recipients are the publication snapshot: no joiners, whatever `campaign.audience.snapshot` says. (4) The announcement delivery is the assignment notice (no separate `campaign_assigned`); reminders and escalations use `announcement_ack_*` templates; reminders open `/announcements/{id}`, escalations open the member page. (5) Acknowledging the announcement completes the assignment in the same transaction and appends one `announcement.acknowledged` audit record that cites the assignment; `/acknowledgements/{id}/complete` refuses announcement assignments (409). (6) Once the announcement expires it cannot be acknowledged: due reminder steps are used up silently, the escalation still fires; the campaign stays active until closed. (7) Archiving closes the campaign (reason "the announcement was archived") without `campaign:manage`; the announcement permission authorises it, as with re-ack (A-16). (8) Announcements published before 0033 get no campaign.</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Product-owner review of J14 and docs/04 §2.7</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>An `announcements.ack.due` / `announcements.escalate_unacked_to_manager` key pair; close the campaign at expiry; a distinct assignment notice</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
           <t>A-33 (FR-W04)</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>Branding accent: docs/20 listed `#4F46E5` as the default while docs/05 §7 and the brand rules make Procera red the default; the default is now `#EE4136`. Any valid colour is accepted (never rejected); the server derives the shades the UI uses by moving it toward black (light theme) or white (dark theme) just enough to pass: links and filled-button labels 4.5:1 on every surface, focus ring 3:1. The logo and the brand mark stay Procera red; `GET /branding` is readable by every member.</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Branding accent: docs/20 listed `#4F46E5` as the default while docs/05 §7 and the brand rules make Procera red the default; the default is now `#EE4136`. Any valid colour is accepted (never rejected); the server derives the shades the UI uses by moving it toward black (light theme) or white (dark theme) just enough to pass: links and filled-button labels 4.5:1 on every surface, focus ring 3:1. The Procera brand mark stays red; `GET /branding` is readable by every member. Logo (`branding.logo`): a clean PNG/JPEG/GIF/WebP up to 512 KB (SVG not accepted yet, since it needs sanitising), served to members by `GET /branding/logo` with metadata stripped; the file is kept out of the orphan purge while a branding setting points to it.</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr"/>
+      <c r="E34" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5140,7 +5167,7 @@
       <c r="N28" s="3" t="inlineStr"/>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-03 accent branding with contrast-safe shades (logo and terminology pending), E2E-R1-04 directory import, E2E-R1-08 new joiner gets open campaigns, E2E-R1-09 location audience (reminders/escalation pending), E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO sweep (21 probes → 404, each audited as access.denied, A-31); plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01, 02, 05..07, 10..13, branding logo and terminology (R1-03), 15, 18, announcement reminders and escalation (R1-09) (several need branding, terminology, template packs, location audiences).</t>
+          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-03 accent branding with contrast-safe shades (logo and terminology pending), E2E-R1-04 directory import, E2E-R1-08 new joiner gets open campaigns, E2E-R1-09 J14 location audience with confirm-by, campaign engine, one escalation, archive closes, E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO sweep (21 probes → 404, each audited as access.denied, A-31); plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01, 02, 05..07, 10..13, branding logo and terminology (R1-03), 15, 18 (several need branding, terminology, template packs, location audiences).</t>
         </is>
       </c>
     </row>
@@ -5721,7 +5748,7 @@
       <c r="N37" s="3" t="inlineStr"/>
       <c r="O37" s="3" t="inlineStr">
         <is>
-          <t>procera-campaigns (migration 0013): acknowledgement campaigns for a published SOP/policy version; audience via the shared resolver (snapshot or dynamic), assignments with in-app + email notices, acknowledgement bound to version id + content hash + statement + auth method, reminder ladder and one-time manager escalation by the scheduler, dynamic new joiners, close/cancel, progress, audited evidence CSV; settings campaign.*; E2E-R1-CMP-01..07. Later: quiz-lite, exemptions, signed PDF evidence, auto re-ack on major publish</t>
+          <t>procera-campaigns (migration 0013): acknowledgement campaigns for a published SOP/policy version; audience via the shared resolver (snapshot or dynamic), assignments with in-app + email notices, acknowledgement bound to version id + content hash + statement + auth method, reminder ladder and one-time manager escalation by the scheduler, dynamic new joiners, close/cancel, progress, audited evidence CSV; settings campaign.*; E2E-R1-CMP-01..07. Later: quiz-lite, exemptions, signed PDF evidence, auto re-ack on major publish Campaign subjects include announcements (0033).</t>
         </is>
       </c>
     </row>
@@ -5786,7 +5813,7 @@
       <c r="N38" s="3" t="inlineStr"/>
       <c r="O38" s="3" t="inlineStr">
         <is>
-          <t>procera-announcements (migration 0014): drafts with block content, audience snapshot, approval per announcements.approval_required with SoD, scheduling + derived expiry, pinned/critical, channels from settings, in-app + email delivery via the outbox, read and acknowledgement receipts, analytics, archive; settings announcements.*; E2E-R1-ANN-01..06. Later: poster scoping, reminders/escalation for unacked, comments/reactions, reach preview Approval loop notifications (A-25): approvers told on submit, author told approved or sent back. E2E-R1-FLOW-04, 06.</t>
+          <t>procera-announcements (migration 0014): drafts with block content, audience snapshot, approval per announcements.approval_required with SoD, scheduling + derived expiry, pinned/critical, channels from settings, in-app + email delivery via the outbox, read and acknowledgement receipts, analytics, archive; settings announcements.*; E2E-R1-ANN-01..06. Later: poster scoping, reminders/escalation for unacked, comments/reactions, reach preview Approval loop notifications (A-25): approvers told on submit, author told approved or sent back. E2E-R1-FLOW-04, 06. Announcement acknowledgements run on the campaign engine (migration 0033, A-32): confirm-by date, reminder ladder, one manager escalation, archive closes; composer Confirm by and drawer link. E2E-R1-09.</t>
         </is>
       </c>
     </row>
@@ -18894,7 +18921,7 @@
       </c>
       <c r="C322" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email (built: a too-light accent shows a live contrast note with the shade text will use; the server derives 4.5:1 text and 3:1 focus shades; every member's app paints them; not yet: logo, terminology overrides) | FR-W04, 05 §7</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email (built: a too-light accent shows a live contrast note with the shade text will use; the server derives 4.5:1 text and 3:1 focus shades; every member's app paints them; a logo uploaded in Settings shows in everyone's sidebar; not yet: terminology overrides) | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D322" s="3" t="inlineStr">
@@ -19056,7 +19083,7 @@
       </c>
       <c r="C328" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct (built: location audience from the directory, only Bangalore members receive it, the acknowledgement shows in receipts; not yet: announcement reminders and manager escalation) | FR-AN01–06, J14</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct (browser: location audience from the directory, confirm-by date, only Bangalore members receive it; the announcement's campaign counts the confirmation; past the deadline the manager of the member who did not confirm is told exactly once; archiving closes the campaign) | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D328" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(web): schedule a publication (Goes live); overview tiles drill into filtered lists; audit filters from the URL (E2E-R1-06, E2E-R1-15)
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -5167,7 +5167,7 @@
       <c r="N28" s="3" t="inlineStr"/>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-03 accent branding with contrast-safe shades (logo and terminology pending), E2E-R1-04 directory import, E2E-R1-08 new joiner gets open campaigns, E2E-R1-09 J14 location audience with confirm-by, campaign engine, one escalation, archive closes, E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO sweep (21 probes → 404, each audited as access.denied, A-31); plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01, 02, 05..07, 10..13, branding logo and terminology (R1-03), 15, 18 (several need branding, terminology, template packs, location audiences).</t>
+          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-03 accent branding with contrast-safe shades (logo and terminology pending), E2E-R1-04 directory import, E2E-R1-06 controlled policy SoD, step-up approve, scheduled go-live, superseded; E2E-R1-08 new joiner gets open campaigns, E2E-R1-09 J14 location audience with confirm-by, campaign engine, one escalation, archive closes, E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-15 overview drill-downs, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO sweep (21 probes → 404, each audited as access.denied, A-31); plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01, 02, 05..07, 10..13, branding logo and terminology (R1-03), 15, 18 (several need branding, terminology, template packs, location audiences).</t>
         </is>
       </c>
     </row>
@@ -19002,7 +19002,7 @@
       </c>
       <c r="C325" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF | FR-G04/G05/G10, FR-PL01</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF (browser: the author's Approve is refused; the reviewer confirms with a code after an aged sign-in; Publish › Goes live schedules v2; `/__test/library/due` makes it due without moving the shared clock; v1's printable export carries the Superseded banner) | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D325" s="3" t="inlineStr">
@@ -19245,7 +19245,7 @@
       </c>
       <c r="C334" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts | FR-A01</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts (browser: open acknowledgements → active campaigns with the same "still to acknowledge"; versions published → audit log filtered to publications with the same event count; announcements published → the Published tab; without two-step → People &amp; access filtered with the same count) | FR-A01</t>
         </is>
       </c>
       <c r="D334" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(library): [protected] collection-scoped grants apply to documents; my_actions per document; E2E-R1-01, 02, 05 (BPMS-024, BPMS-032)
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -197,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E34" headerRowCount="1">
-  <autoFilter ref="A1:E34"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E35" headerRowCount="1">
+  <autoFilter ref="A1:E35"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Source"/>
     <tableColumn id="2" name="ID"/>
@@ -1393,7 +1393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2296,6 +2296,29 @@
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>A-34 (BPMS-024/041)</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Scoped grants on documents: a document filed in a collection is checked against that collection under its ancestors, so a role granted for a collection applies to the documents in it and its sub-collections; holding an authoring permission there also shows that collection's drafts. Unfiled documents use workspace grants only. `GET /artifacts/{id}` returns `my_actions`, the actions the caller may take on that document, and the page offers only those. Creating a document still needs the workspace-level create permission (a new document is not in a collection yet).</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5167,7 +5190,7 @@
       <c r="N28" s="3" t="inlineStr"/>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-03 accent branding with contrast-safe shades (logo and terminology pending), E2E-R1-04 directory import, E2E-R1-06 controlled policy SoD, step-up approve, scheduled go-live, superseded; E2E-R1-08 new joiner gets open campaigns, E2E-R1-09 J14 location audience with confirm-by, campaign engine, one escalation, archive closes, E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-15 overview drill-downs, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO sweep (21 probes → 404, each audited as access.denied, A-31); plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01, 02, 05..07, 10..13, branding logo and terminology (R1-03), 15, 18 (several need branding, terminology, template packs, location audiences).</t>
+          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-01 setup page, E2E-R1-02 new workspaces with owner onboarding, E2E-R1-05 roles with collection scope, E2E-R1-03 accent branding with contrast-safe shades (logo and terminology pending), E2E-R1-04 directory import, E2E-R1-06 controlled policy SoD, step-up approve, scheduled go-live, superseded; E2E-R1-10 announcement approval and expiry, E2E-R1-08 new joiner gets open campaigns, E2E-R1-09 J14 location audience with confirm-by, campaign engine, one escalation, archive closes, E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-15 overview drill-downs, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO sweep (21 probes → 404, each audited as access.denied, A-31); plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01, 02, 05..07, 10..13, branding logo and terminology (R1-03), 15, 18 (several need branding, terminology, template packs, location audiences).</t>
         </is>
       </c>
     </row>
@@ -18867,7 +18890,7 @@
       </c>
       <c r="C320" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work | FR-S01</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work (browser: /setup refuses a bad token or says the platform is already set up; no default account signs in; the full first run needs a fresh database, since the shared E2E database already has system admins) | FR-S01</t>
         </is>
       </c>
       <c r="D320" s="3" t="inlineStr">
@@ -18894,7 +18917,7 @@
       </c>
       <c r="C321" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA | FR-S02/S03, FR-W01</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA (browser: System › New workspace twice; owner A opens the emailed link, creates the account, turns on two-step verification, signs in and lands in the workspace) | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D321" s="3" t="inlineStr">
@@ -18975,7 +18998,7 @@
       </c>
       <c r="C324" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused | FR-W03, J6</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused (browser: Roles &amp; access › Duplicate › grant to a person for the HR collection; a permission change previews "1 person gains 1 permission"; the holder gets Edit on the HR draft but not the Finance one, and the API agrees; an admin putting an owner-only permission into a role gets 403 escalation) | FR-W03, J6</t>
         </is>
       </c>
       <c r="D324" s="3" t="inlineStr">
@@ -19110,7 +19133,7 @@
       </c>
       <c r="C329" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it | FX-C01, FR-AN03</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it (browser: the drawer says approval is needed, the author sends it, a second admin approves, members see it; at expiry it leaves the feed and admins see it as Expired) | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D329" s="3" t="inlineStr">

</xml_diff>

<commit_message>
test(e2e): E2E-R1-07 re-acknowledgement at scale with evidence; the no-sleeps lint allows test timeouts
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -5190,7 +5190,7 @@
       <c r="N28" s="3" t="inlineStr"/>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-01 setup page, E2E-R1-02 new workspaces with owner onboarding, E2E-R1-05 roles with collection scope, E2E-R1-03 accent branding with contrast-safe shades (logo and terminology pending), E2E-R1-04 directory import, E2E-R1-06 controlled policy SoD, step-up approve, scheduled go-live, superseded; E2E-R1-10 announcement approval and expiry, E2E-R1-08 new joiner gets open campaigns, E2E-R1-09 J14 location audience with confirm-by, campaign engine, one escalation, archive closes, E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-15 overview drill-downs, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO sweep (21 probes → 404, each audited as access.denied, A-31); plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01, 02, 05..07, 10..13, branding logo and terminology (R1-03), 15, 18 (several need branding, terminology, template packs, location audiences).</t>
+          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-01 setup page, E2E-R1-02 new workspaces with owner onboarding, E2E-R1-05 roles with collection scope, E2E-R1-03 accent branding with contrast-safe shades (logo and terminology pending), E2E-R1-04 directory import, E2E-R1-06 controlled policy SoD, step-up approve, scheduled go-live, superseded; E2E-R1-10 announcement approval and expiry, E2E-R1-07 re-ack at scale with evidence, E2E-R1-08 new joiner gets open campaigns, E2E-R1-09 J14 location audience with confirm-by, campaign engine, one escalation, archive closes, E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-15 overview drill-downs, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO sweep (21 probes → 404, each audited as access.denied, A-31); plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01, 02, 05..07, 10..13, branding logo and terminology (R1-03), 15, 18 (several need branding, terminology, template packs, location audiences).</t>
         </is>
       </c>
     </row>
@@ -19052,7 +19052,7 @@
       </c>
       <c r="C326" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method | FR-PL03, FR-AK01–04</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method (browser: the owner publishes v2.0 as major, 51 asked; 10 people acknowledge at 390×844 from Home, 40 through the same API; the campaign shows 50 of 51 and the evidence CSV lists the v2 hash and sign-in method for all 50) | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D326" s="3" t="inlineStr">

</xml_diff>

<commit_message>
test(e2e): R1-03 covers terminology overrides; tracker regenerated
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -197,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E35" headerRowCount="1">
-  <autoFilter ref="A1:E35"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E36" headerRowCount="1">
+  <autoFilter ref="A1:E36"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Source"/>
     <tableColumn id="2" name="ID"/>
@@ -1393,7 +1393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2319,6 +2319,33 @@
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>A-36 (CFG-008, FR-W04)</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Terminology overrides are `en` only. docs/20 §2.2 says "per-locale label", but `en` is the only UI and email locale, so the value holds one `{singular, plural}` per term and no locale layer; a per-locale shape (`{en: {...}, de: {...}}`) can be added when a second locale ships. Labels are used as written in headings and tags. Mid-sentence, each word's first letter is lowered unless the word starts with two capitals ("SOP", "HR"), so "Work Instruction" reads "work instruction". Articles ("a"/"an") are avoided around a renamed term rather than guessed. Policies, announcements and campaigns are not renameable terms.</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Per-locale labels and grammatical forms (articles, gender) with the i18n pipeline (UX-033)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -18944,7 +18971,7 @@
       </c>
       <c r="C322" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email (built: a too-light accent shows a live contrast note with the shade text will use; the server derives 4.5:1 text and 3:1 focus shades; every member's app paints them; a logo uploaded in Settings shows in everyone's sidebar; not yet: terminology overrides) | FR-W04, 05 §7</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email (built: a too-light accent shows a live contrast note with the shade text will use; the server derives 4.5:1 text and 3:1 focus shades; every member's app paints them; a logo uploaded in Settings shows in everyone's sidebar; renaming SOP to "Work Instruction" in Settings › Terminology changes the labels other members see; "Request" has no screens until M6, so its override is covered at unit level) | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D322" s="3" t="inlineStr">
@@ -19025,7 +19052,7 @@
       </c>
       <c r="C325" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF (browser: the author's Approve is refused; the reviewer confirms with a code after an aged sign-in; Publish › Goes live schedules v2; `/__test/library/due` makes it due without moving the shared clock; v1's printable export carries the Superseded banner) | FR-G04/G05/G10, FR-PL01</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF (browser: the author's Approve is refused; the reviewer confirms with their password after an aged sign-in; Publish › Goes live schedules v2; `/__test/library/due` makes it due without moving the shared clock; v1's printable export carries the Superseded banner) | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D325" s="3" t="inlineStr">
@@ -19160,7 +19187,7 @@
       </c>
       <c r="C330" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B | FR-F01–F03, SEC-10</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B (browser: a 50 MB attachment with one chunk dropped resumes and its SHA-256 matches; EICAR shows quarantined and gets no link; links last ≤ 5 minutes, a tampered link is refused, workspace B gets 404 for the link and the file) | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D330" s="3" t="inlineStr">

</xml_diff>

<commit_message>
test(e2e): E2E-R1-11, R1-12, R1-13 gate tests; A-37
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -197,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E36" headerRowCount="1">
-  <autoFilter ref="A1:E36"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E38" headerRowCount="1">
+  <autoFilter ref="A1:E38"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Source"/>
     <tableColumn id="2" name="ID"/>
@@ -1393,7 +1393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2328,24 +2328,74 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
+          <t>A-35 (BPMS-028)</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>DataGrid v2 (FR-V02, FR-V04, FR-V07; docs/05 §4 *As built*). (1) **Filter groups:** one level only (docs/05 allows depth ≤ 2): the top level ANDs its plain conditions and its groups; each group matches all (and) or any (or) of its conditions. The state keeps v1 `filters` and adds an optional `groups`, so v1 saved views and `?grid=` links load unchanged. (2) **Role sharing:** a view is personal, shared with everyone, or shared with one role (`shared_role`, a role key), never two of these; any member may share with any role of the workspace (they need not hold it), and `GET /views/roles` lists role keys and names to every member for that picker. Holding a role means an unexpired grant of it at **any scope**, directly or through a group; deleting the role makes its views personal. Only the owner changes or deletes a view, as in v1; workspace admins do not see others' personal views (they are preferences, not content). (3) **XLSX:** built by the server in `POST /exports` (`format: xlsx`) from the header and cells the browser sends, which are exactly the visible columns, rows, order and values the CSV gets, so redaction is the same as on screen; the server checks the shape (one value per column, `rows` = cell rows) but not the values, until the server-driven query model (docs/04 §5) lets it rebuild the rows itself. At most 10 000 rows and an 8 MB request per synchronous export; text cells are always strings, and formula-like text (`= + - @`, tab, CR) also gets Excel's quote prefix, the twin of the CSV apostrophe. Numbers and booleans keep their type; dates stay the text the grid shows.</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Owner review of E2E-R1-13</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Nested groups (depth 2); sharing only with roles the sharer holds; server-rebuilt XLSX rows; async exports</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
           <t>A-36 (CFG-008, FR-W04)</t>
         </is>
       </c>
-      <c r="C36" s="3" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>Terminology overrides are `en` only. docs/20 §2.2 says "per-locale label", but `en` is the only UI and email locale, so the value holds one `{singular, plural}` per term and no locale layer; a per-locale shape (`{en: {...}, de: {...}}`) can be added when a second locale ships. Labels are used as written in headings and tags. Mid-sentence, each word's first letter is lowered unless the word starts with two capitals ("SOP", "HR"), so "Work Instruction" reads "work instruction". Articles ("a"/"an") are avoided around a renamed term rather than guessed. Policies, announcements and campaigns are not renameable terms.</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
+      <c r="E37" s="3" t="inlineStr">
         <is>
           <t>Per-locale labels and grammatical forms (articles, gender) with the i18n pipeline (UX-033)</t>
         </is>
       </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>A-37 (FR-F06/F09)</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Per-file retention class: an admin (`file:delete`) may set or clear a file's class in bulk with a reason (`POST /files/retention`, one `file.retention_changed` audit record per file); a set class wins over the one derived from what holds the file, and the Files view says "(set by an admin)". Legal holds remain BPMS-164.</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5217,7 +5267,7 @@
       <c r="N28" s="3" t="inlineStr"/>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-01 setup page, E2E-R1-02 new workspaces with owner onboarding, E2E-R1-05 roles with collection scope, E2E-R1-03 accent branding with contrast-safe shades (logo and terminology pending), E2E-R1-04 directory import, E2E-R1-06 controlled policy SoD, step-up approve, scheduled go-live, superseded; E2E-R1-10 announcement approval and expiry, E2E-R1-07 re-ack at scale with evidence, E2E-R1-08 new joiner gets open campaigns, E2E-R1-09 J14 location audience with confirm-by, campaign engine, one escalation, archive closes, E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-15 overview drill-downs, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO sweep (21 probes → 404, each audited as access.denied, A-31); plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01, 02, 05..07, 10..13, branding logo and terminology (R1-03), 15, 18 (several need branding, terminology, template packs, location audiences).</t>
+          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-01 setup page, E2E-R1-02 new workspaces with owner onboarding, E2E-R1-05 roles with collection scope, E2E-R1-03 accent branding with contrast-safe shades (logo and terminology pending), E2E-R1-04 directory import, E2E-R1-06 controlled policy SoD, step-up approve, scheduled go-live, superseded; E2E-R1-10 announcement approval and expiry, E2E-R1-07 re-ack at scale with evidence, E2E-R1-11 resumable 50 MB upload and links, E2E-R1-12 Files retention and held files, E2E-R1-13 DataGrid groups, shared views and exports, E2E-R1-08 new joiner gets open campaigns, E2E-R1-09 J14 location audience with confirm-by, campaign engine, one escalation, archive closes, E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-15 overview drill-downs, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO sweep (21 probes → 404, each audited as access.denied, A-31); plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01, 02, 05..07, 10..13, branding logo and terminology (R1-03), 15, 18 (several need branding, terminology, template packs, location audiences).</t>
         </is>
       </c>
     </row>
@@ -19214,7 +19264,7 @@
       </c>
       <c r="C331" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused | FR-F06, FR-V</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused (browser: Quarantined chip and a Name filter; two files changed to Operational with a reason, shown as set by an admin and audited; deleting a file a published version holds is refused) | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D331" s="3" t="inlineStr">
@@ -19241,7 +19291,7 @@
       </c>
       <c r="C332" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction | FR-V01–V07</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction (browser: Status is Published and (Name contains Alpha or Charlie); sort by type then name; view shared with Reviewers opens from the deep link for a reviewer; CSV has exactly the shown rows; XLSX downloads) | FR-V01–V07</t>
         </is>
       </c>
       <c r="D332" s="3" t="inlineStr">

</xml_diff>

<commit_message>
test(e2e): E2E-R1-18 startup day one; AUD-01 covers template install
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -197,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E38" headerRowCount="1">
-  <autoFilter ref="A1:E38"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E39" headerRowCount="1">
+  <autoFilter ref="A1:E39"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Source"/>
     <tableColumn id="2" name="ID"/>
@@ -1393,7 +1393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2396,6 +2396,29 @@
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>A-38 (BPMS-106, FR-G08)</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Template packs, P0 subset (docs/21 §4 *As built*, docs/08 "Templates", docs/05 §3.7 *As built*). (1) **Provenance:** the packs ship in code (`crates/library/src/templates/`), versioned (`policy-ack` 1.0.0, `core-sops` 1.0.0) and changed only by a reviewed commit; the text is written for Procera from general practice, copies no standard or company document, opens with a "Template to adapt" notice, says it is not legal advice and makes no compliance claims. The gallery service, workspace-published templates, role mapping and upgrade diffs (FR-S06, FR-G08 in full) stay with BPMS-106. (2) **Keys on conflict:** a document whose key already exists (any state) is skipped and reported with the existing artifact; only an explicit `on_conflict: copy` creates a copy under the first free `key-N` (2-99) titled "Title (N)". Installing twice never duplicates silently, and every install appends one `template.installed` listing each outcome. (3) **Drafts:** documents install as `standard` criticality drafts owned by the installer, top level (no collection), through the normal create path (`artifact.created` each); review and publication follow the workspace review policy. (4) **Campaign defaults:** a campaign needs a published version (BPMS-046), so install does not create one; it returns a plan (everyone, due 14 days after launch, for the handbook) and the UI links to the new-campaign dialog with the document and date filled in. An automatic "ask on first publish" per document would need a stored acknowledgement requirement (docs/05 §3.21 *Authoring*) and is not built. (5) **Permissions:** browse = `template:browse` (Member has it); install = `template:install` plus `&lt;kind&gt;:create` for each kind created (Workspace Admin/Owner hold both; Process Owner holds `template:install` but not `policy:create`, so it can install `core-sops` only).</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5267,7 +5290,7 @@
       <c r="N28" s="3" t="inlineStr"/>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-01 setup page, E2E-R1-02 new workspaces with owner onboarding, E2E-R1-05 roles with collection scope, E2E-R1-03 accent branding with contrast-safe shades (logo and terminology pending), E2E-R1-04 directory import, E2E-R1-06 controlled policy SoD, step-up approve, scheduled go-live, superseded; E2E-R1-10 announcement approval and expiry, E2E-R1-07 re-ack at scale with evidence, E2E-R1-11 resumable 50 MB upload and links, E2E-R1-12 Files retention and held files, E2E-R1-13 DataGrid groups, shared views and exports, E2E-R1-08 new joiner gets open campaigns, E2E-R1-09 J14 location audience with confirm-by, campaign engine, one escalation, archive closes, E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-15 overview drill-downs, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO sweep (21 probes → 404, each audited as access.denied, A-31); plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01, 02, 05..07, 10..13, branding logo and terminology (R1-03), 15, 18 (several need branding, terminology, template packs, location audiences).</t>
+          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-01 setup page, E2E-R1-02 new workspaces with owner onboarding, E2E-R1-05 roles with collection scope, E2E-R1-03 accent branding with contrast-safe shades (logo and terminology pending), E2E-R1-04 directory import, E2E-R1-06 controlled policy SoD, step-up approve, scheduled go-live, superseded; E2E-R1-10 announcement approval and expiry, E2E-R1-07 re-ack at scale with evidence, E2E-R1-11 resumable 50 MB upload and links, E2E-R1-12 Files retention and held files, E2E-R1-13 DataGrid groups, shared views and exports, E2E-R1-18 startup day one with template packs, E2E-R1-08 new joiner gets open campaigns, E2E-R1-09 J14 location audience with confirm-by, campaign engine, one escalation, archive closes, E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-15 overview drill-downs, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO sweep (21 probes → 404, each audited as access.denied, A-31); plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01, 02, 05..07, 10..13, branding logo and terminology (R1-03), 15, 18 (several need branding, terminology, template packs, location audiences).</t>
         </is>
       </c>
     </row>
@@ -19426,7 +19449,7 @@
       </c>
       <c r="C337" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock | J12</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock (browser: Home › Browse templates › Install the handbook pack (5 drafts) → publish the handbook → launch the campaign → 20 people at 390×844 acknowledge; 20 of 21 done, within 15 minutes) | J12</t>
         </is>
       </c>
       <c r="D337" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(brand): vector logo masters and crisp exports (BPMS-034)
One geometry for the P-ribbon symbol (64-unit grid, fold shading), a flat symbol for
16-32 px, horizontal and stacked lockups for light and dark, app icons and the banner,
generated by assets/brand/vector/build.py with the wordmark outlined from Geist (OFL).
PNGs, favicons and the ICO are exported from the SVGs; the app uses the SVG symbol
and an SVG favicon.

Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -5416,7 +5416,7 @@
       <c r="N30" s="3" t="inlineStr"/>
       <c r="O30" s="3" t="inlineStr">
         <is>
-          <t>Raster assets + brand guide merged; SVG masters and trademark search pending</t>
+          <t>Vector masters (assets/brand/vector, generated by build.py: P-ribbon symbol, flat small symbol, horizontal and stacked lockups light/dark, app icons, banner; wordmark outlined from Geist, OFL); PNGs, favicons and ICO re-exported from them; the app uses the SVG symbol and an SVG favicon. Remaining: trademark search (OQ-01), professional mark review before GA</t>
         </is>
       </c>
     </row>
@@ -19098,7 +19098,7 @@
       </c>
       <c r="C324" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused (browser: Roles &amp; access › Duplicate › grant to a person for the HR collection; a permission change previews "1 person gains 1 permission"; the holder gets Edit on the HR draft but not the Finance one, and the API agrees; an admin putting an owner-only permission into a role gets 403 escalation) | FR-W03, J6</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused (browser: Roles &amp; access › Duplicate › grant to a person for the HR collection; a permission change previews "1 person gains 1 permission"; the holder gets Edit on the HR draft but not the Finance one, and the API agrees; a role manager who lacks audit export cannot put it into a role (403 escalation)) | FR-W03, J6</t>
         </is>
       </c>
       <c r="D324" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: account recovery and admin account controls designed (OQ-15 decided: option A), A-39
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -197,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E39" headerRowCount="1">
-  <autoFilter ref="A1:E39"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E40" headerRowCount="1">
+  <autoFilter ref="A1:E40"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Source"/>
     <tableColumn id="2" name="ID"/>
@@ -1393,7 +1393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2419,6 +2419,29 @@
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>A-39 (OQ-15)</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Account recovery: a password reset or change keeps two-step verification (only an admin's explicit reset removes it); reset links last 30 minutes, are single use and are stored hashed; a reset revokes every session, a signed-in change revokes the others; admin "require password change", "sign out everywhere" and "reset two-step verification" apply only when this is the member's only active workspace (accounts are global), else a system administrator does it; recovery emails are system emails (not in a workspace's mail queue).</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -25166,12 +25189,12 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Forgotten passwords.** Self-service reset by email link, or admin-initiated reset only (the sign-in page today says "Lost access? Ask your workspace admin", and there is no reset flow at all)? What happens to MFA on reset?</t>
+          <t>~~Forgotten passwords~~ **Decided 2026-10-12 (owner): option A.** Self-service "Forgot password?" by email link, change password while signed in, and admin controls (send reset link, require a password change at next sign-in, sign out everywhere, reset two-step verification). Designed in docs/06 §3.6.1; two-step verification is kept on reset (A-39).</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Self-service email reset (single-use 30-minute link, signs out all sessions, keeps MFA so a mailbox alone can't take the account) plus an admin "send reset link" on Members; lost second factor stays admin-assisted with step-up and audit</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -25181,7 +25204,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
chore(tracker): bring statuses up to date (R1 gate done, recovery, profile, roles UI, templates, site; directory UI, settings and IA redesign in progress)
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -197,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E40" headerRowCount="1">
-  <autoFilter ref="A1:E40"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E41" headerRowCount="1">
+  <autoFilter ref="A1:E41"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Source"/>
     <tableColumn id="2" name="ID"/>
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E393" headerRowCount="1">
-  <autoFilter ref="A1:E393"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E398" headerRowCount="1">
+  <autoFilter ref="A1:E398"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -1393,7 +1393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2442,6 +2442,33 @@
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>A-40 (OQ-15, as built)</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Account recovery details the decision left open (docs/06 §3.6.1 *As built*): (1) a **system role** counts as "outside this workspace", so a workspace admin cannot require a password change, sign out or reset two-step verification of a system account; (2) an admin's reset link is not counted against the 3-per-hour self-service budget; (3) "require a password change" does not end current sessions (the admin can also sign the member out everywhere); (4) the change token after `password_change_required` lasts 10 minutes; (5) recovery emails use the system workspace's queue (nil workspace id) rather than a separate table.</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Product-owner review of docs/06 §3.6.1 *As built</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Treat system accounts like any other; count admin links; revoke sessions on "require change"; a separate system mail table</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4533,7 +4560,7 @@
       <c r="N16" s="3" t="inlineStr"/>
       <c r="O16" s="3" t="inlineStr">
         <is>
-          <t>procera-platform + /sysapi/v1: one-time bootstrap token (printed at startup until bootstrapped), system.owner/admin/operator/auditor fixed authz table, MFA required for system plane, workspace create/list/get/rename/suspend/restore/schedule-deletion with If-Match + ETag, profile quotas, platform setting floors seeded, all audited; E2E-R1-SYS-01..05</t>
+          <t>procera-platform + /sysapi/v1: one-time bootstrap token (printed at startup until bootstrapped), system.owner/admin/operator/auditor fixed authz table, MFA required for system plane, workspace create/list/get/rename/suspend/restore/schedule-deletion with If-Match + ETag, profile quotas, platform setting floors seeded, all audited; E2E-R1-SYS-01..05 Workspace rename from workspace Settings (PATCH /api/v1/workspace, audited on the system and workspace chains), E2E-R1-UI-47.</t>
         </is>
       </c>
     </row>
@@ -4598,7 +4625,7 @@
       <c r="N17" s="3" t="inlineStr"/>
       <c r="O17" s="3" t="inlineStr">
         <is>
-          <t>procera-identity + /api/v1/auth: users, Argon2id (policy, rehash, enumeration-safe), JWT access (ADR-0020) + rotating refresh with reuse detection, DB login throttling + per-IP rate limit, logout, sign-out-everywhere, deactivation via token_version; audited; E2E-R1-AUTH-01..05,07</t>
+          <t>procera-identity + /api/v1/auth: users, Argon2id (policy, rehash, enumeration-safe), JWT access (ADR-0020) + rotating refresh with reuse detection, DB login throttling + per-IP rate limit, logout, sign-out-everywhere, deactivation via token_version; audited; E2E-R1-AUTH-01..05,07 Account recovery (migration 0036, docs/06 §3.6.1, A-39/A-40): forgot password with hashed single-use 30-minute reset links (no enumeration, rate limited), reset revokes sessions and keeps two-step, change password, admin-required change at next sign-in; admin account controls on the person page (member:security.manage, step-up and reason, only-workspace rule): send reset link, require password change, sign out everywhere, reset two-step; Account › Profile (name, time zone, language). E2E-R1-UI-46, 48..50, AUD-01.</t>
         </is>
       </c>
     </row>
@@ -4720,7 +4747,7 @@
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L19" s="3" t="inlineStr"/>
@@ -4728,7 +4755,7 @@
       <c r="N19" s="3" t="inlineStr"/>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>procera-members + /api/v1: memberships, invitations (hashed + sealed tokens, 7-day expiry, email-bound, single use; list, revoke, resend), register-by-invite, owner onboarding activates the workspace, workspace switch (ws-scoped JWT), deactivation guards, state gate (423). Directory (migration 0008): department tree (uuid[] paths, sibling-unique names, no moves under descendants), static groups, positions (behind directory.positions.enabled), manager links with cycle rejection, deterministic manager resolution (explicit → nearest department head), per-field source attribution, CSV import with plan/apply. All audited; E2E-R1-MEM-01..03,05..07, E2E-R1-DIR-01..04 Invitation page /invite (GET /invitations/preview, A-24): create account and join, or sign in and join; deep links survive sign-in. E2E-R1-FLOW-01, 02. Directory import UI with a check step and per-row reasons (E2E-R1-04); deactivate from the person page with immediate session exit (E2E-R1-16); person page with department, manager and location.</t>
+          <t>procera-members + /api/v1: memberships, invitations (hashed + sealed tokens, 7-day expiry, email-bound, single use; list, revoke, resend), register-by-invite, owner onboarding activates the workspace, workspace switch (ws-scoped JWT), deactivation guards, state gate (423). Directory (migration 0008): department tree (uuid[] paths, sibling-unique names, no moves under descendants), static groups, positions (behind directory.positions.enabled), manager links with cycle rejection, deterministic manager resolution (explicit → nearest department head), per-field source attribution, CSV import with plan/apply. All audited; E2E-R1-MEM-01..03,05..07, E2E-R1-DIR-01..04 Invitation page /invite (GET /invitations/preview, A-24): create account and join, or sign in and join; deep links survive sign-in. E2E-R1-FLOW-01, 02. Directory import UI with a check step and per-row reasons (E2E-R1-04); deactivate from the person page with immediate session exit (E2E-R1-16); person page with department, manager and location. Remaining (owner: user management missing): directory UI to create, rename and move departments and groups, editable person profile, reactivate, bulk set — in progress.</t>
         </is>
       </c>
     </row>
@@ -4793,7 +4820,7 @@
       <c r="N20" s="3" t="inlineStr"/>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>procera-access: permission catalogue + 12 role templates; custom roles (no escalation on create/edit/grant/revoke, built-ins immutable, clone lineage); grants to members or static groups (migration 0009), scoped (workspace/department/collection/process/case) with expiry, compiled to Cedar; members inherit their department subtree so department-scoped admins reach only it; invariants (workspace isolation, active members only); last-owner protection; role change preview; access_revisions cache; all changes audited. Property tests: no escalation (64 cases) and preview matches effect (48 cases), both against Postgres. E2E-R1-MEM-04,08,09</t>
+          <t>procera-access: permission catalogue + 12 role templates; custom roles (no escalation on create/edit/grant/revoke, built-ins immutable, clone lineage); grants to members or static groups (migration 0009), scoped (workspace/department/collection/process/case) with expiry, compiled to Cedar; members inherit their department subtree so department-scoped admins reach only it; invariants (workspace isolation, active members only); last-owner protection; role change preview; access_revisions cache; all changes audited. Property tests: no escalation (64 cases) and preview matches effect (48 cases), both against Postgres. E2E-R1-MEM-04,08,09 Roles &amp; access UI: roles list and drawer, custom roles, grants with scope and expiry, collection-scoped library grants (A-34); the Member baseline is always granted on accept, so specialist roles add to it (E2E-R1-05).</t>
         </is>
       </c>
     </row>
@@ -4988,7 +5015,7 @@
       <c r="N23" s="3" t="inlineStr"/>
       <c r="O23" s="3" t="inlineStr">
         <is>
-          <t>Catalogue, floors, profiles, explainer (earlier); department overrides as layer 4 with tree inheritance (0021), profile switch plan/apply with If-Match, reason and step-up (CFG-017), effective-settings cache with generation invalidation over Valkey, never authoritative (CFG-004); Settings tabs for departments and profile. E2E-R1-CFG-01..08, E2E-R1-UI-16, 35..36 (A-17)</t>
+          <t>Catalogue, floors, profiles, explainer (earlier); department overrides as layer 4 with tree inheritance (0021), profile switch plan/apply with If-Match, reason and step-up (CFG-017), effective-settings cache with generation invalidation over Valkey, never authoritative (CFG-004); Settings tabs for departments and profile. E2E-R1-CFG-01..08, E2E-R1-UI-16, 35..36 (A-17) Settings redesign (owner: crowded and confusing; docs/design/ia-competitive-analysis.md §6): category index with search, Advanced sections, unbuilt-feature keys hidden — in progress.</t>
         </is>
       </c>
     </row>
@@ -5053,7 +5080,7 @@
       <c r="N24" s="3" t="inlineStr"/>
       <c r="O24" s="3" t="inlineStr">
         <is>
-          <t>DataGrid v1 (web/src/ui/components/DataGrid.tsx): quick search, typed filter builder with chips and plain-language summary, multi-sort with order numbers, columns chooser, density, formula-safe CSV export audited via POST /exports, saved views per list (personal/shared, default, modified marker; migration 0028; /views API) with URL state, selection with shift-range and bulk actions, Enter/Space keyboard, live count, cards below 40rem; adopted by Library and Members. E2E-R1-VIEW-01, E2E-R1-UI-38, E2E-P0-10. Later: server-driven query + cursor paging, XLSX/async export, AND/OR groups, column resize.</t>
+          <t>DataGrid v1 (web/src/ui/components/DataGrid.tsx): quick search, typed filter builder with chips and plain-language summary, multi-sort with order numbers, columns chooser, density, formula-safe CSV export audited via POST /exports, saved views per list (personal/shared, default, modified marker; migration 0028; /views API) with URL state, selection with shift-range and bulk actions, Enter/Space keyboard, live count, cards below 40rem; adopted by Library and Members. E2E-R1-VIEW-01, E2E-R1-UI-38, E2E-P0-10. v2: AND/OR filter groups, views shared with roles (migration 0034), XLSX export (E2E-R1-13). Later: server-driven query + cursor paging, async export, column resize.</t>
         </is>
       </c>
     </row>
@@ -5248,7 +5275,7 @@
       <c r="N27" s="3" t="inlineStr"/>
       <c r="O27" s="3" t="inlineStr">
         <is>
-          <t>Web app on the Notion/Attio direction (owner choice): warm paper palette in tokens (contrast-checked), full-bleed pages with a warm icon sidebar, workspace + account menus (persisted theme), action-first Home (acknowledgements, reviews, announcements with inline actions, library table, activity, people), Library (filters, Attio-style table, New document dialog), document reading view with properties, lifecycle actions (edit, submit, approve, request changes, publish with step-up, new version), acknowledgement callout, Announcements feed with read/ack, Members with invite dialog; split sign-in with product preview; single-flight token refresh. E2E-R1-UI-01..10 with axe. Remaining: ⌘K command palette (search API is ready), system console shell, mobile bottom bar Second UI pass: Geist type, state kit (skeletons, empty states, load errors with retry), ⌘K palette over search + commands (E2E-R1-UI-12..13), admin screens: Manage announcements, Campaigns, Settings, Audit log, Overview, People &amp; access (E2E-R1-UI-14..17, 23); Policies portal and document governance (E2E-R1-UI-18..22). Remaining: system console shell, keyboard nav audit</t>
+          <t>Web app on the Notion/Attio direction (owner choice): warm paper palette in tokens (contrast-checked), full-bleed pages with a warm icon sidebar, workspace + account menus (persisted theme), action-first Home (acknowledgements, reviews, announcements with inline actions, library table, activity, people), Library (filters, Attio-style table, New document dialog), document reading view with properties, lifecycle actions (edit, submit, approve, request changes, publish with step-up, new version), acknowledgement callout, Announcements feed with read/ack, Members with invite dialog; split sign-in with product preview; single-flight token refresh. E2E-R1-UI-01..10 with axe. Second UI pass: Geist type, state kit (skeletons, empty states, load errors with retry), ⌘K palette over search + commands (E2E-R1-UI-12..13), admin screens: Manage announcements, Campaigns, Settings, Audit log, Overview, People &amp; access (E2E-R1-UI-14..17, 23); Policies portal and document governance (E2E-R1-UI-18..22). Keyboard-only journey (E2E-R1-19) and system console shell done. Remaining: persona IA redesign approved 2026-10-12 (docs/design/ia-competitive-analysis.md: persona sidebar, Admin hub, Needs-you Home, workspace onboarding) — in progress; mobile bottom bar</t>
         </is>
       </c>
     </row>
@@ -5305,7 +5332,7 @@
       </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L28" s="3" t="inlineStr"/>
@@ -5313,7 +5340,7 @@
       <c r="N28" s="3" t="inlineStr"/>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-01 setup page, E2E-R1-02 new workspaces with owner onboarding, E2E-R1-05 roles with collection scope, E2E-R1-03 accent branding with contrast-safe shades (logo and terminology pending), E2E-R1-04 directory import, E2E-R1-06 controlled policy SoD, step-up approve, scheduled go-live, superseded; E2E-R1-10 announcement approval and expiry, E2E-R1-07 re-ack at scale with evidence, E2E-R1-11 resumable 50 MB upload and links, E2E-R1-12 Files retention and held files, E2E-R1-13 DataGrid groups, shared views and exports, E2E-R1-18 startup day one with template packs, E2E-R1-08 new joiner gets open campaigns, E2E-R1-09 J14 location audience with confirm-by, campaign engine, one escalation, archive closes, E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-15 overview drill-downs, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO sweep (21 probes → 404, each audited as access.denied, A-31); plus complete flows E2E-R1-FLOW-01..06. Remaining: R1-01, 02, 05..07, 10..13, branding logo and terminology (R1-03), 15, 18 (several need branding, terminology, template packs, location audiences).</t>
+          <t>R1 gate pack started in the browser (packs/r1/gate.ui.spec.ts): E2E-R1-01 setup page, E2E-R1-02 new workspaces with owner onboarding, E2E-R1-05 roles with collection scope, E2E-R1-03 accent branding with contrast-safe shades (logo and terminology pending), E2E-R1-04 directory import, E2E-R1-06 controlled policy SoD, step-up approve, scheduled go-live, superseded; E2E-R1-10 announcement approval and expiry, E2E-R1-07 re-ack at scale with evidence, E2E-R1-11 resumable 50 MB upload and links, E2E-R1-12 Files retention and held files, E2E-R1-13 DataGrid groups, shared views and exports, E2E-R1-18 startup day one with template packs, E2E-R1-08 new joiner gets open campaigns, E2E-R1-09 J14 location audience with confirm-by, campaign engine, one escalation, archive closes, E2E-R1-16 deactivation, E2E-R1-14 audit trail in the browser, E2E-R1-15 overview drill-downs, E2E-R1-17 read-only workspace with banner, E2E-R1-19 keyboard only, E2E-R1-ISO sweep (21 probes → 404, each audited as access.denied, A-31); plus complete flows E2E-R1-FLOW-01..06. All 19 R1 scenarios green in the browser. Notes: R1-01 full bootstrap needs a fresh database (covered by E2E-R1-SYS-01); R1-18 plans the first campaign rather than creating it.</t>
         </is>
       </c>
     </row>
@@ -5439,7 +5466,7 @@
       <c r="N30" s="3" t="inlineStr"/>
       <c r="O30" s="3" t="inlineStr">
         <is>
-          <t>Vector masters (assets/brand/vector, generated by build.py: P-ribbon symbol, flat small symbol, horizontal and stacked lockups light/dark, app icons, banner; wordmark outlined from Geist, OFL); PNGs, favicons and ICO re-exported from them; the app uses the SVG symbol and an SVG favicon. Remaining: trademark search (OQ-01), professional mark review before GA</t>
+          <t>Vector masters (assets/brand/vector, generated by build.py: P-ribbon symbol, flat small symbol, horizontal and stacked lockups light/dark, app icons, banner; wordmark outlined from Geist, OFL); PNGs, favicons and ICO re-exported from them; the app uses the SVG symbol and an SVG favicon. Remaining: trademark search (OQ-01), professional mark review before GA Marketing site (site/, static, generated from tracker data and real screenshots: home, features, user flows, comparison, roadmap, security, open source); not published yet.</t>
         </is>
       </c>
     </row>
@@ -6471,7 +6498,7 @@
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L46" s="3" t="inlineStr"/>
@@ -6479,7 +6506,7 @@
       <c r="N46" s="3" t="inlineStr"/>
       <c r="O46" s="3" t="inlineStr">
         <is>
-          <t>System console (0022): workspaces grid with usage and quotas, suspend/reactivate/schedule deletion with step-up on the system chain, quota defaults per profile with the member quota enforced at invite, platform health, system audit explorer; console shell for system admins (metadata only, never workspace content). E2E-R1-SYS-01..09, E2E-R1-UI-40..41 (A-18)</t>
+          <t>System console (0022): workspaces grid with usage and quotas, suspend/reactivate/schedule deletion with step-up on the system chain, quota defaults per profile with the member quota enforced at invite, platform health, system audit explorer; console shell for system admins (metadata only, never workspace content). E2E-R1-SYS-01..09, E2E-R1-UI-40..41 (A-18) Remaining (docs/20 §3, CFG-006): email delivery (SMTP) settings with test send, public URL and sender, storage and scanning status, /setup continuing to email and the first workspace — next.</t>
         </is>
       </c>
     </row>
@@ -7467,13 +7494,17 @@
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="L62" s="3" t="inlineStr"/>
       <c r="M62" s="3" t="inlineStr"/>
       <c r="N62" s="3" t="inlineStr"/>
-      <c r="O62" s="3" t="inlineStr"/>
+      <c r="O62" s="3" t="inlineStr">
+        <is>
+          <t>P0 subset (A-38): built-in template packs (employee handbook, starter policies) installed as drafts with the right kind permissions, Templates gallery page; E2E-R1-18. Remaining: install wizard, Wave-1 process templates (need the designer and runtime).</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -10377,7 +10408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E393"/>
+  <dimension ref="A1:E398"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -18198,12 +18229,12 @@
       </c>
       <c r="B290" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-01</t>
+          <t>E2E-R1-UI-46</t>
         </is>
       </c>
       <c r="C290" s="3" t="inlineStr">
         <is>
-          <t>Onboarding start to finish: the owner invites from Members; the invitee opens the link from the email, creates an account (password confirmation checked) and lands on Home in the workspace; the link then no longer works; the owner sees them Active and opens their person page | BPMS-023</t>
+          <t>A person opens Account › Profile from the account menu, changes their name and time zone, saves, and the shell and a reload show the new values | BPMS-021</t>
         </is>
       </c>
       <c r="D290" s="3" t="inlineStr">
@@ -18225,12 +18256,12 @@
       </c>
       <c r="B291" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-02</t>
+          <t>E2E-R1-UI-47</t>
         </is>
       </c>
       <c r="C291" s="3" t="inlineStr">
         <is>
-          <t>Someone with an account opens the invitation email, signs in from the page, comes back to it and joins with one click; an unknown link explains itself | BPMS-023</t>
+          <t>An owner renames the workspace from Settings; the switcher shows the new name and it survives a reload (audited on both chains, AUD-01) | BPMS-020</t>
         </is>
       </c>
       <c r="D291" s="3" t="inlineStr">
@@ -18252,12 +18283,12 @@
       </c>
       <c r="B292" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-03</t>
+          <t>E2E-R1-UI-48</t>
         </is>
       </c>
       <c r="C292" s="3" t="inlineStr">
         <is>
-          <t>Policy to evidence: the owner writes and publishes a policy and launches a campaign; a colleague (invited the same way) sees the task on Home, opens the acknowledgement email link, acknowledges on the document; the owner sees them Done, 1 of 2, and downloads the evidence CSV | BPMS-040, 046</t>
+          <t>A member who forgot their password asks for a link, opens it from the email, sets a new password, and signs in with it (the old one fails) | BPMS-021</t>
         </is>
       </c>
       <c r="D292" s="3" t="inlineStr">
@@ -18279,12 +18310,12 @@
       </c>
       <c r="B293" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-04</t>
+          <t>E2E-R1-UI-49</t>
         </is>
       </c>
       <c r="C293" s="3" t="inlineStr">
         <is>
-          <t>Announcement: the owner composes a critical post that needs acknowledgement and publishes it; a colleague opens the email link while signed out, signs in, lands on the open post and confirms; the owner sees the receipt | BPMS-047</t>
+          <t>A member changes their password from Account › Security; a wrong current password is refused on the field; the session stays signed in | BPMS-021</t>
         </is>
       </c>
       <c r="D293" s="3" t="inlineStr">
@@ -18306,12 +18337,12 @@
       </c>
       <c r="B294" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-05</t>
+          <t>E2E-R1-UI-50</t>
         </is>
       </c>
       <c r="C294" s="3" t="inlineStr">
         <is>
-          <t>Review loop: the owner submits a controlled policy; the reviewer (invited as Reviewer) gets the review email, opens it and requests changes with a comment; the owner gets a notification quoting it, edits and resubmits; the reviewer approves from Home; the owner is told it is approved and publishes | BPMS-040</t>
+          <t>An owner requires a member to change their password (reason recorded); at the member's next sign-in they choose a new one and land on Home | BPMS-021</t>
         </is>
       </c>
       <c r="D294" s="3" t="inlineStr">
@@ -18333,12 +18364,12 @@
       </c>
       <c r="B295" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-06</t>
+          <t>E2E-R1-FLOW-01</t>
         </is>
       </c>
       <c r="C295" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval: a second admin joins from the invitation and turns on two-step verification; the owner sends a workspace-wide post for approval; the admin gets the approval email, opens it and sends it back with a note; the owner gets a notification with the note, edits and resubmits; the admin approves and publishes; the owner is told; the post is in the feed | BPMS-047</t>
+          <t>Onboarding start to finish: the owner invites from Members; the invitee opens the link from the email, creates an account (password confirmation checked) and lands on Home in the workspace; the link then no longer works; the owner sees them Active and opens their person page | BPMS-023</t>
         </is>
       </c>
       <c r="D295" s="3" t="inlineStr">
@@ -18360,12 +18391,12 @@
       </c>
       <c r="B296" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-01</t>
+          <t>E2E-R1-FLOW-02</t>
         </is>
       </c>
       <c r="C296" s="3" t="inlineStr">
         <is>
-          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
+          <t>Someone with an account opens the invitation email, signs in from the page, comes back to it and joins with one click; an unknown link explains itself | BPMS-023</t>
         </is>
       </c>
       <c r="D296" s="3" t="inlineStr">
@@ -18387,12 +18418,12 @@
       </c>
       <c r="B297" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-02</t>
+          <t>E2E-R1-FLOW-03</t>
         </is>
       </c>
       <c r="C297" s="3" t="inlineStr">
         <is>
-          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
+          <t>Policy to evidence: the owner writes and publishes a policy and launches a campaign; a colleague (invited the same way) sees the task on Home, opens the acknowledgement email link, acknowledges on the document; the owner sees them Done, 1 of 2, and downloads the evidence CSV | BPMS-040, 046</t>
         </is>
       </c>
       <c r="D297" s="3" t="inlineStr">
@@ -18414,12 +18445,12 @@
       </c>
       <c r="B298" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-03</t>
+          <t>E2E-R1-FLOW-04</t>
         </is>
       </c>
       <c r="C298" s="3" t="inlineStr">
         <is>
-          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
+          <t>Announcement: the owner composes a critical post that needs acknowledgement and publishes it; a colleague opens the email link while signed out, signs in, lands on the open post and confirms; the owner sees the receipt | BPMS-047</t>
         </is>
       </c>
       <c r="D298" s="3" t="inlineStr">
@@ -18441,12 +18472,12 @@
       </c>
       <c r="B299" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-04</t>
+          <t>E2E-R1-FLOW-05</t>
         </is>
       </c>
       <c r="C299" s="3" t="inlineStr">
         <is>
-          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
+          <t>Review loop: the owner submits a controlled policy; the reviewer (invited as Reviewer) gets the review email, opens it and requests changes with a comment; the owner gets a notification quoting it, edits and resubmits; the reviewer approves from Home; the owner is told it is approved and publishes | BPMS-040</t>
         </is>
       </c>
       <c r="D299" s="3" t="inlineStr">
@@ -18468,12 +18499,12 @@
       </c>
       <c r="B300" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-05</t>
+          <t>E2E-R1-FLOW-06</t>
         </is>
       </c>
       <c r="C300" s="3" t="inlineStr">
         <is>
-          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
+          <t>Announcement approval: a second admin joins from the invitation and turns on two-step verification; the owner sends a workspace-wide post for approval; the admin gets the approval email, opens it and sends it back with a note; the owner gets a notification with the note, edits and resubmits; the admin approves and publishes; the owner is told; the post is in the feed | BPMS-047</t>
         </is>
       </c>
       <c r="D300" s="3" t="inlineStr">
@@ -18495,12 +18526,12 @@
       </c>
       <c r="B301" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-06</t>
+          <t>E2E-R1-CMP-01</t>
         </is>
       </c>
       <c r="C301" s="3" t="inlineStr">
         <is>
-          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
+          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
         </is>
       </c>
       <c r="D301" s="3" t="inlineStr">
@@ -18522,12 +18553,12 @@
       </c>
       <c r="B302" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-07</t>
+          <t>E2E-R1-CMP-02</t>
         </is>
       </c>
       <c r="C302" s="3" t="inlineStr">
         <is>
-          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
+          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
         </is>
       </c>
       <c r="D302" s="3" t="inlineStr">
@@ -18549,12 +18580,12 @@
       </c>
       <c r="B303" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-01</t>
+          <t>E2E-R1-CMP-03</t>
         </is>
       </c>
       <c r="C303" s="3" t="inlineStr">
         <is>
-          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
+          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
         </is>
       </c>
       <c r="D303" s="3" t="inlineStr">
@@ -18576,12 +18607,12 @@
       </c>
       <c r="B304" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-02</t>
+          <t>E2E-R1-CMP-04</t>
         </is>
       </c>
       <c r="C304" s="3" t="inlineStr">
         <is>
-          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
+          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
         </is>
       </c>
       <c r="D304" s="3" t="inlineStr">
@@ -18603,12 +18634,12 @@
       </c>
       <c r="B305" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-03</t>
+          <t>E2E-R1-CMP-05</t>
         </is>
       </c>
       <c r="C305" s="3" t="inlineStr">
         <is>
-          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
+          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
         </is>
       </c>
       <c r="D305" s="3" t="inlineStr">
@@ -18630,12 +18661,12 @@
       </c>
       <c r="B306" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-04</t>
+          <t>E2E-R1-CMP-06</t>
         </is>
       </c>
       <c r="C306" s="3" t="inlineStr">
         <is>
-          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
+          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
         </is>
       </c>
       <c r="D306" s="3" t="inlineStr">
@@ -18657,12 +18688,12 @@
       </c>
       <c r="B307" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-05</t>
+          <t>E2E-R1-CMP-07</t>
         </is>
       </c>
       <c r="C307" s="3" t="inlineStr">
         <is>
-          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
+          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D307" s="3" t="inlineStr">
@@ -18684,12 +18715,12 @@
       </c>
       <c r="B308" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-06</t>
+          <t>E2E-R1-ANN-01</t>
         </is>
       </c>
       <c r="C308" s="3" t="inlineStr">
         <is>
-          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
+          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
         </is>
       </c>
       <c r="D308" s="3" t="inlineStr">
@@ -18711,12 +18742,12 @@
       </c>
       <c r="B309" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-01</t>
+          <t>E2E-R1-ANN-02</t>
         </is>
       </c>
       <c r="C309" s="3" t="inlineStr">
         <is>
-          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
+          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
         </is>
       </c>
       <c r="D309" s="3" t="inlineStr">
@@ -18738,12 +18769,12 @@
       </c>
       <c r="B310" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-02</t>
+          <t>E2E-R1-ANN-03</t>
         </is>
       </c>
       <c r="C310" s="3" t="inlineStr">
         <is>
-          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
+          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
         </is>
       </c>
       <c r="D310" s="3" t="inlineStr">
@@ -18765,12 +18796,12 @@
       </c>
       <c r="B311" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-03</t>
+          <t>E2E-R1-ANN-04</t>
         </is>
       </c>
       <c r="C311" s="3" t="inlineStr">
         <is>
-          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
+          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
         </is>
       </c>
       <c r="D311" s="3" t="inlineStr">
@@ -18792,12 +18823,12 @@
       </c>
       <c r="B312" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-01</t>
+          <t>E2E-R1-ANN-05</t>
         </is>
       </c>
       <c r="C312" s="3" t="inlineStr">
         <is>
-          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
+          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D312" s="3" t="inlineStr">
@@ -18819,12 +18850,12 @@
       </c>
       <c r="B313" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-02</t>
+          <t>E2E-R1-ANN-06</t>
         </is>
       </c>
       <c r="C313" s="3" t="inlineStr">
         <is>
-          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
+          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
         </is>
       </c>
       <c r="D313" s="3" t="inlineStr">
@@ -18846,12 +18877,12 @@
       </c>
       <c r="B314" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-03</t>
+          <t>E2E-R1-SRCH-01</t>
         </is>
       </c>
       <c r="C314" s="3" t="inlineStr">
         <is>
-          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
+          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
         </is>
       </c>
       <c r="D314" s="3" t="inlineStr">
@@ -18873,12 +18904,12 @@
       </c>
       <c r="B315" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-04</t>
+          <t>E2E-R1-SRCH-02</t>
         </is>
       </c>
       <c r="C315" s="3" t="inlineStr">
         <is>
-          <t>Chain verify reports intact | FR-T02</t>
+          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
         </is>
       </c>
       <c r="D315" s="3" t="inlineStr">
@@ -18900,12 +18931,12 @@
       </c>
       <c r="B316" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-05</t>
+          <t>E2E-R1-SRCH-03</t>
         </is>
       </c>
       <c r="C316" s="3" t="inlineStr">
         <is>
-          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
+          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
         </is>
       </c>
       <c r="D316" s="3" t="inlineStr">
@@ -18927,12 +18958,12 @@
       </c>
       <c r="B317" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-06</t>
+          <t>E2E-R1-AUDX-01</t>
         </is>
       </c>
       <c r="C317" s="3" t="inlineStr">
         <is>
-          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
+          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
         </is>
       </c>
       <c r="D317" s="3" t="inlineStr">
@@ -18954,12 +18985,12 @@
       </c>
       <c r="B318" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-07</t>
+          <t>E2E-R1-AUDX-02</t>
         </is>
       </c>
       <c r="C318" s="3" t="inlineStr">
         <is>
-          <t>`POST /audit/query`: an AND group (category, action prefix, within P30D) sorted ascending pages by cursor; an OR group returns only matching events; unknown fields or values, bad durations, nesting deeper than 2 and unsupported sorts → 422 | BPMS-064, docs/08 §7.5</t>
+          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
         </is>
       </c>
       <c r="D318" s="3" t="inlineStr">
@@ -18981,12 +19012,12 @@
       </c>
       <c r="B319" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-08</t>
+          <t>E2E-R1-AUDX-03</t>
         </is>
       </c>
       <c r="C319" s="3" t="inlineStr">
         <is>
-          <t>A background export (202) runs as a job, finishes `done` with rows, its CSV downloads through the requester's signed file link, the requester is notified, and both `audit.export_requested` and `audit.exported` are recorded | BPMS-064, FR-T04</t>
+          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
         </is>
       </c>
       <c r="D319" s="3" t="inlineStr">
@@ -19008,12 +19039,12 @@
       </c>
       <c r="B320" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-AUDX-04</t>
         </is>
       </c>
       <c r="C320" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work (browser: /setup refuses a bad token or says the platform is already set up; no default account signs in; the full first run needs a fresh database, since the shared E2E database already has system admins) | FR-S01</t>
+          <t>Chain verify reports intact | FR-T02</t>
         </is>
       </c>
       <c r="D320" s="3" t="inlineStr">
@@ -19035,12 +19066,12 @@
       </c>
       <c r="B321" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-AUDX-05</t>
         </is>
       </c>
       <c r="C321" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA (browser: System › New workspace twice; owner A opens the emailed link, creates the account, turns on two-step verification, signs in and lands in the workspace) | FR-S02/S03, FR-W01</t>
+          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
         </is>
       </c>
       <c r="D321" s="3" t="inlineStr">
@@ -19062,12 +19093,12 @@
       </c>
       <c r="B322" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-AUDX-06</t>
         </is>
       </c>
       <c r="C322" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email (built: a too-light accent shows a live contrast note with the shade text will use; the server derives 4.5:1 text and 3:1 focus shades; every member's app paints them; a logo uploaded in Settings shows in everyone's sidebar; renaming SOP to "Work Instruction" in Settings › Terminology changes the labels other members see; "Request" has no screens until M6, so its override is covered at unit level) | FR-W04, 05 §7</t>
+          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
         </is>
       </c>
       <c r="D322" s="3" t="inlineStr">
@@ -19089,12 +19120,12 @@
       </c>
       <c r="B323" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-AUDX-07</t>
         </is>
       </c>
       <c r="C323" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error (browser: Members › Import directory › Check shows each row; cycle and unknown member refused; Apply saves the rest; person pages show department, manager and location) | FR-W02</t>
+          <t>`POST /audit/query`: an AND group (category, action prefix, within P30D) sorted ascending pages by cursor; an OR group returns only matching events; unknown fields or values, bad durations, nesting deeper than 2 and unsupported sorts → 422 | BPMS-064, docs/08 §7.5</t>
         </is>
       </c>
       <c r="D323" s="3" t="inlineStr">
@@ -19116,12 +19147,12 @@
       </c>
       <c r="B324" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-AUDX-08</t>
         </is>
       </c>
       <c r="C324" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused (browser: Roles &amp; access › Duplicate › grant to a person for the HR collection; a permission change previews "1 person gains 1 permission"; the holder gets Edit on the HR draft but not the Finance one, and the API agrees; a role manager who lacks audit export cannot put it into a role (403 escalation)) | FR-W03, J6</t>
+          <t>A background export (202) runs as a job, finishes `done` with rows, its CSV downloads through the requester's signed file link, the requester is notified, and both `audit.export_requested` and `audit.exported` are recorded | BPMS-064, FR-T04</t>
         </is>
       </c>
       <c r="D324" s="3" t="inlineStr">
@@ -19143,12 +19174,12 @@
       </c>
       <c r="B325" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C325" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF (browser: the author's Approve is refused; the reviewer confirms with their password after an aged sign-in; Publish › Goes live schedules v2; `/__test/library/due` makes it due without moving the shared clock; v1's printable export carries the Superseded banner) | FR-G04/G05/G10, FR-PL01</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work (browser: /setup refuses a bad token or says the platform is already set up; no default account signs in; the full first run needs a fresh database, since the shared E2E database already has system admins) | FR-S01</t>
         </is>
       </c>
       <c r="D325" s="3" t="inlineStr">
@@ -19170,12 +19201,12 @@
       </c>
       <c r="B326" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C326" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method (browser: the owner publishes v2.0 as major, 51 asked; 10 people acknowledge at 390×844 from Home, 40 through the same API; the campaign shows 50 of 51 and the evidence CSV lists the v2 hash and sign-in method for all 50) | FR-PL03, FR-AK01–04</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA (browser: System › New workspace twice; owner A opens the emailed link, creates the account, turns on two-step verification, signs in and lands in the workspace) | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D326" s="3" t="inlineStr">
@@ -19197,12 +19228,12 @@
       </c>
       <c r="B327" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C327" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns (browser: a campaign created with "Also ask people who join later" on; a new hire who joins from the invitation email after launch finds the request on Home, acknowledges, and shows Done) | FR-AK03</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email (built: a too-light accent shows a live contrast note with the shade text will use; the server derives 4.5:1 text and 3:1 focus shades; every member's app paints them; a logo uploaded in Settings shows in everyone's sidebar; renaming SOP to "Work Instruction" in Settings › Terminology changes the labels other members see; "Request" has no screens until M6, so its override is covered at unit level) | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D327" s="3" t="inlineStr">
@@ -19224,12 +19255,12 @@
       </c>
       <c r="B328" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C328" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct (browser: location audience from the directory, confirm-by date, only Bangalore members receive it; the announcement's campaign counts the confirmation; past the deadline the manager of the member who did not confirm is told exactly once; archiving closes the campaign) | FR-AN01–06, J14</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error (browser: Members › Import directory › Check shows each row; cycle and unknown member refused; Apply saves the rest; person pages show department, manager and location) | FR-W02</t>
         </is>
       </c>
       <c r="D328" s="3" t="inlineStr">
@@ -19251,12 +19282,12 @@
       </c>
       <c r="B329" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C329" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it (browser: the drawer says approval is needed, the author sends it, a second admin approves, members see it; at expiry it leaves the feed and admins see it as Expired) | FX-C01, FR-AN03</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused (browser: Roles &amp; access › Duplicate › grant to a person for the HR collection; a permission change previews "1 person gains 1 permission"; the holder gets Edit on the HR draft but not the Finance one, and the API agrees; a role manager who lacks audit export cannot put it into a role (403 escalation)) | FR-W03, J6</t>
         </is>
       </c>
       <c r="D329" s="3" t="inlineStr">
@@ -19278,12 +19309,12 @@
       </c>
       <c r="B330" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C330" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B (browser: a 50 MB attachment with one chunk dropped resumes and its SHA-256 matches; EICAR shows quarantined and gets no link; links last ≤ 5 minutes, a tampered link is refused, workspace B gets 404 for the link and the file) | FR-F01–F03, SEC-10</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF (browser: the author's Approve is refused; the reviewer confirms with their password after an aged sign-in; Publish › Goes live schedules v2; `/__test/library/due` makes it due without moving the shared clock; v1's printable export carries the Superseded banner) | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D330" s="3" t="inlineStr">
@@ -19305,12 +19336,12 @@
       </c>
       <c r="B331" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C331" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused (browser: Quarantined chip and a Name filter; two files changed to Operational with a reason, shown as set by an admin and audited; deleting a file a published version holds is refused) | FR-F06, FR-V</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method (browser: the owner publishes v2.0 as major, 51 asked; 10 people acknowledge at 390×844 from Home, 40 through the same API; the campaign shows 50 of 51 and the evidence CSV lists the v2 hash and sign-in method for all 50) | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D331" s="3" t="inlineStr">
@@ -19332,12 +19363,12 @@
       </c>
       <c r="B332" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C332" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction (browser: Status is Published and (Name contains Alpha or Charlie); sort by type then name; view shared with Reviewers opens from the deep link for a reviewer; CSV has exactly the shown rows; XLSX downloads) | FR-V01–V07</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns (browser: a campaign created with "Also ask people who join later" on; a new hire who joins from the invitation email after launch finds the request on Home, acknowledges, and shows Done) | FR-AK03</t>
         </is>
       </c>
       <c r="D332" s="3" t="inlineStr">
@@ -19359,12 +19390,12 @@
       </c>
       <c r="B333" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C333" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK (browser: Person filter shows only that person's events; a version's timeline is oldest first: three edits, submitted, published; the page shows Chain verified) | FR-T01–T04</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct (browser: location audience from the directory, confirm-by date, only Bangalore members receive it; the announcement's campaign counts the confirmation; past the deadline the manager of the member who did not confirm is told exactly once; archiving closes the campaign) | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D333" s="3" t="inlineStr">
@@ -19386,12 +19417,12 @@
       </c>
       <c r="B334" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C334" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts (browser: open acknowledgements → active campaigns with the same "still to acknowledge"; versions published → audit log filtered to publications with the same event count; announcements published → the Published tab; without two-step → People &amp; access filtered with the same count) | FR-A01</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it (browser: the drawer says approval is needed, the author sends it, a second admin approves, members see it; at expiry it leaves the feed and admins see it as Expired) | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D334" s="3" t="inlineStr">
@@ -19413,12 +19444,12 @@
       </c>
       <c r="B335" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C335" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act (browser: owner deactivates from the person page; the member's open tab is sent to the chooser on the next page; signing in again offers no workspace; the API refuses entry) | SEC-04, FR-W01</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B (browser: a 50 MB attachment with one chunk dropped resumes and its SHA-256 matches; EICAR shows quarantined and gets no link; links last ≤ 5 minutes, a tampered link is refused, workspace B gets 404 for the link and the file) | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D335" s="3" t="inlineStr">
@@ -19440,12 +19471,12 @@
       </c>
       <c r="B336" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C336" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore (browser: reads keep working; the first change is refused and a read-only banner appears on every page; after restore the banner is gone and changes work) | FR-S02, J8</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused (browser: Quarantined chip and a Name filter; two files changed to Operational with a reason, shown as set by an admin and audited; deleting a file a published version holds is refused) | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D336" s="3" t="inlineStr">
@@ -19467,12 +19498,12 @@
       </c>
       <c r="B337" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C337" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock (browser: Home › Browse templates › Install the handbook pack (5 drafts) → publish the handbook → launch the campaign → 20 people at 390×844 acknowledge; 20 of 21 done, within 15 minutes) | J12</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction (browser: Status is Published and (Name contains Alpha or Charlie); sort by type then name; view shared with Reviewers opens from the deep link for a reviewer; CSV has exactly the shown rows; XLSX downloads) | FR-V01–V07</t>
         </is>
       </c>
       <c r="D337" s="3" t="inlineStr">
@@ -19494,12 +19525,12 @@
       </c>
       <c r="B338" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C338" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse (browser: Tab/Enter/typing only, author from Library to Published, colleague from sign-in to Acknowledged) | A11Y-01, T10</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK (browser: Person filter shows only that person's events; a version's timeline is oldest first: three edits, submitted, published; the page shows Chain verified) | FR-T01–T04</t>
         </is>
       </c>
       <c r="D338" s="3" t="inlineStr">
@@ -19521,12 +19552,12 @@
       </c>
       <c r="B339" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C339" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` (built: B's owner probes 21 reads and writes on A's documents, versions, exports, campaigns, announcements, collections, departments, views, files and members → all 404, each recorded in B's audit log as `access.denied` with the object id, B's chain verifies, A unchanged) | SEC-01/02</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts (browser: open acknowledgements → active campaigns with the same "still to acknowledge"; versions published → audit log filtered to publications with the same event count; announcements published → the Published tab; without two-step → People &amp; access filtered with the same count) | FR-A01</t>
         </is>
       </c>
       <c r="D339" s="3" t="inlineStr">
@@ -19548,12 +19579,12 @@
       </c>
       <c r="B340" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C340" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act (browser: owner deactivates from the person page; the member's open tab is sent to the chooser on the next page; signing in again offers no workspace; the API refuses entry) | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D340" s="3" t="inlineStr">
@@ -19575,12 +19606,12 @@
       </c>
       <c r="B341" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C341" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore (browser: reads keep working; the first change is refused and a read-only banner appears on every page; after restore the banner is gone and changes work) | FR-S02, J8</t>
         </is>
       </c>
       <c r="D341" s="3" t="inlineStr">
@@ -19602,12 +19633,12 @@
       </c>
       <c r="B342" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C342" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock (browser: Home › Browse templates › Install the handbook pack (5 drafts) → publish the handbook → launch the campaign → 20 people at 390×844 acknowledge; 20 of 21 done, within 15 minutes) | J12</t>
         </is>
       </c>
       <c r="D342" s="3" t="inlineStr">
@@ -19629,12 +19660,12 @@
       </c>
       <c r="B343" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C343" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse (browser: Tab/Enter/typing only, author from Library to Published, colleague from sign-in to Acknowledged) | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D343" s="3" t="inlineStr">
@@ -19656,12 +19687,12 @@
       </c>
       <c r="B344" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C344" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` (built: B's owner probes 21 reads and writes on A's documents, versions, exports, campaigns, announcements, collections, departments, views, files and members → all 404, each recorded in B's audit log as `access.denied` with the object id, B's chain verifies, A unchanged) | SEC-01/02</t>
         </is>
       </c>
       <c r="D344" s="3" t="inlineStr">
@@ -19683,12 +19714,12 @@
       </c>
       <c r="B345" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C345" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D345" s="3" t="inlineStr">
@@ -19710,12 +19741,12 @@
       </c>
       <c r="B346" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C346" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D346" s="3" t="inlineStr">
@@ -19737,12 +19768,12 @@
       </c>
       <c r="B347" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C347" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D347" s="3" t="inlineStr">
@@ -19764,12 +19795,12 @@
       </c>
       <c r="B348" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C348" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D348" s="3" t="inlineStr">
@@ -19791,12 +19822,12 @@
       </c>
       <c r="B349" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C349" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D349" s="3" t="inlineStr">
@@ -19818,12 +19849,12 @@
       </c>
       <c r="B350" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C350" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D350" s="3" t="inlineStr">
@@ -19845,12 +19876,12 @@
       </c>
       <c r="B351" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C351" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D351" s="3" t="inlineStr">
@@ -19872,12 +19903,12 @@
       </c>
       <c r="B352" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C352" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D352" s="3" t="inlineStr">
@@ -19899,12 +19930,12 @@
       </c>
       <c r="B353" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C353" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D353" s="3" t="inlineStr">
@@ -19926,12 +19957,12 @@
       </c>
       <c r="B354" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C354" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D354" s="3" t="inlineStr">
@@ -19953,12 +19984,12 @@
       </c>
       <c r="B355" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C355" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D355" s="3" t="inlineStr">
@@ -19980,12 +20011,12 @@
       </c>
       <c r="B356" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C356" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D356" s="3" t="inlineStr">
@@ -20007,12 +20038,12 @@
       </c>
       <c r="B357" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C357" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D357" s="3" t="inlineStr">
@@ -20034,12 +20065,12 @@
       </c>
       <c r="B358" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C358" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D358" s="3" t="inlineStr">
@@ -20061,12 +20092,12 @@
       </c>
       <c r="B359" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C359" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D359" s="3" t="inlineStr">
@@ -20088,12 +20119,12 @@
       </c>
       <c r="B360" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C360" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D360" s="3" t="inlineStr">
@@ -20115,12 +20146,12 @@
       </c>
       <c r="B361" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C361" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D361" s="3" t="inlineStr">
@@ -20142,12 +20173,12 @@
       </c>
       <c r="B362" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C362" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D362" s="3" t="inlineStr">
@@ -20169,12 +20200,12 @@
       </c>
       <c r="B363" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C363" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D363" s="3" t="inlineStr">
@@ -20196,12 +20227,12 @@
       </c>
       <c r="B364" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C364" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D364" s="3" t="inlineStr">
@@ -20223,12 +20254,12 @@
       </c>
       <c r="B365" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C365" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D365" s="3" t="inlineStr">
@@ -20250,12 +20281,12 @@
       </c>
       <c r="B366" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C366" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D366" s="3" t="inlineStr">
@@ -20277,12 +20308,12 @@
       </c>
       <c r="B367" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C367" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D367" s="3" t="inlineStr">
@@ -20304,12 +20335,12 @@
       </c>
       <c r="B368" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C368" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D368" s="3" t="inlineStr">
@@ -20331,12 +20362,12 @@
       </c>
       <c r="B369" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C369" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D369" s="3" t="inlineStr">
@@ -20358,12 +20389,12 @@
       </c>
       <c r="B370" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C370" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D370" s="3" t="inlineStr">
@@ -20385,12 +20416,12 @@
       </c>
       <c r="B371" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C371" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D371" s="3" t="inlineStr">
@@ -20412,12 +20443,12 @@
       </c>
       <c r="B372" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C372" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D372" s="3" t="inlineStr">
@@ -20439,12 +20470,12 @@
       </c>
       <c r="B373" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C373" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D373" s="3" t="inlineStr">
@@ -20466,12 +20497,12 @@
       </c>
       <c r="B374" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C374" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D374" s="3" t="inlineStr">
@@ -20493,12 +20524,12 @@
       </c>
       <c r="B375" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C375" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D375" s="3" t="inlineStr">
@@ -20520,12 +20551,12 @@
       </c>
       <c r="B376" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C376" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D376" s="3" t="inlineStr">
@@ -20547,12 +20578,12 @@
       </c>
       <c r="B377" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C377" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D377" s="3" t="inlineStr">
@@ -20574,12 +20605,12 @@
       </c>
       <c r="B378" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C378" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D378" s="3" t="inlineStr">
@@ -20601,12 +20632,12 @@
       </c>
       <c r="B379" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C379" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D379" s="3" t="inlineStr">
@@ -20628,12 +20659,12 @@
       </c>
       <c r="B380" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C380" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D380" s="3" t="inlineStr">
@@ -20655,12 +20686,12 @@
       </c>
       <c r="B381" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C381" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D381" s="3" t="inlineStr">
@@ -20682,12 +20713,12 @@
       </c>
       <c r="B382" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C382" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D382" s="3" t="inlineStr">
@@ -20709,12 +20740,12 @@
       </c>
       <c r="B383" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C383" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D383" s="3" t="inlineStr">
@@ -20736,12 +20767,12 @@
       </c>
       <c r="B384" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C384" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D384" s="3" t="inlineStr">
@@ -20763,12 +20794,12 @@
       </c>
       <c r="B385" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C385" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D385" s="3" t="inlineStr">
@@ -20790,12 +20821,12 @@
       </c>
       <c r="B386" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R4-11</t>
         </is>
       </c>
       <c r="C386" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
         </is>
       </c>
       <c r="D386" s="3" t="inlineStr">
@@ -20817,12 +20848,12 @@
       </c>
       <c r="B387" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R4-ISO</t>
         </is>
       </c>
       <c r="C387" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
         </is>
       </c>
       <c r="D387" s="3" t="inlineStr">
@@ -20844,12 +20875,12 @@
       </c>
       <c r="B388" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R5-01</t>
         </is>
       </c>
       <c r="C388" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
         </is>
       </c>
       <c r="D388" s="3" t="inlineStr">
@@ -20871,12 +20902,12 @@
       </c>
       <c r="B389" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R5-02</t>
         </is>
       </c>
       <c r="C389" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
         </is>
       </c>
       <c r="D389" s="3" t="inlineStr">
@@ -20898,12 +20929,12 @@
       </c>
       <c r="B390" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R5-03</t>
         </is>
       </c>
       <c r="C390" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
         </is>
       </c>
       <c r="D390" s="3" t="inlineStr">
@@ -20925,12 +20956,12 @@
       </c>
       <c r="B391" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R5-04</t>
         </is>
       </c>
       <c r="C391" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
         </is>
       </c>
       <c r="D391" s="3" t="inlineStr">
@@ -20952,12 +20983,12 @@
       </c>
       <c r="B392" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R5-05</t>
         </is>
       </c>
       <c r="C392" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
         </is>
       </c>
       <c r="D392" s="3" t="inlineStr">
@@ -20979,20 +21010,155 @@
       </c>
       <c r="B393" s="3" t="inlineStr">
         <is>
+          <t>E2E-R5-06</t>
+        </is>
+      </c>
+      <c r="C393" s="3" t="inlineStr">
+        <is>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+        </is>
+      </c>
+      <c r="D393" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E393" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B394" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-07</t>
+        </is>
+      </c>
+      <c r="C394" s="3" t="inlineStr">
+        <is>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+        </is>
+      </c>
+      <c r="D394" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E394" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B395" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-08</t>
+        </is>
+      </c>
+      <c r="C395" s="3" t="inlineStr">
+        <is>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+        </is>
+      </c>
+      <c r="D395" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E395" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B396" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-09</t>
+        </is>
+      </c>
+      <c r="C396" s="3" t="inlineStr">
+        <is>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+        </is>
+      </c>
+      <c r="D396" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E396" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B397" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C397" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D397" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E397" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B398" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C393" s="3" t="inlineStr">
+      <c r="C398" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D393" s="3" t="inlineStr">
+      <c r="D398" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E393" s="3" t="inlineStr">
+      <c r="E398" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
chore(tracker): directory UI, settings redesign and persona navigation done
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -197,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E41" headerRowCount="1">
-  <autoFilter ref="A1:E41"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E43" headerRowCount="1">
+  <autoFilter ref="A1:E43"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Source"/>
     <tableColumn id="2" name="ID"/>
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E398" headerRowCount="1">
-  <autoFilter ref="A1:E398"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E407" headerRowCount="1">
+  <autoFilter ref="A1:E407"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -1393,7 +1393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2467,6 +2467,60 @@
       <c r="E41" s="3" t="inlineStr">
         <is>
           <t>Treat system accounts like any other; count admin links; revoke sessions on "require change"; a separate system mail table</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>A-41 (BPMS-023)</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Reactivating a deactivated member (`POST /members/{id}/reactivate`): deactivation removes nothing, so reactivation restores the membership with the role grants (unexpired, at any scope, direct or through a group), group memberships and directory fields it had. Because that restores access, it is treated like granting it: `member:deactivate` on the member, a recent verification (step-up) and a reason (1–500 characters, recorded in `member.reactivated` with the restored role keys); the actor must hold every permission of those roles (the invitation rule, so an admin cannot bring back an owner); a disabled account is refused (a system administrator restores it first); the member takes a seat under the member quota. It emits `membership.reactivated.v1`, which nothing consumes yet: dynamic campaigns are not re-enrolled and nobody is notified. Inviting the person again still works and adds the invited roles to the old ones.</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Reset roles on reactivation; re-enrol dynamic campaigns; tell the person</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>A-43</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Role presets for jobs (HR lead, Finance lead, Engineering lead, Manager, Communications, Security &amp; IT) are custom roles created on first use, not built-in templates: built-in roles don't cover HR (announcements). Editable afterwards.</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Owner direction 2026-10-12</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -4747,7 +4801,7 @@
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L19" s="3" t="inlineStr"/>
@@ -4755,7 +4809,7 @@
       <c r="N19" s="3" t="inlineStr"/>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>procera-members + /api/v1: memberships, invitations (hashed + sealed tokens, 7-day expiry, email-bound, single use; list, revoke, resend), register-by-invite, owner onboarding activates the workspace, workspace switch (ws-scoped JWT), deactivation guards, state gate (423). Directory (migration 0008): department tree (uuid[] paths, sibling-unique names, no moves under descendants), static groups, positions (behind directory.positions.enabled), manager links with cycle rejection, deterministic manager resolution (explicit → nearest department head), per-field source attribution, CSV import with plan/apply. All audited; E2E-R1-MEM-01..03,05..07, E2E-R1-DIR-01..04 Invitation page /invite (GET /invitations/preview, A-24): create account and join, or sign in and join; deep links survive sign-in. E2E-R1-FLOW-01, 02. Directory import UI with a check step and per-row reasons (E2E-R1-04); deactivate from the person page with immediate session exit (E2E-R1-16); person page with department, manager and location. Remaining (owner: user management missing): directory UI to create, rename and move departments and groups, editable person profile, reactivate, bulk set — in progress.</t>
+          <t>procera-members + /api/v1: memberships, invitations (hashed + sealed tokens, 7-day expiry, email-bound, single use; list, revoke, resend), register-by-invite, owner onboarding activates the workspace, workspace switch (ws-scoped JWT), deactivation guards, state gate (423). Directory (migration 0008): department tree (uuid[] paths, sibling-unique names, no moves under descendants), static groups, positions (behind directory.positions.enabled), manager links with cycle rejection, deterministic manager resolution (explicit → nearest department head), per-field source attribution, CSV import with plan/apply. All audited; E2E-R1-MEM-01..03,05..07, E2E-R1-DIR-01..04 Invitation page /invite (GET /invitations/preview, A-24): create account and join, or sign in and join; deep links survive sign-in. E2E-R1-FLOW-01, 02. Directory import UI with a check step and per-row reasons (E2E-R1-04); deactivate from the person page with immediate session exit (E2E-R1-16); person page with department, manager and location. Directory UI: Departments page (tree, add, rename, move, head, delete only when empty), Groups (list, group page, members), editable person profile with groups, reactivate with step-up and reason (A-41), resend and revoke invitations, bulk set department and add to group. E2E-R1-UI-51..55. Later: people list per department, Used by, group owners.</t>
         </is>
       </c>
     </row>
@@ -5015,7 +5069,7 @@
       <c r="N23" s="3" t="inlineStr"/>
       <c r="O23" s="3" t="inlineStr">
         <is>
-          <t>Catalogue, floors, profiles, explainer (earlier); department overrides as layer 4 with tree inheritance (0021), profile switch plan/apply with If-Match, reason and step-up (CFG-017), effective-settings cache with generation invalidation over Valkey, never authoritative (CFG-004); Settings tabs for departments and profile. E2E-R1-CFG-01..08, E2E-R1-UI-16, 35..36 (A-17) Settings redesign (owner: crowded and confusing; docs/design/ia-competitive-analysis.md §6): category index with search, Advanced sections, unbuilt-feature keys hidden — in progress.</t>
+          <t>Catalogue, floors, profiles, explainer (earlier); department overrides as layer 4 with tree inheritance (0021), profile switch plan/apply with If-Match, reason and step-up (CFG-017), effective-settings cache with generation invalidation over Valkey, never authoritative (CFG-004); Settings tabs for departments and profile. E2E-R1-CFG-01..08, E2E-R1-UI-16, 35..36 (A-17) Settings redesign (owner: crowded and confusing; docs/design/ia-competitive-analysis.md §6): seven category pages with search, Advanced sections, unbuilt-feature keys and choices hidden, department overrides on each setting, starting-point banner. E2E-R1-UI-61, 35, 36.</t>
         </is>
       </c>
     </row>
@@ -5275,7 +5329,7 @@
       <c r="N27" s="3" t="inlineStr"/>
       <c r="O27" s="3" t="inlineStr">
         <is>
-          <t>Web app on the Notion/Attio direction (owner choice): warm paper palette in tokens (contrast-checked), full-bleed pages with a warm icon sidebar, workspace + account menus (persisted theme), action-first Home (acknowledgements, reviews, announcements with inline actions, library table, activity, people), Library (filters, Attio-style table, New document dialog), document reading view with properties, lifecycle actions (edit, submit, approve, request changes, publish with step-up, new version), acknowledgement callout, Announcements feed with read/ack, Members with invite dialog; split sign-in with product preview; single-flight token refresh. E2E-R1-UI-01..10 with axe. Second UI pass: Geist type, state kit (skeletons, empty states, load errors with retry), ⌘K palette over search + commands (E2E-R1-UI-12..13), admin screens: Manage announcements, Campaigns, Settings, Audit log, Overview, People &amp; access (E2E-R1-UI-14..17, 23); Policies portal and document governance (E2E-R1-UI-18..22). Keyboard-only journey (E2E-R1-19) and system console shell done. Remaining: persona IA redesign approved 2026-10-12 (docs/design/ia-competitive-analysis.md: persona sidebar, Admin hub, Needs-you Home, workspace onboarding) — in progress; mobile bottom bar</t>
+          <t>Web app on the Notion/Attio direction (owner choice): warm paper palette in tokens (contrast-checked), full-bleed pages with a warm icon sidebar, workspace + account menus (persisted theme), action-first Home (acknowledgements, reviews, announcements with inline actions, library table, activity, people), Library (filters, Attio-style table, New document dialog), document reading view with properties, lifecycle actions (edit, submit, approve, request changes, publish with step-up, new version), acknowledgement callout, Announcements feed with read/ack, Members with invite dialog; split sign-in with product preview; single-flight token refresh. E2E-R1-UI-01..10 with axe. Second UI pass: Geist type, state kit (skeletons, empty states, load errors with retry), ⌘K palette over search + commands (E2E-R1-UI-12..13), admin screens: Manage announcements, Campaigns, Settings, Audit log, Overview, People &amp; access (E2E-R1-UI-14..17, 23); Policies portal and document governance (E2E-R1-UI-18..22). Keyboard-only journey (E2E-R1-19) and system console shell done. Remaining: persona IA redesign approved 2026-10-12 (docs/design/ia-competitive-analysis.md: persona sidebar, Admin hub, Needs-you Home, workspace onboarding) done: persona sidebar, Admin hub and admin mode, Library and Announcements views, Needs you Home, workspace onboarding checklist and /welcome (E2E-R1-UI-62..63). Remaining: role cards on Home, mobile bottom bar</t>
         </is>
       </c>
     </row>
@@ -10408,7 +10462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E398"/>
+  <dimension ref="A1:E407"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -17451,7 +17505,7 @@
       </c>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>Settings: change a value in place with a reason and see why it applies; a step-up key asks to confirm identity | BPMS-031, BPMS-027</t>
+          <t>Settings (Sign-in &amp; security page): change a value in place with a reason and see why it applies; a step-up key asks to confirm identity | BPMS-031, BPMS-027</t>
         </is>
       </c>
       <c r="D261" s="3" t="inlineStr">
@@ -18018,7 +18072,7 @@
       </c>
       <c r="C282" s="3" t="inlineStr">
         <is>
-          <t>Departments: override a setting for a parent department, see a child inherit it, then clear it | BPMS-027</t>
+          <t>Departments: from a setting's "Same for all departments" chip, override it for a parent department, see a child inherit it, then use the workspace value again | BPMS-027</t>
         </is>
       </c>
       <c r="D282" s="3" t="inlineStr">
@@ -18045,7 +18099,7 @@
       </c>
       <c r="C283" s="3" t="inlineStr">
         <is>
-          <t>Configuration profile: preview a switch with every change, then switch with a reason | BPMS-027, CFG-017</t>
+          <t>Starting point: from the Settings index banner, preview a switch with every change, then switch with a reason | BPMS-027, CFG-017</t>
         </is>
       </c>
       <c r="D283" s="3" t="inlineStr">
@@ -18261,7 +18315,7 @@
       </c>
       <c r="C291" s="3" t="inlineStr">
         <is>
-          <t>An owner renames the workspace from Settings; the switcher shows the new name and it survives a reload (audited on both chains, AUD-01) | BPMS-020</t>
+          <t>An owner renames the workspace from Settings › General &amp; branding; the switcher shows the new name and it survives a reload (audited on both chains, AUD-01) | BPMS-020</t>
         </is>
       </c>
       <c r="D291" s="3" t="inlineStr">
@@ -18364,12 +18418,12 @@
       </c>
       <c r="B295" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-01</t>
+          <t>E2E-R1-UI-51</t>
         </is>
       </c>
       <c r="C295" s="3" t="inlineStr">
         <is>
-          <t>Onboarding start to finish: the owner invites from Members; the invitee opens the link from the email, creates an account (password confirmation checked) and lands on Home in the workspace; the link then no longer works; the owner sees them Active and opens their person page | BPMS-023</t>
+          <t>Departments (Admin → People): the empty state offers Add department and Import from CSV; an owner adds a department and one inside it with a head (a name with "/" is refused as typed), renames it inline, cannot delete the parent while it holds a sub-department (the dialog says what to move) nor move it under its own sub-department (not offered, with the reason), moves the child to the top level and deletes the now-empty parent | BPMS-023</t>
         </is>
       </c>
       <c r="D295" s="3" t="inlineStr">
@@ -18391,12 +18445,12 @@
       </c>
       <c r="B296" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-02</t>
+          <t>E2E-R1-UI-52</t>
         </is>
       </c>
       <c r="C296" s="3" t="inlineStr">
         <is>
-          <t>Someone with an account opens the invitation email, signs in from the page, comes back to it and joins with one click; an unknown link explains itself | BPMS-023</t>
+          <t>Groups (Admin → People): the empty state explains groups versus departments; an owner creates a group with a purpose, adds two people with the multi-select picker (searchable), removes one after confirming, sees name, purpose and member count in the list, and deletes the group | BPMS-023</t>
         </is>
       </c>
       <c r="D296" s="3" t="inlineStr">
@@ -18418,12 +18472,12 @@
       </c>
       <c r="B297" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-03</t>
+          <t>E2E-R1-UI-53</t>
         </is>
       </c>
       <c r="C297" s="3" t="inlineStr">
         <is>
-          <t>Policy to evidence: the owner writes and publishes a policy and launches a campaign; a colleague (invited the same way) sees the task on Home, opens the acknowledgement email link, acknowledges on the document; the owner sees them Done, 1 of 2, and downloads the evidence CSV | BPMS-040, 046</t>
+          <t>Person page: an owner edits a member's title, department, manager and location; adds them to a group and removes them after confirming; setting a manager that would create a reporting loop is refused with the reason; a role chip opens that role on Roles &amp; access | BPMS-023</t>
         </is>
       </c>
       <c r="D297" s="3" t="inlineStr">
@@ -18445,12 +18499,12 @@
       </c>
       <c r="B298" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-04</t>
+          <t>E2E-R1-UI-54</t>
         </is>
       </c>
       <c r="C298" s="3" t="inlineStr">
         <is>
-          <t>Announcement: the owner composes a critical post that needs acknowledgement and publishes it; a colleague opens the email link while signed out, signs in, lands on the open post and confirms; the owner sees the receipt | BPMS-047</t>
+          <t>An owner deactivates a member, then reactivates them: a reason is required, the dialog names the roles they get back, and an old sign-in must confirm it's them (step-up) first (docs/22 A-41); on Members, a pending invitation is resent (the old link stops working) and then revoked after confirming | BPMS-023</t>
         </is>
       </c>
       <c r="D298" s="3" t="inlineStr">
@@ -18472,12 +18526,12 @@
       </c>
       <c r="B299" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-05</t>
+          <t>E2E-R1-UI-55</t>
         </is>
       </c>
       <c r="C299" s="3" t="inlineStr">
         <is>
-          <t>Review loop: the owner submits a controlled policy; the reviewer (invited as Reviewer) gets the review email, opens it and requests changes with a comment; the owner gets a notification quoting it, edits and resubmits; the reviewer approves from Home; the owner is told it is approved and publishes | BPMS-040</t>
+          <t>Members bulk actions: an owner selects two members and a pending invitation, sets their department (the dialog previews who moves and says the invitation is skipped), then adds the two to a group | BPMS-023</t>
         </is>
       </c>
       <c r="D299" s="3" t="inlineStr">
@@ -18499,12 +18553,12 @@
       </c>
       <c r="B300" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-06</t>
+          <t>E2E-R1-UI-56</t>
         </is>
       </c>
       <c r="C300" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval: a second admin joins from the invitation and turns on two-step verification; the owner sends a workspace-wide post for approval; the admin gets the approval email, opens it and sends it back with a note; the owner gets a notification with the note, edits and resubmits; the admin approves and publishes; the owner is told; the post is in the feed | BPMS-047</t>
+          <t>Roles for common jobs: an owner adds HR lead from the presets (custom role, A-43) and lands in the grant dialog | BPMS-024</t>
         </is>
       </c>
       <c r="D300" s="3" t="inlineStr">
@@ -18526,12 +18580,12 @@
       </c>
       <c r="B301" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-01</t>
+          <t>E2E-R1-UI-61</t>
         </is>
       </c>
       <c r="C301" s="3" t="inlineStr">
         <is>
-          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
+          <t>Settings index: seven categories with descriptions and the starting point; search (synonyms) opens a setting on its category page; Advanced is collapsed; keys and choices for unshipped features are absent; a department override shows on the setting; a change in place counts on the index; old anchors redirect; axe on index and category | BPMS-027</t>
         </is>
       </c>
       <c r="D301" s="3" t="inlineStr">
@@ -18553,12 +18607,12 @@
       </c>
       <c r="B302" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-02</t>
+          <t>E2E-R1-UI-62</t>
         </is>
       </c>
       <c r="C302" s="3" t="inlineStr">
         <is>
-          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
+          <t>Persona navigation: an employee's sidebar is Home, Library, Announcements (+ bell); an owner reaches grouped admin pages through Admin and comes back; Library and Announcements views are tabs with their own URLs | BPMS-031</t>
         </is>
       </c>
       <c r="D302" s="3" t="inlineStr">
@@ -18580,12 +18634,12 @@
       </c>
       <c r="B303" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-03</t>
+          <t>E2E-R1-UI-63</t>
         </is>
       </c>
       <c r="C303" s="3" t="inlineStr">
         <is>
-          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
+          <t>Workspace onboarding: the owner's setup checklist on Home leads through /welcome (name and accent, starter packs, departments, invitations) and ticks steps from real data | BPMS-031</t>
         </is>
       </c>
       <c r="D303" s="3" t="inlineStr">
@@ -18607,12 +18661,12 @@
       </c>
       <c r="B304" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-04</t>
+          <t>E2E-R1-FLOW-01</t>
         </is>
       </c>
       <c r="C304" s="3" t="inlineStr">
         <is>
-          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
+          <t>Onboarding start to finish: the owner invites from Members; the invitee opens the link from the email, creates an account (password confirmation checked) and lands on Home in the workspace; the link then no longer works; the owner sees them Active and opens their person page | BPMS-023</t>
         </is>
       </c>
       <c r="D304" s="3" t="inlineStr">
@@ -18634,12 +18688,12 @@
       </c>
       <c r="B305" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-05</t>
+          <t>E2E-R1-FLOW-02</t>
         </is>
       </c>
       <c r="C305" s="3" t="inlineStr">
         <is>
-          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
+          <t>Someone with an account opens the invitation email, signs in from the page, comes back to it and joins with one click; an unknown link explains itself | BPMS-023</t>
         </is>
       </c>
       <c r="D305" s="3" t="inlineStr">
@@ -18661,12 +18715,12 @@
       </c>
       <c r="B306" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-06</t>
+          <t>E2E-R1-FLOW-03</t>
         </is>
       </c>
       <c r="C306" s="3" t="inlineStr">
         <is>
-          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
+          <t>Policy to evidence: the owner writes and publishes a policy and launches a campaign; a colleague (invited the same way) sees the task on Home, opens the acknowledgement email link, acknowledges on the document; the owner sees them Done, 1 of 2, and downloads the evidence CSV | BPMS-040, 046</t>
         </is>
       </c>
       <c r="D306" s="3" t="inlineStr">
@@ -18688,12 +18742,12 @@
       </c>
       <c r="B307" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-07</t>
+          <t>E2E-R1-FLOW-04</t>
         </is>
       </c>
       <c r="C307" s="3" t="inlineStr">
         <is>
-          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
+          <t>Announcement: the owner composes a critical post that needs acknowledgement and publishes it; a colleague opens the email link while signed out, signs in, lands on the open post and confirms; the owner sees the receipt | BPMS-047</t>
         </is>
       </c>
       <c r="D307" s="3" t="inlineStr">
@@ -18715,12 +18769,12 @@
       </c>
       <c r="B308" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-01</t>
+          <t>E2E-R1-FLOW-05</t>
         </is>
       </c>
       <c r="C308" s="3" t="inlineStr">
         <is>
-          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
+          <t>Review loop: the owner submits a controlled policy; the reviewer (invited as Reviewer) gets the review email, opens it and requests changes with a comment; the owner gets a notification quoting it, edits and resubmits; the reviewer approves from Home; the owner is told it is approved and publishes | BPMS-040</t>
         </is>
       </c>
       <c r="D308" s="3" t="inlineStr">
@@ -18742,12 +18796,12 @@
       </c>
       <c r="B309" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-02</t>
+          <t>E2E-R1-FLOW-06</t>
         </is>
       </c>
       <c r="C309" s="3" t="inlineStr">
         <is>
-          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
+          <t>Announcement approval: a second admin joins from the invitation and turns on two-step verification; the owner sends a workspace-wide post for approval; the admin gets the approval email, opens it and sends it back with a note; the owner gets a notification with the note, edits and resubmits; the admin approves and publishes; the owner is told; the post is in the feed | BPMS-047</t>
         </is>
       </c>
       <c r="D309" s="3" t="inlineStr">
@@ -18769,12 +18823,12 @@
       </c>
       <c r="B310" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-03</t>
+          <t>E2E-R1-CMP-01</t>
         </is>
       </c>
       <c r="C310" s="3" t="inlineStr">
         <is>
-          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
+          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
         </is>
       </c>
       <c r="D310" s="3" t="inlineStr">
@@ -18796,12 +18850,12 @@
       </c>
       <c r="B311" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-04</t>
+          <t>E2E-R1-CMP-02</t>
         </is>
       </c>
       <c r="C311" s="3" t="inlineStr">
         <is>
-          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
+          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
         </is>
       </c>
       <c r="D311" s="3" t="inlineStr">
@@ -18823,12 +18877,12 @@
       </c>
       <c r="B312" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-05</t>
+          <t>E2E-R1-CMP-03</t>
         </is>
       </c>
       <c r="C312" s="3" t="inlineStr">
         <is>
-          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
+          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
         </is>
       </c>
       <c r="D312" s="3" t="inlineStr">
@@ -18850,12 +18904,12 @@
       </c>
       <c r="B313" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-06</t>
+          <t>E2E-R1-CMP-04</t>
         </is>
       </c>
       <c r="C313" s="3" t="inlineStr">
         <is>
-          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
+          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
         </is>
       </c>
       <c r="D313" s="3" t="inlineStr">
@@ -18877,12 +18931,12 @@
       </c>
       <c r="B314" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-01</t>
+          <t>E2E-R1-CMP-05</t>
         </is>
       </c>
       <c r="C314" s="3" t="inlineStr">
         <is>
-          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
+          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
         </is>
       </c>
       <c r="D314" s="3" t="inlineStr">
@@ -18904,12 +18958,12 @@
       </c>
       <c r="B315" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-02</t>
+          <t>E2E-R1-CMP-06</t>
         </is>
       </c>
       <c r="C315" s="3" t="inlineStr">
         <is>
-          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
+          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
         </is>
       </c>
       <c r="D315" s="3" t="inlineStr">
@@ -18931,12 +18985,12 @@
       </c>
       <c r="B316" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-03</t>
+          <t>E2E-R1-CMP-07</t>
         </is>
       </c>
       <c r="C316" s="3" t="inlineStr">
         <is>
-          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
+          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D316" s="3" t="inlineStr">
@@ -18958,12 +19012,12 @@
       </c>
       <c r="B317" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-01</t>
+          <t>E2E-R1-ANN-01</t>
         </is>
       </c>
       <c r="C317" s="3" t="inlineStr">
         <is>
-          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
+          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
         </is>
       </c>
       <c r="D317" s="3" t="inlineStr">
@@ -18985,12 +19039,12 @@
       </c>
       <c r="B318" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-02</t>
+          <t>E2E-R1-ANN-02</t>
         </is>
       </c>
       <c r="C318" s="3" t="inlineStr">
         <is>
-          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
+          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
         </is>
       </c>
       <c r="D318" s="3" t="inlineStr">
@@ -19012,12 +19066,12 @@
       </c>
       <c r="B319" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-03</t>
+          <t>E2E-R1-ANN-03</t>
         </is>
       </c>
       <c r="C319" s="3" t="inlineStr">
         <is>
-          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
+          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
         </is>
       </c>
       <c r="D319" s="3" t="inlineStr">
@@ -19039,12 +19093,12 @@
       </c>
       <c r="B320" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-04</t>
+          <t>E2E-R1-ANN-04</t>
         </is>
       </c>
       <c r="C320" s="3" t="inlineStr">
         <is>
-          <t>Chain verify reports intact | FR-T02</t>
+          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
         </is>
       </c>
       <c r="D320" s="3" t="inlineStr">
@@ -19066,12 +19120,12 @@
       </c>
       <c r="B321" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-05</t>
+          <t>E2E-R1-ANN-05</t>
         </is>
       </c>
       <c r="C321" s="3" t="inlineStr">
         <is>
-          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
+          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D321" s="3" t="inlineStr">
@@ -19093,12 +19147,12 @@
       </c>
       <c r="B322" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-06</t>
+          <t>E2E-R1-ANN-06</t>
         </is>
       </c>
       <c r="C322" s="3" t="inlineStr">
         <is>
-          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
+          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
         </is>
       </c>
       <c r="D322" s="3" t="inlineStr">
@@ -19120,12 +19174,12 @@
       </c>
       <c r="B323" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-07</t>
+          <t>E2E-R1-SRCH-01</t>
         </is>
       </c>
       <c r="C323" s="3" t="inlineStr">
         <is>
-          <t>`POST /audit/query`: an AND group (category, action prefix, within P30D) sorted ascending pages by cursor; an OR group returns only matching events; unknown fields or values, bad durations, nesting deeper than 2 and unsupported sorts → 422 | BPMS-064, docs/08 §7.5</t>
+          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
         </is>
       </c>
       <c r="D323" s="3" t="inlineStr">
@@ -19147,12 +19201,12 @@
       </c>
       <c r="B324" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-08</t>
+          <t>E2E-R1-SRCH-02</t>
         </is>
       </c>
       <c r="C324" s="3" t="inlineStr">
         <is>
-          <t>A background export (202) runs as a job, finishes `done` with rows, its CSV downloads through the requester's signed file link, the requester is notified, and both `audit.export_requested` and `audit.exported` are recorded | BPMS-064, FR-T04</t>
+          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
         </is>
       </c>
       <c r="D324" s="3" t="inlineStr">
@@ -19174,12 +19228,12 @@
       </c>
       <c r="B325" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-SRCH-03</t>
         </is>
       </c>
       <c r="C325" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work (browser: /setup refuses a bad token or says the platform is already set up; no default account signs in; the full first run needs a fresh database, since the shared E2E database already has system admins) | FR-S01</t>
+          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
         </is>
       </c>
       <c r="D325" s="3" t="inlineStr">
@@ -19201,12 +19255,12 @@
       </c>
       <c r="B326" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-AUDX-01</t>
         </is>
       </c>
       <c r="C326" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA (browser: System › New workspace twice; owner A opens the emailed link, creates the account, turns on two-step verification, signs in and lands in the workspace) | FR-S02/S03, FR-W01</t>
+          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
         </is>
       </c>
       <c r="D326" s="3" t="inlineStr">
@@ -19228,12 +19282,12 @@
       </c>
       <c r="B327" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-AUDX-02</t>
         </is>
       </c>
       <c r="C327" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email (built: a too-light accent shows a live contrast note with the shade text will use; the server derives 4.5:1 text and 3:1 focus shades; every member's app paints them; a logo uploaded in Settings shows in everyone's sidebar; renaming SOP to "Work Instruction" in Settings › Terminology changes the labels other members see; "Request" has no screens until M6, so its override is covered at unit level) | FR-W04, 05 §7</t>
+          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
         </is>
       </c>
       <c r="D327" s="3" t="inlineStr">
@@ -19255,12 +19309,12 @@
       </c>
       <c r="B328" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-AUDX-03</t>
         </is>
       </c>
       <c r="C328" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error (browser: Members › Import directory › Check shows each row; cycle and unknown member refused; Apply saves the rest; person pages show department, manager and location) | FR-W02</t>
+          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
         </is>
       </c>
       <c r="D328" s="3" t="inlineStr">
@@ -19282,12 +19336,12 @@
       </c>
       <c r="B329" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-AUDX-04</t>
         </is>
       </c>
       <c r="C329" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused (browser: Roles &amp; access › Duplicate › grant to a person for the HR collection; a permission change previews "1 person gains 1 permission"; the holder gets Edit on the HR draft but not the Finance one, and the API agrees; a role manager who lacks audit export cannot put it into a role (403 escalation)) | FR-W03, J6</t>
+          <t>Chain verify reports intact | FR-T02</t>
         </is>
       </c>
       <c r="D329" s="3" t="inlineStr">
@@ -19309,12 +19363,12 @@
       </c>
       <c r="B330" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-AUDX-05</t>
         </is>
       </c>
       <c r="C330" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF (browser: the author's Approve is refused; the reviewer confirms with their password after an aged sign-in; Publish › Goes live schedules v2; `/__test/library/due` makes it due without moving the shared clock; v1's printable export carries the Superseded banner) | FR-G04/G05/G10, FR-PL01</t>
+          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
         </is>
       </c>
       <c r="D330" s="3" t="inlineStr">
@@ -19336,12 +19390,12 @@
       </c>
       <c r="B331" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-AUDX-06</t>
         </is>
       </c>
       <c r="C331" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method (browser: the owner publishes v2.0 as major, 51 asked; 10 people acknowledge at 390×844 from Home, 40 through the same API; the campaign shows 50 of 51 and the evidence CSV lists the v2 hash and sign-in method for all 50) | FR-PL03, FR-AK01–04</t>
+          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
         </is>
       </c>
       <c r="D331" s="3" t="inlineStr">
@@ -19363,12 +19417,12 @@
       </c>
       <c r="B332" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-AUDX-07</t>
         </is>
       </c>
       <c r="C332" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns (browser: a campaign created with "Also ask people who join later" on; a new hire who joins from the invitation email after launch finds the request on Home, acknowledges, and shows Done) | FR-AK03</t>
+          <t>`POST /audit/query`: an AND group (category, action prefix, within P30D) sorted ascending pages by cursor; an OR group returns only matching events; unknown fields or values, bad durations, nesting deeper than 2 and unsupported sorts → 422 | BPMS-064, docs/08 §7.5</t>
         </is>
       </c>
       <c r="D332" s="3" t="inlineStr">
@@ -19390,12 +19444,12 @@
       </c>
       <c r="B333" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-AUDX-08</t>
         </is>
       </c>
       <c r="C333" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct (browser: location audience from the directory, confirm-by date, only Bangalore members receive it; the announcement's campaign counts the confirmation; past the deadline the manager of the member who did not confirm is told exactly once; archiving closes the campaign) | FR-AN01–06, J14</t>
+          <t>A background export (202) runs as a job, finishes `done` with rows, its CSV downloads through the requester's signed file link, the requester is notified, and both `audit.export_requested` and `audit.exported` are recorded | BPMS-064, FR-T04</t>
         </is>
       </c>
       <c r="D333" s="3" t="inlineStr">
@@ -19417,12 +19471,12 @@
       </c>
       <c r="B334" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C334" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it (browser: the drawer says approval is needed, the author sends it, a second admin approves, members see it; at expiry it leaves the feed and admins see it as Expired) | FX-C01, FR-AN03</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work (browser: /setup refuses a bad token or says the platform is already set up; no default account signs in; the full first run needs a fresh database, since the shared E2E database already has system admins) | FR-S01</t>
         </is>
       </c>
       <c r="D334" s="3" t="inlineStr">
@@ -19444,12 +19498,12 @@
       </c>
       <c r="B335" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C335" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B (browser: a 50 MB attachment with one chunk dropped resumes and its SHA-256 matches; EICAR shows quarantined and gets no link; links last ≤ 5 minutes, a tampered link is refused, workspace B gets 404 for the link and the file) | FR-F01–F03, SEC-10</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA (browser: System › New workspace twice; owner A opens the emailed link, creates the account, turns on two-step verification, signs in and lands in the workspace) | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D335" s="3" t="inlineStr">
@@ -19471,12 +19525,12 @@
       </c>
       <c r="B336" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C336" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused (browser: Quarantined chip and a Name filter; two files changed to Operational with a reason, shown as set by an admin and audited; deleting a file a published version holds is refused) | FR-F06, FR-V</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email (built: a too-light accent shows a live contrast note with the shade text will use; the server derives 4.5:1 text and 3:1 focus shades; every member's app paints them; a logo uploaded in Settings shows in everyone's sidebar; renaming SOP to "Work Instruction" in Settings › Terminology changes the labels other members see; "Request" has no screens until M6, so its override is covered at unit level) | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D336" s="3" t="inlineStr">
@@ -19498,12 +19552,12 @@
       </c>
       <c r="B337" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C337" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction (browser: Status is Published and (Name contains Alpha or Charlie); sort by type then name; view shared with Reviewers opens from the deep link for a reviewer; CSV has exactly the shown rows; XLSX downloads) | FR-V01–V07</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error (browser: Members › Import directory › Check shows each row; cycle and unknown member refused; Apply saves the rest; person pages show department, manager and location) | FR-W02</t>
         </is>
       </c>
       <c r="D337" s="3" t="inlineStr">
@@ -19525,12 +19579,12 @@
       </c>
       <c r="B338" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C338" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK (browser: Person filter shows only that person's events; a version's timeline is oldest first: three edits, submitted, published; the page shows Chain verified) | FR-T01–T04</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused (browser: Roles &amp; access › Duplicate › grant to a person for the HR collection; a permission change previews "1 person gains 1 permission"; the holder gets Edit on the HR draft but not the Finance one, and the API agrees; a role manager who lacks audit export cannot put it into a role (403 escalation)) | FR-W03, J6</t>
         </is>
       </c>
       <c r="D338" s="3" t="inlineStr">
@@ -19552,12 +19606,12 @@
       </c>
       <c r="B339" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C339" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts (browser: open acknowledgements → active campaigns with the same "still to acknowledge"; versions published → audit log filtered to publications with the same event count; announcements published → the Published tab; without two-step → People &amp; access filtered with the same count) | FR-A01</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF (browser: the author's Approve is refused; the reviewer confirms with their password after an aged sign-in; Publish › Goes live schedules v2; `/__test/library/due` makes it due without moving the shared clock; v1's printable export carries the Superseded banner) | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D339" s="3" t="inlineStr">
@@ -19579,12 +19633,12 @@
       </c>
       <c r="B340" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C340" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act (browser: owner deactivates from the person page; the member's open tab is sent to the chooser on the next page; signing in again offers no workspace; the API refuses entry) | SEC-04, FR-W01</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method (browser: the owner publishes v2.0 as major, 51 asked; 10 people acknowledge at 390×844 from Home, 40 through the same API; the campaign shows 50 of 51 and the evidence CSV lists the v2 hash and sign-in method for all 50) | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D340" s="3" t="inlineStr">
@@ -19606,12 +19660,12 @@
       </c>
       <c r="B341" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C341" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore (browser: reads keep working; the first change is refused and a read-only banner appears on every page; after restore the banner is gone and changes work) | FR-S02, J8</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns (browser: a campaign created with "Also ask people who join later" on; a new hire who joins from the invitation email after launch finds the request on Home, acknowledges, and shows Done) | FR-AK03</t>
         </is>
       </c>
       <c r="D341" s="3" t="inlineStr">
@@ -19633,12 +19687,12 @@
       </c>
       <c r="B342" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C342" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock (browser: Home › Browse templates › Install the handbook pack (5 drafts) → publish the handbook → launch the campaign → 20 people at 390×844 acknowledge; 20 of 21 done, within 15 minutes) | J12</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct (browser: location audience from the directory, confirm-by date, only Bangalore members receive it; the announcement's campaign counts the confirmation; past the deadline the manager of the member who did not confirm is told exactly once; archiving closes the campaign) | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D342" s="3" t="inlineStr">
@@ -19660,12 +19714,12 @@
       </c>
       <c r="B343" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C343" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse (browser: Tab/Enter/typing only, author from Library to Published, colleague from sign-in to Acknowledged) | A11Y-01, T10</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it (browser: the drawer says approval is needed, the author sends it, a second admin approves, members see it; at expiry it leaves the feed and admins see it as Expired) | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D343" s="3" t="inlineStr">
@@ -19687,12 +19741,12 @@
       </c>
       <c r="B344" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C344" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` (built: B's owner probes 21 reads and writes on A's documents, versions, exports, campaigns, announcements, collections, departments, views, files and members → all 404, each recorded in B's audit log as `access.denied` with the object id, B's chain verifies, A unchanged) | SEC-01/02</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B (browser: a 50 MB attachment with one chunk dropped resumes and its SHA-256 matches; EICAR shows quarantined and gets no link; links last ≤ 5 minutes, a tampered link is refused, workspace B gets 404 for the link and the file) | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D344" s="3" t="inlineStr">
@@ -19714,12 +19768,12 @@
       </c>
       <c r="B345" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C345" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused (browser: Quarantined chip and a Name filter; two files changed to Operational with a reason, shown as set by an admin and audited; deleting a file a published version holds is refused) | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D345" s="3" t="inlineStr">
@@ -19741,12 +19795,12 @@
       </c>
       <c r="B346" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C346" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction (browser: Status is Published and (Name contains Alpha or Charlie); sort by type then name; view shared with Reviewers opens from the deep link for a reviewer; CSV has exactly the shown rows; XLSX downloads) | FR-V01–V07</t>
         </is>
       </c>
       <c r="D346" s="3" t="inlineStr">
@@ -19768,12 +19822,12 @@
       </c>
       <c r="B347" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C347" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK (browser: Person filter shows only that person's events; a version's timeline is oldest first: three edits, submitted, published; the page shows Chain verified) | FR-T01–T04</t>
         </is>
       </c>
       <c r="D347" s="3" t="inlineStr">
@@ -19795,12 +19849,12 @@
       </c>
       <c r="B348" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C348" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts (browser: open acknowledgements → active campaigns with the same "still to acknowledge"; versions published → audit log filtered to publications with the same event count; announcements published → the Published tab; without two-step → People &amp; access filtered with the same count) | FR-A01</t>
         </is>
       </c>
       <c r="D348" s="3" t="inlineStr">
@@ -19822,12 +19876,12 @@
       </c>
       <c r="B349" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C349" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act (browser: owner deactivates from the person page; the member's open tab is sent to the chooser on the next page; signing in again offers no workspace; the API refuses entry) | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D349" s="3" t="inlineStr">
@@ -19849,12 +19903,12 @@
       </c>
       <c r="B350" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C350" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore (browser: reads keep working; the first change is refused and a read-only banner appears on every page; after restore the banner is gone and changes work) | FR-S02, J8</t>
         </is>
       </c>
       <c r="D350" s="3" t="inlineStr">
@@ -19876,12 +19930,12 @@
       </c>
       <c r="B351" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C351" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock (browser: Home › Browse templates › Install the handbook pack (5 drafts) → publish the handbook → launch the campaign → 20 people at 390×844 acknowledge; 20 of 21 done, within 15 minutes) | J12</t>
         </is>
       </c>
       <c r="D351" s="3" t="inlineStr">
@@ -19903,12 +19957,12 @@
       </c>
       <c r="B352" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C352" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse (browser: Tab/Enter/typing only, author from Library to Published, colleague from sign-in to Acknowledged) | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D352" s="3" t="inlineStr">
@@ -19930,12 +19984,12 @@
       </c>
       <c r="B353" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C353" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` (built: B's owner probes 21 reads and writes on A's documents, versions, exports, campaigns, announcements, collections, departments, views, files and members → all 404, each recorded in B's audit log as `access.denied` with the object id, B's chain verifies, A unchanged) | SEC-01/02</t>
         </is>
       </c>
       <c r="D353" s="3" t="inlineStr">
@@ -19957,12 +20011,12 @@
       </c>
       <c r="B354" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C354" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D354" s="3" t="inlineStr">
@@ -19984,12 +20038,12 @@
       </c>
       <c r="B355" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C355" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D355" s="3" t="inlineStr">
@@ -20011,12 +20065,12 @@
       </c>
       <c r="B356" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C356" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D356" s="3" t="inlineStr">
@@ -20038,12 +20092,12 @@
       </c>
       <c r="B357" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C357" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D357" s="3" t="inlineStr">
@@ -20065,12 +20119,12 @@
       </c>
       <c r="B358" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C358" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D358" s="3" t="inlineStr">
@@ -20092,12 +20146,12 @@
       </c>
       <c r="B359" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C359" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D359" s="3" t="inlineStr">
@@ -20119,12 +20173,12 @@
       </c>
       <c r="B360" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C360" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D360" s="3" t="inlineStr">
@@ -20146,12 +20200,12 @@
       </c>
       <c r="B361" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C361" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D361" s="3" t="inlineStr">
@@ -20173,12 +20227,12 @@
       </c>
       <c r="B362" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C362" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D362" s="3" t="inlineStr">
@@ -20200,12 +20254,12 @@
       </c>
       <c r="B363" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C363" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D363" s="3" t="inlineStr">
@@ -20227,12 +20281,12 @@
       </c>
       <c r="B364" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C364" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D364" s="3" t="inlineStr">
@@ -20254,12 +20308,12 @@
       </c>
       <c r="B365" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C365" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D365" s="3" t="inlineStr">
@@ -20281,12 +20335,12 @@
       </c>
       <c r="B366" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C366" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D366" s="3" t="inlineStr">
@@ -20308,12 +20362,12 @@
       </c>
       <c r="B367" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C367" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D367" s="3" t="inlineStr">
@@ -20335,12 +20389,12 @@
       </c>
       <c r="B368" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C368" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D368" s="3" t="inlineStr">
@@ -20362,12 +20416,12 @@
       </c>
       <c r="B369" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C369" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D369" s="3" t="inlineStr">
@@ -20389,12 +20443,12 @@
       </c>
       <c r="B370" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C370" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D370" s="3" t="inlineStr">
@@ -20416,12 +20470,12 @@
       </c>
       <c r="B371" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C371" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D371" s="3" t="inlineStr">
@@ -20443,12 +20497,12 @@
       </c>
       <c r="B372" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C372" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D372" s="3" t="inlineStr">
@@ -20470,12 +20524,12 @@
       </c>
       <c r="B373" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C373" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D373" s="3" t="inlineStr">
@@ -20497,12 +20551,12 @@
       </c>
       <c r="B374" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C374" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D374" s="3" t="inlineStr">
@@ -20524,12 +20578,12 @@
       </c>
       <c r="B375" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C375" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D375" s="3" t="inlineStr">
@@ -20551,12 +20605,12 @@
       </c>
       <c r="B376" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C376" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D376" s="3" t="inlineStr">
@@ -20578,12 +20632,12 @@
       </c>
       <c r="B377" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C377" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D377" s="3" t="inlineStr">
@@ -20605,12 +20659,12 @@
       </c>
       <c r="B378" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C378" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D378" s="3" t="inlineStr">
@@ -20632,12 +20686,12 @@
       </c>
       <c r="B379" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C379" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D379" s="3" t="inlineStr">
@@ -20659,12 +20713,12 @@
       </c>
       <c r="B380" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C380" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D380" s="3" t="inlineStr">
@@ -20686,12 +20740,12 @@
       </c>
       <c r="B381" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C381" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D381" s="3" t="inlineStr">
@@ -20713,12 +20767,12 @@
       </c>
       <c r="B382" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C382" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D382" s="3" t="inlineStr">
@@ -20740,12 +20794,12 @@
       </c>
       <c r="B383" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C383" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D383" s="3" t="inlineStr">
@@ -20767,12 +20821,12 @@
       </c>
       <c r="B384" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C384" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D384" s="3" t="inlineStr">
@@ -20794,12 +20848,12 @@
       </c>
       <c r="B385" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C385" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D385" s="3" t="inlineStr">
@@ -20821,12 +20875,12 @@
       </c>
       <c r="B386" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C386" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D386" s="3" t="inlineStr">
@@ -20848,12 +20902,12 @@
       </c>
       <c r="B387" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C387" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D387" s="3" t="inlineStr">
@@ -20875,12 +20929,12 @@
       </c>
       <c r="B388" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C388" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D388" s="3" t="inlineStr">
@@ -20902,12 +20956,12 @@
       </c>
       <c r="B389" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C389" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D389" s="3" t="inlineStr">
@@ -20929,12 +20983,12 @@
       </c>
       <c r="B390" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C390" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D390" s="3" t="inlineStr">
@@ -20956,12 +21010,12 @@
       </c>
       <c r="B391" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C391" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D391" s="3" t="inlineStr">
@@ -20983,12 +21037,12 @@
       </c>
       <c r="B392" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C392" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D392" s="3" t="inlineStr">
@@ -21010,12 +21064,12 @@
       </c>
       <c r="B393" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C393" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D393" s="3" t="inlineStr">
@@ -21037,12 +21091,12 @@
       </c>
       <c r="B394" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C394" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D394" s="3" t="inlineStr">
@@ -21064,12 +21118,12 @@
       </c>
       <c r="B395" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R4-11</t>
         </is>
       </c>
       <c r="C395" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
         </is>
       </c>
       <c r="D395" s="3" t="inlineStr">
@@ -21091,12 +21145,12 @@
       </c>
       <c r="B396" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R4-ISO</t>
         </is>
       </c>
       <c r="C396" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
         </is>
       </c>
       <c r="D396" s="3" t="inlineStr">
@@ -21118,12 +21172,12 @@
       </c>
       <c r="B397" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R5-01</t>
         </is>
       </c>
       <c r="C397" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
         </is>
       </c>
       <c r="D397" s="3" t="inlineStr">
@@ -21145,20 +21199,263 @@
       </c>
       <c r="B398" s="3" t="inlineStr">
         <is>
+          <t>E2E-R5-02</t>
+        </is>
+      </c>
+      <c r="C398" s="3" t="inlineStr">
+        <is>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+        </is>
+      </c>
+      <c r="D398" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E398" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B399" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-03</t>
+        </is>
+      </c>
+      <c r="C399" s="3" t="inlineStr">
+        <is>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+        </is>
+      </c>
+      <c r="D399" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E399" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B400" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-04</t>
+        </is>
+      </c>
+      <c r="C400" s="3" t="inlineStr">
+        <is>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+        </is>
+      </c>
+      <c r="D400" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E400" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B401" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-05</t>
+        </is>
+      </c>
+      <c r="C401" s="3" t="inlineStr">
+        <is>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+        </is>
+      </c>
+      <c r="D401" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E401" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B402" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-06</t>
+        </is>
+      </c>
+      <c r="C402" s="3" t="inlineStr">
+        <is>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+        </is>
+      </c>
+      <c r="D402" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E402" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B403" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-07</t>
+        </is>
+      </c>
+      <c r="C403" s="3" t="inlineStr">
+        <is>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+        </is>
+      </c>
+      <c r="D403" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E403" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B404" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-08</t>
+        </is>
+      </c>
+      <c r="C404" s="3" t="inlineStr">
+        <is>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+        </is>
+      </c>
+      <c r="D404" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E404" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B405" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-09</t>
+        </is>
+      </c>
+      <c r="C405" s="3" t="inlineStr">
+        <is>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+        </is>
+      </c>
+      <c r="D405" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E405" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B406" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C406" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D406" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E406" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B407" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C398" s="3" t="inlineStr">
+      <c r="C407" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D398" s="3" t="inlineStr">
+      <c r="D407" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E398" s="3" t="inlineStr">
+      <c r="E407" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
chore(tracker): email setup done; self-hosting guides, site, audit labels, onboarding and 0.1 polish recorded
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E407" headerRowCount="1">
-  <autoFilter ref="A1:E407"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E409" headerRowCount="1">
+  <autoFilter ref="A1:E409"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -4488,7 +4488,7 @@
       <c r="N14" s="3" t="inlineStr"/>
       <c r="O14" s="3" t="inlineStr">
         <is>
-          <t>e2e feature + /__test controls, Playwright harness, P0 smoke pack (E2E-P0-01..04, REL), compose.e2e stack, CI e2e-smoke job; on main, CI green. Seed A/B + personas land with the first workspace APIs (BPMS-032); full compose boot pending a Docker run</t>
+          <t>e2e feature + /__test controls, Playwright harness, P0 smoke pack (E2E-P0-01..04, REL), compose.e2e stack, CI e2e-smoke job; on main, CI green. Seed A/B + personas land with the first workspace APIs (BPMS-032); full compose boot pending a Docker run Self-hosting: deploy/compose.yml (web+API behind Caddy, Postgres, migrate, optional cache/scan/mail profiles), procera healthcheck, SIGTERM shutdown; guides for Docker Compose install, first-time setup and configuration (docs/guides).</t>
         </is>
       </c>
     </row>
@@ -4744,7 +4744,7 @@
       <c r="N18" s="3" t="inlineStr"/>
       <c r="O18" s="3" t="inlineStr">
         <is>
-          <t>TOTP + recovery codes + step-up + MFA by role (earlier); passkeys (WebAuthn L3, migration 0020): registration, sign-in second factor and step-up, list/rename/remove with step-up, phishing-origin and replay protection, Account › Security page, Use a passkey at sign-in and in step-up. E2E-R1-AUTH-06, 20..23, E2E-R1-UI-30..31. Passkey-only sign-in is P1 (A-19)</t>
+          <t>TOTP + recovery codes + step-up + MFA by role (earlier); passkeys (WebAuthn L3, migration 0020): registration, sign-in second factor and step-up, list/rename/remove with step-up, phishing-origin and replay protection, Account › Security page, Use a passkey at sign-in and in step-up. E2E-R1-AUTH-06, 20..23, E2E-R1-UI-30..31. Passkey-only sign-in is P1 (A-19) No second sign-in after turning on two-step: the confirmed code upgrades the session and its refresh family.</t>
         </is>
       </c>
     </row>
@@ -5329,7 +5329,7 @@
       <c r="N27" s="3" t="inlineStr"/>
       <c r="O27" s="3" t="inlineStr">
         <is>
-          <t>Web app on the Notion/Attio direction (owner choice): warm paper palette in tokens (contrast-checked), full-bleed pages with a warm icon sidebar, workspace + account menus (persisted theme), action-first Home (acknowledgements, reviews, announcements with inline actions, library table, activity, people), Library (filters, Attio-style table, New document dialog), document reading view with properties, lifecycle actions (edit, submit, approve, request changes, publish with step-up, new version), acknowledgement callout, Announcements feed with read/ack, Members with invite dialog; split sign-in with product preview; single-flight token refresh. E2E-R1-UI-01..10 with axe. Second UI pass: Geist type, state kit (skeletons, empty states, load errors with retry), ⌘K palette over search + commands (E2E-R1-UI-12..13), admin screens: Manage announcements, Campaigns, Settings, Audit log, Overview, People &amp; access (E2E-R1-UI-14..17, 23); Policies portal and document governance (E2E-R1-UI-18..22). Keyboard-only journey (E2E-R1-19) and system console shell done. Remaining: persona IA redesign approved 2026-10-12 (docs/design/ia-competitive-analysis.md: persona sidebar, Admin hub, Needs-you Home, workspace onboarding) done: persona sidebar, Admin hub and admin mode, Library and Announcements views, Needs you Home, workspace onboarding checklist and /welcome (E2E-R1-UI-62..63). Remaining: role cards on Home, mobile bottom bar</t>
+          <t>Web app on the Notion/Attio direction (owner choice): warm paper palette in tokens (contrast-checked), full-bleed pages with a warm icon sidebar, workspace + account menus (persisted theme), action-first Home (acknowledgements, reviews, announcements with inline actions, library table, activity, people), Library (filters, Attio-style table, New document dialog), document reading view with properties, lifecycle actions (edit, submit, approve, request changes, publish with step-up, new version), acknowledgement callout, Announcements feed with read/ack, Members with invite dialog; split sign-in with product preview; single-flight token refresh. E2E-R1-UI-01..10 with axe. Second UI pass: Geist type, state kit (skeletons, empty states, load errors with retry), ⌘K palette over search + commands (E2E-R1-UI-12..13), admin screens: Manage announcements, Campaigns, Settings, Audit log, Overview, People &amp; access (E2E-R1-UI-14..17, 23); Policies portal and document governance (E2E-R1-UI-18..22). Keyboard-only journey (E2E-R1-19) and system console shell done. Remaining: persona IA redesign approved 2026-10-12 (docs/design/ia-competitive-analysis.md: persona sidebar, Admin hub, Needs-you Home, workspace onboarding) done: persona sidebar, Admin hub and admin mode, Library and Announcements views, Needs you Home, workspace onboarding checklist and /welcome (E2E-R1-UI-62..63). Home role cards (needs attention, active campaigns); 0.1 polish from a small-company walkthrough (review choice in setup, approver named, authors not offered their own review, merged notifications, document page layout, animated empty-state illustrations). Remaining: mobile bottom bar</t>
         </is>
       </c>
     </row>
@@ -5520,7 +5520,7 @@
       <c r="N30" s="3" t="inlineStr"/>
       <c r="O30" s="3" t="inlineStr">
         <is>
-          <t>Vector masters (assets/brand/vector, generated by build.py: P-ribbon symbol, flat small symbol, horizontal and stacked lockups light/dark, app icons, banner; wordmark outlined from Geist, OFL); PNGs, favicons and ICO re-exported from them; the app uses the SVG symbol and an SVG favicon. Remaining: trademark search (OQ-01), professional mark review before GA Marketing site (site/, static, generated from tracker data and real screenshots: home, features, user flows, comparison, roadmap, security, open source); not published yet.</t>
+          <t>Vector masters (assets/brand/vector, generated by build.py: P-ribbon symbol, flat small symbol, horizontal and stacked lockups light/dark, app icons, banner; wordmark outlined from Geist, OFL); PNGs, favicons and ICO re-exported from them; the app uses the SVG symbol and an SVG favicon. Remaining: trademark search (OQ-01), professional mark review before GA Marketing site (site/, static, generated from tracker data and real screenshots: home, features, user flows, comparison, roadmap, security, open source); not published yet. Revamped site: animated product story, original illustrations, scroll motion, persona tabs, tamper demo, Get started page rendering the guides; published to GitHub Pages.</t>
         </is>
       </c>
     </row>
@@ -6300,7 +6300,7 @@
       <c r="N42" s="3" t="inlineStr"/>
       <c r="O42" s="3" t="inlineStr">
         <is>
-          <t>Image/PDF previews: GET /files/{id}/preview-url (kind image|pdf|none) and GET /files/preview/{token} (own preview HMAC purpose, 2-minute TTL, re-authorized per request; clean PNG/JPEG/GIF/WebP/PDF only by recorded type plus fresh sniff, else 415; inline under CSP sandbox, nosniff, CORP same-origin, no-store; audited file.previewed); JPEG Exif/XMP/IPTC stripped from previews (files.exif_strip); Preview dialog on attachments. E2E-R1-FILE-04, E2E-R1-UI-34. Remaining: separate preview origin, EXIF strip at upload, Office preview (P1).</t>
+          <t>In-app viewer for PDF, Word and spreadsheets in progress. Image/PDF previews: GET /files/{id}/preview-url (kind image|pdf|none) and GET /files/preview/{token} (own preview HMAC purpose, 2-minute TTL, re-authorized per request; clean PNG/JPEG/GIF/WebP/PDF only by recorded type plus fresh sniff, else 415; inline under CSP sandbox, nosniff, CORP same-origin, no-store; audited file.previewed); JPEG Exif/XMP/IPTC stripped from previews (files.exif_strip); Preview dialog on attachments. E2E-R1-FILE-04, E2E-R1-UI-34. Remaining: separate preview origin, EXIF strip at upload, Office preview (P1).</t>
         </is>
       </c>
     </row>
@@ -6495,7 +6495,7 @@
       <c r="N45" s="3" t="inlineStr"/>
       <c r="O45" s="3" t="inlineStr">
         <is>
-          <t>procera_audit::explorer and query: filtered newest-first keyset paging, view-own scope, member names, artifact timelines (own and version events), chain verify, saved queries, capped synchronous CSV/JSONL exports with step-up; POST /audit/query (AND/OR tree, allow-listed fields, depth 2); background export jobs (migration 0029) stored as the requester's encrypted file with notification; Audit log UI with filters, timelines and background exports. E2E-R1-AUDX-01..08, E2E-R1-AUD-01, E2E-R1-UI-17, 39. Later: verify-proof per sequence, the P95 &lt; 2 s at 10 M events benchmark</t>
+          <t>procera_audit::explorer and query: filtered newest-first keyset paging, view-own scope, member names, artifact timelines (own and version events), chain verify, saved queries, capped synchronous CSV/JSONL exports with step-up; POST /audit/query (AND/OR tree, allow-listed fields, depth 2); background export jobs (migration 0029) stored as the requester's encrypted file with notification; Audit log UI with filters, timelines and background exports. E2E-R1-AUDX-01..08, E2E-R1-AUD-01, E2E-R1-UI-17, 39. Later: verify-proof per sequence, the P95 &lt; 2 s at 10 M events benchmark Events name their object (“Expense claims v1”, a person, a campaign).</t>
         </is>
       </c>
     </row>
@@ -6552,7 +6552,7 @@
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L46" s="3" t="inlineStr"/>
@@ -6560,7 +6560,7 @@
       <c r="N46" s="3" t="inlineStr"/>
       <c r="O46" s="3" t="inlineStr">
         <is>
-          <t>System console (0022): workspaces grid with usage and quotas, suspend/reactivate/schedule deletion with step-up on the system chain, quota defaults per profile with the member quota enforced at invite, platform health, system audit explorer; console shell for system admins (metadata only, never workspace content). E2E-R1-SYS-01..09, E2E-R1-UI-40..41 (A-18) Remaining (docs/20 §3, CFG-006): email delivery (SMTP) settings with test send, public URL and sender, storage and scanning status, /setup continuing to email and the first workspace — next.</t>
+          <t>System console (0022): workspaces grid with usage and quotas, suspend/reactivate/schedule deletion with step-up on the system chain, quota defaults per profile with the member quota enforced at invite, platform health, system audit explorer; console shell for system admins (metadata only, never workspace content). E2E-R1-SYS-01..09, E2E-R1-UI-40..41 (A-18) Email &amp; platform (migration 0037): SMTP settings with the password sealed and never returned, test send with plain-language failures, hot reload without restart, environment wins; public URL, storage and scanning status; first-time setup continues to Email and the first workspace. E2E-R1-UI-64..65.</t>
         </is>
       </c>
     </row>
@@ -10462,7 +10462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E407"/>
+  <dimension ref="A1:E409"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -18661,12 +18661,12 @@
       </c>
       <c r="B304" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-01</t>
+          <t>E2E-R1-UI-64</t>
         </is>
       </c>
       <c r="C304" s="3" t="inlineStr">
         <is>
-          <t>Onboarding start to finish: the owner invites from Members; the invitee opens the link from the email, creates an account (password confirmation checked) and lands on Home in the workspace; the link then no longer works; the owner sees them Active and opens their person page | BPMS-023</t>
+          <t>System › Email &amp; platform: save SMTP settings (password write-only, "Leave blank to keep the current password"), a test send to a closed port explains the refusal, both audited; platform basics, storage and scanning shown read-only. E2E builds deliver only through PROCERA_SMTP_URL, so saved settings never drain the shared queue | BPMS-065</t>
         </is>
       </c>
       <c r="D304" s="3" t="inlineStr">
@@ -18688,12 +18688,12 @@
       </c>
       <c r="B305" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-02</t>
+          <t>E2E-R1-UI-65</t>
         </is>
       </c>
       <c r="C305" s="3" t="inlineStr">
         <is>
-          <t>Someone with an account opens the invitation email, signs in from the page, comes back to it and joins with one click; an unknown link explains itself | BPMS-023</t>
+          <t>First-time setup continues at /system/setup: an optional email step (skippable) and Create your first workspace, ending with the owner's invitation | BPMS-065</t>
         </is>
       </c>
       <c r="D305" s="3" t="inlineStr">
@@ -18715,12 +18715,12 @@
       </c>
       <c r="B306" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-03</t>
+          <t>E2E-R1-FLOW-01</t>
         </is>
       </c>
       <c r="C306" s="3" t="inlineStr">
         <is>
-          <t>Policy to evidence: the owner writes and publishes a policy and launches a campaign; a colleague (invited the same way) sees the task on Home, opens the acknowledgement email link, acknowledges on the document; the owner sees them Done, 1 of 2, and downloads the evidence CSV | BPMS-040, 046</t>
+          <t>Onboarding start to finish: the owner invites from Members; the invitee opens the link from the email, creates an account (password confirmation checked) and lands on Home in the workspace; the link then no longer works; the owner sees them Active and opens their person page | BPMS-023</t>
         </is>
       </c>
       <c r="D306" s="3" t="inlineStr">
@@ -18742,12 +18742,12 @@
       </c>
       <c r="B307" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-04</t>
+          <t>E2E-R1-FLOW-02</t>
         </is>
       </c>
       <c r="C307" s="3" t="inlineStr">
         <is>
-          <t>Announcement: the owner composes a critical post that needs acknowledgement and publishes it; a colleague opens the email link while signed out, signs in, lands on the open post and confirms; the owner sees the receipt | BPMS-047</t>
+          <t>Someone with an account opens the invitation email, signs in from the page, comes back to it and joins with one click; an unknown link explains itself | BPMS-023</t>
         </is>
       </c>
       <c r="D307" s="3" t="inlineStr">
@@ -18769,12 +18769,12 @@
       </c>
       <c r="B308" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-05</t>
+          <t>E2E-R1-FLOW-03</t>
         </is>
       </c>
       <c r="C308" s="3" t="inlineStr">
         <is>
-          <t>Review loop: the owner submits a controlled policy; the reviewer (invited as Reviewer) gets the review email, opens it and requests changes with a comment; the owner gets a notification quoting it, edits and resubmits; the reviewer approves from Home; the owner is told it is approved and publishes | BPMS-040</t>
+          <t>Policy to evidence: the owner writes and publishes a policy and launches a campaign; a colleague (invited the same way) sees the task on Home, opens the acknowledgement email link, acknowledges on the document; the owner sees them Done, 1 of 2, and downloads the evidence CSV | BPMS-040, 046</t>
         </is>
       </c>
       <c r="D308" s="3" t="inlineStr">
@@ -18796,12 +18796,12 @@
       </c>
       <c r="B309" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-06</t>
+          <t>E2E-R1-FLOW-04</t>
         </is>
       </c>
       <c r="C309" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval: a second admin joins from the invitation and turns on two-step verification; the owner sends a workspace-wide post for approval; the admin gets the approval email, opens it and sends it back with a note; the owner gets a notification with the note, edits and resubmits; the admin approves and publishes; the owner is told; the post is in the feed | BPMS-047</t>
+          <t>Announcement: the owner composes a critical post that needs acknowledgement and publishes it; a colleague opens the email link while signed out, signs in, lands on the open post and confirms; the owner sees the receipt | BPMS-047</t>
         </is>
       </c>
       <c r="D309" s="3" t="inlineStr">
@@ -18823,12 +18823,12 @@
       </c>
       <c r="B310" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-01</t>
+          <t>E2E-R1-FLOW-05</t>
         </is>
       </c>
       <c r="C310" s="3" t="inlineStr">
         <is>
-          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
+          <t>Review loop: the owner submits a controlled policy; the reviewer (invited as Reviewer) gets the review email, opens it and requests changes with a comment; the owner gets a notification quoting it, edits and resubmits; the reviewer approves from Home; the owner is told it is approved and publishes | BPMS-040</t>
         </is>
       </c>
       <c r="D310" s="3" t="inlineStr">
@@ -18850,12 +18850,12 @@
       </c>
       <c r="B311" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-02</t>
+          <t>E2E-R1-FLOW-06</t>
         </is>
       </c>
       <c r="C311" s="3" t="inlineStr">
         <is>
-          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
+          <t>Announcement approval: a second admin joins from the invitation and turns on two-step verification; the owner sends a workspace-wide post for approval; the admin gets the approval email, opens it and sends it back with a note; the owner gets a notification with the note, edits and resubmits; the admin approves and publishes; the owner is told; the post is in the feed | BPMS-047</t>
         </is>
       </c>
       <c r="D311" s="3" t="inlineStr">
@@ -18877,12 +18877,12 @@
       </c>
       <c r="B312" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-03</t>
+          <t>E2E-R1-CMP-01</t>
         </is>
       </c>
       <c r="C312" s="3" t="inlineStr">
         <is>
-          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
+          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
         </is>
       </c>
       <c r="D312" s="3" t="inlineStr">
@@ -18904,12 +18904,12 @@
       </c>
       <c r="B313" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-04</t>
+          <t>E2E-R1-CMP-02</t>
         </is>
       </c>
       <c r="C313" s="3" t="inlineStr">
         <is>
-          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
+          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
         </is>
       </c>
       <c r="D313" s="3" t="inlineStr">
@@ -18931,12 +18931,12 @@
       </c>
       <c r="B314" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-05</t>
+          <t>E2E-R1-CMP-03</t>
         </is>
       </c>
       <c r="C314" s="3" t="inlineStr">
         <is>
-          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
+          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
         </is>
       </c>
       <c r="D314" s="3" t="inlineStr">
@@ -18958,12 +18958,12 @@
       </c>
       <c r="B315" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-06</t>
+          <t>E2E-R1-CMP-04</t>
         </is>
       </c>
       <c r="C315" s="3" t="inlineStr">
         <is>
-          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
+          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
         </is>
       </c>
       <c r="D315" s="3" t="inlineStr">
@@ -18985,12 +18985,12 @@
       </c>
       <c r="B316" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-07</t>
+          <t>E2E-R1-CMP-05</t>
         </is>
       </c>
       <c r="C316" s="3" t="inlineStr">
         <is>
-          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
+          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
         </is>
       </c>
       <c r="D316" s="3" t="inlineStr">
@@ -19012,12 +19012,12 @@
       </c>
       <c r="B317" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-01</t>
+          <t>E2E-R1-CMP-06</t>
         </is>
       </c>
       <c r="C317" s="3" t="inlineStr">
         <is>
-          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
+          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
         </is>
       </c>
       <c r="D317" s="3" t="inlineStr">
@@ -19039,12 +19039,12 @@
       </c>
       <c r="B318" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-02</t>
+          <t>E2E-R1-CMP-07</t>
         </is>
       </c>
       <c r="C318" s="3" t="inlineStr">
         <is>
-          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
+          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D318" s="3" t="inlineStr">
@@ -19066,12 +19066,12 @@
       </c>
       <c r="B319" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-03</t>
+          <t>E2E-R1-ANN-01</t>
         </is>
       </c>
       <c r="C319" s="3" t="inlineStr">
         <is>
-          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
+          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
         </is>
       </c>
       <c r="D319" s="3" t="inlineStr">
@@ -19093,12 +19093,12 @@
       </c>
       <c r="B320" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-04</t>
+          <t>E2E-R1-ANN-02</t>
         </is>
       </c>
       <c r="C320" s="3" t="inlineStr">
         <is>
-          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
+          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
         </is>
       </c>
       <c r="D320" s="3" t="inlineStr">
@@ -19120,12 +19120,12 @@
       </c>
       <c r="B321" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-05</t>
+          <t>E2E-R1-ANN-03</t>
         </is>
       </c>
       <c r="C321" s="3" t="inlineStr">
         <is>
-          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
+          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
         </is>
       </c>
       <c r="D321" s="3" t="inlineStr">
@@ -19147,12 +19147,12 @@
       </c>
       <c r="B322" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-06</t>
+          <t>E2E-R1-ANN-04</t>
         </is>
       </c>
       <c r="C322" s="3" t="inlineStr">
         <is>
-          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
+          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
         </is>
       </c>
       <c r="D322" s="3" t="inlineStr">
@@ -19174,12 +19174,12 @@
       </c>
       <c r="B323" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-01</t>
+          <t>E2E-R1-ANN-05</t>
         </is>
       </c>
       <c r="C323" s="3" t="inlineStr">
         <is>
-          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
+          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D323" s="3" t="inlineStr">
@@ -19201,12 +19201,12 @@
       </c>
       <c r="B324" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-02</t>
+          <t>E2E-R1-ANN-06</t>
         </is>
       </c>
       <c r="C324" s="3" t="inlineStr">
         <is>
-          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
+          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
         </is>
       </c>
       <c r="D324" s="3" t="inlineStr">
@@ -19228,12 +19228,12 @@
       </c>
       <c r="B325" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-03</t>
+          <t>E2E-R1-SRCH-01</t>
         </is>
       </c>
       <c r="C325" s="3" t="inlineStr">
         <is>
-          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
+          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
         </is>
       </c>
       <c r="D325" s="3" t="inlineStr">
@@ -19255,12 +19255,12 @@
       </c>
       <c r="B326" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-01</t>
+          <t>E2E-R1-SRCH-02</t>
         </is>
       </c>
       <c r="C326" s="3" t="inlineStr">
         <is>
-          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
+          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
         </is>
       </c>
       <c r="D326" s="3" t="inlineStr">
@@ -19282,12 +19282,12 @@
       </c>
       <c r="B327" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-02</t>
+          <t>E2E-R1-SRCH-03</t>
         </is>
       </c>
       <c r="C327" s="3" t="inlineStr">
         <is>
-          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
+          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
         </is>
       </c>
       <c r="D327" s="3" t="inlineStr">
@@ -19309,12 +19309,12 @@
       </c>
       <c r="B328" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-03</t>
+          <t>E2E-R1-AUDX-01</t>
         </is>
       </c>
       <c r="C328" s="3" t="inlineStr">
         <is>
-          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
+          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
         </is>
       </c>
       <c r="D328" s="3" t="inlineStr">
@@ -19336,12 +19336,12 @@
       </c>
       <c r="B329" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-04</t>
+          <t>E2E-R1-AUDX-02</t>
         </is>
       </c>
       <c r="C329" s="3" t="inlineStr">
         <is>
-          <t>Chain verify reports intact | FR-T02</t>
+          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
         </is>
       </c>
       <c r="D329" s="3" t="inlineStr">
@@ -19363,12 +19363,12 @@
       </c>
       <c r="B330" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-05</t>
+          <t>E2E-R1-AUDX-03</t>
         </is>
       </c>
       <c r="C330" s="3" t="inlineStr">
         <is>
-          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
+          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
         </is>
       </c>
       <c r="D330" s="3" t="inlineStr">
@@ -19390,12 +19390,12 @@
       </c>
       <c r="B331" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-06</t>
+          <t>E2E-R1-AUDX-04</t>
         </is>
       </c>
       <c r="C331" s="3" t="inlineStr">
         <is>
-          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
+          <t>Chain verify reports intact | FR-T02</t>
         </is>
       </c>
       <c r="D331" s="3" t="inlineStr">
@@ -19417,12 +19417,12 @@
       </c>
       <c r="B332" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-07</t>
+          <t>E2E-R1-AUDX-05</t>
         </is>
       </c>
       <c r="C332" s="3" t="inlineStr">
         <is>
-          <t>`POST /audit/query`: an AND group (category, action prefix, within P30D) sorted ascending pages by cursor; an OR group returns only matching events; unknown fields or values, bad durations, nesting deeper than 2 and unsupported sorts → 422 | BPMS-064, docs/08 §7.5</t>
+          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
         </is>
       </c>
       <c r="D332" s="3" t="inlineStr">
@@ -19444,12 +19444,12 @@
       </c>
       <c r="B333" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-08</t>
+          <t>E2E-R1-AUDX-06</t>
         </is>
       </c>
       <c r="C333" s="3" t="inlineStr">
         <is>
-          <t>A background export (202) runs as a job, finishes `done` with rows, its CSV downloads through the requester's signed file link, the requester is notified, and both `audit.export_requested` and `audit.exported` are recorded | BPMS-064, FR-T04</t>
+          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
         </is>
       </c>
       <c r="D333" s="3" t="inlineStr">
@@ -19471,12 +19471,12 @@
       </c>
       <c r="B334" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-AUDX-07</t>
         </is>
       </c>
       <c r="C334" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work (browser: /setup refuses a bad token or says the platform is already set up; no default account signs in; the full first run needs a fresh database, since the shared E2E database already has system admins) | FR-S01</t>
+          <t>`POST /audit/query`: an AND group (category, action prefix, within P30D) sorted ascending pages by cursor; an OR group returns only matching events; unknown fields or values, bad durations, nesting deeper than 2 and unsupported sorts → 422 | BPMS-064, docs/08 §7.5</t>
         </is>
       </c>
       <c r="D334" s="3" t="inlineStr">
@@ -19498,12 +19498,12 @@
       </c>
       <c r="B335" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-AUDX-08</t>
         </is>
       </c>
       <c r="C335" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA (browser: System › New workspace twice; owner A opens the emailed link, creates the account, turns on two-step verification, signs in and lands in the workspace) | FR-S02/S03, FR-W01</t>
+          <t>A background export (202) runs as a job, finishes `done` with rows, its CSV downloads through the requester's signed file link, the requester is notified, and both `audit.export_requested` and `audit.exported` are recorded | BPMS-064, FR-T04</t>
         </is>
       </c>
       <c r="D335" s="3" t="inlineStr">
@@ -19525,12 +19525,12 @@
       </c>
       <c r="B336" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C336" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email (built: a too-light accent shows a live contrast note with the shade text will use; the server derives 4.5:1 text and 3:1 focus shades; every member's app paints them; a logo uploaded in Settings shows in everyone's sidebar; renaming SOP to "Work Instruction" in Settings › Terminology changes the labels other members see; "Request" has no screens until M6, so its override is covered at unit level) | FR-W04, 05 §7</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work (browser: /setup refuses a bad token or says the platform is already set up; no default account signs in; the full first run needs a fresh database, since the shared E2E database already has system admins) | FR-S01</t>
         </is>
       </c>
       <c r="D336" s="3" t="inlineStr">
@@ -19552,12 +19552,12 @@
       </c>
       <c r="B337" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C337" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error (browser: Members › Import directory › Check shows each row; cycle and unknown member refused; Apply saves the rest; person pages show department, manager and location) | FR-W02</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA (browser: System › New workspace twice; owner A opens the emailed link, creates the account, turns on two-step verification, signs in and lands in the workspace) | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D337" s="3" t="inlineStr">
@@ -19579,12 +19579,12 @@
       </c>
       <c r="B338" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C338" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused (browser: Roles &amp; access › Duplicate › grant to a person for the HR collection; a permission change previews "1 person gains 1 permission"; the holder gets Edit on the HR draft but not the Finance one, and the API agrees; a role manager who lacks audit export cannot put it into a role (403 escalation)) | FR-W03, J6</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email (built: a too-light accent shows a live contrast note with the shade text will use; the server derives 4.5:1 text and 3:1 focus shades; every member's app paints them; a logo uploaded in Settings shows in everyone's sidebar; renaming SOP to "Work Instruction" in Settings › Terminology changes the labels other members see; "Request" has no screens until M6, so its override is covered at unit level) | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D338" s="3" t="inlineStr">
@@ -19606,12 +19606,12 @@
       </c>
       <c r="B339" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C339" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF (browser: the author's Approve is refused; the reviewer confirms with their password after an aged sign-in; Publish › Goes live schedules v2; `/__test/library/due` makes it due without moving the shared clock; v1's printable export carries the Superseded banner) | FR-G04/G05/G10, FR-PL01</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error (browser: Members › Import directory › Check shows each row; cycle and unknown member refused; Apply saves the rest; person pages show department, manager and location) | FR-W02</t>
         </is>
       </c>
       <c r="D339" s="3" t="inlineStr">
@@ -19633,12 +19633,12 @@
       </c>
       <c r="B340" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C340" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method (browser: the owner publishes v2.0 as major, 51 asked; 10 people acknowledge at 390×844 from Home, 40 through the same API; the campaign shows 50 of 51 and the evidence CSV lists the v2 hash and sign-in method for all 50) | FR-PL03, FR-AK01–04</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused (browser: Roles &amp; access › Duplicate › grant to a person for the HR collection; a permission change previews "1 person gains 1 permission"; the holder gets Edit on the HR draft but not the Finance one, and the API agrees; a role manager who lacks audit export cannot put it into a role (403 escalation)) | FR-W03, J6</t>
         </is>
       </c>
       <c r="D340" s="3" t="inlineStr">
@@ -19660,12 +19660,12 @@
       </c>
       <c r="B341" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C341" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns (browser: a campaign created with "Also ask people who join later" on; a new hire who joins from the invitation email after launch finds the request on Home, acknowledges, and shows Done) | FR-AK03</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF (browser: the author's Approve is refused; the reviewer confirms with their password after an aged sign-in; Publish › Goes live schedules v2; `/__test/library/due` makes it due without moving the shared clock; v1's printable export carries the Superseded banner) | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D341" s="3" t="inlineStr">
@@ -19687,12 +19687,12 @@
       </c>
       <c r="B342" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C342" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct (browser: location audience from the directory, confirm-by date, only Bangalore members receive it; the announcement's campaign counts the confirmation; past the deadline the manager of the member who did not confirm is told exactly once; archiving closes the campaign) | FR-AN01–06, J14</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method (browser: the owner publishes v2.0 as major, 51 asked; 10 people acknowledge at 390×844 from Home, 40 through the same API; the campaign shows 50 of 51 and the evidence CSV lists the v2 hash and sign-in method for all 50) | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D342" s="3" t="inlineStr">
@@ -19714,12 +19714,12 @@
       </c>
       <c r="B343" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C343" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it (browser: the drawer says approval is needed, the author sends it, a second admin approves, members see it; at expiry it leaves the feed and admins see it as Expired) | FX-C01, FR-AN03</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns (browser: a campaign created with "Also ask people who join later" on; a new hire who joins from the invitation email after launch finds the request on Home, acknowledges, and shows Done) | FR-AK03</t>
         </is>
       </c>
       <c r="D343" s="3" t="inlineStr">
@@ -19741,12 +19741,12 @@
       </c>
       <c r="B344" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C344" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B (browser: a 50 MB attachment with one chunk dropped resumes and its SHA-256 matches; EICAR shows quarantined and gets no link; links last ≤ 5 minutes, a tampered link is refused, workspace B gets 404 for the link and the file) | FR-F01–F03, SEC-10</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct (browser: location audience from the directory, confirm-by date, only Bangalore members receive it; the announcement's campaign counts the confirmation; past the deadline the manager of the member who did not confirm is told exactly once; archiving closes the campaign) | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D344" s="3" t="inlineStr">
@@ -19768,12 +19768,12 @@
       </c>
       <c r="B345" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C345" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused (browser: Quarantined chip and a Name filter; two files changed to Operational with a reason, shown as set by an admin and audited; deleting a file a published version holds is refused) | FR-F06, FR-V</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it (browser: the drawer says approval is needed, the author sends it, a second admin approves, members see it; at expiry it leaves the feed and admins see it as Expired) | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D345" s="3" t="inlineStr">
@@ -19795,12 +19795,12 @@
       </c>
       <c r="B346" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C346" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction (browser: Status is Published and (Name contains Alpha or Charlie); sort by type then name; view shared with Reviewers opens from the deep link for a reviewer; CSV has exactly the shown rows; XLSX downloads) | FR-V01–V07</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B (browser: a 50 MB attachment with one chunk dropped resumes and its SHA-256 matches; EICAR shows quarantined and gets no link; links last ≤ 5 minutes, a tampered link is refused, workspace B gets 404 for the link and the file) | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D346" s="3" t="inlineStr">
@@ -19822,12 +19822,12 @@
       </c>
       <c r="B347" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C347" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK (browser: Person filter shows only that person's events; a version's timeline is oldest first: three edits, submitted, published; the page shows Chain verified) | FR-T01–T04</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused (browser: Quarantined chip and a Name filter; two files changed to Operational with a reason, shown as set by an admin and audited; deleting a file a published version holds is refused) | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D347" s="3" t="inlineStr">
@@ -19849,12 +19849,12 @@
       </c>
       <c r="B348" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C348" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts (browser: open acknowledgements → active campaigns with the same "still to acknowledge"; versions published → audit log filtered to publications with the same event count; announcements published → the Published tab; without two-step → People &amp; access filtered with the same count) | FR-A01</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction (browser: Status is Published and (Name contains Alpha or Charlie); sort by type then name; view shared with Reviewers opens from the deep link for a reviewer; CSV has exactly the shown rows; XLSX downloads) | FR-V01–V07</t>
         </is>
       </c>
       <c r="D348" s="3" t="inlineStr">
@@ -19876,12 +19876,12 @@
       </c>
       <c r="B349" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C349" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act (browser: owner deactivates from the person page; the member's open tab is sent to the chooser on the next page; signing in again offers no workspace; the API refuses entry) | SEC-04, FR-W01</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK (browser: Person filter shows only that person's events; a version's timeline is oldest first: three edits, submitted, published; the page shows Chain verified) | FR-T01–T04</t>
         </is>
       </c>
       <c r="D349" s="3" t="inlineStr">
@@ -19903,12 +19903,12 @@
       </c>
       <c r="B350" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C350" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore (browser: reads keep working; the first change is refused and a read-only banner appears on every page; after restore the banner is gone and changes work) | FR-S02, J8</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts (browser: open acknowledgements → active campaigns with the same "still to acknowledge"; versions published → audit log filtered to publications with the same event count; announcements published → the Published tab; without two-step → People &amp; access filtered with the same count) | FR-A01</t>
         </is>
       </c>
       <c r="D350" s="3" t="inlineStr">
@@ -19930,12 +19930,12 @@
       </c>
       <c r="B351" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C351" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock (browser: Home › Browse templates › Install the handbook pack (5 drafts) → publish the handbook → launch the campaign → 20 people at 390×844 acknowledge; 20 of 21 done, within 15 minutes) | J12</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act (browser: owner deactivates from the person page; the member's open tab is sent to the chooser on the next page; signing in again offers no workspace; the API refuses entry) | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D351" s="3" t="inlineStr">
@@ -19957,12 +19957,12 @@
       </c>
       <c r="B352" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C352" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse (browser: Tab/Enter/typing only, author from Library to Published, colleague from sign-in to Acknowledged) | A11Y-01, T10</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore (browser: reads keep working; the first change is refused and a read-only banner appears on every page; after restore the banner is gone and changes work) | FR-S02, J8</t>
         </is>
       </c>
       <c r="D352" s="3" t="inlineStr">
@@ -19984,12 +19984,12 @@
       </c>
       <c r="B353" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C353" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` (built: B's owner probes 21 reads and writes on A's documents, versions, exports, campaigns, announcements, collections, departments, views, files and members → all 404, each recorded in B's audit log as `access.denied` with the object id, B's chain verifies, A unchanged) | SEC-01/02</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock (browser: Home › Browse templates › Install the handbook pack (5 drafts) → publish the handbook → launch the campaign → 20 people at 390×844 acknowledge; 20 of 21 done, within 15 minutes) | J12</t>
         </is>
       </c>
       <c r="D353" s="3" t="inlineStr">
@@ -20011,12 +20011,12 @@
       </c>
       <c r="B354" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C354" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse (browser: Tab/Enter/typing only, author from Library to Published, colleague from sign-in to Acknowledged) | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D354" s="3" t="inlineStr">
@@ -20038,12 +20038,12 @@
       </c>
       <c r="B355" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C355" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` (built: B's owner probes 21 reads and writes on A's documents, versions, exports, campaigns, announcements, collections, departments, views, files and members → all 404, each recorded in B's audit log as `access.denied` with the object id, B's chain verifies, A unchanged) | SEC-01/02</t>
         </is>
       </c>
       <c r="D355" s="3" t="inlineStr">
@@ -20065,12 +20065,12 @@
       </c>
       <c r="B356" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C356" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D356" s="3" t="inlineStr">
@@ -20092,12 +20092,12 @@
       </c>
       <c r="B357" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C357" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D357" s="3" t="inlineStr">
@@ -20119,12 +20119,12 @@
       </c>
       <c r="B358" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C358" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D358" s="3" t="inlineStr">
@@ -20146,12 +20146,12 @@
       </c>
       <c r="B359" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C359" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D359" s="3" t="inlineStr">
@@ -20173,12 +20173,12 @@
       </c>
       <c r="B360" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C360" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D360" s="3" t="inlineStr">
@@ -20200,12 +20200,12 @@
       </c>
       <c r="B361" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C361" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D361" s="3" t="inlineStr">
@@ -20227,12 +20227,12 @@
       </c>
       <c r="B362" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C362" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D362" s="3" t="inlineStr">
@@ -20254,12 +20254,12 @@
       </c>
       <c r="B363" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C363" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D363" s="3" t="inlineStr">
@@ -20281,12 +20281,12 @@
       </c>
       <c r="B364" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C364" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D364" s="3" t="inlineStr">
@@ -20308,12 +20308,12 @@
       </c>
       <c r="B365" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C365" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D365" s="3" t="inlineStr">
@@ -20335,12 +20335,12 @@
       </c>
       <c r="B366" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C366" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D366" s="3" t="inlineStr">
@@ -20362,12 +20362,12 @@
       </c>
       <c r="B367" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C367" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D367" s="3" t="inlineStr">
@@ -20389,12 +20389,12 @@
       </c>
       <c r="B368" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C368" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D368" s="3" t="inlineStr">
@@ -20416,12 +20416,12 @@
       </c>
       <c r="B369" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C369" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D369" s="3" t="inlineStr">
@@ -20443,12 +20443,12 @@
       </c>
       <c r="B370" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C370" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D370" s="3" t="inlineStr">
@@ -20470,12 +20470,12 @@
       </c>
       <c r="B371" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C371" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D371" s="3" t="inlineStr">
@@ -20497,12 +20497,12 @@
       </c>
       <c r="B372" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C372" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D372" s="3" t="inlineStr">
@@ -20524,12 +20524,12 @@
       </c>
       <c r="B373" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C373" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D373" s="3" t="inlineStr">
@@ -20551,12 +20551,12 @@
       </c>
       <c r="B374" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C374" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D374" s="3" t="inlineStr">
@@ -20578,12 +20578,12 @@
       </c>
       <c r="B375" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C375" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D375" s="3" t="inlineStr">
@@ -20605,12 +20605,12 @@
       </c>
       <c r="B376" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C376" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D376" s="3" t="inlineStr">
@@ -20632,12 +20632,12 @@
       </c>
       <c r="B377" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C377" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D377" s="3" t="inlineStr">
@@ -20659,12 +20659,12 @@
       </c>
       <c r="B378" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C378" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D378" s="3" t="inlineStr">
@@ -20686,12 +20686,12 @@
       </c>
       <c r="B379" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C379" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D379" s="3" t="inlineStr">
@@ -20713,12 +20713,12 @@
       </c>
       <c r="B380" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C380" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D380" s="3" t="inlineStr">
@@ -20740,12 +20740,12 @@
       </c>
       <c r="B381" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C381" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D381" s="3" t="inlineStr">
@@ -20767,12 +20767,12 @@
       </c>
       <c r="B382" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C382" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D382" s="3" t="inlineStr">
@@ -20794,12 +20794,12 @@
       </c>
       <c r="B383" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C383" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D383" s="3" t="inlineStr">
@@ -20821,12 +20821,12 @@
       </c>
       <c r="B384" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C384" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D384" s="3" t="inlineStr">
@@ -20848,12 +20848,12 @@
       </c>
       <c r="B385" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C385" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D385" s="3" t="inlineStr">
@@ -20875,12 +20875,12 @@
       </c>
       <c r="B386" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C386" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D386" s="3" t="inlineStr">
@@ -20902,12 +20902,12 @@
       </c>
       <c r="B387" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C387" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D387" s="3" t="inlineStr">
@@ -20929,12 +20929,12 @@
       </c>
       <c r="B388" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C388" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D388" s="3" t="inlineStr">
@@ -20956,12 +20956,12 @@
       </c>
       <c r="B389" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C389" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D389" s="3" t="inlineStr">
@@ -20983,12 +20983,12 @@
       </c>
       <c r="B390" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C390" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D390" s="3" t="inlineStr">
@@ -21010,12 +21010,12 @@
       </c>
       <c r="B391" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C391" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D391" s="3" t="inlineStr">
@@ -21037,12 +21037,12 @@
       </c>
       <c r="B392" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C392" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D392" s="3" t="inlineStr">
@@ -21064,12 +21064,12 @@
       </c>
       <c r="B393" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C393" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D393" s="3" t="inlineStr">
@@ -21091,12 +21091,12 @@
       </c>
       <c r="B394" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C394" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D394" s="3" t="inlineStr">
@@ -21118,12 +21118,12 @@
       </c>
       <c r="B395" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C395" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D395" s="3" t="inlineStr">
@@ -21145,12 +21145,12 @@
       </c>
       <c r="B396" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C396" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D396" s="3" t="inlineStr">
@@ -21172,12 +21172,12 @@
       </c>
       <c r="B397" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-11</t>
         </is>
       </c>
       <c r="C397" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
         </is>
       </c>
       <c r="D397" s="3" t="inlineStr">
@@ -21199,12 +21199,12 @@
       </c>
       <c r="B398" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R4-ISO</t>
         </is>
       </c>
       <c r="C398" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
         </is>
       </c>
       <c r="D398" s="3" t="inlineStr">
@@ -21226,12 +21226,12 @@
       </c>
       <c r="B399" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R5-01</t>
         </is>
       </c>
       <c r="C399" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
         </is>
       </c>
       <c r="D399" s="3" t="inlineStr">
@@ -21253,12 +21253,12 @@
       </c>
       <c r="B400" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R5-02</t>
         </is>
       </c>
       <c r="C400" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
         </is>
       </c>
       <c r="D400" s="3" t="inlineStr">
@@ -21280,12 +21280,12 @@
       </c>
       <c r="B401" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R5-03</t>
         </is>
       </c>
       <c r="C401" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
         </is>
       </c>
       <c r="D401" s="3" t="inlineStr">
@@ -21307,12 +21307,12 @@
       </c>
       <c r="B402" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R5-04</t>
         </is>
       </c>
       <c r="C402" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
         </is>
       </c>
       <c r="D402" s="3" t="inlineStr">
@@ -21334,12 +21334,12 @@
       </c>
       <c r="B403" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R5-05</t>
         </is>
       </c>
       <c r="C403" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
         </is>
       </c>
       <c r="D403" s="3" t="inlineStr">
@@ -21361,12 +21361,12 @@
       </c>
       <c r="B404" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R5-06</t>
         </is>
       </c>
       <c r="C404" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
         </is>
       </c>
       <c r="D404" s="3" t="inlineStr">
@@ -21388,12 +21388,12 @@
       </c>
       <c r="B405" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R5-07</t>
         </is>
       </c>
       <c r="C405" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
         </is>
       </c>
       <c r="D405" s="3" t="inlineStr">
@@ -21415,12 +21415,12 @@
       </c>
       <c r="B406" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R5-08</t>
         </is>
       </c>
       <c r="C406" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
         </is>
       </c>
       <c r="D406" s="3" t="inlineStr">
@@ -21442,20 +21442,74 @@
       </c>
       <c r="B407" s="3" t="inlineStr">
         <is>
+          <t>E2E-R5-09</t>
+        </is>
+      </c>
+      <c r="C407" s="3" t="inlineStr">
+        <is>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+        </is>
+      </c>
+      <c r="D407" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E407" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B408" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C408" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D408" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E408" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B409" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C407" s="3" t="inlineStr">
+      <c r="C409" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D407" s="3" t="inlineStr">
+      <c r="D409" s="3" t="inlineStr">
         <is>
           <t>23-E2E-TEST-PLAN.md</t>
         </is>
       </c>
-      <c r="E407" s="3" t="inlineStr">
+      <c r="E409" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
test(e2e): document preview pack E2E-R1-UI-66..69 and as-built notes (BPMS-061)
preview.ui.spec.ts: a two-page PDF (page nav, 100 %/zoom/fit, keyboard,
search), a DOCX in the script-less frame with its outbound link stripped, CSV
and two-sheet XLSX tables, and the download fallback for a .txt and for a zip
posing as .docx (whose preview link is 415). Fixtures build the files in the
test: pdfPages, a stored-zip writer, tinyDocx and tinyXlsx. UI-34 now expects
Preview on a text attachment too (it opens the fallback).

docs/23 registers UI-66..69 and updates UI-34; docs/05 gets the 0.1 as-built
line; docs/06 §5.7 lists the extended preview allow-list. Tracker note
updated and regenerated.

Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E407" headerRowCount="1">
-  <autoFilter ref="A1:E407"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E413" headerRowCount="1">
+  <autoFilter ref="A1:E413"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -6300,7 +6300,7 @@
       <c r="N42" s="3" t="inlineStr"/>
       <c r="O42" s="3" t="inlineStr">
         <is>
-          <t>Image/PDF previews: GET /files/{id}/preview-url (kind image|pdf|none) and GET /files/preview/{token} (own preview HMAC purpose, 2-minute TTL, re-authorized per request; clean PNG/JPEG/GIF/WebP/PDF only by recorded type plus fresh sniff, else 415; inline under CSP sandbox, nosniff, CORP same-origin, no-store; audited file.previewed); JPEG Exif/XMP/IPTC stripped from previews (files.exif_strip); Preview dialog on attachments. E2E-R1-FILE-04, E2E-R1-UI-34. Remaining: separate preview origin, EXIF strip at upload, Office preview (P1).</t>
+          <t>Image/PDF previews: GET /files/{id}/preview-url (kind image|pdf|none) and GET /files/preview/{token} (own preview HMAC purpose, 2-minute TTL, re-authorized per request; clean PNG/JPEG/GIF/WebP/PDF only by recorded type plus fresh sniff, else 415; inline under CSP sandbox, nosniff, CORP same-origin, no-store; audited file.previewed); JPEG Exif/XMP/IPTC stripped from previews (files.exif_strip); one Preview dialog (attachments, Admin › Files) with pdf.js, docx-preview in a script-less sandboxed frame, SheetJS CE and CSV tables, download fallback; DOCX/XLSX checked against the zip central directory. E2E-R1-FILE-04, E2E-R1-UI-34, E2E-R1-UI-66..69. Remaining: separate preview origin, EXIF strip at upload.</t>
         </is>
       </c>
     </row>
@@ -10462,7 +10462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E407"/>
+  <dimension ref="A1:E413"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -17937,7 +17937,7 @@
       </c>
       <c r="C277" s="3" t="inlineStr">
         <is>
-          <t>An author opens Preview on an image attachment: a dialog named after the file shows the image (axe clean); a text attachment offers no Preview; Escape closes it and focus returns | BPMS-061</t>
+          <t>An author opens Preview on an image attachment: a dialog named after the file shows the image (axe clean); a text attachment also offers Preview (fallback, UI-69); Escape closes it and focus returns | BPMS-061</t>
         </is>
       </c>
       <c r="D277" s="3" t="inlineStr">
@@ -18661,12 +18661,12 @@
       </c>
       <c r="B304" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-01</t>
+          <t>E2E-R1-UI-64</t>
         </is>
       </c>
       <c r="C304" s="3" t="inlineStr">
         <is>
-          <t>Onboarding start to finish: the owner invites from Members; the invitee opens the link from the email, creates an account (password confirmation checked) and lands on Home in the workspace; the link then no longer works; the owner sees them Active and opens their person page | BPMS-023</t>
+          <t>System › Email &amp; platform: save SMTP settings (password write-only, "Leave blank to keep the current password"), a test send to a closed port explains the refusal, both audited; platform basics, storage and scanning shown read-only. E2E builds deliver only through PROCERA_SMTP_URL, so saved settings never drain the shared queue | BPMS-065</t>
         </is>
       </c>
       <c r="D304" s="3" t="inlineStr">
@@ -18688,12 +18688,12 @@
       </c>
       <c r="B305" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-02</t>
+          <t>E2E-R1-UI-65</t>
         </is>
       </c>
       <c r="C305" s="3" t="inlineStr">
         <is>
-          <t>Someone with an account opens the invitation email, signs in from the page, comes back to it and joins with one click; an unknown link explains itself | BPMS-023</t>
+          <t>First-time setup continues at /system/setup: an optional email step (skippable) and Create your first workspace, ending with the owner's invitation | BPMS-065</t>
         </is>
       </c>
       <c r="D305" s="3" t="inlineStr">
@@ -18715,12 +18715,12 @@
       </c>
       <c r="B306" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-03</t>
+          <t>E2E-R1-UI-66</t>
         </is>
       </c>
       <c r="C306" s="3" t="inlineStr">
         <is>
-          <t>Policy to evidence: the owner writes and publishes a policy and launches a campaign; a colleague (invited the same way) sees the task on Home, opens the acknowledgement email link, acknowledges on the document; the owner sees them Done, 1 of 2, and downloads the evidence CSV | BPMS-040, 046</t>
+          <t>A two-page PDF previews with pdf.js: Page 1 of 2, next/previous, 100 %, zoom in/out (125 %, 75 %), Fit width, arrow/Home/End keys on the page region, search jumps to the matching page; axe clean | BPMS-061</t>
         </is>
       </c>
       <c r="D306" s="3" t="inlineStr">
@@ -18742,12 +18742,12 @@
       </c>
       <c r="B307" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-04</t>
+          <t>E2E-R1-UI-67</t>
         </is>
       </c>
       <c r="C307" s="3" t="inlineStr">
         <is>
-          <t>Announcement: the owner composes a critical post that needs acknowledgement and publishes it; a colleague opens the email link while signed out, signs in, lands on the open post and confirms; the owner sees the receipt | BPMS-047</t>
+          <t>A DOCX previews its paragraphs in a `sandbox="allow-same-origin"` frame; its external hyperlink keeps the words but no element has `href`, `src` or a script; axe clean | BPMS-061</t>
         </is>
       </c>
       <c r="D307" s="3" t="inlineStr">
@@ -18769,12 +18769,12 @@
       </c>
       <c r="B308" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-05</t>
+          <t>E2E-R1-UI-68</t>
         </is>
       </c>
       <c r="C308" s="3" t="inlineStr">
         <is>
-          <t>Review loop: the owner submits a controlled policy; the reviewer (invited as Reviewer) gets the review email, opens it and requests changes with a comment; the owner gets a notification quoting it, edits and resubmits; the reviewer approves from Home; the owner is told it is approved and publishes | BPMS-040</t>
+          <t>A CSV shows a read-only table (quoted comma field, row numbers, "Read-only. 3 rows."); a two-sheet XLSX shows Q1, and the Sheets tabs switch to Q2; axe clean | BPMS-061</t>
         </is>
       </c>
       <c r="D308" s="3" t="inlineStr">
@@ -18796,12 +18796,12 @@
       </c>
       <c r="B309" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-06</t>
+          <t>E2E-R1-UI-69</t>
         </is>
       </c>
       <c r="C309" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval: a second admin joins from the invitation and turns on two-step verification; the owner sends a workspace-wide post for approval; the admin gets the approval email, opens it and sends it back with a note; the owner gets a notification with the note, edits and resubmits; the admin approves and publishes; the owner is told; the post is in the feed | BPMS-047</t>
+          <t>A .txt and a zip posing as .docx (no `word/document.xml`; its preview link is 415) both show "No preview for this type — download it." with name, size, type and Download; axe clean | BPMS-061</t>
         </is>
       </c>
       <c r="D309" s="3" t="inlineStr">
@@ -18823,12 +18823,12 @@
       </c>
       <c r="B310" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-01</t>
+          <t>E2E-R1-FLOW-01</t>
         </is>
       </c>
       <c r="C310" s="3" t="inlineStr">
         <is>
-          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
+          <t>Onboarding start to finish: the owner invites from Members; the invitee opens the link from the email, creates an account (password confirmation checked) and lands on Home in the workspace; the link then no longer works; the owner sees them Active and opens their person page | BPMS-023</t>
         </is>
       </c>
       <c r="D310" s="3" t="inlineStr">
@@ -18850,12 +18850,12 @@
       </c>
       <c r="B311" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-02</t>
+          <t>E2E-R1-FLOW-02</t>
         </is>
       </c>
       <c r="C311" s="3" t="inlineStr">
         <is>
-          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
+          <t>Someone with an account opens the invitation email, signs in from the page, comes back to it and joins with one click; an unknown link explains itself | BPMS-023</t>
         </is>
       </c>
       <c r="D311" s="3" t="inlineStr">
@@ -18877,12 +18877,12 @@
       </c>
       <c r="B312" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-03</t>
+          <t>E2E-R1-FLOW-03</t>
         </is>
       </c>
       <c r="C312" s="3" t="inlineStr">
         <is>
-          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
+          <t>Policy to evidence: the owner writes and publishes a policy and launches a campaign; a colleague (invited the same way) sees the task on Home, opens the acknowledgement email link, acknowledges on the document; the owner sees them Done, 1 of 2, and downloads the evidence CSV | BPMS-040, 046</t>
         </is>
       </c>
       <c r="D312" s="3" t="inlineStr">
@@ -18904,12 +18904,12 @@
       </c>
       <c r="B313" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-04</t>
+          <t>E2E-R1-FLOW-04</t>
         </is>
       </c>
       <c r="C313" s="3" t="inlineStr">
         <is>
-          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
+          <t>Announcement: the owner composes a critical post that needs acknowledgement and publishes it; a colleague opens the email link while signed out, signs in, lands on the open post and confirms; the owner sees the receipt | BPMS-047</t>
         </is>
       </c>
       <c r="D313" s="3" t="inlineStr">
@@ -18931,12 +18931,12 @@
       </c>
       <c r="B314" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-05</t>
+          <t>E2E-R1-FLOW-05</t>
         </is>
       </c>
       <c r="C314" s="3" t="inlineStr">
         <is>
-          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
+          <t>Review loop: the owner submits a controlled policy; the reviewer (invited as Reviewer) gets the review email, opens it and requests changes with a comment; the owner gets a notification quoting it, edits and resubmits; the reviewer approves from Home; the owner is told it is approved and publishes | BPMS-040</t>
         </is>
       </c>
       <c r="D314" s="3" t="inlineStr">
@@ -18958,12 +18958,12 @@
       </c>
       <c r="B315" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-06</t>
+          <t>E2E-R1-FLOW-06</t>
         </is>
       </c>
       <c r="C315" s="3" t="inlineStr">
         <is>
-          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
+          <t>Announcement approval: a second admin joins from the invitation and turns on two-step verification; the owner sends a workspace-wide post for approval; the admin gets the approval email, opens it and sends it back with a note; the owner gets a notification with the note, edits and resubmits; the admin approves and publishes; the owner is told; the post is in the feed | BPMS-047</t>
         </is>
       </c>
       <c r="D315" s="3" t="inlineStr">
@@ -18985,12 +18985,12 @@
       </c>
       <c r="B316" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-CMP-07</t>
+          <t>E2E-R1-CMP-01</t>
         </is>
       </c>
       <c r="C316" s="3" t="inlineStr">
         <is>
-          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
+          <t>Launching a campaign snapshots the audience (department) and notifies each assignee in-app and by email; non-audience members get nothing; draft preview counts the audience | FR-AK01, FR-AK02, FR-AN05</t>
         </is>
       </c>
       <c r="D316" s="3" t="inlineStr">
@@ -19012,12 +19012,12 @@
       </c>
       <c r="B317" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-01</t>
+          <t>E2E-R1-CMP-02</t>
         </is>
       </c>
       <c r="C317" s="3" t="inlineStr">
         <is>
-          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
+          <t>Acknowledging records the exact version id, content hash and statement; a stale hash is refused (409 content_changed); progress counts update | FR-AK01, FR-PL03, FR-AK04</t>
         </is>
       </c>
       <c r="D317" s="3" t="inlineStr">
@@ -19039,12 +19039,12 @@
       </c>
       <c r="B318" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-02</t>
+          <t>E2E-R1-CMP-03</t>
         </is>
       </c>
       <c r="C318" s="3" t="inlineStr">
         <is>
-          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
+          <t>Only the assignee can acknowledge (others 404), only once (409), only while active; close/cancel rules | FR-AK01, docs/12 §5</t>
         </is>
       </c>
       <c r="D318" s="3" t="inlineStr">
@@ -19066,12 +19066,12 @@
       </c>
       <c r="B319" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-03</t>
+          <t>E2E-R1-CMP-04</t>
         </is>
       </c>
       <c r="C319" s="3" t="inlineStr">
         <is>
-          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
+          <t>Reminder ladder and manager escalation run by the scheduler via drain; overdue list and counts; overdue can still be acknowledged | FR-AK01, FR-AN04</t>
         </is>
       </c>
       <c r="D319" s="3" t="inlineStr">
@@ -19093,12 +19093,12 @@
       </c>
       <c r="B320" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-04</t>
+          <t>E2E-R1-CMP-05</t>
         </is>
       </c>
       <c r="C320" s="3" t="inlineStr">
         <is>
-          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
+          <t>A new member matching a dynamic audience is enrolled (own window); at-launch campaigns stay fixed | FR-AK03</t>
         </is>
       </c>
       <c r="D320" s="3" t="inlineStr">
@@ -19120,12 +19120,12 @@
       </c>
       <c r="B321" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-05</t>
+          <t>E2E-R1-CMP-06</t>
         </is>
       </c>
       <c r="C321" s="3" t="inlineStr">
         <is>
-          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
+          <t>Evidence CSV lists every assignee with department, timestamps, version, content hash and auth method; members cannot export | FR-AK04, CMP-03</t>
         </is>
       </c>
       <c r="D321" s="3" t="inlineStr">
@@ -19147,12 +19147,12 @@
       </c>
       <c r="B322" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ANN-06</t>
+          <t>E2E-R1-CMP-07</t>
         </is>
       </c>
       <c r="C322" s="3" t="inlineStr">
         <is>
-          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
+          <t>Members cannot manage or track campaigns; a compliance officer can; draft version 409, empty audience 422; another workspace gets 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D322" s="3" t="inlineStr">
@@ -19174,12 +19174,12 @@
       </c>
       <c r="B323" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-01</t>
+          <t>E2E-R1-ANN-01</t>
         </is>
       </c>
       <c r="C323" s="3" t="inlineStr">
         <is>
-          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
+          <t>Compose → edit with If-Match → publish to a department: only its members see it; first read recorded; in-app + email delivery after drain; edits after publish 409; content hash frozen | FR-AN01..03, FR-AN05</t>
         </is>
       </c>
       <c r="D323" s="3" t="inlineStr">
@@ -19201,12 +19201,12 @@
       </c>
       <c r="B324" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-02</t>
+          <t>E2E-R1-ANN-02</t>
         </is>
       </c>
       <c r="C324" s="3" t="inlineStr">
         <is>
-          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
+          <t>Workspace-wide posts need approval; self-approval 403 sod_violation; publisher approves; reject needs a comment and returns the draft | FX-C01, FR-AN02</t>
         </is>
       </c>
       <c r="D324" s="3" t="inlineStr">
@@ -19228,12 +19228,12 @@
       </c>
       <c r="B325" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-SRCH-03</t>
+          <t>E2E-R1-ANN-03</t>
         </is>
       </c>
       <c r="C325" s="3" t="inlineStr">
         <is>
-          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
+          <t>Scheduled announcement goes live after clock + drain; expiry removes it from feeds (state stays published, expired: true) | FR-AN03</t>
         </is>
       </c>
       <c r="D325" s="3" t="inlineStr">
@@ -19255,12 +19255,12 @@
       </c>
       <c r="B326" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-01</t>
+          <t>E2E-R1-ANN-04</t>
         </is>
       </c>
       <c r="C326" s="3" t="inlineStr">
         <is>
-          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
+          <t>Required ack on a critical announcement; idempotent ack; analytics reconcile by department; archive needs a reason | FR-AN04, FR-AN06</t>
         </is>
       </c>
       <c r="D326" s="3" t="inlineStr">
@@ -19282,12 +19282,12 @@
       </c>
       <c r="B327" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-02</t>
+          <t>E2E-R1-ANN-05</t>
         </is>
       </c>
       <c r="C327" s="3" t="inlineStr">
         <is>
-          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
+          <t>Permissions and isolation: members read the feed but cannot compose; authors see only their drafts; other workspaces 404 | docs/12 §5</t>
         </is>
       </c>
       <c r="D327" s="3" t="inlineStr">
@@ -19309,12 +19309,12 @@
       </c>
       <c r="B328" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-03</t>
+          <t>E2E-R1-ANN-06</t>
         </is>
       </c>
       <c r="C328" s="3" t="inlineStr">
         <is>
-          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
+          <t>Settings drive approval, ack default, expiry default and the enabled switch | docs/20 §2.17</t>
         </is>
       </c>
       <c r="D328" s="3" t="inlineStr">
@@ -19336,12 +19336,12 @@
       </c>
       <c r="B329" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-04</t>
+          <t>E2E-R1-SRCH-01</t>
         </is>
       </c>
       <c r="C329" s="3" t="inlineStr">
         <is>
-          <t>Chain verify reports intact | FR-T02</t>
+          <t>Ranked results across SOPs, policies, people, departments, groups; escaped highlighted snippets; typo and prefix matches; type filter; validation errors | BPMS-049, docs/05 §2.4</t>
         </is>
       </c>
       <c r="D329" s="3" t="inlineStr">
@@ -19363,12 +19363,12 @@
       </c>
       <c r="B330" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-05</t>
+          <t>E2E-R1-SRCH-02</t>
         </is>
       </c>
       <c r="C330" s="3" t="inlineStr">
         <is>
-          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
+          <t>A SOP-only role sees only SOP results; other types filtered on the server | docs/12 §3</t>
         </is>
       </c>
       <c r="D330" s="3" t="inlineStr">
@@ -19390,12 +19390,12 @@
       </c>
       <c r="B331" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-06</t>
+          <t>E2E-R1-SRCH-03</t>
         </is>
       </c>
       <c r="C331" s="3" t="inlineStr">
         <is>
-          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
+          <t>Another workspace's content is never found; draft edits are searchable at once | docs/06 T-22</t>
         </is>
       </c>
       <c r="D331" s="3" t="inlineStr">
@@ -19417,12 +19417,12 @@
       </c>
       <c r="B332" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-07</t>
+          <t>E2E-R1-AUDX-01</t>
         </is>
       </c>
       <c r="C332" s="3" t="inlineStr">
         <is>
-          <t>`POST /audit/query`: an AND group (category, action prefix, within P30D) sorted ascending pages by cursor; an OR group returns only matching events; unknown fields or values, bad durations, nesting deeper than 2 and unsupported sorts → 422 | BPMS-064, docs/08 §7.5</t>
+          <t>Explorer filters, newest-first keyset pagination without duplicates, actor names, validation | BPMS-064, FR-T03</t>
         </is>
       </c>
       <c r="D332" s="3" t="inlineStr">
@@ -19444,12 +19444,12 @@
       </c>
       <c r="B333" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-AUDX-08</t>
+          <t>E2E-R1-AUDX-02</t>
         </is>
       </c>
       <c r="C333" s="3" t="inlineStr">
         <is>
-          <t>A background export (202) runs as a job, finishes `done` with rows, its CSV downloads through the requester's signed file link, the requester is notified, and both `audit.export_requested` and `audit.exported` are recorded | BPMS-064, FR-T04</t>
+          <t>audit:view_own sees only own events; verify/export forbidden; no permission 403 | docs/12 §5</t>
         </is>
       </c>
       <c r="D333" s="3" t="inlineStr">
@@ -19471,12 +19471,12 @@
       </c>
       <c r="B334" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-01</t>
+          <t>E2E-R1-AUDX-03</t>
         </is>
       </c>
       <c r="C334" s="3" t="inlineStr">
         <is>
-          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work (browser: /setup refuses a bad token or says the platform is already set up; no default account signs in; the full first run needs a fresh database, since the shared E2E database already has system admins) | FR-S01</t>
+          <t>Artifact timeline covers all versions, oldest first | FR-T04</t>
         </is>
       </c>
       <c r="D334" s="3" t="inlineStr">
@@ -19498,12 +19498,12 @@
       </c>
       <c r="B335" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-02</t>
+          <t>E2E-R1-AUDX-04</t>
         </is>
       </c>
       <c r="C335" s="3" t="inlineStr">
         <is>
-          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA (browser: System › New workspace twice; owner A opens the emailed link, creates the account, turns on two-step verification, signs in and lands in the workspace) | FR-S02/S03, FR-W01</t>
+          <t>Chain verify reports intact | FR-T02</t>
         </is>
       </c>
       <c r="D335" s="3" t="inlineStr">
@@ -19525,12 +19525,12 @@
       </c>
       <c r="B336" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-03</t>
+          <t>E2E-R1-AUDX-05</t>
         </is>
       </c>
       <c r="C336" s="3" t="inlineStr">
         <is>
-          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email (built: a too-light accent shows a live contrast note with the shade text will use; the server derives 4.5:1 text and 3:1 focus shades; every member's app paints them; a logo uploaded in Settings shows in everyone's sidebar; renaming SOP to "Work Instruction" in Settings › Terminology changes the labels other members see; "Request" has no screens until M6, so its override is covered at unit level) | FR-W04, 05 §7</t>
+          <t>Saved queries: create, duplicate 409, validation 422, private per member, delete; audited | FR-T03, FR-T01</t>
         </is>
       </c>
       <c r="D336" s="3" t="inlineStr">
@@ -19552,12 +19552,12 @@
       </c>
       <c r="B337" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-04</t>
+          <t>E2E-R1-AUDX-06</t>
         </is>
       </c>
       <c r="C337" s="3" t="inlineStr">
         <is>
-          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error (browser: Members › Import directory › Check shows each row; cycle and unknown member refused; Apply saves the rest; person pages show department, manager and location) | FR-W02</t>
+          <t>CSV and JSONL exports honour filters, need step-up, and are audited | FR-T01, docs/12 §11</t>
         </is>
       </c>
       <c r="D337" s="3" t="inlineStr">
@@ -19579,12 +19579,12 @@
       </c>
       <c r="B338" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-05</t>
+          <t>E2E-R1-AUDX-07</t>
         </is>
       </c>
       <c r="C338" s="3" t="inlineStr">
         <is>
-          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused (browser: Roles &amp; access › Duplicate › grant to a person for the HR collection; a permission change previews "1 person gains 1 permission"; the holder gets Edit on the HR draft but not the Finance one, and the API agrees; a role manager who lacks audit export cannot put it into a role (403 escalation)) | FR-W03, J6</t>
+          <t>`POST /audit/query`: an AND group (category, action prefix, within P30D) sorted ascending pages by cursor; an OR group returns only matching events; unknown fields or values, bad durations, nesting deeper than 2 and unsupported sorts → 422 | BPMS-064, docs/08 §7.5</t>
         </is>
       </c>
       <c r="D338" s="3" t="inlineStr">
@@ -19606,12 +19606,12 @@
       </c>
       <c r="B339" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-06</t>
+          <t>E2E-R1-AUDX-08</t>
         </is>
       </c>
       <c r="C339" s="3" t="inlineStr">
         <is>
-          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF (browser: the author's Approve is refused; the reviewer confirms with their password after an aged sign-in; Publish › Goes live schedules v2; `/__test/library/due` makes it due without moving the shared clock; v1's printable export carries the Superseded banner) | FR-G04/G05/G10, FR-PL01</t>
+          <t>A background export (202) runs as a job, finishes `done` with rows, its CSV downloads through the requester's signed file link, the requester is notified, and both `audit.export_requested` and `audit.exported` are recorded | BPMS-064, FR-T04</t>
         </is>
       </c>
       <c r="D339" s="3" t="inlineStr">
@@ -19633,12 +19633,12 @@
       </c>
       <c r="B340" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-07</t>
+          <t>E2E-R1-01</t>
         </is>
       </c>
       <c r="C340" s="3" t="inlineStr">
         <is>
-          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method (browser: the owner publishes v2.0 as major, 51 asked; 10 people acknowledge at 390×844 from Home, 40 through the same API; the campaign shows 50 of 51 and the evidence CSV lists the v2 hash and sign-in method for all 50) | FR-PL03, FR-AK01–04</t>
+          <t>Bootstrap: one-time token → system owner enrols MFA → no default credentials work (browser: /setup refuses a bad token or says the platform is already set up; no default account signs in; the full first run needs a fresh database, since the shared E2E database already has system admins) | FR-S01</t>
         </is>
       </c>
       <c r="D340" s="3" t="inlineStr">
@@ -19660,12 +19660,12 @@
       </c>
       <c r="B341" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-08</t>
+          <t>E2E-R1-02</t>
         </is>
       </c>
       <c r="C341" s="3" t="inlineStr">
         <is>
-          <t>New joiner added to a department automatically receives outstanding applicable campaigns (browser: a campaign created with "Also ask people who join later" on; a new hire who joins from the invitation email after launch finds the request on Home, acknowledges, and shows Done) | FR-AK03</t>
+          <t>System admin creates workspace A (Starter) and B (Enterprise), invites owners; owners accept via Mailpit link and enrol MFA (browser: System › New workspace twice; owner A opens the emailed link, creates the account, turns on two-step verification, signs in and lands in the workspace) | FR-S02/S03, FR-W01</t>
         </is>
       </c>
       <c r="D341" s="3" t="inlineStr">
@@ -19687,12 +19687,12 @@
       </c>
       <c r="B342" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-09</t>
+          <t>E2E-R1-03</t>
         </is>
       </c>
       <c r="C342" s="3" t="inlineStr">
         <is>
-          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct (browser: location audience from the directory, confirm-by date, only Bangalore members receive it; the announcement's campaign counts the confirmation; past the deadline the manager of the member who did not confirm is told exactly once; archiving closes the campaign) | FR-AN01–06, J14</t>
+          <t>Workspace owner sets branding; a low-contrast accent is auto-adjusted or rejected; terminology override ("Request" → "Ticket") shows in UI and email (built: a too-light accent shows a live contrast note with the shade text will use; the server derives 4.5:1 text and 3:1 focus shades; every member's app paints them; a logo uploaded in Settings shows in everyone's sidebar; renaming SOP to "Work Instruction" in Settings › Terminology changes the labels other members see; "Request" has no screens until M6, so its override is covered at unit level) | FR-W04, 05 §7</t>
         </is>
       </c>
       <c r="D342" s="3" t="inlineStr">
@@ -19714,12 +19714,12 @@
       </c>
       <c r="B343" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-10</t>
+          <t>E2E-R1-04</t>
         </is>
       </c>
       <c r="C343" s="3" t="inlineStr">
         <is>
-          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it (browser: the drawer says approval is needed, the author sends it, a second admin approves, members see it; at expiry it leaves the feed and admins see it as Expired) | FX-C01, FR-AN03</t>
+          <t>Directory CSV import (departments, managers); a manager cycle is rejected with a clear error (browser: Members › Import directory › Check shows each row; cycle and unknown member refused; Apply saves the rest; person pages show department, manager and location) | FR-W02</t>
         </is>
       </c>
       <c r="D343" s="3" t="inlineStr">
@@ -19741,12 +19741,12 @@
       </c>
       <c r="B344" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-11</t>
+          <t>E2E-R1-05</t>
         </is>
       </c>
       <c r="C344" s="3" t="inlineStr">
         <is>
-          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B (browser: a 50 MB attachment with one chunk dropped resumes and its SHA-256 matches; EICAR shows quarantined and gets no link; links last ≤ 5 minutes, a tampered link is refused, workspace B gets 404 for the link and the file) | FR-F01–F03, SEC-10</t>
+          <t>Clone "Process Designer" → "HR Designer" scoped to the HR collection; preview count is correct; the scope is enforced on UI and API; adding a permission the editor lacks is refused (browser: Roles &amp; access › Duplicate › grant to a person for the HR collection; a permission change previews "1 person gains 1 permission"; the holder gets Edit on the HR draft but not the Finance one, and the API agrees; a role manager who lacks audit export cannot put it into a role (403 escalation)) | FR-W03, J6</t>
         </is>
       </c>
       <c r="D344" s="3" t="inlineStr">
@@ -19768,12 +19768,12 @@
       </c>
       <c r="B345" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-12</t>
+          <t>E2E-R1-06</t>
         </is>
       </c>
       <c r="C345" s="3" t="inlineStr">
         <is>
-          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused (browser: Quarantined chip and a Name filter; two files changed to Operational with a reason, shown as set by an admin and audited; deleting a file a published version holds is refused) | FR-F06, FR-V</t>
+          <t>Policy authored → submitted → self-approval blocked (SoD) → reviewer approves with step-up → scheduled → published at effective date (test clock) → old version watermarked as superseded in PDF (browser: the author's Approve is refused; the reviewer confirms with their password after an aged sign-in; Publish › Goes live schedules v2; `/__test/library/due` makes it due without moving the shared clock; v1's printable export carries the Superseded banner) | FR-G04/G05/G10, FR-PL01</t>
         </is>
       </c>
       <c r="D345" s="3" t="inlineStr">
@@ -19795,12 +19795,12 @@
       </c>
       <c r="B346" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-13</t>
+          <t>E2E-R1-07</t>
         </is>
       </c>
       <c r="C346" s="3" t="inlineStr">
         <is>
-          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction (browser: Status is Published and (Name contains Alpha or Charlie); sort by type then name; view shared with Reviewers opens from the deep link for a reviewer; CSV has exactly the shown rows; XLSX downloads) | FR-V01–V07</t>
+          <t>Major version publish triggers a re-ack campaign; 50 employees ack (10 at mobile viewport); evidence export lists version hash and auth method (browser: the owner publishes v2.0 as major, 51 asked; 10 people acknowledge at 390×844 from Home, 40 through the same API; the campaign shows 50 of 51 and the evidence CSV lists the v2 hash and sign-in method for all 50) | FR-PL03, FR-AK01–04</t>
         </is>
       </c>
       <c r="D346" s="3" t="inlineStr">
@@ -19822,12 +19822,12 @@
       </c>
       <c r="B347" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-14</t>
+          <t>E2E-R1-08</t>
         </is>
       </c>
       <c r="C347" s="3" t="inlineStr">
         <is>
-          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK (browser: Person filter shows only that person's events; a version's timeline is oldest first: three edits, submitted, published; the page shows Chain verified) | FR-T01–T04</t>
+          <t>New joiner added to a department automatically receives outstanding applicable campaigns (browser: a campaign created with "Also ask people who join later" on; a new hire who joins from the invitation email after launch finds the request on Home, acknowledges, and shows Done) | FR-AK03</t>
         </is>
       </c>
       <c r="D347" s="3" t="inlineStr">
@@ -19849,12 +19849,12 @@
       </c>
       <c r="B348" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-15</t>
+          <t>E2E-R1-09</t>
         </is>
       </c>
       <c r="C348" s="3" t="inlineStr">
         <is>
-          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts (browser: open acknowledgements → active campaigns with the same "still to acknowledge"; versions published → audit log filtered to publications with the same event count; announcements published → the Published tab; without two-step → People &amp; access filtered with the same count) | FR-A01</t>
+          <t>Announcement to location "Bangalore" with ack in 3 days; reminders; manager escalation after deadline (test clock); ack % by department correct (browser: location audience from the directory, confirm-by date, only Bangalore members receive it; the announcement's campaign counts the confirmation; past the deadline the manager of the member who did not confirm is told exactly once; archiving closes the campaign) | FR-AN01–06, J14</t>
         </is>
       </c>
       <c r="D348" s="3" t="inlineStr">
@@ -19876,12 +19876,12 @@
       </c>
       <c r="B349" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-16</t>
+          <t>E2E-R1-10</t>
         </is>
       </c>
       <c r="C349" s="3" t="inlineStr">
         <is>
-          <t>Member deactivated → sessions revoked immediately → cannot log in or act (browser: owner deactivates from the person page; the member's open tab is sent to the chooser on the next page; signing in again offers no workspace; the API refuses entry) | SEC-04, FR-W01</t>
+          <t>Announcement approval workflow: draft → reviewer → publish; expiry archives it (browser: the drawer says approval is needed, the author sends it, a second admin approves, members see it; at expiry it leaves the feed and admins see it as Expired) | FX-C01, FR-AN03</t>
         </is>
       </c>
       <c r="D349" s="3" t="inlineStr">
@@ -19903,12 +19903,12 @@
       </c>
       <c r="B350" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-17</t>
+          <t>E2E-R1-11</t>
         </is>
       </c>
       <c r="C350" s="3" t="inlineStr">
         <is>
-          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore (browser: reads keep working; the first change is refused and a read-only banner appears on every page; after restore the banner is gone and changes work) | FR-S02, J8</t>
+          <t>File upload (resumable 50 MB): clean file previews; **EICAR quarantined** and undownloadable; signed URL expires and fails from workspace B (browser: a 50 MB attachment with one chunk dropped resumes and its SHA-256 matches; EICAR shows quarantined and gets no link; links last ≤ 5 minutes, a tampered link is refused, workspace B gets 404 for the link and the file) | FR-F01–F03, SEC-10</t>
         </is>
       </c>
       <c r="D350" s="3" t="inlineStr">
@@ -19930,12 +19930,12 @@
       </c>
       <c r="B351" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-18</t>
+          <t>E2E-R1-12</t>
         </is>
       </c>
       <c r="C351" s="3" t="inlineStr">
         <is>
-          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock (browser: Home › Browse templates › Install the handbook pack (5 drafts) → publish the handbook → launch the campaign → 20 people at 390×844 acknowledge; 20 of 21 done, within 15 minutes) | J12</t>
+          <t>Files view: filter by scan state/type/size, bulk retention change, held file deletion refused (browser: Quarantined chip and a Name filter; two files changed to Operational with a reason, shown as set by an admin and audited; deleting a file a published version holds is refused) | FR-F06, FR-V</t>
         </is>
       </c>
       <c r="D351" s="3" t="inlineStr">
@@ -19957,12 +19957,12 @@
       </c>
       <c r="B352" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-19</t>
+          <t>E2E-R1-13</t>
         </is>
       </c>
       <c r="C352" s="3" t="inlineStr">
         <is>
-          <t>Keyboard-only: publish a policy and acknowledge it without a mouse (browser: Tab/Enter/typing only, author from Library to Published, colleague from sign-in to Acknowledged) | A11Y-01, T10</t>
+          <t>DataGrid: multi-sort, typed filters, AND/OR group, saved view shared to a role, URL deep link restores view, CSV/XLSX export matches view and redaction (browser: Status is Published and (Name contains Alpha or Charlie); sort by type then name; view shared with Reviewers opens from the deep link for a reviewer; CSV has exactly the shown rows; XLSX downloads) | FR-V01–V07</t>
         </is>
       </c>
       <c r="D352" s="3" t="inlineStr">
@@ -19984,12 +19984,12 @@
       </c>
       <c r="B353" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-ISO</t>
+          <t>E2E-R1-14</t>
         </is>
       </c>
       <c r="C353" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` (built: B's owner probes 21 reads and writes on A's documents, versions, exports, campaigns, announcements, collections, departments, views, files and members → all 404, each recorded in B's audit log as `access.denied` with the object id, B's chain verifies, A unchanged) | SEC-01/02</t>
+          <t>Audit: perform 10 actions → audit explorer filter by actor → user timeline shows them in order → `/__test/audit/verify` OK (browser: Person filter shows only that person's events; a version's timeline is oldest first: three edits, submitted, published; the page shows Chain verified) | FR-T01–T04</t>
         </is>
       </c>
       <c r="D353" s="3" t="inlineStr">
@@ -20011,12 +20011,12 @@
       </c>
       <c r="B354" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-01</t>
+          <t>E2E-R1-15</t>
         </is>
       </c>
       <c r="C354" s="3" t="inlineStr">
         <is>
-          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
+          <t>Workspace overview dashboard: every tile drills into a pre-filtered grid with matching counts (browser: open acknowledgements → active campaigns with the same "still to acknowledge"; versions published → audit log filtered to publications with the same event count; announcements published → the Published tab; without two-step → People &amp; access filtered with the same count) | FR-A01</t>
         </is>
       </c>
       <c r="D354" s="3" t="inlineStr">
@@ -20038,12 +20038,12 @@
       </c>
       <c r="B355" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-02</t>
+          <t>E2E-R1-16</t>
         </is>
       </c>
       <c r="C355" s="3" t="inlineStr">
         <is>
-          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
+          <t>Member deactivated → sessions revoked immediately → cannot log in or act (browser: owner deactivates from the person page; the member's open tab is sent to the chooser on the next page; signing in again offers no workspace; the API refuses entry) | SEC-04, FR-W01</t>
         </is>
       </c>
       <c r="D355" s="3" t="inlineStr">
@@ -20065,12 +20065,12 @@
       </c>
       <c r="B356" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-03</t>
+          <t>E2E-R1-17</t>
         </is>
       </c>
       <c r="C356" s="3" t="inlineStr">
         <is>
-          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
+          <t>System admin suspends workspace B (read-only) → writes return 423 with banner → restore (browser: reads keep working; the first change is refused and a read-only banner appears on every page; after restore the banner is gone and changes work) | FR-S02, J8</t>
         </is>
       </c>
       <c r="D356" s="3" t="inlineStr">
@@ -20092,12 +20092,12 @@
       </c>
       <c r="B357" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-04</t>
+          <t>E2E-R1-18</t>
         </is>
       </c>
       <c r="C357" s="3" t="inlineStr">
         <is>
-          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
+          <t>Startup day-one (J12): Starter profile → install policy-ack pack → publish handbook → 20 employees ack on phones in &lt; 15 min wall-clock (browser: Home › Browse templates › Install the handbook pack (5 drafts) → publish the handbook → launch the campaign → 20 people at 390×844 acknowledge; 20 of 21 done, within 15 minutes) | J12</t>
         </is>
       </c>
       <c r="D357" s="3" t="inlineStr">
@@ -20119,12 +20119,12 @@
       </c>
       <c r="B358" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-05</t>
+          <t>E2E-R1-19</t>
         </is>
       </c>
       <c r="C358" s="3" t="inlineStr">
         <is>
-          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
+          <t>Keyboard-only: publish a policy and acknowledge it without a mouse (browser: Tab/Enter/typing only, author from Library to Published, colleague from sign-in to Acknowledged) | A11Y-01, T10</t>
         </is>
       </c>
       <c r="D358" s="3" t="inlineStr">
@@ -20146,12 +20146,12 @@
       </c>
       <c r="B359" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-06</t>
+          <t>E2E-R1-ISO</t>
         </is>
       </c>
       <c r="C359" s="3" t="inlineStr">
         <is>
-          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
+          <t>Isolation sweep: B users probe every A object id captured during the pack → 404 + audit `denied` (built: B's owner probes 21 reads and writes on A's documents, versions, exports, campaigns, announcements, collections, departments, views, files and members → all 404, each recorded in B's audit log as `access.denied` with the object id, B's chain verifies, A unchanged) | SEC-01/02</t>
         </is>
       </c>
       <c r="D359" s="3" t="inlineStr">
@@ -20173,12 +20173,12 @@
       </c>
       <c r="B360" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-07</t>
+          <t>E2E-R2-01</t>
         </is>
       </c>
       <c r="C360" s="3" t="inlineStr">
         <is>
-          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
+          <t>Install "Purchase requisition", map role placeholders, test run (no emails sent, nothing in metrics), publish | FR-G08, FR-E11</t>
         </is>
       </c>
       <c r="D360" s="3" t="inlineStr">
@@ -20200,12 +20200,12 @@
       </c>
       <c r="B361" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-08</t>
+          <t>E2E-R2-02</t>
         </is>
       </c>
       <c r="C361" s="3" t="inlineStr">
         <is>
-          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
+          <t>Purchase 30 000 → manager approves; 120 000 → rule table routes to finance; rule version recorded in timeline | FR-E10, J3</t>
         </is>
       </c>
       <c r="D361" s="3" t="inlineStr">
@@ -20227,12 +20227,12 @@
       </c>
       <c r="B362" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-09</t>
+          <t>E2E-R2-03</t>
         </is>
       </c>
       <c r="C362" s="3" t="inlineStr">
         <is>
-          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
+          <t>Duplicate submit with the same Idempotency-Key returns the same request; a different body returns 409 | 08 §2</t>
         </is>
       </c>
       <c r="D362" s="3" t="inlineStr">
@@ -20254,12 +20254,12 @@
       </c>
       <c r="B363" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-10</t>
+          <t>E2E-R2-04</t>
         </is>
       </c>
       <c r="C363" s="3" t="inlineStr">
         <is>
-          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
+          <t>Double approval race:** two approvers decide concurrently → exactly one commit, the other gets `already_decided` | T01</t>
         </is>
       </c>
       <c r="D363" s="3" t="inlineStr">
@@ -20281,12 +20281,12 @@
       </c>
       <c r="B364" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-11</t>
+          <t>E2E-R2-05</t>
         </is>
       </c>
       <c r="C364" s="3" t="inlineStr">
         <is>
-          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
+          <t>Kill worker after commit** (fault) → instance still progresses after restart; no duplicate email | T02</t>
         </is>
       </c>
       <c r="D364" s="3" t="inlineStr">
@@ -20308,12 +20308,12 @@
       </c>
       <c r="B365" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-12</t>
+          <t>E2E-R2-06</t>
         </is>
       </c>
       <c r="C365" s="3" t="inlineStr">
         <is>
-          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
+          <t>30-day wait timer: publish v2 mid-flight → advance clock 30 d → instance completes on pinned v1 | T03, FR-E07</t>
         </is>
       </c>
       <c r="D365" s="3" t="inlineStr">
@@ -20335,12 +20335,12 @@
       </c>
       <c r="B366" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-13</t>
+          <t>E2E-R2-07</t>
         </is>
       </c>
       <c r="C366" s="3" t="inlineStr">
         <is>
-          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
+          <t>Onboarding (J1): HR starts, manager approves, parallel IT + facilities tasks join, employee tracks progress | J1</t>
         </is>
       </c>
       <c r="D366" s="3" t="inlineStr">
@@ -20362,12 +20362,12 @@
       </c>
       <c r="B367" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-14</t>
+          <t>E2E-R2-08</t>
         </is>
       </c>
       <c r="C367" s="3" t="inlineStr">
         <is>
-          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
+          <t>Out-of-office: manager sets a substitute → new approvals route to them → "on behalf of" recorded → expiry restores routing → substitute who is the initiator is excluded (SoD) | FR-E04, J7, T05</t>
         </is>
       </c>
       <c r="D367" s="3" t="inlineStr">
@@ -20389,12 +20389,12 @@
       </c>
       <c r="B368" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-15</t>
+          <t>E2E-R2-09</t>
         </is>
       </c>
       <c r="C368" s="3" t="inlineStr">
         <is>
-          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
+          <t>Send back to an earlier step with comment → requester edits → resubmits → approver sees diff | FX-E05</t>
         </is>
       </c>
       <c r="D368" s="3" t="inlineStr">
@@ -20416,12 +20416,12 @@
       </c>
       <c r="B369" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-16</t>
+          <t>E2E-R2-10</t>
         </is>
       </c>
       <c r="C369" s="3" t="inlineStr">
         <is>
-          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
+          <t>SLA on business calendar (IN holidays) → at-risk → breach notification to process owner (test clock) | FR-E12</t>
         </is>
       </c>
       <c r="D369" s="3" t="inlineStr">
@@ -20443,12 +20443,12 @@
       </c>
       <c r="B370" s="3" t="inlineStr">
         <is>
-          <t>E2E-R2-ISO</t>
+          <t>E2E-R2-11</t>
         </is>
       </c>
       <c r="C370" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
+          <t>Escalation reassign after P2D; controlled process forbids auto-approve | 11 §3.2</t>
         </is>
       </c>
       <c r="D370" s="3" t="inlineStr">
@@ -20470,12 +20470,12 @@
       </c>
       <c r="B371" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-01</t>
+          <t>E2E-R2-12</t>
         </is>
       </c>
       <c r="C371" s="3" t="inlineStr">
         <is>
-          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
+          <t>Form: calculation, conditional section, repeating line items, URL prefill, server rejects tampered payload | FR-E03, FX-F01–F03</t>
         </is>
       </c>
       <c r="D371" s="3" t="inlineStr">
@@ -20497,12 +20497,12 @@
       </c>
       <c r="B372" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-02</t>
+          <t>E2E-R2-13</t>
         </is>
       </c>
       <c r="C372" s="3" t="inlineStr">
         <is>
-          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
+          <t>Designer keyboard-only: build a 4-step process, validation errors link to nodes, publish | FR-E01, T10</t>
         </is>
       </c>
       <c r="D372" s="3" t="inlineStr">
@@ -20524,12 +20524,12 @@
       </c>
       <c r="B373" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-03</t>
+          <t>E2E-R2-14</t>
         </is>
       </c>
       <c r="C373" s="3" t="inlineStr">
         <is>
-          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
+          <t>Failed step raises an incident → admin retries → instance continues; exactly one open incident | FR-E13</t>
         </is>
       </c>
       <c r="D373" s="3" t="inlineStr">
@@ -20551,12 +20551,12 @@
       </c>
       <c r="B374" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-04</t>
+          <t>E2E-R2-15</t>
         </is>
       </c>
       <c r="C374" s="3" t="inlineStr">
         <is>
-          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
+          <t>My Work: j/k/a triage, decision in ≤ 3 interactions, acks tab shows pending campaigns | FR-R03</t>
         </is>
       </c>
       <c r="D374" s="3" t="inlineStr">
@@ -20578,12 +20578,12 @@
       </c>
       <c r="B375" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-05</t>
+          <t>E2E-R2-16</t>
         </is>
       </c>
       <c r="C375" s="3" t="inlineStr">
         <is>
-          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
+          <t>Restricted variable (salary) hidden from approver without grant in UI, API, export, email body and search | SEC-03</t>
         </is>
       </c>
       <c r="D375" s="3" t="inlineStr">
@@ -20605,12 +20605,12 @@
       </c>
       <c r="B376" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-06</t>
+          <t>E2E-R2-ISO</t>
         </is>
       </c>
       <c r="C376" s="3" t="inlineStr">
         <is>
-          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
+          <t>Isolation sweep incl. work items, requests, forms, rule tables | SEC-01/02</t>
         </is>
       </c>
       <c r="D376" s="3" t="inlineStr">
@@ -20632,12 +20632,12 @@
       </c>
       <c r="B377" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-07</t>
+          <t>E2E-R3-01</t>
         </is>
       </c>
       <c r="C377" s="3" t="inlineStr">
         <is>
-          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
+          <t>Admin monitoring (J9): overview → 12 overdue in Finance → filtered grid → bulk reassign with reason and preview → per-item audit → save view | J9, FR-A02/A03</t>
         </is>
       </c>
       <c r="D377" s="3" t="inlineStr">
@@ -20659,12 +20659,12 @@
       </c>
       <c r="B378" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-08</t>
+          <t>E2E-R3-02</t>
         </is>
       </c>
       <c r="C378" s="3" t="inlineStr">
         <is>
-          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
+          <t>DoA matrix: amount and position limits route to the correct approver; matrix version pinned | FX-D01/D02</t>
         </is>
       </c>
       <c r="D378" s="3" t="inlineStr">
@@ -20686,12 +20686,12 @@
       </c>
       <c r="B379" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-09</t>
+          <t>E2E-R3-03</t>
         </is>
       </c>
       <c r="C379" s="3" t="inlineStr">
         <is>
-          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
+          <t>Recall/withdraw then restart as a linked copy; edit-after-submit with per-step editable fields | FX-E04/E06</t>
         </is>
       </c>
       <c r="D379" s="3" t="inlineStr">
@@ -20713,12 +20713,12 @@
       </c>
       <c r="B380" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-10</t>
+          <t>E2E-R3-04</t>
         </is>
       </c>
       <c r="C380" s="3" t="inlineStr">
         <is>
-          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
+          <t>Request on behalf of: beneficiary sees status; initiator ≠ beneficiary in audit | FX-E03</t>
         </is>
       </c>
       <c r="D380" s="3" t="inlineStr">
@@ -20740,12 +20740,12 @@
       </c>
       <c r="B381" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-11</t>
+          <t>E2E-R3-05</t>
         </is>
       </c>
       <c r="C381" s="3" t="inlineStr">
         <is>
-          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
+          <t>Master data: CSV import of cost centres → cascading dropdown in form → version change doesn't alter running requests | FX-E02</t>
         </is>
       </c>
       <c r="D381" s="3" t="inlineStr">
@@ -20767,12 +20767,12 @@
       </c>
       <c r="B382" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-12</t>
+          <t>E2E-R3-06</t>
         </is>
       </c>
       <c r="C382" s="3" t="inlineStr">
         <is>
-          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
+          <t>E-sign: upload PDF, place fields (mouse and keyboard), sequential then parallel signers, consent step, sign on mobile, certificate of completion, tamper check fails after byte change | FR-DS01–DS06</t>
         </is>
       </c>
       <c r="D382" s="3" t="inlineStr">
@@ -20794,12 +20794,12 @@
       </c>
       <c r="B383" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-MOB</t>
+          <t>E2E-R3-07</t>
         </is>
       </c>
       <c r="C383" s="3" t="inlineStr">
         <is>
-          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
+          <t>Bulk sign 1 000 recipients** (J13): async progress, reminders, decline with reason, manager escalation, overdue export | J13</t>
         </is>
       </c>
       <c r="D383" s="3" t="inlineStr">
@@ -20821,12 +20821,12 @@
       </c>
       <c r="B384" s="3" t="inlineStr">
         <is>
-          <t>E2E-R3-ISO</t>
+          <t>E2E-R3-08</t>
         </is>
       </c>
       <c r="C384" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
+          <t>"Not e-signable" template flag blocks sending with guidance | FX-S06</t>
         </is>
       </c>
       <c r="D384" s="3" t="inlineStr">
@@ -20848,12 +20848,12 @@
       </c>
       <c r="B385" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-01</t>
+          <t>E2E-R3-09</t>
         </is>
       </c>
       <c r="C385" s="3" t="inlineStr">
         <is>
-          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
+          <t>File lifecycle (J11): invoice attached, scanned, previewed, locked on completion, visible in Files view with retention class | J11</t>
         </is>
       </c>
       <c r="D385" s="3" t="inlineStr">
@@ -20875,12 +20875,12 @@
       </c>
       <c r="B386" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-02</t>
+          <t>E2E-R3-10</t>
         </is>
       </c>
       <c r="C386" s="3" t="inlineStr">
         <is>
-          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
+          <t>BPMN import of a sample with an inclusive gateway → compatibility report lists the element id | FR-G09</t>
         </is>
       </c>
       <c r="D386" s="3" t="inlineStr">
@@ -20902,12 +20902,12 @@
       </c>
       <c r="B387" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-03</t>
+          <t>E2E-R3-11</t>
         </is>
       </c>
       <c r="C387" s="3" t="inlineStr">
         <is>
-          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
+          <t>Process health and ops monitor numbers reconcile with raw events | FR-A04/A05</t>
         </is>
       </c>
       <c r="D387" s="3" t="inlineStr">
@@ -20929,12 +20929,12 @@
       </c>
       <c r="B388" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-04</t>
+          <t>E2E-R3-12</t>
         </is>
       </c>
       <c r="C388" s="3" t="inlineStr">
         <is>
-          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
+          <t>All 13 Wave-1 templates: install → test run green (data-driven) | TPL-*, 19</t>
         </is>
       </c>
       <c r="D388" s="3" t="inlineStr">
@@ -20956,12 +20956,12 @@
       </c>
       <c r="B389" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-05</t>
+          <t>E2E-R3-MOB</t>
         </is>
       </c>
       <c r="C389" s="3" t="inlineStr">
         <is>
-          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
+          <t>Mobile pack (360×740, touch): start request, approve, ack, sign | FR-P07</t>
         </is>
       </c>
       <c r="D389" s="3" t="inlineStr">
@@ -20983,12 +20983,12 @@
       </c>
       <c r="B390" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-06</t>
+          <t>E2E-R3-ISO</t>
         </is>
       </c>
       <c r="C390" s="3" t="inlineStr">
         <is>
-          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
+          <t>Isolation sweep incl. envelopes, master data, files | SEC-01/02/10</t>
         </is>
       </c>
       <c r="D390" s="3" t="inlineStr">
@@ -21010,12 +21010,12 @@
       </c>
       <c r="B391" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-07</t>
+          <t>E2E-R4-01</t>
         </is>
       </c>
       <c r="C391" s="3" t="inlineStr">
         <is>
-          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
+          <t>OIDC SSO via Keycloak; SSO enforcement blocks local login except break-glass owner | FR-P02</t>
         </is>
       </c>
       <c r="D391" s="3" t="inlineStr">
@@ -21037,12 +21037,12 @@
       </c>
       <c r="B392" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-08</t>
+          <t>E2E-R4-02</t>
         </is>
       </c>
       <c r="C392" s="3" t="inlineStr">
         <is>
-          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
+          <t>SCIM create/update/deactivate → access revoked and work re-routed &lt; 5 min | INT-003, SEC-04</t>
         </is>
       </c>
       <c r="D392" s="3" t="inlineStr">
@@ -21064,12 +21064,12 @@
       </c>
       <c r="B393" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-09</t>
+          <t>E2E-R4-03</t>
         </is>
       </c>
       <c r="C393" s="3" t="inlineStr">
         <is>
-          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
+          <t>Scoped admin (Finance dept) cannot see or grant outside scope; escalation attempt denied | CFG-018</t>
         </is>
       </c>
       <c r="D393" s="3" t="inlineStr">
@@ -21091,12 +21091,12 @@
       </c>
       <c r="B394" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-10</t>
+          <t>E2E-R4-04</t>
         </is>
       </c>
       <c r="C394" s="3" t="inlineStr">
         <is>
-          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
+          <t>Webhook delivered with valid Standard Webhooks signature; replay outside tolerance rejected by receiver; retries on 500; disabled on 410 | WH-01–04</t>
         </is>
       </c>
       <c r="D394" s="3" t="inlineStr">
@@ -21118,12 +21118,12 @@
       </c>
       <c r="B395" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-11</t>
+          <t>E2E-R4-05</t>
         </is>
       </c>
       <c r="C395" s="3" t="inlineStr">
         <is>
-          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
+          <t>HTTP connector to `169.254.169.254` and to private IP refused (SSRF); allowlisted host OK | SSRF-01–06</t>
         </is>
       </c>
       <c r="D395" s="3" t="inlineStr">
@@ -21145,12 +21145,12 @@
       </c>
       <c r="B396" s="3" t="inlineStr">
         <is>
-          <t>E2E-R4-ISO</t>
+          <t>E2E-R4-06</t>
         </is>
       </c>
       <c r="C396" s="3" t="inlineStr">
         <is>
-          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
+          <t>Email-actionable approval: link → confirm page → approve; reusing link fails; a GET never mutates | FR-N03</t>
         </is>
       </c>
       <c r="D396" s="3" t="inlineStr">
@@ -21172,12 +21172,12 @@
       </c>
       <c r="B397" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-01</t>
+          <t>E2E-R4-07</t>
         </is>
       </c>
       <c r="C397" s="3" t="inlineStr">
         <is>
-          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
+          <t>External signer via magic link + email OTP; link single-use | FR-DS02, FR-P08</t>
         </is>
       </c>
       <c r="D397" s="3" t="inlineStr">
@@ -21199,12 +21199,12 @@
       </c>
       <c r="B398" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-02</t>
+          <t>E2E-R4-08</t>
         </is>
       </c>
       <c r="C398" s="3" t="inlineStr">
         <is>
-          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
+          <t>Envelope correction (change recipient email) audited; DOCX + merge fields; anchor tags place fields | FX-S03/S09</t>
         </is>
       </c>
       <c r="D398" s="3" t="inlineStr">
@@ -21226,12 +21226,12 @@
       </c>
       <c r="B399" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-03</t>
+          <t>E2E-R4-09</t>
         </is>
       </c>
       <c r="C399" s="3" t="inlineStr">
         <is>
-          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
+          <t>Public form with CAPTCHA + rate limit; save &amp; resume | FX-F05/F06</t>
         </is>
       </c>
       <c r="D399" s="3" t="inlineStr">
@@ -21253,12 +21253,12 @@
       </c>
       <c r="B400" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-04</t>
+          <t>E2E-R4-10</t>
         </is>
       </c>
       <c r="C400" s="3" t="inlineStr">
         <is>
-          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
+          <t>Config export from sandbox → import into prod workspace shows diff; secrets absent | FR-W12, FR-P09</t>
         </is>
       </c>
       <c r="D400" s="3" t="inlineStr">
@@ -21280,12 +21280,12 @@
       </c>
       <c r="B401" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-05</t>
+          <t>E2E-R4-11</t>
         </is>
       </c>
       <c r="C401" s="3" t="inlineStr">
         <is>
-          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+          <t>API token scoped to `request:start` cannot read audit | 12 §5</t>
         </is>
       </c>
       <c r="D401" s="3" t="inlineStr">
@@ -21307,12 +21307,12 @@
       </c>
       <c r="B402" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-06</t>
+          <t>E2E-R4-ISO</t>
         </is>
       </c>
       <c r="C402" s="3" t="inlineStr">
         <is>
-          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+          <t>Isolation sweep incl. tokens, webhooks, connectors | SEC-</t>
         </is>
       </c>
       <c r="D402" s="3" t="inlineStr">
@@ -21334,12 +21334,12 @@
       </c>
       <c r="B403" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-07</t>
+          <t>E2E-R5-01</t>
         </is>
       </c>
       <c r="C403" s="3" t="inlineStr">
         <is>
-          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+          <t>Incident case (J4): intake → evidence → ad hoc tasks → closure blocked until checklist done → audit export | J4, FR-C01/C02</t>
         </is>
       </c>
       <c r="D403" s="3" t="inlineStr">
@@ -21361,12 +21361,12 @@
       </c>
       <c r="B404" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-08</t>
+          <t>E2E-R5-02</t>
         </is>
       </c>
       <c r="C404" s="3" t="inlineStr">
         <is>
-          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+          <t>Restricted HR case invisible in global search, reports, dashboards, notifications; admin self-grant is audited and visible to case team | FX-K06, OQ-12</t>
         </is>
       </c>
       <c r="D404" s="3" t="inlineStr">
@@ -21388,12 +21388,12 @@
       </c>
       <c r="B405" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-09</t>
+          <t>E2E-R5-03</t>
         </is>
       </c>
       <c r="C405" s="3" t="inlineStr">
         <is>
-          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+          <t>Investigation (J10): filter `data_access` on `salary` → pin events/files → legal hold → signed export → `procera-verify` offline passes; edited bundle fails | J10, FR-T05/T06, AUD-05</t>
         </is>
       </c>
       <c r="D405" s="3" t="inlineStr">
@@ -21415,12 +21415,12 @@
       </c>
       <c r="B406" s="3" t="inlineStr">
         <is>
-          <t>E2E-R5-10</t>
+          <t>E2E-R5-04</t>
         </is>
       </c>
       <c r="C406" s="3" t="inlineStr">
         <is>
-          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+          <t>Legal hold blocks retention purge and file deletion; release by authorised role resumes | PRV-03</t>
         </is>
       </c>
       <c r="D406" s="3" t="inlineStr">
@@ -21442,20 +21442,182 @@
       </c>
       <c r="B407" s="3" t="inlineStr">
         <is>
+          <t>E2E-R5-05</t>
+        </is>
+      </c>
+      <c r="C407" s="3" t="inlineStr">
+        <is>
+          <t>Part 11 mode: approval requires re-auth; manifestation shows name/time/meaning; signature bound to record hash | ESIG-01–05</t>
+        </is>
+      </c>
+      <c r="D407" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E407" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B408" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-06</t>
+        </is>
+      </c>
+      <c r="C408" s="3" t="inlineStr">
+        <is>
+          <t>Attestation campaign + access review; unconfirmed grants expire | FR-G06, FR-W11</t>
+        </is>
+      </c>
+      <c r="D408" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E408" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B409" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-07</t>
+        </is>
+      </c>
+      <c r="C409" s="3" t="inlineStr">
+        <is>
+          <t>Break-glass: system admin request → workspace approval → read-only session banner → auto-expiry → visible in workspace audit | FR-S07</t>
+        </is>
+      </c>
+      <c r="D409" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E409" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B410" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-08</t>
+        </is>
+      </c>
+      <c r="C410" s="3" t="inlineStr">
+        <is>
+          <t>Separation mode on → workspace admin loses content access → audited self-grant flow | 12 §6.1</t>
+        </is>
+      </c>
+      <c r="D410" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E410" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B411" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-09</t>
+        </is>
+      </c>
+      <c r="C411" s="3" t="inlineStr">
+        <is>
+          <t>Scheduled report re-applies permissions at run time (user lost access → no data sent) | FX-A02</t>
+        </is>
+      </c>
+      <c r="D411" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E411" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B412" s="3" t="inlineStr">
+        <is>
+          <t>E2E-R5-10</t>
+        </is>
+      </c>
+      <c r="C412" s="3" t="inlineStr">
+        <is>
+          <t>AI drafting (when enabled): output is a draft, labelled, provenance in audit; cannot publish or approve | ADR-0006</t>
+        </is>
+      </c>
+      <c r="D412" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E412" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="3" t="inlineStr">
+        <is>
+          <t>E2E scenarios (E2E)</t>
+        </is>
+      </c>
+      <c r="B413" s="3" t="inlineStr">
+        <is>
           <t>E2E-R5-ISO</t>
         </is>
       </c>
-      <c r="C407" s="3" t="inlineStr">
+      <c r="C413" s="3" t="inlineStr">
         <is>
           <t>Isolation sweep incl. cases, investigations, evidence | SEC-</t>
         </is>
       </c>
-      <c r="D407" s="3" t="inlineStr">
-        <is>
-          <t>23-E2E-TEST-PLAN.md</t>
-        </is>
-      </c>
-      <c r="E407" s="3" t="inlineStr">
+      <c r="D413" s="3" t="inlineStr">
+        <is>
+          <t>23-E2E-TEST-PLAN.md</t>
+        </is>
+      </c>
+      <c r="E413" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
chore(tracker): document preview, invite links, reader view, leaving flow, department usage
Signed-off-by: sachin sarwa <schnsrw@gmail.com>
</commit_message>
<xml_diff>
--- a/trackers/Delivery_Tracker.xlsx
+++ b/trackers/Delivery_Tracker.xlsx
@@ -197,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E43" headerRowCount="1">
-  <autoFilter ref="A1:E43"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AssumptionsT" displayName="AssumptionsT" ref="A1:E44" headerRowCount="1">
+  <autoFilter ref="A1:E44"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Source"/>
     <tableColumn id="2" name="ID"/>
@@ -250,8 +250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E413" headerRowCount="1">
-  <autoFilter ref="A1:E413"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DomainBacklogT" displayName="DomainBacklogT" ref="A1:E418" headerRowCount="1">
+  <autoFilter ref="A1:E418"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Domain"/>
     <tableColumn id="2" name="ID"/>
@@ -1393,7 +1393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2519,6 +2519,33 @@
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>22-UNKNOWNS-ASSUMPTIONS-AND-OPEN-QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>A-44 (BPMS-023/046)</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Leaving the organisation (0.1). Deactivation is the leaving step; a 3-step dialog (Review, Hand over, Confirm) deactivates first, then hands documents to a new owner and direct reports to a new manager through the existing audited endpoints (`PUT /artifacts/{id}/owner`, `PATCH /members/{id}`). The hand-over default follows `directory.deactivation.reassign_strategy`: `manager` picks their manager when they have one; `fallback` and `process_owner` (no process owners yet) pick the admin doing it. Their open assignments in active campaigns close as `left` (migration 0038) by the `membership.deactivated.v1` consumer, audited `campaign.recipient_left` by the system, never as acknowledged; `left` assignments are frozen, leave the progress counts (`progress.left` reports them) and are not reopened on reactivation (A-41). Drafts, campaigns, groups and grants are listed for review but not moved: grants stay so reactivation can restore them.</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Owner direction 2026-10-13</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -4809,7 +4836,7 @@
       <c r="N19" s="3" t="inlineStr"/>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>procera-members + /api/v1: memberships, invitations (hashed + sealed tokens, 7-day expiry, email-bound, single use; list, revoke, resend), register-by-invite, owner onboarding activates the workspace, workspace switch (ws-scoped JWT), deactivation guards, state gate (423). Directory (migration 0008): department tree (uuid[] paths, sibling-unique names, no moves under descendants), static groups, positions (behind directory.positions.enabled), manager links with cycle rejection, deterministic manager resolution (explicit → nearest department head), per-field source attribution, CSV import with plan/apply. All audited; E2E-R1-MEM-01..03,05..07, E2E-R1-DIR-01..04 Invitation page /invite (GET /invitations/preview, A-24): create account and join, or sign in and join; deep links survive sign-in. E2E-R1-FLOW-01, 02. Directory import UI with a check step and per-row reasons (E2E-R1-04); deactivate from the person page with immediate session exit (E2E-R1-16); person page with department, manager and location. Directory UI: Departments page (tree, add, rename, move, head, delete only when empty), Groups (list, group page, members), editable person profile with groups, reactivate with step-up and reason (A-41), resend and revoke invitations, bulk set department and add to group. E2E-R1-UI-51..55. Later: people list per department, Used by, group owners.</t>
+          <t>procera-members + /api/v1: memberships, invitations (hashed + sealed tokens, 7-day expiry, email-bound, single use; list, revoke, resend), register-by-invite, owner onboarding activates the workspace, workspace switch (ws-scoped JWT), deactivation guards, state gate (423). Directory (migration 0008): department tree (uuid[] paths, sibling-unique names, no moves under descendants), static groups, positions (behind directory.positions.enabled), manager links with cycle rejection, deterministic manager resolution (explicit → nearest department head), per-field source attribution, CSV import with plan/apply. All audited; E2E-R1-MEM-01..03,05..07, E2E-R1-DIR-01..04 Invitation page /invite (GET /invitations/preview, A-24): create account and join, or sign in and join; deep links survive sign-in. E2E-R1-FLOW-01, 02. Directory import UI with a check step and per-row reasons (E2E-R1-04); deactivate from the person page with immediate session exit (E2E-R1-16); person page with department, manager and location. Directory UI: Departments page (tree, add, rename, move, head, delete only when empty), Groups (list, group page, members), editable person profile with groups, reactivate with step-up and reason (A-41), resend and revoke invitations, bulk set department and add to group. E2E-R1-UI-51..55. Later: people list per department, Used by, group owners. 0.1 gaps: copy an invitation link when email isn't set up (members and the owner invite), leaving the organisation as a 3-step flow (review, hand over, confirm), department people and Used by. E2E-R1-UI-71..72, 74..75.</t>
         </is>
       </c>
     </row>
@@ -5585,7 +5612,7 @@
       <c r="N31" s="3" t="inlineStr"/>
       <c r="O31" s="3" t="inlineStr">
         <is>
-          <t>procera-library (migration 0012): artifacts + versions for SOPs and policies; lifecycle draft → in_review → approved → scheduled/published → deprecated → retired with guarded transitions; one open draft per artifact; reviews in numbered rounds, approvals from governance.review.* settings, author never reviews own version, distinct approvers, comment required to reject; content_hash = SHA-256(JCS) frozen at approval and a trigger forbids changing approved content or moving back (T07); publish supersedes, future effective_at schedules (worker + drain), reason for change on later versions, retire; step-up for controlled approve/publish; outbox artifact.published.v1; every transition audited. E2E-R1-LIB-01..05. Process artifacts arrive with the designer/compiler Review notifications (A-25): reviewers told on submit (in-app + email), author told the outcome with the comment. E2E-R1-FLOW-03, 05.</t>
+          <t>procera-library (migration 0012): artifacts + versions for SOPs and policies; lifecycle draft → in_review → approved → scheduled/published → deprecated → retired with guarded transitions; one open draft per artifact; reviews in numbered rounds, approvals from governance.review.* settings, author never reviews own version, distinct approvers, comment required to reject; content_hash = SHA-256(JCS) frozen at approval and a trigger forbids changing approved content or moving back (T07); publish supersedes, future effective_at schedules (worker + drain), reason for change on later versions, retire; step-up for controlled approve/publish; outbox artifact.published.v1; every transition audited. E2E-R1-LIB-01..05. Process artifacts arrive with the designer/compiler Review notifications (A-25): reviewers told on submit (in-app + email), author told the outcome with the comment. E2E-R1-FLOW-03, 05. Clean reading view for plain readers (details tucked away); authors aren't offered review of their own version. E2E-R1-UI-73.</t>
         </is>
       </c>
     </row>
@@ -5975,7 +6002,7 @@
       <c r="N37" s="3" t="inlineStr"/>
       <c r="O37" s="3" t="inlineStr">
         <is>
-          <t>procera-campaigns (migration 0013): acknowledgement campaigns for a published SOP/policy version; audience via the shared resolver (snapshot or dynamic), assignments with in-app + email notices, acknowledgement bound to version id + content hash + statement + auth method, reminder ladder and one-time manager escalation by the scheduler, dynamic new joiners, close/cancel, progress, audited evidence CSV; settings campaign.*; E2E-R1-CMP-01..07. Later: quiz-lite, exemptions, signed PDF evidence, auto re-ack on major publish Campaign subjects include announcements (0033).</t>
+          <t>procera-campaigns (migration 0013): acknowledgement campaigns for a published SOP/policy version; audience via the shared resolver (snapshot or dynamic), assignments with in-app + email notices, acknowledgement bound to version id + content hash + statement + auth method, reminder ladder and one-time manager escalation by the scheduler, dynamic new joiners, close/cancel, progress, audited evidence CSV; settings campaign.*; E2E-R1-CMP-01..07. Later: quiz-lite, exemptions, signed PDF evidence, auto re-ack on major publish Campaign subjects include announcements (0033). Leavers' pending acknowledgements close as left organisation (migration 0038), excluded from progress, never marked acknowledged.</t>
         </is>
       </c>
     </row>
@@ -10462,7 +10489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E413"/>
+  <dimension ref="A1:E418"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -18823,12 +18850,12 @@
       </c>
       <c r="B310" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-01</t>
+          <t>E2E-R1-UI-71</t>
         </is>
       </c>
       <c r="C310" s="3" t="inlineStr">
         <is>
-          <t>Onboarding start to finish: the owner invites from Members; the invitee opens the link from the email, creates an account (password confirmation checked) and lands on Home in the workspace; the link then no longer works; the owner sees them Active and opens their person page | BPMS-023</t>
+          <t>Copy owner invite link (no email set up): after creating a workspace and again from its row the system admin gets a one-time link; the newer link opens the join page, the earlier one no longer works; both copies on the system audit | BPMS-020</t>
         </is>
       </c>
       <c r="D310" s="3" t="inlineStr">
@@ -18850,12 +18877,12 @@
       </c>
       <c r="B311" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-02</t>
+          <t>E2E-R1-UI-72</t>
         </is>
       </c>
       <c r="C311" s="3" t="inlineStr">
         <is>
-          <t>Someone with an account opens the invitation email, signs in from the page, comes back to it and joins with one click; an unknown link explains itself | BPMS-023</t>
+          <t>Copy invite link on Members for a pending invitation: the dialog shows the link and who it is for; it opens the join page; the token never appears in the invitation list | BPMS-023</t>
         </is>
       </c>
       <c r="D311" s="3" t="inlineStr">
@@ -18877,12 +18904,12 @@
       </c>
       <c r="B312" s="3" t="inlineStr">
         <is>
-          <t>E2E-R1-FLOW-03</t>
+          <t>E2E-R1-UI-73</t>
         </is>
       </c>
       <c r="C312" s="3" t="inlineStr">
         <is>
-          <t>Policy to evidence: the o